<commit_message>
QA 리비전 열 I = 1848231 (video-261014b · 어둠막 0.75)
· I8 = 1848231 · I6 비고. 요약 다섯 수식과 N7 「버전」을 I 열로 옮겼다.
· H(bf98a1c)는 비어 있어도 덮지 않았다 — 그 빌드는 video-261014 태그가 붙었고
  사용자 2차 육안 「Fail 없음」을 받은 빌드다. 태그 붙은 빌드의 열은 기록으로 남긴다.

값 0 · 코드 0.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -294,6 +294,11 @@
           <t xml:space="preserve">#130 T3 DIM·문구</t>
         </is>
       </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">video-261014b · 어둠막 0.55→0.75 (T1·T3) · H(bf98a1c)=video-261014 2차 육안 Fail 0</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -332,7 +337,7 @@
       </c>
       <c r="N7" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">bf98a1c</t>
+          <t xml:space="preserve">1848231</t>
         </is>
       </c>
     </row>
@@ -365,14 +370,18 @@
           <t xml:space="preserve">bf98a1c</t>
         </is>
       </c>
-      <c r="I8" s="2"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1848231</t>
+        </is>
+      </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">PASSrate</t>
         </is>
       </c>
       <c r="N8" s="7">
-        <f>COUNTIF(H9:H111,"Pass")</f>
+        <f>COUNTIF(I9:I111,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -415,7 +424,7 @@
         </is>
       </c>
       <c r="N9" s="7">
-        <f>COUNTIF(H9:H111,"Fail")+COUNTIF(H9:H111,"Broken")</f>
+        <f>COUNTIF(I9:I111,"Fail")+COUNTIF(I9:I111,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -458,7 +467,7 @@
         </is>
       </c>
       <c r="N10" s="7">
-        <f>COUNTIF(H9:H111,"N/A")</f>
+        <f>COUNTIF(I9:I111,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -544,7 +553,7 @@
         </is>
       </c>
       <c r="N12" s="7">
-        <f>TEXT((COUNTA(H9:H111))/103,"0.00%")</f>
+        <f>TEXT((COUNTA(I9:I111))/103,"0.00%")</f>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
QA I열(1848231) — 10-15 코드 세션 실플레이 40칸 (Pass 36 · Fail 4)
576×1024 · 소리 0 · 새 저장 · 튜토리얼 → S1 파밍(T3) → S1 도전 자연 통과 →
「스테이지로」 → 조립 진입 → 새로고침(저장 복원). 지나간 항목만 적고 나머지는 빈 칸.
사용자 지시(10-15) 「문제 발생 시 체크만 하고 다음 스텝으로」 — 멈추지 않고 끝까지 갔다.

Fail 4 (증상은 I6 비고):
· CID_014 「- 일시 정지 -」 오른끝이 마일스톤 카드에 가림
· CID_021 설정에 「보드 좌표 덤프」·「현재 적 전멸」 노출 — 촬영 빌드가 개발 빌드
· CID_032 T3 막이 HUD 위로 안 덮임 — 전장만 어두움(잠금·「도전」 빛남·문구는 정상)
· CID_055 극소 창 결과 단추 잘림 = #122 보류(보통 창 정상)

곁 고침: 조건부 서식 범위 G9:I111 → G9:L111. 어제 J~L 을 늘리면서 안 넓혔다 —
그대로면 J~L 판정이 색을 못 입는다.

값 0 · 코드 0. 고친 결함 0(수정 여부 = 사용자).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -296,7 +296,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">video-261014b · 어둠막 0.55→0.75 (T1·T3) · H(bf98a1c)=video-261014 2차 육안 Fail 0</t>
+          <t xml:space="preserve">video-261014b · 어둠막 0.55→0.75 (T1·T3) · H(bf98a1c)=video-261014 2차 육안 Fail 0 ‖ 10-15 코드 세션 실플레이(576×1024 · 소리 0 · 새 저장 · 튜토→S1 도전 자연 통과→스테이지로→새로고침) · Pass 36 · Fail 4 · 빈 칸 = 안 지나감 · Fail: CID_014 「- 일시 정지 -」 오른끝이 마일스톤 카드에 가림 / CID_021 설정에 「보드 좌표 덤프」·「현재 적 전멸」 노출 = 촬영 빌드가 개발 빌드 / CID_032 T3 막이 HUD(상단 칩·Stage 띠·배지·로봇B/Auto/합체 원형) 위로 안 덮임 — 전장만 어두움(잠금·「도전」 빛남·문구는 정상) / CID_055 극소 창(≈253px) 셋째 단추 잘림 = #122 보류(보통 창은 정상)</t>
         </is>
       </c>
       <c r="J6" s="2"/>
@@ -426,7 +426,11 @@
       </c>
       <c r="G9" s="7"/>
       <c r="H9" s="7"/>
-      <c r="I9" s="7"/>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J9" s="7"/>
       <c r="K9" s="7"/>
       <c r="L9" s="7"/>
@@ -610,7 +614,11 @@
       </c>
       <c r="G13" s="7"/>
       <c r="H13" s="7"/>
-      <c r="I13" s="7"/>
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J13" s="7"/>
       <c r="K13" s="7"/>
       <c r="L13" s="7"/>
@@ -676,7 +684,11 @@
       </c>
       <c r="G15" s="7"/>
       <c r="H15" s="7"/>
-      <c r="I15" s="7"/>
+      <c r="I15" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J15" s="7"/>
       <c r="K15" s="7"/>
       <c r="L15" s="7"/>
@@ -709,7 +721,11 @@
       </c>
       <c r="G16" s="7"/>
       <c r="H16" s="7"/>
-      <c r="I16" s="7"/>
+      <c r="I16" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J16" s="7"/>
       <c r="K16" s="7"/>
       <c r="L16" s="7"/>
@@ -747,7 +763,11 @@
       </c>
       <c r="G17" s="7"/>
       <c r="H17" s="7"/>
-      <c r="I17" s="7"/>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J17" s="7"/>
       <c r="K17" s="7"/>
       <c r="L17" s="7"/>
@@ -884,7 +904,11 @@
       </c>
       <c r="G21" s="7"/>
       <c r="H21" s="7"/>
-      <c r="I21" s="7"/>
+      <c r="I21" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J21" s="7"/>
       <c r="K21" s="7"/>
       <c r="L21" s="7"/>
@@ -922,7 +946,11 @@
       </c>
       <c r="G22" s="7"/>
       <c r="H22" s="7"/>
-      <c r="I22" s="7"/>
+      <c r="I22" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
       <c r="J22" s="7"/>
       <c r="K22" s="7"/>
       <c r="L22" s="7"/>
@@ -1163,7 +1191,11 @@
       </c>
       <c r="G29" s="7"/>
       <c r="H29" s="7"/>
-      <c r="I29" s="7"/>
+      <c r="I29" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
       <c r="J29" s="7"/>
       <c r="K29" s="7"/>
       <c r="L29" s="7"/>
@@ -1196,7 +1228,11 @@
       </c>
       <c r="G30" s="7"/>
       <c r="H30" s="7"/>
-      <c r="I30" s="7"/>
+      <c r="I30" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J30" s="7"/>
       <c r="K30" s="7"/>
       <c r="L30" s="7"/>
@@ -1234,7 +1270,11 @@
       </c>
       <c r="G31" s="7"/>
       <c r="H31" s="7"/>
-      <c r="I31" s="7"/>
+      <c r="I31" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J31" s="7"/>
       <c r="K31" s="7"/>
       <c r="L31" s="7"/>
@@ -1267,7 +1307,11 @@
       </c>
       <c r="G32" s="7"/>
       <c r="H32" s="7"/>
-      <c r="I32" s="7"/>
+      <c r="I32" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J32" s="7"/>
       <c r="K32" s="7"/>
       <c r="L32" s="7"/>
@@ -1300,7 +1344,11 @@
       </c>
       <c r="G33" s="7"/>
       <c r="H33" s="7"/>
-      <c r="I33" s="7"/>
+      <c r="I33" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J33" s="7"/>
       <c r="K33" s="7"/>
       <c r="L33" s="7"/>
@@ -1333,7 +1381,11 @@
       </c>
       <c r="G34" s="7"/>
       <c r="H34" s="7"/>
-      <c r="I34" s="7"/>
+      <c r="I34" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J34" s="7"/>
       <c r="K34" s="7"/>
       <c r="L34" s="7"/>
@@ -1371,7 +1423,11 @@
       </c>
       <c r="G35" s="7"/>
       <c r="H35" s="7"/>
-      <c r="I35" s="7"/>
+      <c r="I35" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J35" s="7"/>
       <c r="K35" s="7"/>
       <c r="L35" s="7"/>
@@ -1404,7 +1460,11 @@
       </c>
       <c r="G36" s="7"/>
       <c r="H36" s="7"/>
-      <c r="I36" s="7"/>
+      <c r="I36" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J36" s="7"/>
       <c r="K36" s="7"/>
       <c r="L36" s="7"/>
@@ -1475,7 +1535,11 @@
       </c>
       <c r="G38" s="7"/>
       <c r="H38" s="7"/>
-      <c r="I38" s="7"/>
+      <c r="I38" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J38" s="7"/>
       <c r="K38" s="7"/>
       <c r="L38" s="7"/>
@@ -1508,7 +1572,11 @@
       </c>
       <c r="G39" s="7"/>
       <c r="H39" s="7"/>
-      <c r="I39" s="7"/>
+      <c r="I39" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J39" s="7"/>
       <c r="K39" s="7"/>
       <c r="L39" s="7"/>
@@ -1546,7 +1614,11 @@
       </c>
       <c r="G40" s="7"/>
       <c r="H40" s="7"/>
-      <c r="I40" s="7"/>
+      <c r="I40" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
       <c r="J40" s="7"/>
       <c r="K40" s="7"/>
       <c r="L40" s="7"/>
@@ -1579,7 +1651,11 @@
       </c>
       <c r="G41" s="7"/>
       <c r="H41" s="7"/>
-      <c r="I41" s="7"/>
+      <c r="I41" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J41" s="7"/>
       <c r="K41" s="7"/>
       <c r="L41" s="7"/>
@@ -1612,7 +1688,11 @@
       </c>
       <c r="G42" s="7"/>
       <c r="H42" s="7"/>
-      <c r="I42" s="7"/>
+      <c r="I42" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J42" s="7"/>
       <c r="K42" s="7"/>
       <c r="L42" s="7"/>
@@ -1645,7 +1725,11 @@
       </c>
       <c r="G43" s="7"/>
       <c r="H43" s="7"/>
-      <c r="I43" s="7"/>
+      <c r="I43" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J43" s="7"/>
       <c r="K43" s="7"/>
       <c r="L43" s="7"/>
@@ -1716,7 +1800,11 @@
       </c>
       <c r="G45" s="7"/>
       <c r="H45" s="7"/>
-      <c r="I45" s="7"/>
+      <c r="I45" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J45" s="7"/>
       <c r="K45" s="7"/>
       <c r="L45" s="7"/>
@@ -1749,7 +1837,11 @@
       </c>
       <c r="G46" s="7"/>
       <c r="H46" s="7"/>
-      <c r="I46" s="7"/>
+      <c r="I46" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J46" s="7"/>
       <c r="K46" s="7"/>
       <c r="L46" s="7"/>
@@ -1886,7 +1978,11 @@
       </c>
       <c r="G50" s="7"/>
       <c r="H50" s="7"/>
-      <c r="I50" s="7"/>
+      <c r="I50" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J50" s="7"/>
       <c r="K50" s="7"/>
       <c r="L50" s="7"/>
@@ -1919,7 +2015,11 @@
       </c>
       <c r="G51" s="7"/>
       <c r="H51" s="7"/>
-      <c r="I51" s="7"/>
+      <c r="I51" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J51" s="7"/>
       <c r="K51" s="7"/>
       <c r="L51" s="7"/>
@@ -2061,7 +2161,11 @@
       </c>
       <c r="G55" s="7"/>
       <c r="H55" s="7"/>
-      <c r="I55" s="7"/>
+      <c r="I55" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J55" s="7"/>
       <c r="K55" s="7"/>
       <c r="L55" s="7"/>
@@ -2094,7 +2198,11 @@
       </c>
       <c r="G56" s="7"/>
       <c r="H56" s="7"/>
-      <c r="I56" s="7"/>
+      <c r="I56" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J56" s="7"/>
       <c r="K56" s="7"/>
       <c r="L56" s="7"/>
@@ -2132,7 +2240,11 @@
       </c>
       <c r="G57" s="7"/>
       <c r="H57" s="7"/>
-      <c r="I57" s="7"/>
+      <c r="I57" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J57" s="7"/>
       <c r="K57" s="7"/>
       <c r="L57" s="7"/>
@@ -2170,7 +2282,11 @@
       </c>
       <c r="G58" s="7"/>
       <c r="H58" s="7"/>
-      <c r="I58" s="7"/>
+      <c r="I58" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J58" s="7"/>
       <c r="K58" s="7"/>
       <c r="L58" s="7"/>
@@ -2269,7 +2385,11 @@
       </c>
       <c r="G61" s="7"/>
       <c r="H61" s="7"/>
-      <c r="I61" s="7"/>
+      <c r="I61" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J61" s="7"/>
       <c r="K61" s="7"/>
       <c r="L61" s="7"/>
@@ -2335,7 +2455,11 @@
       </c>
       <c r="G63" s="7"/>
       <c r="H63" s="7"/>
-      <c r="I63" s="7"/>
+      <c r="I63" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
       <c r="J63" s="7"/>
       <c r="K63" s="7"/>
       <c r="L63" s="7"/>
@@ -2439,7 +2563,11 @@
       </c>
       <c r="G66" s="7"/>
       <c r="H66" s="7"/>
-      <c r="I66" s="7"/>
+      <c r="I66" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J66" s="7"/>
       <c r="K66" s="7"/>
       <c r="L66" s="7"/>
@@ -2505,7 +2633,11 @@
       </c>
       <c r="G68" s="7"/>
       <c r="H68" s="7"/>
-      <c r="I68" s="7"/>
+      <c r="I68" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J68" s="7"/>
       <c r="K68" s="7"/>
       <c r="L68" s="7"/>
@@ -2538,7 +2670,11 @@
       </c>
       <c r="G69" s="7"/>
       <c r="H69" s="7"/>
-      <c r="I69" s="7"/>
+      <c r="I69" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J69" s="7"/>
       <c r="K69" s="7"/>
       <c r="L69" s="7"/>
@@ -3261,7 +3397,11 @@
       </c>
       <c r="G90" s="7"/>
       <c r="H90" s="7"/>
-      <c r="I90" s="7"/>
+      <c r="I90" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J90" s="7"/>
       <c r="K90" s="7"/>
       <c r="L90" s="7"/>
@@ -3327,7 +3467,11 @@
       </c>
       <c r="G92" s="7"/>
       <c r="H92" s="7"/>
-      <c r="I92" s="7"/>
+      <c r="I92" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J92" s="7"/>
       <c r="K92" s="7"/>
       <c r="L92" s="7"/>
@@ -3365,7 +3509,11 @@
       </c>
       <c r="G93" s="7"/>
       <c r="H93" s="7"/>
-      <c r="I93" s="7"/>
+      <c r="I93" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J93" s="7"/>
       <c r="K93" s="7"/>
       <c r="L93" s="7"/>
@@ -3469,7 +3617,11 @@
       </c>
       <c r="G96" s="7"/>
       <c r="H96" s="7"/>
-      <c r="I96" s="7"/>
+      <c r="I96" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J96" s="7"/>
       <c r="K96" s="7"/>
       <c r="L96" s="7"/>
@@ -3875,7 +4027,11 @@
       </c>
       <c r="G108" s="7"/>
       <c r="H108" s="7"/>
-      <c r="I108" s="7"/>
+      <c r="I108" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J108" s="7"/>
       <c r="K108" s="7"/>
       <c r="L108" s="7"/>
@@ -3913,7 +4069,11 @@
       </c>
       <c r="G109" s="7"/>
       <c r="H109" s="7"/>
-      <c r="I109" s="7"/>
+      <c r="I109" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="J109" s="7"/>
       <c r="K109" s="7"/>
       <c r="L109" s="7"/>
@@ -4018,7 +4178,7 @@
     <mergeCell ref="B107:B111"/>
     <mergeCell ref="G7:L7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:I111">
+  <conditionalFormatting sqref="G9:L111">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
QA J열(445bf91) — #133 재확인 34칸 Pass 0 Fail · CID_104 신설 · CID_021 정정
· J8 = 445bf91 (video-261014c 후보) · 비고 J6. 재확인(576×1024 · 소리 0 · 튜토리얼 →
  S1 → T3 → 도전 → 스테이지로)에서 지나간 33칸 + 새 항목 = Pass 34 · Fail 0.
  T3 막이 HUD·원형 셋 위까지(CID_032) · 「- 일시 정지 -」 겹침 0(CID_014) · 해제 정상.
  도전 통과는 「도전 즉시 종료」로 — 자연 통과는 I열(1848231)에서 봤다.
· CID_104 신설(112행 · ID 이어 세기) — 「설정 열면 HUD 가 어둠막 아래」(플랜 지시 · #133).
  요약 수식 다섯 → J9:J112 · 전체 103 → 104 · 조건부 서식 G9:L112 · N7 = 445bf91.
· I29(CID_021) Fail → Pass — 사용자 ⓐ(09-18 결정 유지 · 바로가기·개발 단추 배포에도).
  내 앞 판정 근거 「촬영 빌드가 개발 빌드」는 틀렸다(b784514 에서 정정).

값 0 · 코드 0.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -296,10 +296,14 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">video-261014b · 어둠막 0.55→0.75 (T1·T3) · H(bf98a1c)=video-261014 2차 육안 Fail 0 ‖ 10-15 코드 세션 실플레이(576×1024 · 소리 0 · 새 저장 · 튜토→S1 도전 자연 통과→스테이지로→새로고침) · Pass 36 · Fail 4 · 빈 칸 = 안 지나감 · Fail: CID_014 「- 일시 정지 -」 오른끝이 마일스톤 카드에 가림 / CID_021 설정에 「보드 좌표 덤프」·「현재 적 전멸」 노출 — ⚠️ 정정(10-15): 빌드는 배포 빌드다(BuildOptions.None) · 노출 까닭은 ReviewerShortcuts.ShowTutorial =&gt; true(09-18 사용자 확정 「바로가기 배포에도」) · 「처음부터」·「튜토」도 같은 스위치 · Fail 판정 유지 여부 = 사용자 / CID_032 T3 막이 HUD(상단 칩·Stage 띠·배지·로봇B/Auto/합체 원형) 위로 안 덮임 — 전장만 어두움(잠금·「도전」 빛남·문구는 정상) / CID_055 극소 창(≈253px) 셋째 단추 잘림 = #122 보류(보통 창은 정상)</t>
-        </is>
-      </c>
-      <c r="J6" s="2"/>
+          <t xml:space="preserve">video-261014b · 어둠막 0.55→0.75 (T1·T3) · H(bf98a1c)=video-261014 2차 육안 Fail 0 ‖ 10-15 코드 세션 실플레이(576×1024 · 소리 0 · 새 저장 · 튜토→S1 도전 자연 통과→스테이지로→새로고침) · Pass 36 · Fail 4 · 빈 칸 = 안 지나감 · Fail: CID_014 「- 일시 정지 -」 오른끝이 마일스톤 카드에 가림 / CID_021 설정에 「보드 좌표 덤프」·「현재 적 전멸」 노출 — ⚠️ 정정(10-15): 빌드는 배포 빌드다(BuildOptions.None) · 노출 까닭은 ReviewerShortcuts.ShowTutorial =&gt; true(09-18 사용자 확정 「바로가기 배포에도」) · 「처음부터」·「튜토」도 같은 스위치 · Fail 판정 유지 여부 = 사용자 / CID_032 T3 막이 HUD(상단 칩·Stage 띠·배지·로봇B/Auto/합체 원형) 위로 안 덮임 — 전장만 어두움(잠금·「도전」 빛남·문구는 정상) / CID_055 극소 창(≈253px) 셋째 단추 잘림 = #122 보류(보통 창은 정상) ‖ 10-15 정정: CID_021 Fail→Pass — 사용자 ⓐ(09-18 결정 유지 · 바로가기·개발 단추 배포에도)</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">video-261014c 후보 · #133 결함 수정(T3 막·설정 어둠이 HUD 위로 · 일시 정지 겹침) ‖ 10-15 코드 세션 재확인(576×1024 · 소리 0 · 튜토→S1→T3→도전(「도전 즉시 종료」로 통과)→스테이지로) · Pass 34 · Fail 0 · 빈 칸 = 안 지나감 · CID_020/021 = ⓐ 09-18 결정대로 노출(Pass) · CID_055 = 보통 창만 봄(극소 창 #122 보류라 빈 칸) · CID_104 새 항목</t>
+        </is>
+      </c>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
     </row>
@@ -343,7 +347,7 @@
       </c>
       <c r="N7" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">1848231</t>
+          <t xml:space="preserve">445bf91</t>
         </is>
       </c>
     </row>
@@ -381,7 +385,11 @@
           <t xml:space="preserve">1848231</t>
         </is>
       </c>
-      <c r="J8" s="2"/>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">445bf91</t>
+        </is>
+      </c>
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
       <c r="M8" s="2" t="inlineStr">
@@ -390,7 +398,7 @@
         </is>
       </c>
       <c r="N8" s="7">
-        <f>COUNTIF(I9:I111,"Pass")</f>
+        <f>COUNTIF(J9:J112,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -431,7 +439,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="J9" s="7"/>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K9" s="7"/>
       <c r="L9" s="7"/>
       <c r="M9" s="2" t="inlineStr">
@@ -440,7 +452,7 @@
         </is>
       </c>
       <c r="N9" s="7">
-        <f>COUNTIF(I9:I111,"Fail")+COUNTIF(I9:I111,"Broken")</f>
+        <f>COUNTIF(J9:J112,"Fail")+COUNTIF(J9:J112,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -486,7 +498,7 @@
         </is>
       </c>
       <c r="N10" s="7">
-        <f>COUNTIF(I9:I111,"N/A")</f>
+        <f>COUNTIF(J9:J112,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -532,7 +544,7 @@
         </is>
       </c>
       <c r="N11" s="7">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="12">
@@ -578,7 +590,7 @@
         </is>
       </c>
       <c r="N12" s="7">
-        <f>TEXT((COUNTA(I9:I111))/103,"0.00%")</f>
+        <f>TEXT((COUNTA(J9:J112))/104,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -689,7 +701,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="J15" s="7"/>
+      <c r="J15" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K15" s="7"/>
       <c r="L15" s="7"/>
     </row>
@@ -726,7 +742,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="J16" s="7"/>
+      <c r="J16" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K16" s="7"/>
       <c r="L16" s="7"/>
     </row>
@@ -768,7 +788,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="J17" s="7"/>
+      <c r="J17" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K17" s="7"/>
       <c r="L17" s="7"/>
     </row>
@@ -909,7 +933,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="J21" s="7"/>
+      <c r="J21" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K21" s="7"/>
       <c r="L21" s="7"/>
     </row>
@@ -951,7 +979,11 @@
           <t xml:space="preserve">Fail</t>
         </is>
       </c>
-      <c r="J22" s="7"/>
+      <c r="J22" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K22" s="7"/>
       <c r="L22" s="7"/>
     </row>
@@ -1159,7 +1191,11 @@
       <c r="G28" s="7"/>
       <c r="H28" s="7"/>
       <c r="I28" s="7"/>
-      <c r="J28" s="7"/>
+      <c r="J28" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K28" s="7"/>
       <c r="L28" s="7"/>
     </row>
@@ -1193,7 +1229,7 @@
       <c r="H29" s="7"/>
       <c r="I29" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fail</t>
+          <t xml:space="preserve">Pass</t>
         </is>
       </c>
       <c r="J29" s="7"/>
@@ -1233,7 +1269,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="J30" s="7"/>
+      <c r="J30" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K30" s="7"/>
       <c r="L30" s="7"/>
     </row>
@@ -1275,7 +1315,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="J31" s="7"/>
+      <c r="J31" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K31" s="7"/>
       <c r="L31" s="7"/>
     </row>
@@ -1312,7 +1356,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="J32" s="7"/>
+      <c r="J32" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K32" s="7"/>
       <c r="L32" s="7"/>
     </row>
@@ -1349,7 +1397,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="J33" s="7"/>
+      <c r="J33" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K33" s="7"/>
       <c r="L33" s="7"/>
     </row>
@@ -1386,7 +1438,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="J34" s="7"/>
+      <c r="J34" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K34" s="7"/>
       <c r="L34" s="7"/>
     </row>
@@ -1428,7 +1484,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="J35" s="7"/>
+      <c r="J35" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K35" s="7"/>
       <c r="L35" s="7"/>
     </row>
@@ -1465,7 +1525,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="J36" s="7"/>
+      <c r="J36" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K36" s="7"/>
       <c r="L36" s="7"/>
     </row>
@@ -1540,7 +1604,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="J38" s="7"/>
+      <c r="J38" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K38" s="7"/>
       <c r="L38" s="7"/>
     </row>
@@ -1577,7 +1645,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="J39" s="7"/>
+      <c r="J39" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K39" s="7"/>
       <c r="L39" s="7"/>
     </row>
@@ -1619,7 +1691,11 @@
           <t xml:space="preserve">Fail</t>
         </is>
       </c>
-      <c r="J40" s="7"/>
+      <c r="J40" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K40" s="7"/>
       <c r="L40" s="7"/>
     </row>
@@ -1656,7 +1732,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="J41" s="7"/>
+      <c r="J41" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K41" s="7"/>
       <c r="L41" s="7"/>
     </row>
@@ -1693,7 +1773,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="J42" s="7"/>
+      <c r="J42" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K42" s="7"/>
       <c r="L42" s="7"/>
     </row>
@@ -1730,7 +1814,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="J43" s="7"/>
+      <c r="J43" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K43" s="7"/>
       <c r="L43" s="7"/>
     </row>
@@ -1805,7 +1893,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="J45" s="7"/>
+      <c r="J45" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K45" s="7"/>
       <c r="L45" s="7"/>
     </row>
@@ -1842,7 +1934,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="J46" s="7"/>
+      <c r="J46" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K46" s="7"/>
       <c r="L46" s="7"/>
     </row>
@@ -1983,7 +2079,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="J50" s="7"/>
+      <c r="J50" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K50" s="7"/>
       <c r="L50" s="7"/>
     </row>
@@ -2020,7 +2120,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="J51" s="7"/>
+      <c r="J51" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K51" s="7"/>
       <c r="L51" s="7"/>
     </row>
@@ -2166,7 +2270,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="J55" s="7"/>
+      <c r="J55" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K55" s="7"/>
       <c r="L55" s="7"/>
     </row>
@@ -2245,7 +2353,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="J57" s="7"/>
+      <c r="J57" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K57" s="7"/>
       <c r="L57" s="7"/>
     </row>
@@ -2287,7 +2399,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="J58" s="7"/>
+      <c r="J58" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K58" s="7"/>
       <c r="L58" s="7"/>
     </row>
@@ -2390,7 +2506,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="J61" s="7"/>
+      <c r="J61" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K61" s="7"/>
       <c r="L61" s="7"/>
     </row>
@@ -2675,7 +2795,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="J69" s="7"/>
+      <c r="J69" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K69" s="7"/>
       <c r="L69" s="7"/>
     </row>
@@ -3402,7 +3526,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="J90" s="7"/>
+      <c r="J90" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K90" s="7"/>
       <c r="L90" s="7"/>
     </row>
@@ -3472,7 +3600,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="J92" s="7"/>
+      <c r="J92" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K92" s="7"/>
       <c r="L92" s="7"/>
     </row>
@@ -3514,7 +3646,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="J93" s="7"/>
+      <c r="J93" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K93" s="7"/>
       <c r="L93" s="7"/>
     </row>
@@ -3622,7 +3758,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="J96" s="7"/>
+      <c r="J96" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="K96" s="7"/>
       <c r="L96" s="7"/>
     </row>
@@ -4148,6 +4288,48 @@
       <c r="J111" s="7"/>
       <c r="K111" s="7"/>
       <c r="L111" s="7"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_104</t>
+        </is>
+      </c>
+      <c r="B112" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">설정</t>
+        </is>
+      </c>
+      <c r="C112" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">패널</t>
+        </is>
+      </c>
+      <c r="D112" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">어둠막</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">설정을 열면 상단 칩·Stage 띠·배지·원형 셋(로봇 B·Auto·합체)이 어둠막 아래로 가는가? (판과 「- 일시 정지 -」만 밝다)</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HUD 가 설정 어둠 위에 밝게 남지 않는다 (10-15 #133)</t>
+        </is>
+      </c>
+      <c r="G112" s="7"/>
+      <c r="H112" s="7"/>
+      <c r="I112" s="7"/>
+      <c r="J112" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="K112" s="7"/>
+      <c r="L112" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="26">
@@ -4178,7 +4360,7 @@
     <mergeCell ref="B107:B111"/>
     <mergeCell ref="G7:L7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:L111">
+  <conditionalFormatting sqref="G9:L112">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
QA K열(f53ebe5) — #134 재확인 36칸 Pass 0 Fail · CID_105 신설
· K8 = f53ebe5 (video-261014c 후보) · 비고 K6. 재확인(576×1024 · 소리 0):
  ① 게임 시작 → 설정 → 「메인 메뉴로」 → 메뉴 뜸 → 「게임 시작」 → 하던 판 복귀
  ② 「처음부터」 → 튜토리얼 → S1 → T3 막이 HUD·원형 셋까지 ③ 설정 판(HUD 어둠 아래 ·
  겹침 0) ④ 도전(「도전 즉시 종료」) → 「스테이지로」 → 해제. 콘솔 오류 0.
· CID_105 신설(113행) — 「설정 → 메인 메뉴로 → 메뉴 → 게임 시작 → 하던 판 복귀」.
  요약 수식 → K9:K113 · 전체 104 → 105 · 조건부 서식 G9:L113 · N7 = f53ebe5.

⚠️ 리비전 칸 G~L 여섯 중 다섯째(K)를 썼다 — 남은 칸은 L 하나.

값 0 · 코드 0.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -304,7 +304,11 @@
           <t xml:space="preserve">video-261014c 후보 · #133 결함 수정(T3 막·설정 어둠이 HUD 위로 · 일시 정지 겹침) ‖ 10-15 코드 세션 재확인(576×1024 · 소리 0 · 튜토→S1→T3→도전(「도전 즉시 종료」로 통과)→스테이지로) · Pass 34 · Fail 0 · 빈 칸 = 안 지나감 · CID_020/021 = ⓐ 09-18 결정대로 노출(Pass) · CID_055 = 보통 창만 봄(극소 창 #122 보류라 빈 칸) · CID_104 새 항목</t>
         </is>
       </c>
-      <c r="K6" s="2"/>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">video-261014c 후보 · #134 「메인 메뉴로」 뒤 빈 화면 고침(+#133 셋) ‖ 10-15 코드 세션 재확인(576×1024 · 소리 0 · 게임 시작→설정→메인 메뉴로→메뉴→게임 시작→복귀 · 처음부터→튜토→S1→T3→설정 판→도전(즉시 종료)→스테이지로) · Pass 36 · Fail 0 · 빈 칸 = 안 지나감 · CID_105 새 항목</t>
+        </is>
+      </c>
       <c r="L6" s="2"/>
     </row>
     <row r="7">
@@ -347,7 +351,7 @@
       </c>
       <c r="N7" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">445bf91</t>
+          <t xml:space="preserve">f53ebe5</t>
         </is>
       </c>
     </row>
@@ -390,7 +394,11 @@
           <t xml:space="preserve">445bf91</t>
         </is>
       </c>
-      <c r="K8" s="2"/>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">f53ebe5</t>
+        </is>
+      </c>
       <c r="L8" s="2"/>
       <c r="M8" s="2" t="inlineStr">
         <is>
@@ -398,7 +406,7 @@
         </is>
       </c>
       <c r="N8" s="7">
-        <f>COUNTIF(J9:J112,"Pass")</f>
+        <f>COUNTIF(K9:K113,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -444,7 +452,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K9" s="7"/>
+      <c r="K9" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L9" s="7"/>
       <c r="M9" s="2" t="inlineStr">
         <is>
@@ -452,7 +464,7 @@
         </is>
       </c>
       <c r="N9" s="7">
-        <f>COUNTIF(J9:J112,"Fail")+COUNTIF(J9:J112,"Broken")</f>
+        <f>COUNTIF(K9:K113,"Fail")+COUNTIF(K9:K113,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -498,7 +510,7 @@
         </is>
       </c>
       <c r="N10" s="7">
-        <f>COUNTIF(J9:J112,"N/A")</f>
+        <f>COUNTIF(K9:K113,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -544,7 +556,7 @@
         </is>
       </c>
       <c r="N11" s="7">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="12">
@@ -590,7 +602,7 @@
         </is>
       </c>
       <c r="N12" s="7">
-        <f>TEXT((COUNTA(J9:J112))/104,"0.00%")</f>
+        <f>TEXT((COUNTA(K9:K113))/105,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -706,7 +718,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K15" s="7"/>
+      <c r="K15" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L15" s="7"/>
     </row>
     <row r="16">
@@ -747,7 +763,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K16" s="7"/>
+      <c r="K16" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L16" s="7"/>
     </row>
     <row r="17">
@@ -793,7 +813,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K17" s="7"/>
+      <c r="K17" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L17" s="7"/>
     </row>
     <row r="18">
@@ -938,7 +962,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K21" s="7"/>
+      <c r="K21" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L21" s="7"/>
     </row>
     <row r="22">
@@ -984,7 +1012,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K22" s="7"/>
+      <c r="K22" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L22" s="7"/>
     </row>
     <row r="23">
@@ -1121,7 +1153,11 @@
       <c r="H26" s="7"/>
       <c r="I26" s="7"/>
       <c r="J26" s="7"/>
-      <c r="K26" s="7"/>
+      <c r="K26" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L26" s="7"/>
     </row>
     <row r="27">
@@ -1154,7 +1190,11 @@
       <c r="H27" s="7"/>
       <c r="I27" s="7"/>
       <c r="J27" s="7"/>
-      <c r="K27" s="7"/>
+      <c r="K27" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L27" s="7"/>
     </row>
     <row r="28">
@@ -1196,7 +1236,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K28" s="7"/>
+      <c r="K28" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L28" s="7"/>
     </row>
     <row r="29">
@@ -1233,7 +1277,11 @@
         </is>
       </c>
       <c r="J29" s="7"/>
-      <c r="K29" s="7"/>
+      <c r="K29" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L29" s="7"/>
     </row>
     <row r="30">
@@ -1274,7 +1322,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K30" s="7"/>
+      <c r="K30" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L30" s="7"/>
     </row>
     <row r="31">
@@ -1320,7 +1372,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K31" s="7"/>
+      <c r="K31" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L31" s="7"/>
     </row>
     <row r="32">
@@ -1361,7 +1417,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K32" s="7"/>
+      <c r="K32" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L32" s="7"/>
     </row>
     <row r="33">
@@ -1402,7 +1462,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K33" s="7"/>
+      <c r="K33" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L33" s="7"/>
     </row>
     <row r="34">
@@ -1443,7 +1507,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K34" s="7"/>
+      <c r="K34" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L34" s="7"/>
     </row>
     <row r="35">
@@ -1489,7 +1557,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K35" s="7"/>
+      <c r="K35" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L35" s="7"/>
     </row>
     <row r="36">
@@ -1530,7 +1602,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K36" s="7"/>
+      <c r="K36" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L36" s="7"/>
     </row>
     <row r="37">
@@ -1609,7 +1685,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K38" s="7"/>
+      <c r="K38" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L38" s="7"/>
     </row>
     <row r="39">
@@ -1650,7 +1730,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K39" s="7"/>
+      <c r="K39" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L39" s="7"/>
     </row>
     <row r="40">
@@ -1696,7 +1780,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K40" s="7"/>
+      <c r="K40" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L40" s="7"/>
     </row>
     <row r="41">
@@ -1737,7 +1825,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K41" s="7"/>
+      <c r="K41" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L41" s="7"/>
     </row>
     <row r="42">
@@ -1778,7 +1870,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K42" s="7"/>
+      <c r="K42" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L42" s="7"/>
     </row>
     <row r="43">
@@ -1819,7 +1915,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K43" s="7"/>
+      <c r="K43" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L43" s="7"/>
     </row>
     <row r="44">
@@ -1898,7 +1998,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K45" s="7"/>
+      <c r="K45" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L45" s="7"/>
     </row>
     <row r="46">
@@ -1939,7 +2043,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K46" s="7"/>
+      <c r="K46" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L46" s="7"/>
     </row>
     <row r="47">
@@ -2084,7 +2192,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K50" s="7"/>
+      <c r="K50" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L50" s="7"/>
     </row>
     <row r="51">
@@ -2125,7 +2237,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K51" s="7"/>
+      <c r="K51" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L51" s="7"/>
     </row>
     <row r="52">
@@ -2275,7 +2391,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K55" s="7"/>
+      <c r="K55" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L55" s="7"/>
     </row>
     <row r="56">
@@ -2511,7 +2631,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K61" s="7"/>
+      <c r="K61" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L61" s="7"/>
     </row>
     <row r="62">
@@ -2800,7 +2924,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K69" s="7"/>
+      <c r="K69" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L69" s="7"/>
     </row>
     <row r="70">
@@ -3531,7 +3659,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K90" s="7"/>
+      <c r="K90" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L90" s="7"/>
     </row>
     <row r="91">
@@ -3605,7 +3737,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K92" s="7"/>
+      <c r="K92" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L92" s="7"/>
     </row>
     <row r="93">
@@ -3651,7 +3787,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K93" s="7"/>
+      <c r="K93" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L93" s="7"/>
     </row>
     <row r="94">
@@ -3763,7 +3903,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K96" s="7"/>
+      <c r="K96" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L96" s="7"/>
     </row>
     <row r="97">
@@ -4328,8 +4472,54 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="K112" s="7"/>
+      <c r="K112" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="L112" s="7"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_105</t>
+        </is>
+      </c>
+      <c r="B113" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">설정</t>
+        </is>
+      </c>
+      <c r="C113" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">바로가기</t>
+        </is>
+      </c>
+      <c r="D113" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">메인 메뉴로 복귀</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">설정 → 「메인 메뉴로」 → 메뉴가 뜨고 → 「게임 시작」 → 하던 판으로 돌아오는가? (단추가 하나도 없는 빈 화면이 아닌가)</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">메뉴가 뜨고 게임 시작으로 그 판에 복귀 · 저장·판 그대로 (10-15 #134 · 09-18 부터 빈 화면이던 결함)</t>
+        </is>
+      </c>
+      <c r="G113" s="7"/>
+      <c r="H113" s="7"/>
+      <c r="I113" s="7"/>
+      <c r="J113" s="7"/>
+      <c r="K113" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="L113" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="26">
@@ -4360,7 +4550,7 @@
     <mergeCell ref="B107:B111"/>
     <mergeCell ref="G7:L7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:L112">
+  <conditionalFormatting sqref="G9:L113">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
QA L열(63dafa6) — 중간 후보 재확인 Pass 34 · Fail 2 · CID_106·107 신설
· L8 = 63dafa6 · 비고 L6. 리비전 칸 G~L 여섯을 다 썼다 — 다음은 M·N(요약)을 밀어야 한다.
· Fail 둘:
  CID_055 — 586×410 에서 결과 단추 셋이 아직 한 줄 · 「음 스테이지」 잘림. #136 의 줄 담기 셈이
            단추 폭의 **합**으로 봤는데 그릴 때는 칸을 **고르게** 나눈다 — 합으로는 들어가도 가장 긴
            「다음 스테이지로」가 3분의 1 칸만 받는다. T4 빌드에서 고친다(최댓값 × 개수 + 틈).
  CID_103 — 「처음부터」 뒤 S1 통과 기록이 남는다(열린 판 2/6 · T3 안 섬). ResetSave 뒤 메모리 장부
            (IdleSignals.ClearedStageIds)를 다시 안 싣는다. 기존 결함(#135~#137 무관).
· CID_032 T3 는 위 CID_103 때문에 안 섰다 → 빈 칸.
· CID_106 신설(튜토리얼 보드가 설치 모드로 열림 · Pass) · CID_107 신설(안내 줄 괄호 메모 없음 · Pass).
  요약 → L9:L115 · 전체 107 · 서식 G9:L115 · N7 = 63dafa6.

값 0 · 코드 0.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -309,7 +309,11 @@
           <t xml:space="preserve">video-261014c 후보 · #134 「메인 메뉴로」 뒤 빈 화면 고침(+#133 셋) ‖ 10-15 코드 세션 재확인(576×1024 · 소리 0 · 게임 시작→설정→메인 메뉴로→메뉴→게임 시작→복귀 · 처음부터→튜토→S1→T3→설정 판→도전(즉시 종료)→스테이지로) · Pass 36 · Fail 0 · 빈 칸 = 안 지나감 · CID_105 새 항목</t>
         </is>
       </c>
-      <c r="L6" s="2"/>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">중간 후보 · #135 보드 설치 모드 · #136 결과 단추 줄 바꿈 · #137 안내 줄 괄호 뗌 ‖ 10-15 코드 세션 재확인(576×1024 · 소리 0 · 처음부터→튜토→S1→도전(즉시 종료)→다음 스테이지로→S2 · 결과 패널 586×410) · Pass 34 · Fail 2 · 빈 칸 = 안 지나감 · Fail: CID_055 586×410 에서 결과 단추 셋이 아직 한 줄 · 「음 스테이지」 잘림 — 줄 담기 셈이 단추 폭의 합으로 봐서(그릴 땐 고르게 나눔) · T4 빌드에서 고침 / CID_103 「처음부터」 뒤 S1 통과 기록이 남음(열린 판 2/6) — ResetSave 뒤 메모리 장부(IdleSignals.ClearedStageIds)를 다시 안 실음 · 기존 결함 · CID_032 T3 는 위 CID_103 때문에 안 섬 → 빈 칸 · CID_106·107 새 항목</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -351,7 +355,7 @@
       </c>
       <c r="N7" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">f53ebe5</t>
+          <t xml:space="preserve">63dafa6</t>
         </is>
       </c>
     </row>
@@ -399,14 +403,18 @@
           <t xml:space="preserve">f53ebe5</t>
         </is>
       </c>
-      <c r="L8" s="2"/>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">63dafa6</t>
+        </is>
+      </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">PASSrate</t>
         </is>
       </c>
       <c r="N8" s="7">
-        <f>COUNTIF(K9:K113,"Pass")</f>
+        <f>COUNTIF(L9:L115,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -457,14 +465,18 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="L9" s="7"/>
+      <c r="L9" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FAILrate</t>
         </is>
       </c>
       <c r="N9" s="7">
-        <f>COUNTIF(K9:K113,"Fail")+COUNTIF(K9:K113,"Broken")</f>
+        <f>COUNTIF(L9:L115,"Fail")+COUNTIF(L9:L115,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -510,7 +522,7 @@
         </is>
       </c>
       <c r="N10" s="7">
-        <f>COUNTIF(K9:K113,"N/A")</f>
+        <f>COUNTIF(L9:L115,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -556,7 +568,7 @@
         </is>
       </c>
       <c r="N11" s="7">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="12">
@@ -602,7 +614,7 @@
         </is>
       </c>
       <c r="N12" s="7">
-        <f>TEXT((COUNTA(K9:K113))/105,"0.00%")</f>
+        <f>TEXT((COUNTA(L9:L115))/107,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -723,7 +735,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="L15" s="7"/>
+      <c r="L15" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -768,7 +784,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="L16" s="7"/>
+      <c r="L16" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -818,7 +838,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="L17" s="7"/>
+      <c r="L17" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -967,7 +991,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="L21" s="7"/>
+      <c r="L21" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1017,7 +1045,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="L22" s="7"/>
+      <c r="L22" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -1158,7 +1190,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="L26" s="7"/>
+      <c r="L26" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -1327,7 +1363,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="L30" s="7"/>
+      <c r="L30" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -1377,7 +1417,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="L31" s="7"/>
+      <c r="L31" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -1422,7 +1466,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="L32" s="7"/>
+      <c r="L32" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -1467,7 +1515,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="L33" s="7"/>
+      <c r="L33" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -1512,7 +1564,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="L34" s="7"/>
+      <c r="L34" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -1562,7 +1618,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="L35" s="7"/>
+      <c r="L35" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -1607,7 +1667,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="L36" s="7"/>
+      <c r="L36" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -1690,7 +1754,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="L38" s="7"/>
+      <c r="L38" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -1735,7 +1803,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="L39" s="7"/>
+      <c r="L39" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -1920,7 +1992,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="L43" s="7"/>
+      <c r="L43" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -2003,7 +2079,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="L45" s="7"/>
+      <c r="L45" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -2048,7 +2128,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="L46" s="7"/>
+      <c r="L46" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -2197,7 +2281,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="L50" s="7"/>
+      <c r="L50" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -2242,7 +2330,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="L51" s="7"/>
+      <c r="L51" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -2396,7 +2488,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="L55" s="7"/>
+      <c r="L55" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -2433,7 +2529,11 @@
       </c>
       <c r="J56" s="7"/>
       <c r="K56" s="7"/>
-      <c r="L56" s="7"/>
+      <c r="L56" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -2479,7 +2579,11 @@
         </is>
       </c>
       <c r="K57" s="7"/>
-      <c r="L57" s="7"/>
+      <c r="L57" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -2525,7 +2629,11 @@
         </is>
       </c>
       <c r="K58" s="7"/>
-      <c r="L58" s="7"/>
+      <c r="L58" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -2669,7 +2777,11 @@
       <c r="I62" s="7"/>
       <c r="J62" s="7"/>
       <c r="K62" s="7"/>
-      <c r="L62" s="7"/>
+      <c r="L62" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -2706,7 +2818,11 @@
       </c>
       <c r="J63" s="7"/>
       <c r="K63" s="7"/>
-      <c r="L63" s="7"/>
+      <c r="L63" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -2929,7 +3045,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="L69" s="7"/>
+      <c r="L69" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
@@ -3664,7 +3784,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="L90" s="7"/>
+      <c r="L90" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
@@ -3742,7 +3866,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="L92" s="7"/>
+      <c r="L92" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
@@ -3792,7 +3920,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="L93" s="7"/>
+      <c r="L93" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
@@ -3908,7 +4040,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="L96" s="7"/>
+      <c r="L96" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="7" t="inlineStr">
@@ -4431,7 +4567,11 @@
       <c r="I111" s="7"/>
       <c r="J111" s="7"/>
       <c r="K111" s="7"/>
-      <c r="L111" s="7"/>
+      <c r="L111" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
@@ -4477,7 +4617,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="L112" s="7"/>
+      <c r="L112" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
@@ -4520,6 +4664,90 @@
         </is>
       </c>
       <c r="L113" s="7"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_106</t>
+        </is>
+      </c>
+      <c r="B114" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼</t>
+        </is>
+      </c>
+      <c r="C114" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">보드</t>
+        </is>
+      </c>
+      <c r="D114" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">설치 모드로 열림</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼에서 「▼ 조립」으로 보드를 열면 「이동 모드」가 아니라 「조립(설치) 모드」로 열리고, 모드를 안 바꿔도 벨트가 바로 깔리는가?</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">첫 화면은 전투 화면 · 보드가 열릴 때만 조립 모드 · 튜토리얼 밖은 이동 모드 그대로 (10-15 #135)</t>
+        </is>
+      </c>
+      <c r="G114" s="7"/>
+      <c r="H114" s="7"/>
+      <c r="I114" s="7"/>
+      <c r="J114" s="7"/>
+      <c r="K114" s="7"/>
+      <c r="L114" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_107</t>
+        </is>
+      </c>
+      <c r="B115" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">공통</t>
+        </is>
+      </c>
+      <c r="C115" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">안내 줄</t>
+        </is>
+      </c>
+      <c r="D115" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">괄호 메모 없음</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">배지 안내 줄(「파밍: …」·「목표: …」)에 설계 메모 괄호((온보딩)·(영상B) 등)가 안 나오는가?</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S1 「벨트 연결」 · S2 「모듈 배치」 · S3 「물류 재설계」 · S4 「마운트 강화」 · S6 「합체·버스트」 (10-15 #137)</t>
+        </is>
+      </c>
+      <c r="G115" s="7"/>
+      <c r="H115" s="7"/>
+      <c r="I115" s="7"/>
+      <c r="J115" s="7"/>
+      <c r="K115" s="7"/>
+      <c r="L115" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="26">
@@ -4550,7 +4778,7 @@
     <mergeCell ref="B107:B111"/>
     <mergeCell ref="G7:L7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:L113">
+  <conditionalFormatting sqref="G9:L115">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
QA M열(5de3e87) — T4 빌드 재확인 Pass 44 · Fail 1 · CID_108~113 신설
- 요약 칸 M·N → N·O 로 밈(넓히지 않고 옮김) · 범위 M9:M121 · 전체 113 · 병합 G7:M7 · 조건부 서식 G9:M121
- 세 회차(b98e463 · cebc551 · 5de3e87) 576×1024 · 소리 0 · 처음부터부터 T4 끝까지 + 결과 패널 586×410
- Fail: CID_102 오프라인 보상 판이 S1 배지 카드 밑에 깔림(기존 · 이번 묶음 밖)
- 새 항목: T4 알림 · T4 전투 막 · T4 보드 · T4 끝 · 팝오버 가장자리 글자 · 팔레트 모듈 그림

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -168,8 +168,9 @@
     <col min="10" max="10" width="12" customWidth="1"/>
     <col min="11" max="11" width="12" customWidth="1"/>
     <col min="12" max="12" width="12" customWidth="1"/>
-    <col min="13" max="13" width="11" customWidth="1"/>
+    <col min="13" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="11" customWidth="1"/>
+    <col min="15" max="15" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -312,6 +313,11 @@
       <c r="L6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">중간 후보 · #135 보드 설치 모드 · #136 결과 단추 줄 바꿈 · #137 안내 줄 괄호 뗌 ‖ 10-15 코드 세션 재확인(576×1024 · 소리 0 · 처음부터→튜토→S1→도전(즉시 종료)→다음 스테이지로→S2 · 결과 패널 586×410) · Pass 34 · Fail 2 · 빈 칸 = 안 지나감 · Fail: CID_055 586×410 에서 결과 단추 셋이 아직 한 줄 · 「음 스테이지」 잘림 — 줄 담기 셈이 단추 폭의 합으로 봐서(그릴 땐 고르게 나눔) · T4 빌드에서 고침 / CID_103 「처음부터」 뒤 S1 통과 기록이 남음(열린 판 2/6) — ResetSave 뒤 메모리 장부(IdleSignals.ClearedStageIds)를 다시 안 실음 · 기존 결함 · CID_032 T3 는 위 CID_103 때문에 안 섬 → 빈 칸 · CID_106·107 새 항목</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">video-261014c 후보(T4 빌드) · #138 T4 · #139 팝오버 · #140 팔레트 모듈 그림 · #136 결과 단추 = 「▼ 조립」 규격 · #141 처음부터 장부 + 보드 초기화 ‖ 10-15 코드 세션 재확인(576×1024 · 소리 0 · b98e463·cebc551·5de3e87 세 회차 · 처음부터→튜토→S1→T3→도전(즉시 종료)→다음 스테이지로→S2 알림→T4 막→조립→모듈 탭→대상 노드(7,8)에 M·R 각 한 번→풀림 · 결과 패널 576×1024·586×410) · 빈 칸 = 안 지나감 · Fail: CID_102 오프라인 보상 판이 S1 배지 카드 밑에 깔려 윗줄이 가려짐(기존 · 이번 묶음 밖) · 덧: 스테이지 목록 S5·S6 줄 글자가 유난히 작음(기존 · CID_058 은 Pass) · CID_108~113 새 항목</t>
         </is>
       </c>
     </row>
@@ -348,14 +354,15 @@
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M7" s="2"/>
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">버전</t>
         </is>
       </c>
-      <c r="N7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">63dafa6</t>
+      <c r="O7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5de3e87</t>
         </is>
       </c>
     </row>
@@ -410,11 +417,16 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">5de3e87</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">PASSrate</t>
         </is>
       </c>
-      <c r="N8" s="7">
-        <f>COUNTIF(L9:L115,"Pass")</f>
+      <c r="O8" s="7">
+        <f>COUNTIF(M9:M121,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -470,13 +482,18 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M9" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FAILrate</t>
         </is>
       </c>
-      <c r="N9" s="7">
-        <f>COUNTIF(L9:L115,"Fail")+COUNTIF(L9:L115,"Broken")</f>
+      <c r="O9" s="7">
+        <f>COUNTIF(M9:M121,"Fail")+COUNTIF(M9:M121,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -516,13 +533,14 @@
       <c r="J10" s="7"/>
       <c r="K10" s="7"/>
       <c r="L10" s="7"/>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M10" s="7"/>
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">N/A</t>
         </is>
       </c>
-      <c r="N10" s="7">
-        <f>COUNTIF(L9:L115,"N/A")</f>
+      <c r="O10" s="7">
+        <f>COUNTIF(M9:M121,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -562,13 +580,14 @@
       <c r="J11" s="7"/>
       <c r="K11" s="7"/>
       <c r="L11" s="7"/>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M11" s="7"/>
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">전체 개수</t>
         </is>
       </c>
-      <c r="N11" s="7">
-        <v>107</v>
+      <c r="O11" s="7">
+        <v>113</v>
       </c>
     </row>
     <row r="12">
@@ -608,13 +627,14 @@
       <c r="J12" s="7"/>
       <c r="K12" s="7"/>
       <c r="L12" s="7"/>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M12" s="7"/>
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">진행율</t>
         </is>
       </c>
-      <c r="N12" s="7">
-        <f>TEXT((COUNTA(L9:L115))/107,"0.00%")</f>
+      <c r="O12" s="7">
+        <f>TEXT((COUNTA(M9:M121))/113,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -658,6 +678,7 @@
       <c r="J13" s="7"/>
       <c r="K13" s="7"/>
       <c r="L13" s="7"/>
+      <c r="M13" s="7"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -691,6 +712,7 @@
       <c r="J14" s="7"/>
       <c r="K14" s="7"/>
       <c r="L14" s="7"/>
+      <c r="M14" s="7"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -740,6 +762,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="M15" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -789,6 +816,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="M16" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -839,6 +871,11 @@
         </is>
       </c>
       <c r="L17" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="M17" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -881,6 +918,7 @@
       <c r="J18" s="7"/>
       <c r="K18" s="7"/>
       <c r="L18" s="7"/>
+      <c r="M18" s="7"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -914,6 +952,7 @@
       <c r="J19" s="7"/>
       <c r="K19" s="7"/>
       <c r="L19" s="7"/>
+      <c r="M19" s="7"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -947,6 +986,7 @@
       <c r="J20" s="7"/>
       <c r="K20" s="7"/>
       <c r="L20" s="7"/>
+      <c r="M20" s="7"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -996,6 +1036,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="M21" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1046,6 +1091,11 @@
         </is>
       </c>
       <c r="L22" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="M22" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -1083,6 +1133,7 @@
       <c r="J23" s="7"/>
       <c r="K23" s="7"/>
       <c r="L23" s="7"/>
+      <c r="M23" s="7"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -1116,6 +1167,7 @@
       <c r="J24" s="7"/>
       <c r="K24" s="7"/>
       <c r="L24" s="7"/>
+      <c r="M24" s="7"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -1149,6 +1201,7 @@
       <c r="J25" s="7"/>
       <c r="K25" s="7"/>
       <c r="L25" s="7"/>
+      <c r="M25" s="7"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -1195,6 +1248,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="M26" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -1232,6 +1290,7 @@
         </is>
       </c>
       <c r="L27" s="7"/>
+      <c r="M27" s="7"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -1278,6 +1337,7 @@
         </is>
       </c>
       <c r="L28" s="7"/>
+      <c r="M28" s="7"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -1319,6 +1379,7 @@
         </is>
       </c>
       <c r="L29" s="7"/>
+      <c r="M29" s="7"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -1368,6 +1429,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="M30" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -1422,6 +1488,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="M31" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -1471,6 +1542,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="M32" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -1520,6 +1596,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="M33" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -1569,6 +1650,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="M34" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -1623,6 +1709,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="M35" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -1672,6 +1763,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="M36" s="7"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -1705,6 +1797,7 @@
       <c r="J37" s="7"/>
       <c r="K37" s="7"/>
       <c r="L37" s="7"/>
+      <c r="M37" s="7"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -1759,6 +1852,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="M38" s="7"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -1808,6 +1902,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="M39" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -1858,6 +1957,11 @@
         </is>
       </c>
       <c r="L40" s="7"/>
+      <c r="M40" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -1903,6 +2007,11 @@
         </is>
       </c>
       <c r="L41" s="7"/>
+      <c r="M41" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -1948,6 +2057,7 @@
         </is>
       </c>
       <c r="L42" s="7"/>
+      <c r="M42" s="7"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -1993,6 +2103,11 @@
         </is>
       </c>
       <c r="L43" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="M43" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -2035,6 +2150,7 @@
       <c r="J44" s="7"/>
       <c r="K44" s="7"/>
       <c r="L44" s="7"/>
+      <c r="M44" s="7"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -2084,6 +2200,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="M45" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -2129,6 +2250,11 @@
         </is>
       </c>
       <c r="L46" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="M46" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -2171,6 +2297,7 @@
       <c r="J47" s="7"/>
       <c r="K47" s="7"/>
       <c r="L47" s="7"/>
+      <c r="M47" s="7"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -2204,6 +2331,7 @@
       <c r="J48" s="7"/>
       <c r="K48" s="7"/>
       <c r="L48" s="7"/>
+      <c r="M48" s="7"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -2237,6 +2365,7 @@
       <c r="J49" s="7"/>
       <c r="K49" s="7"/>
       <c r="L49" s="7"/>
+      <c r="M49" s="7"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -2286,6 +2415,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="M50" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -2331,6 +2465,11 @@
         </is>
       </c>
       <c r="L51" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="M51" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -2373,6 +2512,7 @@
       <c r="J52" s="7"/>
       <c r="K52" s="7"/>
       <c r="L52" s="7"/>
+      <c r="M52" s="7"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -2411,6 +2551,7 @@
       <c r="J53" s="7"/>
       <c r="K53" s="7"/>
       <c r="L53" s="7"/>
+      <c r="M53" s="7"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -2444,6 +2585,7 @@
       <c r="J54" s="7"/>
       <c r="K54" s="7"/>
       <c r="L54" s="7"/>
+      <c r="M54" s="7"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -2493,6 +2635,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="M55" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -2534,6 +2681,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="M56" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -2584,6 +2736,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="M57" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -2630,6 +2787,11 @@
       </c>
       <c r="K58" s="7"/>
       <c r="L58" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="M58" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -2667,6 +2829,7 @@
       <c r="J59" s="7"/>
       <c r="K59" s="7"/>
       <c r="L59" s="7"/>
+      <c r="M59" s="7"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -2700,6 +2863,7 @@
       <c r="J60" s="7"/>
       <c r="K60" s="7"/>
       <c r="L60" s="7"/>
+      <c r="M60" s="7"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -2745,6 +2909,7 @@
         </is>
       </c>
       <c r="L61" s="7"/>
+      <c r="M61" s="7"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -2782,6 +2947,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="M62" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -2821,6 +2991,11 @@
       <c r="L63" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
+      <c r="M63" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
         </is>
       </c>
     </row>
@@ -2856,6 +3031,7 @@
       <c r="J64" s="7"/>
       <c r="K64" s="7"/>
       <c r="L64" s="7"/>
+      <c r="M64" s="7"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -2894,6 +3070,7 @@
       <c r="J65" s="7"/>
       <c r="K65" s="7"/>
       <c r="L65" s="7"/>
+      <c r="M65" s="7"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
@@ -2931,6 +3108,11 @@
       <c r="J66" s="7"/>
       <c r="K66" s="7"/>
       <c r="L66" s="7"/>
+      <c r="M66" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -2964,6 +3146,7 @@
       <c r="J67" s="7"/>
       <c r="K67" s="7"/>
       <c r="L67" s="7"/>
+      <c r="M67" s="7"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
@@ -3001,6 +3184,7 @@
       <c r="J68" s="7"/>
       <c r="K68" s="7"/>
       <c r="L68" s="7"/>
+      <c r="M68" s="7"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -3046,6 +3230,11 @@
         </is>
       </c>
       <c r="L69" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="M69" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -3083,6 +3272,7 @@
       <c r="J70" s="7"/>
       <c r="K70" s="7"/>
       <c r="L70" s="7"/>
+      <c r="M70" s="7"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -3121,6 +3311,7 @@
       <c r="J71" s="7"/>
       <c r="K71" s="7"/>
       <c r="L71" s="7"/>
+      <c r="M71" s="7"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
@@ -3154,6 +3345,11 @@
       <c r="J72" s="7"/>
       <c r="K72" s="7"/>
       <c r="L72" s="7"/>
+      <c r="M72" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
@@ -3192,6 +3388,7 @@
       <c r="J73" s="7"/>
       <c r="K73" s="7"/>
       <c r="L73" s="7"/>
+      <c r="M73" s="7"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -3225,6 +3422,7 @@
       <c r="J74" s="7"/>
       <c r="K74" s="7"/>
       <c r="L74" s="7"/>
+      <c r="M74" s="7"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -3258,6 +3456,7 @@
       <c r="J75" s="7"/>
       <c r="K75" s="7"/>
       <c r="L75" s="7"/>
+      <c r="M75" s="7"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -3291,6 +3490,7 @@
       <c r="J76" s="7"/>
       <c r="K76" s="7"/>
       <c r="L76" s="7"/>
+      <c r="M76" s="7"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -3324,6 +3524,7 @@
       <c r="J77" s="7"/>
       <c r="K77" s="7"/>
       <c r="L77" s="7"/>
+      <c r="M77" s="7"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
@@ -3357,6 +3558,7 @@
       <c r="J78" s="7"/>
       <c r="K78" s="7"/>
       <c r="L78" s="7"/>
+      <c r="M78" s="7"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -3395,6 +3597,7 @@
       <c r="J79" s="7"/>
       <c r="K79" s="7"/>
       <c r="L79" s="7"/>
+      <c r="M79" s="7"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
@@ -3428,6 +3631,11 @@
       <c r="J80" s="7"/>
       <c r="K80" s="7"/>
       <c r="L80" s="7"/>
+      <c r="M80" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
@@ -3461,6 +3669,7 @@
       <c r="J81" s="7"/>
       <c r="K81" s="7"/>
       <c r="L81" s="7"/>
+      <c r="M81" s="7"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
@@ -3494,6 +3703,7 @@
       <c r="J82" s="7"/>
       <c r="K82" s="7"/>
       <c r="L82" s="7"/>
+      <c r="M82" s="7"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
@@ -3532,6 +3742,7 @@
       <c r="J83" s="7"/>
       <c r="K83" s="7"/>
       <c r="L83" s="7"/>
+      <c r="M83" s="7"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
@@ -3565,6 +3776,7 @@
       <c r="J84" s="7"/>
       <c r="K84" s="7"/>
       <c r="L84" s="7"/>
+      <c r="M84" s="7"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
@@ -3598,6 +3810,7 @@
       <c r="J85" s="7"/>
       <c r="K85" s="7"/>
       <c r="L85" s="7"/>
+      <c r="M85" s="7"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
@@ -3636,6 +3849,7 @@
       <c r="J86" s="7"/>
       <c r="K86" s="7"/>
       <c r="L86" s="7"/>
+      <c r="M86" s="7"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
@@ -3669,6 +3883,7 @@
       <c r="J87" s="7"/>
       <c r="K87" s="7"/>
       <c r="L87" s="7"/>
+      <c r="M87" s="7"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
@@ -3702,6 +3917,7 @@
       <c r="J88" s="7"/>
       <c r="K88" s="7"/>
       <c r="L88" s="7"/>
+      <c r="M88" s="7"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
@@ -3735,6 +3951,7 @@
       <c r="J89" s="7"/>
       <c r="K89" s="7"/>
       <c r="L89" s="7"/>
+      <c r="M89" s="7"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
@@ -3785,6 +4002,11 @@
         </is>
       </c>
       <c r="L90" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="M90" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -3822,6 +4044,7 @@
       <c r="J91" s="7"/>
       <c r="K91" s="7"/>
       <c r="L91" s="7"/>
+      <c r="M91" s="7"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
@@ -3871,6 +4094,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="M92" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
@@ -3921,6 +4149,11 @@
         </is>
       </c>
       <c r="L93" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="M93" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -3963,6 +4196,7 @@
       <c r="J94" s="7"/>
       <c r="K94" s="7"/>
       <c r="L94" s="7"/>
+      <c r="M94" s="7"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
@@ -3996,6 +4230,7 @@
       <c r="J95" s="7"/>
       <c r="K95" s="7"/>
       <c r="L95" s="7"/>
+      <c r="M95" s="7"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
@@ -4041,6 +4276,11 @@
         </is>
       </c>
       <c r="L96" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="M96" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -4078,6 +4318,7 @@
       <c r="J97" s="7"/>
       <c r="K97" s="7"/>
       <c r="L97" s="7"/>
+      <c r="M97" s="7"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
@@ -4111,6 +4352,7 @@
       <c r="J98" s="7"/>
       <c r="K98" s="7"/>
       <c r="L98" s="7"/>
+      <c r="M98" s="7"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
@@ -4144,6 +4386,7 @@
       <c r="J99" s="7"/>
       <c r="K99" s="7"/>
       <c r="L99" s="7"/>
+      <c r="M99" s="7"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
@@ -4182,6 +4425,7 @@
       <c r="J100" s="7"/>
       <c r="K100" s="7"/>
       <c r="L100" s="7"/>
+      <c r="M100" s="7"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
@@ -4215,6 +4459,7 @@
       <c r="J101" s="7"/>
       <c r="K101" s="7"/>
       <c r="L101" s="7"/>
+      <c r="M101" s="7"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
@@ -4248,6 +4493,7 @@
       <c r="J102" s="7"/>
       <c r="K102" s="7"/>
       <c r="L102" s="7"/>
+      <c r="M102" s="7"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="inlineStr">
@@ -4281,6 +4527,7 @@
       <c r="J103" s="7"/>
       <c r="K103" s="7"/>
       <c r="L103" s="7"/>
+      <c r="M103" s="7"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="inlineStr">
@@ -4319,6 +4566,7 @@
       <c r="J104" s="7"/>
       <c r="K104" s="7"/>
       <c r="L104" s="7"/>
+      <c r="M104" s="7"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
@@ -4352,6 +4600,7 @@
       <c r="J105" s="7"/>
       <c r="K105" s="7"/>
       <c r="L105" s="7"/>
+      <c r="M105" s="7"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
@@ -4385,6 +4634,7 @@
       <c r="J106" s="7"/>
       <c r="K106" s="7"/>
       <c r="L106" s="7"/>
+      <c r="M106" s="7"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
@@ -4418,6 +4668,7 @@
       <c r="J107" s="7"/>
       <c r="K107" s="7"/>
       <c r="L107" s="7"/>
+      <c r="M107" s="7"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
@@ -4455,6 +4706,7 @@
       <c r="J108" s="7"/>
       <c r="K108" s="7"/>
       <c r="L108" s="7"/>
+      <c r="M108" s="7"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="inlineStr">
@@ -4497,6 +4749,7 @@
       <c r="J109" s="7"/>
       <c r="K109" s="7"/>
       <c r="L109" s="7"/>
+      <c r="M109" s="7"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
@@ -4535,6 +4788,11 @@
       <c r="J110" s="7"/>
       <c r="K110" s="7"/>
       <c r="L110" s="7"/>
+      <c r="M110" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
@@ -4572,6 +4830,11 @@
           <t xml:space="preserve">Fail</t>
         </is>
       </c>
+      <c r="M111" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
@@ -4622,6 +4885,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="M112" s="7"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
@@ -4664,6 +4928,7 @@
         </is>
       </c>
       <c r="L113" s="7"/>
+      <c r="M113" s="7"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="inlineStr">
@@ -4706,6 +4971,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="M114" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="7" t="inlineStr">
@@ -4744,6 +5014,269 @@
       <c r="J115" s="7"/>
       <c r="K115" s="7"/>
       <c r="L115" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="M115" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_108</t>
+        </is>
+      </c>
+      <c r="B116" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼</t>
+        </is>
+      </c>
+      <c r="C116" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T4 지급 알림</t>
+        </is>
+      </c>
+      <c r="D116" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">알림 한 번</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S1 통과 뒤 「다음 스테이지로」로 S2 파밍에 처음 들어오면 「모듈 M·R을 받았습니다」 알림이 한 번 뜨는가? (저장 복원으로 곧장 S2 면 안 뜸)</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">표시 4초(가정) · 알림이 걷힌 뒤 막 (10-15 #138)</t>
+        </is>
+      </c>
+      <c r="G116" s="7"/>
+      <c r="H116" s="7"/>
+      <c r="I116" s="7"/>
+      <c r="J116" s="7"/>
+      <c r="K116" s="7"/>
+      <c r="L116" s="7"/>
+      <c r="M116" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_109</t>
+        </is>
+      </c>
+      <c r="B117" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼</t>
+        </is>
+      </c>
+      <c r="C117" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T4 전투 막</t>
+        </is>
+      </c>
+      <c r="D117" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">조립만 열림</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">알림 뒤 「▼ 조립」만 남기고 화면이 어두워지며 「조립 버튼을 눌러 모듈을 붙여보세요」가 뜨고 「도전」·「스테이지」가 잠기는가?</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T3 와 같은 막·잠금 · 「▲ 전투로」 예외 (10-15 #138)</t>
+        </is>
+      </c>
+      <c r="G117" s="7"/>
+      <c r="H117" s="7"/>
+      <c r="I117" s="7"/>
+      <c r="J117" s="7"/>
+      <c r="K117" s="7"/>
+      <c r="L117" s="7"/>
+      <c r="M117" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_110</t>
+        </is>
+      </c>
+      <c r="B118" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼</t>
+        </is>
+      </c>
+      <c r="C118" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T4 보드</t>
+        </is>
+      </c>
+      <c r="D118" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">대상 노드·모듈 탭</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">보드가 조립 모드로 열리고 대상 노드(기초 가공소 (7,8))만 밝으며 고스트 + 「모듈 탭에서 M 또는 R을 고른 뒤 이 노드를 탭하세요」가 보이고, 팔레트는 「모듈」 탭·M/R 만 열리는가?</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">대상 노드 = 하네스 실측 가정 · 안내는 맨 윗줄이라 칸 아래에 앉는다 (10-15 #138)</t>
+        </is>
+      </c>
+      <c r="G118" s="7"/>
+      <c r="H118" s="7"/>
+      <c r="I118" s="7"/>
+      <c r="J118" s="7"/>
+      <c r="K118" s="7"/>
+      <c r="L118" s="7"/>
+      <c r="M118" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_111</t>
+        </is>
+      </c>
+      <c r="B119" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼</t>
+        </is>
+      </c>
+      <c r="C119" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T4 끝</t>
+        </is>
+      </c>
+      <c r="D119" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">붙이면 풀림</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">M 또는 R 을 고르고 대상 노드를 탭하면 붙고(노드에 모듈 그림) 막·고스트·잠금이 함께 풀리며 「도전」·「스테이지」가 열리는가?</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">「처음부터」 뒤 보드도 시작 배치로 돌아가 다시 뜬다 (10-15 #138·#141)</t>
+        </is>
+      </c>
+      <c r="G119" s="7"/>
+      <c r="H119" s="7"/>
+      <c r="I119" s="7"/>
+      <c r="J119" s="7"/>
+      <c r="K119" s="7"/>
+      <c r="L119" s="7"/>
+      <c r="M119" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_112</t>
+        </is>
+      </c>
+      <c r="B120" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">보드</t>
+        </is>
+      </c>
+      <c r="C120" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">노드 팝오버</t>
+        </is>
+      </c>
+      <c r="D120" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">가장자리 글자</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">보드 왼쪽·오른쪽·아래 가장자리 노드를 탭해도 팝오버 글자(90도 돌리기·상태·물품·전력·시간·조합표)가 잘리지 않고 화면 안에 서는가?</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">칸 = 글자에서 잼 · 넘치면 줄바꿈 (10-15 #139) · 이번엔 왼쪽 끝 노드로 봄</t>
+        </is>
+      </c>
+      <c r="G120" s="7"/>
+      <c r="H120" s="7"/>
+      <c r="I120" s="7"/>
+      <c r="J120" s="7"/>
+      <c r="K120" s="7"/>
+      <c r="L120" s="7"/>
+      <c r="M120" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_113</t>
+        </is>
+      </c>
+      <c r="B121" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">보드</t>
+        </is>
+      </c>
+      <c r="C121" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">팔레트</t>
+        </is>
+      </c>
+      <c r="D121" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">모듈 그림</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">팔레트 「모듈」 탭의 생산량·생산속도 단추에 그림이 나오는가? (노드에 붙은 모듈 그림과 같은 그림)</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">그림 없으면 글자만 (10-15 #140)</t>
+        </is>
+      </c>
+      <c r="G121" s="7"/>
+      <c r="H121" s="7"/>
+      <c r="I121" s="7"/>
+      <c r="J121" s="7"/>
+      <c r="K121" s="7"/>
+      <c r="L121" s="7"/>
+      <c r="M121" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -4776,9 +5309,9 @@
     <mergeCell ref="B92:B99"/>
     <mergeCell ref="B100:B106"/>
     <mergeCell ref="B107:B111"/>
-    <mergeCell ref="G7:L7"/>
+    <mergeCell ref="G7:M7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:L115">
+  <conditionalFormatting sqref="G9:M121">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
QA N열(589473d) — #142 재확인 Pass 45 · Fail 0 · CID_102 Pass · CID_114·115 신설
요약 칸 N·O → O·P 로 밈 · 범위 N9:N123 · 전체 115 · 병합 G7:N7 · 조건부 서식 G9:N123. 리포 8123 에서 같은 빌드로 재확인 뒤 8127 갈아엎음(19:28:52). 관찰(판정 없음): T4 보드 막 첫 진입 3/3 깔림(미재현) · ▲전투로 직후 ▼조립 첫 탭 헛돎.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -169,8 +169,9 @@
     <col min="11" max="11" width="12" customWidth="1"/>
     <col min="12" max="12" width="12" customWidth="1"/>
     <col min="13" max="13" width="12" customWidth="1"/>
-    <col min="14" max="14" width="11" customWidth="1"/>
+    <col min="14" max="14" width="12" customWidth="1"/>
     <col min="15" max="15" width="11" customWidth="1"/>
+    <col min="16" max="16" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -318,6 +319,11 @@
       <c r="M6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">video-261014c 후보(T4 빌드) · #138 T4 · #139 팝오버 · #140 팔레트 모듈 그림 · #136 결과 단추 = 「▼ 조립」 규격 · #141 처음부터 장부 + 보드 초기화 ‖ 10-15 코드 세션 재확인(576×1024 · 소리 0 · b98e463·cebc551·5de3e87 세 회차 · 처음부터→튜토→S1→T3→도전(즉시 종료)→다음 스테이지로→S2 알림→T4 막→조립→모듈 탭→대상 노드(7,8)에 M·R 각 한 번→풀림 · 결과 패널 576×1024·586×410) · 빈 칸 = 안 지나감 · Fail: CID_102 오프라인 보상 판이 S1 배지 카드 밑에 깔려 윗줄이 가려짐(기존 · 이번 묶음 밖) · 덧: 스테이지 목록 S5·S6 줄 글자가 유난히 작음(기존 · CID_058 은 Pass) · CID_108~113 새 항목</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">video-261014c 후보 · #142 a HUD 「도전」·「스테이지」 글자 = 「▼ 조립」 규격 · b 오프라인 보상 판을 HUD 맨 위로 · c 스테이지 목록 긴 잠김 줄 두 줄 ‖ 10-15 코드 세션 재확인(리포 8123 에서 같은 빌드 · 576×1024 · 소리 0 · 새로고침→보상 판→처음부터→튜토→S1 T3→도전(즉시 종료)→다음 스테이지로→S2 알림→T4→M 붙여 풀림 · 목록) · 8127 갈아엎음 19:28:52 · 빈 칸 = 안 지나감(CID_112 팝오버·결과 패널 586×410 은 코드 그대로라 앞 칸 M 판정) · 관찰(판정 없음): f T4 보드 막 첫 진입 3/3 깔림 — 미재현 · 보드 막이 T3 막보다 옅게 보임 · ▲전투로 직후 ▼조립 첫 탭이 매번 한 번 헛돎(브라우저 자동화 초점일 수 있음) · CID_114·115 새 항목</t>
         </is>
       </c>
     </row>
@@ -355,14 +361,15 @@
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N7" s="2"/>
+      <c r="O7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">버전</t>
         </is>
       </c>
-      <c r="O7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5de3e87</t>
+      <c r="P7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">589473d</t>
         </is>
       </c>
     </row>
@@ -422,11 +429,16 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">589473d</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">PASSrate</t>
         </is>
       </c>
-      <c r="O8" s="7">
-        <f>COUNTIF(M9:M121,"Pass")</f>
+      <c r="P8" s="7">
+        <f>COUNTIF(N9:N123,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -487,13 +499,18 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N9" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FAILrate</t>
         </is>
       </c>
-      <c r="O9" s="7">
-        <f>COUNTIF(M9:M121,"Fail")+COUNTIF(M9:M121,"Broken")</f>
+      <c r="P9" s="7">
+        <f>COUNTIF(N9:N123,"Fail")+COUNTIF(N9:N123,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -534,13 +551,14 @@
       <c r="K10" s="7"/>
       <c r="L10" s="7"/>
       <c r="M10" s="7"/>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N10" s="7"/>
+      <c r="O10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">N/A</t>
         </is>
       </c>
-      <c r="O10" s="7">
-        <f>COUNTIF(M9:M121,"N/A")</f>
+      <c r="P10" s="7">
+        <f>COUNTIF(N9:N123,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -581,13 +599,14 @@
       <c r="K11" s="7"/>
       <c r="L11" s="7"/>
       <c r="M11" s="7"/>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N11" s="7"/>
+      <c r="O11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">전체 개수</t>
         </is>
       </c>
-      <c r="O11" s="7">
-        <v>113</v>
+      <c r="P11" s="7">
+        <v>115</v>
       </c>
     </row>
     <row r="12">
@@ -628,13 +647,14 @@
       <c r="K12" s="7"/>
       <c r="L12" s="7"/>
       <c r="M12" s="7"/>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N12" s="7"/>
+      <c r="O12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">진행율</t>
         </is>
       </c>
-      <c r="O12" s="7">
-        <f>TEXT((COUNTA(M9:M121))/113,"0.00%")</f>
+      <c r="P12" s="7">
+        <f>TEXT((COUNTA(N9:N123))/115,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -679,6 +699,7 @@
       <c r="K13" s="7"/>
       <c r="L13" s="7"/>
       <c r="M13" s="7"/>
+      <c r="N13" s="7"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -713,6 +734,7 @@
       <c r="K14" s="7"/>
       <c r="L14" s="7"/>
       <c r="M14" s="7"/>
+      <c r="N14" s="7"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -767,6 +789,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="N15" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -821,6 +848,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="N16" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -876,6 +908,11 @@
         </is>
       </c>
       <c r="M17" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="N17" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -919,6 +956,7 @@
       <c r="K18" s="7"/>
       <c r="L18" s="7"/>
       <c r="M18" s="7"/>
+      <c r="N18" s="7"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -953,6 +991,7 @@
       <c r="K19" s="7"/>
       <c r="L19" s="7"/>
       <c r="M19" s="7"/>
+      <c r="N19" s="7"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -987,6 +1026,7 @@
       <c r="K20" s="7"/>
       <c r="L20" s="7"/>
       <c r="M20" s="7"/>
+      <c r="N20" s="7"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1041,6 +1081,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="N21" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1096,6 +1141,11 @@
         </is>
       </c>
       <c r="M22" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="N22" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -1134,6 +1184,7 @@
       <c r="K23" s="7"/>
       <c r="L23" s="7"/>
       <c r="M23" s="7"/>
+      <c r="N23" s="7"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -1168,6 +1219,7 @@
       <c r="K24" s="7"/>
       <c r="L24" s="7"/>
       <c r="M24" s="7"/>
+      <c r="N24" s="7"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -1202,6 +1254,7 @@
       <c r="K25" s="7"/>
       <c r="L25" s="7"/>
       <c r="M25" s="7"/>
+      <c r="N25" s="7"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -1253,6 +1306,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="N26" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -1291,6 +1349,7 @@
       </c>
       <c r="L27" s="7"/>
       <c r="M27" s="7"/>
+      <c r="N27" s="7"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -1338,6 +1397,7 @@
       </c>
       <c r="L28" s="7"/>
       <c r="M28" s="7"/>
+      <c r="N28" s="7"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -1380,6 +1440,7 @@
       </c>
       <c r="L29" s="7"/>
       <c r="M29" s="7"/>
+      <c r="N29" s="7"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -1434,6 +1495,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="N30" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -1493,6 +1559,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="N31" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -1547,6 +1618,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="N32" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -1601,6 +1677,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="N33" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -1655,6 +1736,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="N34" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -1714,6 +1800,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="N35" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -1764,6 +1855,7 @@
         </is>
       </c>
       <c r="M36" s="7"/>
+      <c r="N36" s="7"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -1798,6 +1890,7 @@
       <c r="K37" s="7"/>
       <c r="L37" s="7"/>
       <c r="M37" s="7"/>
+      <c r="N37" s="7"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -1853,6 +1946,7 @@
         </is>
       </c>
       <c r="M38" s="7"/>
+      <c r="N38" s="7"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -1907,6 +2001,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="N39" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -1962,6 +2061,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="N40" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -2012,6 +2116,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="N41" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -2058,6 +2167,7 @@
       </c>
       <c r="L42" s="7"/>
       <c r="M42" s="7"/>
+      <c r="N42" s="7"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -2108,6 +2218,11 @@
         </is>
       </c>
       <c r="M43" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="N43" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -2151,6 +2266,7 @@
       <c r="K44" s="7"/>
       <c r="L44" s="7"/>
       <c r="M44" s="7"/>
+      <c r="N44" s="7"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -2205,6 +2321,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="N45" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -2255,6 +2376,11 @@
         </is>
       </c>
       <c r="M46" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="N46" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -2298,6 +2424,7 @@
       <c r="K47" s="7"/>
       <c r="L47" s="7"/>
       <c r="M47" s="7"/>
+      <c r="N47" s="7"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -2332,6 +2459,7 @@
       <c r="K48" s="7"/>
       <c r="L48" s="7"/>
       <c r="M48" s="7"/>
+      <c r="N48" s="7"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -2366,6 +2494,7 @@
       <c r="K49" s="7"/>
       <c r="L49" s="7"/>
       <c r="M49" s="7"/>
+      <c r="N49" s="7"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -2420,6 +2549,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="N50" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -2470,6 +2604,11 @@
         </is>
       </c>
       <c r="M51" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="N51" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -2513,6 +2652,7 @@
       <c r="K52" s="7"/>
       <c r="L52" s="7"/>
       <c r="M52" s="7"/>
+      <c r="N52" s="7"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -2552,6 +2692,7 @@
       <c r="K53" s="7"/>
       <c r="L53" s="7"/>
       <c r="M53" s="7"/>
+      <c r="N53" s="7"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -2586,6 +2727,7 @@
       <c r="K54" s="7"/>
       <c r="L54" s="7"/>
       <c r="M54" s="7"/>
+      <c r="N54" s="7"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -2640,6 +2782,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="N55" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -2686,6 +2833,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="N56" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -2741,6 +2893,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="N57" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -2792,6 +2949,11 @@
         </is>
       </c>
       <c r="M58" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="N58" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -2830,6 +2992,7 @@
       <c r="K59" s="7"/>
       <c r="L59" s="7"/>
       <c r="M59" s="7"/>
+      <c r="N59" s="7"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -2864,6 +3027,7 @@
       <c r="K60" s="7"/>
       <c r="L60" s="7"/>
       <c r="M60" s="7"/>
+      <c r="N60" s="7"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -2910,6 +3074,7 @@
       </c>
       <c r="L61" s="7"/>
       <c r="M61" s="7"/>
+      <c r="N61" s="7"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -2952,6 +3117,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="N62" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -2998,6 +3168,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="N63" s="7"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -3032,6 +3203,7 @@
       <c r="K64" s="7"/>
       <c r="L64" s="7"/>
       <c r="M64" s="7"/>
+      <c r="N64" s="7"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -3071,6 +3243,7 @@
       <c r="K65" s="7"/>
       <c r="L65" s="7"/>
       <c r="M65" s="7"/>
+      <c r="N65" s="7"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
@@ -3109,6 +3282,11 @@
       <c r="K66" s="7"/>
       <c r="L66" s="7"/>
       <c r="M66" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="N66" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -3147,6 +3325,7 @@
       <c r="K67" s="7"/>
       <c r="L67" s="7"/>
       <c r="M67" s="7"/>
+      <c r="N67" s="7"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
@@ -3185,6 +3364,7 @@
       <c r="K68" s="7"/>
       <c r="L68" s="7"/>
       <c r="M68" s="7"/>
+      <c r="N68" s="7"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -3235,6 +3415,11 @@
         </is>
       </c>
       <c r="M69" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="N69" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -3273,6 +3458,7 @@
       <c r="K70" s="7"/>
       <c r="L70" s="7"/>
       <c r="M70" s="7"/>
+      <c r="N70" s="7"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -3312,6 +3498,7 @@
       <c r="K71" s="7"/>
       <c r="L71" s="7"/>
       <c r="M71" s="7"/>
+      <c r="N71" s="7"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
@@ -3350,6 +3537,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="N72" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
@@ -3389,6 +3581,7 @@
       <c r="K73" s="7"/>
       <c r="L73" s="7"/>
       <c r="M73" s="7"/>
+      <c r="N73" s="7"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -3423,6 +3616,7 @@
       <c r="K74" s="7"/>
       <c r="L74" s="7"/>
       <c r="M74" s="7"/>
+      <c r="N74" s="7"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -3457,6 +3651,7 @@
       <c r="K75" s="7"/>
       <c r="L75" s="7"/>
       <c r="M75" s="7"/>
+      <c r="N75" s="7"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -3491,6 +3686,7 @@
       <c r="K76" s="7"/>
       <c r="L76" s="7"/>
       <c r="M76" s="7"/>
+      <c r="N76" s="7"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -3525,6 +3721,7 @@
       <c r="K77" s="7"/>
       <c r="L77" s="7"/>
       <c r="M77" s="7"/>
+      <c r="N77" s="7"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
@@ -3559,6 +3756,7 @@
       <c r="K78" s="7"/>
       <c r="L78" s="7"/>
       <c r="M78" s="7"/>
+      <c r="N78" s="7"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -3598,6 +3796,7 @@
       <c r="K79" s="7"/>
       <c r="L79" s="7"/>
       <c r="M79" s="7"/>
+      <c r="N79" s="7"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
@@ -3636,6 +3835,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="N80" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
@@ -3670,6 +3874,7 @@
       <c r="K81" s="7"/>
       <c r="L81" s="7"/>
       <c r="M81" s="7"/>
+      <c r="N81" s="7"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
@@ -3704,6 +3909,7 @@
       <c r="K82" s="7"/>
       <c r="L82" s="7"/>
       <c r="M82" s="7"/>
+      <c r="N82" s="7"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
@@ -3743,6 +3949,7 @@
       <c r="K83" s="7"/>
       <c r="L83" s="7"/>
       <c r="M83" s="7"/>
+      <c r="N83" s="7"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
@@ -3777,6 +3984,7 @@
       <c r="K84" s="7"/>
       <c r="L84" s="7"/>
       <c r="M84" s="7"/>
+      <c r="N84" s="7"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
@@ -3811,6 +4019,7 @@
       <c r="K85" s="7"/>
       <c r="L85" s="7"/>
       <c r="M85" s="7"/>
+      <c r="N85" s="7"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
@@ -3850,6 +4059,7 @@
       <c r="K86" s="7"/>
       <c r="L86" s="7"/>
       <c r="M86" s="7"/>
+      <c r="N86" s="7"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
@@ -3884,6 +4094,7 @@
       <c r="K87" s="7"/>
       <c r="L87" s="7"/>
       <c r="M87" s="7"/>
+      <c r="N87" s="7"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
@@ -3918,6 +4129,7 @@
       <c r="K88" s="7"/>
       <c r="L88" s="7"/>
       <c r="M88" s="7"/>
+      <c r="N88" s="7"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
@@ -3952,6 +4164,7 @@
       <c r="K89" s="7"/>
       <c r="L89" s="7"/>
       <c r="M89" s="7"/>
+      <c r="N89" s="7"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
@@ -4007,6 +4220,11 @@
         </is>
       </c>
       <c r="M90" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="N90" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -4045,6 +4263,7 @@
       <c r="K91" s="7"/>
       <c r="L91" s="7"/>
       <c r="M91" s="7"/>
+      <c r="N91" s="7"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
@@ -4099,6 +4318,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="N92" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
@@ -4154,6 +4378,11 @@
         </is>
       </c>
       <c r="M93" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="N93" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -4197,6 +4426,7 @@
       <c r="K94" s="7"/>
       <c r="L94" s="7"/>
       <c r="M94" s="7"/>
+      <c r="N94" s="7"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
@@ -4231,6 +4461,7 @@
       <c r="K95" s="7"/>
       <c r="L95" s="7"/>
       <c r="M95" s="7"/>
+      <c r="N95" s="7"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
@@ -4281,6 +4512,11 @@
         </is>
       </c>
       <c r="M96" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="N96" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -4319,6 +4555,7 @@
       <c r="K97" s="7"/>
       <c r="L97" s="7"/>
       <c r="M97" s="7"/>
+      <c r="N97" s="7"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
@@ -4353,6 +4590,7 @@
       <c r="K98" s="7"/>
       <c r="L98" s="7"/>
       <c r="M98" s="7"/>
+      <c r="N98" s="7"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
@@ -4387,6 +4625,7 @@
       <c r="K99" s="7"/>
       <c r="L99" s="7"/>
       <c r="M99" s="7"/>
+      <c r="N99" s="7"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
@@ -4426,6 +4665,7 @@
       <c r="K100" s="7"/>
       <c r="L100" s="7"/>
       <c r="M100" s="7"/>
+      <c r="N100" s="7"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
@@ -4460,6 +4700,7 @@
       <c r="K101" s="7"/>
       <c r="L101" s="7"/>
       <c r="M101" s="7"/>
+      <c r="N101" s="7"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
@@ -4494,6 +4735,7 @@
       <c r="K102" s="7"/>
       <c r="L102" s="7"/>
       <c r="M102" s="7"/>
+      <c r="N102" s="7"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="inlineStr">
@@ -4528,6 +4770,7 @@
       <c r="K103" s="7"/>
       <c r="L103" s="7"/>
       <c r="M103" s="7"/>
+      <c r="N103" s="7"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="inlineStr">
@@ -4567,6 +4810,7 @@
       <c r="K104" s="7"/>
       <c r="L104" s="7"/>
       <c r="M104" s="7"/>
+      <c r="N104" s="7"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
@@ -4601,6 +4845,7 @@
       <c r="K105" s="7"/>
       <c r="L105" s="7"/>
       <c r="M105" s="7"/>
+      <c r="N105" s="7"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
@@ -4635,6 +4880,7 @@
       <c r="K106" s="7"/>
       <c r="L106" s="7"/>
       <c r="M106" s="7"/>
+      <c r="N106" s="7"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
@@ -4669,6 +4915,7 @@
       <c r="K107" s="7"/>
       <c r="L107" s="7"/>
       <c r="M107" s="7"/>
+      <c r="N107" s="7"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
@@ -4707,6 +4954,7 @@
       <c r="K108" s="7"/>
       <c r="L108" s="7"/>
       <c r="M108" s="7"/>
+      <c r="N108" s="7"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="inlineStr">
@@ -4750,6 +4998,7 @@
       <c r="K109" s="7"/>
       <c r="L109" s="7"/>
       <c r="M109" s="7"/>
+      <c r="N109" s="7"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
@@ -4793,6 +5042,11 @@
           <t xml:space="preserve">Fail</t>
         </is>
       </c>
+      <c r="N110" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
@@ -4835,6 +5089,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="N111" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
@@ -4886,6 +5145,7 @@
         </is>
       </c>
       <c r="M112" s="7"/>
+      <c r="N112" s="7"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
@@ -4929,6 +5189,7 @@
       </c>
       <c r="L113" s="7"/>
       <c r="M113" s="7"/>
+      <c r="N113" s="7"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="inlineStr">
@@ -4976,6 +5237,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="N114" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="7" t="inlineStr">
@@ -5019,6 +5285,11 @@
         </is>
       </c>
       <c r="M115" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="N115" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -5066,6 +5337,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="N116" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
@@ -5109,6 +5385,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="N117" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
@@ -5152,6 +5433,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="N118" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="7" t="inlineStr">
@@ -5195,6 +5481,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="N119" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="7" t="inlineStr">
@@ -5238,6 +5529,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="N120" s="7"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="inlineStr">
@@ -5277,6 +5569,99 @@
       <c r="K121" s="7"/>
       <c r="L121" s="7"/>
       <c r="M121" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="N121" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_114</t>
+        </is>
+      </c>
+      <c r="B122" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">상단</t>
+        </is>
+      </c>
+      <c r="C122" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HUD 단추</t>
+        </is>
+      </c>
+      <c r="D122" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">글자 크기</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">파밍 화면 「도전」·「스테이지」 글자가 「▼ 조립」 단추와 같은 크기이고, 두 칸이 같은 크기로 글자를 다 담는가? (T3 막 구멍도 그 칸에 맞는가)</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">칸이 글자를 따라감 (10-15 #142 a)</t>
+        </is>
+      </c>
+      <c r="G122" s="7"/>
+      <c r="H122" s="7"/>
+      <c r="I122" s="7"/>
+      <c r="J122" s="7"/>
+      <c r="K122" s="7"/>
+      <c r="L122" s="7"/>
+      <c r="M122" s="7"/>
+      <c r="N122" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_115</t>
+        </is>
+      </c>
+      <c r="B123" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">스테이지 목록</t>
+        </is>
+      </c>
+      <c r="C123" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">출력</t>
+        </is>
+      </c>
+      <c r="D123" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">줄 글자 같음</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">스테이지 목록 여섯 줄 글자가 모두 같은 크기인가? (긴 잠김 줄은 「잠김 · S5 — 이름」/「(앞 판 도전 통과 필요)」 두 줄)</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">문구 불변 · 줄 높이는 글자에서 (10-15 #142 c)</t>
+        </is>
+      </c>
+      <c r="G123" s="7"/>
+      <c r="H123" s="7"/>
+      <c r="I123" s="7"/>
+      <c r="J123" s="7"/>
+      <c r="K123" s="7"/>
+      <c r="L123" s="7"/>
+      <c r="M123" s="7"/>
+      <c r="N123" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -5309,9 +5694,9 @@
     <mergeCell ref="B92:B99"/>
     <mergeCell ref="B100:B106"/>
     <mergeCell ref="B107:B111"/>
-    <mergeCell ref="G7:M7"/>
+    <mergeCell ref="G7:N7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:M121">
+  <conditionalFormatting sqref="G9:N123">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
QA O열(4dbd244) — #143·#144 재확인 Pass 28 · Fail 0 · CID_116·117 신설 · CID_086·087 폐기 표기
요약 O·P → P·Q 로 밈 · 범위 O9:O125 · 전체 117 · 병합 G7:O7 · 조건부 서식 G9:O125. 리포 8123 에서 같은 빌드로 재확인 뒤 8127 갈아엎음(19:49:09).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -170,8 +170,9 @@
     <col min="12" max="12" width="12" customWidth="1"/>
     <col min="13" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="12" customWidth="1"/>
-    <col min="15" max="15" width="11" customWidth="1"/>
+    <col min="15" max="15" width="12" customWidth="1"/>
     <col min="16" max="16" width="11" customWidth="1"/>
+    <col min="17" max="17" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -324,6 +325,11 @@
       <c r="N6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">video-261014c 후보 · #142 a HUD 「도전」·「스테이지」 글자 = 「▼ 조립」 규격 · b 오프라인 보상 판을 HUD 맨 위로 · c 스테이지 목록 긴 잠김 줄 두 줄 ‖ 10-15 코드 세션 재확인(리포 8123 에서 같은 빌드 · 576×1024 · 소리 0 · 새로고침→보상 판→처음부터→튜토→S1 T3→도전(즉시 종료)→다음 스테이지로→S2 알림→T4→M 붙여 풀림 · 목록) · 8127 갈아엎음 19:28:52 · 빈 칸 = 안 지나감(CID_112 팝오버·결과 패널 586×410 은 코드 그대로라 앞 칸 M 판정) · 관찰(판정 없음): f T4 보드 막 첫 진입 3/3 깔림 — 미재현 · 보드 막이 T3 막보다 옅게 보임 · ▲전투로 직후 ▼조립 첫 탭이 매번 한 번 헛돎(브라우저 자동화 초점일 수 있음) · CID_114·115 새 항목</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">video-261014c 후보 · #143 도전 중 보드 모드 단추 「도전 중 변경 불가」 흐림 · #144 태그 원형 셋(로봇 B·Auto·합체)은 로봇 B 해금 뒤에만 ‖ 10-15 코드 세션 재확인(리포 8123 같은 빌드 · 576×1024 · 소리 0 · S1 파밍 원형 없음 → 도전 → 조립: 모드 판 흐림·눌러도 그대로 → S5 점프: 태그·Auto·합체 보임 → 처음부터 → 튜토 판 모드 단추 그대로 → 튜토·S1 원형 없음 → T3 막 구멍 그대로) · 8127 갈아엎음 19:49:09 · 빈 칸 = 안 지나감 · CID_086·087 은 비고에 폐기 표기(#144 · CID_117 로 갈음) · CID_116·117 새 항목</t>
         </is>
       </c>
     </row>
@@ -362,14 +368,15 @@
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
       <c r="N7" s="2"/>
-      <c r="O7" s="2" t="inlineStr">
+      <c r="O7" s="2"/>
+      <c r="P7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">버전</t>
         </is>
       </c>
-      <c r="P7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">589473d</t>
+      <c r="Q7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4dbd244</t>
         </is>
       </c>
     </row>
@@ -434,11 +441,16 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">4dbd244</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">PASSrate</t>
         </is>
       </c>
-      <c r="P8" s="7">
-        <f>COUNTIF(N9:N123,"Pass")</f>
+      <c r="Q8" s="7">
+        <f>COUNTIF(O9:O125,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -504,13 +516,18 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="O9" s="2" t="inlineStr">
+      <c r="O9" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FAILrate</t>
         </is>
       </c>
-      <c r="P9" s="7">
-        <f>COUNTIF(N9:N123,"Fail")+COUNTIF(N9:N123,"Broken")</f>
+      <c r="Q9" s="7">
+        <f>COUNTIF(O9:O125,"Fail")+COUNTIF(O9:O125,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -552,13 +569,14 @@
       <c r="L10" s="7"/>
       <c r="M10" s="7"/>
       <c r="N10" s="7"/>
-      <c r="O10" s="2" t="inlineStr">
+      <c r="O10" s="7"/>
+      <c r="P10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">N/A</t>
         </is>
       </c>
-      <c r="P10" s="7">
-        <f>COUNTIF(N9:N123,"N/A")</f>
+      <c r="Q10" s="7">
+        <f>COUNTIF(O9:O125,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -600,13 +618,14 @@
       <c r="L11" s="7"/>
       <c r="M11" s="7"/>
       <c r="N11" s="7"/>
-      <c r="O11" s="2" t="inlineStr">
+      <c r="O11" s="7"/>
+      <c r="P11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">전체 개수</t>
         </is>
       </c>
-      <c r="P11" s="7">
-        <v>115</v>
+      <c r="Q11" s="7">
+        <v>117</v>
       </c>
     </row>
     <row r="12">
@@ -648,13 +667,14 @@
       <c r="L12" s="7"/>
       <c r="M12" s="7"/>
       <c r="N12" s="7"/>
-      <c r="O12" s="2" t="inlineStr">
+      <c r="O12" s="7"/>
+      <c r="P12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">진행율</t>
         </is>
       </c>
-      <c r="P12" s="7">
-        <f>TEXT((COUNTA(N9:N123))/115,"0.00%")</f>
+      <c r="Q12" s="7">
+        <f>TEXT((COUNTA(O9:O125))/117,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -700,6 +720,7 @@
       <c r="L13" s="7"/>
       <c r="M13" s="7"/>
       <c r="N13" s="7"/>
+      <c r="O13" s="7"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -735,6 +756,7 @@
       <c r="L14" s="7"/>
       <c r="M14" s="7"/>
       <c r="N14" s="7"/>
+      <c r="O14" s="7"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -794,6 +816,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O15" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -853,6 +880,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O16" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -913,6 +945,11 @@
         </is>
       </c>
       <c r="N17" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="O17" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -957,6 +994,7 @@
       <c r="L18" s="7"/>
       <c r="M18" s="7"/>
       <c r="N18" s="7"/>
+      <c r="O18" s="7"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -992,6 +1030,7 @@
       <c r="L19" s="7"/>
       <c r="M19" s="7"/>
       <c r="N19" s="7"/>
+      <c r="O19" s="7"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1027,6 +1066,7 @@
       <c r="L20" s="7"/>
       <c r="M20" s="7"/>
       <c r="N20" s="7"/>
+      <c r="O20" s="7"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1086,6 +1126,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O21" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1150,6 +1195,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O22" s="7"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -1185,6 +1231,11 @@
       <c r="L23" s="7"/>
       <c r="M23" s="7"/>
       <c r="N23" s="7"/>
+      <c r="O23" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -1220,6 +1271,7 @@
       <c r="L24" s="7"/>
       <c r="M24" s="7"/>
       <c r="N24" s="7"/>
+      <c r="O24" s="7"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -1255,6 +1307,7 @@
       <c r="L25" s="7"/>
       <c r="M25" s="7"/>
       <c r="N25" s="7"/>
+      <c r="O25" s="7"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -1311,6 +1364,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O26" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -1350,6 +1408,7 @@
       <c r="L27" s="7"/>
       <c r="M27" s="7"/>
       <c r="N27" s="7"/>
+      <c r="O27" s="7"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -1398,6 +1457,7 @@
       <c r="L28" s="7"/>
       <c r="M28" s="7"/>
       <c r="N28" s="7"/>
+      <c r="O28" s="7"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -1441,6 +1501,7 @@
       <c r="L29" s="7"/>
       <c r="M29" s="7"/>
       <c r="N29" s="7"/>
+      <c r="O29" s="7"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -1500,6 +1561,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O30" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -1564,6 +1630,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O31" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -1623,6 +1694,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O32" s="7"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -1682,6 +1754,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O33" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -1741,6 +1818,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O34" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -1805,6 +1887,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O35" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -1856,6 +1943,7 @@
       </c>
       <c r="M36" s="7"/>
       <c r="N36" s="7"/>
+      <c r="O36" s="7"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -1891,6 +1979,7 @@
       <c r="L37" s="7"/>
       <c r="M37" s="7"/>
       <c r="N37" s="7"/>
+      <c r="O37" s="7"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -1947,6 +2036,7 @@
       </c>
       <c r="M38" s="7"/>
       <c r="N38" s="7"/>
+      <c r="O38" s="7"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -2006,6 +2096,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O39" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -2066,6 +2161,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O40" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -2121,6 +2221,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O41" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -2168,6 +2273,7 @@
       <c r="L42" s="7"/>
       <c r="M42" s="7"/>
       <c r="N42" s="7"/>
+      <c r="O42" s="7"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -2223,6 +2329,11 @@
         </is>
       </c>
       <c r="N43" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="O43" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -2267,6 +2378,7 @@
       <c r="L44" s="7"/>
       <c r="M44" s="7"/>
       <c r="N44" s="7"/>
+      <c r="O44" s="7"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -2326,6 +2438,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O45" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -2381,6 +2498,11 @@
         </is>
       </c>
       <c r="N46" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="O46" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -2425,6 +2547,7 @@
       <c r="L47" s="7"/>
       <c r="M47" s="7"/>
       <c r="N47" s="7"/>
+      <c r="O47" s="7"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -2460,6 +2583,7 @@
       <c r="L48" s="7"/>
       <c r="M48" s="7"/>
       <c r="N48" s="7"/>
+      <c r="O48" s="7"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -2495,6 +2619,7 @@
       <c r="L49" s="7"/>
       <c r="M49" s="7"/>
       <c r="N49" s="7"/>
+      <c r="O49" s="7"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -2554,6 +2679,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O50" s="7"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -2613,6 +2739,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O51" s="7"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -2653,6 +2780,7 @@
       <c r="L52" s="7"/>
       <c r="M52" s="7"/>
       <c r="N52" s="7"/>
+      <c r="O52" s="7"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -2693,6 +2821,7 @@
       <c r="L53" s="7"/>
       <c r="M53" s="7"/>
       <c r="N53" s="7"/>
+      <c r="O53" s="7"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -2728,6 +2857,7 @@
       <c r="L54" s="7"/>
       <c r="M54" s="7"/>
       <c r="N54" s="7"/>
+      <c r="O54" s="7"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -2787,6 +2917,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O55" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -2838,6 +2973,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O56" s="7"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -2898,6 +3034,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O57" s="7"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -2958,6 +3095,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O58" s="7"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -2993,6 +3131,7 @@
       <c r="L59" s="7"/>
       <c r="M59" s="7"/>
       <c r="N59" s="7"/>
+      <c r="O59" s="7"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -3028,6 +3167,7 @@
       <c r="L60" s="7"/>
       <c r="M60" s="7"/>
       <c r="N60" s="7"/>
+      <c r="O60" s="7"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -3075,6 +3215,7 @@
       <c r="L61" s="7"/>
       <c r="M61" s="7"/>
       <c r="N61" s="7"/>
+      <c r="O61" s="7"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -3122,6 +3263,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O62" s="7"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -3169,6 +3311,7 @@
         </is>
       </c>
       <c r="N63" s="7"/>
+      <c r="O63" s="7"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -3204,6 +3347,7 @@
       <c r="L64" s="7"/>
       <c r="M64" s="7"/>
       <c r="N64" s="7"/>
+      <c r="O64" s="7"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -3244,6 +3388,7 @@
       <c r="L65" s="7"/>
       <c r="M65" s="7"/>
       <c r="N65" s="7"/>
+      <c r="O65" s="7"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
@@ -3291,6 +3436,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O66" s="7"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -3326,6 +3472,7 @@
       <c r="L67" s="7"/>
       <c r="M67" s="7"/>
       <c r="N67" s="7"/>
+      <c r="O67" s="7"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
@@ -3365,6 +3512,7 @@
       <c r="L68" s="7"/>
       <c r="M68" s="7"/>
       <c r="N68" s="7"/>
+      <c r="O68" s="7"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -3420,6 +3568,11 @@
         </is>
       </c>
       <c r="N69" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="O69" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -3459,6 +3612,7 @@
       <c r="L70" s="7"/>
       <c r="M70" s="7"/>
       <c r="N70" s="7"/>
+      <c r="O70" s="7"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -3499,6 +3653,7 @@
       <c r="L71" s="7"/>
       <c r="M71" s="7"/>
       <c r="N71" s="7"/>
+      <c r="O71" s="7"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
@@ -3542,6 +3697,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O72" s="7"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
@@ -3582,6 +3738,7 @@
       <c r="L73" s="7"/>
       <c r="M73" s="7"/>
       <c r="N73" s="7"/>
+      <c r="O73" s="7"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -3617,6 +3774,7 @@
       <c r="L74" s="7"/>
       <c r="M74" s="7"/>
       <c r="N74" s="7"/>
+      <c r="O74" s="7"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -3652,6 +3810,7 @@
       <c r="L75" s="7"/>
       <c r="M75" s="7"/>
       <c r="N75" s="7"/>
+      <c r="O75" s="7"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -3687,6 +3846,7 @@
       <c r="L76" s="7"/>
       <c r="M76" s="7"/>
       <c r="N76" s="7"/>
+      <c r="O76" s="7"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -3722,6 +3882,7 @@
       <c r="L77" s="7"/>
       <c r="M77" s="7"/>
       <c r="N77" s="7"/>
+      <c r="O77" s="7"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
@@ -3757,6 +3918,7 @@
       <c r="L78" s="7"/>
       <c r="M78" s="7"/>
       <c r="N78" s="7"/>
+      <c r="O78" s="7"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -3797,6 +3959,7 @@
       <c r="L79" s="7"/>
       <c r="M79" s="7"/>
       <c r="N79" s="7"/>
+      <c r="O79" s="7"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
@@ -3840,6 +4003,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O80" s="7"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
@@ -3875,6 +4039,7 @@
       <c r="L81" s="7"/>
       <c r="M81" s="7"/>
       <c r="N81" s="7"/>
+      <c r="O81" s="7"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
@@ -3910,6 +4075,7 @@
       <c r="L82" s="7"/>
       <c r="M82" s="7"/>
       <c r="N82" s="7"/>
+      <c r="O82" s="7"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
@@ -3950,6 +4116,7 @@
       <c r="L83" s="7"/>
       <c r="M83" s="7"/>
       <c r="N83" s="7"/>
+      <c r="O83" s="7"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
@@ -3985,6 +4152,7 @@
       <c r="L84" s="7"/>
       <c r="M84" s="7"/>
       <c r="N84" s="7"/>
+      <c r="O84" s="7"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
@@ -4020,6 +4188,7 @@
       <c r="L85" s="7"/>
       <c r="M85" s="7"/>
       <c r="N85" s="7"/>
+      <c r="O85" s="7"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
@@ -4060,6 +4229,7 @@
       <c r="L86" s="7"/>
       <c r="M86" s="7"/>
       <c r="N86" s="7"/>
+      <c r="O86" s="7"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
@@ -4095,6 +4265,7 @@
       <c r="L87" s="7"/>
       <c r="M87" s="7"/>
       <c r="N87" s="7"/>
+      <c r="O87" s="7"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
@@ -4130,6 +4301,7 @@
       <c r="L88" s="7"/>
       <c r="M88" s="7"/>
       <c r="N88" s="7"/>
+      <c r="O88" s="7"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
@@ -4165,6 +4337,7 @@
       <c r="L89" s="7"/>
       <c r="M89" s="7"/>
       <c r="N89" s="7"/>
+      <c r="O89" s="7"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
@@ -4229,6 +4402,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O90" s="7"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
@@ -4264,6 +4438,7 @@
       <c r="L91" s="7"/>
       <c r="M91" s="7"/>
       <c r="N91" s="7"/>
+      <c r="O91" s="7"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
@@ -4323,6 +4498,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O92" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
@@ -4387,6 +4567,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O93" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
@@ -4416,7 +4601,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t xml:space="preserve">10-13 수정분</t>
+          <t xml:space="preserve">10-13 수정분 · 🗑️ 폐기(10-15 #144 — 미해금 동안 원형 자체를 안 그림 · CID_117 로 갈음)</t>
         </is>
       </c>
       <c r="G94" s="7"/>
@@ -4427,6 +4612,7 @@
       <c r="L94" s="7"/>
       <c r="M94" s="7"/>
       <c r="N94" s="7"/>
+      <c r="O94" s="7"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
@@ -4452,6 +4638,11 @@
       <c r="E95" t="inlineStr">
         <is>
           <t xml:space="preserve">「Auto」 토글이 S4 전엔 돌지 않는가?</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">🗑️ 폐기(10-15 #144 — 미해금 동안 원형 자체를 안 그림 · CID_117 로 갈음)</t>
         </is>
       </c>
       <c r="G95" s="7"/>
@@ -4462,6 +4653,7 @@
       <c r="L95" s="7"/>
       <c r="M95" s="7"/>
       <c r="N95" s="7"/>
+      <c r="O95" s="7"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
@@ -4521,6 +4713,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O96" s="7"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="inlineStr">
@@ -4556,6 +4749,7 @@
       <c r="L97" s="7"/>
       <c r="M97" s="7"/>
       <c r="N97" s="7"/>
+      <c r="O97" s="7"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
@@ -4591,6 +4785,7 @@
       <c r="L98" s="7"/>
       <c r="M98" s="7"/>
       <c r="N98" s="7"/>
+      <c r="O98" s="7"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
@@ -4626,6 +4821,7 @@
       <c r="L99" s="7"/>
       <c r="M99" s="7"/>
       <c r="N99" s="7"/>
+      <c r="O99" s="7"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
@@ -4666,6 +4862,11 @@
       <c r="L100" s="7"/>
       <c r="M100" s="7"/>
       <c r="N100" s="7"/>
+      <c r="O100" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
@@ -4701,6 +4902,7 @@
       <c r="L101" s="7"/>
       <c r="M101" s="7"/>
       <c r="N101" s="7"/>
+      <c r="O101" s="7"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
@@ -4736,6 +4938,7 @@
       <c r="L102" s="7"/>
       <c r="M102" s="7"/>
       <c r="N102" s="7"/>
+      <c r="O102" s="7"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="inlineStr">
@@ -4771,6 +4974,7 @@
       <c r="L103" s="7"/>
       <c r="M103" s="7"/>
       <c r="N103" s="7"/>
+      <c r="O103" s="7"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="inlineStr">
@@ -4811,6 +5015,7 @@
       <c r="L104" s="7"/>
       <c r="M104" s="7"/>
       <c r="N104" s="7"/>
+      <c r="O104" s="7"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
@@ -4846,6 +5051,7 @@
       <c r="L105" s="7"/>
       <c r="M105" s="7"/>
       <c r="N105" s="7"/>
+      <c r="O105" s="7"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
@@ -4881,6 +5087,7 @@
       <c r="L106" s="7"/>
       <c r="M106" s="7"/>
       <c r="N106" s="7"/>
+      <c r="O106" s="7"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
@@ -4916,6 +5123,7 @@
       <c r="L107" s="7"/>
       <c r="M107" s="7"/>
       <c r="N107" s="7"/>
+      <c r="O107" s="7"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
@@ -4955,6 +5163,7 @@
       <c r="L108" s="7"/>
       <c r="M108" s="7"/>
       <c r="N108" s="7"/>
+      <c r="O108" s="7"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="inlineStr">
@@ -4999,6 +5208,7 @@
       <c r="L109" s="7"/>
       <c r="M109" s="7"/>
       <c r="N109" s="7"/>
+      <c r="O109" s="7"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
@@ -5047,6 +5257,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O110" s="7"/>
     </row>
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
@@ -5094,6 +5305,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O111" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
@@ -5146,6 +5362,7 @@
       </c>
       <c r="M112" s="7"/>
       <c r="N112" s="7"/>
+      <c r="O112" s="7"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
@@ -5190,6 +5407,7 @@
       <c r="L113" s="7"/>
       <c r="M113" s="7"/>
       <c r="N113" s="7"/>
+      <c r="O113" s="7"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="inlineStr">
@@ -5242,6 +5460,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O114" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="7" t="inlineStr">
@@ -5294,6 +5517,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O115" s="7"/>
     </row>
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
@@ -5342,6 +5566,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O116" s="7"/>
     </row>
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
@@ -5390,6 +5615,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O117" s="7"/>
     </row>
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
@@ -5438,6 +5664,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O118" s="7"/>
     </row>
     <row r="119">
       <c r="A119" s="7" t="inlineStr">
@@ -5486,6 +5713,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O119" s="7"/>
     </row>
     <row r="120">
       <c r="A120" s="7" t="inlineStr">
@@ -5530,6 +5758,7 @@
         </is>
       </c>
       <c r="N120" s="7"/>
+      <c r="O120" s="7"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="inlineStr">
@@ -5578,6 +5807,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O121" s="7"/>
     </row>
     <row r="122">
       <c r="A122" s="7" t="inlineStr">
@@ -5622,6 +5852,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="O122" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="7" t="inlineStr">
@@ -5662,6 +5897,97 @@
       <c r="L123" s="7"/>
       <c r="M123" s="7"/>
       <c r="N123" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="O123" s="7"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_116</t>
+        </is>
+      </c>
+      <c r="B124" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">보드</t>
+        </is>
+      </c>
+      <c r="C124" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">모드 단추</t>
+        </is>
+      </c>
+      <c r="D124" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도전 중 잠김</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도전 층에서 조립 보드에 들어가면 모드 단추가 「도전 중 변경 불가」로 흐리고 눌러도 안 바뀌는가? (파밍 층·튜토리얼 판은 그대로 「조립/이동 모드 (바꾸기)」)</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#123 「들어가되 못 고친다」의 화면 표현 (10-15 #143)</t>
+        </is>
+      </c>
+      <c r="G124" s="7"/>
+      <c r="H124" s="7"/>
+      <c r="I124" s="7"/>
+      <c r="J124" s="7"/>
+      <c r="K124" s="7"/>
+      <c r="L124" s="7"/>
+      <c r="M124" s="7"/>
+      <c r="N124" s="7"/>
+      <c r="O124" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_117</t>
+        </is>
+      </c>
+      <c r="B125" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">태그</t>
+        </is>
+      </c>
+      <c r="C125" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">노출</t>
+        </is>
+      </c>
+      <c r="D125" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">해금 뒤에만</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">로봇 B 해금 전(S4 통과 전 · S4 이하)에는 「로봇 B」·「Auto」·「합체」 원형과 링이 안 보이고, S4 통과 또는 S5·S6 점프 뒤에는 보이는가?</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">「로봇 B 미해금」 표시 폐기 (10-15 #144)</t>
+        </is>
+      </c>
+      <c r="G125" s="7"/>
+      <c r="H125" s="7"/>
+      <c r="I125" s="7"/>
+      <c r="J125" s="7"/>
+      <c r="K125" s="7"/>
+      <c r="L125" s="7"/>
+      <c r="M125" s="7"/>
+      <c r="N125" s="7"/>
+      <c r="O125" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -5694,9 +6020,9 @@
     <mergeCell ref="B92:B99"/>
     <mergeCell ref="B100:B106"/>
     <mergeCell ref="B107:B111"/>
-    <mergeCell ref="G7:N7"/>
+    <mergeCell ref="G7:O7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:N123">
+  <conditionalFormatting sqref="G9:O125">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
QA P열(9c2b4a0) — #145~#147 · S2 알림 재확인 Pass 37 · Fail 0 · CID_118~121 신설
요약 P·Q → Q·R 로 밈 · 범위 P9:P129 · 전체 121 · 병합 G7:P7 · 조건부 서식 G9:P129 · CID_108·110 비고에 #147 문안 덧. 리포 8123 에서 같은 빌드로 재확인 뒤 8127 갈아엎음(20:32:26).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -171,8 +171,9 @@
     <col min="13" max="13" width="12" customWidth="1"/>
     <col min="14" max="14" width="12" customWidth="1"/>
     <col min="15" max="15" width="12" customWidth="1"/>
-    <col min="16" max="16" width="11" customWidth="1"/>
+    <col min="16" max="16" width="12" customWidth="1"/>
     <col min="17" max="17" width="11" customWidth="1"/>
+    <col min="18" max="18" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -330,6 +331,11 @@
       <c r="O6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">video-261014c 후보 · #143 도전 중 보드 모드 단추 「도전 중 변경 불가」 흐림 · #144 태그 원형 셋(로봇 B·Auto·합체)은 로봇 B 해금 뒤에만 ‖ 10-15 코드 세션 재확인(리포 8123 같은 빌드 · 576×1024 · 소리 0 · S1 파밍 원형 없음 → 도전 → 조립: 모드 판 흐림·눌러도 그대로 → S5 점프: 태그·Auto·합체 보임 → 처음부터 → 튜토 판 모드 단추 그대로 → 튜토·S1 원형 없음 → T3 막 구멍 그대로) · 8127 갈아엎음 19:49:09 · 빈 칸 = 안 지나감 · CID_086·087 은 비고에 폐기 표기(#144 · CID_117 로 갈음) · CID_116·117 새 항목</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">video-261014c 후보 · #145 튜토리얼 목표 줄 「(지금/40)」 · #146 도전 층 보드 이동 모드 고정 · #147 「생산량·생산속도 모듈」 · S2 지급 알림 결함(세션에 한 번이라 같은 창 처음부터 뒤 안 뜸 · 설정이 가린 동안 시계가 흘러 놓침) 고침 ‖ 10-15 코드 세션 재확인(리포 8123 · d28d8b2·cfc72d3·9c2b4a0 세 회차 · 576×1024 · 소리 0 · 튜토 (0/40)→(14/40)→(30/40)→(36/40) · S1 도전 중 조립: 이동 모드·끌기 됨·모드 판 흐림 → 파밍 오면 조립 모드로 되돌아옴 · 다음 스테이지로 알림 · 탭으로 닫힘 · 설정 바로가기 S2 후 8초 늦게 닫아도 알림 · 같은 창 처음부터 → 다음 스테이지로 알림 다시 · T4 안내·팔레트·팝오버 「생산량 모듈」) · 8127 갈아엎음 20:32:26 · 빈 칸 = 안 지나감 · 관찰(판정 없음): 결과 화면 직후 설정을 열어 바로가기로 판을 옮기면 S1 통과가 안 남았다(시험 손 · 「스테이지로」를 거치면 남음) · CID_118~121 새 항목</t>
         </is>
       </c>
     </row>
@@ -369,14 +375,15 @@
       <c r="M7" s="2"/>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
-      <c r="P7" s="2" t="inlineStr">
+      <c r="P7" s="2"/>
+      <c r="Q7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">버전</t>
         </is>
       </c>
-      <c r="Q7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4dbd244</t>
+      <c r="R7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9c2b4a0</t>
         </is>
       </c>
     </row>
@@ -446,11 +453,16 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">9c2b4a0</t>
+        </is>
+      </c>
+      <c r="Q8" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">PASSrate</t>
         </is>
       </c>
-      <c r="Q8" s="7">
-        <f>COUNTIF(O9:O125,"Pass")</f>
+      <c r="R8" s="7">
+        <f>COUNTIF(P9:P129,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -521,13 +533,18 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="P9" s="2" t="inlineStr">
+      <c r="P9" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="Q9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FAILrate</t>
         </is>
       </c>
-      <c r="Q9" s="7">
-        <f>COUNTIF(O9:O125,"Fail")+COUNTIF(O9:O125,"Broken")</f>
+      <c r="R9" s="7">
+        <f>COUNTIF(P9:P129,"Fail")+COUNTIF(P9:P129,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -570,13 +587,14 @@
       <c r="M10" s="7"/>
       <c r="N10" s="7"/>
       <c r="O10" s="7"/>
-      <c r="P10" s="2" t="inlineStr">
+      <c r="P10" s="7"/>
+      <c r="Q10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">N/A</t>
         </is>
       </c>
-      <c r="Q10" s="7">
-        <f>COUNTIF(O9:O125,"N/A")</f>
+      <c r="R10" s="7">
+        <f>COUNTIF(P9:P129,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -619,13 +637,14 @@
       <c r="M11" s="7"/>
       <c r="N11" s="7"/>
       <c r="O11" s="7"/>
-      <c r="P11" s="2" t="inlineStr">
+      <c r="P11" s="7"/>
+      <c r="Q11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">전체 개수</t>
         </is>
       </c>
-      <c r="Q11" s="7">
-        <v>117</v>
+      <c r="R11" s="7">
+        <v>121</v>
       </c>
     </row>
     <row r="12">
@@ -668,13 +687,14 @@
       <c r="M12" s="7"/>
       <c r="N12" s="7"/>
       <c r="O12" s="7"/>
-      <c r="P12" s="2" t="inlineStr">
+      <c r="P12" s="7"/>
+      <c r="Q12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">진행율</t>
         </is>
       </c>
-      <c r="Q12" s="7">
-        <f>TEXT((COUNTA(O9:O125))/117,"0.00%")</f>
+      <c r="R12" s="7">
+        <f>TEXT((COUNTA(P9:P129))/121,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -721,6 +741,7 @@
       <c r="M13" s="7"/>
       <c r="N13" s="7"/>
       <c r="O13" s="7"/>
+      <c r="P13" s="7"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -757,6 +778,7 @@
       <c r="M14" s="7"/>
       <c r="N14" s="7"/>
       <c r="O14" s="7"/>
+      <c r="P14" s="7"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -821,6 +843,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="P15" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -885,6 +912,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="P16" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -950,6 +982,11 @@
         </is>
       </c>
       <c r="O17" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="P17" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -995,6 +1032,7 @@
       <c r="M18" s="7"/>
       <c r="N18" s="7"/>
       <c r="O18" s="7"/>
+      <c r="P18" s="7"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -1031,6 +1069,7 @@
       <c r="M19" s="7"/>
       <c r="N19" s="7"/>
       <c r="O19" s="7"/>
+      <c r="P19" s="7"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1067,6 +1106,7 @@
       <c r="M20" s="7"/>
       <c r="N20" s="7"/>
       <c r="O20" s="7"/>
+      <c r="P20" s="7"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1131,6 +1171,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="P21" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1196,6 +1241,7 @@
         </is>
       </c>
       <c r="O22" s="7"/>
+      <c r="P22" s="7"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -1236,6 +1282,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="P23" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -1272,6 +1323,7 @@
       <c r="M24" s="7"/>
       <c r="N24" s="7"/>
       <c r="O24" s="7"/>
+      <c r="P24" s="7"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -1308,6 +1360,7 @@
       <c r="M25" s="7"/>
       <c r="N25" s="7"/>
       <c r="O25" s="7"/>
+      <c r="P25" s="7"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -1369,6 +1422,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="P26" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -1409,6 +1467,7 @@
       <c r="M27" s="7"/>
       <c r="N27" s="7"/>
       <c r="O27" s="7"/>
+      <c r="P27" s="7"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -1458,6 +1517,7 @@
       <c r="M28" s="7"/>
       <c r="N28" s="7"/>
       <c r="O28" s="7"/>
+      <c r="P28" s="7"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -1502,6 +1562,7 @@
       <c r="M29" s="7"/>
       <c r="N29" s="7"/>
       <c r="O29" s="7"/>
+      <c r="P29" s="7"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -1566,6 +1627,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="P30" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -1635,6 +1701,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="P31" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -1695,6 +1766,7 @@
         </is>
       </c>
       <c r="O32" s="7"/>
+      <c r="P32" s="7"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -1759,6 +1831,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="P33" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -1823,6 +1900,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="P34" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -1892,6 +1974,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="P35" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -1944,6 +2031,7 @@
       <c r="M36" s="7"/>
       <c r="N36" s="7"/>
       <c r="O36" s="7"/>
+      <c r="P36" s="7"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -1980,6 +2068,7 @@
       <c r="M37" s="7"/>
       <c r="N37" s="7"/>
       <c r="O37" s="7"/>
+      <c r="P37" s="7"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -2037,6 +2126,7 @@
       <c r="M38" s="7"/>
       <c r="N38" s="7"/>
       <c r="O38" s="7"/>
+      <c r="P38" s="7"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -2101,6 +2191,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="P39" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -2166,6 +2261,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="P40" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -2222,6 +2322,11 @@
         </is>
       </c>
       <c r="O41" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="P41" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -2274,6 +2379,7 @@
       <c r="M42" s="7"/>
       <c r="N42" s="7"/>
       <c r="O42" s="7"/>
+      <c r="P42" s="7"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -2334,6 +2440,11 @@
         </is>
       </c>
       <c r="O43" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="P43" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -2379,6 +2490,7 @@
       <c r="M44" s="7"/>
       <c r="N44" s="7"/>
       <c r="O44" s="7"/>
+      <c r="P44" s="7"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -2443,6 +2555,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="P45" s="7"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -2507,6 +2620,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="P46" s="7"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -2548,6 +2662,7 @@
       <c r="M47" s="7"/>
       <c r="N47" s="7"/>
       <c r="O47" s="7"/>
+      <c r="P47" s="7"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -2584,6 +2699,7 @@
       <c r="M48" s="7"/>
       <c r="N48" s="7"/>
       <c r="O48" s="7"/>
+      <c r="P48" s="7"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -2620,6 +2736,7 @@
       <c r="M49" s="7"/>
       <c r="N49" s="7"/>
       <c r="O49" s="7"/>
+      <c r="P49" s="7"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -2680,6 +2797,7 @@
         </is>
       </c>
       <c r="O50" s="7"/>
+      <c r="P50" s="7"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -2740,6 +2858,7 @@
         </is>
       </c>
       <c r="O51" s="7"/>
+      <c r="P51" s="7"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -2781,6 +2900,7 @@
       <c r="M52" s="7"/>
       <c r="N52" s="7"/>
       <c r="O52" s="7"/>
+      <c r="P52" s="7"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -2822,6 +2942,7 @@
       <c r="M53" s="7"/>
       <c r="N53" s="7"/>
       <c r="O53" s="7"/>
+      <c r="P53" s="7"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -2858,6 +2979,7 @@
       <c r="M54" s="7"/>
       <c r="N54" s="7"/>
       <c r="O54" s="7"/>
+      <c r="P54" s="7"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -2922,6 +3044,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="P55" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -2974,6 +3101,7 @@
         </is>
       </c>
       <c r="O56" s="7"/>
+      <c r="P56" s="7"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -3035,6 +3163,7 @@
         </is>
       </c>
       <c r="O57" s="7"/>
+      <c r="P57" s="7"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -3096,6 +3225,11 @@
         </is>
       </c>
       <c r="O58" s="7"/>
+      <c r="P58" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -3132,6 +3266,7 @@
       <c r="M59" s="7"/>
       <c r="N59" s="7"/>
       <c r="O59" s="7"/>
+      <c r="P59" s="7"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -3168,6 +3303,7 @@
       <c r="M60" s="7"/>
       <c r="N60" s="7"/>
       <c r="O60" s="7"/>
+      <c r="P60" s="7"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -3216,6 +3352,7 @@
       <c r="M61" s="7"/>
       <c r="N61" s="7"/>
       <c r="O61" s="7"/>
+      <c r="P61" s="7"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -3264,6 +3401,11 @@
         </is>
       </c>
       <c r="O62" s="7"/>
+      <c r="P62" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -3312,6 +3454,7 @@
       </c>
       <c r="N63" s="7"/>
       <c r="O63" s="7"/>
+      <c r="P63" s="7"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -3348,6 +3491,7 @@
       <c r="M64" s="7"/>
       <c r="N64" s="7"/>
       <c r="O64" s="7"/>
+      <c r="P64" s="7"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -3389,6 +3533,7 @@
       <c r="M65" s="7"/>
       <c r="N65" s="7"/>
       <c r="O65" s="7"/>
+      <c r="P65" s="7"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
@@ -3437,6 +3582,7 @@
         </is>
       </c>
       <c r="O66" s="7"/>
+      <c r="P66" s="7"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -3473,6 +3619,7 @@
       <c r="M67" s="7"/>
       <c r="N67" s="7"/>
       <c r="O67" s="7"/>
+      <c r="P67" s="7"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
@@ -3513,6 +3660,7 @@
       <c r="M68" s="7"/>
       <c r="N68" s="7"/>
       <c r="O68" s="7"/>
+      <c r="P68" s="7"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -3573,6 +3721,11 @@
         </is>
       </c>
       <c r="O69" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="P69" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -3613,6 +3766,7 @@
       <c r="M70" s="7"/>
       <c r="N70" s="7"/>
       <c r="O70" s="7"/>
+      <c r="P70" s="7"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -3654,6 +3808,7 @@
       <c r="M71" s="7"/>
       <c r="N71" s="7"/>
       <c r="O71" s="7"/>
+      <c r="P71" s="7"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
@@ -3698,6 +3853,11 @@
         </is>
       </c>
       <c r="O72" s="7"/>
+      <c r="P72" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
@@ -3739,6 +3899,7 @@
       <c r="M73" s="7"/>
       <c r="N73" s="7"/>
       <c r="O73" s="7"/>
+      <c r="P73" s="7"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -3775,6 +3936,7 @@
       <c r="M74" s="7"/>
       <c r="N74" s="7"/>
       <c r="O74" s="7"/>
+      <c r="P74" s="7"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -3811,6 +3973,7 @@
       <c r="M75" s="7"/>
       <c r="N75" s="7"/>
       <c r="O75" s="7"/>
+      <c r="P75" s="7"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -3847,6 +4010,7 @@
       <c r="M76" s="7"/>
       <c r="N76" s="7"/>
       <c r="O76" s="7"/>
+      <c r="P76" s="7"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -3883,6 +4047,7 @@
       <c r="M77" s="7"/>
       <c r="N77" s="7"/>
       <c r="O77" s="7"/>
+      <c r="P77" s="7"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
@@ -3919,6 +4084,7 @@
       <c r="M78" s="7"/>
       <c r="N78" s="7"/>
       <c r="O78" s="7"/>
+      <c r="P78" s="7"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -3960,6 +4126,7 @@
       <c r="M79" s="7"/>
       <c r="N79" s="7"/>
       <c r="O79" s="7"/>
+      <c r="P79" s="7"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
@@ -4004,6 +4171,11 @@
         </is>
       </c>
       <c r="O80" s="7"/>
+      <c r="P80" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
@@ -4040,6 +4212,7 @@
       <c r="M81" s="7"/>
       <c r="N81" s="7"/>
       <c r="O81" s="7"/>
+      <c r="P81" s="7"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
@@ -4076,6 +4249,7 @@
       <c r="M82" s="7"/>
       <c r="N82" s="7"/>
       <c r="O82" s="7"/>
+      <c r="P82" s="7"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
@@ -4117,6 +4291,7 @@
       <c r="M83" s="7"/>
       <c r="N83" s="7"/>
       <c r="O83" s="7"/>
+      <c r="P83" s="7"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
@@ -4153,6 +4328,7 @@
       <c r="M84" s="7"/>
       <c r="N84" s="7"/>
       <c r="O84" s="7"/>
+      <c r="P84" s="7"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
@@ -4189,6 +4365,7 @@
       <c r="M85" s="7"/>
       <c r="N85" s="7"/>
       <c r="O85" s="7"/>
+      <c r="P85" s="7"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
@@ -4230,6 +4407,7 @@
       <c r="M86" s="7"/>
       <c r="N86" s="7"/>
       <c r="O86" s="7"/>
+      <c r="P86" s="7"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
@@ -4266,6 +4444,7 @@
       <c r="M87" s="7"/>
       <c r="N87" s="7"/>
       <c r="O87" s="7"/>
+      <c r="P87" s="7"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
@@ -4302,6 +4481,7 @@
       <c r="M88" s="7"/>
       <c r="N88" s="7"/>
       <c r="O88" s="7"/>
+      <c r="P88" s="7"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
@@ -4338,6 +4518,7 @@
       <c r="M89" s="7"/>
       <c r="N89" s="7"/>
       <c r="O89" s="7"/>
+      <c r="P89" s="7"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
@@ -4403,6 +4584,7 @@
         </is>
       </c>
       <c r="O90" s="7"/>
+      <c r="P90" s="7"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
@@ -4439,6 +4621,7 @@
       <c r="M91" s="7"/>
       <c r="N91" s="7"/>
       <c r="O91" s="7"/>
+      <c r="P91" s="7"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
@@ -4503,6 +4686,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="P92" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
@@ -4568,6 +4756,11 @@
         </is>
       </c>
       <c r="O93" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="P93" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -4613,6 +4806,7 @@
       <c r="M94" s="7"/>
       <c r="N94" s="7"/>
       <c r="O94" s="7"/>
+      <c r="P94" s="7"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
@@ -4654,6 +4848,7 @@
       <c r="M95" s="7"/>
       <c r="N95" s="7"/>
       <c r="O95" s="7"/>
+      <c r="P95" s="7"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
@@ -4714,6 +4909,7 @@
         </is>
       </c>
       <c r="O96" s="7"/>
+      <c r="P96" s="7"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="inlineStr">
@@ -4750,6 +4946,7 @@
       <c r="M97" s="7"/>
       <c r="N97" s="7"/>
       <c r="O97" s="7"/>
+      <c r="P97" s="7"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
@@ -4786,6 +4983,7 @@
       <c r="M98" s="7"/>
       <c r="N98" s="7"/>
       <c r="O98" s="7"/>
+      <c r="P98" s="7"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
@@ -4822,6 +5020,7 @@
       <c r="M99" s="7"/>
       <c r="N99" s="7"/>
       <c r="O99" s="7"/>
+      <c r="P99" s="7"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
@@ -4867,6 +5066,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="P100" s="7"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
@@ -4903,6 +5103,7 @@
       <c r="M101" s="7"/>
       <c r="N101" s="7"/>
       <c r="O101" s="7"/>
+      <c r="P101" s="7"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
@@ -4939,6 +5140,7 @@
       <c r="M102" s="7"/>
       <c r="N102" s="7"/>
       <c r="O102" s="7"/>
+      <c r="P102" s="7"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="inlineStr">
@@ -4975,6 +5177,7 @@
       <c r="M103" s="7"/>
       <c r="N103" s="7"/>
       <c r="O103" s="7"/>
+      <c r="P103" s="7"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="inlineStr">
@@ -5016,6 +5219,7 @@
       <c r="M104" s="7"/>
       <c r="N104" s="7"/>
       <c r="O104" s="7"/>
+      <c r="P104" s="7"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
@@ -5052,6 +5256,7 @@
       <c r="M105" s="7"/>
       <c r="N105" s="7"/>
       <c r="O105" s="7"/>
+      <c r="P105" s="7"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
@@ -5088,6 +5293,7 @@
       <c r="M106" s="7"/>
       <c r="N106" s="7"/>
       <c r="O106" s="7"/>
+      <c r="P106" s="7"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
@@ -5124,6 +5330,7 @@
       <c r="M107" s="7"/>
       <c r="N107" s="7"/>
       <c r="O107" s="7"/>
+      <c r="P107" s="7"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
@@ -5164,6 +5371,7 @@
       <c r="M108" s="7"/>
       <c r="N108" s="7"/>
       <c r="O108" s="7"/>
+      <c r="P108" s="7"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="inlineStr">
@@ -5209,6 +5417,7 @@
       <c r="M109" s="7"/>
       <c r="N109" s="7"/>
       <c r="O109" s="7"/>
+      <c r="P109" s="7"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
@@ -5258,6 +5467,11 @@
         </is>
       </c>
       <c r="O110" s="7"/>
+      <c r="P110" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
@@ -5310,6 +5524,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="P111" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
@@ -5363,6 +5582,7 @@
       <c r="M112" s="7"/>
       <c r="N112" s="7"/>
       <c r="O112" s="7"/>
+      <c r="P112" s="7"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
@@ -5408,6 +5628,7 @@
       <c r="M113" s="7"/>
       <c r="N113" s="7"/>
       <c r="O113" s="7"/>
+      <c r="P113" s="7"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="inlineStr">
@@ -5465,6 +5686,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="P114" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="7" t="inlineStr">
@@ -5518,6 +5744,7 @@
         </is>
       </c>
       <c r="O115" s="7"/>
+      <c r="P115" s="7"/>
     </row>
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
@@ -5547,7 +5774,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t xml:space="preserve">표시 4초(가정) · 알림이 걷힌 뒤 막 (10-15 #138)</t>
+          <t xml:space="preserve">표시 4초(가정) · 알림이 걷힌 뒤 막 (10-15 #138) · 10-15 #147 로 문안 「생산량·생산속도 모듈을 받았습니다」 · 경로 무관(CID_121)</t>
         </is>
       </c>
       <c r="G116" s="7"/>
@@ -5567,6 +5794,11 @@
         </is>
       </c>
       <c r="O116" s="7"/>
+      <c r="P116" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
@@ -5616,6 +5848,11 @@
         </is>
       </c>
       <c r="O117" s="7"/>
+      <c r="P117" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
@@ -5645,7 +5882,7 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t xml:space="preserve">대상 노드 = 하네스 실측 가정 · 안내는 맨 윗줄이라 칸 아래에 앉는다 (10-15 #138)</t>
+          <t xml:space="preserve">대상 노드 = 하네스 실측 가정 · 안내는 맨 윗줄이라 칸 아래에 앉는다 (10-15 #138) · 10-15 #147 로 안내 「모듈 탭에서 생산량 또는 생산속도 모듈을 고른 뒤 이 노드를 탭하세요」</t>
         </is>
       </c>
       <c r="G118" s="7"/>
@@ -5665,6 +5902,11 @@
         </is>
       </c>
       <c r="O118" s="7"/>
+      <c r="P118" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="7" t="inlineStr">
@@ -5714,6 +5956,7 @@
         </is>
       </c>
       <c r="O119" s="7"/>
+      <c r="P119" s="7"/>
     </row>
     <row r="120">
       <c r="A120" s="7" t="inlineStr">
@@ -5759,6 +6002,7 @@
       </c>
       <c r="N120" s="7"/>
       <c r="O120" s="7"/>
+      <c r="P120" s="7"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="inlineStr">
@@ -5808,6 +6052,11 @@
         </is>
       </c>
       <c r="O121" s="7"/>
+      <c r="P121" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="7" t="inlineStr">
@@ -5857,6 +6106,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="P122" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="7" t="inlineStr">
@@ -5902,6 +6156,7 @@
         </is>
       </c>
       <c r="O123" s="7"/>
+      <c r="P123" s="7"/>
     </row>
     <row r="124">
       <c r="A124" s="7" t="inlineStr">
@@ -5947,6 +6202,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="P124" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="7" t="inlineStr">
@@ -5988,6 +6248,191 @@
       <c r="M125" s="7"/>
       <c r="N125" s="7"/>
       <c r="O125" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="P125" s="7"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_118</t>
+        </is>
+      </c>
+      <c r="B126" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼</t>
+        </is>
+      </c>
+      <c r="C126" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">마일스톤</t>
+        </is>
+      </c>
+      <c r="D126" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">마운트 수치</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">마일스톤 「마운트가 가득 찬다」 옆에 (지금 보유량 / 목표 보유량)이 붙어 오르는가? (예 (14/40) · 다 차면 (40/40))</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">목표 수 = 전 슬롯 기준 40 (10-15 #145 · 꼴 가정)</t>
+        </is>
+      </c>
+      <c r="G126" s="7"/>
+      <c r="H126" s="7"/>
+      <c r="I126" s="7"/>
+      <c r="J126" s="7"/>
+      <c r="K126" s="7"/>
+      <c r="L126" s="7"/>
+      <c r="M126" s="7"/>
+      <c r="N126" s="7"/>
+      <c r="O126" s="7"/>
+      <c r="P126" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_119</t>
+        </is>
+      </c>
+      <c r="B127" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">보드</t>
+        </is>
+      </c>
+      <c r="C127" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도전 층</t>
+        </is>
+      </c>
+      <c r="D127" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">이동 모드 고정</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도전 중 조립 보드에 들어가면 이동 모드로 서서 끌면 화면이 움직이고, 파밍으로 돌아오면 전에 쓰던 모드로 되돌아오는가?</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">모드 판은 「도전 중 변경 불가」 흐림 그대로 (10-15 #146)</t>
+        </is>
+      </c>
+      <c r="G127" s="7"/>
+      <c r="H127" s="7"/>
+      <c r="I127" s="7"/>
+      <c r="J127" s="7"/>
+      <c r="K127" s="7"/>
+      <c r="L127" s="7"/>
+      <c r="M127" s="7"/>
+      <c r="N127" s="7"/>
+      <c r="O127" s="7"/>
+      <c r="P127" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_120</t>
+        </is>
+      </c>
+      <c r="B128" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">보드</t>
+        </is>
+      </c>
+      <c r="C128" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">모듈</t>
+        </is>
+      </c>
+      <c r="D128" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">이름</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">팔레트 단추·노드 팝오버 「붙은 모듈」·T4 안내·지급 알림이 「생산량 모듈」·「생산속도 모듈」로 적히는가? (글자 M/R 없음 · 노드 위 그림은 그대로)</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">자산 이름 + 「 모듈」 (10-15 #147)</t>
+        </is>
+      </c>
+      <c r="G128" s="7"/>
+      <c r="H128" s="7"/>
+      <c r="I128" s="7"/>
+      <c r="J128" s="7"/>
+      <c r="K128" s="7"/>
+      <c r="L128" s="7"/>
+      <c r="M128" s="7"/>
+      <c r="N128" s="7"/>
+      <c r="O128" s="7"/>
+      <c r="P128" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_121</t>
+        </is>
+      </c>
+      <c r="B129" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼</t>
+        </is>
+      </c>
+      <c r="C129" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T4 알림</t>
+        </is>
+      </c>
+      <c r="D129" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">진입 경로 무관</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S1 통과 뒤 「다음 스테이지로」든 설정 바로가기 S2 든 지급 알림이 뜨는가? 같은 창에서 「처음부터」 뒤 다시 돌아도 뜨고, 설정을 늦게 닫아도 놓치지 않는가?</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6초(가정) 또는 탭으로 닫힘 (10-15 결함 고침)</t>
+        </is>
+      </c>
+      <c r="G129" s="7"/>
+      <c r="H129" s="7"/>
+      <c r="I129" s="7"/>
+      <c r="J129" s="7"/>
+      <c r="K129" s="7"/>
+      <c r="L129" s="7"/>
+      <c r="M129" s="7"/>
+      <c r="N129" s="7"/>
+      <c r="O129" s="7"/>
+      <c r="P129" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -6020,9 +6465,9 @@
     <mergeCell ref="B92:B99"/>
     <mergeCell ref="B100:B106"/>
     <mergeCell ref="B107:B111"/>
-    <mergeCell ref="G7:O7"/>
+    <mergeCell ref="G7:P7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:O125">
+  <conditionalFormatting sqref="G9:P129">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
QA Q열(9d3a11e) — #148 재확인 Pass 25 · Fail 0 · CID_122 신설
요약 Q·R → R·S 로 밈 · 범위 Q9:Q130 · 전체 122 · 병합 G7:Q7 · 조건부 서식 G9:Q130. 리포 8123 에서 같은 빌드로 재확인 뒤 8127 갈아엎음(20:49:22).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -172,8 +172,9 @@
     <col min="14" max="14" width="12" customWidth="1"/>
     <col min="15" max="15" width="12" customWidth="1"/>
     <col min="16" max="16" width="12" customWidth="1"/>
-    <col min="17" max="17" width="11" customWidth="1"/>
+    <col min="17" max="17" width="12" customWidth="1"/>
     <col min="18" max="18" width="11" customWidth="1"/>
+    <col min="19" max="19" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -336,6 +337,11 @@
       <c r="P6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">video-261014c 후보 · #145 튜토리얼 목표 줄 「(지금/40)」 · #146 도전 층 보드 이동 모드 고정 · #147 「생산량·생산속도 모듈」 · S2 지급 알림 결함(세션에 한 번이라 같은 창 처음부터 뒤 안 뜸 · 설정이 가린 동안 시계가 흘러 놓침) 고침 ‖ 10-15 코드 세션 재확인(리포 8123 · d28d8b2·cfc72d3·9c2b4a0 세 회차 · 576×1024 · 소리 0 · 튜토 (0/40)→(14/40)→(30/40)→(36/40) · S1 도전 중 조립: 이동 모드·끌기 됨·모드 판 흐림 → 파밍 오면 조립 모드로 되돌아옴 · 다음 스테이지로 알림 · 탭으로 닫힘 · 설정 바로가기 S2 후 8초 늦게 닫아도 알림 · 같은 창 처음부터 → 다음 스테이지로 알림 다시 · T4 안내·팔레트·팝오버 「생산량 모듈」) · 8127 갈아엎음 20:32:26 · 빈 칸 = 안 지나감 · 관찰(판정 없음): 결과 화면 직후 설정을 열어 바로가기로 판을 옮기면 S1 통과가 안 남았다(시험 손 · 「스테이지로」를 거치면 남음) · CID_118~121 새 항목</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">video-261014c 후보 · #148 도전 층 이동 모드: 끌면 이동 · 탭 = 팝오버(보기) · 팝오버 편집 행(90도 돌리기·떼기·조합표·탄종) 흐림 · 도전 층을 나오면 팝오버 닫음 ‖ 10-15 코드 세션 재확인(리포 8123 · dfbf6c8·9d3a11e · 576×1024 · 소리 0 · S1 도전 중 조립: 노드 탭 팝오버 · 편집 행 흐림 · 흐린 조합표 눌러도 그대로 · 팝오버 연 채 전투로 → 즉시 종료 → 다음 스테이지로 → 알림 · 탭 닫힘 → 조립: 팝오버 닫혀 있음 · 조립 모드 · 생산속도 모듈 붙여 T4 풀림) · 8127 갈아엎음 시각은 README · 빈 칸 = 안 지나감 · 관찰(판정 없음): 보드를 연 직후 첫 탭이 한 번 헛돎(브라우저 자동화 초점일 수 있음) · CID_122 새 항목</t>
         </is>
       </c>
     </row>
@@ -376,14 +382,15 @@
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
       <c r="P7" s="2"/>
-      <c r="Q7" s="2" t="inlineStr">
+      <c r="Q7" s="2"/>
+      <c r="R7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">버전</t>
         </is>
       </c>
-      <c r="R7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">9c2b4a0</t>
+      <c r="S7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9d3a11e</t>
         </is>
       </c>
     </row>
@@ -458,11 +465,16 @@
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">9d3a11e</t>
+        </is>
+      </c>
+      <c r="R8" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">PASSrate</t>
         </is>
       </c>
-      <c r="R8" s="7">
-        <f>COUNTIF(P9:P129,"Pass")</f>
+      <c r="S8" s="7">
+        <f>COUNTIF(Q9:Q130,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -538,13 +550,18 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="Q9" s="2" t="inlineStr">
+      <c r="Q9" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="R9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FAILrate</t>
         </is>
       </c>
-      <c r="R9" s="7">
-        <f>COUNTIF(P9:P129,"Fail")+COUNTIF(P9:P129,"Broken")</f>
+      <c r="S9" s="7">
+        <f>COUNTIF(Q9:Q130,"Fail")+COUNTIF(Q9:Q130,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -588,13 +605,14 @@
       <c r="N10" s="7"/>
       <c r="O10" s="7"/>
       <c r="P10" s="7"/>
-      <c r="Q10" s="2" t="inlineStr">
+      <c r="Q10" s="7"/>
+      <c r="R10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">N/A</t>
         </is>
       </c>
-      <c r="R10" s="7">
-        <f>COUNTIF(P9:P129,"N/A")</f>
+      <c r="S10" s="7">
+        <f>COUNTIF(Q9:Q130,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -638,13 +656,14 @@
       <c r="N11" s="7"/>
       <c r="O11" s="7"/>
       <c r="P11" s="7"/>
-      <c r="Q11" s="2" t="inlineStr">
+      <c r="Q11" s="7"/>
+      <c r="R11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">전체 개수</t>
         </is>
       </c>
-      <c r="R11" s="7">
-        <v>121</v>
+      <c r="S11" s="7">
+        <v>122</v>
       </c>
     </row>
     <row r="12">
@@ -688,13 +707,14 @@
       <c r="N12" s="7"/>
       <c r="O12" s="7"/>
       <c r="P12" s="7"/>
-      <c r="Q12" s="2" t="inlineStr">
+      <c r="Q12" s="7"/>
+      <c r="R12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">진행율</t>
         </is>
       </c>
-      <c r="R12" s="7">
-        <f>TEXT((COUNTA(P9:P129))/121,"0.00%")</f>
+      <c r="S12" s="7">
+        <f>TEXT((COUNTA(Q9:Q130))/122,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -742,6 +762,7 @@
       <c r="N13" s="7"/>
       <c r="O13" s="7"/>
       <c r="P13" s="7"/>
+      <c r="Q13" s="7"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -779,6 +800,7 @@
       <c r="N14" s="7"/>
       <c r="O14" s="7"/>
       <c r="P14" s="7"/>
+      <c r="Q14" s="7"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -848,6 +870,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Q15" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -917,6 +944,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Q16" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -987,6 +1019,11 @@
         </is>
       </c>
       <c r="P17" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="Q17" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -1033,6 +1070,7 @@
       <c r="N18" s="7"/>
       <c r="O18" s="7"/>
       <c r="P18" s="7"/>
+      <c r="Q18" s="7"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -1070,6 +1108,7 @@
       <c r="N19" s="7"/>
       <c r="O19" s="7"/>
       <c r="P19" s="7"/>
+      <c r="Q19" s="7"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1107,6 +1146,7 @@
       <c r="N20" s="7"/>
       <c r="O20" s="7"/>
       <c r="P20" s="7"/>
+      <c r="Q20" s="7"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1176,6 +1216,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Q21" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1242,6 +1287,7 @@
       </c>
       <c r="O22" s="7"/>
       <c r="P22" s="7"/>
+      <c r="Q22" s="7"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -1287,6 +1333,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Q23" s="7"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -1324,6 +1371,7 @@
       <c r="N24" s="7"/>
       <c r="O24" s="7"/>
       <c r="P24" s="7"/>
+      <c r="Q24" s="7"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -1361,6 +1409,7 @@
       <c r="N25" s="7"/>
       <c r="O25" s="7"/>
       <c r="P25" s="7"/>
+      <c r="Q25" s="7"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -1427,6 +1476,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Q26" s="7"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -1468,6 +1518,7 @@
       <c r="N27" s="7"/>
       <c r="O27" s="7"/>
       <c r="P27" s="7"/>
+      <c r="Q27" s="7"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -1518,6 +1569,7 @@
       <c r="N28" s="7"/>
       <c r="O28" s="7"/>
       <c r="P28" s="7"/>
+      <c r="Q28" s="7"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -1563,6 +1615,7 @@
       <c r="N29" s="7"/>
       <c r="O29" s="7"/>
       <c r="P29" s="7"/>
+      <c r="Q29" s="7"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -1632,6 +1685,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Q30" s="7"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -1706,6 +1760,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Q31" s="7"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -1767,6 +1822,7 @@
       </c>
       <c r="O32" s="7"/>
       <c r="P32" s="7"/>
+      <c r="Q32" s="7"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -1836,6 +1892,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Q33" s="7"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -1905,6 +1962,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Q34" s="7"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -1979,6 +2037,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Q35" s="7"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -2032,6 +2091,7 @@
       <c r="N36" s="7"/>
       <c r="O36" s="7"/>
       <c r="P36" s="7"/>
+      <c r="Q36" s="7"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -2069,6 +2129,7 @@
       <c r="N37" s="7"/>
       <c r="O37" s="7"/>
       <c r="P37" s="7"/>
+      <c r="Q37" s="7"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -2127,6 +2188,7 @@
       <c r="N38" s="7"/>
       <c r="O38" s="7"/>
       <c r="P38" s="7"/>
+      <c r="Q38" s="7"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -2196,6 +2258,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Q39" s="7"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -2266,6 +2329,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Q40" s="7"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -2331,6 +2395,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Q41" s="7"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -2380,6 +2445,7 @@
       <c r="N42" s="7"/>
       <c r="O42" s="7"/>
       <c r="P42" s="7"/>
+      <c r="Q42" s="7"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -2449,6 +2515,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Q43" s="7"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -2491,6 +2558,7 @@
       <c r="N44" s="7"/>
       <c r="O44" s="7"/>
       <c r="P44" s="7"/>
+      <c r="Q44" s="7"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -2556,6 +2624,7 @@
         </is>
       </c>
       <c r="P45" s="7"/>
+      <c r="Q45" s="7"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -2621,6 +2690,7 @@
         </is>
       </c>
       <c r="P46" s="7"/>
+      <c r="Q46" s="7"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -2663,6 +2733,7 @@
       <c r="N47" s="7"/>
       <c r="O47" s="7"/>
       <c r="P47" s="7"/>
+      <c r="Q47" s="7"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -2700,6 +2771,7 @@
       <c r="N48" s="7"/>
       <c r="O48" s="7"/>
       <c r="P48" s="7"/>
+      <c r="Q48" s="7"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -2737,6 +2809,7 @@
       <c r="N49" s="7"/>
       <c r="O49" s="7"/>
       <c r="P49" s="7"/>
+      <c r="Q49" s="7"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -2798,6 +2871,7 @@
       </c>
       <c r="O50" s="7"/>
       <c r="P50" s="7"/>
+      <c r="Q50" s="7"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -2859,6 +2933,7 @@
       </c>
       <c r="O51" s="7"/>
       <c r="P51" s="7"/>
+      <c r="Q51" s="7"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -2901,6 +2976,7 @@
       <c r="N52" s="7"/>
       <c r="O52" s="7"/>
       <c r="P52" s="7"/>
+      <c r="Q52" s="7"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -2943,6 +3019,7 @@
       <c r="N53" s="7"/>
       <c r="O53" s="7"/>
       <c r="P53" s="7"/>
+      <c r="Q53" s="7"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -2980,6 +3057,7 @@
       <c r="N54" s="7"/>
       <c r="O54" s="7"/>
       <c r="P54" s="7"/>
+      <c r="Q54" s="7"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -3049,6 +3127,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Q55" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -3102,6 +3185,7 @@
       </c>
       <c r="O56" s="7"/>
       <c r="P56" s="7"/>
+      <c r="Q56" s="7"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -3164,6 +3248,7 @@
       </c>
       <c r="O57" s="7"/>
       <c r="P57" s="7"/>
+      <c r="Q57" s="7"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -3226,6 +3311,11 @@
       </c>
       <c r="O58" s="7"/>
       <c r="P58" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="Q58" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -3267,6 +3357,7 @@
       <c r="N59" s="7"/>
       <c r="O59" s="7"/>
       <c r="P59" s="7"/>
+      <c r="Q59" s="7"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -3304,6 +3395,7 @@
       <c r="N60" s="7"/>
       <c r="O60" s="7"/>
       <c r="P60" s="7"/>
+      <c r="Q60" s="7"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -3353,6 +3445,7 @@
       <c r="N61" s="7"/>
       <c r="O61" s="7"/>
       <c r="P61" s="7"/>
+      <c r="Q61" s="7"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -3406,6 +3499,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Q62" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -3455,6 +3553,7 @@
       <c r="N63" s="7"/>
       <c r="O63" s="7"/>
       <c r="P63" s="7"/>
+      <c r="Q63" s="7"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -3492,6 +3591,7 @@
       <c r="N64" s="7"/>
       <c r="O64" s="7"/>
       <c r="P64" s="7"/>
+      <c r="Q64" s="7"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -3534,6 +3634,7 @@
       <c r="N65" s="7"/>
       <c r="O65" s="7"/>
       <c r="P65" s="7"/>
+      <c r="Q65" s="7"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
@@ -3583,6 +3684,7 @@
       </c>
       <c r="O66" s="7"/>
       <c r="P66" s="7"/>
+      <c r="Q66" s="7"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -3620,6 +3722,7 @@
       <c r="N67" s="7"/>
       <c r="O67" s="7"/>
       <c r="P67" s="7"/>
+      <c r="Q67" s="7"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
@@ -3661,6 +3764,7 @@
       <c r="N68" s="7"/>
       <c r="O68" s="7"/>
       <c r="P68" s="7"/>
+      <c r="Q68" s="7"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -3726,6 +3830,11 @@
         </is>
       </c>
       <c r="P69" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="Q69" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -3767,6 +3876,7 @@
       <c r="N70" s="7"/>
       <c r="O70" s="7"/>
       <c r="P70" s="7"/>
+      <c r="Q70" s="7"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -3809,6 +3919,7 @@
       <c r="N71" s="7"/>
       <c r="O71" s="7"/>
       <c r="P71" s="7"/>
+      <c r="Q71" s="7"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
@@ -3854,6 +3965,11 @@
       </c>
       <c r="O72" s="7"/>
       <c r="P72" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="Q72" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -3900,6 +4016,7 @@
       <c r="N73" s="7"/>
       <c r="O73" s="7"/>
       <c r="P73" s="7"/>
+      <c r="Q73" s="7"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -3937,6 +4054,7 @@
       <c r="N74" s="7"/>
       <c r="O74" s="7"/>
       <c r="P74" s="7"/>
+      <c r="Q74" s="7"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -3974,6 +4092,7 @@
       <c r="N75" s="7"/>
       <c r="O75" s="7"/>
       <c r="P75" s="7"/>
+      <c r="Q75" s="7"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -4011,6 +4130,7 @@
       <c r="N76" s="7"/>
       <c r="O76" s="7"/>
       <c r="P76" s="7"/>
+      <c r="Q76" s="7"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -4048,6 +4168,11 @@
       <c r="N77" s="7"/>
       <c r="O77" s="7"/>
       <c r="P77" s="7"/>
+      <c r="Q77" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
@@ -4085,6 +4210,7 @@
       <c r="N78" s="7"/>
       <c r="O78" s="7"/>
       <c r="P78" s="7"/>
+      <c r="Q78" s="7"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -4127,6 +4253,7 @@
       <c r="N79" s="7"/>
       <c r="O79" s="7"/>
       <c r="P79" s="7"/>
+      <c r="Q79" s="7"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
@@ -4172,6 +4299,11 @@
       </c>
       <c r="O80" s="7"/>
       <c r="P80" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="Q80" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -4213,6 +4345,7 @@
       <c r="N81" s="7"/>
       <c r="O81" s="7"/>
       <c r="P81" s="7"/>
+      <c r="Q81" s="7"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
@@ -4250,6 +4383,7 @@
       <c r="N82" s="7"/>
       <c r="O82" s="7"/>
       <c r="P82" s="7"/>
+      <c r="Q82" s="7"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
@@ -4292,6 +4426,7 @@
       <c r="N83" s="7"/>
       <c r="O83" s="7"/>
       <c r="P83" s="7"/>
+      <c r="Q83" s="7"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
@@ -4329,6 +4464,7 @@
       <c r="N84" s="7"/>
       <c r="O84" s="7"/>
       <c r="P84" s="7"/>
+      <c r="Q84" s="7"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
@@ -4366,6 +4502,7 @@
       <c r="N85" s="7"/>
       <c r="O85" s="7"/>
       <c r="P85" s="7"/>
+      <c r="Q85" s="7"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
@@ -4408,6 +4545,7 @@
       <c r="N86" s="7"/>
       <c r="O86" s="7"/>
       <c r="P86" s="7"/>
+      <c r="Q86" s="7"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
@@ -4445,6 +4583,7 @@
       <c r="N87" s="7"/>
       <c r="O87" s="7"/>
       <c r="P87" s="7"/>
+      <c r="Q87" s="7"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
@@ -4482,6 +4621,7 @@
       <c r="N88" s="7"/>
       <c r="O88" s="7"/>
       <c r="P88" s="7"/>
+      <c r="Q88" s="7"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
@@ -4519,6 +4659,7 @@
       <c r="N89" s="7"/>
       <c r="O89" s="7"/>
       <c r="P89" s="7"/>
+      <c r="Q89" s="7"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
@@ -4585,6 +4726,7 @@
       </c>
       <c r="O90" s="7"/>
       <c r="P90" s="7"/>
+      <c r="Q90" s="7"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
@@ -4622,6 +4764,7 @@
       <c r="N91" s="7"/>
       <c r="O91" s="7"/>
       <c r="P91" s="7"/>
+      <c r="Q91" s="7"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
@@ -4691,6 +4834,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Q92" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
@@ -4761,6 +4909,11 @@
         </is>
       </c>
       <c r="P93" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="Q93" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -4807,6 +4960,7 @@
       <c r="N94" s="7"/>
       <c r="O94" s="7"/>
       <c r="P94" s="7"/>
+      <c r="Q94" s="7"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
@@ -4849,6 +5003,7 @@
       <c r="N95" s="7"/>
       <c r="O95" s="7"/>
       <c r="P95" s="7"/>
+      <c r="Q95" s="7"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
@@ -4910,6 +5065,7 @@
       </c>
       <c r="O96" s="7"/>
       <c r="P96" s="7"/>
+      <c r="Q96" s="7"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="inlineStr">
@@ -4947,6 +5103,7 @@
       <c r="N97" s="7"/>
       <c r="O97" s="7"/>
       <c r="P97" s="7"/>
+      <c r="Q97" s="7"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
@@ -4984,6 +5141,7 @@
       <c r="N98" s="7"/>
       <c r="O98" s="7"/>
       <c r="P98" s="7"/>
+      <c r="Q98" s="7"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
@@ -5021,6 +5179,7 @@
       <c r="N99" s="7"/>
       <c r="O99" s="7"/>
       <c r="P99" s="7"/>
+      <c r="Q99" s="7"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
@@ -5067,6 +5226,7 @@
         </is>
       </c>
       <c r="P100" s="7"/>
+      <c r="Q100" s="7"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
@@ -5104,6 +5264,7 @@
       <c r="N101" s="7"/>
       <c r="O101" s="7"/>
       <c r="P101" s="7"/>
+      <c r="Q101" s="7"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
@@ -5141,6 +5302,7 @@
       <c r="N102" s="7"/>
       <c r="O102" s="7"/>
       <c r="P102" s="7"/>
+      <c r="Q102" s="7"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="inlineStr">
@@ -5178,6 +5340,7 @@
       <c r="N103" s="7"/>
       <c r="O103" s="7"/>
       <c r="P103" s="7"/>
+      <c r="Q103" s="7"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="inlineStr">
@@ -5220,6 +5383,7 @@
       <c r="N104" s="7"/>
       <c r="O104" s="7"/>
       <c r="P104" s="7"/>
+      <c r="Q104" s="7"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
@@ -5257,6 +5421,7 @@
       <c r="N105" s="7"/>
       <c r="O105" s="7"/>
       <c r="P105" s="7"/>
+      <c r="Q105" s="7"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
@@ -5294,6 +5459,7 @@
       <c r="N106" s="7"/>
       <c r="O106" s="7"/>
       <c r="P106" s="7"/>
+      <c r="Q106" s="7"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
@@ -5331,6 +5497,7 @@
       <c r="N107" s="7"/>
       <c r="O107" s="7"/>
       <c r="P107" s="7"/>
+      <c r="Q107" s="7"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
@@ -5372,6 +5539,7 @@
       <c r="N108" s="7"/>
       <c r="O108" s="7"/>
       <c r="P108" s="7"/>
+      <c r="Q108" s="7"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="inlineStr">
@@ -5418,6 +5586,7 @@
       <c r="N109" s="7"/>
       <c r="O109" s="7"/>
       <c r="P109" s="7"/>
+      <c r="Q109" s="7"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
@@ -5472,6 +5641,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Q110" s="7"/>
     </row>
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
@@ -5529,6 +5699,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Q111" s="7"/>
     </row>
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
@@ -5583,6 +5754,7 @@
       <c r="N112" s="7"/>
       <c r="O112" s="7"/>
       <c r="P112" s="7"/>
+      <c r="Q112" s="7"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
@@ -5629,6 +5801,7 @@
       <c r="N113" s="7"/>
       <c r="O113" s="7"/>
       <c r="P113" s="7"/>
+      <c r="Q113" s="7"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="inlineStr">
@@ -5691,6 +5864,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Q114" s="7"/>
     </row>
     <row r="115">
       <c r="A115" s="7" t="inlineStr">
@@ -5745,6 +5919,7 @@
       </c>
       <c r="O115" s="7"/>
       <c r="P115" s="7"/>
+      <c r="Q115" s="7"/>
     </row>
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
@@ -5799,6 +5974,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Q116" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
@@ -5853,6 +6033,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Q117" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
@@ -5907,6 +6092,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Q118" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="7" t="inlineStr">
@@ -5957,6 +6147,11 @@
       </c>
       <c r="O119" s="7"/>
       <c r="P119" s="7"/>
+      <c r="Q119" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="7" t="inlineStr">
@@ -6003,6 +6198,7 @@
       <c r="N120" s="7"/>
       <c r="O120" s="7"/>
       <c r="P120" s="7"/>
+      <c r="Q120" s="7"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="inlineStr">
@@ -6053,6 +6249,11 @@
       </c>
       <c r="O121" s="7"/>
       <c r="P121" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="Q121" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -6111,6 +6312,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Q122" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="7" t="inlineStr">
@@ -6157,6 +6363,7 @@
       </c>
       <c r="O123" s="7"/>
       <c r="P123" s="7"/>
+      <c r="Q123" s="7"/>
     </row>
     <row r="124">
       <c r="A124" s="7" t="inlineStr">
@@ -6207,6 +6414,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Q124" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="7" t="inlineStr">
@@ -6253,6 +6465,7 @@
         </is>
       </c>
       <c r="P125" s="7"/>
+      <c r="Q125" s="7"/>
     </row>
     <row r="126">
       <c r="A126" s="7" t="inlineStr">
@@ -6299,6 +6512,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Q126" s="7"/>
     </row>
     <row r="127">
       <c r="A127" s="7" t="inlineStr">
@@ -6345,6 +6559,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Q127" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="7" t="inlineStr">
@@ -6391,6 +6610,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Q128" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="7" t="inlineStr">
@@ -6433,6 +6657,58 @@
       <c r="N129" s="7"/>
       <c r="O129" s="7"/>
       <c r="P129" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="Q129" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_122</t>
+        </is>
+      </c>
+      <c r="B130" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">보드</t>
+        </is>
+      </c>
+      <c r="C130" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도전 층</t>
+        </is>
+      </c>
+      <c r="D130" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">탭 = 팝오버 보기</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도전 중 조립 보드에서 노드를 탭하면 팝오버가 뜨고(끌면 이동), 90도 돌리기·떼기·조합표·탄종은 흐려 안 눌리며 상태·물품·전력·붙은 모듈은 읽히는가? 도전을 나오면 팝오버가 닫히는가?</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#123 「보는 것은 막지 않는다」 · 파밍 층 그대로 (10-15 #148)</t>
+        </is>
+      </c>
+      <c r="G130" s="7"/>
+      <c r="H130" s="7"/>
+      <c r="I130" s="7"/>
+      <c r="J130" s="7"/>
+      <c r="K130" s="7"/>
+      <c r="L130" s="7"/>
+      <c r="M130" s="7"/>
+      <c r="N130" s="7"/>
+      <c r="O130" s="7"/>
+      <c r="P130" s="7"/>
+      <c r="Q130" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -6465,9 +6741,9 @@
     <mergeCell ref="B92:B99"/>
     <mergeCell ref="B100:B106"/>
     <mergeCell ref="B107:B111"/>
-    <mergeCell ref="G7:P7"/>
+    <mergeCell ref="G7:Q7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:P129">
+  <conditionalFormatting sqref="G9:Q130">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
QA R열(f710a05) — #149·#150·#151 재확인 Pass 4 · Fail 0 · CID_123~126 신설
사본 _261016 · 8128 · 576×1024 · 소리 0. S1 승리(남은 00:21) · S2 자연 승리(남은 00:13) ·
S3·S4 시간 초과(남은 16 · 23 = 하네스 미등장+생존과 같다) · 강화 단추 → 「강화 ×1.45 적용」 · 새로고침 유지 ·
S6 시간 초과. 빈 칸 = 안 지나감(바로가기 점프라 튜토리얼·T4 는 안 지나감).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -173,8 +173,9 @@
     <col min="15" max="15" width="12" customWidth="1"/>
     <col min="16" max="16" width="12" customWidth="1"/>
     <col min="17" max="17" width="12" customWidth="1"/>
-    <col min="18" max="18" width="11" customWidth="1"/>
+    <col min="18" max="18" width="12" customWidth="1"/>
     <col min="19" max="19" width="11" customWidth="1"/>
+    <col min="20" max="20" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -342,6 +343,11 @@
       <c r="Q6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">video-261014c 후보 · #148 도전 층 이동 모드: 끌면 이동 · 탭 = 팝오버(보기) · 팝오버 편집 행(90도 돌리기·떼기·조합표·탄종) 흐림 · 도전 층을 나오면 팝오버 닫음 ‖ 10-15 코드 세션 재확인(리포 8123 · dfbf6c8·9d3a11e · 576×1024 · 소리 0 · S1 도전 중 조립: 노드 탭 팝오버 · 편집 행 흐림 · 흐린 조합표 눌러도 그대로 · 팝오버 연 채 전투로 → 즉시 종료 → 다음 스테이지로 → 알림 · 탭 닫힘 → 조립: 팝오버 닫혀 있음 · 조립 모드 · 생산속도 모듈 붙여 T4 풀림) · 8127 갈아엎음 시각은 README · 빈 칸 = 안 지나감 · 관찰(판정 없음): 보드를 연 직후 첫 탭이 한 번 헛돎(브라우저 자동화 초점일 수 있음) · CID_122 새 항목</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">video-261016 후보 · #149 moduleMult 1.5 · 몬스터 hp 성장 절반 · #150 강화 단추(설정 판 · 재료 100 → ×1.45 · 계수 = 강화 표식) · #151 도전 몬스터 수·제한 시간 절반(60초 · S6 강적 18000) ‖ 10-16 코드 세션 재확인(사본 _261016 · 8128 · 576×1024 · 소리 0 · 처음부터 → 바로가기 S1 도전 50기 01:00 → 승리(남은 00:21) → 다음 스테이지로 S2 55기 → 승리(남은 00:13) → S3 패배 시간 초과 남은 16(하네스 = 미등장 11 + 생존 5 와 같다) → 다시 도전 · 도전 즉시 종료 → 다음 스테이지로 S4 파밍 → 설정 강화 단추 밝음 → 누름 → 「강화 ×1.45 적용」 흐림 → 새로고침 뒤 그대로 → S4 도전 패배 시간 초과 남은 23(하네스 = 미등장 22 + 생존 1) → S6 도전 패배 시간 초과(자동 · 합체 안 누름)) · 8128 갈아엎음 16:45:57(869c521 → f710a05) · 빈 칸 = 안 지나감 · 관찰(판정 없음): S3·S4 는 60초 안에 적이 다 안 나온다(마지막 스폰 예정 67.2초·76.8초) · 바로가기 점프라 튜토리얼·T4 는 안 지나감 · CID_123~126 새 항목</t>
         </is>
       </c>
     </row>
@@ -383,14 +389,15 @@
       <c r="O7" s="2"/>
       <c r="P7" s="2"/>
       <c r="Q7" s="2"/>
-      <c r="R7" s="2" t="inlineStr">
+      <c r="R7" s="2"/>
+      <c r="S7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">버전</t>
         </is>
       </c>
-      <c r="S7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">9d3a11e</t>
+      <c r="T7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">f710a05</t>
         </is>
       </c>
     </row>
@@ -470,11 +477,16 @@
       </c>
       <c r="R8" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">f710a05</t>
+        </is>
+      </c>
+      <c r="S8" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">PASSrate</t>
         </is>
       </c>
-      <c r="S8" s="7">
-        <f>COUNTIF(Q9:Q130,"Pass")</f>
+      <c r="T8" s="7">
+        <f>COUNTIF(R9:R134,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -555,13 +567,14 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="R9" s="2" t="inlineStr">
+      <c r="R9" s="7"/>
+      <c r="S9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FAILrate</t>
         </is>
       </c>
-      <c r="S9" s="7">
-        <f>COUNTIF(Q9:Q130,"Fail")+COUNTIF(Q9:Q130,"Broken")</f>
+      <c r="T9" s="7">
+        <f>COUNTIF(R9:R134,"Fail")+COUNTIF(R9:R134,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -606,13 +619,14 @@
       <c r="O10" s="7"/>
       <c r="P10" s="7"/>
       <c r="Q10" s="7"/>
-      <c r="R10" s="2" t="inlineStr">
+      <c r="R10" s="7"/>
+      <c r="S10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">N/A</t>
         </is>
       </c>
-      <c r="S10" s="7">
-        <f>COUNTIF(Q9:Q130,"N/A")</f>
+      <c r="T10" s="7">
+        <f>COUNTIF(R9:R134,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -657,13 +671,14 @@
       <c r="O11" s="7"/>
       <c r="P11" s="7"/>
       <c r="Q11" s="7"/>
-      <c r="R11" s="2" t="inlineStr">
+      <c r="R11" s="7"/>
+      <c r="S11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">전체 개수</t>
         </is>
       </c>
-      <c r="S11" s="7">
-        <v>122</v>
+      <c r="T11" s="7">
+        <v>126</v>
       </c>
     </row>
     <row r="12">
@@ -708,13 +723,14 @@
       <c r="O12" s="7"/>
       <c r="P12" s="7"/>
       <c r="Q12" s="7"/>
-      <c r="R12" s="2" t="inlineStr">
+      <c r="R12" s="7"/>
+      <c r="S12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">진행율</t>
         </is>
       </c>
-      <c r="S12" s="7">
-        <f>TEXT((COUNTA(Q9:Q130))/122,"0.00%")</f>
+      <c r="T12" s="7">
+        <f>TEXT((COUNTA(R9:R134))/126,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -763,6 +779,7 @@
       <c r="O13" s="7"/>
       <c r="P13" s="7"/>
       <c r="Q13" s="7"/>
+      <c r="R13" s="7"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -801,6 +818,7 @@
       <c r="O14" s="7"/>
       <c r="P14" s="7"/>
       <c r="Q14" s="7"/>
+      <c r="R14" s="7"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -875,6 +893,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="R15" s="7"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -949,6 +968,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="R16" s="7"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -1028,6 +1048,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="R17" s="7"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -1071,6 +1092,7 @@
       <c r="O18" s="7"/>
       <c r="P18" s="7"/>
       <c r="Q18" s="7"/>
+      <c r="R18" s="7"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -1109,6 +1131,7 @@
       <c r="O19" s="7"/>
       <c r="P19" s="7"/>
       <c r="Q19" s="7"/>
+      <c r="R19" s="7"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1147,6 +1170,7 @@
       <c r="O20" s="7"/>
       <c r="P20" s="7"/>
       <c r="Q20" s="7"/>
+      <c r="R20" s="7"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1221,6 +1245,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="R21" s="7"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1288,6 +1313,7 @@
       <c r="O22" s="7"/>
       <c r="P22" s="7"/>
       <c r="Q22" s="7"/>
+      <c r="R22" s="7"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -1334,6 +1360,7 @@
         </is>
       </c>
       <c r="Q23" s="7"/>
+      <c r="R23" s="7"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -1372,6 +1399,7 @@
       <c r="O24" s="7"/>
       <c r="P24" s="7"/>
       <c r="Q24" s="7"/>
+      <c r="R24" s="7"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -1410,6 +1438,7 @@
       <c r="O25" s="7"/>
       <c r="P25" s="7"/>
       <c r="Q25" s="7"/>
+      <c r="R25" s="7"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -1477,6 +1506,7 @@
         </is>
       </c>
       <c r="Q26" s="7"/>
+      <c r="R26" s="7"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -1519,6 +1549,7 @@
       <c r="O27" s="7"/>
       <c r="P27" s="7"/>
       <c r="Q27" s="7"/>
+      <c r="R27" s="7"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -1570,6 +1601,7 @@
       <c r="O28" s="7"/>
       <c r="P28" s="7"/>
       <c r="Q28" s="7"/>
+      <c r="R28" s="7"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -1616,6 +1648,7 @@
       <c r="O29" s="7"/>
       <c r="P29" s="7"/>
       <c r="Q29" s="7"/>
+      <c r="R29" s="7"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -1686,6 +1719,7 @@
         </is>
       </c>
       <c r="Q30" s="7"/>
+      <c r="R30" s="7"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -1761,6 +1795,7 @@
         </is>
       </c>
       <c r="Q31" s="7"/>
+      <c r="R31" s="7"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -1823,6 +1858,7 @@
       <c r="O32" s="7"/>
       <c r="P32" s="7"/>
       <c r="Q32" s="7"/>
+      <c r="R32" s="7"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -1893,6 +1929,7 @@
         </is>
       </c>
       <c r="Q33" s="7"/>
+      <c r="R33" s="7"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -1963,6 +2000,7 @@
         </is>
       </c>
       <c r="Q34" s="7"/>
+      <c r="R34" s="7"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -2038,6 +2076,7 @@
         </is>
       </c>
       <c r="Q35" s="7"/>
+      <c r="R35" s="7"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -2092,6 +2131,7 @@
       <c r="O36" s="7"/>
       <c r="P36" s="7"/>
       <c r="Q36" s="7"/>
+      <c r="R36" s="7"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -2130,6 +2170,7 @@
       <c r="O37" s="7"/>
       <c r="P37" s="7"/>
       <c r="Q37" s="7"/>
+      <c r="R37" s="7"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -2189,6 +2230,7 @@
       <c r="O38" s="7"/>
       <c r="P38" s="7"/>
       <c r="Q38" s="7"/>
+      <c r="R38" s="7"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -2259,6 +2301,7 @@
         </is>
       </c>
       <c r="Q39" s="7"/>
+      <c r="R39" s="7"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -2330,6 +2373,7 @@
         </is>
       </c>
       <c r="Q40" s="7"/>
+      <c r="R40" s="7"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -2396,6 +2440,7 @@
         </is>
       </c>
       <c r="Q41" s="7"/>
+      <c r="R41" s="7"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -2446,6 +2491,7 @@
       <c r="O42" s="7"/>
       <c r="P42" s="7"/>
       <c r="Q42" s="7"/>
+      <c r="R42" s="7"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -2516,6 +2562,7 @@
         </is>
       </c>
       <c r="Q43" s="7"/>
+      <c r="R43" s="7"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -2559,6 +2606,7 @@
       <c r="O44" s="7"/>
       <c r="P44" s="7"/>
       <c r="Q44" s="7"/>
+      <c r="R44" s="7"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -2625,6 +2673,7 @@
       </c>
       <c r="P45" s="7"/>
       <c r="Q45" s="7"/>
+      <c r="R45" s="7"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -2691,6 +2740,7 @@
       </c>
       <c r="P46" s="7"/>
       <c r="Q46" s="7"/>
+      <c r="R46" s="7"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -2734,6 +2784,7 @@
       <c r="O47" s="7"/>
       <c r="P47" s="7"/>
       <c r="Q47" s="7"/>
+      <c r="R47" s="7"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -2772,6 +2823,7 @@
       <c r="O48" s="7"/>
       <c r="P48" s="7"/>
       <c r="Q48" s="7"/>
+      <c r="R48" s="7"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -2810,6 +2862,7 @@
       <c r="O49" s="7"/>
       <c r="P49" s="7"/>
       <c r="Q49" s="7"/>
+      <c r="R49" s="7"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -2872,6 +2925,7 @@
       <c r="O50" s="7"/>
       <c r="P50" s="7"/>
       <c r="Q50" s="7"/>
+      <c r="R50" s="7"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -2934,6 +2988,7 @@
       <c r="O51" s="7"/>
       <c r="P51" s="7"/>
       <c r="Q51" s="7"/>
+      <c r="R51" s="7"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -2977,6 +3032,7 @@
       <c r="O52" s="7"/>
       <c r="P52" s="7"/>
       <c r="Q52" s="7"/>
+      <c r="R52" s="7"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -3020,6 +3076,7 @@
       <c r="O53" s="7"/>
       <c r="P53" s="7"/>
       <c r="Q53" s="7"/>
+      <c r="R53" s="7"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -3058,6 +3115,7 @@
       <c r="O54" s="7"/>
       <c r="P54" s="7"/>
       <c r="Q54" s="7"/>
+      <c r="R54" s="7"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -3132,6 +3190,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="R55" s="7"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -3186,6 +3245,7 @@
       <c r="O56" s="7"/>
       <c r="P56" s="7"/>
       <c r="Q56" s="7"/>
+      <c r="R56" s="7"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -3249,6 +3309,7 @@
       <c r="O57" s="7"/>
       <c r="P57" s="7"/>
       <c r="Q57" s="7"/>
+      <c r="R57" s="7"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -3320,6 +3381,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="R58" s="7"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -3358,6 +3420,7 @@
       <c r="O59" s="7"/>
       <c r="P59" s="7"/>
       <c r="Q59" s="7"/>
+      <c r="R59" s="7"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -3396,6 +3459,7 @@
       <c r="O60" s="7"/>
       <c r="P60" s="7"/>
       <c r="Q60" s="7"/>
+      <c r="R60" s="7"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -3446,6 +3510,7 @@
       <c r="O61" s="7"/>
       <c r="P61" s="7"/>
       <c r="Q61" s="7"/>
+      <c r="R61" s="7"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -3504,6 +3569,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="R62" s="7"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -3554,6 +3620,7 @@
       <c r="O63" s="7"/>
       <c r="P63" s="7"/>
       <c r="Q63" s="7"/>
+      <c r="R63" s="7"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -3592,6 +3659,7 @@
       <c r="O64" s="7"/>
       <c r="P64" s="7"/>
       <c r="Q64" s="7"/>
+      <c r="R64" s="7"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -3635,6 +3703,7 @@
       <c r="O65" s="7"/>
       <c r="P65" s="7"/>
       <c r="Q65" s="7"/>
+      <c r="R65" s="7"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
@@ -3685,6 +3754,7 @@
       <c r="O66" s="7"/>
       <c r="P66" s="7"/>
       <c r="Q66" s="7"/>
+      <c r="R66" s="7"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -3723,6 +3793,7 @@
       <c r="O67" s="7"/>
       <c r="P67" s="7"/>
       <c r="Q67" s="7"/>
+      <c r="R67" s="7"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
@@ -3765,6 +3836,7 @@
       <c r="O68" s="7"/>
       <c r="P68" s="7"/>
       <c r="Q68" s="7"/>
+      <c r="R68" s="7"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -3839,6 +3911,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="R69" s="7"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
@@ -3877,6 +3950,7 @@
       <c r="O70" s="7"/>
       <c r="P70" s="7"/>
       <c r="Q70" s="7"/>
+      <c r="R70" s="7"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -3920,6 +3994,7 @@
       <c r="O71" s="7"/>
       <c r="P71" s="7"/>
       <c r="Q71" s="7"/>
+      <c r="R71" s="7"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
@@ -3974,6 +4049,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="R72" s="7"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
@@ -4017,6 +4093,7 @@
       <c r="O73" s="7"/>
       <c r="P73" s="7"/>
       <c r="Q73" s="7"/>
+      <c r="R73" s="7"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -4055,6 +4132,7 @@
       <c r="O74" s="7"/>
       <c r="P74" s="7"/>
       <c r="Q74" s="7"/>
+      <c r="R74" s="7"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -4093,6 +4171,7 @@
       <c r="O75" s="7"/>
       <c r="P75" s="7"/>
       <c r="Q75" s="7"/>
+      <c r="R75" s="7"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -4131,6 +4210,7 @@
       <c r="O76" s="7"/>
       <c r="P76" s="7"/>
       <c r="Q76" s="7"/>
+      <c r="R76" s="7"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -4173,6 +4253,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="R77" s="7"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
@@ -4211,6 +4292,7 @@
       <c r="O78" s="7"/>
       <c r="P78" s="7"/>
       <c r="Q78" s="7"/>
+      <c r="R78" s="7"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -4254,6 +4336,7 @@
       <c r="O79" s="7"/>
       <c r="P79" s="7"/>
       <c r="Q79" s="7"/>
+      <c r="R79" s="7"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
@@ -4308,6 +4391,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="R80" s="7"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
@@ -4346,6 +4430,7 @@
       <c r="O81" s="7"/>
       <c r="P81" s="7"/>
       <c r="Q81" s="7"/>
+      <c r="R81" s="7"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
@@ -4384,6 +4469,7 @@
       <c r="O82" s="7"/>
       <c r="P82" s="7"/>
       <c r="Q82" s="7"/>
+      <c r="R82" s="7"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
@@ -4427,6 +4513,7 @@
       <c r="O83" s="7"/>
       <c r="P83" s="7"/>
       <c r="Q83" s="7"/>
+      <c r="R83" s="7"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
@@ -4465,6 +4552,7 @@
       <c r="O84" s="7"/>
       <c r="P84" s="7"/>
       <c r="Q84" s="7"/>
+      <c r="R84" s="7"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
@@ -4503,6 +4591,7 @@
       <c r="O85" s="7"/>
       <c r="P85" s="7"/>
       <c r="Q85" s="7"/>
+      <c r="R85" s="7"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
@@ -4546,6 +4635,7 @@
       <c r="O86" s="7"/>
       <c r="P86" s="7"/>
       <c r="Q86" s="7"/>
+      <c r="R86" s="7"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
@@ -4584,6 +4674,7 @@
       <c r="O87" s="7"/>
       <c r="P87" s="7"/>
       <c r="Q87" s="7"/>
+      <c r="R87" s="7"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
@@ -4622,6 +4713,7 @@
       <c r="O88" s="7"/>
       <c r="P88" s="7"/>
       <c r="Q88" s="7"/>
+      <c r="R88" s="7"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
@@ -4660,6 +4752,7 @@
       <c r="O89" s="7"/>
       <c r="P89" s="7"/>
       <c r="Q89" s="7"/>
+      <c r="R89" s="7"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
@@ -4727,6 +4820,7 @@
       <c r="O90" s="7"/>
       <c r="P90" s="7"/>
       <c r="Q90" s="7"/>
+      <c r="R90" s="7"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
@@ -4765,6 +4859,7 @@
       <c r="O91" s="7"/>
       <c r="P91" s="7"/>
       <c r="Q91" s="7"/>
+      <c r="R91" s="7"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
@@ -4839,6 +4934,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="R92" s="7"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
@@ -4918,6 +5014,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="R93" s="7"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
@@ -4961,6 +5058,7 @@
       <c r="O94" s="7"/>
       <c r="P94" s="7"/>
       <c r="Q94" s="7"/>
+      <c r="R94" s="7"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
@@ -5004,6 +5102,7 @@
       <c r="O95" s="7"/>
       <c r="P95" s="7"/>
       <c r="Q95" s="7"/>
+      <c r="R95" s="7"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
@@ -5066,6 +5165,7 @@
       <c r="O96" s="7"/>
       <c r="P96" s="7"/>
       <c r="Q96" s="7"/>
+      <c r="R96" s="7"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="inlineStr">
@@ -5104,6 +5204,7 @@
       <c r="O97" s="7"/>
       <c r="P97" s="7"/>
       <c r="Q97" s="7"/>
+      <c r="R97" s="7"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
@@ -5142,6 +5243,7 @@
       <c r="O98" s="7"/>
       <c r="P98" s="7"/>
       <c r="Q98" s="7"/>
+      <c r="R98" s="7"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
@@ -5180,6 +5282,7 @@
       <c r="O99" s="7"/>
       <c r="P99" s="7"/>
       <c r="Q99" s="7"/>
+      <c r="R99" s="7"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
@@ -5227,6 +5330,7 @@
       </c>
       <c r="P100" s="7"/>
       <c r="Q100" s="7"/>
+      <c r="R100" s="7"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
@@ -5265,6 +5369,7 @@
       <c r="O101" s="7"/>
       <c r="P101" s="7"/>
       <c r="Q101" s="7"/>
+      <c r="R101" s="7"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
@@ -5303,6 +5408,7 @@
       <c r="O102" s="7"/>
       <c r="P102" s="7"/>
       <c r="Q102" s="7"/>
+      <c r="R102" s="7"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="inlineStr">
@@ -5341,6 +5447,7 @@
       <c r="O103" s="7"/>
       <c r="P103" s="7"/>
       <c r="Q103" s="7"/>
+      <c r="R103" s="7"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="inlineStr">
@@ -5384,6 +5491,7 @@
       <c r="O104" s="7"/>
       <c r="P104" s="7"/>
       <c r="Q104" s="7"/>
+      <c r="R104" s="7"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
@@ -5422,6 +5530,7 @@
       <c r="O105" s="7"/>
       <c r="P105" s="7"/>
       <c r="Q105" s="7"/>
+      <c r="R105" s="7"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
@@ -5460,6 +5569,7 @@
       <c r="O106" s="7"/>
       <c r="P106" s="7"/>
       <c r="Q106" s="7"/>
+      <c r="R106" s="7"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
@@ -5498,6 +5608,7 @@
       <c r="O107" s="7"/>
       <c r="P107" s="7"/>
       <c r="Q107" s="7"/>
+      <c r="R107" s="7"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
@@ -5540,6 +5651,7 @@
       <c r="O108" s="7"/>
       <c r="P108" s="7"/>
       <c r="Q108" s="7"/>
+      <c r="R108" s="7"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="inlineStr">
@@ -5587,6 +5699,7 @@
       <c r="O109" s="7"/>
       <c r="P109" s="7"/>
       <c r="Q109" s="7"/>
+      <c r="R109" s="7"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
@@ -5642,6 +5755,7 @@
         </is>
       </c>
       <c r="Q110" s="7"/>
+      <c r="R110" s="7"/>
     </row>
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
@@ -5700,6 +5814,7 @@
         </is>
       </c>
       <c r="Q111" s="7"/>
+      <c r="R111" s="7"/>
     </row>
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
@@ -5755,6 +5870,7 @@
       <c r="O112" s="7"/>
       <c r="P112" s="7"/>
       <c r="Q112" s="7"/>
+      <c r="R112" s="7"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
@@ -5802,6 +5918,7 @@
       <c r="O113" s="7"/>
       <c r="P113" s="7"/>
       <c r="Q113" s="7"/>
+      <c r="R113" s="7"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="inlineStr">
@@ -5865,6 +5982,7 @@
         </is>
       </c>
       <c r="Q114" s="7"/>
+      <c r="R114" s="7"/>
     </row>
     <row r="115">
       <c r="A115" s="7" t="inlineStr">
@@ -5920,6 +6038,7 @@
       <c r="O115" s="7"/>
       <c r="P115" s="7"/>
       <c r="Q115" s="7"/>
+      <c r="R115" s="7"/>
     </row>
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
@@ -5979,6 +6098,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="R116" s="7"/>
     </row>
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
@@ -6038,6 +6158,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="R117" s="7"/>
     </row>
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
@@ -6097,6 +6218,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="R118" s="7"/>
     </row>
     <row r="119">
       <c r="A119" s="7" t="inlineStr">
@@ -6152,6 +6274,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="R119" s="7"/>
     </row>
     <row r="120">
       <c r="A120" s="7" t="inlineStr">
@@ -6199,6 +6322,7 @@
       <c r="O120" s="7"/>
       <c r="P120" s="7"/>
       <c r="Q120" s="7"/>
+      <c r="R120" s="7"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="inlineStr">
@@ -6258,6 +6382,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="R121" s="7"/>
     </row>
     <row r="122">
       <c r="A122" s="7" t="inlineStr">
@@ -6317,6 +6442,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="R122" s="7"/>
     </row>
     <row r="123">
       <c r="A123" s="7" t="inlineStr">
@@ -6364,6 +6490,7 @@
       <c r="O123" s="7"/>
       <c r="P123" s="7"/>
       <c r="Q123" s="7"/>
+      <c r="R123" s="7"/>
     </row>
     <row r="124">
       <c r="A124" s="7" t="inlineStr">
@@ -6419,6 +6546,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="R124" s="7"/>
     </row>
     <row r="125">
       <c r="A125" s="7" t="inlineStr">
@@ -6466,6 +6594,7 @@
       </c>
       <c r="P125" s="7"/>
       <c r="Q125" s="7"/>
+      <c r="R125" s="7"/>
     </row>
     <row r="126">
       <c r="A126" s="7" t="inlineStr">
@@ -6513,6 +6642,7 @@
         </is>
       </c>
       <c r="Q126" s="7"/>
+      <c r="R126" s="7"/>
     </row>
     <row r="127">
       <c r="A127" s="7" t="inlineStr">
@@ -6564,6 +6694,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="R127" s="7"/>
     </row>
     <row r="128">
       <c r="A128" s="7" t="inlineStr">
@@ -6615,6 +6746,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="R128" s="7"/>
     </row>
     <row r="129">
       <c r="A129" s="7" t="inlineStr">
@@ -6666,6 +6798,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="R129" s="7"/>
     </row>
     <row r="130">
       <c r="A130" s="7" t="inlineStr">
@@ -6709,6 +6842,199 @@
       <c r="O130" s="7"/>
       <c r="P130" s="7"/>
       <c r="Q130" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="R130" s="7"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_123</t>
+        </is>
+      </c>
+      <c r="B131" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">강화</t>
+        </is>
+      </c>
+      <c r="C131" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">설정 판</t>
+        </is>
+      </c>
+      <c r="D131" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">강화 단추</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">재료 100 이상이면 설정 판 「강화 (재료 전부 투입)」이 밝고, 누르면 「강화 ×1.45 적용」으로 바뀌어 흐리며, 새로고침 뒤에도 그대로인가? 100 미만이면 흐린가?</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">자리 = 설정 판(구현 판단) · 문구 가정 · 처음부터면 꺼짐 (10-16 #150)</t>
+        </is>
+      </c>
+      <c r="G131" s="7"/>
+      <c r="H131" s="7"/>
+      <c r="I131" s="7"/>
+      <c r="J131" s="7"/>
+      <c r="K131" s="7"/>
+      <c r="L131" s="7"/>
+      <c r="M131" s="7"/>
+      <c r="N131" s="7"/>
+      <c r="O131" s="7"/>
+      <c r="P131" s="7"/>
+      <c r="Q131" s="7"/>
+      <c r="R131" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_124</t>
+        </is>
+      </c>
+      <c r="B132" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C132" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2</t>
+        </is>
+      </c>
+      <c r="D132" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">자연 통과</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">시작 보드(마운트 강화 없음)로 S2 도전을 그대로 두면 제한 시간 안에 전멸 승리하는가?</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#149 피해 ×1.5 · hp 성장 절반 (10-16)</t>
+        </is>
+      </c>
+      <c r="G132" s="7"/>
+      <c r="H132" s="7"/>
+      <c r="I132" s="7"/>
+      <c r="J132" s="7"/>
+      <c r="K132" s="7"/>
+      <c r="L132" s="7"/>
+      <c r="M132" s="7"/>
+      <c r="N132" s="7"/>
+      <c r="O132" s="7"/>
+      <c r="P132" s="7"/>
+      <c r="Q132" s="7"/>
+      <c r="R132" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_125</t>
+        </is>
+      </c>
+      <c r="B133" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">경제</t>
+        </is>
+      </c>
+      <c r="C133" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">강화 재료</t>
+        </is>
+      </c>
+      <c r="D133" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">적립</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S1·S2·S3 를 처음 통과할 때마다 강화 재료가 쌓여 셋 뒤 100 이 되는가?(30+33+37 · 다시 통과하면 안 쌓임)</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">단추가 S1·S2 뒤 흐림 · S3 뒤 밝음으로 간접 확인 (10-16)</t>
+        </is>
+      </c>
+      <c r="G133" s="7"/>
+      <c r="H133" s="7"/>
+      <c r="I133" s="7"/>
+      <c r="J133" s="7"/>
+      <c r="K133" s="7"/>
+      <c r="L133" s="7"/>
+      <c r="M133" s="7"/>
+      <c r="N133" s="7"/>
+      <c r="O133" s="7"/>
+      <c r="P133" s="7"/>
+      <c r="Q133" s="7"/>
+      <c r="R133" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_126</t>
+        </is>
+      </c>
+      <c r="B134" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C134" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도전</t>
+        </is>
+      </c>
+      <c r="D134" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">60초</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도전에 들어가면 「남은 시간 01:00」에서 줄고, 몬스터 수가 절반(S1 50 · S2 55 · S3 87 · S4 98 · S5 7 · S6 1)인가?</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#151 (10-16) · 시작 표시 01:00</t>
+        </is>
+      </c>
+      <c r="G134" s="7"/>
+      <c r="H134" s="7"/>
+      <c r="I134" s="7"/>
+      <c r="J134" s="7"/>
+      <c r="K134" s="7"/>
+      <c r="L134" s="7"/>
+      <c r="M134" s="7"/>
+      <c r="N134" s="7"/>
+      <c r="O134" s="7"/>
+      <c r="P134" s="7"/>
+      <c r="Q134" s="7"/>
+      <c r="R134" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -6741,9 +7067,9 @@
     <mergeCell ref="B92:B99"/>
     <mergeCell ref="B100:B106"/>
     <mergeCell ref="B107:B111"/>
-    <mergeCell ref="G7:Q7"/>
+    <mergeCell ref="G7:R7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:Q130">
+  <conditionalFormatting sqref="G9:R134">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
QA S열(08ec1c7) — #152 재확인 Pass 4 · Fail 0 · CID_127~128 신설
8128 처음부터 → S1 승리(남은 00:27) → S2 승리(남은 00:02 · HP 약 875) · 8123 S4 로봇 파괴 약 13초 · 98기 동시 브라우저 약 83/초.
CID_128 의 「멀어져도 계속 쫓음」은 시험(MonsterAggroTests)으로 보고 화면은 「제자리 → 깸」까지 봤다.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -174,8 +174,9 @@
     <col min="16" max="16" width="12" customWidth="1"/>
     <col min="17" max="17" width="12" customWidth="1"/>
     <col min="18" max="18" width="12" customWidth="1"/>
-    <col min="19" max="19" width="11" customWidth="1"/>
+    <col min="19" max="19" width="12" customWidth="1"/>
     <col min="20" max="20" width="11" customWidth="1"/>
+    <col min="21" max="21" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -348,6 +349,11 @@
       <c r="R6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">video-261016 후보 · #149 moduleMult 1.5 · 몬스터 hp 성장 절반 · #150 강화 단추(설정 판 · 재료 100 → ×1.45 · 계수 = 강화 표식) · #151 도전 몬스터 수·제한 시간 절반(60초 · S6 강적 18000) ‖ 10-16 코드 세션 재확인(사본 _261016 · 8128 · 576×1024 · 소리 0 · 처음부터 → 바로가기 S1 도전 50기 01:00 → 승리(남은 00:21) → 다음 스테이지로 S2 55기 → 승리(남은 00:13) → S3 패배 시간 초과 남은 16(하네스 = 미등장 11 + 생존 5 와 같다) → 다시 도전 · 도전 즉시 종료 → 다음 스테이지로 S4 파밍 → 설정 강화 단추 밝음 → 누름 → 「강화 ×1.45 적용」 흐림 → 새로고침 뒤 그대로 → S4 도전 패배 시간 초과 남은 23(하네스 = 미등장 22 + 생존 1) → S6 도전 패배 시간 초과(자동 · 합체 안 누름)) · 8128 갈아엎음 16:45:57(869c521 → f710a05) · 빈 칸 = 안 지나감 · 관찰(판정 없음): S3·S4 는 60초 안에 적이 다 안 나온다(마지막 스폰 예정 67.2초·76.8초) · 바로가기 점프라 튜토리얼·T4 는 안 지나감 · CID_123~126 새 항목</t>
+        </is>
+      </c>
+      <c r="S6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">video-261016 후보 · #152 도전 층 전원 스폰 · 몬스터 탐색 범위 9.2(밖이면 제자리 · 들면 깨어 끝까지 추격) ‖ 10-16 코드 세션 재확인(리포 8123 S4 + 사본 _261016 · 8128 · 576×1024 · 소리 0 · 처음부터 → 바로가기 S1 도전 50기 전원 서고 제자리 → 승리(남은 00:27 · HP 가득) → 다음 스테이지로 S2 → 승리(남은 00:02 · HP 약 875) · 8123 S4 도전 98기 → 로봇 파괴 약 13초(남은 93 · 바로가기라 마운트 빈손) · 브라우저 프레임 약 83/초(rAF · 98기 동시)) · 8128 갈아엎음 17:18:45(f710a05 → 08ec1c7) · 빈 칸 = 안 지나감 · 관찰(판정 없음): S3·S4 는 깨어 있는 적이 한 번에 19~26 기라 로봇이 버티지 못한다(하네스) · CID_127~128 새 항목</t>
         </is>
       </c>
     </row>
@@ -390,14 +396,15 @@
       <c r="P7" s="2"/>
       <c r="Q7" s="2"/>
       <c r="R7" s="2"/>
-      <c r="S7" s="2" t="inlineStr">
+      <c r="S7" s="2"/>
+      <c r="T7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">버전</t>
         </is>
       </c>
-      <c r="T7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">f710a05</t>
+      <c r="U7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">08ec1c7</t>
         </is>
       </c>
     </row>
@@ -482,11 +489,16 @@
       </c>
       <c r="S8" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">08ec1c7</t>
+        </is>
+      </c>
+      <c r="T8" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">PASSrate</t>
         </is>
       </c>
-      <c r="T8" s="7">
-        <f>COUNTIF(R9:R134,"Pass")</f>
+      <c r="U8" s="7">
+        <f>COUNTIF(S9:S136,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -568,13 +580,14 @@
         </is>
       </c>
       <c r="R9" s="7"/>
-      <c r="S9" s="2" t="inlineStr">
+      <c r="S9" s="7"/>
+      <c r="T9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FAILrate</t>
         </is>
       </c>
-      <c r="T9" s="7">
-        <f>COUNTIF(R9:R134,"Fail")+COUNTIF(R9:R134,"Broken")</f>
+      <c r="U9" s="7">
+        <f>COUNTIF(S9:S136,"Fail")+COUNTIF(S9:S136,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -620,13 +633,14 @@
       <c r="P10" s="7"/>
       <c r="Q10" s="7"/>
       <c r="R10" s="7"/>
-      <c r="S10" s="2" t="inlineStr">
+      <c r="S10" s="7"/>
+      <c r="T10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">N/A</t>
         </is>
       </c>
-      <c r="T10" s="7">
-        <f>COUNTIF(R9:R134,"N/A")</f>
+      <c r="U10" s="7">
+        <f>COUNTIF(S9:S136,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -672,13 +686,14 @@
       <c r="P11" s="7"/>
       <c r="Q11" s="7"/>
       <c r="R11" s="7"/>
-      <c r="S11" s="2" t="inlineStr">
+      <c r="S11" s="7"/>
+      <c r="T11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">전체 개수</t>
         </is>
       </c>
-      <c r="T11" s="7">
-        <v>126</v>
+      <c r="U11" s="7">
+        <v>128</v>
       </c>
     </row>
     <row r="12">
@@ -724,13 +739,14 @@
       <c r="P12" s="7"/>
       <c r="Q12" s="7"/>
       <c r="R12" s="7"/>
-      <c r="S12" s="2" t="inlineStr">
+      <c r="S12" s="7"/>
+      <c r="T12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">진행율</t>
         </is>
       </c>
-      <c r="T12" s="7">
-        <f>TEXT((COUNTA(R9:R134))/126,"0.00%")</f>
+      <c r="U12" s="7">
+        <f>TEXT((COUNTA(S9:S136))/128,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -780,6 +796,7 @@
       <c r="P13" s="7"/>
       <c r="Q13" s="7"/>
       <c r="R13" s="7"/>
+      <c r="S13" s="7"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -819,6 +836,7 @@
       <c r="P14" s="7"/>
       <c r="Q14" s="7"/>
       <c r="R14" s="7"/>
+      <c r="S14" s="7"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -894,6 +912,7 @@
         </is>
       </c>
       <c r="R15" s="7"/>
+      <c r="S15" s="7"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -969,6 +988,7 @@
         </is>
       </c>
       <c r="R16" s="7"/>
+      <c r="S16" s="7"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -1049,6 +1069,7 @@
         </is>
       </c>
       <c r="R17" s="7"/>
+      <c r="S17" s="7"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -1093,6 +1114,7 @@
       <c r="P18" s="7"/>
       <c r="Q18" s="7"/>
       <c r="R18" s="7"/>
+      <c r="S18" s="7"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -1132,6 +1154,7 @@
       <c r="P19" s="7"/>
       <c r="Q19" s="7"/>
       <c r="R19" s="7"/>
+      <c r="S19" s="7"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1171,6 +1194,7 @@
       <c r="P20" s="7"/>
       <c r="Q20" s="7"/>
       <c r="R20" s="7"/>
+      <c r="S20" s="7"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1246,6 +1270,7 @@
         </is>
       </c>
       <c r="R21" s="7"/>
+      <c r="S21" s="7"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1314,6 +1339,7 @@
       <c r="P22" s="7"/>
       <c r="Q22" s="7"/>
       <c r="R22" s="7"/>
+      <c r="S22" s="7"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -1361,6 +1387,7 @@
       </c>
       <c r="Q23" s="7"/>
       <c r="R23" s="7"/>
+      <c r="S23" s="7"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -1400,6 +1427,7 @@
       <c r="P24" s="7"/>
       <c r="Q24" s="7"/>
       <c r="R24" s="7"/>
+      <c r="S24" s="7"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -1439,6 +1467,7 @@
       <c r="P25" s="7"/>
       <c r="Q25" s="7"/>
       <c r="R25" s="7"/>
+      <c r="S25" s="7"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -1507,6 +1536,7 @@
       </c>
       <c r="Q26" s="7"/>
       <c r="R26" s="7"/>
+      <c r="S26" s="7"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -1550,6 +1580,7 @@
       <c r="P27" s="7"/>
       <c r="Q27" s="7"/>
       <c r="R27" s="7"/>
+      <c r="S27" s="7"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -1602,6 +1633,7 @@
       <c r="P28" s="7"/>
       <c r="Q28" s="7"/>
       <c r="R28" s="7"/>
+      <c r="S28" s="7"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -1649,6 +1681,7 @@
       <c r="P29" s="7"/>
       <c r="Q29" s="7"/>
       <c r="R29" s="7"/>
+      <c r="S29" s="7"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -1720,6 +1753,7 @@
       </c>
       <c r="Q30" s="7"/>
       <c r="R30" s="7"/>
+      <c r="S30" s="7"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -1796,6 +1830,7 @@
       </c>
       <c r="Q31" s="7"/>
       <c r="R31" s="7"/>
+      <c r="S31" s="7"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -1859,6 +1894,7 @@
       <c r="P32" s="7"/>
       <c r="Q32" s="7"/>
       <c r="R32" s="7"/>
+      <c r="S32" s="7"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -1930,6 +1966,7 @@
       </c>
       <c r="Q33" s="7"/>
       <c r="R33" s="7"/>
+      <c r="S33" s="7"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -2001,6 +2038,7 @@
       </c>
       <c r="Q34" s="7"/>
       <c r="R34" s="7"/>
+      <c r="S34" s="7"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -2077,6 +2115,7 @@
       </c>
       <c r="Q35" s="7"/>
       <c r="R35" s="7"/>
+      <c r="S35" s="7"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -2132,6 +2171,7 @@
       <c r="P36" s="7"/>
       <c r="Q36" s="7"/>
       <c r="R36" s="7"/>
+      <c r="S36" s="7"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -2171,6 +2211,7 @@
       <c r="P37" s="7"/>
       <c r="Q37" s="7"/>
       <c r="R37" s="7"/>
+      <c r="S37" s="7"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -2231,6 +2272,7 @@
       <c r="P38" s="7"/>
       <c r="Q38" s="7"/>
       <c r="R38" s="7"/>
+      <c r="S38" s="7"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -2302,6 +2344,7 @@
       </c>
       <c r="Q39" s="7"/>
       <c r="R39" s="7"/>
+      <c r="S39" s="7"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -2374,6 +2417,7 @@
       </c>
       <c r="Q40" s="7"/>
       <c r="R40" s="7"/>
+      <c r="S40" s="7"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -2441,6 +2485,7 @@
       </c>
       <c r="Q41" s="7"/>
       <c r="R41" s="7"/>
+      <c r="S41" s="7"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -2492,6 +2537,7 @@
       <c r="P42" s="7"/>
       <c r="Q42" s="7"/>
       <c r="R42" s="7"/>
+      <c r="S42" s="7"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -2563,6 +2609,7 @@
       </c>
       <c r="Q43" s="7"/>
       <c r="R43" s="7"/>
+      <c r="S43" s="7"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -2607,6 +2654,7 @@
       <c r="P44" s="7"/>
       <c r="Q44" s="7"/>
       <c r="R44" s="7"/>
+      <c r="S44" s="7"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -2674,6 +2722,7 @@
       <c r="P45" s="7"/>
       <c r="Q45" s="7"/>
       <c r="R45" s="7"/>
+      <c r="S45" s="7"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -2741,6 +2790,7 @@
       <c r="P46" s="7"/>
       <c r="Q46" s="7"/>
       <c r="R46" s="7"/>
+      <c r="S46" s="7"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -2785,6 +2835,7 @@
       <c r="P47" s="7"/>
       <c r="Q47" s="7"/>
       <c r="R47" s="7"/>
+      <c r="S47" s="7"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -2824,6 +2875,7 @@
       <c r="P48" s="7"/>
       <c r="Q48" s="7"/>
       <c r="R48" s="7"/>
+      <c r="S48" s="7"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -2863,6 +2915,7 @@
       <c r="P49" s="7"/>
       <c r="Q49" s="7"/>
       <c r="R49" s="7"/>
+      <c r="S49" s="7"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -2926,6 +2979,7 @@
       <c r="P50" s="7"/>
       <c r="Q50" s="7"/>
       <c r="R50" s="7"/>
+      <c r="S50" s="7"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -2989,6 +3043,7 @@
       <c r="P51" s="7"/>
       <c r="Q51" s="7"/>
       <c r="R51" s="7"/>
+      <c r="S51" s="7"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -3033,6 +3088,7 @@
       <c r="P52" s="7"/>
       <c r="Q52" s="7"/>
       <c r="R52" s="7"/>
+      <c r="S52" s="7"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -3077,6 +3133,7 @@
       <c r="P53" s="7"/>
       <c r="Q53" s="7"/>
       <c r="R53" s="7"/>
+      <c r="S53" s="7"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -3116,6 +3173,7 @@
       <c r="P54" s="7"/>
       <c r="Q54" s="7"/>
       <c r="R54" s="7"/>
+      <c r="S54" s="7"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -3191,6 +3249,7 @@
         </is>
       </c>
       <c r="R55" s="7"/>
+      <c r="S55" s="7"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -3246,6 +3305,7 @@
       <c r="P56" s="7"/>
       <c r="Q56" s="7"/>
       <c r="R56" s="7"/>
+      <c r="S56" s="7"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -3310,6 +3370,7 @@
       <c r="P57" s="7"/>
       <c r="Q57" s="7"/>
       <c r="R57" s="7"/>
+      <c r="S57" s="7"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -3382,6 +3443,7 @@
         </is>
       </c>
       <c r="R58" s="7"/>
+      <c r="S58" s="7"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -3421,6 +3483,7 @@
       <c r="P59" s="7"/>
       <c r="Q59" s="7"/>
       <c r="R59" s="7"/>
+      <c r="S59" s="7"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -3460,6 +3523,7 @@
       <c r="P60" s="7"/>
       <c r="Q60" s="7"/>
       <c r="R60" s="7"/>
+      <c r="S60" s="7"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -3511,6 +3575,7 @@
       <c r="P61" s="7"/>
       <c r="Q61" s="7"/>
       <c r="R61" s="7"/>
+      <c r="S61" s="7"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -3570,6 +3635,7 @@
         </is>
       </c>
       <c r="R62" s="7"/>
+      <c r="S62" s="7"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -3621,6 +3687,7 @@
       <c r="P63" s="7"/>
       <c r="Q63" s="7"/>
       <c r="R63" s="7"/>
+      <c r="S63" s="7"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -3660,6 +3727,7 @@
       <c r="P64" s="7"/>
       <c r="Q64" s="7"/>
       <c r="R64" s="7"/>
+      <c r="S64" s="7"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -3704,6 +3772,7 @@
       <c r="P65" s="7"/>
       <c r="Q65" s="7"/>
       <c r="R65" s="7"/>
+      <c r="S65" s="7"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
@@ -3755,6 +3824,7 @@
       <c r="P66" s="7"/>
       <c r="Q66" s="7"/>
       <c r="R66" s="7"/>
+      <c r="S66" s="7"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -3794,6 +3864,7 @@
       <c r="P67" s="7"/>
       <c r="Q67" s="7"/>
       <c r="R67" s="7"/>
+      <c r="S67" s="7"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
@@ -3837,6 +3908,7 @@
       <c r="P68" s="7"/>
       <c r="Q68" s="7"/>
       <c r="R68" s="7"/>
+      <c r="S68" s="7"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -3912,6 +3984,7 @@
         </is>
       </c>
       <c r="R69" s="7"/>
+      <c r="S69" s="7"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
@@ -3951,6 +4024,7 @@
       <c r="P70" s="7"/>
       <c r="Q70" s="7"/>
       <c r="R70" s="7"/>
+      <c r="S70" s="7"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -3995,6 +4069,7 @@
       <c r="P71" s="7"/>
       <c r="Q71" s="7"/>
       <c r="R71" s="7"/>
+      <c r="S71" s="7"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
@@ -4050,6 +4125,7 @@
         </is>
       </c>
       <c r="R72" s="7"/>
+      <c r="S72" s="7"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
@@ -4094,6 +4170,7 @@
       <c r="P73" s="7"/>
       <c r="Q73" s="7"/>
       <c r="R73" s="7"/>
+      <c r="S73" s="7"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -4133,6 +4210,7 @@
       <c r="P74" s="7"/>
       <c r="Q74" s="7"/>
       <c r="R74" s="7"/>
+      <c r="S74" s="7"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -4172,6 +4250,7 @@
       <c r="P75" s="7"/>
       <c r="Q75" s="7"/>
       <c r="R75" s="7"/>
+      <c r="S75" s="7"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -4211,6 +4290,7 @@
       <c r="P76" s="7"/>
       <c r="Q76" s="7"/>
       <c r="R76" s="7"/>
+      <c r="S76" s="7"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -4254,6 +4334,7 @@
         </is>
       </c>
       <c r="R77" s="7"/>
+      <c r="S77" s="7"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
@@ -4293,6 +4374,7 @@
       <c r="P78" s="7"/>
       <c r="Q78" s="7"/>
       <c r="R78" s="7"/>
+      <c r="S78" s="7"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -4337,6 +4419,7 @@
       <c r="P79" s="7"/>
       <c r="Q79" s="7"/>
       <c r="R79" s="7"/>
+      <c r="S79" s="7"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
@@ -4392,6 +4475,7 @@
         </is>
       </c>
       <c r="R80" s="7"/>
+      <c r="S80" s="7"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
@@ -4431,6 +4515,7 @@
       <c r="P81" s="7"/>
       <c r="Q81" s="7"/>
       <c r="R81" s="7"/>
+      <c r="S81" s="7"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
@@ -4470,6 +4555,7 @@
       <c r="P82" s="7"/>
       <c r="Q82" s="7"/>
       <c r="R82" s="7"/>
+      <c r="S82" s="7"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
@@ -4514,6 +4600,7 @@
       <c r="P83" s="7"/>
       <c r="Q83" s="7"/>
       <c r="R83" s="7"/>
+      <c r="S83" s="7"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
@@ -4553,6 +4640,7 @@
       <c r="P84" s="7"/>
       <c r="Q84" s="7"/>
       <c r="R84" s="7"/>
+      <c r="S84" s="7"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
@@ -4592,6 +4680,7 @@
       <c r="P85" s="7"/>
       <c r="Q85" s="7"/>
       <c r="R85" s="7"/>
+      <c r="S85" s="7"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
@@ -4636,6 +4725,7 @@
       <c r="P86" s="7"/>
       <c r="Q86" s="7"/>
       <c r="R86" s="7"/>
+      <c r="S86" s="7"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
@@ -4675,6 +4765,7 @@
       <c r="P87" s="7"/>
       <c r="Q87" s="7"/>
       <c r="R87" s="7"/>
+      <c r="S87" s="7"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
@@ -4714,6 +4805,7 @@
       <c r="P88" s="7"/>
       <c r="Q88" s="7"/>
       <c r="R88" s="7"/>
+      <c r="S88" s="7"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
@@ -4753,6 +4845,7 @@
       <c r="P89" s="7"/>
       <c r="Q89" s="7"/>
       <c r="R89" s="7"/>
+      <c r="S89" s="7"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
@@ -4821,6 +4914,7 @@
       <c r="P90" s="7"/>
       <c r="Q90" s="7"/>
       <c r="R90" s="7"/>
+      <c r="S90" s="7"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
@@ -4860,6 +4954,7 @@
       <c r="P91" s="7"/>
       <c r="Q91" s="7"/>
       <c r="R91" s="7"/>
+      <c r="S91" s="7"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
@@ -4935,6 +5030,7 @@
         </is>
       </c>
       <c r="R92" s="7"/>
+      <c r="S92" s="7"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
@@ -5015,6 +5111,7 @@
         </is>
       </c>
       <c r="R93" s="7"/>
+      <c r="S93" s="7"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
@@ -5059,6 +5156,7 @@
       <c r="P94" s="7"/>
       <c r="Q94" s="7"/>
       <c r="R94" s="7"/>
+      <c r="S94" s="7"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
@@ -5103,6 +5201,7 @@
       <c r="P95" s="7"/>
       <c r="Q95" s="7"/>
       <c r="R95" s="7"/>
+      <c r="S95" s="7"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
@@ -5166,6 +5265,7 @@
       <c r="P96" s="7"/>
       <c r="Q96" s="7"/>
       <c r="R96" s="7"/>
+      <c r="S96" s="7"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="inlineStr">
@@ -5205,6 +5305,7 @@
       <c r="P97" s="7"/>
       <c r="Q97" s="7"/>
       <c r="R97" s="7"/>
+      <c r="S97" s="7"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
@@ -5244,6 +5345,7 @@
       <c r="P98" s="7"/>
       <c r="Q98" s="7"/>
       <c r="R98" s="7"/>
+      <c r="S98" s="7"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
@@ -5283,6 +5385,7 @@
       <c r="P99" s="7"/>
       <c r="Q99" s="7"/>
       <c r="R99" s="7"/>
+      <c r="S99" s="7"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
@@ -5331,6 +5434,7 @@
       <c r="P100" s="7"/>
       <c r="Q100" s="7"/>
       <c r="R100" s="7"/>
+      <c r="S100" s="7"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
@@ -5370,6 +5474,7 @@
       <c r="P101" s="7"/>
       <c r="Q101" s="7"/>
       <c r="R101" s="7"/>
+      <c r="S101" s="7"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
@@ -5409,6 +5514,7 @@
       <c r="P102" s="7"/>
       <c r="Q102" s="7"/>
       <c r="R102" s="7"/>
+      <c r="S102" s="7"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="inlineStr">
@@ -5448,6 +5554,7 @@
       <c r="P103" s="7"/>
       <c r="Q103" s="7"/>
       <c r="R103" s="7"/>
+      <c r="S103" s="7"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="inlineStr">
@@ -5492,6 +5599,7 @@
       <c r="P104" s="7"/>
       <c r="Q104" s="7"/>
       <c r="R104" s="7"/>
+      <c r="S104" s="7"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
@@ -5531,6 +5639,7 @@
       <c r="P105" s="7"/>
       <c r="Q105" s="7"/>
       <c r="R105" s="7"/>
+      <c r="S105" s="7"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
@@ -5570,6 +5679,7 @@
       <c r="P106" s="7"/>
       <c r="Q106" s="7"/>
       <c r="R106" s="7"/>
+      <c r="S106" s="7"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
@@ -5609,6 +5719,7 @@
       <c r="P107" s="7"/>
       <c r="Q107" s="7"/>
       <c r="R107" s="7"/>
+      <c r="S107" s="7"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
@@ -5652,6 +5763,7 @@
       <c r="P108" s="7"/>
       <c r="Q108" s="7"/>
       <c r="R108" s="7"/>
+      <c r="S108" s="7"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="inlineStr">
@@ -5700,6 +5812,7 @@
       <c r="P109" s="7"/>
       <c r="Q109" s="7"/>
       <c r="R109" s="7"/>
+      <c r="S109" s="7"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
@@ -5756,6 +5869,7 @@
       </c>
       <c r="Q110" s="7"/>
       <c r="R110" s="7"/>
+      <c r="S110" s="7"/>
     </row>
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
@@ -5815,6 +5929,7 @@
       </c>
       <c r="Q111" s="7"/>
       <c r="R111" s="7"/>
+      <c r="S111" s="7"/>
     </row>
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
@@ -5871,6 +5986,7 @@
       <c r="P112" s="7"/>
       <c r="Q112" s="7"/>
       <c r="R112" s="7"/>
+      <c r="S112" s="7"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
@@ -5919,6 +6035,7 @@
       <c r="P113" s="7"/>
       <c r="Q113" s="7"/>
       <c r="R113" s="7"/>
+      <c r="S113" s="7"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="inlineStr">
@@ -5983,6 +6100,7 @@
       </c>
       <c r="Q114" s="7"/>
       <c r="R114" s="7"/>
+      <c r="S114" s="7"/>
     </row>
     <row r="115">
       <c r="A115" s="7" t="inlineStr">
@@ -6039,6 +6157,7 @@
       <c r="P115" s="7"/>
       <c r="Q115" s="7"/>
       <c r="R115" s="7"/>
+      <c r="S115" s="7"/>
     </row>
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
@@ -6099,6 +6218,7 @@
         </is>
       </c>
       <c r="R116" s="7"/>
+      <c r="S116" s="7"/>
     </row>
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
@@ -6159,6 +6279,7 @@
         </is>
       </c>
       <c r="R117" s="7"/>
+      <c r="S117" s="7"/>
     </row>
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
@@ -6219,6 +6340,7 @@
         </is>
       </c>
       <c r="R118" s="7"/>
+      <c r="S118" s="7"/>
     </row>
     <row r="119">
       <c r="A119" s="7" t="inlineStr">
@@ -6275,6 +6397,7 @@
         </is>
       </c>
       <c r="R119" s="7"/>
+      <c r="S119" s="7"/>
     </row>
     <row r="120">
       <c r="A120" s="7" t="inlineStr">
@@ -6323,6 +6446,7 @@
       <c r="P120" s="7"/>
       <c r="Q120" s="7"/>
       <c r="R120" s="7"/>
+      <c r="S120" s="7"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="inlineStr">
@@ -6383,6 +6507,7 @@
         </is>
       </c>
       <c r="R121" s="7"/>
+      <c r="S121" s="7"/>
     </row>
     <row r="122">
       <c r="A122" s="7" t="inlineStr">
@@ -6443,6 +6568,7 @@
         </is>
       </c>
       <c r="R122" s="7"/>
+      <c r="S122" s="7"/>
     </row>
     <row r="123">
       <c r="A123" s="7" t="inlineStr">
@@ -6491,6 +6617,7 @@
       <c r="P123" s="7"/>
       <c r="Q123" s="7"/>
       <c r="R123" s="7"/>
+      <c r="S123" s="7"/>
     </row>
     <row r="124">
       <c r="A124" s="7" t="inlineStr">
@@ -6547,6 +6674,7 @@
         </is>
       </c>
       <c r="R124" s="7"/>
+      <c r="S124" s="7"/>
     </row>
     <row r="125">
       <c r="A125" s="7" t="inlineStr">
@@ -6595,6 +6723,7 @@
       <c r="P125" s="7"/>
       <c r="Q125" s="7"/>
       <c r="R125" s="7"/>
+      <c r="S125" s="7"/>
     </row>
     <row r="126">
       <c r="A126" s="7" t="inlineStr">
@@ -6643,6 +6772,7 @@
       </c>
       <c r="Q126" s="7"/>
       <c r="R126" s="7"/>
+      <c r="S126" s="7"/>
     </row>
     <row r="127">
       <c r="A127" s="7" t="inlineStr">
@@ -6695,6 +6825,7 @@
         </is>
       </c>
       <c r="R127" s="7"/>
+      <c r="S127" s="7"/>
     </row>
     <row r="128">
       <c r="A128" s="7" t="inlineStr">
@@ -6747,6 +6878,7 @@
         </is>
       </c>
       <c r="R128" s="7"/>
+      <c r="S128" s="7"/>
     </row>
     <row r="129">
       <c r="A129" s="7" t="inlineStr">
@@ -6799,6 +6931,7 @@
         </is>
       </c>
       <c r="R129" s="7"/>
+      <c r="S129" s="7"/>
     </row>
     <row r="130">
       <c r="A130" s="7" t="inlineStr">
@@ -6847,6 +6980,7 @@
         </is>
       </c>
       <c r="R130" s="7"/>
+      <c r="S130" s="7"/>
     </row>
     <row r="131">
       <c r="A131" s="7" t="inlineStr">
@@ -6895,6 +7029,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="S131" s="7"/>
     </row>
     <row r="132">
       <c r="A132" s="7" t="inlineStr">
@@ -6943,6 +7078,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="S132" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="7" t="inlineStr">
@@ -6991,6 +7131,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="S133" s="7"/>
     </row>
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
@@ -7035,6 +7176,109 @@
       <c r="P134" s="7"/>
       <c r="Q134" s="7"/>
       <c r="R134" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="S134" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_127</t>
+        </is>
+      </c>
+      <c r="B135" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C135" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도전</t>
+        </is>
+      </c>
+      <c r="D135" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전원 스폰</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도전에 들어가면 그 판의 몬스터가 첫 순간에 전부 서고(「남은 몬스터」가 판 전체 수), 서로 겹치지 않는가?</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">🗑️ 도전 층 묶음 스폰 폐기 · 파밍 층은 그대로 (10-16 #152)</t>
+        </is>
+      </c>
+      <c r="G135" s="7"/>
+      <c r="H135" s="7"/>
+      <c r="I135" s="7"/>
+      <c r="J135" s="7"/>
+      <c r="K135" s="7"/>
+      <c r="L135" s="7"/>
+      <c r="M135" s="7"/>
+      <c r="N135" s="7"/>
+      <c r="O135" s="7"/>
+      <c r="P135" s="7"/>
+      <c r="Q135" s="7"/>
+      <c r="R135" s="7"/>
+      <c r="S135" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_128</t>
+        </is>
+      </c>
+      <c r="B136" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C136" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">몬스터</t>
+        </is>
+      </c>
+      <c r="D136" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">탐색 범위</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">로봇과 먼 몬스터는 제자리에 서서 쏘지도 않다가, 로봇이 다가가면(탐색 범위 9.2) 그때부터 쫓아오고 다시 멀어져도 계속 쫓는가?</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">범위 = COMBAT_RULE_DATA enemyAggroRangeTbd (10-16 #152)</t>
+        </is>
+      </c>
+      <c r="G136" s="7"/>
+      <c r="H136" s="7"/>
+      <c r="I136" s="7"/>
+      <c r="J136" s="7"/>
+      <c r="K136" s="7"/>
+      <c r="L136" s="7"/>
+      <c r="M136" s="7"/>
+      <c r="N136" s="7"/>
+      <c r="O136" s="7"/>
+      <c r="P136" s="7"/>
+      <c r="Q136" s="7"/>
+      <c r="R136" s="7"/>
+      <c r="S136" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -7067,9 +7311,9 @@
     <mergeCell ref="B92:B99"/>
     <mergeCell ref="B100:B106"/>
     <mergeCell ref="B107:B111"/>
-    <mergeCell ref="G7:R7"/>
+    <mergeCell ref="G7:S7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:R134">
+  <conditionalFormatting sqref="G9:S136">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
QA T열(983f3f6) — #153 재확인 Pass 10 · Fail 0 · CID_129~132 신설
8128 처음부터 → S1·S2·S3 자연 승리 → S4 강화 전 시간 초과(벽) → 강화 단추 → S4 승리 · 파밍 적 바로 다가옴 ·
S6 보스 제자리 → 맞고 다가옴. S5 시간 초과(Auto 태그 안 켬).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -175,8 +175,9 @@
     <col min="17" max="17" width="12" customWidth="1"/>
     <col min="18" max="18" width="12" customWidth="1"/>
     <col min="19" max="19" width="12" customWidth="1"/>
-    <col min="20" max="20" width="11" customWidth="1"/>
+    <col min="20" max="20" width="12" customWidth="1"/>
     <col min="21" max="21" width="11" customWidth="1"/>
+    <col min="22" max="22" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -354,6 +355,11 @@
       <c r="S6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">video-261016 후보 · #152 도전 층 전원 스폰 · 몬스터 탐색 범위 9.2(밖이면 제자리 · 들면 깨어 끝까지 추격) ‖ 10-16 코드 세션 재확인(리포 8123 S4 + 사본 _261016 · 8128 · 576×1024 · 소리 0 · 처음부터 → 바로가기 S1 도전 50기 전원 서고 제자리 → 승리(남은 00:27 · HP 가득) → 다음 스테이지로 S2 → 승리(남은 00:02 · HP 약 875) · 8123 S4 도전 98기 → 로봇 파괴 약 13초(남은 93 · 바로가기라 마운트 빈손) · 브라우저 프레임 약 83/초(rAF · 98기 동시)) · 8128 갈아엎음 17:18:45(f710a05 → 08ec1c7) · 빈 칸 = 안 지나감 · 관찰(판정 없음): S3·S4 는 깨어 있는 적이 한 번에 19~26 기라 로봇이 버티지 못한다(하네스) · CID_127~128 새 항목</t>
+        </is>
+      </c>
+      <c r="T6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">video-261016 후보 · #153 맞으면 깸 · 탐색 범위 6 · 탐색·전원 스폰은 도전 층만 · S3 87→30 · S4 98→24 ‖ 10-16 코드 세션 재확인(사본 _261016 · 8128 · 576×1024 · 소리 0 · 처음부터 → 바로가기 S1 파밍: 적이 바로 다가옴 → S1 도전 승리(남은 00:34) → S2 승리(남은 00:14 · HP 가득) → S3 자연 승리(남은 00:07 · HP 가득) → S4 파밍 적 다가옴 → S4 도전 시간 초과 남은 3(벽) → 설정 강화 단추 밝음 → 누름 → 「강화 ×1.45 적용」 → 다시 도전 S4 승리(남은 00:10) → S5 시간 초과 0/7(Auto 태그 안 켬) → 바로가기 S6 시간 초과(보스 제자리 → 맞고 다가옴)) · 8128 갈아엎음 17:48:54(08ec1c7 → 983f3f6) · 빈 칸 = 안 지나감 · CID_129~132 새 항목</t>
         </is>
       </c>
     </row>
@@ -397,14 +403,15 @@
       <c r="Q7" s="2"/>
       <c r="R7" s="2"/>
       <c r="S7" s="2"/>
-      <c r="T7" s="2" t="inlineStr">
+      <c r="T7" s="2"/>
+      <c r="U7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">버전</t>
         </is>
       </c>
-      <c r="U7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">08ec1c7</t>
+      <c r="V7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">983f3f6</t>
         </is>
       </c>
     </row>
@@ -494,11 +501,16 @@
       </c>
       <c r="T8" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">983f3f6</t>
+        </is>
+      </c>
+      <c r="U8" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">PASSrate</t>
         </is>
       </c>
-      <c r="U8" s="7">
-        <f>COUNTIF(S9:S136,"Pass")</f>
+      <c r="V8" s="7">
+        <f>COUNTIF(T9:T140,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -581,13 +593,14 @@
       </c>
       <c r="R9" s="7"/>
       <c r="S9" s="7"/>
-      <c r="T9" s="2" t="inlineStr">
+      <c r="T9" s="7"/>
+      <c r="U9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FAILrate</t>
         </is>
       </c>
-      <c r="U9" s="7">
-        <f>COUNTIF(S9:S136,"Fail")+COUNTIF(S9:S136,"Broken")</f>
+      <c r="V9" s="7">
+        <f>COUNTIF(T9:T140,"Fail")+COUNTIF(T9:T140,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -634,13 +647,14 @@
       <c r="Q10" s="7"/>
       <c r="R10" s="7"/>
       <c r="S10" s="7"/>
-      <c r="T10" s="2" t="inlineStr">
+      <c r="T10" s="7"/>
+      <c r="U10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">N/A</t>
         </is>
       </c>
-      <c r="U10" s="7">
-        <f>COUNTIF(S9:S136,"N/A")</f>
+      <c r="V10" s="7">
+        <f>COUNTIF(T9:T140,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -687,13 +701,14 @@
       <c r="Q11" s="7"/>
       <c r="R11" s="7"/>
       <c r="S11" s="7"/>
-      <c r="T11" s="2" t="inlineStr">
+      <c r="T11" s="7"/>
+      <c r="U11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">전체 개수</t>
         </is>
       </c>
-      <c r="U11" s="7">
-        <v>128</v>
+      <c r="V11" s="7">
+        <v>132</v>
       </c>
     </row>
     <row r="12">
@@ -740,13 +755,14 @@
       <c r="Q12" s="7"/>
       <c r="R12" s="7"/>
       <c r="S12" s="7"/>
-      <c r="T12" s="2" t="inlineStr">
+      <c r="T12" s="7"/>
+      <c r="U12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">진행율</t>
         </is>
       </c>
-      <c r="U12" s="7">
-        <f>TEXT((COUNTA(S9:S136))/128,"0.00%")</f>
+      <c r="V12" s="7">
+        <f>TEXT((COUNTA(T9:T140))/132,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -797,6 +813,7 @@
       <c r="Q13" s="7"/>
       <c r="R13" s="7"/>
       <c r="S13" s="7"/>
+      <c r="T13" s="7"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -837,6 +854,7 @@
       <c r="Q14" s="7"/>
       <c r="R14" s="7"/>
       <c r="S14" s="7"/>
+      <c r="T14" s="7"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -913,6 +931,7 @@
       </c>
       <c r="R15" s="7"/>
       <c r="S15" s="7"/>
+      <c r="T15" s="7"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -989,6 +1008,7 @@
       </c>
       <c r="R16" s="7"/>
       <c r="S16" s="7"/>
+      <c r="T16" s="7"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -1070,6 +1090,7 @@
       </c>
       <c r="R17" s="7"/>
       <c r="S17" s="7"/>
+      <c r="T17" s="7"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -1115,6 +1136,7 @@
       <c r="Q18" s="7"/>
       <c r="R18" s="7"/>
       <c r="S18" s="7"/>
+      <c r="T18" s="7"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -1155,6 +1177,7 @@
       <c r="Q19" s="7"/>
       <c r="R19" s="7"/>
       <c r="S19" s="7"/>
+      <c r="T19" s="7"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1195,6 +1218,7 @@
       <c r="Q20" s="7"/>
       <c r="R20" s="7"/>
       <c r="S20" s="7"/>
+      <c r="T20" s="7"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1271,6 +1295,7 @@
       </c>
       <c r="R21" s="7"/>
       <c r="S21" s="7"/>
+      <c r="T21" s="7"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1340,6 +1365,7 @@
       <c r="Q22" s="7"/>
       <c r="R22" s="7"/>
       <c r="S22" s="7"/>
+      <c r="T22" s="7"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -1388,6 +1414,7 @@
       <c r="Q23" s="7"/>
       <c r="R23" s="7"/>
       <c r="S23" s="7"/>
+      <c r="T23" s="7"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -1428,6 +1455,7 @@
       <c r="Q24" s="7"/>
       <c r="R24" s="7"/>
       <c r="S24" s="7"/>
+      <c r="T24" s="7"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -1468,6 +1496,7 @@
       <c r="Q25" s="7"/>
       <c r="R25" s="7"/>
       <c r="S25" s="7"/>
+      <c r="T25" s="7"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -1537,6 +1566,7 @@
       <c r="Q26" s="7"/>
       <c r="R26" s="7"/>
       <c r="S26" s="7"/>
+      <c r="T26" s="7"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -1581,6 +1611,7 @@
       <c r="Q27" s="7"/>
       <c r="R27" s="7"/>
       <c r="S27" s="7"/>
+      <c r="T27" s="7"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -1634,6 +1665,7 @@
       <c r="Q28" s="7"/>
       <c r="R28" s="7"/>
       <c r="S28" s="7"/>
+      <c r="T28" s="7"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -1682,6 +1714,7 @@
       <c r="Q29" s="7"/>
       <c r="R29" s="7"/>
       <c r="S29" s="7"/>
+      <c r="T29" s="7"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -1754,6 +1787,7 @@
       <c r="Q30" s="7"/>
       <c r="R30" s="7"/>
       <c r="S30" s="7"/>
+      <c r="T30" s="7"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -1831,6 +1865,7 @@
       <c r="Q31" s="7"/>
       <c r="R31" s="7"/>
       <c r="S31" s="7"/>
+      <c r="T31" s="7"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -1895,6 +1930,7 @@
       <c r="Q32" s="7"/>
       <c r="R32" s="7"/>
       <c r="S32" s="7"/>
+      <c r="T32" s="7"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -1967,6 +2003,7 @@
       <c r="Q33" s="7"/>
       <c r="R33" s="7"/>
       <c r="S33" s="7"/>
+      <c r="T33" s="7"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -2039,6 +2076,7 @@
       <c r="Q34" s="7"/>
       <c r="R34" s="7"/>
       <c r="S34" s="7"/>
+      <c r="T34" s="7"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -2116,6 +2154,7 @@
       <c r="Q35" s="7"/>
       <c r="R35" s="7"/>
       <c r="S35" s="7"/>
+      <c r="T35" s="7"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -2172,6 +2211,7 @@
       <c r="Q36" s="7"/>
       <c r="R36" s="7"/>
       <c r="S36" s="7"/>
+      <c r="T36" s="7"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -2212,6 +2252,7 @@
       <c r="Q37" s="7"/>
       <c r="R37" s="7"/>
       <c r="S37" s="7"/>
+      <c r="T37" s="7"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -2273,6 +2314,7 @@
       <c r="Q38" s="7"/>
       <c r="R38" s="7"/>
       <c r="S38" s="7"/>
+      <c r="T38" s="7"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -2345,6 +2387,7 @@
       <c r="Q39" s="7"/>
       <c r="R39" s="7"/>
       <c r="S39" s="7"/>
+      <c r="T39" s="7"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -2418,6 +2461,7 @@
       <c r="Q40" s="7"/>
       <c r="R40" s="7"/>
       <c r="S40" s="7"/>
+      <c r="T40" s="7"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -2486,6 +2530,7 @@
       <c r="Q41" s="7"/>
       <c r="R41" s="7"/>
       <c r="S41" s="7"/>
+      <c r="T41" s="7"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -2538,6 +2583,7 @@
       <c r="Q42" s="7"/>
       <c r="R42" s="7"/>
       <c r="S42" s="7"/>
+      <c r="T42" s="7"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -2610,6 +2656,7 @@
       <c r="Q43" s="7"/>
       <c r="R43" s="7"/>
       <c r="S43" s="7"/>
+      <c r="T43" s="7"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -2655,6 +2702,7 @@
       <c r="Q44" s="7"/>
       <c r="R44" s="7"/>
       <c r="S44" s="7"/>
+      <c r="T44" s="7"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -2723,6 +2771,7 @@
       <c r="Q45" s="7"/>
       <c r="R45" s="7"/>
       <c r="S45" s="7"/>
+      <c r="T45" s="7"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -2791,6 +2840,7 @@
       <c r="Q46" s="7"/>
       <c r="R46" s="7"/>
       <c r="S46" s="7"/>
+      <c r="T46" s="7"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -2836,6 +2886,7 @@
       <c r="Q47" s="7"/>
       <c r="R47" s="7"/>
       <c r="S47" s="7"/>
+      <c r="T47" s="7"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -2876,6 +2927,7 @@
       <c r="Q48" s="7"/>
       <c r="R48" s="7"/>
       <c r="S48" s="7"/>
+      <c r="T48" s="7"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -2916,6 +2968,7 @@
       <c r="Q49" s="7"/>
       <c r="R49" s="7"/>
       <c r="S49" s="7"/>
+      <c r="T49" s="7"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -2980,6 +3033,7 @@
       <c r="Q50" s="7"/>
       <c r="R50" s="7"/>
       <c r="S50" s="7"/>
+      <c r="T50" s="7"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -3044,6 +3098,7 @@
       <c r="Q51" s="7"/>
       <c r="R51" s="7"/>
       <c r="S51" s="7"/>
+      <c r="T51" s="7"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -3089,6 +3144,7 @@
       <c r="Q52" s="7"/>
       <c r="R52" s="7"/>
       <c r="S52" s="7"/>
+      <c r="T52" s="7"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -3134,6 +3190,7 @@
       <c r="Q53" s="7"/>
       <c r="R53" s="7"/>
       <c r="S53" s="7"/>
+      <c r="T53" s="7"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -3174,6 +3231,7 @@
       <c r="Q54" s="7"/>
       <c r="R54" s="7"/>
       <c r="S54" s="7"/>
+      <c r="T54" s="7"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -3250,6 +3308,7 @@
       </c>
       <c r="R55" s="7"/>
       <c r="S55" s="7"/>
+      <c r="T55" s="7"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -3306,6 +3365,7 @@
       <c r="Q56" s="7"/>
       <c r="R56" s="7"/>
       <c r="S56" s="7"/>
+      <c r="T56" s="7"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -3371,6 +3431,7 @@
       <c r="Q57" s="7"/>
       <c r="R57" s="7"/>
       <c r="S57" s="7"/>
+      <c r="T57" s="7"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -3444,6 +3505,7 @@
       </c>
       <c r="R58" s="7"/>
       <c r="S58" s="7"/>
+      <c r="T58" s="7"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -3484,6 +3546,7 @@
       <c r="Q59" s="7"/>
       <c r="R59" s="7"/>
       <c r="S59" s="7"/>
+      <c r="T59" s="7"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -3524,6 +3587,7 @@
       <c r="Q60" s="7"/>
       <c r="R60" s="7"/>
       <c r="S60" s="7"/>
+      <c r="T60" s="7"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -3576,6 +3640,7 @@
       <c r="Q61" s="7"/>
       <c r="R61" s="7"/>
       <c r="S61" s="7"/>
+      <c r="T61" s="7"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -3636,6 +3701,7 @@
       </c>
       <c r="R62" s="7"/>
       <c r="S62" s="7"/>
+      <c r="T62" s="7"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -3688,6 +3754,7 @@
       <c r="Q63" s="7"/>
       <c r="R63" s="7"/>
       <c r="S63" s="7"/>
+      <c r="T63" s="7"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -3728,6 +3795,7 @@
       <c r="Q64" s="7"/>
       <c r="R64" s="7"/>
       <c r="S64" s="7"/>
+      <c r="T64" s="7"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -3773,6 +3841,7 @@
       <c r="Q65" s="7"/>
       <c r="R65" s="7"/>
       <c r="S65" s="7"/>
+      <c r="T65" s="7"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
@@ -3825,6 +3894,7 @@
       <c r="Q66" s="7"/>
       <c r="R66" s="7"/>
       <c r="S66" s="7"/>
+      <c r="T66" s="7"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -3865,6 +3935,7 @@
       <c r="Q67" s="7"/>
       <c r="R67" s="7"/>
       <c r="S67" s="7"/>
+      <c r="T67" s="7"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
@@ -3909,6 +3980,7 @@
       <c r="Q68" s="7"/>
       <c r="R68" s="7"/>
       <c r="S68" s="7"/>
+      <c r="T68" s="7"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -3985,6 +4057,7 @@
       </c>
       <c r="R69" s="7"/>
       <c r="S69" s="7"/>
+      <c r="T69" s="7"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
@@ -4025,6 +4098,7 @@
       <c r="Q70" s="7"/>
       <c r="R70" s="7"/>
       <c r="S70" s="7"/>
+      <c r="T70" s="7"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -4070,6 +4144,7 @@
       <c r="Q71" s="7"/>
       <c r="R71" s="7"/>
       <c r="S71" s="7"/>
+      <c r="T71" s="7"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
@@ -4126,6 +4201,7 @@
       </c>
       <c r="R72" s="7"/>
       <c r="S72" s="7"/>
+      <c r="T72" s="7"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
@@ -4171,6 +4247,7 @@
       <c r="Q73" s="7"/>
       <c r="R73" s="7"/>
       <c r="S73" s="7"/>
+      <c r="T73" s="7"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -4211,6 +4288,7 @@
       <c r="Q74" s="7"/>
       <c r="R74" s="7"/>
       <c r="S74" s="7"/>
+      <c r="T74" s="7"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -4251,6 +4329,7 @@
       <c r="Q75" s="7"/>
       <c r="R75" s="7"/>
       <c r="S75" s="7"/>
+      <c r="T75" s="7"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -4291,6 +4370,7 @@
       <c r="Q76" s="7"/>
       <c r="R76" s="7"/>
       <c r="S76" s="7"/>
+      <c r="T76" s="7"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -4335,6 +4415,7 @@
       </c>
       <c r="R77" s="7"/>
       <c r="S77" s="7"/>
+      <c r="T77" s="7"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
@@ -4375,6 +4456,7 @@
       <c r="Q78" s="7"/>
       <c r="R78" s="7"/>
       <c r="S78" s="7"/>
+      <c r="T78" s="7"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -4420,6 +4502,7 @@
       <c r="Q79" s="7"/>
       <c r="R79" s="7"/>
       <c r="S79" s="7"/>
+      <c r="T79" s="7"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
@@ -4476,6 +4559,7 @@
       </c>
       <c r="R80" s="7"/>
       <c r="S80" s="7"/>
+      <c r="T80" s="7"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
@@ -4516,6 +4600,7 @@
       <c r="Q81" s="7"/>
       <c r="R81" s="7"/>
       <c r="S81" s="7"/>
+      <c r="T81" s="7"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
@@ -4556,6 +4641,7 @@
       <c r="Q82" s="7"/>
       <c r="R82" s="7"/>
       <c r="S82" s="7"/>
+      <c r="T82" s="7"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
@@ -4601,6 +4687,7 @@
       <c r="Q83" s="7"/>
       <c r="R83" s="7"/>
       <c r="S83" s="7"/>
+      <c r="T83" s="7"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
@@ -4641,6 +4728,7 @@
       <c r="Q84" s="7"/>
       <c r="R84" s="7"/>
       <c r="S84" s="7"/>
+      <c r="T84" s="7"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
@@ -4681,6 +4769,7 @@
       <c r="Q85" s="7"/>
       <c r="R85" s="7"/>
       <c r="S85" s="7"/>
+      <c r="T85" s="7"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
@@ -4726,6 +4815,7 @@
       <c r="Q86" s="7"/>
       <c r="R86" s="7"/>
       <c r="S86" s="7"/>
+      <c r="T86" s="7"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
@@ -4766,6 +4856,7 @@
       <c r="Q87" s="7"/>
       <c r="R87" s="7"/>
       <c r="S87" s="7"/>
+      <c r="T87" s="7"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
@@ -4806,6 +4897,7 @@
       <c r="Q88" s="7"/>
       <c r="R88" s="7"/>
       <c r="S88" s="7"/>
+      <c r="T88" s="7"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
@@ -4846,6 +4938,7 @@
       <c r="Q89" s="7"/>
       <c r="R89" s="7"/>
       <c r="S89" s="7"/>
+      <c r="T89" s="7"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
@@ -4915,6 +5008,7 @@
       <c r="Q90" s="7"/>
       <c r="R90" s="7"/>
       <c r="S90" s="7"/>
+      <c r="T90" s="7"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
@@ -4955,6 +5049,7 @@
       <c r="Q91" s="7"/>
       <c r="R91" s="7"/>
       <c r="S91" s="7"/>
+      <c r="T91" s="7"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
@@ -5031,6 +5126,7 @@
       </c>
       <c r="R92" s="7"/>
       <c r="S92" s="7"/>
+      <c r="T92" s="7"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
@@ -5112,6 +5208,7 @@
       </c>
       <c r="R93" s="7"/>
       <c r="S93" s="7"/>
+      <c r="T93" s="7"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
@@ -5157,6 +5254,7 @@
       <c r="Q94" s="7"/>
       <c r="R94" s="7"/>
       <c r="S94" s="7"/>
+      <c r="T94" s="7"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
@@ -5202,6 +5300,7 @@
       <c r="Q95" s="7"/>
       <c r="R95" s="7"/>
       <c r="S95" s="7"/>
+      <c r="T95" s="7"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
@@ -5266,6 +5365,7 @@
       <c r="Q96" s="7"/>
       <c r="R96" s="7"/>
       <c r="S96" s="7"/>
+      <c r="T96" s="7"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="inlineStr">
@@ -5306,6 +5406,7 @@
       <c r="Q97" s="7"/>
       <c r="R97" s="7"/>
       <c r="S97" s="7"/>
+      <c r="T97" s="7"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
@@ -5346,6 +5447,7 @@
       <c r="Q98" s="7"/>
       <c r="R98" s="7"/>
       <c r="S98" s="7"/>
+      <c r="T98" s="7"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
@@ -5386,6 +5488,7 @@
       <c r="Q99" s="7"/>
       <c r="R99" s="7"/>
       <c r="S99" s="7"/>
+      <c r="T99" s="7"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
@@ -5435,6 +5538,7 @@
       <c r="Q100" s="7"/>
       <c r="R100" s="7"/>
       <c r="S100" s="7"/>
+      <c r="T100" s="7"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
@@ -5475,6 +5579,7 @@
       <c r="Q101" s="7"/>
       <c r="R101" s="7"/>
       <c r="S101" s="7"/>
+      <c r="T101" s="7"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
@@ -5515,6 +5620,7 @@
       <c r="Q102" s="7"/>
       <c r="R102" s="7"/>
       <c r="S102" s="7"/>
+      <c r="T102" s="7"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="inlineStr">
@@ -5555,6 +5661,7 @@
       <c r="Q103" s="7"/>
       <c r="R103" s="7"/>
       <c r="S103" s="7"/>
+      <c r="T103" s="7"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="inlineStr">
@@ -5600,6 +5707,7 @@
       <c r="Q104" s="7"/>
       <c r="R104" s="7"/>
       <c r="S104" s="7"/>
+      <c r="T104" s="7"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
@@ -5640,6 +5748,7 @@
       <c r="Q105" s="7"/>
       <c r="R105" s="7"/>
       <c r="S105" s="7"/>
+      <c r="T105" s="7"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
@@ -5680,6 +5789,7 @@
       <c r="Q106" s="7"/>
       <c r="R106" s="7"/>
       <c r="S106" s="7"/>
+      <c r="T106" s="7"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
@@ -5720,6 +5830,7 @@
       <c r="Q107" s="7"/>
       <c r="R107" s="7"/>
       <c r="S107" s="7"/>
+      <c r="T107" s="7"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
@@ -5764,6 +5875,7 @@
       <c r="Q108" s="7"/>
       <c r="R108" s="7"/>
       <c r="S108" s="7"/>
+      <c r="T108" s="7"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="inlineStr">
@@ -5813,6 +5925,7 @@
       <c r="Q109" s="7"/>
       <c r="R109" s="7"/>
       <c r="S109" s="7"/>
+      <c r="T109" s="7"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
@@ -5870,6 +5983,7 @@
       <c r="Q110" s="7"/>
       <c r="R110" s="7"/>
       <c r="S110" s="7"/>
+      <c r="T110" s="7"/>
     </row>
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
@@ -5930,6 +6044,7 @@
       <c r="Q111" s="7"/>
       <c r="R111" s="7"/>
       <c r="S111" s="7"/>
+      <c r="T111" s="7"/>
     </row>
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
@@ -5987,6 +6102,7 @@
       <c r="Q112" s="7"/>
       <c r="R112" s="7"/>
       <c r="S112" s="7"/>
+      <c r="T112" s="7"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
@@ -6036,6 +6152,7 @@
       <c r="Q113" s="7"/>
       <c r="R113" s="7"/>
       <c r="S113" s="7"/>
+      <c r="T113" s="7"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="inlineStr">
@@ -6101,6 +6218,7 @@
       <c r="Q114" s="7"/>
       <c r="R114" s="7"/>
       <c r="S114" s="7"/>
+      <c r="T114" s="7"/>
     </row>
     <row r="115">
       <c r="A115" s="7" t="inlineStr">
@@ -6158,6 +6276,7 @@
       <c r="Q115" s="7"/>
       <c r="R115" s="7"/>
       <c r="S115" s="7"/>
+      <c r="T115" s="7"/>
     </row>
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
@@ -6219,6 +6338,7 @@
       </c>
       <c r="R116" s="7"/>
       <c r="S116" s="7"/>
+      <c r="T116" s="7"/>
     </row>
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
@@ -6280,6 +6400,7 @@
       </c>
       <c r="R117" s="7"/>
       <c r="S117" s="7"/>
+      <c r="T117" s="7"/>
     </row>
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
@@ -6341,6 +6462,7 @@
       </c>
       <c r="R118" s="7"/>
       <c r="S118" s="7"/>
+      <c r="T118" s="7"/>
     </row>
     <row r="119">
       <c r="A119" s="7" t="inlineStr">
@@ -6398,6 +6520,7 @@
       </c>
       <c r="R119" s="7"/>
       <c r="S119" s="7"/>
+      <c r="T119" s="7"/>
     </row>
     <row r="120">
       <c r="A120" s="7" t="inlineStr">
@@ -6447,6 +6570,7 @@
       <c r="Q120" s="7"/>
       <c r="R120" s="7"/>
       <c r="S120" s="7"/>
+      <c r="T120" s="7"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="inlineStr">
@@ -6508,6 +6632,7 @@
       </c>
       <c r="R121" s="7"/>
       <c r="S121" s="7"/>
+      <c r="T121" s="7"/>
     </row>
     <row r="122">
       <c r="A122" s="7" t="inlineStr">
@@ -6569,6 +6694,7 @@
       </c>
       <c r="R122" s="7"/>
       <c r="S122" s="7"/>
+      <c r="T122" s="7"/>
     </row>
     <row r="123">
       <c r="A123" s="7" t="inlineStr">
@@ -6618,6 +6744,7 @@
       <c r="Q123" s="7"/>
       <c r="R123" s="7"/>
       <c r="S123" s="7"/>
+      <c r="T123" s="7"/>
     </row>
     <row r="124">
       <c r="A124" s="7" t="inlineStr">
@@ -6675,6 +6802,7 @@
       </c>
       <c r="R124" s="7"/>
       <c r="S124" s="7"/>
+      <c r="T124" s="7"/>
     </row>
     <row r="125">
       <c r="A125" s="7" t="inlineStr">
@@ -6724,6 +6852,7 @@
       <c r="Q125" s="7"/>
       <c r="R125" s="7"/>
       <c r="S125" s="7"/>
+      <c r="T125" s="7"/>
     </row>
     <row r="126">
       <c r="A126" s="7" t="inlineStr">
@@ -6773,6 +6902,7 @@
       <c r="Q126" s="7"/>
       <c r="R126" s="7"/>
       <c r="S126" s="7"/>
+      <c r="T126" s="7"/>
     </row>
     <row r="127">
       <c r="A127" s="7" t="inlineStr">
@@ -6826,6 +6956,7 @@
       </c>
       <c r="R127" s="7"/>
       <c r="S127" s="7"/>
+      <c r="T127" s="7"/>
     </row>
     <row r="128">
       <c r="A128" s="7" t="inlineStr">
@@ -6879,6 +7010,7 @@
       </c>
       <c r="R128" s="7"/>
       <c r="S128" s="7"/>
+      <c r="T128" s="7"/>
     </row>
     <row r="129">
       <c r="A129" s="7" t="inlineStr">
@@ -6932,6 +7064,7 @@
       </c>
       <c r="R129" s="7"/>
       <c r="S129" s="7"/>
+      <c r="T129" s="7"/>
     </row>
     <row r="130">
       <c r="A130" s="7" t="inlineStr">
@@ -6981,6 +7114,7 @@
       </c>
       <c r="R130" s="7"/>
       <c r="S130" s="7"/>
+      <c r="T130" s="7"/>
     </row>
     <row r="131">
       <c r="A131" s="7" t="inlineStr">
@@ -7030,6 +7164,11 @@
         </is>
       </c>
       <c r="S131" s="7"/>
+      <c r="T131" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="7" t="inlineStr">
@@ -7083,6 +7222,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="T132" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="7" t="inlineStr">
@@ -7132,6 +7276,11 @@
         </is>
       </c>
       <c r="S133" s="7"/>
+      <c r="T133" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
@@ -7181,6 +7330,11 @@
         </is>
       </c>
       <c r="S134" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="T134" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -7234,6 +7388,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="T135" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="7" t="inlineStr">
@@ -7279,6 +7438,211 @@
       <c r="Q136" s="7"/>
       <c r="R136" s="7"/>
       <c r="S136" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="T136" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_129</t>
+        </is>
+      </c>
+      <c r="B137" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C137" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">몬스터</t>
+        </is>
+      </c>
+      <c r="D137" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">맞으면 깸</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도전 층에서 탐색 범위 밖에 서 있던 몬스터(보스 포함)가 로봇에게 맞으면 그때부터 다가오는가? (맞은 적만 · 둘레 무리는 그대로)</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">탐색 범위 6 (10-16 #153)</t>
+        </is>
+      </c>
+      <c r="G137" s="7"/>
+      <c r="H137" s="7"/>
+      <c r="I137" s="7"/>
+      <c r="J137" s="7"/>
+      <c r="K137" s="7"/>
+      <c r="L137" s="7"/>
+      <c r="M137" s="7"/>
+      <c r="N137" s="7"/>
+      <c r="O137" s="7"/>
+      <c r="P137" s="7"/>
+      <c r="Q137" s="7"/>
+      <c r="R137" s="7"/>
+      <c r="S137" s="7"/>
+      <c r="T137" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_130</t>
+        </is>
+      </c>
+      <c r="B138" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C138" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">파밍 층</t>
+        </is>
+      </c>
+      <c r="D138" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">보충·접근</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">파밍 층에서는 몬스터가 정원·주기대로 보충되고 나오자마자 로봇에게 다가오는가? (도전 층의 전원 스폰·대기 규칙이 안 걸림)</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도전 층만 (10-16 #153)</t>
+        </is>
+      </c>
+      <c r="G138" s="7"/>
+      <c r="H138" s="7"/>
+      <c r="I138" s="7"/>
+      <c r="J138" s="7"/>
+      <c r="K138" s="7"/>
+      <c r="L138" s="7"/>
+      <c r="M138" s="7"/>
+      <c r="N138" s="7"/>
+      <c r="O138" s="7"/>
+      <c r="P138" s="7"/>
+      <c r="Q138" s="7"/>
+      <c r="R138" s="7"/>
+      <c r="S138" s="7"/>
+      <c r="T138" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_131</t>
+        </is>
+      </c>
+      <c r="B139" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C139" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3</t>
+        </is>
+      </c>
+      <c r="D139" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">자연 통과</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">강화 없이(시작 보드) S3 도전을 그대로 두면 60초 안에 전멸 승리하는가?</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 30기 (10-16 #153 ④)</t>
+        </is>
+      </c>
+      <c r="G139" s="7"/>
+      <c r="H139" s="7"/>
+      <c r="I139" s="7"/>
+      <c r="J139" s="7"/>
+      <c r="K139" s="7"/>
+      <c r="L139" s="7"/>
+      <c r="M139" s="7"/>
+      <c r="N139" s="7"/>
+      <c r="O139" s="7"/>
+      <c r="P139" s="7"/>
+      <c r="Q139" s="7"/>
+      <c r="R139" s="7"/>
+      <c r="S139" s="7"/>
+      <c r="T139" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_132</t>
+        </is>
+      </c>
+      <c r="B140" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C140" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4</t>
+        </is>
+      </c>
+      <c r="D140" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">강화 벽</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">강화 전 S4 도전은 60초 안에 다 못 잡고(시간 초과), 강화 단추를 누른 뒤 다시 도전하면 승리하는가?</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 24기 (10-16 #153 ④)</t>
+        </is>
+      </c>
+      <c r="G140" s="7"/>
+      <c r="H140" s="7"/>
+      <c r="I140" s="7"/>
+      <c r="J140" s="7"/>
+      <c r="K140" s="7"/>
+      <c r="L140" s="7"/>
+      <c r="M140" s="7"/>
+      <c r="N140" s="7"/>
+      <c r="O140" s="7"/>
+      <c r="P140" s="7"/>
+      <c r="Q140" s="7"/>
+      <c r="R140" s="7"/>
+      <c r="S140" s="7"/>
+      <c r="T140" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -7311,9 +7675,9 @@
     <mergeCell ref="B92:B99"/>
     <mergeCell ref="B100:B106"/>
     <mergeCell ref="B107:B111"/>
-    <mergeCell ref="G7:S7"/>
+    <mergeCell ref="G7:T7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:S136">
+  <conditionalFormatting sqref="G9:T140">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
QA U열(d08ddfc) — Pass 14 · Fail 1(CID_139 S6 화면) · CID_133~139 신설
도전 안내 창 · 물류 유지 · 합체 게이지 이어 감 · T3 안내 창 · 바로가기 만충 · 합체 중 B 드론 Pass.
S6 화면(태그 Auto 꺼짐 · 사람이 태그·합체) 시간 초과 Fail — 조건·내용은 플랜 세션에 전달.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -176,8 +176,9 @@
     <col min="18" max="18" width="12" customWidth="1"/>
     <col min="19" max="19" width="12" customWidth="1"/>
     <col min="20" max="20" width="12" customWidth="1"/>
-    <col min="21" max="21" width="11" customWidth="1"/>
+    <col min="21" max="21" width="12" customWidth="1"/>
     <col min="22" max="22" width="11" customWidth="1"/>
+    <col min="23" max="23" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -360,6 +361,11 @@
       <c r="T6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">video-261016 후보 · #153 맞으면 깸 · 탐색 범위 6 · 탐색·전원 스폰은 도전 층만 · S3 87→30 · S4 98→24 ‖ 10-16 코드 세션 재확인(사본 _261016 · 8128 · 576×1024 · 소리 0 · 처음부터 → 바로가기 S1 파밍: 적이 바로 다가옴 → S1 도전 승리(남은 00:34) → S2 승리(남은 00:14 · HP 가득) → S3 자연 승리(남은 00:07 · HP 가득) → S4 파밍 적 다가옴 → S4 도전 시간 초과 남은 3(벽) → 설정 강화 단추 밝음 → 누름 → 「강화 ×1.45 적용」 → 다시 도전 S4 승리(남은 00:10) → S5 시간 초과 0/7(Auto 태그 안 켬) → 바로가기 S6 시간 초과(보스 제자리 → 맞고 다가옴)) · 8128 갈아엎음 17:48:54(08ec1c7 → 983f3f6) · 빈 칸 = 안 지나감 · CID_129~132 새 항목</t>
+        </is>
+      </c>
+      <c r="U6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">video-261016 후보 · 사용자 직접 지시 ②③(물류 유지 · 도전 안내 창) · #155 합체 게이지 이어 감 · T3 안내 창 · S6 보스 13500 · #156 바로가기 만충 · #157 합체 중 A 탄 + B 드론 ‖ 10-16 코드 세션 재확인(8128 · 576×1024 · 소리 0 · ad5b7db 판: 처음부터 → 튜토리얼 벨트 이음 → T3 안내 창 [도전 시작] 하나(A 40/40) → S1 승(남 29초) → T4 모듈 → S2 승(남 3초) → S3 자연 승(남 5초) → 강화 → S4 승(남 8초) · 게이지가 판 넘어 차 S4 파밍에서 합체 발동 밝음 · 새로고침 뒤 S6 안내 창 게이지 100% · d08ddfc 판: 8123·8128 바로가기 S6 안내 창 A 40/40 · B 40/40 · 게이지 47%/100% · 태그 → 합체 → 합체 중 B 드론 나감 → S6 시간 초과(보스 약 30% 남음 · 태그 Auto 꺼짐 · 사람이 누름 · 하네스는 Auto 켬으로 Win)) · 8128 갈아엎음 19:30:01(ad5b7db → d08ddfc) · 빈 칸 = 안 지나감 · CID_133~139 새 항목 · S6 Fail 은 플랜에 조건·내용 전달</t>
         </is>
       </c>
     </row>
@@ -404,14 +410,15 @@
       <c r="R7" s="2"/>
       <c r="S7" s="2"/>
       <c r="T7" s="2"/>
-      <c r="U7" s="2" t="inlineStr">
+      <c r="U7" s="2"/>
+      <c r="V7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">버전</t>
         </is>
       </c>
-      <c r="V7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">983f3f6</t>
+      <c r="W7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">d08ddfc</t>
         </is>
       </c>
     </row>
@@ -506,11 +513,16 @@
       </c>
       <c r="U8" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">d08ddfc</t>
+        </is>
+      </c>
+      <c r="V8" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">PASSrate</t>
         </is>
       </c>
-      <c r="V8" s="7">
-        <f>COUNTIF(T9:T140,"Pass")</f>
+      <c r="W8" s="7">
+        <f>COUNTIF(U9:U147,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -594,13 +606,14 @@
       <c r="R9" s="7"/>
       <c r="S9" s="7"/>
       <c r="T9" s="7"/>
-      <c r="U9" s="2" t="inlineStr">
+      <c r="U9" s="7"/>
+      <c r="V9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FAILrate</t>
         </is>
       </c>
-      <c r="V9" s="7">
-        <f>COUNTIF(T9:T140,"Fail")+COUNTIF(T9:T140,"Broken")</f>
+      <c r="W9" s="7">
+        <f>COUNTIF(U9:U147,"Fail")+COUNTIF(U9:U147,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -648,13 +661,14 @@
       <c r="R10" s="7"/>
       <c r="S10" s="7"/>
       <c r="T10" s="7"/>
-      <c r="U10" s="2" t="inlineStr">
+      <c r="U10" s="7"/>
+      <c r="V10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">N/A</t>
         </is>
       </c>
-      <c r="V10" s="7">
-        <f>COUNTIF(T9:T140,"N/A")</f>
+      <c r="W10" s="7">
+        <f>COUNTIF(U9:U147,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -702,13 +716,14 @@
       <c r="R11" s="7"/>
       <c r="S11" s="7"/>
       <c r="T11" s="7"/>
-      <c r="U11" s="2" t="inlineStr">
+      <c r="U11" s="7"/>
+      <c r="V11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">전체 개수</t>
         </is>
       </c>
-      <c r="V11" s="7">
-        <v>132</v>
+      <c r="W11" s="7">
+        <v>139</v>
       </c>
     </row>
     <row r="12">
@@ -756,13 +771,14 @@
       <c r="R12" s="7"/>
       <c r="S12" s="7"/>
       <c r="T12" s="7"/>
-      <c r="U12" s="2" t="inlineStr">
+      <c r="U12" s="7"/>
+      <c r="V12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">진행율</t>
         </is>
       </c>
-      <c r="V12" s="7">
-        <f>TEXT((COUNTA(T9:T140))/132,"0.00%")</f>
+      <c r="W12" s="7">
+        <f>TEXT((COUNTA(U9:U147))/139,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -814,6 +830,7 @@
       <c r="R13" s="7"/>
       <c r="S13" s="7"/>
       <c r="T13" s="7"/>
+      <c r="U13" s="7"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -855,6 +872,7 @@
       <c r="R14" s="7"/>
       <c r="S14" s="7"/>
       <c r="T14" s="7"/>
+      <c r="U14" s="7"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -932,6 +950,7 @@
       <c r="R15" s="7"/>
       <c r="S15" s="7"/>
       <c r="T15" s="7"/>
+      <c r="U15" s="7"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -1009,6 +1028,7 @@
       <c r="R16" s="7"/>
       <c r="S16" s="7"/>
       <c r="T16" s="7"/>
+      <c r="U16" s="7"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -1091,6 +1111,7 @@
       <c r="R17" s="7"/>
       <c r="S17" s="7"/>
       <c r="T17" s="7"/>
+      <c r="U17" s="7"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -1137,6 +1158,7 @@
       <c r="R18" s="7"/>
       <c r="S18" s="7"/>
       <c r="T18" s="7"/>
+      <c r="U18" s="7"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -1178,6 +1200,7 @@
       <c r="R19" s="7"/>
       <c r="S19" s="7"/>
       <c r="T19" s="7"/>
+      <c r="U19" s="7"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1219,6 +1242,7 @@
       <c r="R20" s="7"/>
       <c r="S20" s="7"/>
       <c r="T20" s="7"/>
+      <c r="U20" s="7"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1296,6 +1320,7 @@
       <c r="R21" s="7"/>
       <c r="S21" s="7"/>
       <c r="T21" s="7"/>
+      <c r="U21" s="7"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1366,6 +1391,7 @@
       <c r="R22" s="7"/>
       <c r="S22" s="7"/>
       <c r="T22" s="7"/>
+      <c r="U22" s="7"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -1415,6 +1441,7 @@
       <c r="R23" s="7"/>
       <c r="S23" s="7"/>
       <c r="T23" s="7"/>
+      <c r="U23" s="7"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -1456,6 +1483,7 @@
       <c r="R24" s="7"/>
       <c r="S24" s="7"/>
       <c r="T24" s="7"/>
+      <c r="U24" s="7"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -1497,6 +1525,7 @@
       <c r="R25" s="7"/>
       <c r="S25" s="7"/>
       <c r="T25" s="7"/>
+      <c r="U25" s="7"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -1567,6 +1596,7 @@
       <c r="R26" s="7"/>
       <c r="S26" s="7"/>
       <c r="T26" s="7"/>
+      <c r="U26" s="7"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -1612,6 +1642,7 @@
       <c r="R27" s="7"/>
       <c r="S27" s="7"/>
       <c r="T27" s="7"/>
+      <c r="U27" s="7"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -1666,6 +1697,7 @@
       <c r="R28" s="7"/>
       <c r="S28" s="7"/>
       <c r="T28" s="7"/>
+      <c r="U28" s="7"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -1715,6 +1747,7 @@
       <c r="R29" s="7"/>
       <c r="S29" s="7"/>
       <c r="T29" s="7"/>
+      <c r="U29" s="7"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -1788,6 +1821,7 @@
       <c r="R30" s="7"/>
       <c r="S30" s="7"/>
       <c r="T30" s="7"/>
+      <c r="U30" s="7"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -1866,6 +1900,7 @@
       <c r="R31" s="7"/>
       <c r="S31" s="7"/>
       <c r="T31" s="7"/>
+      <c r="U31" s="7"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -1931,6 +1966,7 @@
       <c r="R32" s="7"/>
       <c r="S32" s="7"/>
       <c r="T32" s="7"/>
+      <c r="U32" s="7"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -2004,6 +2040,7 @@
       <c r="R33" s="7"/>
       <c r="S33" s="7"/>
       <c r="T33" s="7"/>
+      <c r="U33" s="7"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -2077,6 +2114,7 @@
       <c r="R34" s="7"/>
       <c r="S34" s="7"/>
       <c r="T34" s="7"/>
+      <c r="U34" s="7"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -2155,6 +2193,7 @@
       <c r="R35" s="7"/>
       <c r="S35" s="7"/>
       <c r="T35" s="7"/>
+      <c r="U35" s="7"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -2212,6 +2251,7 @@
       <c r="R36" s="7"/>
       <c r="S36" s="7"/>
       <c r="T36" s="7"/>
+      <c r="U36" s="7"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -2253,6 +2293,7 @@
       <c r="R37" s="7"/>
       <c r="S37" s="7"/>
       <c r="T37" s="7"/>
+      <c r="U37" s="7"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -2315,6 +2356,7 @@
       <c r="R38" s="7"/>
       <c r="S38" s="7"/>
       <c r="T38" s="7"/>
+      <c r="U38" s="7"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -2388,6 +2430,7 @@
       <c r="R39" s="7"/>
       <c r="S39" s="7"/>
       <c r="T39" s="7"/>
+      <c r="U39" s="7"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -2462,6 +2505,7 @@
       <c r="R40" s="7"/>
       <c r="S40" s="7"/>
       <c r="T40" s="7"/>
+      <c r="U40" s="7"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -2531,6 +2575,7 @@
       <c r="R41" s="7"/>
       <c r="S41" s="7"/>
       <c r="T41" s="7"/>
+      <c r="U41" s="7"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -2584,6 +2629,7 @@
       <c r="R42" s="7"/>
       <c r="S42" s="7"/>
       <c r="T42" s="7"/>
+      <c r="U42" s="7"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -2657,6 +2703,7 @@
       <c r="R43" s="7"/>
       <c r="S43" s="7"/>
       <c r="T43" s="7"/>
+      <c r="U43" s="7"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -2703,6 +2750,7 @@
       <c r="R44" s="7"/>
       <c r="S44" s="7"/>
       <c r="T44" s="7"/>
+      <c r="U44" s="7"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -2772,6 +2820,7 @@
       <c r="R45" s="7"/>
       <c r="S45" s="7"/>
       <c r="T45" s="7"/>
+      <c r="U45" s="7"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -2841,6 +2890,7 @@
       <c r="R46" s="7"/>
       <c r="S46" s="7"/>
       <c r="T46" s="7"/>
+      <c r="U46" s="7"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -2887,6 +2937,7 @@
       <c r="R47" s="7"/>
       <c r="S47" s="7"/>
       <c r="T47" s="7"/>
+      <c r="U47" s="7"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -2928,6 +2979,7 @@
       <c r="R48" s="7"/>
       <c r="S48" s="7"/>
       <c r="T48" s="7"/>
+      <c r="U48" s="7"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -2969,6 +3021,7 @@
       <c r="R49" s="7"/>
       <c r="S49" s="7"/>
       <c r="T49" s="7"/>
+      <c r="U49" s="7"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -3034,6 +3087,7 @@
       <c r="R50" s="7"/>
       <c r="S50" s="7"/>
       <c r="T50" s="7"/>
+      <c r="U50" s="7"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -3099,6 +3153,7 @@
       <c r="R51" s="7"/>
       <c r="S51" s="7"/>
       <c r="T51" s="7"/>
+      <c r="U51" s="7"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -3145,6 +3200,7 @@
       <c r="R52" s="7"/>
       <c r="S52" s="7"/>
       <c r="T52" s="7"/>
+      <c r="U52" s="7"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -3191,6 +3247,7 @@
       <c r="R53" s="7"/>
       <c r="S53" s="7"/>
       <c r="T53" s="7"/>
+      <c r="U53" s="7"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -3232,6 +3289,7 @@
       <c r="R54" s="7"/>
       <c r="S54" s="7"/>
       <c r="T54" s="7"/>
+      <c r="U54" s="7"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -3309,6 +3367,7 @@
       <c r="R55" s="7"/>
       <c r="S55" s="7"/>
       <c r="T55" s="7"/>
+      <c r="U55" s="7"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -3366,6 +3425,7 @@
       <c r="R56" s="7"/>
       <c r="S56" s="7"/>
       <c r="T56" s="7"/>
+      <c r="U56" s="7"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -3432,6 +3492,7 @@
       <c r="R57" s="7"/>
       <c r="S57" s="7"/>
       <c r="T57" s="7"/>
+      <c r="U57" s="7"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -3506,6 +3567,7 @@
       <c r="R58" s="7"/>
       <c r="S58" s="7"/>
       <c r="T58" s="7"/>
+      <c r="U58" s="7"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -3547,6 +3609,7 @@
       <c r="R59" s="7"/>
       <c r="S59" s="7"/>
       <c r="T59" s="7"/>
+      <c r="U59" s="7"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -3588,6 +3651,7 @@
       <c r="R60" s="7"/>
       <c r="S60" s="7"/>
       <c r="T60" s="7"/>
+      <c r="U60" s="7"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -3641,6 +3705,7 @@
       <c r="R61" s="7"/>
       <c r="S61" s="7"/>
       <c r="T61" s="7"/>
+      <c r="U61" s="7"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -3702,6 +3767,7 @@
       <c r="R62" s="7"/>
       <c r="S62" s="7"/>
       <c r="T62" s="7"/>
+      <c r="U62" s="7"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -3755,6 +3821,7 @@
       <c r="R63" s="7"/>
       <c r="S63" s="7"/>
       <c r="T63" s="7"/>
+      <c r="U63" s="7"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -3796,6 +3863,7 @@
       <c r="R64" s="7"/>
       <c r="S64" s="7"/>
       <c r="T64" s="7"/>
+      <c r="U64" s="7"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -3842,6 +3910,7 @@
       <c r="R65" s="7"/>
       <c r="S65" s="7"/>
       <c r="T65" s="7"/>
+      <c r="U65" s="7"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
@@ -3895,6 +3964,7 @@
       <c r="R66" s="7"/>
       <c r="S66" s="7"/>
       <c r="T66" s="7"/>
+      <c r="U66" s="7"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -3936,6 +4006,7 @@
       <c r="R67" s="7"/>
       <c r="S67" s="7"/>
       <c r="T67" s="7"/>
+      <c r="U67" s="7"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
@@ -3981,6 +4052,7 @@
       <c r="R68" s="7"/>
       <c r="S68" s="7"/>
       <c r="T68" s="7"/>
+      <c r="U68" s="7"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -4058,6 +4130,7 @@
       <c r="R69" s="7"/>
       <c r="S69" s="7"/>
       <c r="T69" s="7"/>
+      <c r="U69" s="7"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
@@ -4099,6 +4172,7 @@
       <c r="R70" s="7"/>
       <c r="S70" s="7"/>
       <c r="T70" s="7"/>
+      <c r="U70" s="7"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -4145,6 +4219,7 @@
       <c r="R71" s="7"/>
       <c r="S71" s="7"/>
       <c r="T71" s="7"/>
+      <c r="U71" s="7"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
@@ -4202,6 +4277,7 @@
       <c r="R72" s="7"/>
       <c r="S72" s="7"/>
       <c r="T72" s="7"/>
+      <c r="U72" s="7"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
@@ -4248,6 +4324,7 @@
       <c r="R73" s="7"/>
       <c r="S73" s="7"/>
       <c r="T73" s="7"/>
+      <c r="U73" s="7"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -4289,6 +4366,7 @@
       <c r="R74" s="7"/>
       <c r="S74" s="7"/>
       <c r="T74" s="7"/>
+      <c r="U74" s="7"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -4330,6 +4408,7 @@
       <c r="R75" s="7"/>
       <c r="S75" s="7"/>
       <c r="T75" s="7"/>
+      <c r="U75" s="7"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -4371,6 +4450,7 @@
       <c r="R76" s="7"/>
       <c r="S76" s="7"/>
       <c r="T76" s="7"/>
+      <c r="U76" s="7"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -4416,6 +4496,7 @@
       <c r="R77" s="7"/>
       <c r="S77" s="7"/>
       <c r="T77" s="7"/>
+      <c r="U77" s="7"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
@@ -4457,6 +4538,7 @@
       <c r="R78" s="7"/>
       <c r="S78" s="7"/>
       <c r="T78" s="7"/>
+      <c r="U78" s="7"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -4503,6 +4585,7 @@
       <c r="R79" s="7"/>
       <c r="S79" s="7"/>
       <c r="T79" s="7"/>
+      <c r="U79" s="7"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
@@ -4560,6 +4643,7 @@
       <c r="R80" s="7"/>
       <c r="S80" s="7"/>
       <c r="T80" s="7"/>
+      <c r="U80" s="7"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
@@ -4601,6 +4685,7 @@
       <c r="R81" s="7"/>
       <c r="S81" s="7"/>
       <c r="T81" s="7"/>
+      <c r="U81" s="7"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
@@ -4642,6 +4727,7 @@
       <c r="R82" s="7"/>
       <c r="S82" s="7"/>
       <c r="T82" s="7"/>
+      <c r="U82" s="7"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
@@ -4688,6 +4774,7 @@
       <c r="R83" s="7"/>
       <c r="S83" s="7"/>
       <c r="T83" s="7"/>
+      <c r="U83" s="7"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
@@ -4729,6 +4816,7 @@
       <c r="R84" s="7"/>
       <c r="S84" s="7"/>
       <c r="T84" s="7"/>
+      <c r="U84" s="7"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
@@ -4770,6 +4858,7 @@
       <c r="R85" s="7"/>
       <c r="S85" s="7"/>
       <c r="T85" s="7"/>
+      <c r="U85" s="7"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
@@ -4816,6 +4905,7 @@
       <c r="R86" s="7"/>
       <c r="S86" s="7"/>
       <c r="T86" s="7"/>
+      <c r="U86" s="7"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
@@ -4857,6 +4947,7 @@
       <c r="R87" s="7"/>
       <c r="S87" s="7"/>
       <c r="T87" s="7"/>
+      <c r="U87" s="7"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
@@ -4898,6 +4989,7 @@
       <c r="R88" s="7"/>
       <c r="S88" s="7"/>
       <c r="T88" s="7"/>
+      <c r="U88" s="7"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
@@ -4939,6 +5031,7 @@
       <c r="R89" s="7"/>
       <c r="S89" s="7"/>
       <c r="T89" s="7"/>
+      <c r="U89" s="7"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
@@ -5009,6 +5102,7 @@
       <c r="R90" s="7"/>
       <c r="S90" s="7"/>
       <c r="T90" s="7"/>
+      <c r="U90" s="7"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
@@ -5050,6 +5144,7 @@
       <c r="R91" s="7"/>
       <c r="S91" s="7"/>
       <c r="T91" s="7"/>
+      <c r="U91" s="7"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
@@ -5127,6 +5222,7 @@
       <c r="R92" s="7"/>
       <c r="S92" s="7"/>
       <c r="T92" s="7"/>
+      <c r="U92" s="7"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
@@ -5209,6 +5305,7 @@
       <c r="R93" s="7"/>
       <c r="S93" s="7"/>
       <c r="T93" s="7"/>
+      <c r="U93" s="7"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
@@ -5255,6 +5352,7 @@
       <c r="R94" s="7"/>
       <c r="S94" s="7"/>
       <c r="T94" s="7"/>
+      <c r="U94" s="7"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
@@ -5301,6 +5399,7 @@
       <c r="R95" s="7"/>
       <c r="S95" s="7"/>
       <c r="T95" s="7"/>
+      <c r="U95" s="7"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
@@ -5366,6 +5465,7 @@
       <c r="R96" s="7"/>
       <c r="S96" s="7"/>
       <c r="T96" s="7"/>
+      <c r="U96" s="7"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="inlineStr">
@@ -5407,6 +5507,7 @@
       <c r="R97" s="7"/>
       <c r="S97" s="7"/>
       <c r="T97" s="7"/>
+      <c r="U97" s="7"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
@@ -5448,6 +5549,7 @@
       <c r="R98" s="7"/>
       <c r="S98" s="7"/>
       <c r="T98" s="7"/>
+      <c r="U98" s="7"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
@@ -5489,6 +5591,7 @@
       <c r="R99" s="7"/>
       <c r="S99" s="7"/>
       <c r="T99" s="7"/>
+      <c r="U99" s="7"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
@@ -5539,6 +5642,7 @@
       <c r="R100" s="7"/>
       <c r="S100" s="7"/>
       <c r="T100" s="7"/>
+      <c r="U100" s="7"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
@@ -5580,6 +5684,7 @@
       <c r="R101" s="7"/>
       <c r="S101" s="7"/>
       <c r="T101" s="7"/>
+      <c r="U101" s="7"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
@@ -5621,6 +5726,7 @@
       <c r="R102" s="7"/>
       <c r="S102" s="7"/>
       <c r="T102" s="7"/>
+      <c r="U102" s="7"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="inlineStr">
@@ -5662,6 +5768,7 @@
       <c r="R103" s="7"/>
       <c r="S103" s="7"/>
       <c r="T103" s="7"/>
+      <c r="U103" s="7"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="inlineStr">
@@ -5708,6 +5815,7 @@
       <c r="R104" s="7"/>
       <c r="S104" s="7"/>
       <c r="T104" s="7"/>
+      <c r="U104" s="7"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
@@ -5749,6 +5857,7 @@
       <c r="R105" s="7"/>
       <c r="S105" s="7"/>
       <c r="T105" s="7"/>
+      <c r="U105" s="7"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
@@ -5790,6 +5899,7 @@
       <c r="R106" s="7"/>
       <c r="S106" s="7"/>
       <c r="T106" s="7"/>
+      <c r="U106" s="7"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
@@ -5831,6 +5941,7 @@
       <c r="R107" s="7"/>
       <c r="S107" s="7"/>
       <c r="T107" s="7"/>
+      <c r="U107" s="7"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
@@ -5876,6 +5987,7 @@
       <c r="R108" s="7"/>
       <c r="S108" s="7"/>
       <c r="T108" s="7"/>
+      <c r="U108" s="7"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="inlineStr">
@@ -5926,6 +6038,7 @@
       <c r="R109" s="7"/>
       <c r="S109" s="7"/>
       <c r="T109" s="7"/>
+      <c r="U109" s="7"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
@@ -5984,6 +6097,7 @@
       <c r="R110" s="7"/>
       <c r="S110" s="7"/>
       <c r="T110" s="7"/>
+      <c r="U110" s="7"/>
     </row>
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
@@ -6045,6 +6159,7 @@
       <c r="R111" s="7"/>
       <c r="S111" s="7"/>
       <c r="T111" s="7"/>
+      <c r="U111" s="7"/>
     </row>
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
@@ -6103,6 +6218,7 @@
       <c r="R112" s="7"/>
       <c r="S112" s="7"/>
       <c r="T112" s="7"/>
+      <c r="U112" s="7"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
@@ -6153,6 +6269,7 @@
       <c r="R113" s="7"/>
       <c r="S113" s="7"/>
       <c r="T113" s="7"/>
+      <c r="U113" s="7"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="inlineStr">
@@ -6219,6 +6336,7 @@
       <c r="R114" s="7"/>
       <c r="S114" s="7"/>
       <c r="T114" s="7"/>
+      <c r="U114" s="7"/>
     </row>
     <row r="115">
       <c r="A115" s="7" t="inlineStr">
@@ -6277,6 +6395,7 @@
       <c r="R115" s="7"/>
       <c r="S115" s="7"/>
       <c r="T115" s="7"/>
+      <c r="U115" s="7"/>
     </row>
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
@@ -6339,6 +6458,7 @@
       <c r="R116" s="7"/>
       <c r="S116" s="7"/>
       <c r="T116" s="7"/>
+      <c r="U116" s="7"/>
     </row>
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
@@ -6401,6 +6521,7 @@
       <c r="R117" s="7"/>
       <c r="S117" s="7"/>
       <c r="T117" s="7"/>
+      <c r="U117" s="7"/>
     </row>
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
@@ -6463,6 +6584,7 @@
       <c r="R118" s="7"/>
       <c r="S118" s="7"/>
       <c r="T118" s="7"/>
+      <c r="U118" s="7"/>
     </row>
     <row r="119">
       <c r="A119" s="7" t="inlineStr">
@@ -6521,6 +6643,7 @@
       <c r="R119" s="7"/>
       <c r="S119" s="7"/>
       <c r="T119" s="7"/>
+      <c r="U119" s="7"/>
     </row>
     <row r="120">
       <c r="A120" s="7" t="inlineStr">
@@ -6571,6 +6694,7 @@
       <c r="R120" s="7"/>
       <c r="S120" s="7"/>
       <c r="T120" s="7"/>
+      <c r="U120" s="7"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="inlineStr">
@@ -6633,6 +6757,7 @@
       <c r="R121" s="7"/>
       <c r="S121" s="7"/>
       <c r="T121" s="7"/>
+      <c r="U121" s="7"/>
     </row>
     <row r="122">
       <c r="A122" s="7" t="inlineStr">
@@ -6695,6 +6820,7 @@
       <c r="R122" s="7"/>
       <c r="S122" s="7"/>
       <c r="T122" s="7"/>
+      <c r="U122" s="7"/>
     </row>
     <row r="123">
       <c r="A123" s="7" t="inlineStr">
@@ -6745,6 +6871,7 @@
       <c r="R123" s="7"/>
       <c r="S123" s="7"/>
       <c r="T123" s="7"/>
+      <c r="U123" s="7"/>
     </row>
     <row r="124">
       <c r="A124" s="7" t="inlineStr">
@@ -6803,6 +6930,7 @@
       <c r="R124" s="7"/>
       <c r="S124" s="7"/>
       <c r="T124" s="7"/>
+      <c r="U124" s="7"/>
     </row>
     <row r="125">
       <c r="A125" s="7" t="inlineStr">
@@ -6853,6 +6981,7 @@
       <c r="R125" s="7"/>
       <c r="S125" s="7"/>
       <c r="T125" s="7"/>
+      <c r="U125" s="7"/>
     </row>
     <row r="126">
       <c r="A126" s="7" t="inlineStr">
@@ -6903,6 +7032,7 @@
       <c r="R126" s="7"/>
       <c r="S126" s="7"/>
       <c r="T126" s="7"/>
+      <c r="U126" s="7"/>
     </row>
     <row r="127">
       <c r="A127" s="7" t="inlineStr">
@@ -6957,6 +7087,7 @@
       <c r="R127" s="7"/>
       <c r="S127" s="7"/>
       <c r="T127" s="7"/>
+      <c r="U127" s="7"/>
     </row>
     <row r="128">
       <c r="A128" s="7" t="inlineStr">
@@ -7011,6 +7142,7 @@
       <c r="R128" s="7"/>
       <c r="S128" s="7"/>
       <c r="T128" s="7"/>
+      <c r="U128" s="7"/>
     </row>
     <row r="129">
       <c r="A129" s="7" t="inlineStr">
@@ -7065,6 +7197,7 @@
       <c r="R129" s="7"/>
       <c r="S129" s="7"/>
       <c r="T129" s="7"/>
+      <c r="U129" s="7"/>
     </row>
     <row r="130">
       <c r="A130" s="7" t="inlineStr">
@@ -7115,6 +7248,7 @@
       <c r="R130" s="7"/>
       <c r="S130" s="7"/>
       <c r="T130" s="7"/>
+      <c r="U130" s="7"/>
     </row>
     <row r="131">
       <c r="A131" s="7" t="inlineStr">
@@ -7169,6 +7303,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="U131" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="7" t="inlineStr">
@@ -7227,6 +7366,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="U132" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="7" t="inlineStr">
@@ -7281,6 +7425,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="U133" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
@@ -7339,6 +7488,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="U134" s="7"/>
     </row>
     <row r="135">
       <c r="A135" s="7" t="inlineStr">
@@ -7393,6 +7543,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="U135" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="7" t="inlineStr">
@@ -7443,6 +7598,11 @@
         </is>
       </c>
       <c r="T136" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="U136" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -7497,6 +7657,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="U137" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="7" t="inlineStr">
@@ -7547,6 +7712,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="U138" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="7" t="inlineStr">
@@ -7597,6 +7767,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="U139" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="7" t="inlineStr">
@@ -7645,6 +7820,364 @@
       <c r="T140" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="U140" s="7"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_133</t>
+        </is>
+      </c>
+      <c r="B141" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C141" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도전</t>
+        </is>
+      </c>
+      <c r="D141" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">안내 창</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">「도전」·「다시 도전」을 누르면 바로 안 들어가고 「도전 시작 / 지금 마운트에 실린 물류를 그대로 가지고 도전합니다 / 로봇 A 마운트 탄환 n/40 / (B 해금 뒤) 로봇 B 마운트 드론 n/40 · 합체 게이지 n%」 창이 뜨고 [도전 시작]을 눌러야 들어가는가? [취소]는 닫는가?</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">사용자 직접 지시 10-16 · 글자 가정</t>
+        </is>
+      </c>
+      <c r="G141" s="7"/>
+      <c r="H141" s="7"/>
+      <c r="I141" s="7"/>
+      <c r="J141" s="7"/>
+      <c r="K141" s="7"/>
+      <c r="L141" s="7"/>
+      <c r="M141" s="7"/>
+      <c r="N141" s="7"/>
+      <c r="O141" s="7"/>
+      <c r="P141" s="7"/>
+      <c r="Q141" s="7"/>
+      <c r="R141" s="7"/>
+      <c r="S141" s="7"/>
+      <c r="T141" s="7"/>
+      <c r="U141" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_134</t>
+        </is>
+      </c>
+      <c r="B142" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C142" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도전</t>
+        </is>
+      </c>
+      <c r="D142" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">물류 유지</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도전에 들어가도 로봇 A 마운트 탄환·로봇 B 마운트 드론이 들어가기 직전 양 그대로인가?</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">사용자 직접 지시 10-16 · 콘솔 로그 「들어가기 전」=「들고 온」</t>
+        </is>
+      </c>
+      <c r="G142" s="7"/>
+      <c r="H142" s="7"/>
+      <c r="I142" s="7"/>
+      <c r="J142" s="7"/>
+      <c r="K142" s="7"/>
+      <c r="L142" s="7"/>
+      <c r="M142" s="7"/>
+      <c r="N142" s="7"/>
+      <c r="O142" s="7"/>
+      <c r="P142" s="7"/>
+      <c r="Q142" s="7"/>
+      <c r="R142" s="7"/>
+      <c r="S142" s="7"/>
+      <c r="T142" s="7"/>
+      <c r="U142" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_135</t>
+        </is>
+      </c>
+      <c r="B143" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C143" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">합체</t>
+        </is>
+      </c>
+      <c r="D143" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">게이지 이어 감</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">합체 게이지가 파밍→도전 · 다음 스테이지로 등 판이 바뀌어도 이어지고, 새로고침 뒤에도 남는가? 합체를 쓰거나 「처음부터」면 0 인가?</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#155</t>
+        </is>
+      </c>
+      <c r="G143" s="7"/>
+      <c r="H143" s="7"/>
+      <c r="I143" s="7"/>
+      <c r="J143" s="7"/>
+      <c r="K143" s="7"/>
+      <c r="L143" s="7"/>
+      <c r="M143" s="7"/>
+      <c r="N143" s="7"/>
+      <c r="O143" s="7"/>
+      <c r="P143" s="7"/>
+      <c r="Q143" s="7"/>
+      <c r="R143" s="7"/>
+      <c r="S143" s="7"/>
+      <c r="T143" s="7"/>
+      <c r="U143" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_136</t>
+        </is>
+      </c>
+      <c r="B144" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼</t>
+        </is>
+      </c>
+      <c r="C144" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T3</t>
+        </is>
+      </c>
+      <c r="D144" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">안내 창</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T3(첫 도전 안내) 국면에서 「도전」을 누르면 흐림막 위에 안내 창이 뜨고 [도전 시작] 하나만 있는가?</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#155 결 · 취소 숨김(구현 판단)</t>
+        </is>
+      </c>
+      <c r="G144" s="7"/>
+      <c r="H144" s="7"/>
+      <c r="I144" s="7"/>
+      <c r="J144" s="7"/>
+      <c r="K144" s="7"/>
+      <c r="L144" s="7"/>
+      <c r="M144" s="7"/>
+      <c r="N144" s="7"/>
+      <c r="O144" s="7"/>
+      <c r="P144" s="7"/>
+      <c r="Q144" s="7"/>
+      <c r="R144" s="7"/>
+      <c r="S144" s="7"/>
+      <c r="T144" s="7"/>
+      <c r="U144" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_137</t>
+        </is>
+      </c>
+      <c r="B145" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">설정</t>
+        </is>
+      </c>
+      <c r="C145" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">바로가기</t>
+        </is>
+      </c>
+      <c r="D145" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">만충 진입</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t xml:space="preserve">설정 바로가기(S1~S6)로 판을 옮기면 로봇 A·B 마운트가 가득(40/40 · 40/40)이고 합체 게이지는 그대로인가? 튜토리얼 점프는 안 채우는가?</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#156</t>
+        </is>
+      </c>
+      <c r="G145" s="7"/>
+      <c r="H145" s="7"/>
+      <c r="I145" s="7"/>
+      <c r="J145" s="7"/>
+      <c r="K145" s="7"/>
+      <c r="L145" s="7"/>
+      <c r="M145" s="7"/>
+      <c r="N145" s="7"/>
+      <c r="O145" s="7"/>
+      <c r="P145" s="7"/>
+      <c r="Q145" s="7"/>
+      <c r="R145" s="7"/>
+      <c r="S145" s="7"/>
+      <c r="T145" s="7"/>
+      <c r="U145" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_138</t>
+        </is>
+      </c>
+      <c r="B146" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C146" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">합체</t>
+        </is>
+      </c>
+      <c r="D146" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B 드론</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t xml:space="preserve">합체 중에 A 의 탄과 함께 B 의 드론도 나가는가(A 가 나가 있던 채 합체해도)?</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#157</t>
+        </is>
+      </c>
+      <c r="G146" s="7"/>
+      <c r="H146" s="7"/>
+      <c r="I146" s="7"/>
+      <c r="J146" s="7"/>
+      <c r="K146" s="7"/>
+      <c r="L146" s="7"/>
+      <c r="M146" s="7"/>
+      <c r="N146" s="7"/>
+      <c r="O146" s="7"/>
+      <c r="P146" s="7"/>
+      <c r="Q146" s="7"/>
+      <c r="R146" s="7"/>
+      <c r="S146" s="7"/>
+      <c r="T146" s="7"/>
+      <c r="U146" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_139</t>
+        </is>
+      </c>
+      <c r="B147" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C147" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S6</t>
+        </is>
+      </c>
+      <c r="D147" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">통과</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t xml:space="preserve">강화 뒤 · 마운트 가득으로 S6 도전에서 태그·합체를 쓰면 60초 안에 보스(13500)를 잡는가?</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t xml:space="preserve">하네스 Win(태그 Auto 켬) · 화면 사람 조작 Fail(10-16)</t>
+        </is>
+      </c>
+      <c r="G147" s="7"/>
+      <c r="H147" s="7"/>
+      <c r="I147" s="7"/>
+      <c r="J147" s="7"/>
+      <c r="K147" s="7"/>
+      <c r="L147" s="7"/>
+      <c r="M147" s="7"/>
+      <c r="N147" s="7"/>
+      <c r="O147" s="7"/>
+      <c r="P147" s="7"/>
+      <c r="Q147" s="7"/>
+      <c r="R147" s="7"/>
+      <c r="S147" s="7"/>
+      <c r="T147" s="7"/>
+      <c r="U147" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
         </is>
       </c>
     </row>
@@ -7675,9 +8208,9 @@
     <mergeCell ref="B92:B99"/>
     <mergeCell ref="B100:B106"/>
     <mergeCell ref="B107:B111"/>
-    <mergeCell ref="G7:T7"/>
+    <mergeCell ref="G7:U7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:T140">
+  <conditionalFormatting sqref="G9:U147">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
QA V열(0749886) — #158 재확인 Pass 5 · Fail 0 · CID_140 신설 · CID_139 S6 Pass
8128: Auto 켜진 채 합체만 → S6 승리(남은 00:12). Auto 끄고 태그 안 누르면 시간 초과(예상대로).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -177,8 +177,9 @@
     <col min="19" max="19" width="12" customWidth="1"/>
     <col min="20" max="20" width="12" customWidth="1"/>
     <col min="21" max="21" width="12" customWidth="1"/>
-    <col min="22" max="22" width="11" customWidth="1"/>
+    <col min="22" max="22" width="12" customWidth="1"/>
     <col min="23" max="23" width="11" customWidth="1"/>
+    <col min="24" max="24" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -366,6 +367,11 @@
       <c r="U6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">video-261016 후보 · 사용자 직접 지시 ②③(물류 유지 · 도전 안내 창) · #155 합체 게이지 이어 감 · T3 안내 창 · S6 보스 13500 · #156 바로가기 만충 · #157 합체 중 A 탄 + B 드론 ‖ 10-16 코드 세션 재확인(8128 · 576×1024 · 소리 0 · ad5b7db 판: 처음부터 → 튜토리얼 벨트 이음 → T3 안내 창 [도전 시작] 하나(A 40/40) → S1 승(남 29초) → T4 모듈 → S2 승(남 3초) → S3 자연 승(남 5초) → 강화 → S4 승(남 8초) · 게이지가 판 넘어 차 S4 파밍에서 합체 발동 밝음 · 새로고침 뒤 S6 안내 창 게이지 100% · d08ddfc 판: 8123·8128 바로가기 S6 안내 창 A 40/40 · B 40/40 · 게이지 47%/100% · 태그 → 합체 → 합체 중 B 드론 나감 → S6 시간 초과(보스 약 30% 남음 · 태그 Auto 꺼짐 · 사람이 누름 · 하네스는 Auto 켬으로 Win)) · 8128 갈아엎음 19:30:01(ad5b7db → d08ddfc) · 빈 칸 = 안 지나감 · CID_133~139 새 항목 · S6 Fail 은 플랜에 조건·내용 전달</t>
+        </is>
+      </c>
+      <c r="V6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">video-261016 후보 · #158 태그 Auto 기본 켜짐 ‖ 10-16 코드 세션 재확인(8123 · 8128 · 576×1024 · 소리 0 · 8123: 처음부터 → 바로가기 S6 파밍에서 B 로 저절로 교대(Auto 켜짐) · 8128(강화된 저장): 바로가기 S6 · 게이지 채움 · Auto 켜진 채 그대로 → 도전 7초쯤 합체만 누름 → **승리(남은 00:12)** · Auto 끄고 같은 판(바로가기 만충 · 게이지 채움 · 합체만 누름 · 태그 안 누름) → 남은 00:06 에 보스 약 90% · 시간 초과(사람이 태그를 안 누른 판 · 예상대로)) · 8128 갈아엎음 21:02:33(d08ddfc → 0749886) · 빈 칸 = 안 지나감(T3 영향은 시험·B 해금 문으로 봄 · 화면 미확인) · CID_140 새 항목</t>
         </is>
       </c>
     </row>
@@ -411,14 +417,15 @@
       <c r="S7" s="2"/>
       <c r="T7" s="2"/>
       <c r="U7" s="2"/>
-      <c r="V7" s="2" t="inlineStr">
+      <c r="V7" s="2"/>
+      <c r="W7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">버전</t>
         </is>
       </c>
-      <c r="W7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">d08ddfc</t>
+      <c r="X7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0749886</t>
         </is>
       </c>
     </row>
@@ -518,11 +525,16 @@
       </c>
       <c r="V8" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">0749886</t>
+        </is>
+      </c>
+      <c r="W8" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">PASSrate</t>
         </is>
       </c>
-      <c r="W8" s="7">
-        <f>COUNTIF(U9:U147,"Pass")</f>
+      <c r="X8" s="7">
+        <f>COUNTIF(V9:V148,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -607,13 +619,14 @@
       <c r="S9" s="7"/>
       <c r="T9" s="7"/>
       <c r="U9" s="7"/>
-      <c r="V9" s="2" t="inlineStr">
+      <c r="V9" s="7"/>
+      <c r="W9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FAILrate</t>
         </is>
       </c>
-      <c r="W9" s="7">
-        <f>COUNTIF(U9:U147,"Fail")+COUNTIF(U9:U147,"Broken")</f>
+      <c r="X9" s="7">
+        <f>COUNTIF(V9:V148,"Fail")+COUNTIF(V9:V148,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -662,13 +675,14 @@
       <c r="S10" s="7"/>
       <c r="T10" s="7"/>
       <c r="U10" s="7"/>
-      <c r="V10" s="2" t="inlineStr">
+      <c r="V10" s="7"/>
+      <c r="W10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">N/A</t>
         </is>
       </c>
-      <c r="W10" s="7">
-        <f>COUNTIF(U9:U147,"N/A")</f>
+      <c r="X10" s="7">
+        <f>COUNTIF(V9:V148,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -717,13 +731,14 @@
       <c r="S11" s="7"/>
       <c r="T11" s="7"/>
       <c r="U11" s="7"/>
-      <c r="V11" s="2" t="inlineStr">
+      <c r="V11" s="7"/>
+      <c r="W11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">전체 개수</t>
         </is>
       </c>
-      <c r="W11" s="7">
-        <v>139</v>
+      <c r="X11" s="7">
+        <v>140</v>
       </c>
     </row>
     <row r="12">
@@ -772,13 +787,14 @@
       <c r="S12" s="7"/>
       <c r="T12" s="7"/>
       <c r="U12" s="7"/>
-      <c r="V12" s="2" t="inlineStr">
+      <c r="V12" s="7"/>
+      <c r="W12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">진행율</t>
         </is>
       </c>
-      <c r="W12" s="7">
-        <f>TEXT((COUNTA(U9:U147))/139,"0.00%")</f>
+      <c r="X12" s="7">
+        <f>TEXT((COUNTA(V9:V148))/140,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -831,6 +847,7 @@
       <c r="S13" s="7"/>
       <c r="T13" s="7"/>
       <c r="U13" s="7"/>
+      <c r="V13" s="7"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -873,6 +890,7 @@
       <c r="S14" s="7"/>
       <c r="T14" s="7"/>
       <c r="U14" s="7"/>
+      <c r="V14" s="7"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -951,6 +969,7 @@
       <c r="S15" s="7"/>
       <c r="T15" s="7"/>
       <c r="U15" s="7"/>
+      <c r="V15" s="7"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -1029,6 +1048,7 @@
       <c r="S16" s="7"/>
       <c r="T16" s="7"/>
       <c r="U16" s="7"/>
+      <c r="V16" s="7"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -1112,6 +1132,7 @@
       <c r="S17" s="7"/>
       <c r="T17" s="7"/>
       <c r="U17" s="7"/>
+      <c r="V17" s="7"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -1159,6 +1180,7 @@
       <c r="S18" s="7"/>
       <c r="T18" s="7"/>
       <c r="U18" s="7"/>
+      <c r="V18" s="7"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -1201,6 +1223,7 @@
       <c r="S19" s="7"/>
       <c r="T19" s="7"/>
       <c r="U19" s="7"/>
+      <c r="V19" s="7"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1243,6 +1266,7 @@
       <c r="S20" s="7"/>
       <c r="T20" s="7"/>
       <c r="U20" s="7"/>
+      <c r="V20" s="7"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1321,6 +1345,7 @@
       <c r="S21" s="7"/>
       <c r="T21" s="7"/>
       <c r="U21" s="7"/>
+      <c r="V21" s="7"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1392,6 +1417,7 @@
       <c r="S22" s="7"/>
       <c r="T22" s="7"/>
       <c r="U22" s="7"/>
+      <c r="V22" s="7"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -1442,6 +1468,7 @@
       <c r="S23" s="7"/>
       <c r="T23" s="7"/>
       <c r="U23" s="7"/>
+      <c r="V23" s="7"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -1484,6 +1511,7 @@
       <c r="S24" s="7"/>
       <c r="T24" s="7"/>
       <c r="U24" s="7"/>
+      <c r="V24" s="7"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -1526,6 +1554,7 @@
       <c r="S25" s="7"/>
       <c r="T25" s="7"/>
       <c r="U25" s="7"/>
+      <c r="V25" s="7"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -1597,6 +1626,7 @@
       <c r="S26" s="7"/>
       <c r="T26" s="7"/>
       <c r="U26" s="7"/>
+      <c r="V26" s="7"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -1643,6 +1673,7 @@
       <c r="S27" s="7"/>
       <c r="T27" s="7"/>
       <c r="U27" s="7"/>
+      <c r="V27" s="7"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -1698,6 +1729,7 @@
       <c r="S28" s="7"/>
       <c r="T28" s="7"/>
       <c r="U28" s="7"/>
+      <c r="V28" s="7"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -1748,6 +1780,7 @@
       <c r="S29" s="7"/>
       <c r="T29" s="7"/>
       <c r="U29" s="7"/>
+      <c r="V29" s="7"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -1822,6 +1855,7 @@
       <c r="S30" s="7"/>
       <c r="T30" s="7"/>
       <c r="U30" s="7"/>
+      <c r="V30" s="7"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -1901,6 +1935,7 @@
       <c r="S31" s="7"/>
       <c r="T31" s="7"/>
       <c r="U31" s="7"/>
+      <c r="V31" s="7"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -1967,6 +2002,7 @@
       <c r="S32" s="7"/>
       <c r="T32" s="7"/>
       <c r="U32" s="7"/>
+      <c r="V32" s="7"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -2041,6 +2077,7 @@
       <c r="S33" s="7"/>
       <c r="T33" s="7"/>
       <c r="U33" s="7"/>
+      <c r="V33" s="7"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -2115,6 +2152,7 @@
       <c r="S34" s="7"/>
       <c r="T34" s="7"/>
       <c r="U34" s="7"/>
+      <c r="V34" s="7"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -2194,6 +2232,7 @@
       <c r="S35" s="7"/>
       <c r="T35" s="7"/>
       <c r="U35" s="7"/>
+      <c r="V35" s="7"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -2252,6 +2291,7 @@
       <c r="S36" s="7"/>
       <c r="T36" s="7"/>
       <c r="U36" s="7"/>
+      <c r="V36" s="7"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -2294,6 +2334,7 @@
       <c r="S37" s="7"/>
       <c r="T37" s="7"/>
       <c r="U37" s="7"/>
+      <c r="V37" s="7"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -2357,6 +2398,7 @@
       <c r="S38" s="7"/>
       <c r="T38" s="7"/>
       <c r="U38" s="7"/>
+      <c r="V38" s="7"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -2431,6 +2473,7 @@
       <c r="S39" s="7"/>
       <c r="T39" s="7"/>
       <c r="U39" s="7"/>
+      <c r="V39" s="7"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -2506,6 +2549,7 @@
       <c r="S40" s="7"/>
       <c r="T40" s="7"/>
       <c r="U40" s="7"/>
+      <c r="V40" s="7"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -2576,6 +2620,7 @@
       <c r="S41" s="7"/>
       <c r="T41" s="7"/>
       <c r="U41" s="7"/>
+      <c r="V41" s="7"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -2630,6 +2675,7 @@
       <c r="S42" s="7"/>
       <c r="T42" s="7"/>
       <c r="U42" s="7"/>
+      <c r="V42" s="7"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -2704,6 +2750,7 @@
       <c r="S43" s="7"/>
       <c r="T43" s="7"/>
       <c r="U43" s="7"/>
+      <c r="V43" s="7"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -2751,6 +2798,7 @@
       <c r="S44" s="7"/>
       <c r="T44" s="7"/>
       <c r="U44" s="7"/>
+      <c r="V44" s="7"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -2821,6 +2869,7 @@
       <c r="S45" s="7"/>
       <c r="T45" s="7"/>
       <c r="U45" s="7"/>
+      <c r="V45" s="7"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -2891,6 +2940,7 @@
       <c r="S46" s="7"/>
       <c r="T46" s="7"/>
       <c r="U46" s="7"/>
+      <c r="V46" s="7"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -2938,6 +2988,7 @@
       <c r="S47" s="7"/>
       <c r="T47" s="7"/>
       <c r="U47" s="7"/>
+      <c r="V47" s="7"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -2980,6 +3031,7 @@
       <c r="S48" s="7"/>
       <c r="T48" s="7"/>
       <c r="U48" s="7"/>
+      <c r="V48" s="7"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -3022,6 +3074,7 @@
       <c r="S49" s="7"/>
       <c r="T49" s="7"/>
       <c r="U49" s="7"/>
+      <c r="V49" s="7"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -3088,6 +3141,7 @@
       <c r="S50" s="7"/>
       <c r="T50" s="7"/>
       <c r="U50" s="7"/>
+      <c r="V50" s="7"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -3154,6 +3208,7 @@
       <c r="S51" s="7"/>
       <c r="T51" s="7"/>
       <c r="U51" s="7"/>
+      <c r="V51" s="7"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -3201,6 +3256,7 @@
       <c r="S52" s="7"/>
       <c r="T52" s="7"/>
       <c r="U52" s="7"/>
+      <c r="V52" s="7"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -3248,6 +3304,7 @@
       <c r="S53" s="7"/>
       <c r="T53" s="7"/>
       <c r="U53" s="7"/>
+      <c r="V53" s="7"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -3290,6 +3347,7 @@
       <c r="S54" s="7"/>
       <c r="T54" s="7"/>
       <c r="U54" s="7"/>
+      <c r="V54" s="7"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -3368,6 +3426,7 @@
       <c r="S55" s="7"/>
       <c r="T55" s="7"/>
       <c r="U55" s="7"/>
+      <c r="V55" s="7"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -3426,6 +3485,7 @@
       <c r="S56" s="7"/>
       <c r="T56" s="7"/>
       <c r="U56" s="7"/>
+      <c r="V56" s="7"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -3493,6 +3553,7 @@
       <c r="S57" s="7"/>
       <c r="T57" s="7"/>
       <c r="U57" s="7"/>
+      <c r="V57" s="7"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -3568,6 +3629,7 @@
       <c r="S58" s="7"/>
       <c r="T58" s="7"/>
       <c r="U58" s="7"/>
+      <c r="V58" s="7"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -3610,6 +3672,7 @@
       <c r="S59" s="7"/>
       <c r="T59" s="7"/>
       <c r="U59" s="7"/>
+      <c r="V59" s="7"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -3652,6 +3715,7 @@
       <c r="S60" s="7"/>
       <c r="T60" s="7"/>
       <c r="U60" s="7"/>
+      <c r="V60" s="7"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -3706,6 +3770,7 @@
       <c r="S61" s="7"/>
       <c r="T61" s="7"/>
       <c r="U61" s="7"/>
+      <c r="V61" s="7"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -3768,6 +3833,7 @@
       <c r="S62" s="7"/>
       <c r="T62" s="7"/>
       <c r="U62" s="7"/>
+      <c r="V62" s="7"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -3822,6 +3888,7 @@
       <c r="S63" s="7"/>
       <c r="T63" s="7"/>
       <c r="U63" s="7"/>
+      <c r="V63" s="7"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -3864,6 +3931,7 @@
       <c r="S64" s="7"/>
       <c r="T64" s="7"/>
       <c r="U64" s="7"/>
+      <c r="V64" s="7"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -3911,6 +3979,7 @@
       <c r="S65" s="7"/>
       <c r="T65" s="7"/>
       <c r="U65" s="7"/>
+      <c r="V65" s="7"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
@@ -3965,6 +4034,7 @@
       <c r="S66" s="7"/>
       <c r="T66" s="7"/>
       <c r="U66" s="7"/>
+      <c r="V66" s="7"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -4007,6 +4077,7 @@
       <c r="S67" s="7"/>
       <c r="T67" s="7"/>
       <c r="U67" s="7"/>
+      <c r="V67" s="7"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
@@ -4053,6 +4124,7 @@
       <c r="S68" s="7"/>
       <c r="T68" s="7"/>
       <c r="U68" s="7"/>
+      <c r="V68" s="7"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -4131,6 +4203,7 @@
       <c r="S69" s="7"/>
       <c r="T69" s="7"/>
       <c r="U69" s="7"/>
+      <c r="V69" s="7"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
@@ -4173,6 +4246,7 @@
       <c r="S70" s="7"/>
       <c r="T70" s="7"/>
       <c r="U70" s="7"/>
+      <c r="V70" s="7"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -4220,6 +4294,7 @@
       <c r="S71" s="7"/>
       <c r="T71" s="7"/>
       <c r="U71" s="7"/>
+      <c r="V71" s="7"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
@@ -4278,6 +4353,7 @@
       <c r="S72" s="7"/>
       <c r="T72" s="7"/>
       <c r="U72" s="7"/>
+      <c r="V72" s="7"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
@@ -4325,6 +4401,7 @@
       <c r="S73" s="7"/>
       <c r="T73" s="7"/>
       <c r="U73" s="7"/>
+      <c r="V73" s="7"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -4367,6 +4444,7 @@
       <c r="S74" s="7"/>
       <c r="T74" s="7"/>
       <c r="U74" s="7"/>
+      <c r="V74" s="7"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -4409,6 +4487,7 @@
       <c r="S75" s="7"/>
       <c r="T75" s="7"/>
       <c r="U75" s="7"/>
+      <c r="V75" s="7"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -4451,6 +4530,7 @@
       <c r="S76" s="7"/>
       <c r="T76" s="7"/>
       <c r="U76" s="7"/>
+      <c r="V76" s="7"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -4497,6 +4577,7 @@
       <c r="S77" s="7"/>
       <c r="T77" s="7"/>
       <c r="U77" s="7"/>
+      <c r="V77" s="7"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
@@ -4539,6 +4620,7 @@
       <c r="S78" s="7"/>
       <c r="T78" s="7"/>
       <c r="U78" s="7"/>
+      <c r="V78" s="7"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -4586,6 +4668,7 @@
       <c r="S79" s="7"/>
       <c r="T79" s="7"/>
       <c r="U79" s="7"/>
+      <c r="V79" s="7"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
@@ -4644,6 +4727,7 @@
       <c r="S80" s="7"/>
       <c r="T80" s="7"/>
       <c r="U80" s="7"/>
+      <c r="V80" s="7"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
@@ -4686,6 +4770,7 @@
       <c r="S81" s="7"/>
       <c r="T81" s="7"/>
       <c r="U81" s="7"/>
+      <c r="V81" s="7"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
@@ -4728,6 +4813,7 @@
       <c r="S82" s="7"/>
       <c r="T82" s="7"/>
       <c r="U82" s="7"/>
+      <c r="V82" s="7"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
@@ -4775,6 +4861,7 @@
       <c r="S83" s="7"/>
       <c r="T83" s="7"/>
       <c r="U83" s="7"/>
+      <c r="V83" s="7"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
@@ -4817,6 +4904,7 @@
       <c r="S84" s="7"/>
       <c r="T84" s="7"/>
       <c r="U84" s="7"/>
+      <c r="V84" s="7"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
@@ -4859,6 +4947,7 @@
       <c r="S85" s="7"/>
       <c r="T85" s="7"/>
       <c r="U85" s="7"/>
+      <c r="V85" s="7"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
@@ -4906,6 +4995,7 @@
       <c r="S86" s="7"/>
       <c r="T86" s="7"/>
       <c r="U86" s="7"/>
+      <c r="V86" s="7"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
@@ -4948,6 +5038,7 @@
       <c r="S87" s="7"/>
       <c r="T87" s="7"/>
       <c r="U87" s="7"/>
+      <c r="V87" s="7"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
@@ -4990,6 +5081,7 @@
       <c r="S88" s="7"/>
       <c r="T88" s="7"/>
       <c r="U88" s="7"/>
+      <c r="V88" s="7"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
@@ -5032,6 +5124,7 @@
       <c r="S89" s="7"/>
       <c r="T89" s="7"/>
       <c r="U89" s="7"/>
+      <c r="V89" s="7"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
@@ -5103,6 +5196,7 @@
       <c r="S90" s="7"/>
       <c r="T90" s="7"/>
       <c r="U90" s="7"/>
+      <c r="V90" s="7"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
@@ -5145,6 +5239,7 @@
       <c r="S91" s="7"/>
       <c r="T91" s="7"/>
       <c r="U91" s="7"/>
+      <c r="V91" s="7"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
@@ -5223,6 +5318,7 @@
       <c r="S92" s="7"/>
       <c r="T92" s="7"/>
       <c r="U92" s="7"/>
+      <c r="V92" s="7"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
@@ -5306,6 +5402,7 @@
       <c r="S93" s="7"/>
       <c r="T93" s="7"/>
       <c r="U93" s="7"/>
+      <c r="V93" s="7"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
@@ -5353,6 +5450,7 @@
       <c r="S94" s="7"/>
       <c r="T94" s="7"/>
       <c r="U94" s="7"/>
+      <c r="V94" s="7"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
@@ -5400,6 +5498,7 @@
       <c r="S95" s="7"/>
       <c r="T95" s="7"/>
       <c r="U95" s="7"/>
+      <c r="V95" s="7"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
@@ -5466,6 +5565,7 @@
       <c r="S96" s="7"/>
       <c r="T96" s="7"/>
       <c r="U96" s="7"/>
+      <c r="V96" s="7"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="inlineStr">
@@ -5508,6 +5608,7 @@
       <c r="S97" s="7"/>
       <c r="T97" s="7"/>
       <c r="U97" s="7"/>
+      <c r="V97" s="7"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
@@ -5550,6 +5651,7 @@
       <c r="S98" s="7"/>
       <c r="T98" s="7"/>
       <c r="U98" s="7"/>
+      <c r="V98" s="7"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
@@ -5592,6 +5694,7 @@
       <c r="S99" s="7"/>
       <c r="T99" s="7"/>
       <c r="U99" s="7"/>
+      <c r="V99" s="7"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
@@ -5643,6 +5746,7 @@
       <c r="S100" s="7"/>
       <c r="T100" s="7"/>
       <c r="U100" s="7"/>
+      <c r="V100" s="7"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
@@ -5685,6 +5789,7 @@
       <c r="S101" s="7"/>
       <c r="T101" s="7"/>
       <c r="U101" s="7"/>
+      <c r="V101" s="7"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
@@ -5727,6 +5832,7 @@
       <c r="S102" s="7"/>
       <c r="T102" s="7"/>
       <c r="U102" s="7"/>
+      <c r="V102" s="7"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="inlineStr">
@@ -5769,6 +5875,7 @@
       <c r="S103" s="7"/>
       <c r="T103" s="7"/>
       <c r="U103" s="7"/>
+      <c r="V103" s="7"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="inlineStr">
@@ -5816,6 +5923,7 @@
       <c r="S104" s="7"/>
       <c r="T104" s="7"/>
       <c r="U104" s="7"/>
+      <c r="V104" s="7"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
@@ -5858,6 +5966,7 @@
       <c r="S105" s="7"/>
       <c r="T105" s="7"/>
       <c r="U105" s="7"/>
+      <c r="V105" s="7"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
@@ -5900,6 +6009,7 @@
       <c r="S106" s="7"/>
       <c r="T106" s="7"/>
       <c r="U106" s="7"/>
+      <c r="V106" s="7"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
@@ -5942,6 +6052,7 @@
       <c r="S107" s="7"/>
       <c r="T107" s="7"/>
       <c r="U107" s="7"/>
+      <c r="V107" s="7"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
@@ -5988,6 +6099,7 @@
       <c r="S108" s="7"/>
       <c r="T108" s="7"/>
       <c r="U108" s="7"/>
+      <c r="V108" s="7"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="inlineStr">
@@ -6039,6 +6151,7 @@
       <c r="S109" s="7"/>
       <c r="T109" s="7"/>
       <c r="U109" s="7"/>
+      <c r="V109" s="7"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
@@ -6098,6 +6211,7 @@
       <c r="S110" s="7"/>
       <c r="T110" s="7"/>
       <c r="U110" s="7"/>
+      <c r="V110" s="7"/>
     </row>
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
@@ -6160,6 +6274,7 @@
       <c r="S111" s="7"/>
       <c r="T111" s="7"/>
       <c r="U111" s="7"/>
+      <c r="V111" s="7"/>
     </row>
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
@@ -6219,6 +6334,7 @@
       <c r="S112" s="7"/>
       <c r="T112" s="7"/>
       <c r="U112" s="7"/>
+      <c r="V112" s="7"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
@@ -6270,6 +6386,7 @@
       <c r="S113" s="7"/>
       <c r="T113" s="7"/>
       <c r="U113" s="7"/>
+      <c r="V113" s="7"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="inlineStr">
@@ -6337,6 +6454,7 @@
       <c r="S114" s="7"/>
       <c r="T114" s="7"/>
       <c r="U114" s="7"/>
+      <c r="V114" s="7"/>
     </row>
     <row r="115">
       <c r="A115" s="7" t="inlineStr">
@@ -6396,6 +6514,7 @@
       <c r="S115" s="7"/>
       <c r="T115" s="7"/>
       <c r="U115" s="7"/>
+      <c r="V115" s="7"/>
     </row>
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
@@ -6459,6 +6578,7 @@
       <c r="S116" s="7"/>
       <c r="T116" s="7"/>
       <c r="U116" s="7"/>
+      <c r="V116" s="7"/>
     </row>
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
@@ -6522,6 +6642,7 @@
       <c r="S117" s="7"/>
       <c r="T117" s="7"/>
       <c r="U117" s="7"/>
+      <c r="V117" s="7"/>
     </row>
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
@@ -6585,6 +6706,7 @@
       <c r="S118" s="7"/>
       <c r="T118" s="7"/>
       <c r="U118" s="7"/>
+      <c r="V118" s="7"/>
     </row>
     <row r="119">
       <c r="A119" s="7" t="inlineStr">
@@ -6644,6 +6766,7 @@
       <c r="S119" s="7"/>
       <c r="T119" s="7"/>
       <c r="U119" s="7"/>
+      <c r="V119" s="7"/>
     </row>
     <row r="120">
       <c r="A120" s="7" t="inlineStr">
@@ -6695,6 +6818,7 @@
       <c r="S120" s="7"/>
       <c r="T120" s="7"/>
       <c r="U120" s="7"/>
+      <c r="V120" s="7"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="inlineStr">
@@ -6758,6 +6882,7 @@
       <c r="S121" s="7"/>
       <c r="T121" s="7"/>
       <c r="U121" s="7"/>
+      <c r="V121" s="7"/>
     </row>
     <row r="122">
       <c r="A122" s="7" t="inlineStr">
@@ -6821,6 +6946,7 @@
       <c r="S122" s="7"/>
       <c r="T122" s="7"/>
       <c r="U122" s="7"/>
+      <c r="V122" s="7"/>
     </row>
     <row r="123">
       <c r="A123" s="7" t="inlineStr">
@@ -6872,6 +6998,7 @@
       <c r="S123" s="7"/>
       <c r="T123" s="7"/>
       <c r="U123" s="7"/>
+      <c r="V123" s="7"/>
     </row>
     <row r="124">
       <c r="A124" s="7" t="inlineStr">
@@ -6931,6 +7058,7 @@
       <c r="S124" s="7"/>
       <c r="T124" s="7"/>
       <c r="U124" s="7"/>
+      <c r="V124" s="7"/>
     </row>
     <row r="125">
       <c r="A125" s="7" t="inlineStr">
@@ -6982,6 +7110,7 @@
       <c r="S125" s="7"/>
       <c r="T125" s="7"/>
       <c r="U125" s="7"/>
+      <c r="V125" s="7"/>
     </row>
     <row r="126">
       <c r="A126" s="7" t="inlineStr">
@@ -7033,6 +7162,7 @@
       <c r="S126" s="7"/>
       <c r="T126" s="7"/>
       <c r="U126" s="7"/>
+      <c r="V126" s="7"/>
     </row>
     <row r="127">
       <c r="A127" s="7" t="inlineStr">
@@ -7088,6 +7218,7 @@
       <c r="S127" s="7"/>
       <c r="T127" s="7"/>
       <c r="U127" s="7"/>
+      <c r="V127" s="7"/>
     </row>
     <row r="128">
       <c r="A128" s="7" t="inlineStr">
@@ -7143,6 +7274,7 @@
       <c r="S128" s="7"/>
       <c r="T128" s="7"/>
       <c r="U128" s="7"/>
+      <c r="V128" s="7"/>
     </row>
     <row r="129">
       <c r="A129" s="7" t="inlineStr">
@@ -7198,6 +7330,7 @@
       <c r="S129" s="7"/>
       <c r="T129" s="7"/>
       <c r="U129" s="7"/>
+      <c r="V129" s="7"/>
     </row>
     <row r="130">
       <c r="A130" s="7" t="inlineStr">
@@ -7249,6 +7382,7 @@
       <c r="S130" s="7"/>
       <c r="T130" s="7"/>
       <c r="U130" s="7"/>
+      <c r="V130" s="7"/>
     </row>
     <row r="131">
       <c r="A131" s="7" t="inlineStr">
@@ -7308,6 +7442,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="V131" s="7"/>
     </row>
     <row r="132">
       <c r="A132" s="7" t="inlineStr">
@@ -7371,6 +7506,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="V132" s="7"/>
     </row>
     <row r="133">
       <c r="A133" s="7" t="inlineStr">
@@ -7430,6 +7566,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="V133" s="7"/>
     </row>
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
@@ -7489,6 +7626,7 @@
         </is>
       </c>
       <c r="U134" s="7"/>
+      <c r="V134" s="7"/>
     </row>
     <row r="135">
       <c r="A135" s="7" t="inlineStr">
@@ -7548,6 +7686,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="V135" s="7"/>
     </row>
     <row r="136">
       <c r="A136" s="7" t="inlineStr">
@@ -7607,6 +7746,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="V136" s="7"/>
     </row>
     <row r="137">
       <c r="A137" s="7" t="inlineStr">
@@ -7662,6 +7802,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="V137" s="7"/>
     </row>
     <row r="138">
       <c r="A138" s="7" t="inlineStr">
@@ -7717,6 +7858,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="V138" s="7"/>
     </row>
     <row r="139">
       <c r="A139" s="7" t="inlineStr">
@@ -7772,6 +7914,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="V139" s="7"/>
     </row>
     <row r="140">
       <c r="A140" s="7" t="inlineStr">
@@ -7823,6 +7966,7 @@
         </is>
       </c>
       <c r="U140" s="7"/>
+      <c r="V140" s="7"/>
     </row>
     <row r="141">
       <c r="A141" s="7" t="inlineStr">
@@ -7874,6 +8018,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="V141" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="7" t="inlineStr">
@@ -7925,6 +8074,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="V142" s="7"/>
     </row>
     <row r="143">
       <c r="A143" s="7" t="inlineStr">
@@ -7976,6 +8126,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="V143" s="7"/>
     </row>
     <row r="144">
       <c r="A144" s="7" t="inlineStr">
@@ -8027,6 +8178,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="V144" s="7"/>
     </row>
     <row r="145">
       <c r="A145" s="7" t="inlineStr">
@@ -8078,6 +8230,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="V145" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="7" t="inlineStr">
@@ -8129,6 +8286,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="V146" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="7" t="inlineStr">
@@ -8178,6 +8340,63 @@
       <c r="U147" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
+      <c r="V147" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_140</t>
+        </is>
+      </c>
+      <c r="B148" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C148" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">태그</t>
+        </is>
+      </c>
+      <c r="D148" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Auto 기본 켜짐</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t xml:space="preserve">새 저장·「처음부터」 뒤 로봇 B 가 해금된 판에서 태그 Auto 가 켜진 채로 시작해, 사람이 안 눌러도 만충 순간 교대·태그 스킬이 나가는가? Auto 단추로 끌 수 있는가?</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#158 · B 해금 전엔 무관</t>
+        </is>
+      </c>
+      <c r="G148" s="7"/>
+      <c r="H148" s="7"/>
+      <c r="I148" s="7"/>
+      <c r="J148" s="7"/>
+      <c r="K148" s="7"/>
+      <c r="L148" s="7"/>
+      <c r="M148" s="7"/>
+      <c r="N148" s="7"/>
+      <c r="O148" s="7"/>
+      <c r="P148" s="7"/>
+      <c r="Q148" s="7"/>
+      <c r="R148" s="7"/>
+      <c r="S148" s="7"/>
+      <c r="T148" s="7"/>
+      <c r="U148" s="7"/>
+      <c r="V148" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
         </is>
       </c>
     </row>
@@ -8208,9 +8427,9 @@
     <mergeCell ref="B92:B99"/>
     <mergeCell ref="B100:B106"/>
     <mergeCell ref="B107:B111"/>
-    <mergeCell ref="G7:U7"/>
+    <mergeCell ref="G7:V7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:U147">
+  <conditionalFormatting sqref="G9:V148">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
QA W열(9529be7) — #159·#160 재확인 Pass 5 · Fail 0 · CID_141~143 신설 · CID_139 빈 칸(강화 뒤 화면 미확인)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -178,8 +178,9 @@
     <col min="20" max="20" width="12" customWidth="1"/>
     <col min="21" max="21" width="12" customWidth="1"/>
     <col min="22" max="22" width="12" customWidth="1"/>
-    <col min="23" max="23" width="11" customWidth="1"/>
+    <col min="23" max="23" width="12" customWidth="1"/>
     <col min="24" max="24" width="11" customWidth="1"/>
+    <col min="25" max="25" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -372,6 +373,11 @@
       <c r="V6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">video-261016 후보 · #158 태그 Auto 기본 켜짐 ‖ 10-16 코드 세션 재확인(8123 · 8128 · 576×1024 · 소리 0 · 8123: 처음부터 → 바로가기 S6 파밍에서 B 로 저절로 교대(Auto 켜짐) · 8128(강화된 저장): 바로가기 S6 · 게이지 채움 · Auto 켜진 채 그대로 → 도전 7초쯤 합체만 누름 → **승리(남은 00:12)** · Auto 끄고 같은 판(바로가기 만충 · 게이지 채움 · 합체만 누름 · 태그 안 누름) → 남은 00:06 에 보스 약 90% · 시간 초과(사람이 태그를 안 누른 판 · 예상대로)) · 8128 갈아엎음 21:02:33(d08ddfc → 0749886) · 빈 칸 = 안 지나감(T3 영향은 시험·B 해금 문으로 봄 · 화면 미확인) · CID_140 새 항목</t>
+        </is>
+      </c>
+      <c r="W6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">video-261016 후보 · #159 설정 소리 줄 여백 · #160 도전 층 합체 연출(게이지 차오름 · 원형 펄스) ‖ 10-16 코드 세션 재확인(8123 · 720×1280 · 소리 0 · 설정 판: 소리 세 줄 높이 줄어 판이 짧아짐 · 바로가기 S6 → 파밍 몇 초 → 도전(안내 창 A 40/40 · B 0/40 · 게이지 100%) → 만충이라 합체 원형 펄스(1.0↔1.15) → 누르니 멈추고 합체 19.7s · 강화 전 저장(골드 15 · 강화 못 함)이라 시간 초과 = 하네스 「강화 전 = 패배」와 같음 · 강화 뒤 승리는 화면 미확인(골드 100 길 없음 · 하네스 58.4초 Win) · 「다시 도전」(게이지 0%) → 도전 시작 뒤 19% → 54% → 100% → 「발동」 펄스 · ⚠️ 빌드 셋 동시 실행 못 함(앱 브라우저 뒤 탭 멈춤 · Chrome 미연결 · 한 탭) · 8128 갈아엎음 23:42:28(0749886 → 9529be7) · 빈 칸 = 안 지나감 · CID_141~143 새 항목</t>
         </is>
       </c>
     </row>
@@ -418,14 +424,15 @@
       <c r="T7" s="2"/>
       <c r="U7" s="2"/>
       <c r="V7" s="2"/>
-      <c r="W7" s="2" t="inlineStr">
+      <c r="W7" s="2"/>
+      <c r="X7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">버전</t>
         </is>
       </c>
-      <c r="X7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0749886</t>
+      <c r="Y7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9529be7</t>
         </is>
       </c>
     </row>
@@ -530,11 +537,16 @@
       </c>
       <c r="W8" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">9529be7</t>
+        </is>
+      </c>
+      <c r="X8" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">PASSrate</t>
         </is>
       </c>
-      <c r="X8" s="7">
-        <f>COUNTIF(V9:V148,"Pass")</f>
+      <c r="Y8" s="7">
+        <f>COUNTIF(W9:W151,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -620,13 +632,14 @@
       <c r="T9" s="7"/>
       <c r="U9" s="7"/>
       <c r="V9" s="7"/>
-      <c r="W9" s="2" t="inlineStr">
+      <c r="W9" s="7"/>
+      <c r="X9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FAILrate</t>
         </is>
       </c>
-      <c r="X9" s="7">
-        <f>COUNTIF(V9:V148,"Fail")+COUNTIF(V9:V148,"Broken")</f>
+      <c r="Y9" s="7">
+        <f>COUNTIF(W9:W151,"Fail")+COUNTIF(W9:W151,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -676,13 +689,14 @@
       <c r="T10" s="7"/>
       <c r="U10" s="7"/>
       <c r="V10" s="7"/>
-      <c r="W10" s="2" t="inlineStr">
+      <c r="W10" s="7"/>
+      <c r="X10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">N/A</t>
         </is>
       </c>
-      <c r="X10" s="7">
-        <f>COUNTIF(V9:V148,"N/A")</f>
+      <c r="Y10" s="7">
+        <f>COUNTIF(W9:W151,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -732,13 +746,14 @@
       <c r="T11" s="7"/>
       <c r="U11" s="7"/>
       <c r="V11" s="7"/>
-      <c r="W11" s="2" t="inlineStr">
+      <c r="W11" s="7"/>
+      <c r="X11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">전체 개수</t>
         </is>
       </c>
-      <c r="X11" s="7">
-        <v>140</v>
+      <c r="Y11" s="7">
+        <v>143</v>
       </c>
     </row>
     <row r="12">
@@ -788,13 +803,14 @@
       <c r="T12" s="7"/>
       <c r="U12" s="7"/>
       <c r="V12" s="7"/>
-      <c r="W12" s="2" t="inlineStr">
+      <c r="W12" s="7"/>
+      <c r="X12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">진행율</t>
         </is>
       </c>
-      <c r="X12" s="7">
-        <f>TEXT((COUNTA(V9:V148))/140,"0.00%")</f>
+      <c r="Y12" s="7">
+        <f>TEXT((COUNTA(W9:W151))/143,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -848,6 +864,7 @@
       <c r="T13" s="7"/>
       <c r="U13" s="7"/>
       <c r="V13" s="7"/>
+      <c r="W13" s="7"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -891,6 +908,7 @@
       <c r="T14" s="7"/>
       <c r="U14" s="7"/>
       <c r="V14" s="7"/>
+      <c r="W14" s="7"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -970,6 +988,7 @@
       <c r="T15" s="7"/>
       <c r="U15" s="7"/>
       <c r="V15" s="7"/>
+      <c r="W15" s="7"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -1049,6 +1068,7 @@
       <c r="T16" s="7"/>
       <c r="U16" s="7"/>
       <c r="V16" s="7"/>
+      <c r="W16" s="7"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -1133,6 +1153,7 @@
       <c r="T17" s="7"/>
       <c r="U17" s="7"/>
       <c r="V17" s="7"/>
+      <c r="W17" s="7"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -1181,6 +1202,7 @@
       <c r="T18" s="7"/>
       <c r="U18" s="7"/>
       <c r="V18" s="7"/>
+      <c r="W18" s="7"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -1224,6 +1246,7 @@
       <c r="T19" s="7"/>
       <c r="U19" s="7"/>
       <c r="V19" s="7"/>
+      <c r="W19" s="7"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1267,6 +1290,7 @@
       <c r="T20" s="7"/>
       <c r="U20" s="7"/>
       <c r="V20" s="7"/>
+      <c r="W20" s="7"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1346,6 +1370,7 @@
       <c r="T21" s="7"/>
       <c r="U21" s="7"/>
       <c r="V21" s="7"/>
+      <c r="W21" s="7"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1418,6 +1443,7 @@
       <c r="T22" s="7"/>
       <c r="U22" s="7"/>
       <c r="V22" s="7"/>
+      <c r="W22" s="7"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -1469,6 +1495,7 @@
       <c r="T23" s="7"/>
       <c r="U23" s="7"/>
       <c r="V23" s="7"/>
+      <c r="W23" s="7"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -1512,6 +1539,7 @@
       <c r="T24" s="7"/>
       <c r="U24" s="7"/>
       <c r="V24" s="7"/>
+      <c r="W24" s="7"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -1555,6 +1583,7 @@
       <c r="T25" s="7"/>
       <c r="U25" s="7"/>
       <c r="V25" s="7"/>
+      <c r="W25" s="7"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -1627,6 +1656,7 @@
       <c r="T26" s="7"/>
       <c r="U26" s="7"/>
       <c r="V26" s="7"/>
+      <c r="W26" s="7"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -1674,6 +1704,7 @@
       <c r="T27" s="7"/>
       <c r="U27" s="7"/>
       <c r="V27" s="7"/>
+      <c r="W27" s="7"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -1730,6 +1761,7 @@
       <c r="T28" s="7"/>
       <c r="U28" s="7"/>
       <c r="V28" s="7"/>
+      <c r="W28" s="7"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -1781,6 +1813,7 @@
       <c r="T29" s="7"/>
       <c r="U29" s="7"/>
       <c r="V29" s="7"/>
+      <c r="W29" s="7"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -1856,6 +1889,7 @@
       <c r="T30" s="7"/>
       <c r="U30" s="7"/>
       <c r="V30" s="7"/>
+      <c r="W30" s="7"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -1936,6 +1970,7 @@
       <c r="T31" s="7"/>
       <c r="U31" s="7"/>
       <c r="V31" s="7"/>
+      <c r="W31" s="7"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -2003,6 +2038,7 @@
       <c r="T32" s="7"/>
       <c r="U32" s="7"/>
       <c r="V32" s="7"/>
+      <c r="W32" s="7"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -2078,6 +2114,7 @@
       <c r="T33" s="7"/>
       <c r="U33" s="7"/>
       <c r="V33" s="7"/>
+      <c r="W33" s="7"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -2153,6 +2190,7 @@
       <c r="T34" s="7"/>
       <c r="U34" s="7"/>
       <c r="V34" s="7"/>
+      <c r="W34" s="7"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -2233,6 +2271,7 @@
       <c r="T35" s="7"/>
       <c r="U35" s="7"/>
       <c r="V35" s="7"/>
+      <c r="W35" s="7"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -2292,6 +2331,7 @@
       <c r="T36" s="7"/>
       <c r="U36" s="7"/>
       <c r="V36" s="7"/>
+      <c r="W36" s="7"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -2335,6 +2375,7 @@
       <c r="T37" s="7"/>
       <c r="U37" s="7"/>
       <c r="V37" s="7"/>
+      <c r="W37" s="7"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -2399,6 +2440,7 @@
       <c r="T38" s="7"/>
       <c r="U38" s="7"/>
       <c r="V38" s="7"/>
+      <c r="W38" s="7"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -2474,6 +2516,7 @@
       <c r="T39" s="7"/>
       <c r="U39" s="7"/>
       <c r="V39" s="7"/>
+      <c r="W39" s="7"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -2550,6 +2593,7 @@
       <c r="T40" s="7"/>
       <c r="U40" s="7"/>
       <c r="V40" s="7"/>
+      <c r="W40" s="7"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -2621,6 +2665,7 @@
       <c r="T41" s="7"/>
       <c r="U41" s="7"/>
       <c r="V41" s="7"/>
+      <c r="W41" s="7"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -2676,6 +2721,7 @@
       <c r="T42" s="7"/>
       <c r="U42" s="7"/>
       <c r="V42" s="7"/>
+      <c r="W42" s="7"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -2751,6 +2797,7 @@
       <c r="T43" s="7"/>
       <c r="U43" s="7"/>
       <c r="V43" s="7"/>
+      <c r="W43" s="7"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -2799,6 +2846,7 @@
       <c r="T44" s="7"/>
       <c r="U44" s="7"/>
       <c r="V44" s="7"/>
+      <c r="W44" s="7"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -2870,6 +2918,7 @@
       <c r="T45" s="7"/>
       <c r="U45" s="7"/>
       <c r="V45" s="7"/>
+      <c r="W45" s="7"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -2941,6 +2990,7 @@
       <c r="T46" s="7"/>
       <c r="U46" s="7"/>
       <c r="V46" s="7"/>
+      <c r="W46" s="7"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -2989,6 +3039,7 @@
       <c r="T47" s="7"/>
       <c r="U47" s="7"/>
       <c r="V47" s="7"/>
+      <c r="W47" s="7"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -3032,6 +3083,7 @@
       <c r="T48" s="7"/>
       <c r="U48" s="7"/>
       <c r="V48" s="7"/>
+      <c r="W48" s="7"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -3075,6 +3127,7 @@
       <c r="T49" s="7"/>
       <c r="U49" s="7"/>
       <c r="V49" s="7"/>
+      <c r="W49" s="7"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -3142,6 +3195,7 @@
       <c r="T50" s="7"/>
       <c r="U50" s="7"/>
       <c r="V50" s="7"/>
+      <c r="W50" s="7"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -3209,6 +3263,7 @@
       <c r="T51" s="7"/>
       <c r="U51" s="7"/>
       <c r="V51" s="7"/>
+      <c r="W51" s="7"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -3257,6 +3312,7 @@
       <c r="T52" s="7"/>
       <c r="U52" s="7"/>
       <c r="V52" s="7"/>
+      <c r="W52" s="7"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -3305,6 +3361,7 @@
       <c r="T53" s="7"/>
       <c r="U53" s="7"/>
       <c r="V53" s="7"/>
+      <c r="W53" s="7"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -3348,6 +3405,7 @@
       <c r="T54" s="7"/>
       <c r="U54" s="7"/>
       <c r="V54" s="7"/>
+      <c r="W54" s="7"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -3427,6 +3485,7 @@
       <c r="T55" s="7"/>
       <c r="U55" s="7"/>
       <c r="V55" s="7"/>
+      <c r="W55" s="7"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -3486,6 +3545,7 @@
       <c r="T56" s="7"/>
       <c r="U56" s="7"/>
       <c r="V56" s="7"/>
+      <c r="W56" s="7"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -3554,6 +3614,7 @@
       <c r="T57" s="7"/>
       <c r="U57" s="7"/>
       <c r="V57" s="7"/>
+      <c r="W57" s="7"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -3630,6 +3691,7 @@
       <c r="T58" s="7"/>
       <c r="U58" s="7"/>
       <c r="V58" s="7"/>
+      <c r="W58" s="7"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -3673,6 +3735,7 @@
       <c r="T59" s="7"/>
       <c r="U59" s="7"/>
       <c r="V59" s="7"/>
+      <c r="W59" s="7"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -3716,6 +3779,7 @@
       <c r="T60" s="7"/>
       <c r="U60" s="7"/>
       <c r="V60" s="7"/>
+      <c r="W60" s="7"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -3771,6 +3835,7 @@
       <c r="T61" s="7"/>
       <c r="U61" s="7"/>
       <c r="V61" s="7"/>
+      <c r="W61" s="7"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -3834,6 +3899,7 @@
       <c r="T62" s="7"/>
       <c r="U62" s="7"/>
       <c r="V62" s="7"/>
+      <c r="W62" s="7"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -3889,6 +3955,7 @@
       <c r="T63" s="7"/>
       <c r="U63" s="7"/>
       <c r="V63" s="7"/>
+      <c r="W63" s="7"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -3932,6 +3999,7 @@
       <c r="T64" s="7"/>
       <c r="U64" s="7"/>
       <c r="V64" s="7"/>
+      <c r="W64" s="7"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -3980,6 +4048,7 @@
       <c r="T65" s="7"/>
       <c r="U65" s="7"/>
       <c r="V65" s="7"/>
+      <c r="W65" s="7"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
@@ -4035,6 +4104,7 @@
       <c r="T66" s="7"/>
       <c r="U66" s="7"/>
       <c r="V66" s="7"/>
+      <c r="W66" s="7"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -4078,6 +4148,7 @@
       <c r="T67" s="7"/>
       <c r="U67" s="7"/>
       <c r="V67" s="7"/>
+      <c r="W67" s="7"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
@@ -4125,6 +4196,7 @@
       <c r="T68" s="7"/>
       <c r="U68" s="7"/>
       <c r="V68" s="7"/>
+      <c r="W68" s="7"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -4204,6 +4276,7 @@
       <c r="T69" s="7"/>
       <c r="U69" s="7"/>
       <c r="V69" s="7"/>
+      <c r="W69" s="7"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
@@ -4247,6 +4320,7 @@
       <c r="T70" s="7"/>
       <c r="U70" s="7"/>
       <c r="V70" s="7"/>
+      <c r="W70" s="7"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -4295,6 +4369,7 @@
       <c r="T71" s="7"/>
       <c r="U71" s="7"/>
       <c r="V71" s="7"/>
+      <c r="W71" s="7"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
@@ -4354,6 +4429,7 @@
       <c r="T72" s="7"/>
       <c r="U72" s="7"/>
       <c r="V72" s="7"/>
+      <c r="W72" s="7"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
@@ -4402,6 +4478,7 @@
       <c r="T73" s="7"/>
       <c r="U73" s="7"/>
       <c r="V73" s="7"/>
+      <c r="W73" s="7"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -4445,6 +4522,7 @@
       <c r="T74" s="7"/>
       <c r="U74" s="7"/>
       <c r="V74" s="7"/>
+      <c r="W74" s="7"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -4488,6 +4566,7 @@
       <c r="T75" s="7"/>
       <c r="U75" s="7"/>
       <c r="V75" s="7"/>
+      <c r="W75" s="7"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -4531,6 +4610,7 @@
       <c r="T76" s="7"/>
       <c r="U76" s="7"/>
       <c r="V76" s="7"/>
+      <c r="W76" s="7"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -4578,6 +4658,7 @@
       <c r="T77" s="7"/>
       <c r="U77" s="7"/>
       <c r="V77" s="7"/>
+      <c r="W77" s="7"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
@@ -4621,6 +4702,7 @@
       <c r="T78" s="7"/>
       <c r="U78" s="7"/>
       <c r="V78" s="7"/>
+      <c r="W78" s="7"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -4669,6 +4751,7 @@
       <c r="T79" s="7"/>
       <c r="U79" s="7"/>
       <c r="V79" s="7"/>
+      <c r="W79" s="7"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
@@ -4728,6 +4811,7 @@
       <c r="T80" s="7"/>
       <c r="U80" s="7"/>
       <c r="V80" s="7"/>
+      <c r="W80" s="7"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
@@ -4771,6 +4855,7 @@
       <c r="T81" s="7"/>
       <c r="U81" s="7"/>
       <c r="V81" s="7"/>
+      <c r="W81" s="7"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
@@ -4814,6 +4899,7 @@
       <c r="T82" s="7"/>
       <c r="U82" s="7"/>
       <c r="V82" s="7"/>
+      <c r="W82" s="7"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
@@ -4862,6 +4948,7 @@
       <c r="T83" s="7"/>
       <c r="U83" s="7"/>
       <c r="V83" s="7"/>
+      <c r="W83" s="7"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
@@ -4905,6 +4992,7 @@
       <c r="T84" s="7"/>
       <c r="U84" s="7"/>
       <c r="V84" s="7"/>
+      <c r="W84" s="7"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
@@ -4948,6 +5036,7 @@
       <c r="T85" s="7"/>
       <c r="U85" s="7"/>
       <c r="V85" s="7"/>
+      <c r="W85" s="7"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
@@ -4996,6 +5085,7 @@
       <c r="T86" s="7"/>
       <c r="U86" s="7"/>
       <c r="V86" s="7"/>
+      <c r="W86" s="7"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
@@ -5039,6 +5129,7 @@
       <c r="T87" s="7"/>
       <c r="U87" s="7"/>
       <c r="V87" s="7"/>
+      <c r="W87" s="7"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
@@ -5082,6 +5173,7 @@
       <c r="T88" s="7"/>
       <c r="U88" s="7"/>
       <c r="V88" s="7"/>
+      <c r="W88" s="7"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
@@ -5125,6 +5217,7 @@
       <c r="T89" s="7"/>
       <c r="U89" s="7"/>
       <c r="V89" s="7"/>
+      <c r="W89" s="7"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
@@ -5197,6 +5290,7 @@
       <c r="T90" s="7"/>
       <c r="U90" s="7"/>
       <c r="V90" s="7"/>
+      <c r="W90" s="7"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
@@ -5240,6 +5334,7 @@
       <c r="T91" s="7"/>
       <c r="U91" s="7"/>
       <c r="V91" s="7"/>
+      <c r="W91" s="7"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
@@ -5319,6 +5414,7 @@
       <c r="T92" s="7"/>
       <c r="U92" s="7"/>
       <c r="V92" s="7"/>
+      <c r="W92" s="7"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
@@ -5403,6 +5499,7 @@
       <c r="T93" s="7"/>
       <c r="U93" s="7"/>
       <c r="V93" s="7"/>
+      <c r="W93" s="7"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
@@ -5451,6 +5548,7 @@
       <c r="T94" s="7"/>
       <c r="U94" s="7"/>
       <c r="V94" s="7"/>
+      <c r="W94" s="7"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
@@ -5499,6 +5597,7 @@
       <c r="T95" s="7"/>
       <c r="U95" s="7"/>
       <c r="V95" s="7"/>
+      <c r="W95" s="7"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
@@ -5566,6 +5665,7 @@
       <c r="T96" s="7"/>
       <c r="U96" s="7"/>
       <c r="V96" s="7"/>
+      <c r="W96" s="7"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="inlineStr">
@@ -5609,6 +5709,7 @@
       <c r="T97" s="7"/>
       <c r="U97" s="7"/>
       <c r="V97" s="7"/>
+      <c r="W97" s="7"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
@@ -5652,6 +5753,7 @@
       <c r="T98" s="7"/>
       <c r="U98" s="7"/>
       <c r="V98" s="7"/>
+      <c r="W98" s="7"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
@@ -5695,6 +5797,7 @@
       <c r="T99" s="7"/>
       <c r="U99" s="7"/>
       <c r="V99" s="7"/>
+      <c r="W99" s="7"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
@@ -5747,6 +5850,7 @@
       <c r="T100" s="7"/>
       <c r="U100" s="7"/>
       <c r="V100" s="7"/>
+      <c r="W100" s="7"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
@@ -5790,6 +5894,7 @@
       <c r="T101" s="7"/>
       <c r="U101" s="7"/>
       <c r="V101" s="7"/>
+      <c r="W101" s="7"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
@@ -5833,6 +5938,7 @@
       <c r="T102" s="7"/>
       <c r="U102" s="7"/>
       <c r="V102" s="7"/>
+      <c r="W102" s="7"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="inlineStr">
@@ -5876,6 +5982,7 @@
       <c r="T103" s="7"/>
       <c r="U103" s="7"/>
       <c r="V103" s="7"/>
+      <c r="W103" s="7"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="inlineStr">
@@ -5924,6 +6031,7 @@
       <c r="T104" s="7"/>
       <c r="U104" s="7"/>
       <c r="V104" s="7"/>
+      <c r="W104" s="7"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
@@ -5967,6 +6075,7 @@
       <c r="T105" s="7"/>
       <c r="U105" s="7"/>
       <c r="V105" s="7"/>
+      <c r="W105" s="7"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
@@ -6010,6 +6119,7 @@
       <c r="T106" s="7"/>
       <c r="U106" s="7"/>
       <c r="V106" s="7"/>
+      <c r="W106" s="7"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
@@ -6053,6 +6163,7 @@
       <c r="T107" s="7"/>
       <c r="U107" s="7"/>
       <c r="V107" s="7"/>
+      <c r="W107" s="7"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
@@ -6100,6 +6211,7 @@
       <c r="T108" s="7"/>
       <c r="U108" s="7"/>
       <c r="V108" s="7"/>
+      <c r="W108" s="7"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="inlineStr">
@@ -6152,6 +6264,7 @@
       <c r="T109" s="7"/>
       <c r="U109" s="7"/>
       <c r="V109" s="7"/>
+      <c r="W109" s="7"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
@@ -6212,6 +6325,7 @@
       <c r="T110" s="7"/>
       <c r="U110" s="7"/>
       <c r="V110" s="7"/>
+      <c r="W110" s="7"/>
     </row>
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
@@ -6275,6 +6389,7 @@
       <c r="T111" s="7"/>
       <c r="U111" s="7"/>
       <c r="V111" s="7"/>
+      <c r="W111" s="7"/>
     </row>
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
@@ -6335,6 +6450,7 @@
       <c r="T112" s="7"/>
       <c r="U112" s="7"/>
       <c r="V112" s="7"/>
+      <c r="W112" s="7"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
@@ -6387,6 +6503,7 @@
       <c r="T113" s="7"/>
       <c r="U113" s="7"/>
       <c r="V113" s="7"/>
+      <c r="W113" s="7"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="inlineStr">
@@ -6455,6 +6572,7 @@
       <c r="T114" s="7"/>
       <c r="U114" s="7"/>
       <c r="V114" s="7"/>
+      <c r="W114" s="7"/>
     </row>
     <row r="115">
       <c r="A115" s="7" t="inlineStr">
@@ -6515,6 +6633,7 @@
       <c r="T115" s="7"/>
       <c r="U115" s="7"/>
       <c r="V115" s="7"/>
+      <c r="W115" s="7"/>
     </row>
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
@@ -6579,6 +6698,7 @@
       <c r="T116" s="7"/>
       <c r="U116" s="7"/>
       <c r="V116" s="7"/>
+      <c r="W116" s="7"/>
     </row>
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
@@ -6643,6 +6763,7 @@
       <c r="T117" s="7"/>
       <c r="U117" s="7"/>
       <c r="V117" s="7"/>
+      <c r="W117" s="7"/>
     </row>
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
@@ -6707,6 +6828,7 @@
       <c r="T118" s="7"/>
       <c r="U118" s="7"/>
       <c r="V118" s="7"/>
+      <c r="W118" s="7"/>
     </row>
     <row r="119">
       <c r="A119" s="7" t="inlineStr">
@@ -6767,6 +6889,7 @@
       <c r="T119" s="7"/>
       <c r="U119" s="7"/>
       <c r="V119" s="7"/>
+      <c r="W119" s="7"/>
     </row>
     <row r="120">
       <c r="A120" s="7" t="inlineStr">
@@ -6819,6 +6942,7 @@
       <c r="T120" s="7"/>
       <c r="U120" s="7"/>
       <c r="V120" s="7"/>
+      <c r="W120" s="7"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="inlineStr">
@@ -6883,6 +7007,7 @@
       <c r="T121" s="7"/>
       <c r="U121" s="7"/>
       <c r="V121" s="7"/>
+      <c r="W121" s="7"/>
     </row>
     <row r="122">
       <c r="A122" s="7" t="inlineStr">
@@ -6947,6 +7072,7 @@
       <c r="T122" s="7"/>
       <c r="U122" s="7"/>
       <c r="V122" s="7"/>
+      <c r="W122" s="7"/>
     </row>
     <row r="123">
       <c r="A123" s="7" t="inlineStr">
@@ -6999,6 +7125,7 @@
       <c r="T123" s="7"/>
       <c r="U123" s="7"/>
       <c r="V123" s="7"/>
+      <c r="W123" s="7"/>
     </row>
     <row r="124">
       <c r="A124" s="7" t="inlineStr">
@@ -7059,6 +7186,7 @@
       <c r="T124" s="7"/>
       <c r="U124" s="7"/>
       <c r="V124" s="7"/>
+      <c r="W124" s="7"/>
     </row>
     <row r="125">
       <c r="A125" s="7" t="inlineStr">
@@ -7111,6 +7239,7 @@
       <c r="T125" s="7"/>
       <c r="U125" s="7"/>
       <c r="V125" s="7"/>
+      <c r="W125" s="7"/>
     </row>
     <row r="126">
       <c r="A126" s="7" t="inlineStr">
@@ -7163,6 +7292,7 @@
       <c r="T126" s="7"/>
       <c r="U126" s="7"/>
       <c r="V126" s="7"/>
+      <c r="W126" s="7"/>
     </row>
     <row r="127">
       <c r="A127" s="7" t="inlineStr">
@@ -7219,6 +7349,7 @@
       <c r="T127" s="7"/>
       <c r="U127" s="7"/>
       <c r="V127" s="7"/>
+      <c r="W127" s="7"/>
     </row>
     <row r="128">
       <c r="A128" s="7" t="inlineStr">
@@ -7275,6 +7406,7 @@
       <c r="T128" s="7"/>
       <c r="U128" s="7"/>
       <c r="V128" s="7"/>
+      <c r="W128" s="7"/>
     </row>
     <row r="129">
       <c r="A129" s="7" t="inlineStr">
@@ -7331,6 +7463,7 @@
       <c r="T129" s="7"/>
       <c r="U129" s="7"/>
       <c r="V129" s="7"/>
+      <c r="W129" s="7"/>
     </row>
     <row r="130">
       <c r="A130" s="7" t="inlineStr">
@@ -7383,6 +7516,7 @@
       <c r="T130" s="7"/>
       <c r="U130" s="7"/>
       <c r="V130" s="7"/>
+      <c r="W130" s="7"/>
     </row>
     <row r="131">
       <c r="A131" s="7" t="inlineStr">
@@ -7443,6 +7577,7 @@
         </is>
       </c>
       <c r="V131" s="7"/>
+      <c r="W131" s="7"/>
     </row>
     <row r="132">
       <c r="A132" s="7" t="inlineStr">
@@ -7507,6 +7642,7 @@
         </is>
       </c>
       <c r="V132" s="7"/>
+      <c r="W132" s="7"/>
     </row>
     <row r="133">
       <c r="A133" s="7" t="inlineStr">
@@ -7567,6 +7703,7 @@
         </is>
       </c>
       <c r="V133" s="7"/>
+      <c r="W133" s="7"/>
     </row>
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
@@ -7627,6 +7764,7 @@
       </c>
       <c r="U134" s="7"/>
       <c r="V134" s="7"/>
+      <c r="W134" s="7"/>
     </row>
     <row r="135">
       <c r="A135" s="7" t="inlineStr">
@@ -7687,6 +7825,7 @@
         </is>
       </c>
       <c r="V135" s="7"/>
+      <c r="W135" s="7"/>
     </row>
     <row r="136">
       <c r="A136" s="7" t="inlineStr">
@@ -7747,6 +7886,7 @@
         </is>
       </c>
       <c r="V136" s="7"/>
+      <c r="W136" s="7"/>
     </row>
     <row r="137">
       <c r="A137" s="7" t="inlineStr">
@@ -7803,6 +7943,7 @@
         </is>
       </c>
       <c r="V137" s="7"/>
+      <c r="W137" s="7"/>
     </row>
     <row r="138">
       <c r="A138" s="7" t="inlineStr">
@@ -7859,6 +8000,7 @@
         </is>
       </c>
       <c r="V138" s="7"/>
+      <c r="W138" s="7"/>
     </row>
     <row r="139">
       <c r="A139" s="7" t="inlineStr">
@@ -7915,6 +8057,7 @@
         </is>
       </c>
       <c r="V139" s="7"/>
+      <c r="W139" s="7"/>
     </row>
     <row r="140">
       <c r="A140" s="7" t="inlineStr">
@@ -7967,6 +8110,7 @@
       </c>
       <c r="U140" s="7"/>
       <c r="V140" s="7"/>
+      <c r="W140" s="7"/>
     </row>
     <row r="141">
       <c r="A141" s="7" t="inlineStr">
@@ -8023,6 +8167,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="W141" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="7" t="inlineStr">
@@ -8075,6 +8224,7 @@
         </is>
       </c>
       <c r="V142" s="7"/>
+      <c r="W142" s="7"/>
     </row>
     <row r="143">
       <c r="A143" s="7" t="inlineStr">
@@ -8127,6 +8277,7 @@
         </is>
       </c>
       <c r="V143" s="7"/>
+      <c r="W143" s="7"/>
     </row>
     <row r="144">
       <c r="A144" s="7" t="inlineStr">
@@ -8179,6 +8330,7 @@
         </is>
       </c>
       <c r="V144" s="7"/>
+      <c r="W144" s="7"/>
     </row>
     <row r="145">
       <c r="A145" s="7" t="inlineStr">
@@ -8235,6 +8387,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="W145" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="7" t="inlineStr">
@@ -8291,6 +8448,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="W146" s="7"/>
     </row>
     <row r="147">
       <c r="A147" s="7" t="inlineStr">
@@ -8347,6 +8505,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="W147" s="7"/>
     </row>
     <row r="148">
       <c r="A148" s="7" t="inlineStr">
@@ -8395,6 +8554,166 @@
       <c r="T148" s="7"/>
       <c r="U148" s="7"/>
       <c r="V148" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="W148" s="7"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_141</t>
+        </is>
+      </c>
+      <c r="B149" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C149" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">합체</t>
+        </is>
+      </c>
+      <c r="D149" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">게이지 차오름</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t xml:space="preserve">합체가 있는 도전 층(로봇 B 해금 뒤)에 들어가면 합체 게이지가 약 3초 동안 지금 값에서 100% 로 눈에 띄게 차오르는가? 파밍 층은 90초 그대로인가?</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#160 · 3초 가정</t>
+        </is>
+      </c>
+      <c r="G149" s="7"/>
+      <c r="H149" s="7"/>
+      <c r="I149" s="7"/>
+      <c r="J149" s="7"/>
+      <c r="K149" s="7"/>
+      <c r="L149" s="7"/>
+      <c r="M149" s="7"/>
+      <c r="N149" s="7"/>
+      <c r="O149" s="7"/>
+      <c r="P149" s="7"/>
+      <c r="Q149" s="7"/>
+      <c r="R149" s="7"/>
+      <c r="S149" s="7"/>
+      <c r="T149" s="7"/>
+      <c r="U149" s="7"/>
+      <c r="V149" s="7"/>
+      <c r="W149" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_142</t>
+        </is>
+      </c>
+      <c r="B150" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C150" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">합체</t>
+        </is>
+      </c>
+      <c r="D150" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">원형 펄스</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도전 층에서 합체 게이지가 100% 면 합체 원형이 커졌다 작아졌다(1.0↔1.15 · 0.6초) 하며 누를 때까지 강조되고, 누르면 멈추는가?</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#160 · 값 가정</t>
+        </is>
+      </c>
+      <c r="G150" s="7"/>
+      <c r="H150" s="7"/>
+      <c r="I150" s="7"/>
+      <c r="J150" s="7"/>
+      <c r="K150" s="7"/>
+      <c r="L150" s="7"/>
+      <c r="M150" s="7"/>
+      <c r="N150" s="7"/>
+      <c r="O150" s="7"/>
+      <c r="P150" s="7"/>
+      <c r="Q150" s="7"/>
+      <c r="R150" s="7"/>
+      <c r="S150" s="7"/>
+      <c r="T150" s="7"/>
+      <c r="U150" s="7"/>
+      <c r="V150" s="7"/>
+      <c r="W150" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_143</t>
+        </is>
+      </c>
+      <c r="B151" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">설정</t>
+        </is>
+      </c>
+      <c r="C151" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">소리</t>
+        </is>
+      </c>
+      <c r="D151" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">여백</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t xml:space="preserve">설정 판의 소리 세 줄(배경 음악·효과음·조작음) 위아래 여백이 줄어 판 높이가 짧아졌는가? 글자 크기는 그대로인가?</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#159 · 한 줄 70→39 가정</t>
+        </is>
+      </c>
+      <c r="G151" s="7"/>
+      <c r="H151" s="7"/>
+      <c r="I151" s="7"/>
+      <c r="J151" s="7"/>
+      <c r="K151" s="7"/>
+      <c r="L151" s="7"/>
+      <c r="M151" s="7"/>
+      <c r="N151" s="7"/>
+      <c r="O151" s="7"/>
+      <c r="P151" s="7"/>
+      <c r="Q151" s="7"/>
+      <c r="R151" s="7"/>
+      <c r="S151" s="7"/>
+      <c r="T151" s="7"/>
+      <c r="U151" s="7"/>
+      <c r="V151" s="7"/>
+      <c r="W151" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -8427,9 +8746,9 @@
     <mergeCell ref="B92:B99"/>
     <mergeCell ref="B100:B106"/>
     <mergeCell ref="B107:B111"/>
-    <mergeCell ref="G7:V7"/>
+    <mergeCell ref="G7:W7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:V148">
+  <conditionalFormatting sqref="G9:W151">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
QA X열(aa2be1b) — #161·#162·#163 재확인 Pass 7 · Fail 0 · CID_139 S6 화면 승리 채움 · CID_144~146 신설(146 빈 칸 · 화면 순간 미확인)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -179,8 +179,9 @@
     <col min="21" max="21" width="12" customWidth="1"/>
     <col min="22" max="22" width="12" customWidth="1"/>
     <col min="23" max="23" width="12" customWidth="1"/>
-    <col min="24" max="24" width="11" customWidth="1"/>
+    <col min="24" max="24" width="12" customWidth="1"/>
     <col min="25" max="25" width="11" customWidth="1"/>
+    <col min="26" max="26" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -378,6 +379,11 @@
       <c r="W6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">video-261016 후보 · #159 설정 소리 줄 여백 · #160 도전 층 합체 연출(게이지 차오름 · 원형 펄스) ‖ 10-16 코드 세션 재확인(8123 · 720×1280 · 소리 0 · 설정 판: 소리 세 줄 높이 줄어 판이 짧아짐 · 바로가기 S6 → 파밍 몇 초 → 도전(안내 창 A 40/40 · B 0/40 · 게이지 100%) → 만충이라 합체 원형 펄스(1.0↔1.15) → 누르니 멈추고 합체 19.7s · 강화 전 저장(골드 15 · 강화 못 함)이라 시간 초과 = 하네스 「강화 전 = 패배」와 같음 · 강화 뒤 승리는 화면 미확인(골드 100 길 없음 · 하네스 58.4초 Win) · 「다시 도전」(게이지 0%) → 도전 시작 뒤 19% → 54% → 100% → 「발동」 펄스 · ⚠️ 빌드 셋 동시 실행 못 함(앱 브라우저 뒤 탭 멈춤 · Chrome 미연결 · 한 탭) · 8128 갈아엎음 23:42:28(0749886 → 9529be7) · 빈 칸 = 안 지나감 · CID_141~143 새 항목</t>
+        </is>
+      </c>
+      <c r="X6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">video-261016 후보 · #161 S6 보스 12000 · #162 바로가기 S4 이상 = 강화 표식 · #163 합체 중 태그 스킬 ‖ 10-17 코드 세션 재확인(8123 · 800×600 창 · 소리 0 · 처음부터 → 바로가기 S3: 설정 단추 「강화 (재료 전부 투입)」(강화 전) → S4: 「강화 ×1.45 적용」 → S6 → 파밍 약 9초(A·B 둘 다 파밍에서 씀) → 도전 안내 A 0/40 · B 11/40 · 게이지 12% → 3초에 만충 · 원형 펄스 → 남은 00:51 에 합체 → **승리 — 적 전멸(남은 00:04)** · ⚠️ 합체 중 태그 스킬이 실제로 나간 순간은 화면에서 못 잡음(캡처 간격) · 하네스 = 45초 합체 55.0초 Win(#163 전 패배) · 즉시 합체 58.4초 · ⚠️ 빌드 셋 동시 실행 못 함(앱 브라우저 한 탭) · 8128 갈아엎음 00:02:38(9529be7 → aa2be1b) · 빈 칸 = 안 지나감 · CID_144~146 새 항목</t>
         </is>
       </c>
     </row>
@@ -425,14 +431,15 @@
       <c r="U7" s="2"/>
       <c r="V7" s="2"/>
       <c r="W7" s="2"/>
-      <c r="X7" s="2" t="inlineStr">
+      <c r="X7" s="2"/>
+      <c r="Y7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">버전</t>
         </is>
       </c>
-      <c r="Y7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">9529be7</t>
+      <c r="Z7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">aa2be1b</t>
         </is>
       </c>
     </row>
@@ -542,11 +549,16 @@
       </c>
       <c r="X8" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">aa2be1b</t>
+        </is>
+      </c>
+      <c r="Y8" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">PASSrate</t>
         </is>
       </c>
-      <c r="Y8" s="7">
-        <f>COUNTIF(W9:W151,"Pass")</f>
+      <c r="Z8" s="7">
+        <f>COUNTIF(X9:X154,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -633,13 +645,14 @@
       <c r="U9" s="7"/>
       <c r="V9" s="7"/>
       <c r="W9" s="7"/>
-      <c r="X9" s="2" t="inlineStr">
+      <c r="X9" s="7"/>
+      <c r="Y9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FAILrate</t>
         </is>
       </c>
-      <c r="Y9" s="7">
-        <f>COUNTIF(W9:W151,"Fail")+COUNTIF(W9:W151,"Broken")</f>
+      <c r="Z9" s="7">
+        <f>COUNTIF(X9:X154,"Fail")+COUNTIF(X9:X154,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -690,13 +703,14 @@
       <c r="U10" s="7"/>
       <c r="V10" s="7"/>
       <c r="W10" s="7"/>
-      <c r="X10" s="2" t="inlineStr">
+      <c r="X10" s="7"/>
+      <c r="Y10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">N/A</t>
         </is>
       </c>
-      <c r="Y10" s="7">
-        <f>COUNTIF(W9:W151,"N/A")</f>
+      <c r="Z10" s="7">
+        <f>COUNTIF(X9:X154,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -747,13 +761,14 @@
       <c r="U11" s="7"/>
       <c r="V11" s="7"/>
       <c r="W11" s="7"/>
-      <c r="X11" s="2" t="inlineStr">
+      <c r="X11" s="7"/>
+      <c r="Y11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">전체 개수</t>
         </is>
       </c>
-      <c r="Y11" s="7">
-        <v>143</v>
+      <c r="Z11" s="7">
+        <v>146</v>
       </c>
     </row>
     <row r="12">
@@ -804,13 +819,14 @@
       <c r="U12" s="7"/>
       <c r="V12" s="7"/>
       <c r="W12" s="7"/>
-      <c r="X12" s="2" t="inlineStr">
+      <c r="X12" s="7"/>
+      <c r="Y12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">진행율</t>
         </is>
       </c>
-      <c r="Y12" s="7">
-        <f>TEXT((COUNTA(W9:W151))/143,"0.00%")</f>
+      <c r="Z12" s="7">
+        <f>TEXT((COUNTA(X9:X154))/146,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -865,6 +881,7 @@
       <c r="U13" s="7"/>
       <c r="V13" s="7"/>
       <c r="W13" s="7"/>
+      <c r="X13" s="7"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -909,6 +926,7 @@
       <c r="U14" s="7"/>
       <c r="V14" s="7"/>
       <c r="W14" s="7"/>
+      <c r="X14" s="7"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -989,6 +1007,7 @@
       <c r="U15" s="7"/>
       <c r="V15" s="7"/>
       <c r="W15" s="7"/>
+      <c r="X15" s="7"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -1069,6 +1088,7 @@
       <c r="U16" s="7"/>
       <c r="V16" s="7"/>
       <c r="W16" s="7"/>
+      <c r="X16" s="7"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -1154,6 +1174,7 @@
       <c r="U17" s="7"/>
       <c r="V17" s="7"/>
       <c r="W17" s="7"/>
+      <c r="X17" s="7"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -1203,6 +1224,7 @@
       <c r="U18" s="7"/>
       <c r="V18" s="7"/>
       <c r="W18" s="7"/>
+      <c r="X18" s="7"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -1247,6 +1269,7 @@
       <c r="U19" s="7"/>
       <c r="V19" s="7"/>
       <c r="W19" s="7"/>
+      <c r="X19" s="7"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1291,6 +1314,7 @@
       <c r="U20" s="7"/>
       <c r="V20" s="7"/>
       <c r="W20" s="7"/>
+      <c r="X20" s="7"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1371,6 +1395,7 @@
       <c r="U21" s="7"/>
       <c r="V21" s="7"/>
       <c r="W21" s="7"/>
+      <c r="X21" s="7"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1444,6 +1469,7 @@
       <c r="U22" s="7"/>
       <c r="V22" s="7"/>
       <c r="W22" s="7"/>
+      <c r="X22" s="7"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -1496,6 +1522,7 @@
       <c r="U23" s="7"/>
       <c r="V23" s="7"/>
       <c r="W23" s="7"/>
+      <c r="X23" s="7"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -1540,6 +1567,7 @@
       <c r="U24" s="7"/>
       <c r="V24" s="7"/>
       <c r="W24" s="7"/>
+      <c r="X24" s="7"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -1584,6 +1612,7 @@
       <c r="U25" s="7"/>
       <c r="V25" s="7"/>
       <c r="W25" s="7"/>
+      <c r="X25" s="7"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -1657,6 +1686,7 @@
       <c r="U26" s="7"/>
       <c r="V26" s="7"/>
       <c r="W26" s="7"/>
+      <c r="X26" s="7"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -1705,6 +1735,7 @@
       <c r="U27" s="7"/>
       <c r="V27" s="7"/>
       <c r="W27" s="7"/>
+      <c r="X27" s="7"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -1762,6 +1793,7 @@
       <c r="U28" s="7"/>
       <c r="V28" s="7"/>
       <c r="W28" s="7"/>
+      <c r="X28" s="7"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -1814,6 +1846,7 @@
       <c r="U29" s="7"/>
       <c r="V29" s="7"/>
       <c r="W29" s="7"/>
+      <c r="X29" s="7"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -1890,6 +1923,7 @@
       <c r="U30" s="7"/>
       <c r="V30" s="7"/>
       <c r="W30" s="7"/>
+      <c r="X30" s="7"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -1971,6 +2005,7 @@
       <c r="U31" s="7"/>
       <c r="V31" s="7"/>
       <c r="W31" s="7"/>
+      <c r="X31" s="7"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -2039,6 +2074,7 @@
       <c r="U32" s="7"/>
       <c r="V32" s="7"/>
       <c r="W32" s="7"/>
+      <c r="X32" s="7"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -2115,6 +2151,7 @@
       <c r="U33" s="7"/>
       <c r="V33" s="7"/>
       <c r="W33" s="7"/>
+      <c r="X33" s="7"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -2191,6 +2228,7 @@
       <c r="U34" s="7"/>
       <c r="V34" s="7"/>
       <c r="W34" s="7"/>
+      <c r="X34" s="7"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -2272,6 +2310,7 @@
       <c r="U35" s="7"/>
       <c r="V35" s="7"/>
       <c r="W35" s="7"/>
+      <c r="X35" s="7"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -2332,6 +2371,7 @@
       <c r="U36" s="7"/>
       <c r="V36" s="7"/>
       <c r="W36" s="7"/>
+      <c r="X36" s="7"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -2376,6 +2416,7 @@
       <c r="U37" s="7"/>
       <c r="V37" s="7"/>
       <c r="W37" s="7"/>
+      <c r="X37" s="7"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -2441,6 +2482,7 @@
       <c r="U38" s="7"/>
       <c r="V38" s="7"/>
       <c r="W38" s="7"/>
+      <c r="X38" s="7"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -2517,6 +2559,7 @@
       <c r="U39" s="7"/>
       <c r="V39" s="7"/>
       <c r="W39" s="7"/>
+      <c r="X39" s="7"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -2594,6 +2637,7 @@
       <c r="U40" s="7"/>
       <c r="V40" s="7"/>
       <c r="W40" s="7"/>
+      <c r="X40" s="7"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -2666,6 +2710,7 @@
       <c r="U41" s="7"/>
       <c r="V41" s="7"/>
       <c r="W41" s="7"/>
+      <c r="X41" s="7"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -2722,6 +2767,7 @@
       <c r="U42" s="7"/>
       <c r="V42" s="7"/>
       <c r="W42" s="7"/>
+      <c r="X42" s="7"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -2798,6 +2844,7 @@
       <c r="U43" s="7"/>
       <c r="V43" s="7"/>
       <c r="W43" s="7"/>
+      <c r="X43" s="7"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -2847,6 +2894,7 @@
       <c r="U44" s="7"/>
       <c r="V44" s="7"/>
       <c r="W44" s="7"/>
+      <c r="X44" s="7"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -2919,6 +2967,7 @@
       <c r="U45" s="7"/>
       <c r="V45" s="7"/>
       <c r="W45" s="7"/>
+      <c r="X45" s="7"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -2991,6 +3040,7 @@
       <c r="U46" s="7"/>
       <c r="V46" s="7"/>
       <c r="W46" s="7"/>
+      <c r="X46" s="7"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -3040,6 +3090,7 @@
       <c r="U47" s="7"/>
       <c r="V47" s="7"/>
       <c r="W47" s="7"/>
+      <c r="X47" s="7"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -3084,6 +3135,7 @@
       <c r="U48" s="7"/>
       <c r="V48" s="7"/>
       <c r="W48" s="7"/>
+      <c r="X48" s="7"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -3128,6 +3180,7 @@
       <c r="U49" s="7"/>
       <c r="V49" s="7"/>
       <c r="W49" s="7"/>
+      <c r="X49" s="7"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -3196,6 +3249,7 @@
       <c r="U50" s="7"/>
       <c r="V50" s="7"/>
       <c r="W50" s="7"/>
+      <c r="X50" s="7"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -3264,6 +3318,7 @@
       <c r="U51" s="7"/>
       <c r="V51" s="7"/>
       <c r="W51" s="7"/>
+      <c r="X51" s="7"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -3313,6 +3368,7 @@
       <c r="U52" s="7"/>
       <c r="V52" s="7"/>
       <c r="W52" s="7"/>
+      <c r="X52" s="7"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -3362,6 +3418,7 @@
       <c r="U53" s="7"/>
       <c r="V53" s="7"/>
       <c r="W53" s="7"/>
+      <c r="X53" s="7"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -3406,6 +3463,7 @@
       <c r="U54" s="7"/>
       <c r="V54" s="7"/>
       <c r="W54" s="7"/>
+      <c r="X54" s="7"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -3486,6 +3544,7 @@
       <c r="U55" s="7"/>
       <c r="V55" s="7"/>
       <c r="W55" s="7"/>
+      <c r="X55" s="7"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -3546,6 +3605,7 @@
       <c r="U56" s="7"/>
       <c r="V56" s="7"/>
       <c r="W56" s="7"/>
+      <c r="X56" s="7"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -3615,6 +3675,7 @@
       <c r="U57" s="7"/>
       <c r="V57" s="7"/>
       <c r="W57" s="7"/>
+      <c r="X57" s="7"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -3692,6 +3753,7 @@
       <c r="U58" s="7"/>
       <c r="V58" s="7"/>
       <c r="W58" s="7"/>
+      <c r="X58" s="7"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -3736,6 +3798,7 @@
       <c r="U59" s="7"/>
       <c r="V59" s="7"/>
       <c r="W59" s="7"/>
+      <c r="X59" s="7"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -3780,6 +3843,7 @@
       <c r="U60" s="7"/>
       <c r="V60" s="7"/>
       <c r="W60" s="7"/>
+      <c r="X60" s="7"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -3836,6 +3900,7 @@
       <c r="U61" s="7"/>
       <c r="V61" s="7"/>
       <c r="W61" s="7"/>
+      <c r="X61" s="7"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -3900,6 +3965,7 @@
       <c r="U62" s="7"/>
       <c r="V62" s="7"/>
       <c r="W62" s="7"/>
+      <c r="X62" s="7"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -3956,6 +4022,7 @@
       <c r="U63" s="7"/>
       <c r="V63" s="7"/>
       <c r="W63" s="7"/>
+      <c r="X63" s="7"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -4000,6 +4067,7 @@
       <c r="U64" s="7"/>
       <c r="V64" s="7"/>
       <c r="W64" s="7"/>
+      <c r="X64" s="7"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -4049,6 +4117,7 @@
       <c r="U65" s="7"/>
       <c r="V65" s="7"/>
       <c r="W65" s="7"/>
+      <c r="X65" s="7"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
@@ -4105,6 +4174,7 @@
       <c r="U66" s="7"/>
       <c r="V66" s="7"/>
       <c r="W66" s="7"/>
+      <c r="X66" s="7"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -4149,6 +4219,7 @@
       <c r="U67" s="7"/>
       <c r="V67" s="7"/>
       <c r="W67" s="7"/>
+      <c r="X67" s="7"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
@@ -4197,6 +4268,7 @@
       <c r="U68" s="7"/>
       <c r="V68" s="7"/>
       <c r="W68" s="7"/>
+      <c r="X68" s="7"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -4277,6 +4349,7 @@
       <c r="U69" s="7"/>
       <c r="V69" s="7"/>
       <c r="W69" s="7"/>
+      <c r="X69" s="7"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
@@ -4321,6 +4394,7 @@
       <c r="U70" s="7"/>
       <c r="V70" s="7"/>
       <c r="W70" s="7"/>
+      <c r="X70" s="7"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -4370,6 +4444,7 @@
       <c r="U71" s="7"/>
       <c r="V71" s="7"/>
       <c r="W71" s="7"/>
+      <c r="X71" s="7"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
@@ -4430,6 +4505,7 @@
       <c r="U72" s="7"/>
       <c r="V72" s="7"/>
       <c r="W72" s="7"/>
+      <c r="X72" s="7"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
@@ -4479,6 +4555,7 @@
       <c r="U73" s="7"/>
       <c r="V73" s="7"/>
       <c r="W73" s="7"/>
+      <c r="X73" s="7"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -4523,6 +4600,7 @@
       <c r="U74" s="7"/>
       <c r="V74" s="7"/>
       <c r="W74" s="7"/>
+      <c r="X74" s="7"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -4567,6 +4645,7 @@
       <c r="U75" s="7"/>
       <c r="V75" s="7"/>
       <c r="W75" s="7"/>
+      <c r="X75" s="7"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -4611,6 +4690,7 @@
       <c r="U76" s="7"/>
       <c r="V76" s="7"/>
       <c r="W76" s="7"/>
+      <c r="X76" s="7"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -4659,6 +4739,7 @@
       <c r="U77" s="7"/>
       <c r="V77" s="7"/>
       <c r="W77" s="7"/>
+      <c r="X77" s="7"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
@@ -4703,6 +4784,7 @@
       <c r="U78" s="7"/>
       <c r="V78" s="7"/>
       <c r="W78" s="7"/>
+      <c r="X78" s="7"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -4752,6 +4834,7 @@
       <c r="U79" s="7"/>
       <c r="V79" s="7"/>
       <c r="W79" s="7"/>
+      <c r="X79" s="7"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
@@ -4812,6 +4895,7 @@
       <c r="U80" s="7"/>
       <c r="V80" s="7"/>
       <c r="W80" s="7"/>
+      <c r="X80" s="7"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
@@ -4856,6 +4940,7 @@
       <c r="U81" s="7"/>
       <c r="V81" s="7"/>
       <c r="W81" s="7"/>
+      <c r="X81" s="7"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
@@ -4900,6 +4985,7 @@
       <c r="U82" s="7"/>
       <c r="V82" s="7"/>
       <c r="W82" s="7"/>
+      <c r="X82" s="7"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
@@ -4949,6 +5035,7 @@
       <c r="U83" s="7"/>
       <c r="V83" s="7"/>
       <c r="W83" s="7"/>
+      <c r="X83" s="7"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
@@ -4993,6 +5080,7 @@
       <c r="U84" s="7"/>
       <c r="V84" s="7"/>
       <c r="W84" s="7"/>
+      <c r="X84" s="7"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
@@ -5037,6 +5125,7 @@
       <c r="U85" s="7"/>
       <c r="V85" s="7"/>
       <c r="W85" s="7"/>
+      <c r="X85" s="7"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
@@ -5086,6 +5175,7 @@
       <c r="U86" s="7"/>
       <c r="V86" s="7"/>
       <c r="W86" s="7"/>
+      <c r="X86" s="7"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
@@ -5130,6 +5220,7 @@
       <c r="U87" s="7"/>
       <c r="V87" s="7"/>
       <c r="W87" s="7"/>
+      <c r="X87" s="7"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
@@ -5174,6 +5265,7 @@
       <c r="U88" s="7"/>
       <c r="V88" s="7"/>
       <c r="W88" s="7"/>
+      <c r="X88" s="7"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
@@ -5218,6 +5310,7 @@
       <c r="U89" s="7"/>
       <c r="V89" s="7"/>
       <c r="W89" s="7"/>
+      <c r="X89" s="7"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
@@ -5291,6 +5384,7 @@
       <c r="U90" s="7"/>
       <c r="V90" s="7"/>
       <c r="W90" s="7"/>
+      <c r="X90" s="7"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
@@ -5335,6 +5429,7 @@
       <c r="U91" s="7"/>
       <c r="V91" s="7"/>
       <c r="W91" s="7"/>
+      <c r="X91" s="7"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
@@ -5415,6 +5510,7 @@
       <c r="U92" s="7"/>
       <c r="V92" s="7"/>
       <c r="W92" s="7"/>
+      <c r="X92" s="7"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
@@ -5500,6 +5596,7 @@
       <c r="U93" s="7"/>
       <c r="V93" s="7"/>
       <c r="W93" s="7"/>
+      <c r="X93" s="7"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
@@ -5549,6 +5646,7 @@
       <c r="U94" s="7"/>
       <c r="V94" s="7"/>
       <c r="W94" s="7"/>
+      <c r="X94" s="7"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
@@ -5598,6 +5696,7 @@
       <c r="U95" s="7"/>
       <c r="V95" s="7"/>
       <c r="W95" s="7"/>
+      <c r="X95" s="7"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
@@ -5666,6 +5765,7 @@
       <c r="U96" s="7"/>
       <c r="V96" s="7"/>
       <c r="W96" s="7"/>
+      <c r="X96" s="7"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="inlineStr">
@@ -5710,6 +5810,7 @@
       <c r="U97" s="7"/>
       <c r="V97" s="7"/>
       <c r="W97" s="7"/>
+      <c r="X97" s="7"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
@@ -5754,6 +5855,7 @@
       <c r="U98" s="7"/>
       <c r="V98" s="7"/>
       <c r="W98" s="7"/>
+      <c r="X98" s="7"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
@@ -5798,6 +5900,7 @@
       <c r="U99" s="7"/>
       <c r="V99" s="7"/>
       <c r="W99" s="7"/>
+      <c r="X99" s="7"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
@@ -5851,6 +5954,7 @@
       <c r="U100" s="7"/>
       <c r="V100" s="7"/>
       <c r="W100" s="7"/>
+      <c r="X100" s="7"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
@@ -5895,6 +5999,7 @@
       <c r="U101" s="7"/>
       <c r="V101" s="7"/>
       <c r="W101" s="7"/>
+      <c r="X101" s="7"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
@@ -5939,6 +6044,7 @@
       <c r="U102" s="7"/>
       <c r="V102" s="7"/>
       <c r="W102" s="7"/>
+      <c r="X102" s="7"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="inlineStr">
@@ -5983,6 +6089,7 @@
       <c r="U103" s="7"/>
       <c r="V103" s="7"/>
       <c r="W103" s="7"/>
+      <c r="X103" s="7"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="inlineStr">
@@ -6032,6 +6139,7 @@
       <c r="U104" s="7"/>
       <c r="V104" s="7"/>
       <c r="W104" s="7"/>
+      <c r="X104" s="7"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
@@ -6076,6 +6184,7 @@
       <c r="U105" s="7"/>
       <c r="V105" s="7"/>
       <c r="W105" s="7"/>
+      <c r="X105" s="7"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
@@ -6120,6 +6229,7 @@
       <c r="U106" s="7"/>
       <c r="V106" s="7"/>
       <c r="W106" s="7"/>
+      <c r="X106" s="7"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
@@ -6164,6 +6274,7 @@
       <c r="U107" s="7"/>
       <c r="V107" s="7"/>
       <c r="W107" s="7"/>
+      <c r="X107" s="7"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
@@ -6212,6 +6323,7 @@
       <c r="U108" s="7"/>
       <c r="V108" s="7"/>
       <c r="W108" s="7"/>
+      <c r="X108" s="7"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="inlineStr">
@@ -6265,6 +6377,7 @@
       <c r="U109" s="7"/>
       <c r="V109" s="7"/>
       <c r="W109" s="7"/>
+      <c r="X109" s="7"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
@@ -6326,6 +6439,7 @@
       <c r="U110" s="7"/>
       <c r="V110" s="7"/>
       <c r="W110" s="7"/>
+      <c r="X110" s="7"/>
     </row>
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
@@ -6390,6 +6504,7 @@
       <c r="U111" s="7"/>
       <c r="V111" s="7"/>
       <c r="W111" s="7"/>
+      <c r="X111" s="7"/>
     </row>
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
@@ -6451,6 +6566,7 @@
       <c r="U112" s="7"/>
       <c r="V112" s="7"/>
       <c r="W112" s="7"/>
+      <c r="X112" s="7"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
@@ -6504,6 +6620,7 @@
       <c r="U113" s="7"/>
       <c r="V113" s="7"/>
       <c r="W113" s="7"/>
+      <c r="X113" s="7"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="inlineStr">
@@ -6573,6 +6690,7 @@
       <c r="U114" s="7"/>
       <c r="V114" s="7"/>
       <c r="W114" s="7"/>
+      <c r="X114" s="7"/>
     </row>
     <row r="115">
       <c r="A115" s="7" t="inlineStr">
@@ -6634,6 +6752,7 @@
       <c r="U115" s="7"/>
       <c r="V115" s="7"/>
       <c r="W115" s="7"/>
+      <c r="X115" s="7"/>
     </row>
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
@@ -6699,6 +6818,7 @@
       <c r="U116" s="7"/>
       <c r="V116" s="7"/>
       <c r="W116" s="7"/>
+      <c r="X116" s="7"/>
     </row>
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
@@ -6764,6 +6884,7 @@
       <c r="U117" s="7"/>
       <c r="V117" s="7"/>
       <c r="W117" s="7"/>
+      <c r="X117" s="7"/>
     </row>
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
@@ -6829,6 +6950,7 @@
       <c r="U118" s="7"/>
       <c r="V118" s="7"/>
       <c r="W118" s="7"/>
+      <c r="X118" s="7"/>
     </row>
     <row r="119">
       <c r="A119" s="7" t="inlineStr">
@@ -6890,6 +7012,7 @@
       <c r="U119" s="7"/>
       <c r="V119" s="7"/>
       <c r="W119" s="7"/>
+      <c r="X119" s="7"/>
     </row>
     <row r="120">
       <c r="A120" s="7" t="inlineStr">
@@ -6943,6 +7066,7 @@
       <c r="U120" s="7"/>
       <c r="V120" s="7"/>
       <c r="W120" s="7"/>
+      <c r="X120" s="7"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="inlineStr">
@@ -7008,6 +7132,7 @@
       <c r="U121" s="7"/>
       <c r="V121" s="7"/>
       <c r="W121" s="7"/>
+      <c r="X121" s="7"/>
     </row>
     <row r="122">
       <c r="A122" s="7" t="inlineStr">
@@ -7073,6 +7198,7 @@
       <c r="U122" s="7"/>
       <c r="V122" s="7"/>
       <c r="W122" s="7"/>
+      <c r="X122" s="7"/>
     </row>
     <row r="123">
       <c r="A123" s="7" t="inlineStr">
@@ -7126,6 +7252,7 @@
       <c r="U123" s="7"/>
       <c r="V123" s="7"/>
       <c r="W123" s="7"/>
+      <c r="X123" s="7"/>
     </row>
     <row r="124">
       <c r="A124" s="7" t="inlineStr">
@@ -7187,6 +7314,7 @@
       <c r="U124" s="7"/>
       <c r="V124" s="7"/>
       <c r="W124" s="7"/>
+      <c r="X124" s="7"/>
     </row>
     <row r="125">
       <c r="A125" s="7" t="inlineStr">
@@ -7240,6 +7368,7 @@
       <c r="U125" s="7"/>
       <c r="V125" s="7"/>
       <c r="W125" s="7"/>
+      <c r="X125" s="7"/>
     </row>
     <row r="126">
       <c r="A126" s="7" t="inlineStr">
@@ -7293,6 +7422,7 @@
       <c r="U126" s="7"/>
       <c r="V126" s="7"/>
       <c r="W126" s="7"/>
+      <c r="X126" s="7"/>
     </row>
     <row r="127">
       <c r="A127" s="7" t="inlineStr">
@@ -7350,6 +7480,7 @@
       <c r="U127" s="7"/>
       <c r="V127" s="7"/>
       <c r="W127" s="7"/>
+      <c r="X127" s="7"/>
     </row>
     <row r="128">
       <c r="A128" s="7" t="inlineStr">
@@ -7407,6 +7538,7 @@
       <c r="U128" s="7"/>
       <c r="V128" s="7"/>
       <c r="W128" s="7"/>
+      <c r="X128" s="7"/>
     </row>
     <row r="129">
       <c r="A129" s="7" t="inlineStr">
@@ -7464,6 +7596,7 @@
       <c r="U129" s="7"/>
       <c r="V129" s="7"/>
       <c r="W129" s="7"/>
+      <c r="X129" s="7"/>
     </row>
     <row r="130">
       <c r="A130" s="7" t="inlineStr">
@@ -7517,6 +7650,7 @@
       <c r="U130" s="7"/>
       <c r="V130" s="7"/>
       <c r="W130" s="7"/>
+      <c r="X130" s="7"/>
     </row>
     <row r="131">
       <c r="A131" s="7" t="inlineStr">
@@ -7578,6 +7712,7 @@
       </c>
       <c r="V131" s="7"/>
       <c r="W131" s="7"/>
+      <c r="X131" s="7"/>
     </row>
     <row r="132">
       <c r="A132" s="7" t="inlineStr">
@@ -7643,6 +7778,7 @@
       </c>
       <c r="V132" s="7"/>
       <c r="W132" s="7"/>
+      <c r="X132" s="7"/>
     </row>
     <row r="133">
       <c r="A133" s="7" t="inlineStr">
@@ -7704,6 +7840,7 @@
       </c>
       <c r="V133" s="7"/>
       <c r="W133" s="7"/>
+      <c r="X133" s="7"/>
     </row>
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
@@ -7765,6 +7902,7 @@
       <c r="U134" s="7"/>
       <c r="V134" s="7"/>
       <c r="W134" s="7"/>
+      <c r="X134" s="7"/>
     </row>
     <row r="135">
       <c r="A135" s="7" t="inlineStr">
@@ -7826,6 +7964,7 @@
       </c>
       <c r="V135" s="7"/>
       <c r="W135" s="7"/>
+      <c r="X135" s="7"/>
     </row>
     <row r="136">
       <c r="A136" s="7" t="inlineStr">
@@ -7887,6 +8026,7 @@
       </c>
       <c r="V136" s="7"/>
       <c r="W136" s="7"/>
+      <c r="X136" s="7"/>
     </row>
     <row r="137">
       <c r="A137" s="7" t="inlineStr">
@@ -7944,6 +8084,7 @@
       </c>
       <c r="V137" s="7"/>
       <c r="W137" s="7"/>
+      <c r="X137" s="7"/>
     </row>
     <row r="138">
       <c r="A138" s="7" t="inlineStr">
@@ -8001,6 +8142,7 @@
       </c>
       <c r="V138" s="7"/>
       <c r="W138" s="7"/>
+      <c r="X138" s="7"/>
     </row>
     <row r="139">
       <c r="A139" s="7" t="inlineStr">
@@ -8058,6 +8200,7 @@
       </c>
       <c r="V139" s="7"/>
       <c r="W139" s="7"/>
+      <c r="X139" s="7"/>
     </row>
     <row r="140">
       <c r="A140" s="7" t="inlineStr">
@@ -8111,6 +8254,7 @@
       <c r="U140" s="7"/>
       <c r="V140" s="7"/>
       <c r="W140" s="7"/>
+      <c r="X140" s="7"/>
     </row>
     <row r="141">
       <c r="A141" s="7" t="inlineStr">
@@ -8172,6 +8316,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="X141" s="7"/>
     </row>
     <row r="142">
       <c r="A142" s="7" t="inlineStr">
@@ -8225,6 +8370,7 @@
       </c>
       <c r="V142" s="7"/>
       <c r="W142" s="7"/>
+      <c r="X142" s="7"/>
     </row>
     <row r="143">
       <c r="A143" s="7" t="inlineStr">
@@ -8278,6 +8424,7 @@
       </c>
       <c r="V143" s="7"/>
       <c r="W143" s="7"/>
+      <c r="X143" s="7"/>
     </row>
     <row r="144">
       <c r="A144" s="7" t="inlineStr">
@@ -8331,6 +8478,7 @@
       </c>
       <c r="V144" s="7"/>
       <c r="W144" s="7"/>
+      <c r="X144" s="7"/>
     </row>
     <row r="145">
       <c r="A145" s="7" t="inlineStr">
@@ -8392,6 +8540,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="X145" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="7" t="inlineStr">
@@ -8449,6 +8602,7 @@
         </is>
       </c>
       <c r="W146" s="7"/>
+      <c r="X146" s="7"/>
     </row>
     <row r="147">
       <c r="A147" s="7" t="inlineStr">
@@ -8506,6 +8660,11 @@
         </is>
       </c>
       <c r="W147" s="7"/>
+      <c r="X147" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="7" t="inlineStr">
@@ -8559,6 +8718,7 @@
         </is>
       </c>
       <c r="W148" s="7"/>
+      <c r="X148" s="7"/>
     </row>
     <row r="149">
       <c r="A149" s="7" t="inlineStr">
@@ -8612,6 +8772,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="X149" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="7" t="inlineStr">
@@ -8665,6 +8830,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="X150" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="7" t="inlineStr">
@@ -8718,6 +8888,169 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="X151" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_144</t>
+        </is>
+      </c>
+      <c r="B152" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">설정</t>
+        </is>
+      </c>
+      <c r="C152" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">바로가기</t>
+        </is>
+      </c>
+      <c r="D152" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">점프 시 강화</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">처음부터 뒤 바로가기 S4 이상으로 점프하면 설정 판 강화 단추가 「강화 ×1.45 적용」으로 바뀌고(재료는 그대로), S1~S3 점프는 강화 전 그대로인가?</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#162</t>
+        </is>
+      </c>
+      <c r="G152" s="7"/>
+      <c r="H152" s="7"/>
+      <c r="I152" s="7"/>
+      <c r="J152" s="7"/>
+      <c r="K152" s="7"/>
+      <c r="L152" s="7"/>
+      <c r="M152" s="7"/>
+      <c r="N152" s="7"/>
+      <c r="O152" s="7"/>
+      <c r="P152" s="7"/>
+      <c r="Q152" s="7"/>
+      <c r="R152" s="7"/>
+      <c r="S152" s="7"/>
+      <c r="T152" s="7"/>
+      <c r="U152" s="7"/>
+      <c r="V152" s="7"/>
+      <c r="W152" s="7"/>
+      <c r="X152" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_145</t>
+        </is>
+      </c>
+      <c r="B153" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C153" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S6</t>
+        </is>
+      </c>
+      <c r="D153" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">보스 HP</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S6 도전 보스 HP 가 12000 인가(바 · 하네스)? 강화 뒤 합체를 써서 60초 안에 잡히는가?</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#161 · 화면 승리 00:04 남음</t>
+        </is>
+      </c>
+      <c r="G153" s="7"/>
+      <c r="H153" s="7"/>
+      <c r="I153" s="7"/>
+      <c r="J153" s="7"/>
+      <c r="K153" s="7"/>
+      <c r="L153" s="7"/>
+      <c r="M153" s="7"/>
+      <c r="N153" s="7"/>
+      <c r="O153" s="7"/>
+      <c r="P153" s="7"/>
+      <c r="Q153" s="7"/>
+      <c r="R153" s="7"/>
+      <c r="S153" s="7"/>
+      <c r="T153" s="7"/>
+      <c r="U153" s="7"/>
+      <c r="V153" s="7"/>
+      <c r="W153" s="7"/>
+      <c r="X153" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_146</t>
+        </is>
+      </c>
+      <c r="B154" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C154" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">합체</t>
+        </is>
+      </c>
+      <c r="D154" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">합체 중 태그 스킬</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">합체 중 대기 로봇 마운트가 만충이면 교대 없이 태그 스킬이 나가고(자동·수동), 교대는 잠긴 채인가? 태그 원형이 「태그 스킬」/쿨다운/「태그 잠금」을 맞게 보이는가?</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#163 · 화면 순간 미확인</t>
+        </is>
+      </c>
+      <c r="G154" s="7"/>
+      <c r="H154" s="7"/>
+      <c r="I154" s="7"/>
+      <c r="J154" s="7"/>
+      <c r="K154" s="7"/>
+      <c r="L154" s="7"/>
+      <c r="M154" s="7"/>
+      <c r="N154" s="7"/>
+      <c r="O154" s="7"/>
+      <c r="P154" s="7"/>
+      <c r="Q154" s="7"/>
+      <c r="R154" s="7"/>
+      <c r="S154" s="7"/>
+      <c r="T154" s="7"/>
+      <c r="U154" s="7"/>
+      <c r="V154" s="7"/>
+      <c r="W154" s="7"/>
+      <c r="X154" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="26">
@@ -8746,9 +9079,9 @@
     <mergeCell ref="B92:B99"/>
     <mergeCell ref="B100:B106"/>
     <mergeCell ref="B107:B111"/>
-    <mergeCell ref="G7:W7"/>
+    <mergeCell ref="G7:X7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:W151">
+  <conditionalFormatting sqref="G9:X154">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
QA Y열(99067dc) — #164 재확인 Pass 6 · Fail 0 · CID_139 S6 화면 승리(남은 00:26 · 긴 파밍 00:23) · 요약 칸 Z→AA(열 셈 고침)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -180,8 +180,9 @@
     <col min="22" max="22" width="12" customWidth="1"/>
     <col min="23" max="23" width="12" customWidth="1"/>
     <col min="24" max="24" width="12" customWidth="1"/>
-    <col min="25" max="25" width="11" customWidth="1"/>
+    <col min="25" max="25" width="12" customWidth="1"/>
     <col min="26" max="26" width="11" customWidth="1"/>
+    <col min="27" max="27" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -384,6 +385,11 @@
       <c r="X6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">video-261016 후보 · #161 S6 보스 12000 · #162 바로가기 S4 이상 = 강화 표식 · #163 합체 중 태그 스킬 ‖ 10-17 코드 세션 재확인(8123 · 800×600 창 · 소리 0 · 처음부터 → 바로가기 S3: 설정 단추 「강화 (재료 전부 투입)」(강화 전) → S4: 「강화 ×1.45 적용」 → S6 → 파밍 약 9초(A·B 둘 다 파밍에서 씀) → 도전 안내 A 0/40 · B 11/40 · 게이지 12% → 3초에 만충 · 원형 펄스 → 남은 00:51 에 합체 → **승리 — 적 전멸(남은 00:04)** · ⚠️ 합체 중 태그 스킬이 실제로 나간 순간은 화면에서 못 잡음(캡처 간격) · 하네스 = 45초 합체 55.0초 Win(#163 전 패배) · 즉시 합체 58.4초 · ⚠️ 빌드 셋 동시 실행 못 함(앱 브라우저 한 탭) · 8128 갈아엎음 00:02:38(9529be7 → aa2be1b) · 빈 칸 = 안 지나감 · CID_144~146 새 항목</t>
+        </is>
+      </c>
+      <c r="Y6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">video-261016 후보 · #164 S6 보스 HP 15000 ‖ 10-17 코드 세션 재확인(8123 · 800×600 창 · 소리 0 · 처음부터 → 바로가기 S6(강화 ×1.45 적용) → 파밍 약 1초 → 도전 안내 A 40/40 · B 0/40 · 게이지 1% → 3초 만충 · 펄스 → 남은 00:54 에 합체 → **승리(남은 00:26)** · 바로가기 S6 다시 → 파밍 약 10초 → 도전 안내 A 22/40 · B 18/40 · 게이지 12% → 즉시 합체 → **승리(남은 00:23)** · 하네스(×2 태운 판 · 즉시 합체 44.1초)보다 화면이 빠름(보드 차이 · 하네스 시작 보드 vs 처음부터 바로가기 보드) · ⚠️ 빌드 셋 동시 실행 못 함(앱 브라우저 한 탭) · 8128 갈아엎음 08:18:22(aa2be1b → 99067dc) · 빈 칸 = 안 지나감 · 새 CID 없음</t>
         </is>
       </c>
     </row>
@@ -432,14 +438,15 @@
       <c r="V7" s="2"/>
       <c r="W7" s="2"/>
       <c r="X7" s="2"/>
-      <c r="Y7" s="2" t="inlineStr">
+      <c r="Y7" s="2"/>
+      <c r="Z7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">버전</t>
         </is>
       </c>
-      <c r="Z7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">aa2be1b</t>
+      <c r="AA7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">99067dc</t>
         </is>
       </c>
     </row>
@@ -554,11 +561,16 @@
       </c>
       <c r="Y8" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">99067dc</t>
+        </is>
+      </c>
+      <c r="Z8" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">PASSrate</t>
         </is>
       </c>
-      <c r="Z8" s="7">
-        <f>COUNTIF(X9:X154,"Pass")</f>
+      <c r="AA8" s="7">
+        <f>COUNTIF(Y9:Y154,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -646,13 +658,14 @@
       <c r="V9" s="7"/>
       <c r="W9" s="7"/>
       <c r="X9" s="7"/>
-      <c r="Y9" s="2" t="inlineStr">
+      <c r="Y9" s="7"/>
+      <c r="Z9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FAILrate</t>
         </is>
       </c>
-      <c r="Z9" s="7">
-        <f>COUNTIF(X9:X154,"Fail")+COUNTIF(X9:X154,"Broken")</f>
+      <c r="AA9" s="7">
+        <f>COUNTIF(Y9:Y154,"Fail")+COUNTIF(Y9:Y154,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -704,13 +717,14 @@
       <c r="V10" s="7"/>
       <c r="W10" s="7"/>
       <c r="X10" s="7"/>
-      <c r="Y10" s="2" t="inlineStr">
+      <c r="Y10" s="7"/>
+      <c r="Z10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">N/A</t>
         </is>
       </c>
-      <c r="Z10" s="7">
-        <f>COUNTIF(X9:X154,"N/A")</f>
+      <c r="AA10" s="7">
+        <f>COUNTIF(Y9:Y154,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -762,12 +776,13 @@
       <c r="V11" s="7"/>
       <c r="W11" s="7"/>
       <c r="X11" s="7"/>
-      <c r="Y11" s="2" t="inlineStr">
+      <c r="Y11" s="7"/>
+      <c r="Z11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">전체 개수</t>
         </is>
       </c>
-      <c r="Z11" s="7">
+      <c r="AA11" s="7">
         <v>146</v>
       </c>
     </row>
@@ -820,13 +835,14 @@
       <c r="V12" s="7"/>
       <c r="W12" s="7"/>
       <c r="X12" s="7"/>
-      <c r="Y12" s="2" t="inlineStr">
+      <c r="Y12" s="7"/>
+      <c r="Z12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">진행율</t>
         </is>
       </c>
-      <c r="Z12" s="7">
-        <f>TEXT((COUNTA(X9:X154))/146,"0.00%")</f>
+      <c r="AA12" s="7">
+        <f>TEXT((COUNTA(Y9:Y154))/146,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -882,6 +898,7 @@
       <c r="V13" s="7"/>
       <c r="W13" s="7"/>
       <c r="X13" s="7"/>
+      <c r="Y13" s="7"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -927,6 +944,7 @@
       <c r="V14" s="7"/>
       <c r="W14" s="7"/>
       <c r="X14" s="7"/>
+      <c r="Y14" s="7"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -1008,6 +1026,7 @@
       <c r="V15" s="7"/>
       <c r="W15" s="7"/>
       <c r="X15" s="7"/>
+      <c r="Y15" s="7"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -1089,6 +1108,7 @@
       <c r="V16" s="7"/>
       <c r="W16" s="7"/>
       <c r="X16" s="7"/>
+      <c r="Y16" s="7"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -1175,6 +1195,7 @@
       <c r="V17" s="7"/>
       <c r="W17" s="7"/>
       <c r="X17" s="7"/>
+      <c r="Y17" s="7"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -1225,6 +1246,7 @@
       <c r="V18" s="7"/>
       <c r="W18" s="7"/>
       <c r="X18" s="7"/>
+      <c r="Y18" s="7"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -1270,6 +1292,7 @@
       <c r="V19" s="7"/>
       <c r="W19" s="7"/>
       <c r="X19" s="7"/>
+      <c r="Y19" s="7"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1315,6 +1338,7 @@
       <c r="V20" s="7"/>
       <c r="W20" s="7"/>
       <c r="X20" s="7"/>
+      <c r="Y20" s="7"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1396,6 +1420,7 @@
       <c r="V21" s="7"/>
       <c r="W21" s="7"/>
       <c r="X21" s="7"/>
+      <c r="Y21" s="7"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1470,6 +1495,7 @@
       <c r="V22" s="7"/>
       <c r="W22" s="7"/>
       <c r="X22" s="7"/>
+      <c r="Y22" s="7"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -1523,6 +1549,7 @@
       <c r="V23" s="7"/>
       <c r="W23" s="7"/>
       <c r="X23" s="7"/>
+      <c r="Y23" s="7"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -1568,6 +1595,7 @@
       <c r="V24" s="7"/>
       <c r="W24" s="7"/>
       <c r="X24" s="7"/>
+      <c r="Y24" s="7"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -1613,6 +1641,7 @@
       <c r="V25" s="7"/>
       <c r="W25" s="7"/>
       <c r="X25" s="7"/>
+      <c r="Y25" s="7"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -1687,6 +1716,7 @@
       <c r="V26" s="7"/>
       <c r="W26" s="7"/>
       <c r="X26" s="7"/>
+      <c r="Y26" s="7"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -1736,6 +1766,7 @@
       <c r="V27" s="7"/>
       <c r="W27" s="7"/>
       <c r="X27" s="7"/>
+      <c r="Y27" s="7"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -1794,6 +1825,7 @@
       <c r="V28" s="7"/>
       <c r="W28" s="7"/>
       <c r="X28" s="7"/>
+      <c r="Y28" s="7"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -1847,6 +1879,7 @@
       <c r="V29" s="7"/>
       <c r="W29" s="7"/>
       <c r="X29" s="7"/>
+      <c r="Y29" s="7"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -1924,6 +1957,7 @@
       <c r="V30" s="7"/>
       <c r="W30" s="7"/>
       <c r="X30" s="7"/>
+      <c r="Y30" s="7"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -2006,6 +2040,7 @@
       <c r="V31" s="7"/>
       <c r="W31" s="7"/>
       <c r="X31" s="7"/>
+      <c r="Y31" s="7"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -2075,6 +2110,7 @@
       <c r="V32" s="7"/>
       <c r="W32" s="7"/>
       <c r="X32" s="7"/>
+      <c r="Y32" s="7"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -2152,6 +2188,7 @@
       <c r="V33" s="7"/>
       <c r="W33" s="7"/>
       <c r="X33" s="7"/>
+      <c r="Y33" s="7"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -2229,6 +2266,7 @@
       <c r="V34" s="7"/>
       <c r="W34" s="7"/>
       <c r="X34" s="7"/>
+      <c r="Y34" s="7"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -2311,6 +2349,7 @@
       <c r="V35" s="7"/>
       <c r="W35" s="7"/>
       <c r="X35" s="7"/>
+      <c r="Y35" s="7"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -2372,6 +2411,7 @@
       <c r="V36" s="7"/>
       <c r="W36" s="7"/>
       <c r="X36" s="7"/>
+      <c r="Y36" s="7"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -2417,6 +2457,7 @@
       <c r="V37" s="7"/>
       <c r="W37" s="7"/>
       <c r="X37" s="7"/>
+      <c r="Y37" s="7"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -2483,6 +2524,7 @@
       <c r="V38" s="7"/>
       <c r="W38" s="7"/>
       <c r="X38" s="7"/>
+      <c r="Y38" s="7"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -2560,6 +2602,7 @@
       <c r="V39" s="7"/>
       <c r="W39" s="7"/>
       <c r="X39" s="7"/>
+      <c r="Y39" s="7"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -2638,6 +2681,7 @@
       <c r="V40" s="7"/>
       <c r="W40" s="7"/>
       <c r="X40" s="7"/>
+      <c r="Y40" s="7"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -2711,6 +2755,7 @@
       <c r="V41" s="7"/>
       <c r="W41" s="7"/>
       <c r="X41" s="7"/>
+      <c r="Y41" s="7"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -2768,6 +2813,7 @@
       <c r="V42" s="7"/>
       <c r="W42" s="7"/>
       <c r="X42" s="7"/>
+      <c r="Y42" s="7"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -2845,6 +2891,7 @@
       <c r="V43" s="7"/>
       <c r="W43" s="7"/>
       <c r="X43" s="7"/>
+      <c r="Y43" s="7"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -2895,6 +2942,7 @@
       <c r="V44" s="7"/>
       <c r="W44" s="7"/>
       <c r="X44" s="7"/>
+      <c r="Y44" s="7"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -2968,6 +3016,7 @@
       <c r="V45" s="7"/>
       <c r="W45" s="7"/>
       <c r="X45" s="7"/>
+      <c r="Y45" s="7"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -3041,6 +3090,7 @@
       <c r="V46" s="7"/>
       <c r="W46" s="7"/>
       <c r="X46" s="7"/>
+      <c r="Y46" s="7"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -3091,6 +3141,7 @@
       <c r="V47" s="7"/>
       <c r="W47" s="7"/>
       <c r="X47" s="7"/>
+      <c r="Y47" s="7"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -3136,6 +3187,7 @@
       <c r="V48" s="7"/>
       <c r="W48" s="7"/>
       <c r="X48" s="7"/>
+      <c r="Y48" s="7"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -3181,6 +3233,7 @@
       <c r="V49" s="7"/>
       <c r="W49" s="7"/>
       <c r="X49" s="7"/>
+      <c r="Y49" s="7"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -3250,6 +3303,7 @@
       <c r="V50" s="7"/>
       <c r="W50" s="7"/>
       <c r="X50" s="7"/>
+      <c r="Y50" s="7"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -3319,6 +3373,7 @@
       <c r="V51" s="7"/>
       <c r="W51" s="7"/>
       <c r="X51" s="7"/>
+      <c r="Y51" s="7"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -3369,6 +3424,7 @@
       <c r="V52" s="7"/>
       <c r="W52" s="7"/>
       <c r="X52" s="7"/>
+      <c r="Y52" s="7"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -3419,6 +3475,7 @@
       <c r="V53" s="7"/>
       <c r="W53" s="7"/>
       <c r="X53" s="7"/>
+      <c r="Y53" s="7"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -3464,6 +3521,7 @@
       <c r="V54" s="7"/>
       <c r="W54" s="7"/>
       <c r="X54" s="7"/>
+      <c r="Y54" s="7"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -3545,6 +3603,7 @@
       <c r="V55" s="7"/>
       <c r="W55" s="7"/>
       <c r="X55" s="7"/>
+      <c r="Y55" s="7"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -3606,6 +3665,7 @@
       <c r="V56" s="7"/>
       <c r="W56" s="7"/>
       <c r="X56" s="7"/>
+      <c r="Y56" s="7"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -3676,6 +3736,7 @@
       <c r="V57" s="7"/>
       <c r="W57" s="7"/>
       <c r="X57" s="7"/>
+      <c r="Y57" s="7"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -3754,6 +3815,7 @@
       <c r="V58" s="7"/>
       <c r="W58" s="7"/>
       <c r="X58" s="7"/>
+      <c r="Y58" s="7"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -3799,6 +3861,7 @@
       <c r="V59" s="7"/>
       <c r="W59" s="7"/>
       <c r="X59" s="7"/>
+      <c r="Y59" s="7"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -3844,6 +3907,7 @@
       <c r="V60" s="7"/>
       <c r="W60" s="7"/>
       <c r="X60" s="7"/>
+      <c r="Y60" s="7"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -3901,6 +3965,7 @@
       <c r="V61" s="7"/>
       <c r="W61" s="7"/>
       <c r="X61" s="7"/>
+      <c r="Y61" s="7"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -3966,6 +4031,7 @@
       <c r="V62" s="7"/>
       <c r="W62" s="7"/>
       <c r="X62" s="7"/>
+      <c r="Y62" s="7"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -4023,6 +4089,7 @@
       <c r="V63" s="7"/>
       <c r="W63" s="7"/>
       <c r="X63" s="7"/>
+      <c r="Y63" s="7"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -4068,6 +4135,7 @@
       <c r="V64" s="7"/>
       <c r="W64" s="7"/>
       <c r="X64" s="7"/>
+      <c r="Y64" s="7"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -4118,6 +4186,7 @@
       <c r="V65" s="7"/>
       <c r="W65" s="7"/>
       <c r="X65" s="7"/>
+      <c r="Y65" s="7"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
@@ -4175,6 +4244,7 @@
       <c r="V66" s="7"/>
       <c r="W66" s="7"/>
       <c r="X66" s="7"/>
+      <c r="Y66" s="7"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -4220,6 +4290,7 @@
       <c r="V67" s="7"/>
       <c r="W67" s="7"/>
       <c r="X67" s="7"/>
+      <c r="Y67" s="7"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
@@ -4269,6 +4340,7 @@
       <c r="V68" s="7"/>
       <c r="W68" s="7"/>
       <c r="X68" s="7"/>
+      <c r="Y68" s="7"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -4350,6 +4422,7 @@
       <c r="V69" s="7"/>
       <c r="W69" s="7"/>
       <c r="X69" s="7"/>
+      <c r="Y69" s="7"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
@@ -4395,6 +4468,7 @@
       <c r="V70" s="7"/>
       <c r="W70" s="7"/>
       <c r="X70" s="7"/>
+      <c r="Y70" s="7"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -4445,6 +4519,7 @@
       <c r="V71" s="7"/>
       <c r="W71" s="7"/>
       <c r="X71" s="7"/>
+      <c r="Y71" s="7"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
@@ -4506,6 +4581,7 @@
       <c r="V72" s="7"/>
       <c r="W72" s="7"/>
       <c r="X72" s="7"/>
+      <c r="Y72" s="7"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
@@ -4556,6 +4632,7 @@
       <c r="V73" s="7"/>
       <c r="W73" s="7"/>
       <c r="X73" s="7"/>
+      <c r="Y73" s="7"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -4601,6 +4678,7 @@
       <c r="V74" s="7"/>
       <c r="W74" s="7"/>
       <c r="X74" s="7"/>
+      <c r="Y74" s="7"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -4646,6 +4724,7 @@
       <c r="V75" s="7"/>
       <c r="W75" s="7"/>
       <c r="X75" s="7"/>
+      <c r="Y75" s="7"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -4691,6 +4770,7 @@
       <c r="V76" s="7"/>
       <c r="W76" s="7"/>
       <c r="X76" s="7"/>
+      <c r="Y76" s="7"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -4740,6 +4820,7 @@
       <c r="V77" s="7"/>
       <c r="W77" s="7"/>
       <c r="X77" s="7"/>
+      <c r="Y77" s="7"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
@@ -4785,6 +4866,7 @@
       <c r="V78" s="7"/>
       <c r="W78" s="7"/>
       <c r="X78" s="7"/>
+      <c r="Y78" s="7"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -4835,6 +4917,7 @@
       <c r="V79" s="7"/>
       <c r="W79" s="7"/>
       <c r="X79" s="7"/>
+      <c r="Y79" s="7"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
@@ -4896,6 +4979,7 @@
       <c r="V80" s="7"/>
       <c r="W80" s="7"/>
       <c r="X80" s="7"/>
+      <c r="Y80" s="7"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
@@ -4941,6 +5025,7 @@
       <c r="V81" s="7"/>
       <c r="W81" s="7"/>
       <c r="X81" s="7"/>
+      <c r="Y81" s="7"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
@@ -4986,6 +5071,7 @@
       <c r="V82" s="7"/>
       <c r="W82" s="7"/>
       <c r="X82" s="7"/>
+      <c r="Y82" s="7"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
@@ -5036,6 +5122,7 @@
       <c r="V83" s="7"/>
       <c r="W83" s="7"/>
       <c r="X83" s="7"/>
+      <c r="Y83" s="7"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
@@ -5081,6 +5168,7 @@
       <c r="V84" s="7"/>
       <c r="W84" s="7"/>
       <c r="X84" s="7"/>
+      <c r="Y84" s="7"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
@@ -5126,6 +5214,7 @@
       <c r="V85" s="7"/>
       <c r="W85" s="7"/>
       <c r="X85" s="7"/>
+      <c r="Y85" s="7"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
@@ -5176,6 +5265,7 @@
       <c r="V86" s="7"/>
       <c r="W86" s="7"/>
       <c r="X86" s="7"/>
+      <c r="Y86" s="7"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
@@ -5221,6 +5311,7 @@
       <c r="V87" s="7"/>
       <c r="W87" s="7"/>
       <c r="X87" s="7"/>
+      <c r="Y87" s="7"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
@@ -5266,6 +5357,7 @@
       <c r="V88" s="7"/>
       <c r="W88" s="7"/>
       <c r="X88" s="7"/>
+      <c r="Y88" s="7"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
@@ -5311,6 +5403,7 @@
       <c r="V89" s="7"/>
       <c r="W89" s="7"/>
       <c r="X89" s="7"/>
+      <c r="Y89" s="7"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
@@ -5385,6 +5478,7 @@
       <c r="V90" s="7"/>
       <c r="W90" s="7"/>
       <c r="X90" s="7"/>
+      <c r="Y90" s="7"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
@@ -5430,6 +5524,7 @@
       <c r="V91" s="7"/>
       <c r="W91" s="7"/>
       <c r="X91" s="7"/>
+      <c r="Y91" s="7"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
@@ -5511,6 +5606,7 @@
       <c r="V92" s="7"/>
       <c r="W92" s="7"/>
       <c r="X92" s="7"/>
+      <c r="Y92" s="7"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
@@ -5597,6 +5693,7 @@
       <c r="V93" s="7"/>
       <c r="W93" s="7"/>
       <c r="X93" s="7"/>
+      <c r="Y93" s="7"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
@@ -5647,6 +5744,7 @@
       <c r="V94" s="7"/>
       <c r="W94" s="7"/>
       <c r="X94" s="7"/>
+      <c r="Y94" s="7"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
@@ -5697,6 +5795,7 @@
       <c r="V95" s="7"/>
       <c r="W95" s="7"/>
       <c r="X95" s="7"/>
+      <c r="Y95" s="7"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
@@ -5766,6 +5865,7 @@
       <c r="V96" s="7"/>
       <c r="W96" s="7"/>
       <c r="X96" s="7"/>
+      <c r="Y96" s="7"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="inlineStr">
@@ -5811,6 +5911,7 @@
       <c r="V97" s="7"/>
       <c r="W97" s="7"/>
       <c r="X97" s="7"/>
+      <c r="Y97" s="7"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
@@ -5856,6 +5957,7 @@
       <c r="V98" s="7"/>
       <c r="W98" s="7"/>
       <c r="X98" s="7"/>
+      <c r="Y98" s="7"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
@@ -5901,6 +6003,7 @@
       <c r="V99" s="7"/>
       <c r="W99" s="7"/>
       <c r="X99" s="7"/>
+      <c r="Y99" s="7"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
@@ -5955,6 +6058,7 @@
       <c r="V100" s="7"/>
       <c r="W100" s="7"/>
       <c r="X100" s="7"/>
+      <c r="Y100" s="7"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
@@ -6000,6 +6104,7 @@
       <c r="V101" s="7"/>
       <c r="W101" s="7"/>
       <c r="X101" s="7"/>
+      <c r="Y101" s="7"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
@@ -6045,6 +6150,7 @@
       <c r="V102" s="7"/>
       <c r="W102" s="7"/>
       <c r="X102" s="7"/>
+      <c r="Y102" s="7"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="inlineStr">
@@ -6090,6 +6196,7 @@
       <c r="V103" s="7"/>
       <c r="W103" s="7"/>
       <c r="X103" s="7"/>
+      <c r="Y103" s="7"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="inlineStr">
@@ -6140,6 +6247,7 @@
       <c r="V104" s="7"/>
       <c r="W104" s="7"/>
       <c r="X104" s="7"/>
+      <c r="Y104" s="7"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
@@ -6185,6 +6293,7 @@
       <c r="V105" s="7"/>
       <c r="W105" s="7"/>
       <c r="X105" s="7"/>
+      <c r="Y105" s="7"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
@@ -6230,6 +6339,7 @@
       <c r="V106" s="7"/>
       <c r="W106" s="7"/>
       <c r="X106" s="7"/>
+      <c r="Y106" s="7"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
@@ -6275,6 +6385,7 @@
       <c r="V107" s="7"/>
       <c r="W107" s="7"/>
       <c r="X107" s="7"/>
+      <c r="Y107" s="7"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
@@ -6324,6 +6435,7 @@
       <c r="V108" s="7"/>
       <c r="W108" s="7"/>
       <c r="X108" s="7"/>
+      <c r="Y108" s="7"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="inlineStr">
@@ -6378,6 +6490,7 @@
       <c r="V109" s="7"/>
       <c r="W109" s="7"/>
       <c r="X109" s="7"/>
+      <c r="Y109" s="7"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
@@ -6440,6 +6553,7 @@
       <c r="V110" s="7"/>
       <c r="W110" s="7"/>
       <c r="X110" s="7"/>
+      <c r="Y110" s="7"/>
     </row>
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
@@ -6505,6 +6619,7 @@
       <c r="V111" s="7"/>
       <c r="W111" s="7"/>
       <c r="X111" s="7"/>
+      <c r="Y111" s="7"/>
     </row>
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
@@ -6567,6 +6682,7 @@
       <c r="V112" s="7"/>
       <c r="W112" s="7"/>
       <c r="X112" s="7"/>
+      <c r="Y112" s="7"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
@@ -6621,6 +6737,7 @@
       <c r="V113" s="7"/>
       <c r="W113" s="7"/>
       <c r="X113" s="7"/>
+      <c r="Y113" s="7"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="inlineStr">
@@ -6691,6 +6808,7 @@
       <c r="V114" s="7"/>
       <c r="W114" s="7"/>
       <c r="X114" s="7"/>
+      <c r="Y114" s="7"/>
     </row>
     <row r="115">
       <c r="A115" s="7" t="inlineStr">
@@ -6753,6 +6871,7 @@
       <c r="V115" s="7"/>
       <c r="W115" s="7"/>
       <c r="X115" s="7"/>
+      <c r="Y115" s="7"/>
     </row>
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
@@ -6819,6 +6938,7 @@
       <c r="V116" s="7"/>
       <c r="W116" s="7"/>
       <c r="X116" s="7"/>
+      <c r="Y116" s="7"/>
     </row>
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
@@ -6885,6 +7005,7 @@
       <c r="V117" s="7"/>
       <c r="W117" s="7"/>
       <c r="X117" s="7"/>
+      <c r="Y117" s="7"/>
     </row>
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
@@ -6951,6 +7072,7 @@
       <c r="V118" s="7"/>
       <c r="W118" s="7"/>
       <c r="X118" s="7"/>
+      <c r="Y118" s="7"/>
     </row>
     <row r="119">
       <c r="A119" s="7" t="inlineStr">
@@ -7013,6 +7135,7 @@
       <c r="V119" s="7"/>
       <c r="W119" s="7"/>
       <c r="X119" s="7"/>
+      <c r="Y119" s="7"/>
     </row>
     <row r="120">
       <c r="A120" s="7" t="inlineStr">
@@ -7067,6 +7190,7 @@
       <c r="V120" s="7"/>
       <c r="W120" s="7"/>
       <c r="X120" s="7"/>
+      <c r="Y120" s="7"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="inlineStr">
@@ -7133,6 +7257,7 @@
       <c r="V121" s="7"/>
       <c r="W121" s="7"/>
       <c r="X121" s="7"/>
+      <c r="Y121" s="7"/>
     </row>
     <row r="122">
       <c r="A122" s="7" t="inlineStr">
@@ -7199,6 +7324,7 @@
       <c r="V122" s="7"/>
       <c r="W122" s="7"/>
       <c r="X122" s="7"/>
+      <c r="Y122" s="7"/>
     </row>
     <row r="123">
       <c r="A123" s="7" t="inlineStr">
@@ -7253,6 +7379,7 @@
       <c r="V123" s="7"/>
       <c r="W123" s="7"/>
       <c r="X123" s="7"/>
+      <c r="Y123" s="7"/>
     </row>
     <row r="124">
       <c r="A124" s="7" t="inlineStr">
@@ -7315,6 +7442,7 @@
       <c r="V124" s="7"/>
       <c r="W124" s="7"/>
       <c r="X124" s="7"/>
+      <c r="Y124" s="7"/>
     </row>
     <row r="125">
       <c r="A125" s="7" t="inlineStr">
@@ -7369,6 +7497,7 @@
       <c r="V125" s="7"/>
       <c r="W125" s="7"/>
       <c r="X125" s="7"/>
+      <c r="Y125" s="7"/>
     </row>
     <row r="126">
       <c r="A126" s="7" t="inlineStr">
@@ -7423,6 +7552,7 @@
       <c r="V126" s="7"/>
       <c r="W126" s="7"/>
       <c r="X126" s="7"/>
+      <c r="Y126" s="7"/>
     </row>
     <row r="127">
       <c r="A127" s="7" t="inlineStr">
@@ -7481,6 +7611,7 @@
       <c r="V127" s="7"/>
       <c r="W127" s="7"/>
       <c r="X127" s="7"/>
+      <c r="Y127" s="7"/>
     </row>
     <row r="128">
       <c r="A128" s="7" t="inlineStr">
@@ -7539,6 +7670,7 @@
       <c r="V128" s="7"/>
       <c r="W128" s="7"/>
       <c r="X128" s="7"/>
+      <c r="Y128" s="7"/>
     </row>
     <row r="129">
       <c r="A129" s="7" t="inlineStr">
@@ -7597,6 +7729,7 @@
       <c r="V129" s="7"/>
       <c r="W129" s="7"/>
       <c r="X129" s="7"/>
+      <c r="Y129" s="7"/>
     </row>
     <row r="130">
       <c r="A130" s="7" t="inlineStr">
@@ -7651,6 +7784,7 @@
       <c r="V130" s="7"/>
       <c r="W130" s="7"/>
       <c r="X130" s="7"/>
+      <c r="Y130" s="7"/>
     </row>
     <row r="131">
       <c r="A131" s="7" t="inlineStr">
@@ -7713,6 +7847,7 @@
       <c r="V131" s="7"/>
       <c r="W131" s="7"/>
       <c r="X131" s="7"/>
+      <c r="Y131" s="7"/>
     </row>
     <row r="132">
       <c r="A132" s="7" t="inlineStr">
@@ -7779,6 +7914,7 @@
       <c r="V132" s="7"/>
       <c r="W132" s="7"/>
       <c r="X132" s="7"/>
+      <c r="Y132" s="7"/>
     </row>
     <row r="133">
       <c r="A133" s="7" t="inlineStr">
@@ -7841,6 +7977,7 @@
       <c r="V133" s="7"/>
       <c r="W133" s="7"/>
       <c r="X133" s="7"/>
+      <c r="Y133" s="7"/>
     </row>
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
@@ -7903,6 +8040,7 @@
       <c r="V134" s="7"/>
       <c r="W134" s="7"/>
       <c r="X134" s="7"/>
+      <c r="Y134" s="7"/>
     </row>
     <row r="135">
       <c r="A135" s="7" t="inlineStr">
@@ -7965,6 +8103,7 @@
       <c r="V135" s="7"/>
       <c r="W135" s="7"/>
       <c r="X135" s="7"/>
+      <c r="Y135" s="7"/>
     </row>
     <row r="136">
       <c r="A136" s="7" t="inlineStr">
@@ -8027,6 +8166,7 @@
       <c r="V136" s="7"/>
       <c r="W136" s="7"/>
       <c r="X136" s="7"/>
+      <c r="Y136" s="7"/>
     </row>
     <row r="137">
       <c r="A137" s="7" t="inlineStr">
@@ -8085,6 +8225,7 @@
       <c r="V137" s="7"/>
       <c r="W137" s="7"/>
       <c r="X137" s="7"/>
+      <c r="Y137" s="7"/>
     </row>
     <row r="138">
       <c r="A138" s="7" t="inlineStr">
@@ -8143,6 +8284,7 @@
       <c r="V138" s="7"/>
       <c r="W138" s="7"/>
       <c r="X138" s="7"/>
+      <c r="Y138" s="7"/>
     </row>
     <row r="139">
       <c r="A139" s="7" t="inlineStr">
@@ -8201,6 +8343,7 @@
       <c r="V139" s="7"/>
       <c r="W139" s="7"/>
       <c r="X139" s="7"/>
+      <c r="Y139" s="7"/>
     </row>
     <row r="140">
       <c r="A140" s="7" t="inlineStr">
@@ -8255,6 +8398,7 @@
       <c r="V140" s="7"/>
       <c r="W140" s="7"/>
       <c r="X140" s="7"/>
+      <c r="Y140" s="7"/>
     </row>
     <row r="141">
       <c r="A141" s="7" t="inlineStr">
@@ -8317,6 +8461,7 @@
         </is>
       </c>
       <c r="X141" s="7"/>
+      <c r="Y141" s="7"/>
     </row>
     <row r="142">
       <c r="A142" s="7" t="inlineStr">
@@ -8371,6 +8516,7 @@
       <c r="V142" s="7"/>
       <c r="W142" s="7"/>
       <c r="X142" s="7"/>
+      <c r="Y142" s="7"/>
     </row>
     <row r="143">
       <c r="A143" s="7" t="inlineStr">
@@ -8425,6 +8571,7 @@
       <c r="V143" s="7"/>
       <c r="W143" s="7"/>
       <c r="X143" s="7"/>
+      <c r="Y143" s="7"/>
     </row>
     <row r="144">
       <c r="A144" s="7" t="inlineStr">
@@ -8479,6 +8626,7 @@
       <c r="V144" s="7"/>
       <c r="W144" s="7"/>
       <c r="X144" s="7"/>
+      <c r="Y144" s="7"/>
     </row>
     <row r="145">
       <c r="A145" s="7" t="inlineStr">
@@ -8545,6 +8693,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Y145" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="7" t="inlineStr">
@@ -8603,6 +8756,7 @@
       </c>
       <c r="W146" s="7"/>
       <c r="X146" s="7"/>
+      <c r="Y146" s="7"/>
     </row>
     <row r="147">
       <c r="A147" s="7" t="inlineStr">
@@ -8661,6 +8815,11 @@
       </c>
       <c r="W147" s="7"/>
       <c r="X147" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="Y147" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -8719,6 +8878,7 @@
       </c>
       <c r="W148" s="7"/>
       <c r="X148" s="7"/>
+      <c r="Y148" s="7"/>
     </row>
     <row r="149">
       <c r="A149" s="7" t="inlineStr">
@@ -8777,6 +8937,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Y149" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="7" t="inlineStr">
@@ -8835,6 +9000,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Y150" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="7" t="inlineStr">
@@ -8893,6 +9063,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Y151" s="7"/>
     </row>
     <row r="152">
       <c r="A152" s="7" t="inlineStr">
@@ -8947,6 +9118,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Y152" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="7" t="inlineStr">
@@ -8976,7 +9152,7 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t xml:space="preserve">#161 · 화면 승리 00:04 남음</t>
+          <t xml:space="preserve">#161 · 화면 승리 00:04 남음 · #164 → 15000(10-17 · 화면 남은 00:26 / 00:23)</t>
         </is>
       </c>
       <c r="G153" s="7"/>
@@ -9001,6 +9177,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="Y153" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="7" t="inlineStr">
@@ -9051,6 +9232,7 @@
       <c r="V154" s="7"/>
       <c r="W154" s="7"/>
       <c r="X154" s="7"/>
+      <c r="Y154" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="26">
@@ -9079,9 +9261,9 @@
     <mergeCell ref="B92:B99"/>
     <mergeCell ref="B100:B106"/>
     <mergeCell ref="B107:B111"/>
-    <mergeCell ref="G7:X7"/>
+    <mergeCell ref="G7:Y7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:X154">
+  <conditionalFormatting sqref="G9:Y154">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
QA AG열(1675623) — #180 · #181 재확인 Pass 2 · CID_173~174 신설(도전 배지 문구 · 줌아웃 하한)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -188,8 +188,9 @@
     <col min="30" max="30" width="12" customWidth="1"/>
     <col min="31" max="31" width="12" customWidth="1"/>
     <col min="32" max="32" width="12" customWidth="1"/>
-    <col min="33" max="33" width="11" customWidth="1"/>
+    <col min="33" max="33" width="12" customWidth="1"/>
     <col min="34" max="34" width="11" customWidth="1"/>
+    <col min="35" max="35" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -432,6 +433,11 @@
       <c r="AF6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">video-261019b 후보 갈아엎음 · #176 정정(팔레트 단추 안 값 표시 폐기 · 안내 줄에 고른 것 값) · #179 설정 판 강화 단추 폐기 ‖ 10-19 코드 세션 재확인(8123 · 캔버스 직접 캡처) · 설정 판: 강화 줄 없음 · 튜토/S1~S6 줄이 소리 줄 바로 아래 · 도전 중엔 「도전 즉시 종료」 더해 정상 · 처음부터 → 바로가기 S1 → S1·S2·S3 즉시 종료 통과 → S4 파밍 → 조립 A 마운트 탭 → 팝오버 「강화 재료 100/100 · [고철 아이콘] 602/300」 밝음 → 누름 → 「0/100 · 302/300 · 강화 ×1.45 적용」 · 조립 B 탭 「로봇 B · [골드 아이콘] 50」(#177 화면 확인) · 팔레트 변환기 고름 → 노랑 테두리 · 보드 안내 줄 「변환기 · [고철 아이콘] 20」 · 576×1024 팔레트: 노드 여섯 = 그림 + 이름 한 줄 · 값 없음 · 데스크톱 판(좁음): 「기초 가공소」 · 「복합 가공소」가 바닥 글자에서도 넘쳐 두 줄 「기초 가공 / 소」(가정 ⓐ 두 줄 허용) · 8131 갈아엎음 14:19:54 · 빈 칸 = 안 지나감 · CID_171~172 새 항목)</t>
+        </is>
+      </c>
+      <c r="AG6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">video-261019b 후보 갈아엎음 · #180 도전 배지 「전투력 n 넘기기」 · #181 줌아웃 하한 1/1.5 ‖ 10-19 코드 세션 재확인(8123 · 캔버스 직접 캡처) · 바로가기 S1 → 도전 → 배지 「목표: 벨트 연결 · 전투력 18 넘기기」 · 조립 휠 아래 두 번 → 최저 배율 · 칸 크기 약 2/3 · 보이는 칸 늘어남(데스크톱 판 · 576×1024 둘 다) · 노드 이름판 읽힘(「기초 가공소」 포함) · 최저 배율에서 코어 탭 = 코어 팝오버 · 선택 테두리 그 칸(탭 좌표 맞음) · 벨트 드래그는 이번 판 미확인(도전 층 · 튜토리얼 판) · 보드 전체 12×14 가 한 화면에 다 들지는 않음 · 8131 갈아엎음 14:51:37 · 빈 칸 = 안 지나감 · CID_173~174 새 항목)</t>
         </is>
       </c>
     </row>
@@ -488,14 +494,15 @@
       <c r="AD7" s="2"/>
       <c r="AE7" s="2"/>
       <c r="AF7" s="2"/>
-      <c r="AG7" s="2" t="inlineStr">
+      <c r="AG7" s="2"/>
+      <c r="AH7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">버전</t>
         </is>
       </c>
-      <c r="AH7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">bd5061e</t>
+      <c r="AI7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1675623</t>
         </is>
       </c>
     </row>
@@ -650,11 +657,16 @@
       </c>
       <c r="AG8" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">1675623</t>
+        </is>
+      </c>
+      <c r="AH8" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">PASSrate</t>
         </is>
       </c>
-      <c r="AH8" s="7">
-        <f>COUNTIF(AF9:AF180,"Pass")</f>
+      <c r="AI8" s="7">
+        <f>COUNTIF(AG9:AG182,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -750,13 +762,14 @@
       <c r="AD9" s="7"/>
       <c r="AE9" s="7"/>
       <c r="AF9" s="7"/>
-      <c r="AG9" s="2" t="inlineStr">
+      <c r="AG9" s="7"/>
+      <c r="AH9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FAILrate</t>
         </is>
       </c>
-      <c r="AH9" s="7">
-        <f>COUNTIF(AF9:AF180,"Fail")+COUNTIF(AF9:AF180,"Broken")</f>
+      <c r="AI9" s="7">
+        <f>COUNTIF(AG9:AG182,"Fail")+COUNTIF(AG9:AG182,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -816,13 +829,14 @@
       <c r="AD10" s="7"/>
       <c r="AE10" s="7"/>
       <c r="AF10" s="7"/>
-      <c r="AG10" s="2" t="inlineStr">
+      <c r="AG10" s="7"/>
+      <c r="AH10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">N/A</t>
         </is>
       </c>
-      <c r="AH10" s="7">
-        <f>COUNTIF(AF9:AF180,"N/A")</f>
+      <c r="AI10" s="7">
+        <f>COUNTIF(AG9:AG182,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -882,13 +896,14 @@
       <c r="AD11" s="7"/>
       <c r="AE11" s="7"/>
       <c r="AF11" s="7"/>
-      <c r="AG11" s="2" t="inlineStr">
+      <c r="AG11" s="7"/>
+      <c r="AH11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">전체 개수</t>
         </is>
       </c>
-      <c r="AH11" s="7">
-        <v>172</v>
+      <c r="AI11" s="7">
+        <v>174</v>
       </c>
     </row>
     <row r="12">
@@ -948,13 +963,14 @@
       <c r="AD12" s="7"/>
       <c r="AE12" s="7"/>
       <c r="AF12" s="7"/>
-      <c r="AG12" s="2" t="inlineStr">
+      <c r="AG12" s="7"/>
+      <c r="AH12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">진행율</t>
         </is>
       </c>
-      <c r="AH12" s="7">
-        <f>TEXT((COUNTA(AF9:AF180))/172,"0.00%")</f>
+      <c r="AI12" s="7">
+        <f>TEXT((COUNTA(AG9:AG182))/174,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -1018,6 +1034,7 @@
       <c r="AD13" s="7"/>
       <c r="AE13" s="7"/>
       <c r="AF13" s="7"/>
+      <c r="AG13" s="7"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -1071,6 +1088,7 @@
       <c r="AD14" s="7"/>
       <c r="AE14" s="7"/>
       <c r="AF14" s="7"/>
+      <c r="AG14" s="7"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -1160,6 +1178,7 @@
       <c r="AD15" s="7"/>
       <c r="AE15" s="7"/>
       <c r="AF15" s="7"/>
+      <c r="AG15" s="7"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -1249,6 +1268,7 @@
       <c r="AD16" s="7"/>
       <c r="AE16" s="7"/>
       <c r="AF16" s="7"/>
+      <c r="AG16" s="7"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -1343,6 +1363,7 @@
       <c r="AD17" s="7"/>
       <c r="AE17" s="7"/>
       <c r="AF17" s="7"/>
+      <c r="AG17" s="7"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -1401,6 +1422,7 @@
       <c r="AD18" s="7"/>
       <c r="AE18" s="7"/>
       <c r="AF18" s="7"/>
+      <c r="AG18" s="7"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -1454,6 +1476,7 @@
       <c r="AD19" s="7"/>
       <c r="AE19" s="7"/>
       <c r="AF19" s="7"/>
+      <c r="AG19" s="7"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1507,6 +1530,7 @@
       <c r="AD20" s="7"/>
       <c r="AE20" s="7"/>
       <c r="AF20" s="7"/>
+      <c r="AG20" s="7"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1596,6 +1620,7 @@
       <c r="AD21" s="7"/>
       <c r="AE21" s="7"/>
       <c r="AF21" s="7"/>
+      <c r="AG21" s="7"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1678,6 +1703,7 @@
       <c r="AD22" s="7"/>
       <c r="AE22" s="7"/>
       <c r="AF22" s="7"/>
+      <c r="AG22" s="7"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -1739,6 +1765,7 @@
       <c r="AD23" s="7"/>
       <c r="AE23" s="7"/>
       <c r="AF23" s="7"/>
+      <c r="AG23" s="7"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -1792,6 +1819,7 @@
       <c r="AD24" s="7"/>
       <c r="AE24" s="7"/>
       <c r="AF24" s="7"/>
+      <c r="AG24" s="7"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -1845,6 +1873,7 @@
       <c r="AD25" s="7"/>
       <c r="AE25" s="7"/>
       <c r="AF25" s="7"/>
+      <c r="AG25" s="7"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -1927,6 +1956,7 @@
       <c r="AD26" s="7"/>
       <c r="AE26" s="7"/>
       <c r="AF26" s="7"/>
+      <c r="AG26" s="7"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -1984,6 +2014,7 @@
       <c r="AD27" s="7"/>
       <c r="AE27" s="7"/>
       <c r="AF27" s="7"/>
+      <c r="AG27" s="7"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -2050,6 +2081,7 @@
       <c r="AD28" s="7"/>
       <c r="AE28" s="7"/>
       <c r="AF28" s="7"/>
+      <c r="AG28" s="7"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -2111,6 +2143,7 @@
       <c r="AD29" s="7"/>
       <c r="AE29" s="7"/>
       <c r="AF29" s="7"/>
+      <c r="AG29" s="7"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -2196,6 +2229,7 @@
       <c r="AD30" s="7"/>
       <c r="AE30" s="7"/>
       <c r="AF30" s="7"/>
+      <c r="AG30" s="7"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -2286,6 +2320,7 @@
       <c r="AD31" s="7"/>
       <c r="AE31" s="7"/>
       <c r="AF31" s="7"/>
+      <c r="AG31" s="7"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -2363,6 +2398,7 @@
       <c r="AD32" s="7"/>
       <c r="AE32" s="7"/>
       <c r="AF32" s="7"/>
+      <c r="AG32" s="7"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -2448,6 +2484,7 @@
       <c r="AD33" s="7"/>
       <c r="AE33" s="7"/>
       <c r="AF33" s="7"/>
+      <c r="AG33" s="7"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -2533,6 +2570,7 @@
       <c r="AD34" s="7"/>
       <c r="AE34" s="7"/>
       <c r="AF34" s="7"/>
+      <c r="AG34" s="7"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -2627,6 +2665,7 @@
       <c r="AD35" s="7"/>
       <c r="AE35" s="7"/>
       <c r="AF35" s="7"/>
+      <c r="AG35" s="7"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -2696,6 +2735,7 @@
       <c r="AD36" s="7"/>
       <c r="AE36" s="7"/>
       <c r="AF36" s="7"/>
+      <c r="AG36" s="7"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -2749,6 +2789,7 @@
       <c r="AD37" s="7"/>
       <c r="AE37" s="7"/>
       <c r="AF37" s="7"/>
+      <c r="AG37" s="7"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -2823,6 +2864,7 @@
       <c r="AD38" s="7"/>
       <c r="AE38" s="7"/>
       <c r="AF38" s="7"/>
+      <c r="AG38" s="7"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -2908,6 +2950,7 @@
       <c r="AD39" s="7"/>
       <c r="AE39" s="7"/>
       <c r="AF39" s="7"/>
+      <c r="AG39" s="7"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -2994,6 +3037,7 @@
       <c r="AD40" s="7"/>
       <c r="AE40" s="7"/>
       <c r="AF40" s="7"/>
+      <c r="AG40" s="7"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -3075,6 +3119,7 @@
       <c r="AD41" s="7"/>
       <c r="AE41" s="7"/>
       <c r="AF41" s="7"/>
+      <c r="AG41" s="7"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -3140,6 +3185,7 @@
       <c r="AD42" s="7"/>
       <c r="AE42" s="7"/>
       <c r="AF42" s="7"/>
+      <c r="AG42" s="7"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -3225,6 +3271,7 @@
       <c r="AD43" s="7"/>
       <c r="AE43" s="7"/>
       <c r="AF43" s="7"/>
+      <c r="AG43" s="7"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -3283,6 +3330,7 @@
       <c r="AD44" s="7"/>
       <c r="AE44" s="7"/>
       <c r="AF44" s="7"/>
+      <c r="AG44" s="7"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -3364,6 +3412,7 @@
       <c r="AD45" s="7"/>
       <c r="AE45" s="7"/>
       <c r="AF45" s="7"/>
+      <c r="AG45" s="7"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -3445,6 +3494,7 @@
       <c r="AD46" s="7"/>
       <c r="AE46" s="7"/>
       <c r="AF46" s="7"/>
+      <c r="AG46" s="7"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -3503,6 +3553,7 @@
       <c r="AD47" s="7"/>
       <c r="AE47" s="7"/>
       <c r="AF47" s="7"/>
+      <c r="AG47" s="7"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -3556,6 +3607,7 @@
       <c r="AD48" s="7"/>
       <c r="AE48" s="7"/>
       <c r="AF48" s="7"/>
+      <c r="AG48" s="7"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -3609,6 +3661,7 @@
       <c r="AD49" s="7"/>
       <c r="AE49" s="7"/>
       <c r="AF49" s="7"/>
+      <c r="AG49" s="7"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -3686,6 +3739,7 @@
       <c r="AD50" s="7"/>
       <c r="AE50" s="7"/>
       <c r="AF50" s="7"/>
+      <c r="AG50" s="7"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -3763,6 +3817,7 @@
       <c r="AD51" s="7"/>
       <c r="AE51" s="7"/>
       <c r="AF51" s="7"/>
+      <c r="AG51" s="7"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -3821,6 +3876,7 @@
       <c r="AD52" s="7"/>
       <c r="AE52" s="7"/>
       <c r="AF52" s="7"/>
+      <c r="AG52" s="7"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -3879,6 +3935,7 @@
       <c r="AD53" s="7"/>
       <c r="AE53" s="7"/>
       <c r="AF53" s="7"/>
+      <c r="AG53" s="7"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -3932,6 +3989,7 @@
       <c r="AD54" s="7"/>
       <c r="AE54" s="7"/>
       <c r="AF54" s="7"/>
+      <c r="AG54" s="7"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -4021,6 +4079,7 @@
       <c r="AD55" s="7"/>
       <c r="AE55" s="7"/>
       <c r="AF55" s="7"/>
+      <c r="AG55" s="7"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -4090,6 +4149,7 @@
       <c r="AD56" s="7"/>
       <c r="AE56" s="7"/>
       <c r="AF56" s="7"/>
+      <c r="AG56" s="7"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -4168,6 +4228,7 @@
       <c r="AD57" s="7"/>
       <c r="AE57" s="7"/>
       <c r="AF57" s="7"/>
+      <c r="AG57" s="7"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -4254,6 +4315,7 @@
       <c r="AD58" s="7"/>
       <c r="AE58" s="7"/>
       <c r="AF58" s="7"/>
+      <c r="AG58" s="7"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -4307,6 +4369,7 @@
       <c r="AD59" s="7"/>
       <c r="AE59" s="7"/>
       <c r="AF59" s="7"/>
+      <c r="AG59" s="7"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -4360,6 +4423,7 @@
       <c r="AD60" s="7"/>
       <c r="AE60" s="7"/>
       <c r="AF60" s="7"/>
+      <c r="AG60" s="7"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -4425,6 +4489,7 @@
       <c r="AD61" s="7"/>
       <c r="AE61" s="7"/>
       <c r="AF61" s="7"/>
+      <c r="AG61" s="7"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -4498,6 +4563,7 @@
       <c r="AD62" s="7"/>
       <c r="AE62" s="7"/>
       <c r="AF62" s="7"/>
+      <c r="AG62" s="7"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -4563,6 +4629,7 @@
       <c r="AD63" s="7"/>
       <c r="AE63" s="7"/>
       <c r="AF63" s="7"/>
+      <c r="AG63" s="7"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -4616,6 +4683,7 @@
       <c r="AD64" s="7"/>
       <c r="AE64" s="7"/>
       <c r="AF64" s="7"/>
+      <c r="AG64" s="7"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -4674,6 +4742,7 @@
       <c r="AD65" s="7"/>
       <c r="AE65" s="7"/>
       <c r="AF65" s="7"/>
+      <c r="AG65" s="7"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
@@ -4739,6 +4808,7 @@
       <c r="AD66" s="7"/>
       <c r="AE66" s="7"/>
       <c r="AF66" s="7"/>
+      <c r="AG66" s="7"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -4792,6 +4862,7 @@
       <c r="AD67" s="7"/>
       <c r="AE67" s="7"/>
       <c r="AF67" s="7"/>
+      <c r="AG67" s="7"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
@@ -4849,6 +4920,7 @@
       <c r="AD68" s="7"/>
       <c r="AE68" s="7"/>
       <c r="AF68" s="7"/>
+      <c r="AG68" s="7"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -4938,6 +5010,7 @@
       <c r="AD69" s="7"/>
       <c r="AE69" s="7"/>
       <c r="AF69" s="7"/>
+      <c r="AG69" s="7"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
@@ -4991,6 +5064,7 @@
       <c r="AD70" s="7"/>
       <c r="AE70" s="7"/>
       <c r="AF70" s="7"/>
+      <c r="AG70" s="7"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -5049,6 +5123,7 @@
       <c r="AD71" s="7"/>
       <c r="AE71" s="7"/>
       <c r="AF71" s="7"/>
+      <c r="AG71" s="7"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
@@ -5118,6 +5193,7 @@
       <c r="AD72" s="7"/>
       <c r="AE72" s="7"/>
       <c r="AF72" s="7"/>
+      <c r="AG72" s="7"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
@@ -5176,6 +5252,7 @@
       <c r="AD73" s="7"/>
       <c r="AE73" s="7"/>
       <c r="AF73" s="7"/>
+      <c r="AG73" s="7"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -5229,6 +5306,7 @@
       <c r="AD74" s="7"/>
       <c r="AE74" s="7"/>
       <c r="AF74" s="7"/>
+      <c r="AG74" s="7"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -5282,6 +5360,7 @@
       <c r="AD75" s="7"/>
       <c r="AE75" s="7"/>
       <c r="AF75" s="7"/>
+      <c r="AG75" s="7"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -5335,6 +5414,7 @@
       <c r="AD76" s="7"/>
       <c r="AE76" s="7"/>
       <c r="AF76" s="7"/>
+      <c r="AG76" s="7"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -5392,6 +5472,7 @@
       <c r="AD77" s="7"/>
       <c r="AE77" s="7"/>
       <c r="AF77" s="7"/>
+      <c r="AG77" s="7"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
@@ -5445,6 +5526,7 @@
       <c r="AD78" s="7"/>
       <c r="AE78" s="7"/>
       <c r="AF78" s="7"/>
+      <c r="AG78" s="7"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -5503,6 +5585,7 @@
       <c r="AD79" s="7"/>
       <c r="AE79" s="7"/>
       <c r="AF79" s="7"/>
+      <c r="AG79" s="7"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
@@ -5572,6 +5655,7 @@
       <c r="AD80" s="7"/>
       <c r="AE80" s="7"/>
       <c r="AF80" s="7"/>
+      <c r="AG80" s="7"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
@@ -5629,6 +5713,7 @@
       <c r="AD81" s="7"/>
       <c r="AE81" s="7"/>
       <c r="AF81" s="7"/>
+      <c r="AG81" s="7"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
@@ -5682,6 +5767,7 @@
       <c r="AD82" s="7"/>
       <c r="AE82" s="7"/>
       <c r="AF82" s="7"/>
+      <c r="AG82" s="7"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
@@ -5740,6 +5826,7 @@
       <c r="AD83" s="7"/>
       <c r="AE83" s="7"/>
       <c r="AF83" s="7"/>
+      <c r="AG83" s="7"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
@@ -5793,6 +5880,7 @@
       <c r="AD84" s="7"/>
       <c r="AE84" s="7"/>
       <c r="AF84" s="7"/>
+      <c r="AG84" s="7"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
@@ -5846,6 +5934,7 @@
       <c r="AD85" s="7"/>
       <c r="AE85" s="7"/>
       <c r="AF85" s="7"/>
+      <c r="AG85" s="7"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
@@ -5904,6 +5993,7 @@
       <c r="AD86" s="7"/>
       <c r="AE86" s="7"/>
       <c r="AF86" s="7"/>
+      <c r="AG86" s="7"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
@@ -5957,6 +6047,7 @@
       <c r="AD87" s="7"/>
       <c r="AE87" s="7"/>
       <c r="AF87" s="7"/>
+      <c r="AG87" s="7"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
@@ -6010,6 +6101,7 @@
       <c r="AD88" s="7"/>
       <c r="AE88" s="7"/>
       <c r="AF88" s="7"/>
+      <c r="AG88" s="7"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
@@ -6063,6 +6155,7 @@
       <c r="AD89" s="7"/>
       <c r="AE89" s="7"/>
       <c r="AF89" s="7"/>
+      <c r="AG89" s="7"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
@@ -6145,6 +6238,7 @@
       <c r="AD90" s="7"/>
       <c r="AE90" s="7"/>
       <c r="AF90" s="7"/>
+      <c r="AG90" s="7"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
@@ -6198,6 +6292,7 @@
       <c r="AD91" s="7"/>
       <c r="AE91" s="7"/>
       <c r="AF91" s="7"/>
+      <c r="AG91" s="7"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
@@ -6287,6 +6382,7 @@
       <c r="AD92" s="7"/>
       <c r="AE92" s="7"/>
       <c r="AF92" s="7"/>
+      <c r="AG92" s="7"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
@@ -6381,6 +6477,7 @@
       <c r="AD93" s="7"/>
       <c r="AE93" s="7"/>
       <c r="AF93" s="7"/>
+      <c r="AG93" s="7"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
@@ -6439,6 +6536,7 @@
       <c r="AD94" s="7"/>
       <c r="AE94" s="7"/>
       <c r="AF94" s="7"/>
+      <c r="AG94" s="7"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
@@ -6497,6 +6595,7 @@
       <c r="AD95" s="7"/>
       <c r="AE95" s="7"/>
       <c r="AF95" s="7"/>
+      <c r="AG95" s="7"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
@@ -6574,6 +6673,7 @@
       <c r="AD96" s="7"/>
       <c r="AE96" s="7"/>
       <c r="AF96" s="7"/>
+      <c r="AG96" s="7"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="inlineStr">
@@ -6627,6 +6727,7 @@
       <c r="AD97" s="7"/>
       <c r="AE97" s="7"/>
       <c r="AF97" s="7"/>
+      <c r="AG97" s="7"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
@@ -6680,6 +6781,7 @@
       <c r="AD98" s="7"/>
       <c r="AE98" s="7"/>
       <c r="AF98" s="7"/>
+      <c r="AG98" s="7"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
@@ -6733,6 +6835,7 @@
       <c r="AD99" s="7"/>
       <c r="AE99" s="7"/>
       <c r="AF99" s="7"/>
+      <c r="AG99" s="7"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
@@ -6795,6 +6898,7 @@
       <c r="AD100" s="7"/>
       <c r="AE100" s="7"/>
       <c r="AF100" s="7"/>
+      <c r="AG100" s="7"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
@@ -6848,6 +6952,7 @@
       <c r="AD101" s="7"/>
       <c r="AE101" s="7"/>
       <c r="AF101" s="7"/>
+      <c r="AG101" s="7"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
@@ -6901,6 +7006,7 @@
       <c r="AD102" s="7"/>
       <c r="AE102" s="7"/>
       <c r="AF102" s="7"/>
+      <c r="AG102" s="7"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="inlineStr">
@@ -6954,6 +7060,7 @@
       <c r="AD103" s="7"/>
       <c r="AE103" s="7"/>
       <c r="AF103" s="7"/>
+      <c r="AG103" s="7"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="inlineStr">
@@ -7012,6 +7119,7 @@
       <c r="AD104" s="7"/>
       <c r="AE104" s="7"/>
       <c r="AF104" s="7"/>
+      <c r="AG104" s="7"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
@@ -7065,6 +7173,7 @@
       <c r="AD105" s="7"/>
       <c r="AE105" s="7"/>
       <c r="AF105" s="7"/>
+      <c r="AG105" s="7"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
@@ -7118,6 +7227,7 @@
       <c r="AD106" s="7"/>
       <c r="AE106" s="7"/>
       <c r="AF106" s="7"/>
+      <c r="AG106" s="7"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
@@ -7171,6 +7281,7 @@
       <c r="AD107" s="7"/>
       <c r="AE107" s="7"/>
       <c r="AF107" s="7"/>
+      <c r="AG107" s="7"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
@@ -7228,6 +7339,7 @@
       <c r="AD108" s="7"/>
       <c r="AE108" s="7"/>
       <c r="AF108" s="7"/>
+      <c r="AG108" s="7"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="inlineStr">
@@ -7290,6 +7402,7 @@
       <c r="AD109" s="7"/>
       <c r="AE109" s="7"/>
       <c r="AF109" s="7"/>
+      <c r="AG109" s="7"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
@@ -7360,6 +7473,7 @@
       <c r="AD110" s="7"/>
       <c r="AE110" s="7"/>
       <c r="AF110" s="7"/>
+      <c r="AG110" s="7"/>
     </row>
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
@@ -7433,6 +7547,7 @@
       <c r="AD111" s="7"/>
       <c r="AE111" s="7"/>
       <c r="AF111" s="7"/>
+      <c r="AG111" s="7"/>
     </row>
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
@@ -7503,6 +7618,7 @@
       <c r="AD112" s="7"/>
       <c r="AE112" s="7"/>
       <c r="AF112" s="7"/>
+      <c r="AG112" s="7"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
@@ -7565,6 +7681,7 @@
       <c r="AD113" s="7"/>
       <c r="AE113" s="7"/>
       <c r="AF113" s="7"/>
+      <c r="AG113" s="7"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="inlineStr">
@@ -7643,6 +7760,7 @@
       <c r="AD114" s="7"/>
       <c r="AE114" s="7"/>
       <c r="AF114" s="7"/>
+      <c r="AG114" s="7"/>
     </row>
     <row r="115">
       <c r="A115" s="7" t="inlineStr">
@@ -7713,6 +7831,7 @@
       <c r="AD115" s="7"/>
       <c r="AE115" s="7"/>
       <c r="AF115" s="7"/>
+      <c r="AG115" s="7"/>
     </row>
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
@@ -7787,6 +7906,7 @@
       <c r="AD116" s="7"/>
       <c r="AE116" s="7"/>
       <c r="AF116" s="7"/>
+      <c r="AG116" s="7"/>
     </row>
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
@@ -7861,6 +7981,7 @@
       <c r="AD117" s="7"/>
       <c r="AE117" s="7"/>
       <c r="AF117" s="7"/>
+      <c r="AG117" s="7"/>
     </row>
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
@@ -7935,6 +8056,7 @@
       <c r="AD118" s="7"/>
       <c r="AE118" s="7"/>
       <c r="AF118" s="7"/>
+      <c r="AG118" s="7"/>
     </row>
     <row r="119">
       <c r="A119" s="7" t="inlineStr">
@@ -8005,6 +8127,7 @@
       <c r="AD119" s="7"/>
       <c r="AE119" s="7"/>
       <c r="AF119" s="7"/>
+      <c r="AG119" s="7"/>
     </row>
     <row r="120">
       <c r="A120" s="7" t="inlineStr">
@@ -8067,6 +8190,7 @@
       <c r="AD120" s="7"/>
       <c r="AE120" s="7"/>
       <c r="AF120" s="7"/>
+      <c r="AG120" s="7"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="inlineStr">
@@ -8141,6 +8265,7 @@
       <c r="AD121" s="7"/>
       <c r="AE121" s="7"/>
       <c r="AF121" s="7"/>
+      <c r="AG121" s="7"/>
     </row>
     <row r="122">
       <c r="A122" s="7" t="inlineStr">
@@ -8215,6 +8340,7 @@
       <c r="AD122" s="7"/>
       <c r="AE122" s="7"/>
       <c r="AF122" s="7"/>
+      <c r="AG122" s="7"/>
     </row>
     <row r="123">
       <c r="A123" s="7" t="inlineStr">
@@ -8277,6 +8403,7 @@
       <c r="AD123" s="7"/>
       <c r="AE123" s="7"/>
       <c r="AF123" s="7"/>
+      <c r="AG123" s="7"/>
     </row>
     <row r="124">
       <c r="A124" s="7" t="inlineStr">
@@ -8347,6 +8474,7 @@
       <c r="AD124" s="7"/>
       <c r="AE124" s="7"/>
       <c r="AF124" s="7"/>
+      <c r="AG124" s="7"/>
     </row>
     <row r="125">
       <c r="A125" s="7" t="inlineStr">
@@ -8409,6 +8537,7 @@
       <c r="AD125" s="7"/>
       <c r="AE125" s="7"/>
       <c r="AF125" s="7"/>
+      <c r="AG125" s="7"/>
     </row>
     <row r="126">
       <c r="A126" s="7" t="inlineStr">
@@ -8471,6 +8600,7 @@
       <c r="AD126" s="7"/>
       <c r="AE126" s="7"/>
       <c r="AF126" s="7"/>
+      <c r="AG126" s="7"/>
     </row>
     <row r="127">
       <c r="A127" s="7" t="inlineStr">
@@ -8537,6 +8667,7 @@
       <c r="AD127" s="7"/>
       <c r="AE127" s="7"/>
       <c r="AF127" s="7"/>
+      <c r="AG127" s="7"/>
     </row>
     <row r="128">
       <c r="A128" s="7" t="inlineStr">
@@ -8603,6 +8734,7 @@
       <c r="AD128" s="7"/>
       <c r="AE128" s="7"/>
       <c r="AF128" s="7"/>
+      <c r="AG128" s="7"/>
     </row>
     <row r="129">
       <c r="A129" s="7" t="inlineStr">
@@ -8669,6 +8801,7 @@
       <c r="AD129" s="7"/>
       <c r="AE129" s="7"/>
       <c r="AF129" s="7"/>
+      <c r="AG129" s="7"/>
     </row>
     <row r="130">
       <c r="A130" s="7" t="inlineStr">
@@ -8731,6 +8864,7 @@
       <c r="AD130" s="7"/>
       <c r="AE130" s="7"/>
       <c r="AF130" s="7"/>
+      <c r="AG130" s="7"/>
     </row>
     <row r="131">
       <c r="A131" s="7" t="inlineStr">
@@ -8801,6 +8935,7 @@
       <c r="AD131" s="7"/>
       <c r="AE131" s="7"/>
       <c r="AF131" s="7"/>
+      <c r="AG131" s="7"/>
     </row>
     <row r="132">
       <c r="A132" s="7" t="inlineStr">
@@ -8875,6 +9010,7 @@
       <c r="AD132" s="7"/>
       <c r="AE132" s="7"/>
       <c r="AF132" s="7"/>
+      <c r="AG132" s="7"/>
     </row>
     <row r="133">
       <c r="A133" s="7" t="inlineStr">
@@ -8949,6 +9085,7 @@
       <c r="AD133" s="7"/>
       <c r="AE133" s="7"/>
       <c r="AF133" s="7"/>
+      <c r="AG133" s="7"/>
     </row>
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
@@ -9019,6 +9156,7 @@
       <c r="AD134" s="7"/>
       <c r="AE134" s="7"/>
       <c r="AF134" s="7"/>
+      <c r="AG134" s="7"/>
     </row>
     <row r="135">
       <c r="A135" s="7" t="inlineStr">
@@ -9089,6 +9227,7 @@
       <c r="AD135" s="7"/>
       <c r="AE135" s="7"/>
       <c r="AF135" s="7"/>
+      <c r="AG135" s="7"/>
     </row>
     <row r="136">
       <c r="A136" s="7" t="inlineStr">
@@ -9159,6 +9298,7 @@
       <c r="AD136" s="7"/>
       <c r="AE136" s="7"/>
       <c r="AF136" s="7"/>
+      <c r="AG136" s="7"/>
     </row>
     <row r="137">
       <c r="A137" s="7" t="inlineStr">
@@ -9225,6 +9365,7 @@
       <c r="AD137" s="7"/>
       <c r="AE137" s="7"/>
       <c r="AF137" s="7"/>
+      <c r="AG137" s="7"/>
     </row>
     <row r="138">
       <c r="A138" s="7" t="inlineStr">
@@ -9291,6 +9432,7 @@
       <c r="AD138" s="7"/>
       <c r="AE138" s="7"/>
       <c r="AF138" s="7"/>
+      <c r="AG138" s="7"/>
     </row>
     <row r="139">
       <c r="A139" s="7" t="inlineStr">
@@ -9357,6 +9499,7 @@
       <c r="AD139" s="7"/>
       <c r="AE139" s="7"/>
       <c r="AF139" s="7"/>
+      <c r="AG139" s="7"/>
     </row>
     <row r="140">
       <c r="A140" s="7" t="inlineStr">
@@ -9419,6 +9562,7 @@
       <c r="AD140" s="7"/>
       <c r="AE140" s="7"/>
       <c r="AF140" s="7"/>
+      <c r="AG140" s="7"/>
     </row>
     <row r="141">
       <c r="A141" s="7" t="inlineStr">
@@ -9493,6 +9637,7 @@
       <c r="AD141" s="7"/>
       <c r="AE141" s="7"/>
       <c r="AF141" s="7"/>
+      <c r="AG141" s="7"/>
     </row>
     <row r="142">
       <c r="A142" s="7" t="inlineStr">
@@ -9555,6 +9700,7 @@
       <c r="AD142" s="7"/>
       <c r="AE142" s="7"/>
       <c r="AF142" s="7"/>
+      <c r="AG142" s="7"/>
     </row>
     <row r="143">
       <c r="A143" s="7" t="inlineStr">
@@ -9617,6 +9763,7 @@
       <c r="AD143" s="7"/>
       <c r="AE143" s="7"/>
       <c r="AF143" s="7"/>
+      <c r="AG143" s="7"/>
     </row>
     <row r="144">
       <c r="A144" s="7" t="inlineStr">
@@ -9679,6 +9826,7 @@
       <c r="AD144" s="7"/>
       <c r="AE144" s="7"/>
       <c r="AF144" s="7"/>
+      <c r="AG144" s="7"/>
     </row>
     <row r="145">
       <c r="A145" s="7" t="inlineStr">
@@ -9757,6 +9905,7 @@
       <c r="AD145" s="7"/>
       <c r="AE145" s="7"/>
       <c r="AF145" s="7"/>
+      <c r="AG145" s="7"/>
     </row>
     <row r="146">
       <c r="A146" s="7" t="inlineStr">
@@ -9823,6 +9972,7 @@
       <c r="AD146" s="7"/>
       <c r="AE146" s="7"/>
       <c r="AF146" s="7"/>
+      <c r="AG146" s="7"/>
     </row>
     <row r="147">
       <c r="A147" s="7" t="inlineStr">
@@ -9901,6 +10051,7 @@
       <c r="AD147" s="7"/>
       <c r="AE147" s="7"/>
       <c r="AF147" s="7"/>
+      <c r="AG147" s="7"/>
     </row>
     <row r="148">
       <c r="A148" s="7" t="inlineStr">
@@ -9963,6 +10114,7 @@
       <c r="AD148" s="7"/>
       <c r="AE148" s="7"/>
       <c r="AF148" s="7"/>
+      <c r="AG148" s="7"/>
     </row>
     <row r="149">
       <c r="A149" s="7" t="inlineStr">
@@ -10033,6 +10185,7 @@
       <c r="AD149" s="7"/>
       <c r="AE149" s="7"/>
       <c r="AF149" s="7"/>
+      <c r="AG149" s="7"/>
     </row>
     <row r="150">
       <c r="A150" s="7" t="inlineStr">
@@ -10107,6 +10260,7 @@
       <c r="AD150" s="7"/>
       <c r="AE150" s="7"/>
       <c r="AF150" s="7"/>
+      <c r="AG150" s="7"/>
     </row>
     <row r="151">
       <c r="A151" s="7" t="inlineStr">
@@ -10173,6 +10327,7 @@
       <c r="AD151" s="7"/>
       <c r="AE151" s="7"/>
       <c r="AF151" s="7"/>
+      <c r="AG151" s="7"/>
     </row>
     <row r="152">
       <c r="A152" s="7" t="inlineStr">
@@ -10243,6 +10398,7 @@
       <c r="AD152" s="7"/>
       <c r="AE152" s="7"/>
       <c r="AF152" s="7"/>
+      <c r="AG152" s="7"/>
     </row>
     <row r="153">
       <c r="A153" s="7" t="inlineStr">
@@ -10313,6 +10469,7 @@
       <c r="AD153" s="7"/>
       <c r="AE153" s="7"/>
       <c r="AF153" s="7"/>
+      <c r="AG153" s="7"/>
     </row>
     <row r="154">
       <c r="A154" s="7" t="inlineStr">
@@ -10371,6 +10528,7 @@
       <c r="AD154" s="7"/>
       <c r="AE154" s="7"/>
       <c r="AF154" s="7"/>
+      <c r="AG154" s="7"/>
     </row>
     <row r="155">
       <c r="A155" s="7" t="inlineStr">
@@ -10433,6 +10591,7 @@
       <c r="AD155" s="7"/>
       <c r="AE155" s="7"/>
       <c r="AF155" s="7"/>
+      <c r="AG155" s="7"/>
     </row>
     <row r="156">
       <c r="A156" s="7" t="inlineStr">
@@ -10499,6 +10658,7 @@
       <c r="AD156" s="7"/>
       <c r="AE156" s="7"/>
       <c r="AF156" s="7"/>
+      <c r="AG156" s="7"/>
     </row>
     <row r="157">
       <c r="A157" s="7" t="inlineStr">
@@ -10561,6 +10721,7 @@
       <c r="AD157" s="7"/>
       <c r="AE157" s="7"/>
       <c r="AF157" s="7"/>
+      <c r="AG157" s="7"/>
     </row>
     <row r="158">
       <c r="A158" s="7" t="inlineStr">
@@ -10623,6 +10784,7 @@
       <c r="AD158" s="7"/>
       <c r="AE158" s="7"/>
       <c r="AF158" s="7"/>
+      <c r="AG158" s="7"/>
     </row>
     <row r="159">
       <c r="A159" s="7" t="inlineStr">
@@ -10685,6 +10847,7 @@
       <c r="AD159" s="7"/>
       <c r="AE159" s="7"/>
       <c r="AF159" s="7"/>
+      <c r="AG159" s="7"/>
     </row>
     <row r="160">
       <c r="A160" s="7" t="inlineStr">
@@ -10747,6 +10910,7 @@
       <c r="AD160" s="7"/>
       <c r="AE160" s="7"/>
       <c r="AF160" s="7"/>
+      <c r="AG160" s="7"/>
     </row>
     <row r="161">
       <c r="A161" s="7" t="inlineStr">
@@ -10813,6 +10977,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AG161" s="7"/>
     </row>
     <row r="162">
       <c r="A162" s="7" t="inlineStr">
@@ -10875,6 +11040,7 @@
       <c r="AD162" s="7"/>
       <c r="AE162" s="7"/>
       <c r="AF162" s="7"/>
+      <c r="AG162" s="7"/>
     </row>
     <row r="163">
       <c r="A163" s="7" t="inlineStr">
@@ -10937,6 +11103,7 @@
       <c r="AD163" s="7"/>
       <c r="AE163" s="7"/>
       <c r="AF163" s="7"/>
+      <c r="AG163" s="7"/>
     </row>
     <row r="164">
       <c r="A164" s="7" t="inlineStr">
@@ -10999,6 +11166,7 @@
       <c r="AD164" s="7"/>
       <c r="AE164" s="7"/>
       <c r="AF164" s="7"/>
+      <c r="AG164" s="7"/>
     </row>
     <row r="165">
       <c r="A165" s="7" t="inlineStr">
@@ -11061,6 +11229,7 @@
       <c r="AD165" s="7"/>
       <c r="AE165" s="7"/>
       <c r="AF165" s="7"/>
+      <c r="AG165" s="7"/>
     </row>
     <row r="166">
       <c r="A166" s="7" t="inlineStr">
@@ -11127,6 +11296,7 @@
       </c>
       <c r="AE166" s="7"/>
       <c r="AF166" s="7"/>
+      <c r="AG166" s="7"/>
     </row>
     <row r="167">
       <c r="A167" s="7" t="inlineStr">
@@ -11189,6 +11359,7 @@
       <c r="AD167" s="7"/>
       <c r="AE167" s="7"/>
       <c r="AF167" s="7"/>
+      <c r="AG167" s="7"/>
     </row>
     <row r="168">
       <c r="A168" s="7" t="inlineStr">
@@ -11251,6 +11422,7 @@
       <c r="AD168" s="7"/>
       <c r="AE168" s="7"/>
       <c r="AF168" s="7"/>
+      <c r="AG168" s="7"/>
     </row>
     <row r="169">
       <c r="A169" s="7" t="inlineStr">
@@ -11313,6 +11485,7 @@
       </c>
       <c r="AE169" s="7"/>
       <c r="AF169" s="7"/>
+      <c r="AG169" s="7"/>
     </row>
     <row r="170">
       <c r="A170" s="7" t="inlineStr">
@@ -11379,6 +11552,7 @@
         </is>
       </c>
       <c r="AF170" s="7"/>
+      <c r="AG170" s="7"/>
     </row>
     <row r="171">
       <c r="A171" s="7" t="inlineStr">
@@ -11437,6 +11611,7 @@
       <c r="AD171" s="7"/>
       <c r="AE171" s="7"/>
       <c r="AF171" s="7"/>
+      <c r="AG171" s="7"/>
     </row>
     <row r="172">
       <c r="A172" s="7" t="inlineStr">
@@ -11495,6 +11670,7 @@
       <c r="AD172" s="7"/>
       <c r="AE172" s="7"/>
       <c r="AF172" s="7"/>
+      <c r="AG172" s="7"/>
     </row>
     <row r="173">
       <c r="A173" s="7" t="inlineStr">
@@ -11561,6 +11737,7 @@
         </is>
       </c>
       <c r="AF173" s="7"/>
+      <c r="AG173" s="7"/>
     </row>
     <row r="174">
       <c r="A174" s="7" t="inlineStr">
@@ -11623,6 +11800,7 @@
       </c>
       <c r="AE174" s="7"/>
       <c r="AF174" s="7"/>
+      <c r="AG174" s="7"/>
     </row>
     <row r="175">
       <c r="A175" s="7" t="inlineStr">
@@ -11689,6 +11867,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AG175" s="7"/>
     </row>
     <row r="176">
       <c r="A176" s="7" t="inlineStr">
@@ -11751,6 +11930,7 @@
         </is>
       </c>
       <c r="AF176" s="7"/>
+      <c r="AG176" s="7"/>
     </row>
     <row r="177">
       <c r="A177" s="7" t="inlineStr">
@@ -11813,6 +11993,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AG177" s="7"/>
     </row>
     <row r="178">
       <c r="A178" s="7" t="inlineStr">
@@ -11875,6 +12056,7 @@
         </is>
       </c>
       <c r="AF178" s="7"/>
+      <c r="AG178" s="7"/>
     </row>
     <row r="179">
       <c r="A179" s="7" t="inlineStr">
@@ -11937,6 +12119,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AG179" s="7"/>
     </row>
     <row r="180">
       <c r="A180" s="7" t="inlineStr">
@@ -11995,6 +12178,133 @@
       <c r="AD180" s="7"/>
       <c r="AE180" s="7"/>
       <c r="AF180" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="AG180" s="7"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_173</t>
+        </is>
+      </c>
+      <c r="B181" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C181" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도전 배지</t>
+        </is>
+      </c>
+      <c r="D181" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">목표 줄 문구</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도전 층 배지 목표 줄이 「목표: {주제} · 전투력 {요구치} 넘기기」로 보이는가?(「출력」 아님 · 수는 그대로 · 파밍 줄 그대로)</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#180</t>
+        </is>
+      </c>
+      <c r="G181" s="7"/>
+      <c r="H181" s="7"/>
+      <c r="I181" s="7"/>
+      <c r="J181" s="7"/>
+      <c r="K181" s="7"/>
+      <c r="L181" s="7"/>
+      <c r="M181" s="7"/>
+      <c r="N181" s="7"/>
+      <c r="O181" s="7"/>
+      <c r="P181" s="7"/>
+      <c r="Q181" s="7"/>
+      <c r="R181" s="7"/>
+      <c r="S181" s="7"/>
+      <c r="T181" s="7"/>
+      <c r="U181" s="7"/>
+      <c r="V181" s="7"/>
+      <c r="W181" s="7"/>
+      <c r="X181" s="7"/>
+      <c r="Y181" s="7"/>
+      <c r="Z181" s="7"/>
+      <c r="AA181" s="7"/>
+      <c r="AB181" s="7"/>
+      <c r="AC181" s="7"/>
+      <c r="AD181" s="7"/>
+      <c r="AE181" s="7"/>
+      <c r="AF181" s="7"/>
+      <c r="AG181" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_174</t>
+        </is>
+      </c>
+      <c r="B182" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">조립</t>
+        </is>
+      </c>
+      <c r="C182" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">보드</t>
+        </is>
+      </c>
+      <c r="D182" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">줌아웃 하한</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t xml:space="preserve">조립 화면에서 휠 · 핀치로 줌아웃하면 종전보다 1.5배 더 멀리(칸이 2/3 크기) 보이고, 그 배율에서도 노드 이름판이 읽히며 탭 · 벨트 드래그가 맞는 칸에 먹는가?</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#181</t>
+        </is>
+      </c>
+      <c r="G182" s="7"/>
+      <c r="H182" s="7"/>
+      <c r="I182" s="7"/>
+      <c r="J182" s="7"/>
+      <c r="K182" s="7"/>
+      <c r="L182" s="7"/>
+      <c r="M182" s="7"/>
+      <c r="N182" s="7"/>
+      <c r="O182" s="7"/>
+      <c r="P182" s="7"/>
+      <c r="Q182" s="7"/>
+      <c r="R182" s="7"/>
+      <c r="S182" s="7"/>
+      <c r="T182" s="7"/>
+      <c r="U182" s="7"/>
+      <c r="V182" s="7"/>
+      <c r="W182" s="7"/>
+      <c r="X182" s="7"/>
+      <c r="Y182" s="7"/>
+      <c r="Z182" s="7"/>
+      <c r="AA182" s="7"/>
+      <c r="AB182" s="7"/>
+      <c r="AC182" s="7"/>
+      <c r="AD182" s="7"/>
+      <c r="AE182" s="7"/>
+      <c r="AF182" s="7"/>
+      <c r="AG182" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -12027,9 +12337,9 @@
     <mergeCell ref="B92:B99"/>
     <mergeCell ref="B100:B106"/>
     <mergeCell ref="B107:B111"/>
-    <mergeCell ref="G7:AF7"/>
+    <mergeCell ref="G7:AG7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:AF180">
+  <conditionalFormatting sqref="G9:AG182">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
docs: QA AH열(d70b00c · CID_175~180) · 촬영 가이드 8132 후보 · 해금 컷 넣지 않음
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -189,8 +189,9 @@
     <col min="31" max="31" width="12" customWidth="1"/>
     <col min="32" max="32" width="12" customWidth="1"/>
     <col min="33" max="33" width="12" customWidth="1"/>
-    <col min="34" max="34" width="11" customWidth="1"/>
+    <col min="34" max="34" width="12" customWidth="1"/>
     <col min="35" max="35" width="11" customWidth="1"/>
+    <col min="36" max="36" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -438,6 +439,11 @@
       <c r="AG6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">video-261019b 후보 갈아엎음 · #180 도전 배지 「전투력 n 넘기기」 · #181 줌아웃 하한 1/1.5 ‖ 10-19 코드 세션 재확인(8123 · 캔버스 직접 캡처) · 바로가기 S1 → 도전 → 배지 「목표: 벨트 연결 · 전투력 18 넘기기」 · 조립 휠 아래 두 번 → 최저 배율 · 칸 크기 약 2/3 · 보이는 칸 늘어남(데스크톱 판 · 576×1024 둘 다) · 노드 이름판 읽힘(「기초 가공소」 포함) · 최저 배율에서 코어 탭 = 코어 팝오버 · 선택 테두리 그 칸(탭 좌표 맞음) · 벨트 드래그는 이번 판 미확인(도전 층 · 튜토리얼 판) · 보드 전체 12×14 가 한 화면에 다 들지는 않음 · 8131 갈아엎음 14:51:37 · 빈 칸 = 안 지나감 · CID_173~174 새 항목)</t>
+        </is>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">video-261019c 후보(8132 · 새 사본 · 8131 동결) · #182 S4 강화 최소 안내 · #183 T1 노드 단추 전부 잠금 · #184 T4 알림 「…모듈이 열렸습니다」 ‖ 10-19 코드 세션 재확인(인앱 브라우저 · 새 저장 · 소리 0): T1 노드 단추 흐림(고스트 채운 뒤에도) → 벨트 드래그로 채움 → 마운트 가득 → S1 T3 → 도전 → 배지 「전투력 18 넘기기」 → 전멸 → S2 알림 「생산량·생산속도 모듈이 열렸습니다」 → T4 → S2 · S3 전멸 → S4 파밍 해금 막 → 해금(골드 −50) → 둘째 막(「▼ 조립」 구멍 · 「조립에서 마운트를 탭해 강화해보세요」 · 「도전」 눌러도 안 열림) → 조립 = 시야가 A 마운트로 옮겨짐 · 「마운트를 탭한 뒤 강화를 누르세요」 → 포트 칸 탭 = 팝오버(재료 100/100 · 고철 796/300) → 강화 → 「강화 ×1.45 적용」 · 고철 −300 · 탭 줄 다시 밝음 → 전투 = 막 없음 · 「도전」·「스테이지」 밝음 · 빈 칸 = 화면으로 못 만든 조건(재료·고철 부족 · 바로가기 S4) — 시험이 든다(EnhanceMountTutorialTests) · ⚠️ 보드 어둠막은 캡처에서 또렷이 구별 안 됨(T1 판도 같음) · 8132 복사 16:16:17 · CID_175~180 새 항목)</t>
         </is>
       </c>
     </row>
@@ -495,14 +501,15 @@
       <c r="AE7" s="2"/>
       <c r="AF7" s="2"/>
       <c r="AG7" s="2"/>
-      <c r="AH7" s="2" t="inlineStr">
+      <c r="AH7" s="2"/>
+      <c r="AI7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">버전</t>
         </is>
       </c>
-      <c r="AI7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1675623</t>
+      <c r="AJ7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">d70b00c</t>
         </is>
       </c>
     </row>
@@ -662,11 +669,16 @@
       </c>
       <c r="AH8" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">d70b00c</t>
+        </is>
+      </c>
+      <c r="AI8" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">PASSrate</t>
         </is>
       </c>
-      <c r="AI8" s="7">
-        <f>COUNTIF(AG9:AG182,"Pass")</f>
+      <c r="AJ8" s="7">
+        <f>COUNTIF(AH9:AH188,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -763,13 +775,14 @@
       <c r="AE9" s="7"/>
       <c r="AF9" s="7"/>
       <c r="AG9" s="7"/>
-      <c r="AH9" s="2" t="inlineStr">
+      <c r="AH9" s="7"/>
+      <c r="AI9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FAILrate</t>
         </is>
       </c>
-      <c r="AI9" s="7">
-        <f>COUNTIF(AG9:AG182,"Fail")+COUNTIF(AG9:AG182,"Broken")</f>
+      <c r="AJ9" s="7">
+        <f>COUNTIF(AH9:AH188,"Fail")+COUNTIF(AH9:AH188,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -830,13 +843,14 @@
       <c r="AE10" s="7"/>
       <c r="AF10" s="7"/>
       <c r="AG10" s="7"/>
-      <c r="AH10" s="2" t="inlineStr">
+      <c r="AH10" s="7"/>
+      <c r="AI10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">N/A</t>
         </is>
       </c>
-      <c r="AI10" s="7">
-        <f>COUNTIF(AG9:AG182,"N/A")</f>
+      <c r="AJ10" s="7">
+        <f>COUNTIF(AH9:AH188,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -897,13 +911,14 @@
       <c r="AE11" s="7"/>
       <c r="AF11" s="7"/>
       <c r="AG11" s="7"/>
-      <c r="AH11" s="2" t="inlineStr">
+      <c r="AH11" s="7"/>
+      <c r="AI11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">전체 개수</t>
         </is>
       </c>
-      <c r="AI11" s="7">
-        <v>174</v>
+      <c r="AJ11" s="7">
+        <v>180</v>
       </c>
     </row>
     <row r="12">
@@ -964,13 +979,14 @@
       <c r="AE12" s="7"/>
       <c r="AF12" s="7"/>
       <c r="AG12" s="7"/>
-      <c r="AH12" s="2" t="inlineStr">
+      <c r="AH12" s="7"/>
+      <c r="AI12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">진행율</t>
         </is>
       </c>
-      <c r="AI12" s="7">
-        <f>TEXT((COUNTA(AG9:AG182))/174,"0.00%")</f>
+      <c r="AJ12" s="7">
+        <f>TEXT((COUNTA(AH9:AH188))/180,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -1035,6 +1051,7 @@
       <c r="AE13" s="7"/>
       <c r="AF13" s="7"/>
       <c r="AG13" s="7"/>
+      <c r="AH13" s="7"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -1089,6 +1106,7 @@
       <c r="AE14" s="7"/>
       <c r="AF14" s="7"/>
       <c r="AG14" s="7"/>
+      <c r="AH14" s="7"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -1179,6 +1197,7 @@
       <c r="AE15" s="7"/>
       <c r="AF15" s="7"/>
       <c r="AG15" s="7"/>
+      <c r="AH15" s="7"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -1269,6 +1288,7 @@
       <c r="AE16" s="7"/>
       <c r="AF16" s="7"/>
       <c r="AG16" s="7"/>
+      <c r="AH16" s="7"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -1364,6 +1384,7 @@
       <c r="AE17" s="7"/>
       <c r="AF17" s="7"/>
       <c r="AG17" s="7"/>
+      <c r="AH17" s="7"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -1423,6 +1444,7 @@
       <c r="AE18" s="7"/>
       <c r="AF18" s="7"/>
       <c r="AG18" s="7"/>
+      <c r="AH18" s="7"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -1477,6 +1499,7 @@
       <c r="AE19" s="7"/>
       <c r="AF19" s="7"/>
       <c r="AG19" s="7"/>
+      <c r="AH19" s="7"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1531,6 +1554,7 @@
       <c r="AE20" s="7"/>
       <c r="AF20" s="7"/>
       <c r="AG20" s="7"/>
+      <c r="AH20" s="7"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1621,6 +1645,7 @@
       <c r="AE21" s="7"/>
       <c r="AF21" s="7"/>
       <c r="AG21" s="7"/>
+      <c r="AH21" s="7"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1704,6 +1729,7 @@
       <c r="AE22" s="7"/>
       <c r="AF22" s="7"/>
       <c r="AG22" s="7"/>
+      <c r="AH22" s="7"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -1766,6 +1792,7 @@
       <c r="AE23" s="7"/>
       <c r="AF23" s="7"/>
       <c r="AG23" s="7"/>
+      <c r="AH23" s="7"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -1820,6 +1847,7 @@
       <c r="AE24" s="7"/>
       <c r="AF24" s="7"/>
       <c r="AG24" s="7"/>
+      <c r="AH24" s="7"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -1874,6 +1902,7 @@
       <c r="AE25" s="7"/>
       <c r="AF25" s="7"/>
       <c r="AG25" s="7"/>
+      <c r="AH25" s="7"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -1957,6 +1986,7 @@
       <c r="AE26" s="7"/>
       <c r="AF26" s="7"/>
       <c r="AG26" s="7"/>
+      <c r="AH26" s="7"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -2015,6 +2045,7 @@
       <c r="AE27" s="7"/>
       <c r="AF27" s="7"/>
       <c r="AG27" s="7"/>
+      <c r="AH27" s="7"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -2082,6 +2113,7 @@
       <c r="AE28" s="7"/>
       <c r="AF28" s="7"/>
       <c r="AG28" s="7"/>
+      <c r="AH28" s="7"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -2144,6 +2176,7 @@
       <c r="AE29" s="7"/>
       <c r="AF29" s="7"/>
       <c r="AG29" s="7"/>
+      <c r="AH29" s="7"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -2230,6 +2263,7 @@
       <c r="AE30" s="7"/>
       <c r="AF30" s="7"/>
       <c r="AG30" s="7"/>
+      <c r="AH30" s="7"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -2321,6 +2355,7 @@
       <c r="AE31" s="7"/>
       <c r="AF31" s="7"/>
       <c r="AG31" s="7"/>
+      <c r="AH31" s="7"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -2399,6 +2434,7 @@
       <c r="AE32" s="7"/>
       <c r="AF32" s="7"/>
       <c r="AG32" s="7"/>
+      <c r="AH32" s="7"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -2485,6 +2521,7 @@
       <c r="AE33" s="7"/>
       <c r="AF33" s="7"/>
       <c r="AG33" s="7"/>
+      <c r="AH33" s="7"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -2571,6 +2608,7 @@
       <c r="AE34" s="7"/>
       <c r="AF34" s="7"/>
       <c r="AG34" s="7"/>
+      <c r="AH34" s="7"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -2666,6 +2704,7 @@
       <c r="AE35" s="7"/>
       <c r="AF35" s="7"/>
       <c r="AG35" s="7"/>
+      <c r="AH35" s="7"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -2736,6 +2775,7 @@
       <c r="AE36" s="7"/>
       <c r="AF36" s="7"/>
       <c r="AG36" s="7"/>
+      <c r="AH36" s="7"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -2790,6 +2830,7 @@
       <c r="AE37" s="7"/>
       <c r="AF37" s="7"/>
       <c r="AG37" s="7"/>
+      <c r="AH37" s="7"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -2865,6 +2906,7 @@
       <c r="AE38" s="7"/>
       <c r="AF38" s="7"/>
       <c r="AG38" s="7"/>
+      <c r="AH38" s="7"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -2951,6 +2993,7 @@
       <c r="AE39" s="7"/>
       <c r="AF39" s="7"/>
       <c r="AG39" s="7"/>
+      <c r="AH39" s="7"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -3038,6 +3081,7 @@
       <c r="AE40" s="7"/>
       <c r="AF40" s="7"/>
       <c r="AG40" s="7"/>
+      <c r="AH40" s="7"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -3120,6 +3164,7 @@
       <c r="AE41" s="7"/>
       <c r="AF41" s="7"/>
       <c r="AG41" s="7"/>
+      <c r="AH41" s="7"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -3186,6 +3231,7 @@
       <c r="AE42" s="7"/>
       <c r="AF42" s="7"/>
       <c r="AG42" s="7"/>
+      <c r="AH42" s="7"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -3272,6 +3318,7 @@
       <c r="AE43" s="7"/>
       <c r="AF43" s="7"/>
       <c r="AG43" s="7"/>
+      <c r="AH43" s="7"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -3331,6 +3378,7 @@
       <c r="AE44" s="7"/>
       <c r="AF44" s="7"/>
       <c r="AG44" s="7"/>
+      <c r="AH44" s="7"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -3413,6 +3461,7 @@
       <c r="AE45" s="7"/>
       <c r="AF45" s="7"/>
       <c r="AG45" s="7"/>
+      <c r="AH45" s="7"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -3495,6 +3544,7 @@
       <c r="AE46" s="7"/>
       <c r="AF46" s="7"/>
       <c r="AG46" s="7"/>
+      <c r="AH46" s="7"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -3554,6 +3604,7 @@
       <c r="AE47" s="7"/>
       <c r="AF47" s="7"/>
       <c r="AG47" s="7"/>
+      <c r="AH47" s="7"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -3608,6 +3659,7 @@
       <c r="AE48" s="7"/>
       <c r="AF48" s="7"/>
       <c r="AG48" s="7"/>
+      <c r="AH48" s="7"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -3662,6 +3714,7 @@
       <c r="AE49" s="7"/>
       <c r="AF49" s="7"/>
       <c r="AG49" s="7"/>
+      <c r="AH49" s="7"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -3740,6 +3793,7 @@
       <c r="AE50" s="7"/>
       <c r="AF50" s="7"/>
       <c r="AG50" s="7"/>
+      <c r="AH50" s="7"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -3818,6 +3872,7 @@
       <c r="AE51" s="7"/>
       <c r="AF51" s="7"/>
       <c r="AG51" s="7"/>
+      <c r="AH51" s="7"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -3877,6 +3932,7 @@
       <c r="AE52" s="7"/>
       <c r="AF52" s="7"/>
       <c r="AG52" s="7"/>
+      <c r="AH52" s="7"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -3936,6 +3992,7 @@
       <c r="AE53" s="7"/>
       <c r="AF53" s="7"/>
       <c r="AG53" s="7"/>
+      <c r="AH53" s="7"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -3990,6 +4047,7 @@
       <c r="AE54" s="7"/>
       <c r="AF54" s="7"/>
       <c r="AG54" s="7"/>
+      <c r="AH54" s="7"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -4080,6 +4138,7 @@
       <c r="AE55" s="7"/>
       <c r="AF55" s="7"/>
       <c r="AG55" s="7"/>
+      <c r="AH55" s="7"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -4150,6 +4209,7 @@
       <c r="AE56" s="7"/>
       <c r="AF56" s="7"/>
       <c r="AG56" s="7"/>
+      <c r="AH56" s="7"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -4229,6 +4289,7 @@
       <c r="AE57" s="7"/>
       <c r="AF57" s="7"/>
       <c r="AG57" s="7"/>
+      <c r="AH57" s="7"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -4316,6 +4377,7 @@
       <c r="AE58" s="7"/>
       <c r="AF58" s="7"/>
       <c r="AG58" s="7"/>
+      <c r="AH58" s="7"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -4370,6 +4432,7 @@
       <c r="AE59" s="7"/>
       <c r="AF59" s="7"/>
       <c r="AG59" s="7"/>
+      <c r="AH59" s="7"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -4424,6 +4487,7 @@
       <c r="AE60" s="7"/>
       <c r="AF60" s="7"/>
       <c r="AG60" s="7"/>
+      <c r="AH60" s="7"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -4490,6 +4554,7 @@
       <c r="AE61" s="7"/>
       <c r="AF61" s="7"/>
       <c r="AG61" s="7"/>
+      <c r="AH61" s="7"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -4564,6 +4629,7 @@
       <c r="AE62" s="7"/>
       <c r="AF62" s="7"/>
       <c r="AG62" s="7"/>
+      <c r="AH62" s="7"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -4630,6 +4696,7 @@
       <c r="AE63" s="7"/>
       <c r="AF63" s="7"/>
       <c r="AG63" s="7"/>
+      <c r="AH63" s="7"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -4684,6 +4751,7 @@
       <c r="AE64" s="7"/>
       <c r="AF64" s="7"/>
       <c r="AG64" s="7"/>
+      <c r="AH64" s="7"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -4743,6 +4811,7 @@
       <c r="AE65" s="7"/>
       <c r="AF65" s="7"/>
       <c r="AG65" s="7"/>
+      <c r="AH65" s="7"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
@@ -4809,6 +4878,7 @@
       <c r="AE66" s="7"/>
       <c r="AF66" s="7"/>
       <c r="AG66" s="7"/>
+      <c r="AH66" s="7"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -4863,6 +4933,7 @@
       <c r="AE67" s="7"/>
       <c r="AF67" s="7"/>
       <c r="AG67" s="7"/>
+      <c r="AH67" s="7"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
@@ -4921,6 +4992,7 @@
       <c r="AE68" s="7"/>
       <c r="AF68" s="7"/>
       <c r="AG68" s="7"/>
+      <c r="AH68" s="7"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -5011,6 +5083,7 @@
       <c r="AE69" s="7"/>
       <c r="AF69" s="7"/>
       <c r="AG69" s="7"/>
+      <c r="AH69" s="7"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
@@ -5065,6 +5138,7 @@
       <c r="AE70" s="7"/>
       <c r="AF70" s="7"/>
       <c r="AG70" s="7"/>
+      <c r="AH70" s="7"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -5124,6 +5198,7 @@
       <c r="AE71" s="7"/>
       <c r="AF71" s="7"/>
       <c r="AG71" s="7"/>
+      <c r="AH71" s="7"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
@@ -5194,6 +5269,7 @@
       <c r="AE72" s="7"/>
       <c r="AF72" s="7"/>
       <c r="AG72" s="7"/>
+      <c r="AH72" s="7"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
@@ -5253,6 +5329,7 @@
       <c r="AE73" s="7"/>
       <c r="AF73" s="7"/>
       <c r="AG73" s="7"/>
+      <c r="AH73" s="7"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -5307,6 +5384,7 @@
       <c r="AE74" s="7"/>
       <c r="AF74" s="7"/>
       <c r="AG74" s="7"/>
+      <c r="AH74" s="7"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -5361,6 +5439,7 @@
       <c r="AE75" s="7"/>
       <c r="AF75" s="7"/>
       <c r="AG75" s="7"/>
+      <c r="AH75" s="7"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -5415,6 +5494,7 @@
       <c r="AE76" s="7"/>
       <c r="AF76" s="7"/>
       <c r="AG76" s="7"/>
+      <c r="AH76" s="7"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -5473,6 +5553,7 @@
       <c r="AE77" s="7"/>
       <c r="AF77" s="7"/>
       <c r="AG77" s="7"/>
+      <c r="AH77" s="7"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
@@ -5527,6 +5608,7 @@
       <c r="AE78" s="7"/>
       <c r="AF78" s="7"/>
       <c r="AG78" s="7"/>
+      <c r="AH78" s="7"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -5586,6 +5668,7 @@
       <c r="AE79" s="7"/>
       <c r="AF79" s="7"/>
       <c r="AG79" s="7"/>
+      <c r="AH79" s="7"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
@@ -5656,6 +5739,7 @@
       <c r="AE80" s="7"/>
       <c r="AF80" s="7"/>
       <c r="AG80" s="7"/>
+      <c r="AH80" s="7"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
@@ -5714,6 +5798,7 @@
       <c r="AE81" s="7"/>
       <c r="AF81" s="7"/>
       <c r="AG81" s="7"/>
+      <c r="AH81" s="7"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
@@ -5768,6 +5853,7 @@
       <c r="AE82" s="7"/>
       <c r="AF82" s="7"/>
       <c r="AG82" s="7"/>
+      <c r="AH82" s="7"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
@@ -5827,6 +5913,7 @@
       <c r="AE83" s="7"/>
       <c r="AF83" s="7"/>
       <c r="AG83" s="7"/>
+      <c r="AH83" s="7"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
@@ -5881,6 +5968,7 @@
       <c r="AE84" s="7"/>
       <c r="AF84" s="7"/>
       <c r="AG84" s="7"/>
+      <c r="AH84" s="7"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
@@ -5935,6 +6023,7 @@
       <c r="AE85" s="7"/>
       <c r="AF85" s="7"/>
       <c r="AG85" s="7"/>
+      <c r="AH85" s="7"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
@@ -5994,6 +6083,7 @@
       <c r="AE86" s="7"/>
       <c r="AF86" s="7"/>
       <c r="AG86" s="7"/>
+      <c r="AH86" s="7"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
@@ -6048,6 +6138,7 @@
       <c r="AE87" s="7"/>
       <c r="AF87" s="7"/>
       <c r="AG87" s="7"/>
+      <c r="AH87" s="7"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
@@ -6102,6 +6193,7 @@
       <c r="AE88" s="7"/>
       <c r="AF88" s="7"/>
       <c r="AG88" s="7"/>
+      <c r="AH88" s="7"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
@@ -6156,6 +6248,7 @@
       <c r="AE89" s="7"/>
       <c r="AF89" s="7"/>
       <c r="AG89" s="7"/>
+      <c r="AH89" s="7"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
@@ -6239,6 +6332,7 @@
       <c r="AE90" s="7"/>
       <c r="AF90" s="7"/>
       <c r="AG90" s="7"/>
+      <c r="AH90" s="7"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
@@ -6293,6 +6387,7 @@
       <c r="AE91" s="7"/>
       <c r="AF91" s="7"/>
       <c r="AG91" s="7"/>
+      <c r="AH91" s="7"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
@@ -6383,6 +6478,7 @@
       <c r="AE92" s="7"/>
       <c r="AF92" s="7"/>
       <c r="AG92" s="7"/>
+      <c r="AH92" s="7"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
@@ -6478,6 +6574,7 @@
       <c r="AE93" s="7"/>
       <c r="AF93" s="7"/>
       <c r="AG93" s="7"/>
+      <c r="AH93" s="7"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
@@ -6537,6 +6634,7 @@
       <c r="AE94" s="7"/>
       <c r="AF94" s="7"/>
       <c r="AG94" s="7"/>
+      <c r="AH94" s="7"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
@@ -6596,6 +6694,7 @@
       <c r="AE95" s="7"/>
       <c r="AF95" s="7"/>
       <c r="AG95" s="7"/>
+      <c r="AH95" s="7"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
@@ -6674,6 +6773,7 @@
       <c r="AE96" s="7"/>
       <c r="AF96" s="7"/>
       <c r="AG96" s="7"/>
+      <c r="AH96" s="7"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="inlineStr">
@@ -6728,6 +6828,7 @@
       <c r="AE97" s="7"/>
       <c r="AF97" s="7"/>
       <c r="AG97" s="7"/>
+      <c r="AH97" s="7"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
@@ -6782,6 +6883,7 @@
       <c r="AE98" s="7"/>
       <c r="AF98" s="7"/>
       <c r="AG98" s="7"/>
+      <c r="AH98" s="7"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
@@ -6836,6 +6938,7 @@
       <c r="AE99" s="7"/>
       <c r="AF99" s="7"/>
       <c r="AG99" s="7"/>
+      <c r="AH99" s="7"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
@@ -6899,6 +7002,7 @@
       <c r="AE100" s="7"/>
       <c r="AF100" s="7"/>
       <c r="AG100" s="7"/>
+      <c r="AH100" s="7"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
@@ -6953,6 +7057,7 @@
       <c r="AE101" s="7"/>
       <c r="AF101" s="7"/>
       <c r="AG101" s="7"/>
+      <c r="AH101" s="7"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
@@ -7007,6 +7112,7 @@
       <c r="AE102" s="7"/>
       <c r="AF102" s="7"/>
       <c r="AG102" s="7"/>
+      <c r="AH102" s="7"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="inlineStr">
@@ -7061,6 +7167,7 @@
       <c r="AE103" s="7"/>
       <c r="AF103" s="7"/>
       <c r="AG103" s="7"/>
+      <c r="AH103" s="7"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="inlineStr">
@@ -7120,6 +7227,7 @@
       <c r="AE104" s="7"/>
       <c r="AF104" s="7"/>
       <c r="AG104" s="7"/>
+      <c r="AH104" s="7"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
@@ -7174,6 +7282,7 @@
       <c r="AE105" s="7"/>
       <c r="AF105" s="7"/>
       <c r="AG105" s="7"/>
+      <c r="AH105" s="7"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
@@ -7228,6 +7337,7 @@
       <c r="AE106" s="7"/>
       <c r="AF106" s="7"/>
       <c r="AG106" s="7"/>
+      <c r="AH106" s="7"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
@@ -7282,6 +7392,7 @@
       <c r="AE107" s="7"/>
       <c r="AF107" s="7"/>
       <c r="AG107" s="7"/>
+      <c r="AH107" s="7"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
@@ -7340,6 +7451,7 @@
       <c r="AE108" s="7"/>
       <c r="AF108" s="7"/>
       <c r="AG108" s="7"/>
+      <c r="AH108" s="7"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="inlineStr">
@@ -7403,6 +7515,7 @@
       <c r="AE109" s="7"/>
       <c r="AF109" s="7"/>
       <c r="AG109" s="7"/>
+      <c r="AH109" s="7"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
@@ -7474,6 +7587,7 @@
       <c r="AE110" s="7"/>
       <c r="AF110" s="7"/>
       <c r="AG110" s="7"/>
+      <c r="AH110" s="7"/>
     </row>
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
@@ -7548,6 +7662,7 @@
       <c r="AE111" s="7"/>
       <c r="AF111" s="7"/>
       <c r="AG111" s="7"/>
+      <c r="AH111" s="7"/>
     </row>
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
@@ -7619,6 +7734,7 @@
       <c r="AE112" s="7"/>
       <c r="AF112" s="7"/>
       <c r="AG112" s="7"/>
+      <c r="AH112" s="7"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
@@ -7682,6 +7798,7 @@
       <c r="AE113" s="7"/>
       <c r="AF113" s="7"/>
       <c r="AG113" s="7"/>
+      <c r="AH113" s="7"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="inlineStr">
@@ -7761,6 +7878,7 @@
       <c r="AE114" s="7"/>
       <c r="AF114" s="7"/>
       <c r="AG114" s="7"/>
+      <c r="AH114" s="7"/>
     </row>
     <row r="115">
       <c r="A115" s="7" t="inlineStr">
@@ -7832,6 +7950,7 @@
       <c r="AE115" s="7"/>
       <c r="AF115" s="7"/>
       <c r="AG115" s="7"/>
+      <c r="AH115" s="7"/>
     </row>
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
@@ -7861,7 +7980,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t xml:space="preserve">표시 4초(가정) · 알림이 걷힌 뒤 막 (10-15 #138) · 10-15 #147 로 문안 「생산량·생산속도 모듈을 받았습니다」 · 경로 무관(CID_121)</t>
+          <t xml:space="preserve">표시 4초(가정) · 알림이 걷힌 뒤 막 (10-15 #138) · 10-15 #147 로 문안 「생산량·생산속도 모듈을 받았습니다」 · 경로 무관(CID_121) · 10-19 #184 로 문안 「생산량·생산속도 모듈이 열렸습니다」</t>
         </is>
       </c>
       <c r="G116" s="7"/>
@@ -7907,6 +8026,11 @@
       <c r="AE116" s="7"/>
       <c r="AF116" s="7"/>
       <c r="AG116" s="7"/>
+      <c r="AH116" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
@@ -7982,6 +8106,7 @@
       <c r="AE117" s="7"/>
       <c r="AF117" s="7"/>
       <c r="AG117" s="7"/>
+      <c r="AH117" s="7"/>
     </row>
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
@@ -8057,6 +8182,7 @@
       <c r="AE118" s="7"/>
       <c r="AF118" s="7"/>
       <c r="AG118" s="7"/>
+      <c r="AH118" s="7"/>
     </row>
     <row r="119">
       <c r="A119" s="7" t="inlineStr">
@@ -8128,6 +8254,7 @@
       <c r="AE119" s="7"/>
       <c r="AF119" s="7"/>
       <c r="AG119" s="7"/>
+      <c r="AH119" s="7"/>
     </row>
     <row r="120">
       <c r="A120" s="7" t="inlineStr">
@@ -8191,6 +8318,7 @@
       <c r="AE120" s="7"/>
       <c r="AF120" s="7"/>
       <c r="AG120" s="7"/>
+      <c r="AH120" s="7"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="inlineStr">
@@ -8266,6 +8394,7 @@
       <c r="AE121" s="7"/>
       <c r="AF121" s="7"/>
       <c r="AG121" s="7"/>
+      <c r="AH121" s="7"/>
     </row>
     <row r="122">
       <c r="A122" s="7" t="inlineStr">
@@ -8341,6 +8470,7 @@
       <c r="AE122" s="7"/>
       <c r="AF122" s="7"/>
       <c r="AG122" s="7"/>
+      <c r="AH122" s="7"/>
     </row>
     <row r="123">
       <c r="A123" s="7" t="inlineStr">
@@ -8404,6 +8534,7 @@
       <c r="AE123" s="7"/>
       <c r="AF123" s="7"/>
       <c r="AG123" s="7"/>
+      <c r="AH123" s="7"/>
     </row>
     <row r="124">
       <c r="A124" s="7" t="inlineStr">
@@ -8475,6 +8606,7 @@
       <c r="AE124" s="7"/>
       <c r="AF124" s="7"/>
       <c r="AG124" s="7"/>
+      <c r="AH124" s="7"/>
     </row>
     <row r="125">
       <c r="A125" s="7" t="inlineStr">
@@ -8538,6 +8670,7 @@
       <c r="AE125" s="7"/>
       <c r="AF125" s="7"/>
       <c r="AG125" s="7"/>
+      <c r="AH125" s="7"/>
     </row>
     <row r="126">
       <c r="A126" s="7" t="inlineStr">
@@ -8601,6 +8734,7 @@
       <c r="AE126" s="7"/>
       <c r="AF126" s="7"/>
       <c r="AG126" s="7"/>
+      <c r="AH126" s="7"/>
     </row>
     <row r="127">
       <c r="A127" s="7" t="inlineStr">
@@ -8668,6 +8802,7 @@
       <c r="AE127" s="7"/>
       <c r="AF127" s="7"/>
       <c r="AG127" s="7"/>
+      <c r="AH127" s="7"/>
     </row>
     <row r="128">
       <c r="A128" s="7" t="inlineStr">
@@ -8735,6 +8870,7 @@
       <c r="AE128" s="7"/>
       <c r="AF128" s="7"/>
       <c r="AG128" s="7"/>
+      <c r="AH128" s="7"/>
     </row>
     <row r="129">
       <c r="A129" s="7" t="inlineStr">
@@ -8802,6 +8938,7 @@
       <c r="AE129" s="7"/>
       <c r="AF129" s="7"/>
       <c r="AG129" s="7"/>
+      <c r="AH129" s="7"/>
     </row>
     <row r="130">
       <c r="A130" s="7" t="inlineStr">
@@ -8865,6 +9002,7 @@
       <c r="AE130" s="7"/>
       <c r="AF130" s="7"/>
       <c r="AG130" s="7"/>
+      <c r="AH130" s="7"/>
     </row>
     <row r="131">
       <c r="A131" s="7" t="inlineStr">
@@ -8936,6 +9074,7 @@
       <c r="AE131" s="7"/>
       <c r="AF131" s="7"/>
       <c r="AG131" s="7"/>
+      <c r="AH131" s="7"/>
     </row>
     <row r="132">
       <c r="A132" s="7" t="inlineStr">
@@ -9011,6 +9150,7 @@
       <c r="AE132" s="7"/>
       <c r="AF132" s="7"/>
       <c r="AG132" s="7"/>
+      <c r="AH132" s="7"/>
     </row>
     <row r="133">
       <c r="A133" s="7" t="inlineStr">
@@ -9086,6 +9226,7 @@
       <c r="AE133" s="7"/>
       <c r="AF133" s="7"/>
       <c r="AG133" s="7"/>
+      <c r="AH133" s="7"/>
     </row>
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
@@ -9157,6 +9298,7 @@
       <c r="AE134" s="7"/>
       <c r="AF134" s="7"/>
       <c r="AG134" s="7"/>
+      <c r="AH134" s="7"/>
     </row>
     <row r="135">
       <c r="A135" s="7" t="inlineStr">
@@ -9228,6 +9370,7 @@
       <c r="AE135" s="7"/>
       <c r="AF135" s="7"/>
       <c r="AG135" s="7"/>
+      <c r="AH135" s="7"/>
     </row>
     <row r="136">
       <c r="A136" s="7" t="inlineStr">
@@ -9299,6 +9442,7 @@
       <c r="AE136" s="7"/>
       <c r="AF136" s="7"/>
       <c r="AG136" s="7"/>
+      <c r="AH136" s="7"/>
     </row>
     <row r="137">
       <c r="A137" s="7" t="inlineStr">
@@ -9366,6 +9510,7 @@
       <c r="AE137" s="7"/>
       <c r="AF137" s="7"/>
       <c r="AG137" s="7"/>
+      <c r="AH137" s="7"/>
     </row>
     <row r="138">
       <c r="A138" s="7" t="inlineStr">
@@ -9433,6 +9578,7 @@
       <c r="AE138" s="7"/>
       <c r="AF138" s="7"/>
       <c r="AG138" s="7"/>
+      <c r="AH138" s="7"/>
     </row>
     <row r="139">
       <c r="A139" s="7" t="inlineStr">
@@ -9500,6 +9646,7 @@
       <c r="AE139" s="7"/>
       <c r="AF139" s="7"/>
       <c r="AG139" s="7"/>
+      <c r="AH139" s="7"/>
     </row>
     <row r="140">
       <c r="A140" s="7" t="inlineStr">
@@ -9563,6 +9710,7 @@
       <c r="AE140" s="7"/>
       <c r="AF140" s="7"/>
       <c r="AG140" s="7"/>
+      <c r="AH140" s="7"/>
     </row>
     <row r="141">
       <c r="A141" s="7" t="inlineStr">
@@ -9638,6 +9786,7 @@
       <c r="AE141" s="7"/>
       <c r="AF141" s="7"/>
       <c r="AG141" s="7"/>
+      <c r="AH141" s="7"/>
     </row>
     <row r="142">
       <c r="A142" s="7" t="inlineStr">
@@ -9701,6 +9850,7 @@
       <c r="AE142" s="7"/>
       <c r="AF142" s="7"/>
       <c r="AG142" s="7"/>
+      <c r="AH142" s="7"/>
     </row>
     <row r="143">
       <c r="A143" s="7" t="inlineStr">
@@ -9764,6 +9914,7 @@
       <c r="AE143" s="7"/>
       <c r="AF143" s="7"/>
       <c r="AG143" s="7"/>
+      <c r="AH143" s="7"/>
     </row>
     <row r="144">
       <c r="A144" s="7" t="inlineStr">
@@ -9827,6 +9978,7 @@
       <c r="AE144" s="7"/>
       <c r="AF144" s="7"/>
       <c r="AG144" s="7"/>
+      <c r="AH144" s="7"/>
     </row>
     <row r="145">
       <c r="A145" s="7" t="inlineStr">
@@ -9906,6 +10058,7 @@
       <c r="AE145" s="7"/>
       <c r="AF145" s="7"/>
       <c r="AG145" s="7"/>
+      <c r="AH145" s="7"/>
     </row>
     <row r="146">
       <c r="A146" s="7" t="inlineStr">
@@ -9973,6 +10126,7 @@
       <c r="AE146" s="7"/>
       <c r="AF146" s="7"/>
       <c r="AG146" s="7"/>
+      <c r="AH146" s="7"/>
     </row>
     <row r="147">
       <c r="A147" s="7" t="inlineStr">
@@ -10052,6 +10206,7 @@
       <c r="AE147" s="7"/>
       <c r="AF147" s="7"/>
       <c r="AG147" s="7"/>
+      <c r="AH147" s="7"/>
     </row>
     <row r="148">
       <c r="A148" s="7" t="inlineStr">
@@ -10115,6 +10270,7 @@
       <c r="AE148" s="7"/>
       <c r="AF148" s="7"/>
       <c r="AG148" s="7"/>
+      <c r="AH148" s="7"/>
     </row>
     <row r="149">
       <c r="A149" s="7" t="inlineStr">
@@ -10186,6 +10342,7 @@
       <c r="AE149" s="7"/>
       <c r="AF149" s="7"/>
       <c r="AG149" s="7"/>
+      <c r="AH149" s="7"/>
     </row>
     <row r="150">
       <c r="A150" s="7" t="inlineStr">
@@ -10261,6 +10418,7 @@
       <c r="AE150" s="7"/>
       <c r="AF150" s="7"/>
       <c r="AG150" s="7"/>
+      <c r="AH150" s="7"/>
     </row>
     <row r="151">
       <c r="A151" s="7" t="inlineStr">
@@ -10328,6 +10486,7 @@
       <c r="AE151" s="7"/>
       <c r="AF151" s="7"/>
       <c r="AG151" s="7"/>
+      <c r="AH151" s="7"/>
     </row>
     <row r="152">
       <c r="A152" s="7" t="inlineStr">
@@ -10399,6 +10558,7 @@
       <c r="AE152" s="7"/>
       <c r="AF152" s="7"/>
       <c r="AG152" s="7"/>
+      <c r="AH152" s="7"/>
     </row>
     <row r="153">
       <c r="A153" s="7" t="inlineStr">
@@ -10470,6 +10630,7 @@
       <c r="AE153" s="7"/>
       <c r="AF153" s="7"/>
       <c r="AG153" s="7"/>
+      <c r="AH153" s="7"/>
     </row>
     <row r="154">
       <c r="A154" s="7" t="inlineStr">
@@ -10529,6 +10690,7 @@
       <c r="AE154" s="7"/>
       <c r="AF154" s="7"/>
       <c r="AG154" s="7"/>
+      <c r="AH154" s="7"/>
     </row>
     <row r="155">
       <c r="A155" s="7" t="inlineStr">
@@ -10592,6 +10754,7 @@
       <c r="AE155" s="7"/>
       <c r="AF155" s="7"/>
       <c r="AG155" s="7"/>
+      <c r="AH155" s="7"/>
     </row>
     <row r="156">
       <c r="A156" s="7" t="inlineStr">
@@ -10659,6 +10822,7 @@
       <c r="AE156" s="7"/>
       <c r="AF156" s="7"/>
       <c r="AG156" s="7"/>
+      <c r="AH156" s="7"/>
     </row>
     <row r="157">
       <c r="A157" s="7" t="inlineStr">
@@ -10722,6 +10886,7 @@
       <c r="AE157" s="7"/>
       <c r="AF157" s="7"/>
       <c r="AG157" s="7"/>
+      <c r="AH157" s="7"/>
     </row>
     <row r="158">
       <c r="A158" s="7" t="inlineStr">
@@ -10785,6 +10950,7 @@
       <c r="AE158" s="7"/>
       <c r="AF158" s="7"/>
       <c r="AG158" s="7"/>
+      <c r="AH158" s="7"/>
     </row>
     <row r="159">
       <c r="A159" s="7" t="inlineStr">
@@ -10848,6 +11014,7 @@
       <c r="AE159" s="7"/>
       <c r="AF159" s="7"/>
       <c r="AG159" s="7"/>
+      <c r="AH159" s="7"/>
     </row>
     <row r="160">
       <c r="A160" s="7" t="inlineStr">
@@ -10911,6 +11078,7 @@
       <c r="AE160" s="7"/>
       <c r="AF160" s="7"/>
       <c r="AG160" s="7"/>
+      <c r="AH160" s="7"/>
     </row>
     <row r="161">
       <c r="A161" s="7" t="inlineStr">
@@ -10978,6 +11146,7 @@
         </is>
       </c>
       <c r="AG161" s="7"/>
+      <c r="AH161" s="7"/>
     </row>
     <row r="162">
       <c r="A162" s="7" t="inlineStr">
@@ -11041,6 +11210,7 @@
       <c r="AE162" s="7"/>
       <c r="AF162" s="7"/>
       <c r="AG162" s="7"/>
+      <c r="AH162" s="7"/>
     </row>
     <row r="163">
       <c r="A163" s="7" t="inlineStr">
@@ -11104,6 +11274,7 @@
       <c r="AE163" s="7"/>
       <c r="AF163" s="7"/>
       <c r="AG163" s="7"/>
+      <c r="AH163" s="7"/>
     </row>
     <row r="164">
       <c r="A164" s="7" t="inlineStr">
@@ -11167,6 +11338,7 @@
       <c r="AE164" s="7"/>
       <c r="AF164" s="7"/>
       <c r="AG164" s="7"/>
+      <c r="AH164" s="7"/>
     </row>
     <row r="165">
       <c r="A165" s="7" t="inlineStr">
@@ -11230,6 +11402,7 @@
       <c r="AE165" s="7"/>
       <c r="AF165" s="7"/>
       <c r="AG165" s="7"/>
+      <c r="AH165" s="7"/>
     </row>
     <row r="166">
       <c r="A166" s="7" t="inlineStr">
@@ -11297,6 +11470,7 @@
       <c r="AE166" s="7"/>
       <c r="AF166" s="7"/>
       <c r="AG166" s="7"/>
+      <c r="AH166" s="7"/>
     </row>
     <row r="167">
       <c r="A167" s="7" t="inlineStr">
@@ -11360,6 +11534,7 @@
       <c r="AE167" s="7"/>
       <c r="AF167" s="7"/>
       <c r="AG167" s="7"/>
+      <c r="AH167" s="7"/>
     </row>
     <row r="168">
       <c r="A168" s="7" t="inlineStr">
@@ -11423,6 +11598,7 @@
       <c r="AE168" s="7"/>
       <c r="AF168" s="7"/>
       <c r="AG168" s="7"/>
+      <c r="AH168" s="7"/>
     </row>
     <row r="169">
       <c r="A169" s="7" t="inlineStr">
@@ -11486,6 +11662,7 @@
       <c r="AE169" s="7"/>
       <c r="AF169" s="7"/>
       <c r="AG169" s="7"/>
+      <c r="AH169" s="7"/>
     </row>
     <row r="170">
       <c r="A170" s="7" t="inlineStr">
@@ -11553,6 +11730,7 @@
       </c>
       <c r="AF170" s="7"/>
       <c r="AG170" s="7"/>
+      <c r="AH170" s="7"/>
     </row>
     <row r="171">
       <c r="A171" s="7" t="inlineStr">
@@ -11612,6 +11790,7 @@
       <c r="AE171" s="7"/>
       <c r="AF171" s="7"/>
       <c r="AG171" s="7"/>
+      <c r="AH171" s="7"/>
     </row>
     <row r="172">
       <c r="A172" s="7" t="inlineStr">
@@ -11671,6 +11850,7 @@
       <c r="AE172" s="7"/>
       <c r="AF172" s="7"/>
       <c r="AG172" s="7"/>
+      <c r="AH172" s="7"/>
     </row>
     <row r="173">
       <c r="A173" s="7" t="inlineStr">
@@ -11738,6 +11918,7 @@
       </c>
       <c r="AF173" s="7"/>
       <c r="AG173" s="7"/>
+      <c r="AH173" s="7"/>
     </row>
     <row r="174">
       <c r="A174" s="7" t="inlineStr">
@@ -11801,6 +11982,7 @@
       <c r="AE174" s="7"/>
       <c r="AF174" s="7"/>
       <c r="AG174" s="7"/>
+      <c r="AH174" s="7"/>
     </row>
     <row r="175">
       <c r="A175" s="7" t="inlineStr">
@@ -11868,6 +12050,7 @@
         </is>
       </c>
       <c r="AG175" s="7"/>
+      <c r="AH175" s="7"/>
     </row>
     <row r="176">
       <c r="A176" s="7" t="inlineStr">
@@ -11931,6 +12114,7 @@
       </c>
       <c r="AF176" s="7"/>
       <c r="AG176" s="7"/>
+      <c r="AH176" s="7"/>
     </row>
     <row r="177">
       <c r="A177" s="7" t="inlineStr">
@@ -11994,6 +12178,7 @@
         </is>
       </c>
       <c r="AG177" s="7"/>
+      <c r="AH177" s="7"/>
     </row>
     <row r="178">
       <c r="A178" s="7" t="inlineStr">
@@ -12057,6 +12242,7 @@
       </c>
       <c r="AF178" s="7"/>
       <c r="AG178" s="7"/>
+      <c r="AH178" s="7"/>
     </row>
     <row r="179">
       <c r="A179" s="7" t="inlineStr">
@@ -12120,6 +12306,7 @@
         </is>
       </c>
       <c r="AG179" s="7"/>
+      <c r="AH179" s="7"/>
     </row>
     <row r="180">
       <c r="A180" s="7" t="inlineStr">
@@ -12183,6 +12370,7 @@
         </is>
       </c>
       <c r="AG180" s="7"/>
+      <c r="AH180" s="7"/>
     </row>
     <row r="181">
       <c r="A181" s="7" t="inlineStr">
@@ -12246,6 +12434,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AH181" s="7"/>
     </row>
     <row r="182">
       <c r="A182" s="7" t="inlineStr">
@@ -12309,6 +12498,387 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AH182" s="7"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_175</t>
+        </is>
+      </c>
+      <c r="B183" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼</t>
+        </is>
+      </c>
+      <c r="C183" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 강화 안내</t>
+        </is>
+      </c>
+      <c r="D183" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투 막</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 파밍에서 로봇 B 를 해금한 뒤(재료 ≥ 100 · 고철 ≥ 300) 막 + 「▼ 조립」 구멍 + 「조립에서 마운트를 탭해 강화해보세요」가 뜨고 「도전」·「스테이지」가 잠기는가? (「▲ 전투로」 예외)</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#182 · 문구 ⚠️ 가정</t>
+        </is>
+      </c>
+      <c r="G183" s="7"/>
+      <c r="H183" s="7"/>
+      <c r="I183" s="7"/>
+      <c r="J183" s="7"/>
+      <c r="K183" s="7"/>
+      <c r="L183" s="7"/>
+      <c r="M183" s="7"/>
+      <c r="N183" s="7"/>
+      <c r="O183" s="7"/>
+      <c r="P183" s="7"/>
+      <c r="Q183" s="7"/>
+      <c r="R183" s="7"/>
+      <c r="S183" s="7"/>
+      <c r="T183" s="7"/>
+      <c r="U183" s="7"/>
+      <c r="V183" s="7"/>
+      <c r="W183" s="7"/>
+      <c r="X183" s="7"/>
+      <c r="Y183" s="7"/>
+      <c r="Z183" s="7"/>
+      <c r="AA183" s="7"/>
+      <c r="AB183" s="7"/>
+      <c r="AC183" s="7"/>
+      <c r="AD183" s="7"/>
+      <c r="AE183" s="7"/>
+      <c r="AF183" s="7"/>
+      <c r="AG183" s="7"/>
+      <c r="AH183" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_176</t>
+        </is>
+      </c>
+      <c r="B184" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼</t>
+        </is>
+      </c>
+      <c r="C184" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 강화 안내</t>
+        </is>
+      </c>
+      <c r="D184" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">조건</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t xml:space="preserve">재료 100 미만 또는 고철 300 미만이면 막이 안 뜨고, 바로가기 S4+ 점프(강화 자동 #162)에서도 안 뜨는가?</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#182 · 갇힘 방지 · 저장 장부 신설 0</t>
+        </is>
+      </c>
+      <c r="G184" s="7"/>
+      <c r="H184" s="7"/>
+      <c r="I184" s="7"/>
+      <c r="J184" s="7"/>
+      <c r="K184" s="7"/>
+      <c r="L184" s="7"/>
+      <c r="M184" s="7"/>
+      <c r="N184" s="7"/>
+      <c r="O184" s="7"/>
+      <c r="P184" s="7"/>
+      <c r="Q184" s="7"/>
+      <c r="R184" s="7"/>
+      <c r="S184" s="7"/>
+      <c r="T184" s="7"/>
+      <c r="U184" s="7"/>
+      <c r="V184" s="7"/>
+      <c r="W184" s="7"/>
+      <c r="X184" s="7"/>
+      <c r="Y184" s="7"/>
+      <c r="Z184" s="7"/>
+      <c r="AA184" s="7"/>
+      <c r="AB184" s="7"/>
+      <c r="AC184" s="7"/>
+      <c r="AD184" s="7"/>
+      <c r="AE184" s="7"/>
+      <c r="AF184" s="7"/>
+      <c r="AG184" s="7"/>
+      <c r="AH184" s="7"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_177</t>
+        </is>
+      </c>
+      <c r="B185" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼</t>
+        </is>
+      </c>
+      <c r="C185" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 강화 안내</t>
+        </is>
+      </c>
+      <c r="D185" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">보드 막</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t xml:space="preserve">조립에 들어가면 A 마운트 칸 (1,4) 만 남기고 덮이며(화면 밖이면 시야가 그 칸으로) 「마운트를 탭한 뒤 강화를 누르세요」가 보이고, 마운트 칸 탭 = 팝오버가 열리는가? (팔레트 잠김 · 모드 단추 열림)</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#182 · T1 막 재사용 · 문구 ⚠️ 가정</t>
+        </is>
+      </c>
+      <c r="G185" s="7"/>
+      <c r="H185" s="7"/>
+      <c r="I185" s="7"/>
+      <c r="J185" s="7"/>
+      <c r="K185" s="7"/>
+      <c r="L185" s="7"/>
+      <c r="M185" s="7"/>
+      <c r="N185" s="7"/>
+      <c r="O185" s="7"/>
+      <c r="P185" s="7"/>
+      <c r="Q185" s="7"/>
+      <c r="R185" s="7"/>
+      <c r="S185" s="7"/>
+      <c r="T185" s="7"/>
+      <c r="U185" s="7"/>
+      <c r="V185" s="7"/>
+      <c r="W185" s="7"/>
+      <c r="X185" s="7"/>
+      <c r="Y185" s="7"/>
+      <c r="Z185" s="7"/>
+      <c r="AA185" s="7"/>
+      <c r="AB185" s="7"/>
+      <c r="AC185" s="7"/>
+      <c r="AD185" s="7"/>
+      <c r="AE185" s="7"/>
+      <c r="AF185" s="7"/>
+      <c r="AG185" s="7"/>
+      <c r="AH185" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_178</t>
+        </is>
+      </c>
+      <c r="B186" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼</t>
+        </is>
+      </c>
+      <c r="C186" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 강화 안내</t>
+        </is>
+      </c>
+      <c r="D186" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">해제</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t xml:space="preserve">팝오버 「강화」를 누르면 막 · 안내가 걷히고 전투 화면 「도전」·「스테이지」가 다시 눌리며 그 뒤 안내가 다시 안 뜨는가?</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#182 · 끝 = 강화 표식</t>
+        </is>
+      </c>
+      <c r="G186" s="7"/>
+      <c r="H186" s="7"/>
+      <c r="I186" s="7"/>
+      <c r="J186" s="7"/>
+      <c r="K186" s="7"/>
+      <c r="L186" s="7"/>
+      <c r="M186" s="7"/>
+      <c r="N186" s="7"/>
+      <c r="O186" s="7"/>
+      <c r="P186" s="7"/>
+      <c r="Q186" s="7"/>
+      <c r="R186" s="7"/>
+      <c r="S186" s="7"/>
+      <c r="T186" s="7"/>
+      <c r="U186" s="7"/>
+      <c r="V186" s="7"/>
+      <c r="W186" s="7"/>
+      <c r="X186" s="7"/>
+      <c r="Y186" s="7"/>
+      <c r="Z186" s="7"/>
+      <c r="AA186" s="7"/>
+      <c r="AB186" s="7"/>
+      <c r="AC186" s="7"/>
+      <c r="AD186" s="7"/>
+      <c r="AE186" s="7"/>
+      <c r="AF186" s="7"/>
+      <c r="AG186" s="7"/>
+      <c r="AH186" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_179</t>
+        </is>
+      </c>
+      <c r="B187" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼</t>
+        </is>
+      </c>
+      <c r="C187" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T1</t>
+        </is>
+      </c>
+      <c r="D187" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">노드 단추 잠금</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼 전용 판(T1) 동안 팔레트 노드 단추가 전부 흐리고(기초 가공소 포함 · 고스트를 채운 뒤에도) 고스트 칸은 벨트 드래그로만 채워지는가?</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#183 · S-3 ① 닫힘</t>
+        </is>
+      </c>
+      <c r="G187" s="7"/>
+      <c r="H187" s="7"/>
+      <c r="I187" s="7"/>
+      <c r="J187" s="7"/>
+      <c r="K187" s="7"/>
+      <c r="L187" s="7"/>
+      <c r="M187" s="7"/>
+      <c r="N187" s="7"/>
+      <c r="O187" s="7"/>
+      <c r="P187" s="7"/>
+      <c r="Q187" s="7"/>
+      <c r="R187" s="7"/>
+      <c r="S187" s="7"/>
+      <c r="T187" s="7"/>
+      <c r="U187" s="7"/>
+      <c r="V187" s="7"/>
+      <c r="W187" s="7"/>
+      <c r="X187" s="7"/>
+      <c r="Y187" s="7"/>
+      <c r="Z187" s="7"/>
+      <c r="AA187" s="7"/>
+      <c r="AB187" s="7"/>
+      <c r="AC187" s="7"/>
+      <c r="AD187" s="7"/>
+      <c r="AE187" s="7"/>
+      <c r="AF187" s="7"/>
+      <c r="AG187" s="7"/>
+      <c r="AH187" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_180</t>
+        </is>
+      </c>
+      <c r="B188" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼</t>
+        </is>
+      </c>
+      <c r="C188" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">T4 지급 알림</t>
+        </is>
+      </c>
+      <c r="D188" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">문안</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S2 파밍 첫 진입 알림이 「생산량·생산속도 모듈이 열렸습니다」인가?</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#184</t>
+        </is>
+      </c>
+      <c r="G188" s="7"/>
+      <c r="H188" s="7"/>
+      <c r="I188" s="7"/>
+      <c r="J188" s="7"/>
+      <c r="K188" s="7"/>
+      <c r="L188" s="7"/>
+      <c r="M188" s="7"/>
+      <c r="N188" s="7"/>
+      <c r="O188" s="7"/>
+      <c r="P188" s="7"/>
+      <c r="Q188" s="7"/>
+      <c r="R188" s="7"/>
+      <c r="S188" s="7"/>
+      <c r="T188" s="7"/>
+      <c r="U188" s="7"/>
+      <c r="V188" s="7"/>
+      <c r="W188" s="7"/>
+      <c r="X188" s="7"/>
+      <c r="Y188" s="7"/>
+      <c r="Z188" s="7"/>
+      <c r="AA188" s="7"/>
+      <c r="AB188" s="7"/>
+      <c r="AC188" s="7"/>
+      <c r="AD188" s="7"/>
+      <c r="AE188" s="7"/>
+      <c r="AF188" s="7"/>
+      <c r="AG188" s="7"/>
+      <c r="AH188" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="26">
@@ -12337,9 +12907,9 @@
     <mergeCell ref="B92:B99"/>
     <mergeCell ref="B100:B106"/>
     <mergeCell ref="B107:B111"/>
-    <mergeCell ref="G7:AG7"/>
+    <mergeCell ref="G7:AH7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:AG182">
+  <conditionalFormatting sqref="G9:AH188">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
docs: QA AI열(38a0ccf · CID_181~183) · 촬영 가이드 8132 후보 38a0ccf · 태그 링 줄
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -190,8 +190,9 @@
     <col min="32" max="32" width="12" customWidth="1"/>
     <col min="33" max="33" width="12" customWidth="1"/>
     <col min="34" max="34" width="12" customWidth="1"/>
-    <col min="35" max="35" width="11" customWidth="1"/>
+    <col min="35" max="35" width="12" customWidth="1"/>
     <col min="36" max="36" width="11" customWidth="1"/>
+    <col min="37" max="37" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -444,6 +445,11 @@
       <c r="AH6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">video-261019c 후보(8132 · 새 사본 · 8131 동결) · #182 S4 강화 최소 안내 · #183 T1 노드 단추 전부 잠금 · #184 T4 알림 「…모듈이 열렸습니다」 ‖ 10-19 코드 세션 재확인(인앱 브라우저 · 새 저장 · 소리 0): T1 노드 단추 흐림(고스트 채운 뒤에도) → 벨트 드래그로 채움 → 마운트 가득 → S1 T3 → 도전 → 배지 「전투력 18 넘기기」 → 전멸 → S2 알림 「생산량·생산속도 모듈이 열렸습니다」 → T4 → S2 · S3 전멸 → S4 파밍 해금 막 → 해금(골드 −50) → 둘째 막(「▼ 조립」 구멍 · 「조립에서 마운트를 탭해 강화해보세요」 · 「도전」 눌러도 안 열림) → 조립 = 시야가 A 마운트로 옮겨짐 · 「마운트를 탭한 뒤 강화를 누르세요」 → 포트 칸 탭 = 팝오버(재료 100/100 · 고철 796/300) → 강화 → 「강화 ×1.45 적용」 · 고철 −300 · 탭 줄 다시 밝음 → 전투 = 막 없음 · 「도전」·「스테이지」 밝음 · 빈 칸 = 화면으로 못 만든 조건(재료·고철 부족 · 바로가기 S4) — 시험이 든다(EnhanceMountTutorialTests) · ⚠️ 보드 어둠막은 캡처에서 또렷이 구별 안 됨(T1 판도 같음) · 8132 복사 16:16:17 · CID_175~180 새 항목)</t>
+        </is>
+      </c>
+      <c r="AI6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">video-261019c 후보 갈아엎음(8132 · 16:46:47) · #185 태그 원형 링 하나 · #186 상태 띠 문제 있을 때만 ‖ 10-19 코드 세션 재확인(8123 · 캔버스 직접 캡처): 바로가기 S5 → 링 하늘색 + 「쿨다운 0.7s」(안쪽 주황 띠 없음 · 네모 없음) → Auto 끔 → 대기 마운트 차오름(하늘색 부분 링) → 만충 = 노란 링 + 「태그 스킬」 → 태그 누름 = 「쿨다운 4.3s」 · 링 하늘색 → 다시 만충 = 노랑 · 하단 띠: 문제 0 = 전투 · 조립 둘 다 띠 없음 · ⚠️ 알람 띠는 화면으로 못 세움(A · B 판 벨트 두 칸씩 끊었으나 물류 판정이 문제로 안 잡음 — 재고 남음) → CID_183 빈 칸 · 코드 경로는 종전 그대로 · CID_181~183 새 항목)</t>
         </is>
       </c>
     </row>
@@ -502,14 +508,15 @@
       <c r="AF7" s="2"/>
       <c r="AG7" s="2"/>
       <c r="AH7" s="2"/>
-      <c r="AI7" s="2" t="inlineStr">
+      <c r="AI7" s="2"/>
+      <c r="AJ7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">버전</t>
         </is>
       </c>
-      <c r="AJ7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">d70b00c</t>
+      <c r="AK7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">38a0ccf</t>
         </is>
       </c>
     </row>
@@ -674,11 +681,16 @@
       </c>
       <c r="AI8" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">38a0ccf</t>
+        </is>
+      </c>
+      <c r="AJ8" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">PASSrate</t>
         </is>
       </c>
-      <c r="AJ8" s="7">
-        <f>COUNTIF(AH9:AH188,"Pass")</f>
+      <c r="AK8" s="7">
+        <f>COUNTIF(AI9:AI191,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -776,13 +788,14 @@
       <c r="AF9" s="7"/>
       <c r="AG9" s="7"/>
       <c r="AH9" s="7"/>
-      <c r="AI9" s="2" t="inlineStr">
+      <c r="AI9" s="7"/>
+      <c r="AJ9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FAILrate</t>
         </is>
       </c>
-      <c r="AJ9" s="7">
-        <f>COUNTIF(AH9:AH188,"Fail")+COUNTIF(AH9:AH188,"Broken")</f>
+      <c r="AK9" s="7">
+        <f>COUNTIF(AI9:AI191,"Fail")+COUNTIF(AI9:AI191,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -844,13 +857,14 @@
       <c r="AF10" s="7"/>
       <c r="AG10" s="7"/>
       <c r="AH10" s="7"/>
-      <c r="AI10" s="2" t="inlineStr">
+      <c r="AI10" s="7"/>
+      <c r="AJ10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">N/A</t>
         </is>
       </c>
-      <c r="AJ10" s="7">
-        <f>COUNTIF(AH9:AH188,"N/A")</f>
+      <c r="AK10" s="7">
+        <f>COUNTIF(AI9:AI191,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -912,13 +926,14 @@
       <c r="AF11" s="7"/>
       <c r="AG11" s="7"/>
       <c r="AH11" s="7"/>
-      <c r="AI11" s="2" t="inlineStr">
+      <c r="AI11" s="7"/>
+      <c r="AJ11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">전체 개수</t>
         </is>
       </c>
-      <c r="AJ11" s="7">
-        <v>180</v>
+      <c r="AK11" s="7">
+        <v>183</v>
       </c>
     </row>
     <row r="12">
@@ -980,13 +995,14 @@
       <c r="AF12" s="7"/>
       <c r="AG12" s="7"/>
       <c r="AH12" s="7"/>
-      <c r="AI12" s="2" t="inlineStr">
+      <c r="AI12" s="7"/>
+      <c r="AJ12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">진행율</t>
         </is>
       </c>
-      <c r="AJ12" s="7">
-        <f>TEXT((COUNTA(AH9:AH188))/180,"0.00%")</f>
+      <c r="AK12" s="7">
+        <f>TEXT((COUNTA(AI9:AI191))/183,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -1052,6 +1068,7 @@
       <c r="AF13" s="7"/>
       <c r="AG13" s="7"/>
       <c r="AH13" s="7"/>
+      <c r="AI13" s="7"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -1107,6 +1124,7 @@
       <c r="AF14" s="7"/>
       <c r="AG14" s="7"/>
       <c r="AH14" s="7"/>
+      <c r="AI14" s="7"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -1198,6 +1216,7 @@
       <c r="AF15" s="7"/>
       <c r="AG15" s="7"/>
       <c r="AH15" s="7"/>
+      <c r="AI15" s="7"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -1289,6 +1308,7 @@
       <c r="AF16" s="7"/>
       <c r="AG16" s="7"/>
       <c r="AH16" s="7"/>
+      <c r="AI16" s="7"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -1385,6 +1405,7 @@
       <c r="AF17" s="7"/>
       <c r="AG17" s="7"/>
       <c r="AH17" s="7"/>
+      <c r="AI17" s="7"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -1445,6 +1466,7 @@
       <c r="AF18" s="7"/>
       <c r="AG18" s="7"/>
       <c r="AH18" s="7"/>
+      <c r="AI18" s="7"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -1500,6 +1522,7 @@
       <c r="AF19" s="7"/>
       <c r="AG19" s="7"/>
       <c r="AH19" s="7"/>
+      <c r="AI19" s="7"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1555,6 +1578,7 @@
       <c r="AF20" s="7"/>
       <c r="AG20" s="7"/>
       <c r="AH20" s="7"/>
+      <c r="AI20" s="7"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1646,6 +1670,7 @@
       <c r="AF21" s="7"/>
       <c r="AG21" s="7"/>
       <c r="AH21" s="7"/>
+      <c r="AI21" s="7"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1730,6 +1755,7 @@
       <c r="AF22" s="7"/>
       <c r="AG22" s="7"/>
       <c r="AH22" s="7"/>
+      <c r="AI22" s="7"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -1793,6 +1819,7 @@
       <c r="AF23" s="7"/>
       <c r="AG23" s="7"/>
       <c r="AH23" s="7"/>
+      <c r="AI23" s="7"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -1848,6 +1875,7 @@
       <c r="AF24" s="7"/>
       <c r="AG24" s="7"/>
       <c r="AH24" s="7"/>
+      <c r="AI24" s="7"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -1903,6 +1931,7 @@
       <c r="AF25" s="7"/>
       <c r="AG25" s="7"/>
       <c r="AH25" s="7"/>
+      <c r="AI25" s="7"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -1987,6 +2016,7 @@
       <c r="AF26" s="7"/>
       <c r="AG26" s="7"/>
       <c r="AH26" s="7"/>
+      <c r="AI26" s="7"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -2046,6 +2076,7 @@
       <c r="AF27" s="7"/>
       <c r="AG27" s="7"/>
       <c r="AH27" s="7"/>
+      <c r="AI27" s="7"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -2114,6 +2145,7 @@
       <c r="AF28" s="7"/>
       <c r="AG28" s="7"/>
       <c r="AH28" s="7"/>
+      <c r="AI28" s="7"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -2177,6 +2209,7 @@
       <c r="AF29" s="7"/>
       <c r="AG29" s="7"/>
       <c r="AH29" s="7"/>
+      <c r="AI29" s="7"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -2264,6 +2297,7 @@
       <c r="AF30" s="7"/>
       <c r="AG30" s="7"/>
       <c r="AH30" s="7"/>
+      <c r="AI30" s="7"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -2356,6 +2390,7 @@
       <c r="AF31" s="7"/>
       <c r="AG31" s="7"/>
       <c r="AH31" s="7"/>
+      <c r="AI31" s="7"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -2435,6 +2470,7 @@
       <c r="AF32" s="7"/>
       <c r="AG32" s="7"/>
       <c r="AH32" s="7"/>
+      <c r="AI32" s="7"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -2522,6 +2558,7 @@
       <c r="AF33" s="7"/>
       <c r="AG33" s="7"/>
       <c r="AH33" s="7"/>
+      <c r="AI33" s="7"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -2609,6 +2646,7 @@
       <c r="AF34" s="7"/>
       <c r="AG34" s="7"/>
       <c r="AH34" s="7"/>
+      <c r="AI34" s="7"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -2705,6 +2743,7 @@
       <c r="AF35" s="7"/>
       <c r="AG35" s="7"/>
       <c r="AH35" s="7"/>
+      <c r="AI35" s="7"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -2776,6 +2815,7 @@
       <c r="AF36" s="7"/>
       <c r="AG36" s="7"/>
       <c r="AH36" s="7"/>
+      <c r="AI36" s="7"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -2831,6 +2871,7 @@
       <c r="AF37" s="7"/>
       <c r="AG37" s="7"/>
       <c r="AH37" s="7"/>
+      <c r="AI37" s="7"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -2907,6 +2948,7 @@
       <c r="AF38" s="7"/>
       <c r="AG38" s="7"/>
       <c r="AH38" s="7"/>
+      <c r="AI38" s="7"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -2994,6 +3036,7 @@
       <c r="AF39" s="7"/>
       <c r="AG39" s="7"/>
       <c r="AH39" s="7"/>
+      <c r="AI39" s="7"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -3082,6 +3125,7 @@
       <c r="AF40" s="7"/>
       <c r="AG40" s="7"/>
       <c r="AH40" s="7"/>
+      <c r="AI40" s="7"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -3165,6 +3209,7 @@
       <c r="AF41" s="7"/>
       <c r="AG41" s="7"/>
       <c r="AH41" s="7"/>
+      <c r="AI41" s="7"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -3232,6 +3277,7 @@
       <c r="AF42" s="7"/>
       <c r="AG42" s="7"/>
       <c r="AH42" s="7"/>
+      <c r="AI42" s="7"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -3319,6 +3365,7 @@
       <c r="AF43" s="7"/>
       <c r="AG43" s="7"/>
       <c r="AH43" s="7"/>
+      <c r="AI43" s="7"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -3379,6 +3426,7 @@
       <c r="AF44" s="7"/>
       <c r="AG44" s="7"/>
       <c r="AH44" s="7"/>
+      <c r="AI44" s="7"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -3462,6 +3510,7 @@
       <c r="AF45" s="7"/>
       <c r="AG45" s="7"/>
       <c r="AH45" s="7"/>
+      <c r="AI45" s="7"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -3545,6 +3594,7 @@
       <c r="AF46" s="7"/>
       <c r="AG46" s="7"/>
       <c r="AH46" s="7"/>
+      <c r="AI46" s="7"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -3605,6 +3655,7 @@
       <c r="AF47" s="7"/>
       <c r="AG47" s="7"/>
       <c r="AH47" s="7"/>
+      <c r="AI47" s="7"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -3660,6 +3711,7 @@
       <c r="AF48" s="7"/>
       <c r="AG48" s="7"/>
       <c r="AH48" s="7"/>
+      <c r="AI48" s="7"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -3715,6 +3767,7 @@
       <c r="AF49" s="7"/>
       <c r="AG49" s="7"/>
       <c r="AH49" s="7"/>
+      <c r="AI49" s="7"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -3794,6 +3847,7 @@
       <c r="AF50" s="7"/>
       <c r="AG50" s="7"/>
       <c r="AH50" s="7"/>
+      <c r="AI50" s="7"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -3873,6 +3927,7 @@
       <c r="AF51" s="7"/>
       <c r="AG51" s="7"/>
       <c r="AH51" s="7"/>
+      <c r="AI51" s="7"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -3933,6 +3988,7 @@
       <c r="AF52" s="7"/>
       <c r="AG52" s="7"/>
       <c r="AH52" s="7"/>
+      <c r="AI52" s="7"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -3993,6 +4049,7 @@
       <c r="AF53" s="7"/>
       <c r="AG53" s="7"/>
       <c r="AH53" s="7"/>
+      <c r="AI53" s="7"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -4048,6 +4105,7 @@
       <c r="AF54" s="7"/>
       <c r="AG54" s="7"/>
       <c r="AH54" s="7"/>
+      <c r="AI54" s="7"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -4139,6 +4197,7 @@
       <c r="AF55" s="7"/>
       <c r="AG55" s="7"/>
       <c r="AH55" s="7"/>
+      <c r="AI55" s="7"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -4210,6 +4269,7 @@
       <c r="AF56" s="7"/>
       <c r="AG56" s="7"/>
       <c r="AH56" s="7"/>
+      <c r="AI56" s="7"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -4290,6 +4350,7 @@
       <c r="AF57" s="7"/>
       <c r="AG57" s="7"/>
       <c r="AH57" s="7"/>
+      <c r="AI57" s="7"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -4378,6 +4439,7 @@
       <c r="AF58" s="7"/>
       <c r="AG58" s="7"/>
       <c r="AH58" s="7"/>
+      <c r="AI58" s="7"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -4433,6 +4495,7 @@
       <c r="AF59" s="7"/>
       <c r="AG59" s="7"/>
       <c r="AH59" s="7"/>
+      <c r="AI59" s="7"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -4488,6 +4551,7 @@
       <c r="AF60" s="7"/>
       <c r="AG60" s="7"/>
       <c r="AH60" s="7"/>
+      <c r="AI60" s="7"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -4555,6 +4619,7 @@
       <c r="AF61" s="7"/>
       <c r="AG61" s="7"/>
       <c r="AH61" s="7"/>
+      <c r="AI61" s="7"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -4630,6 +4695,7 @@
       <c r="AF62" s="7"/>
       <c r="AG62" s="7"/>
       <c r="AH62" s="7"/>
+      <c r="AI62" s="7"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -4697,6 +4763,7 @@
       <c r="AF63" s="7"/>
       <c r="AG63" s="7"/>
       <c r="AH63" s="7"/>
+      <c r="AI63" s="7"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -4752,6 +4819,7 @@
       <c r="AF64" s="7"/>
       <c r="AG64" s="7"/>
       <c r="AH64" s="7"/>
+      <c r="AI64" s="7"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -4812,6 +4880,7 @@
       <c r="AF65" s="7"/>
       <c r="AG65" s="7"/>
       <c r="AH65" s="7"/>
+      <c r="AI65" s="7"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
@@ -4879,6 +4948,7 @@
       <c r="AF66" s="7"/>
       <c r="AG66" s="7"/>
       <c r="AH66" s="7"/>
+      <c r="AI66" s="7"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -4934,6 +5004,7 @@
       <c r="AF67" s="7"/>
       <c r="AG67" s="7"/>
       <c r="AH67" s="7"/>
+      <c r="AI67" s="7"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
@@ -4993,6 +5064,7 @@
       <c r="AF68" s="7"/>
       <c r="AG68" s="7"/>
       <c r="AH68" s="7"/>
+      <c r="AI68" s="7"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -5084,6 +5156,7 @@
       <c r="AF69" s="7"/>
       <c r="AG69" s="7"/>
       <c r="AH69" s="7"/>
+      <c r="AI69" s="7"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
@@ -5139,6 +5212,7 @@
       <c r="AF70" s="7"/>
       <c r="AG70" s="7"/>
       <c r="AH70" s="7"/>
+      <c r="AI70" s="7"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -5199,6 +5273,7 @@
       <c r="AF71" s="7"/>
       <c r="AG71" s="7"/>
       <c r="AH71" s="7"/>
+      <c r="AI71" s="7"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
@@ -5270,6 +5345,7 @@
       <c r="AF72" s="7"/>
       <c r="AG72" s="7"/>
       <c r="AH72" s="7"/>
+      <c r="AI72" s="7"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
@@ -5330,6 +5406,7 @@
       <c r="AF73" s="7"/>
       <c r="AG73" s="7"/>
       <c r="AH73" s="7"/>
+      <c r="AI73" s="7"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -5385,6 +5462,7 @@
       <c r="AF74" s="7"/>
       <c r="AG74" s="7"/>
       <c r="AH74" s="7"/>
+      <c r="AI74" s="7"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -5440,6 +5518,7 @@
       <c r="AF75" s="7"/>
       <c r="AG75" s="7"/>
       <c r="AH75" s="7"/>
+      <c r="AI75" s="7"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -5495,6 +5574,7 @@
       <c r="AF76" s="7"/>
       <c r="AG76" s="7"/>
       <c r="AH76" s="7"/>
+      <c r="AI76" s="7"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -5554,6 +5634,7 @@
       <c r="AF77" s="7"/>
       <c r="AG77" s="7"/>
       <c r="AH77" s="7"/>
+      <c r="AI77" s="7"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
@@ -5609,6 +5690,7 @@
       <c r="AF78" s="7"/>
       <c r="AG78" s="7"/>
       <c r="AH78" s="7"/>
+      <c r="AI78" s="7"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -5669,6 +5751,7 @@
       <c r="AF79" s="7"/>
       <c r="AG79" s="7"/>
       <c r="AH79" s="7"/>
+      <c r="AI79" s="7"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
@@ -5740,6 +5823,7 @@
       <c r="AF80" s="7"/>
       <c r="AG80" s="7"/>
       <c r="AH80" s="7"/>
+      <c r="AI80" s="7"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
@@ -5799,6 +5883,7 @@
       <c r="AF81" s="7"/>
       <c r="AG81" s="7"/>
       <c r="AH81" s="7"/>
+      <c r="AI81" s="7"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
@@ -5854,6 +5939,7 @@
       <c r="AF82" s="7"/>
       <c r="AG82" s="7"/>
       <c r="AH82" s="7"/>
+      <c r="AI82" s="7"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
@@ -5914,6 +6000,7 @@
       <c r="AF83" s="7"/>
       <c r="AG83" s="7"/>
       <c r="AH83" s="7"/>
+      <c r="AI83" s="7"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
@@ -5969,6 +6056,7 @@
       <c r="AF84" s="7"/>
       <c r="AG84" s="7"/>
       <c r="AH84" s="7"/>
+      <c r="AI84" s="7"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
@@ -6024,6 +6112,7 @@
       <c r="AF85" s="7"/>
       <c r="AG85" s="7"/>
       <c r="AH85" s="7"/>
+      <c r="AI85" s="7"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
@@ -6084,6 +6173,7 @@
       <c r="AF86" s="7"/>
       <c r="AG86" s="7"/>
       <c r="AH86" s="7"/>
+      <c r="AI86" s="7"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
@@ -6139,6 +6229,7 @@
       <c r="AF87" s="7"/>
       <c r="AG87" s="7"/>
       <c r="AH87" s="7"/>
+      <c r="AI87" s="7"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
@@ -6194,6 +6285,7 @@
       <c r="AF88" s="7"/>
       <c r="AG88" s="7"/>
       <c r="AH88" s="7"/>
+      <c r="AI88" s="7"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
@@ -6249,6 +6341,7 @@
       <c r="AF89" s="7"/>
       <c r="AG89" s="7"/>
       <c r="AH89" s="7"/>
+      <c r="AI89" s="7"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
@@ -6333,6 +6426,7 @@
       <c r="AF90" s="7"/>
       <c r="AG90" s="7"/>
       <c r="AH90" s="7"/>
+      <c r="AI90" s="7"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
@@ -6388,6 +6482,7 @@
       <c r="AF91" s="7"/>
       <c r="AG91" s="7"/>
       <c r="AH91" s="7"/>
+      <c r="AI91" s="7"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
@@ -6479,6 +6574,7 @@
       <c r="AF92" s="7"/>
       <c r="AG92" s="7"/>
       <c r="AH92" s="7"/>
+      <c r="AI92" s="7"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
@@ -6575,6 +6671,7 @@
       <c r="AF93" s="7"/>
       <c r="AG93" s="7"/>
       <c r="AH93" s="7"/>
+      <c r="AI93" s="7"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
@@ -6635,6 +6732,7 @@
       <c r="AF94" s="7"/>
       <c r="AG94" s="7"/>
       <c r="AH94" s="7"/>
+      <c r="AI94" s="7"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
@@ -6695,6 +6793,7 @@
       <c r="AF95" s="7"/>
       <c r="AG95" s="7"/>
       <c r="AH95" s="7"/>
+      <c r="AI95" s="7"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
@@ -6774,6 +6873,7 @@
       <c r="AF96" s="7"/>
       <c r="AG96" s="7"/>
       <c r="AH96" s="7"/>
+      <c r="AI96" s="7"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="inlineStr">
@@ -6829,6 +6929,7 @@
       <c r="AF97" s="7"/>
       <c r="AG97" s="7"/>
       <c r="AH97" s="7"/>
+      <c r="AI97" s="7"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
@@ -6884,6 +6985,7 @@
       <c r="AF98" s="7"/>
       <c r="AG98" s="7"/>
       <c r="AH98" s="7"/>
+      <c r="AI98" s="7"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
@@ -6939,6 +7041,7 @@
       <c r="AF99" s="7"/>
       <c r="AG99" s="7"/>
       <c r="AH99" s="7"/>
+      <c r="AI99" s="7"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
@@ -7003,6 +7106,7 @@
       <c r="AF100" s="7"/>
       <c r="AG100" s="7"/>
       <c r="AH100" s="7"/>
+      <c r="AI100" s="7"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
@@ -7058,6 +7162,7 @@
       <c r="AF101" s="7"/>
       <c r="AG101" s="7"/>
       <c r="AH101" s="7"/>
+      <c r="AI101" s="7"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
@@ -7113,6 +7218,7 @@
       <c r="AF102" s="7"/>
       <c r="AG102" s="7"/>
       <c r="AH102" s="7"/>
+      <c r="AI102" s="7"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="inlineStr">
@@ -7168,6 +7274,7 @@
       <c r="AF103" s="7"/>
       <c r="AG103" s="7"/>
       <c r="AH103" s="7"/>
+      <c r="AI103" s="7"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="inlineStr">
@@ -7228,6 +7335,7 @@
       <c r="AF104" s="7"/>
       <c r="AG104" s="7"/>
       <c r="AH104" s="7"/>
+      <c r="AI104" s="7"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
@@ -7283,6 +7391,7 @@
       <c r="AF105" s="7"/>
       <c r="AG105" s="7"/>
       <c r="AH105" s="7"/>
+      <c r="AI105" s="7"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
@@ -7338,6 +7447,7 @@
       <c r="AF106" s="7"/>
       <c r="AG106" s="7"/>
       <c r="AH106" s="7"/>
+      <c r="AI106" s="7"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
@@ -7393,6 +7503,7 @@
       <c r="AF107" s="7"/>
       <c r="AG107" s="7"/>
       <c r="AH107" s="7"/>
+      <c r="AI107" s="7"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
@@ -7452,6 +7563,7 @@
       <c r="AF108" s="7"/>
       <c r="AG108" s="7"/>
       <c r="AH108" s="7"/>
+      <c r="AI108" s="7"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="inlineStr">
@@ -7516,6 +7628,7 @@
       <c r="AF109" s="7"/>
       <c r="AG109" s="7"/>
       <c r="AH109" s="7"/>
+      <c r="AI109" s="7"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
@@ -7588,6 +7701,7 @@
       <c r="AF110" s="7"/>
       <c r="AG110" s="7"/>
       <c r="AH110" s="7"/>
+      <c r="AI110" s="7"/>
     </row>
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
@@ -7663,6 +7777,7 @@
       <c r="AF111" s="7"/>
       <c r="AG111" s="7"/>
       <c r="AH111" s="7"/>
+      <c r="AI111" s="7"/>
     </row>
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
@@ -7735,6 +7850,7 @@
       <c r="AF112" s="7"/>
       <c r="AG112" s="7"/>
       <c r="AH112" s="7"/>
+      <c r="AI112" s="7"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
@@ -7799,6 +7915,7 @@
       <c r="AF113" s="7"/>
       <c r="AG113" s="7"/>
       <c r="AH113" s="7"/>
+      <c r="AI113" s="7"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="inlineStr">
@@ -7879,6 +7996,7 @@
       <c r="AF114" s="7"/>
       <c r="AG114" s="7"/>
       <c r="AH114" s="7"/>
+      <c r="AI114" s="7"/>
     </row>
     <row r="115">
       <c r="A115" s="7" t="inlineStr">
@@ -7951,6 +8069,7 @@
       <c r="AF115" s="7"/>
       <c r="AG115" s="7"/>
       <c r="AH115" s="7"/>
+      <c r="AI115" s="7"/>
     </row>
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
@@ -8031,6 +8150,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AI116" s="7"/>
     </row>
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
@@ -8107,6 +8227,7 @@
       <c r="AF117" s="7"/>
       <c r="AG117" s="7"/>
       <c r="AH117" s="7"/>
+      <c r="AI117" s="7"/>
     </row>
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
@@ -8183,6 +8304,7 @@
       <c r="AF118" s="7"/>
       <c r="AG118" s="7"/>
       <c r="AH118" s="7"/>
+      <c r="AI118" s="7"/>
     </row>
     <row r="119">
       <c r="A119" s="7" t="inlineStr">
@@ -8255,6 +8377,7 @@
       <c r="AF119" s="7"/>
       <c r="AG119" s="7"/>
       <c r="AH119" s="7"/>
+      <c r="AI119" s="7"/>
     </row>
     <row r="120">
       <c r="A120" s="7" t="inlineStr">
@@ -8319,6 +8442,7 @@
       <c r="AF120" s="7"/>
       <c r="AG120" s="7"/>
       <c r="AH120" s="7"/>
+      <c r="AI120" s="7"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="inlineStr">
@@ -8395,6 +8519,7 @@
       <c r="AF121" s="7"/>
       <c r="AG121" s="7"/>
       <c r="AH121" s="7"/>
+      <c r="AI121" s="7"/>
     </row>
     <row r="122">
       <c r="A122" s="7" t="inlineStr">
@@ -8471,6 +8596,7 @@
       <c r="AF122" s="7"/>
       <c r="AG122" s="7"/>
       <c r="AH122" s="7"/>
+      <c r="AI122" s="7"/>
     </row>
     <row r="123">
       <c r="A123" s="7" t="inlineStr">
@@ -8535,6 +8661,7 @@
       <c r="AF123" s="7"/>
       <c r="AG123" s="7"/>
       <c r="AH123" s="7"/>
+      <c r="AI123" s="7"/>
     </row>
     <row r="124">
       <c r="A124" s="7" t="inlineStr">
@@ -8607,6 +8734,7 @@
       <c r="AF124" s="7"/>
       <c r="AG124" s="7"/>
       <c r="AH124" s="7"/>
+      <c r="AI124" s="7"/>
     </row>
     <row r="125">
       <c r="A125" s="7" t="inlineStr">
@@ -8671,6 +8799,7 @@
       <c r="AF125" s="7"/>
       <c r="AG125" s="7"/>
       <c r="AH125" s="7"/>
+      <c r="AI125" s="7"/>
     </row>
     <row r="126">
       <c r="A126" s="7" t="inlineStr">
@@ -8735,6 +8864,7 @@
       <c r="AF126" s="7"/>
       <c r="AG126" s="7"/>
       <c r="AH126" s="7"/>
+      <c r="AI126" s="7"/>
     </row>
     <row r="127">
       <c r="A127" s="7" t="inlineStr">
@@ -8803,6 +8933,7 @@
       <c r="AF127" s="7"/>
       <c r="AG127" s="7"/>
       <c r="AH127" s="7"/>
+      <c r="AI127" s="7"/>
     </row>
     <row r="128">
       <c r="A128" s="7" t="inlineStr">
@@ -8871,6 +9002,7 @@
       <c r="AF128" s="7"/>
       <c r="AG128" s="7"/>
       <c r="AH128" s="7"/>
+      <c r="AI128" s="7"/>
     </row>
     <row r="129">
       <c r="A129" s="7" t="inlineStr">
@@ -8939,6 +9071,7 @@
       <c r="AF129" s="7"/>
       <c r="AG129" s="7"/>
       <c r="AH129" s="7"/>
+      <c r="AI129" s="7"/>
     </row>
     <row r="130">
       <c r="A130" s="7" t="inlineStr">
@@ -9003,6 +9136,7 @@
       <c r="AF130" s="7"/>
       <c r="AG130" s="7"/>
       <c r="AH130" s="7"/>
+      <c r="AI130" s="7"/>
     </row>
     <row r="131">
       <c r="A131" s="7" t="inlineStr">
@@ -9075,6 +9209,7 @@
       <c r="AF131" s="7"/>
       <c r="AG131" s="7"/>
       <c r="AH131" s="7"/>
+      <c r="AI131" s="7"/>
     </row>
     <row r="132">
       <c r="A132" s="7" t="inlineStr">
@@ -9151,6 +9286,7 @@
       <c r="AF132" s="7"/>
       <c r="AG132" s="7"/>
       <c r="AH132" s="7"/>
+      <c r="AI132" s="7"/>
     </row>
     <row r="133">
       <c r="A133" s="7" t="inlineStr">
@@ -9227,6 +9363,7 @@
       <c r="AF133" s="7"/>
       <c r="AG133" s="7"/>
       <c r="AH133" s="7"/>
+      <c r="AI133" s="7"/>
     </row>
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
@@ -9299,6 +9436,7 @@
       <c r="AF134" s="7"/>
       <c r="AG134" s="7"/>
       <c r="AH134" s="7"/>
+      <c r="AI134" s="7"/>
     </row>
     <row r="135">
       <c r="A135" s="7" t="inlineStr">
@@ -9371,6 +9509,7 @@
       <c r="AF135" s="7"/>
       <c r="AG135" s="7"/>
       <c r="AH135" s="7"/>
+      <c r="AI135" s="7"/>
     </row>
     <row r="136">
       <c r="A136" s="7" t="inlineStr">
@@ -9443,6 +9582,7 @@
       <c r="AF136" s="7"/>
       <c r="AG136" s="7"/>
       <c r="AH136" s="7"/>
+      <c r="AI136" s="7"/>
     </row>
     <row r="137">
       <c r="A137" s="7" t="inlineStr">
@@ -9511,6 +9651,7 @@
       <c r="AF137" s="7"/>
       <c r="AG137" s="7"/>
       <c r="AH137" s="7"/>
+      <c r="AI137" s="7"/>
     </row>
     <row r="138">
       <c r="A138" s="7" t="inlineStr">
@@ -9579,6 +9720,7 @@
       <c r="AF138" s="7"/>
       <c r="AG138" s="7"/>
       <c r="AH138" s="7"/>
+      <c r="AI138" s="7"/>
     </row>
     <row r="139">
       <c r="A139" s="7" t="inlineStr">
@@ -9647,6 +9789,7 @@
       <c r="AF139" s="7"/>
       <c r="AG139" s="7"/>
       <c r="AH139" s="7"/>
+      <c r="AI139" s="7"/>
     </row>
     <row r="140">
       <c r="A140" s="7" t="inlineStr">
@@ -9711,6 +9854,7 @@
       <c r="AF140" s="7"/>
       <c r="AG140" s="7"/>
       <c r="AH140" s="7"/>
+      <c r="AI140" s="7"/>
     </row>
     <row r="141">
       <c r="A141" s="7" t="inlineStr">
@@ -9787,6 +9931,7 @@
       <c r="AF141" s="7"/>
       <c r="AG141" s="7"/>
       <c r="AH141" s="7"/>
+      <c r="AI141" s="7"/>
     </row>
     <row r="142">
       <c r="A142" s="7" t="inlineStr">
@@ -9851,6 +9996,7 @@
       <c r="AF142" s="7"/>
       <c r="AG142" s="7"/>
       <c r="AH142" s="7"/>
+      <c r="AI142" s="7"/>
     </row>
     <row r="143">
       <c r="A143" s="7" t="inlineStr">
@@ -9915,6 +10061,7 @@
       <c r="AF143" s="7"/>
       <c r="AG143" s="7"/>
       <c r="AH143" s="7"/>
+      <c r="AI143" s="7"/>
     </row>
     <row r="144">
       <c r="A144" s="7" t="inlineStr">
@@ -9979,6 +10126,7 @@
       <c r="AF144" s="7"/>
       <c r="AG144" s="7"/>
       <c r="AH144" s="7"/>
+      <c r="AI144" s="7"/>
     </row>
     <row r="145">
       <c r="A145" s="7" t="inlineStr">
@@ -10059,6 +10207,7 @@
       <c r="AF145" s="7"/>
       <c r="AG145" s="7"/>
       <c r="AH145" s="7"/>
+      <c r="AI145" s="7"/>
     </row>
     <row r="146">
       <c r="A146" s="7" t="inlineStr">
@@ -10127,6 +10276,7 @@
       <c r="AF146" s="7"/>
       <c r="AG146" s="7"/>
       <c r="AH146" s="7"/>
+      <c r="AI146" s="7"/>
     </row>
     <row r="147">
       <c r="A147" s="7" t="inlineStr">
@@ -10207,6 +10357,7 @@
       <c r="AF147" s="7"/>
       <c r="AG147" s="7"/>
       <c r="AH147" s="7"/>
+      <c r="AI147" s="7"/>
     </row>
     <row r="148">
       <c r="A148" s="7" t="inlineStr">
@@ -10271,6 +10422,7 @@
       <c r="AF148" s="7"/>
       <c r="AG148" s="7"/>
       <c r="AH148" s="7"/>
+      <c r="AI148" s="7"/>
     </row>
     <row r="149">
       <c r="A149" s="7" t="inlineStr">
@@ -10343,6 +10495,7 @@
       <c r="AF149" s="7"/>
       <c r="AG149" s="7"/>
       <c r="AH149" s="7"/>
+      <c r="AI149" s="7"/>
     </row>
     <row r="150">
       <c r="A150" s="7" t="inlineStr">
@@ -10419,6 +10572,7 @@
       <c r="AF150" s="7"/>
       <c r="AG150" s="7"/>
       <c r="AH150" s="7"/>
+      <c r="AI150" s="7"/>
     </row>
     <row r="151">
       <c r="A151" s="7" t="inlineStr">
@@ -10487,6 +10641,7 @@
       <c r="AF151" s="7"/>
       <c r="AG151" s="7"/>
       <c r="AH151" s="7"/>
+      <c r="AI151" s="7"/>
     </row>
     <row r="152">
       <c r="A152" s="7" t="inlineStr">
@@ -10559,6 +10714,7 @@
       <c r="AF152" s="7"/>
       <c r="AG152" s="7"/>
       <c r="AH152" s="7"/>
+      <c r="AI152" s="7"/>
     </row>
     <row r="153">
       <c r="A153" s="7" t="inlineStr">
@@ -10631,6 +10787,7 @@
       <c r="AF153" s="7"/>
       <c r="AG153" s="7"/>
       <c r="AH153" s="7"/>
+      <c r="AI153" s="7"/>
     </row>
     <row r="154">
       <c r="A154" s="7" t="inlineStr">
@@ -10691,6 +10848,7 @@
       <c r="AF154" s="7"/>
       <c r="AG154" s="7"/>
       <c r="AH154" s="7"/>
+      <c r="AI154" s="7"/>
     </row>
     <row r="155">
       <c r="A155" s="7" t="inlineStr">
@@ -10755,6 +10913,7 @@
       <c r="AF155" s="7"/>
       <c r="AG155" s="7"/>
       <c r="AH155" s="7"/>
+      <c r="AI155" s="7"/>
     </row>
     <row r="156">
       <c r="A156" s="7" t="inlineStr">
@@ -10823,6 +10982,7 @@
       <c r="AF156" s="7"/>
       <c r="AG156" s="7"/>
       <c r="AH156" s="7"/>
+      <c r="AI156" s="7"/>
     </row>
     <row r="157">
       <c r="A157" s="7" t="inlineStr">
@@ -10887,6 +11047,7 @@
       <c r="AF157" s="7"/>
       <c r="AG157" s="7"/>
       <c r="AH157" s="7"/>
+      <c r="AI157" s="7"/>
     </row>
     <row r="158">
       <c r="A158" s="7" t="inlineStr">
@@ -10951,6 +11112,7 @@
       <c r="AF158" s="7"/>
       <c r="AG158" s="7"/>
       <c r="AH158" s="7"/>
+      <c r="AI158" s="7"/>
     </row>
     <row r="159">
       <c r="A159" s="7" t="inlineStr">
@@ -11015,6 +11177,7 @@
       <c r="AF159" s="7"/>
       <c r="AG159" s="7"/>
       <c r="AH159" s="7"/>
+      <c r="AI159" s="7"/>
     </row>
     <row r="160">
       <c r="A160" s="7" t="inlineStr">
@@ -11079,6 +11242,7 @@
       <c r="AF160" s="7"/>
       <c r="AG160" s="7"/>
       <c r="AH160" s="7"/>
+      <c r="AI160" s="7"/>
     </row>
     <row r="161">
       <c r="A161" s="7" t="inlineStr">
@@ -11147,6 +11311,7 @@
       </c>
       <c r="AG161" s="7"/>
       <c r="AH161" s="7"/>
+      <c r="AI161" s="7"/>
     </row>
     <row r="162">
       <c r="A162" s="7" t="inlineStr">
@@ -11211,6 +11376,7 @@
       <c r="AF162" s="7"/>
       <c r="AG162" s="7"/>
       <c r="AH162" s="7"/>
+      <c r="AI162" s="7"/>
     </row>
     <row r="163">
       <c r="A163" s="7" t="inlineStr">
@@ -11275,6 +11441,7 @@
       <c r="AF163" s="7"/>
       <c r="AG163" s="7"/>
       <c r="AH163" s="7"/>
+      <c r="AI163" s="7"/>
     </row>
     <row r="164">
       <c r="A164" s="7" t="inlineStr">
@@ -11339,6 +11506,7 @@
       <c r="AF164" s="7"/>
       <c r="AG164" s="7"/>
       <c r="AH164" s="7"/>
+      <c r="AI164" s="7"/>
     </row>
     <row r="165">
       <c r="A165" s="7" t="inlineStr">
@@ -11403,6 +11571,7 @@
       <c r="AF165" s="7"/>
       <c r="AG165" s="7"/>
       <c r="AH165" s="7"/>
+      <c r="AI165" s="7"/>
     </row>
     <row r="166">
       <c r="A166" s="7" t="inlineStr">
@@ -11471,6 +11640,7 @@
       <c r="AF166" s="7"/>
       <c r="AG166" s="7"/>
       <c r="AH166" s="7"/>
+      <c r="AI166" s="7"/>
     </row>
     <row r="167">
       <c r="A167" s="7" t="inlineStr">
@@ -11535,6 +11705,7 @@
       <c r="AF167" s="7"/>
       <c r="AG167" s="7"/>
       <c r="AH167" s="7"/>
+      <c r="AI167" s="7"/>
     </row>
     <row r="168">
       <c r="A168" s="7" t="inlineStr">
@@ -11599,6 +11770,7 @@
       <c r="AF168" s="7"/>
       <c r="AG168" s="7"/>
       <c r="AH168" s="7"/>
+      <c r="AI168" s="7"/>
     </row>
     <row r="169">
       <c r="A169" s="7" t="inlineStr">
@@ -11663,6 +11835,7 @@
       <c r="AF169" s="7"/>
       <c r="AG169" s="7"/>
       <c r="AH169" s="7"/>
+      <c r="AI169" s="7"/>
     </row>
     <row r="170">
       <c r="A170" s="7" t="inlineStr">
@@ -11731,6 +11904,7 @@
       <c r="AF170" s="7"/>
       <c r="AG170" s="7"/>
       <c r="AH170" s="7"/>
+      <c r="AI170" s="7"/>
     </row>
     <row r="171">
       <c r="A171" s="7" t="inlineStr">
@@ -11791,6 +11965,7 @@
       <c r="AF171" s="7"/>
       <c r="AG171" s="7"/>
       <c r="AH171" s="7"/>
+      <c r="AI171" s="7"/>
     </row>
     <row r="172">
       <c r="A172" s="7" t="inlineStr">
@@ -11851,6 +12026,7 @@
       <c r="AF172" s="7"/>
       <c r="AG172" s="7"/>
       <c r="AH172" s="7"/>
+      <c r="AI172" s="7"/>
     </row>
     <row r="173">
       <c r="A173" s="7" t="inlineStr">
@@ -11919,6 +12095,7 @@
       <c r="AF173" s="7"/>
       <c r="AG173" s="7"/>
       <c r="AH173" s="7"/>
+      <c r="AI173" s="7"/>
     </row>
     <row r="174">
       <c r="A174" s="7" t="inlineStr">
@@ -11983,6 +12160,7 @@
       <c r="AF174" s="7"/>
       <c r="AG174" s="7"/>
       <c r="AH174" s="7"/>
+      <c r="AI174" s="7"/>
     </row>
     <row r="175">
       <c r="A175" s="7" t="inlineStr">
@@ -12051,6 +12229,7 @@
       </c>
       <c r="AG175" s="7"/>
       <c r="AH175" s="7"/>
+      <c r="AI175" s="7"/>
     </row>
     <row r="176">
       <c r="A176" s="7" t="inlineStr">
@@ -12115,6 +12294,7 @@
       <c r="AF176" s="7"/>
       <c r="AG176" s="7"/>
       <c r="AH176" s="7"/>
+      <c r="AI176" s="7"/>
     </row>
     <row r="177">
       <c r="A177" s="7" t="inlineStr">
@@ -12179,6 +12359,7 @@
       </c>
       <c r="AG177" s="7"/>
       <c r="AH177" s="7"/>
+      <c r="AI177" s="7"/>
     </row>
     <row r="178">
       <c r="A178" s="7" t="inlineStr">
@@ -12243,6 +12424,7 @@
       <c r="AF178" s="7"/>
       <c r="AG178" s="7"/>
       <c r="AH178" s="7"/>
+      <c r="AI178" s="7"/>
     </row>
     <row r="179">
       <c r="A179" s="7" t="inlineStr">
@@ -12307,6 +12489,7 @@
       </c>
       <c r="AG179" s="7"/>
       <c r="AH179" s="7"/>
+      <c r="AI179" s="7"/>
     </row>
     <row r="180">
       <c r="A180" s="7" t="inlineStr">
@@ -12371,6 +12554,7 @@
       </c>
       <c r="AG180" s="7"/>
       <c r="AH180" s="7"/>
+      <c r="AI180" s="7"/>
     </row>
     <row r="181">
       <c r="A181" s="7" t="inlineStr">
@@ -12435,6 +12619,7 @@
         </is>
       </c>
       <c r="AH181" s="7"/>
+      <c r="AI181" s="7"/>
     </row>
     <row r="182">
       <c r="A182" s="7" t="inlineStr">
@@ -12499,6 +12684,7 @@
         </is>
       </c>
       <c r="AH182" s="7"/>
+      <c r="AI182" s="7"/>
     </row>
     <row r="183">
       <c r="A183" s="7" t="inlineStr">
@@ -12563,6 +12749,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AI183" s="7"/>
     </row>
     <row r="184">
       <c r="A184" s="7" t="inlineStr">
@@ -12623,6 +12810,7 @@
       <c r="AF184" s="7"/>
       <c r="AG184" s="7"/>
       <c r="AH184" s="7"/>
+      <c r="AI184" s="7"/>
     </row>
     <row r="185">
       <c r="A185" s="7" t="inlineStr">
@@ -12687,6 +12875,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AI185" s="7"/>
     </row>
     <row r="186">
       <c r="A186" s="7" t="inlineStr">
@@ -12751,6 +12940,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AI186" s="7"/>
     </row>
     <row r="187">
       <c r="A187" s="7" t="inlineStr">
@@ -12815,6 +13005,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AI187" s="7"/>
     </row>
     <row r="188">
       <c r="A188" s="7" t="inlineStr">
@@ -12879,6 +13070,198 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AI188" s="7"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_181</t>
+        </is>
+      </c>
+      <c r="B189" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C189" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">태그 원형</t>
+        </is>
+      </c>
+      <c r="D189" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">링 하나 · 색</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t xml:space="preserve">태그 원형에 링이 하나(적재)만 있고, 대기 마운트 만충 + 스킬 조건이 참이면 노랑 · 그 밖(채우는 중 · 쿨다운)은 하늘색이며 쿨다운은 글자 「쿨다운 n.ns」로만 보이는가? (노란 네모 · 안쪽 주황 띠 없음)</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#185 · 노랑 = TagSkillRingColor 재사용 ⚠️ 가정</t>
+        </is>
+      </c>
+      <c r="G189" s="7"/>
+      <c r="H189" s="7"/>
+      <c r="I189" s="7"/>
+      <c r="J189" s="7"/>
+      <c r="K189" s="7"/>
+      <c r="L189" s="7"/>
+      <c r="M189" s="7"/>
+      <c r="N189" s="7"/>
+      <c r="O189" s="7"/>
+      <c r="P189" s="7"/>
+      <c r="Q189" s="7"/>
+      <c r="R189" s="7"/>
+      <c r="S189" s="7"/>
+      <c r="T189" s="7"/>
+      <c r="U189" s="7"/>
+      <c r="V189" s="7"/>
+      <c r="W189" s="7"/>
+      <c r="X189" s="7"/>
+      <c r="Y189" s="7"/>
+      <c r="Z189" s="7"/>
+      <c r="AA189" s="7"/>
+      <c r="AB189" s="7"/>
+      <c r="AC189" s="7"/>
+      <c r="AD189" s="7"/>
+      <c r="AE189" s="7"/>
+      <c r="AF189" s="7"/>
+      <c r="AG189" s="7"/>
+      <c r="AH189" s="7"/>
+      <c r="AI189" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_182</t>
+        </is>
+      </c>
+      <c r="B190" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C190" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">하단 상태 띠</t>
+        </is>
+      </c>
+      <c r="D190" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">문제 없음 = 안 띄움</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t xml:space="preserve">물류 문제가 없을 때 전투 · 조립 화면 하단에 상태 띠(「문제 없음」 줄)가 아예 안 뜨는가? (자리 재배치 없음)</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#186</t>
+        </is>
+      </c>
+      <c r="G190" s="7"/>
+      <c r="H190" s="7"/>
+      <c r="I190" s="7"/>
+      <c r="J190" s="7"/>
+      <c r="K190" s="7"/>
+      <c r="L190" s="7"/>
+      <c r="M190" s="7"/>
+      <c r="N190" s="7"/>
+      <c r="O190" s="7"/>
+      <c r="P190" s="7"/>
+      <c r="Q190" s="7"/>
+      <c r="R190" s="7"/>
+      <c r="S190" s="7"/>
+      <c r="T190" s="7"/>
+      <c r="U190" s="7"/>
+      <c r="V190" s="7"/>
+      <c r="W190" s="7"/>
+      <c r="X190" s="7"/>
+      <c r="Y190" s="7"/>
+      <c r="Z190" s="7"/>
+      <c r="AA190" s="7"/>
+      <c r="AB190" s="7"/>
+      <c r="AC190" s="7"/>
+      <c r="AD190" s="7"/>
+      <c r="AE190" s="7"/>
+      <c r="AF190" s="7"/>
+      <c r="AG190" s="7"/>
+      <c r="AH190" s="7"/>
+      <c r="AI190" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_183</t>
+        </is>
+      </c>
+      <c r="B191" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C191" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">하단 상태 띠</t>
+        </is>
+      </c>
+      <c r="D191" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">문제 있을 때</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미연결 · 생산 정지 · 전력 부족 · 마운트 빔 · 고철 부족 중 하나라도 있으면 종전처럼 빨간 점멸 띠 + 문구가 뜨고, 풀리면 사라지는가?</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#186</t>
+        </is>
+      </c>
+      <c r="G191" s="7"/>
+      <c r="H191" s="7"/>
+      <c r="I191" s="7"/>
+      <c r="J191" s="7"/>
+      <c r="K191" s="7"/>
+      <c r="L191" s="7"/>
+      <c r="M191" s="7"/>
+      <c r="N191" s="7"/>
+      <c r="O191" s="7"/>
+      <c r="P191" s="7"/>
+      <c r="Q191" s="7"/>
+      <c r="R191" s="7"/>
+      <c r="S191" s="7"/>
+      <c r="T191" s="7"/>
+      <c r="U191" s="7"/>
+      <c r="V191" s="7"/>
+      <c r="W191" s="7"/>
+      <c r="X191" s="7"/>
+      <c r="Y191" s="7"/>
+      <c r="Z191" s="7"/>
+      <c r="AA191" s="7"/>
+      <c r="AB191" s="7"/>
+      <c r="AC191" s="7"/>
+      <c r="AD191" s="7"/>
+      <c r="AE191" s="7"/>
+      <c r="AF191" s="7"/>
+      <c r="AG191" s="7"/>
+      <c r="AH191" s="7"/>
+      <c r="AI191" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="26">
@@ -12907,9 +13290,9 @@
     <mergeCell ref="B92:B99"/>
     <mergeCell ref="B100:B106"/>
     <mergeCell ref="B107:B111"/>
-    <mergeCell ref="G7:AH7"/>
+    <mergeCell ref="G7:AI7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:AH188">
+  <conditionalFormatting sqref="G9:AI191">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
docs: QA AJ열(caf9133 · CID_184) · 촬영 가이드 8133 후보
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -191,8 +191,9 @@
     <col min="33" max="33" width="12" customWidth="1"/>
     <col min="34" max="34" width="12" customWidth="1"/>
     <col min="35" max="35" width="12" customWidth="1"/>
-    <col min="36" max="36" width="11" customWidth="1"/>
+    <col min="36" max="36" width="12" customWidth="1"/>
     <col min="37" max="37" width="11" customWidth="1"/>
+    <col min="38" max="38" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -450,6 +451,11 @@
       <c r="AI6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">video-261019c 후보 갈아엎음(8132 · 16:46:47) · #185 태그 원형 링 하나 · #186 상태 띠 문제 있을 때만 ‖ 10-19 코드 세션 재확인(8123 · 캔버스 직접 캡처): 바로가기 S5 → 링 하늘색 + 「쿨다운 0.7s」(안쪽 주황 띠 없음 · 네모 없음) → Auto 끔 → 대기 마운트 차오름(하늘색 부분 링) → 만충 = 노란 링 + 「태그 스킬」 → 태그 누름 = 「쿨다운 4.3s」 · 링 하늘색 → 다시 만충 = 노랑 · 하단 띠: 문제 0 = 전투 · 조립 둘 다 띠 없음 · ⚠️ 알람 띠는 화면으로 못 세움(A · B 판 벨트 두 칸씩 끊었으나 물류 판정이 문제로 안 잡음 — 재고 남음) → CID_183 빈 칸 · 코드 경로는 종전 그대로 · CID_181~183 새 항목)</t>
+        </is>
+      </c>
+      <c r="AJ6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">video-261019d 후보(8133 · 새 사본 · 8132 동결) · #187 탄약 소진 아이콘 머리 위 ‖ 10-19 코드 세션 재확인(8123 · 캔버스 캡처): 「처음부터」 → 튜토리얼 판(마운트 0/40 · 고스트 빈 칸) = 주황 「물류 마크」가 로봇 머리 위 · HP · 쉴드 막대 · 회피 눈금과 겹침 0 · 같은 화면에 띠 「⚠ 생산 정지 — 만드는 것이 없다 외 1건」(② · ④) → 조립에서 고스트 채움(조립 화면 위 전투 인셋에도 머리 위) → 30초 뒤 마운트 차오름 = 아이콘 · 띠 사라짐 · ⚠️ 로봇 B · 합체 몸은 화면 미확인(몸 윗변을 그려진 사각에서 읽는 같은 길) · 576×1024 · 1024×768 창 미확인(인앱 프레임 하나) · 8133 복사 17:37:00 · CID_184 새 항목)</t>
         </is>
       </c>
     </row>
@@ -509,14 +515,15 @@
       <c r="AG7" s="2"/>
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
-      <c r="AJ7" s="2" t="inlineStr">
+      <c r="AJ7" s="2"/>
+      <c r="AK7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">버전</t>
         </is>
       </c>
-      <c r="AK7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">38a0ccf</t>
+      <c r="AL7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">caf9133</t>
         </is>
       </c>
     </row>
@@ -686,11 +693,16 @@
       </c>
       <c r="AJ8" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">caf9133</t>
+        </is>
+      </c>
+      <c r="AK8" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">PASSrate</t>
         </is>
       </c>
-      <c r="AK8" s="7">
-        <f>COUNTIF(AI9:AI191,"Pass")</f>
+      <c r="AL8" s="7">
+        <f>COUNTIF(AJ9:AJ192,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -789,13 +801,14 @@
       <c r="AG9" s="7"/>
       <c r="AH9" s="7"/>
       <c r="AI9" s="7"/>
-      <c r="AJ9" s="2" t="inlineStr">
+      <c r="AJ9" s="7"/>
+      <c r="AK9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FAILrate</t>
         </is>
       </c>
-      <c r="AK9" s="7">
-        <f>COUNTIF(AI9:AI191,"Fail")+COUNTIF(AI9:AI191,"Broken")</f>
+      <c r="AL9" s="7">
+        <f>COUNTIF(AJ9:AJ192,"Fail")+COUNTIF(AJ9:AJ192,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -858,13 +871,14 @@
       <c r="AG10" s="7"/>
       <c r="AH10" s="7"/>
       <c r="AI10" s="7"/>
-      <c r="AJ10" s="2" t="inlineStr">
+      <c r="AJ10" s="7"/>
+      <c r="AK10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">N/A</t>
         </is>
       </c>
-      <c r="AK10" s="7">
-        <f>COUNTIF(AI9:AI191,"N/A")</f>
+      <c r="AL10" s="7">
+        <f>COUNTIF(AJ9:AJ192,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -927,13 +941,14 @@
       <c r="AG11" s="7"/>
       <c r="AH11" s="7"/>
       <c r="AI11" s="7"/>
-      <c r="AJ11" s="2" t="inlineStr">
+      <c r="AJ11" s="7"/>
+      <c r="AK11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">전체 개수</t>
         </is>
       </c>
-      <c r="AK11" s="7">
-        <v>183</v>
+      <c r="AL11" s="7">
+        <v>184</v>
       </c>
     </row>
     <row r="12">
@@ -996,13 +1011,14 @@
       <c r="AG12" s="7"/>
       <c r="AH12" s="7"/>
       <c r="AI12" s="7"/>
-      <c r="AJ12" s="2" t="inlineStr">
+      <c r="AJ12" s="7"/>
+      <c r="AK12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">진행율</t>
         </is>
       </c>
-      <c r="AK12" s="7">
-        <f>TEXT((COUNTA(AI9:AI191))/183,"0.00%")</f>
+      <c r="AL12" s="7">
+        <f>TEXT((COUNTA(AJ9:AJ192))/184,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -1069,6 +1085,7 @@
       <c r="AG13" s="7"/>
       <c r="AH13" s="7"/>
       <c r="AI13" s="7"/>
+      <c r="AJ13" s="7"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -1125,6 +1142,7 @@
       <c r="AG14" s="7"/>
       <c r="AH14" s="7"/>
       <c r="AI14" s="7"/>
+      <c r="AJ14" s="7"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -1217,6 +1235,7 @@
       <c r="AG15" s="7"/>
       <c r="AH15" s="7"/>
       <c r="AI15" s="7"/>
+      <c r="AJ15" s="7"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -1309,6 +1328,7 @@
       <c r="AG16" s="7"/>
       <c r="AH16" s="7"/>
       <c r="AI16" s="7"/>
+      <c r="AJ16" s="7"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -1406,6 +1426,7 @@
       <c r="AG17" s="7"/>
       <c r="AH17" s="7"/>
       <c r="AI17" s="7"/>
+      <c r="AJ17" s="7"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -1467,6 +1488,7 @@
       <c r="AG18" s="7"/>
       <c r="AH18" s="7"/>
       <c r="AI18" s="7"/>
+      <c r="AJ18" s="7"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -1523,6 +1545,7 @@
       <c r="AG19" s="7"/>
       <c r="AH19" s="7"/>
       <c r="AI19" s="7"/>
+      <c r="AJ19" s="7"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1579,6 +1602,7 @@
       <c r="AG20" s="7"/>
       <c r="AH20" s="7"/>
       <c r="AI20" s="7"/>
+      <c r="AJ20" s="7"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1671,6 +1695,7 @@
       <c r="AG21" s="7"/>
       <c r="AH21" s="7"/>
       <c r="AI21" s="7"/>
+      <c r="AJ21" s="7"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1756,6 +1781,7 @@
       <c r="AG22" s="7"/>
       <c r="AH22" s="7"/>
       <c r="AI22" s="7"/>
+      <c r="AJ22" s="7"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -1820,6 +1846,7 @@
       <c r="AG23" s="7"/>
       <c r="AH23" s="7"/>
       <c r="AI23" s="7"/>
+      <c r="AJ23" s="7"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -1876,6 +1903,7 @@
       <c r="AG24" s="7"/>
       <c r="AH24" s="7"/>
       <c r="AI24" s="7"/>
+      <c r="AJ24" s="7"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -1932,6 +1960,7 @@
       <c r="AG25" s="7"/>
       <c r="AH25" s="7"/>
       <c r="AI25" s="7"/>
+      <c r="AJ25" s="7"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -2017,6 +2046,7 @@
       <c r="AG26" s="7"/>
       <c r="AH26" s="7"/>
       <c r="AI26" s="7"/>
+      <c r="AJ26" s="7"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -2077,6 +2107,7 @@
       <c r="AG27" s="7"/>
       <c r="AH27" s="7"/>
       <c r="AI27" s="7"/>
+      <c r="AJ27" s="7"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -2146,6 +2177,7 @@
       <c r="AG28" s="7"/>
       <c r="AH28" s="7"/>
       <c r="AI28" s="7"/>
+      <c r="AJ28" s="7"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -2210,6 +2242,7 @@
       <c r="AG29" s="7"/>
       <c r="AH29" s="7"/>
       <c r="AI29" s="7"/>
+      <c r="AJ29" s="7"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -2298,6 +2331,7 @@
       <c r="AG30" s="7"/>
       <c r="AH30" s="7"/>
       <c r="AI30" s="7"/>
+      <c r="AJ30" s="7"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -2391,6 +2425,7 @@
       <c r="AG31" s="7"/>
       <c r="AH31" s="7"/>
       <c r="AI31" s="7"/>
+      <c r="AJ31" s="7"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -2471,6 +2506,7 @@
       <c r="AG32" s="7"/>
       <c r="AH32" s="7"/>
       <c r="AI32" s="7"/>
+      <c r="AJ32" s="7"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -2559,6 +2595,7 @@
       <c r="AG33" s="7"/>
       <c r="AH33" s="7"/>
       <c r="AI33" s="7"/>
+      <c r="AJ33" s="7"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -2647,6 +2684,7 @@
       <c r="AG34" s="7"/>
       <c r="AH34" s="7"/>
       <c r="AI34" s="7"/>
+      <c r="AJ34" s="7"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -2744,6 +2782,7 @@
       <c r="AG35" s="7"/>
       <c r="AH35" s="7"/>
       <c r="AI35" s="7"/>
+      <c r="AJ35" s="7"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -2816,6 +2855,7 @@
       <c r="AG36" s="7"/>
       <c r="AH36" s="7"/>
       <c r="AI36" s="7"/>
+      <c r="AJ36" s="7"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -2872,6 +2912,7 @@
       <c r="AG37" s="7"/>
       <c r="AH37" s="7"/>
       <c r="AI37" s="7"/>
+      <c r="AJ37" s="7"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -2949,6 +2990,7 @@
       <c r="AG38" s="7"/>
       <c r="AH38" s="7"/>
       <c r="AI38" s="7"/>
+      <c r="AJ38" s="7"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -3037,6 +3079,7 @@
       <c r="AG39" s="7"/>
       <c r="AH39" s="7"/>
       <c r="AI39" s="7"/>
+      <c r="AJ39" s="7"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -3126,6 +3169,7 @@
       <c r="AG40" s="7"/>
       <c r="AH40" s="7"/>
       <c r="AI40" s="7"/>
+      <c r="AJ40" s="7"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -3210,6 +3254,7 @@
       <c r="AG41" s="7"/>
       <c r="AH41" s="7"/>
       <c r="AI41" s="7"/>
+      <c r="AJ41" s="7"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -3278,6 +3323,7 @@
       <c r="AG42" s="7"/>
       <c r="AH42" s="7"/>
       <c r="AI42" s="7"/>
+      <c r="AJ42" s="7"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -3366,6 +3412,7 @@
       <c r="AG43" s="7"/>
       <c r="AH43" s="7"/>
       <c r="AI43" s="7"/>
+      <c r="AJ43" s="7"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -3427,6 +3474,7 @@
       <c r="AG44" s="7"/>
       <c r="AH44" s="7"/>
       <c r="AI44" s="7"/>
+      <c r="AJ44" s="7"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -3511,6 +3559,7 @@
       <c r="AG45" s="7"/>
       <c r="AH45" s="7"/>
       <c r="AI45" s="7"/>
+      <c r="AJ45" s="7"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -3595,6 +3644,7 @@
       <c r="AG46" s="7"/>
       <c r="AH46" s="7"/>
       <c r="AI46" s="7"/>
+      <c r="AJ46" s="7"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -3656,6 +3706,7 @@
       <c r="AG47" s="7"/>
       <c r="AH47" s="7"/>
       <c r="AI47" s="7"/>
+      <c r="AJ47" s="7"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -3712,6 +3763,7 @@
       <c r="AG48" s="7"/>
       <c r="AH48" s="7"/>
       <c r="AI48" s="7"/>
+      <c r="AJ48" s="7"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -3768,6 +3820,7 @@
       <c r="AG49" s="7"/>
       <c r="AH49" s="7"/>
       <c r="AI49" s="7"/>
+      <c r="AJ49" s="7"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -3848,6 +3901,7 @@
       <c r="AG50" s="7"/>
       <c r="AH50" s="7"/>
       <c r="AI50" s="7"/>
+      <c r="AJ50" s="7"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -3928,6 +3982,7 @@
       <c r="AG51" s="7"/>
       <c r="AH51" s="7"/>
       <c r="AI51" s="7"/>
+      <c r="AJ51" s="7"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -3989,6 +4044,7 @@
       <c r="AG52" s="7"/>
       <c r="AH52" s="7"/>
       <c r="AI52" s="7"/>
+      <c r="AJ52" s="7"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -4050,6 +4106,7 @@
       <c r="AG53" s="7"/>
       <c r="AH53" s="7"/>
       <c r="AI53" s="7"/>
+      <c r="AJ53" s="7"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -4106,6 +4163,7 @@
       <c r="AG54" s="7"/>
       <c r="AH54" s="7"/>
       <c r="AI54" s="7"/>
+      <c r="AJ54" s="7"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -4198,6 +4256,7 @@
       <c r="AG55" s="7"/>
       <c r="AH55" s="7"/>
       <c r="AI55" s="7"/>
+      <c r="AJ55" s="7"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -4270,6 +4329,7 @@
       <c r="AG56" s="7"/>
       <c r="AH56" s="7"/>
       <c r="AI56" s="7"/>
+      <c r="AJ56" s="7"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -4351,6 +4411,7 @@
       <c r="AG57" s="7"/>
       <c r="AH57" s="7"/>
       <c r="AI57" s="7"/>
+      <c r="AJ57" s="7"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -4440,6 +4501,7 @@
       <c r="AG58" s="7"/>
       <c r="AH58" s="7"/>
       <c r="AI58" s="7"/>
+      <c r="AJ58" s="7"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -4496,6 +4558,7 @@
       <c r="AG59" s="7"/>
       <c r="AH59" s="7"/>
       <c r="AI59" s="7"/>
+      <c r="AJ59" s="7"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -4552,6 +4615,7 @@
       <c r="AG60" s="7"/>
       <c r="AH60" s="7"/>
       <c r="AI60" s="7"/>
+      <c r="AJ60" s="7"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -4620,6 +4684,7 @@
       <c r="AG61" s="7"/>
       <c r="AH61" s="7"/>
       <c r="AI61" s="7"/>
+      <c r="AJ61" s="7"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -4696,6 +4761,7 @@
       <c r="AG62" s="7"/>
       <c r="AH62" s="7"/>
       <c r="AI62" s="7"/>
+      <c r="AJ62" s="7"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -4764,6 +4830,7 @@
       <c r="AG63" s="7"/>
       <c r="AH63" s="7"/>
       <c r="AI63" s="7"/>
+      <c r="AJ63" s="7"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -4820,6 +4887,7 @@
       <c r="AG64" s="7"/>
       <c r="AH64" s="7"/>
       <c r="AI64" s="7"/>
+      <c r="AJ64" s="7"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -4881,6 +4949,7 @@
       <c r="AG65" s="7"/>
       <c r="AH65" s="7"/>
       <c r="AI65" s="7"/>
+      <c r="AJ65" s="7"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
@@ -4949,6 +5018,7 @@
       <c r="AG66" s="7"/>
       <c r="AH66" s="7"/>
       <c r="AI66" s="7"/>
+      <c r="AJ66" s="7"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -5005,6 +5075,7 @@
       <c r="AG67" s="7"/>
       <c r="AH67" s="7"/>
       <c r="AI67" s="7"/>
+      <c r="AJ67" s="7"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
@@ -5065,6 +5136,7 @@
       <c r="AG68" s="7"/>
       <c r="AH68" s="7"/>
       <c r="AI68" s="7"/>
+      <c r="AJ68" s="7"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -5157,6 +5229,7 @@
       <c r="AG69" s="7"/>
       <c r="AH69" s="7"/>
       <c r="AI69" s="7"/>
+      <c r="AJ69" s="7"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
@@ -5213,6 +5286,7 @@
       <c r="AG70" s="7"/>
       <c r="AH70" s="7"/>
       <c r="AI70" s="7"/>
+      <c r="AJ70" s="7"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -5274,6 +5348,7 @@
       <c r="AG71" s="7"/>
       <c r="AH71" s="7"/>
       <c r="AI71" s="7"/>
+      <c r="AJ71" s="7"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
@@ -5346,6 +5421,7 @@
       <c r="AG72" s="7"/>
       <c r="AH72" s="7"/>
       <c r="AI72" s="7"/>
+      <c r="AJ72" s="7"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
@@ -5407,6 +5483,7 @@
       <c r="AG73" s="7"/>
       <c r="AH73" s="7"/>
       <c r="AI73" s="7"/>
+      <c r="AJ73" s="7"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -5463,6 +5540,7 @@
       <c r="AG74" s="7"/>
       <c r="AH74" s="7"/>
       <c r="AI74" s="7"/>
+      <c r="AJ74" s="7"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -5519,6 +5597,7 @@
       <c r="AG75" s="7"/>
       <c r="AH75" s="7"/>
       <c r="AI75" s="7"/>
+      <c r="AJ75" s="7"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -5575,6 +5654,7 @@
       <c r="AG76" s="7"/>
       <c r="AH76" s="7"/>
       <c r="AI76" s="7"/>
+      <c r="AJ76" s="7"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -5635,6 +5715,7 @@
       <c r="AG77" s="7"/>
       <c r="AH77" s="7"/>
       <c r="AI77" s="7"/>
+      <c r="AJ77" s="7"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
@@ -5691,6 +5772,7 @@
       <c r="AG78" s="7"/>
       <c r="AH78" s="7"/>
       <c r="AI78" s="7"/>
+      <c r="AJ78" s="7"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -5752,6 +5834,7 @@
       <c r="AG79" s="7"/>
       <c r="AH79" s="7"/>
       <c r="AI79" s="7"/>
+      <c r="AJ79" s="7"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
@@ -5824,6 +5907,7 @@
       <c r="AG80" s="7"/>
       <c r="AH80" s="7"/>
       <c r="AI80" s="7"/>
+      <c r="AJ80" s="7"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
@@ -5884,6 +5968,7 @@
       <c r="AG81" s="7"/>
       <c r="AH81" s="7"/>
       <c r="AI81" s="7"/>
+      <c r="AJ81" s="7"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
@@ -5940,6 +6025,7 @@
       <c r="AG82" s="7"/>
       <c r="AH82" s="7"/>
       <c r="AI82" s="7"/>
+      <c r="AJ82" s="7"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
@@ -6001,6 +6087,7 @@
       <c r="AG83" s="7"/>
       <c r="AH83" s="7"/>
       <c r="AI83" s="7"/>
+      <c r="AJ83" s="7"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
@@ -6057,6 +6144,7 @@
       <c r="AG84" s="7"/>
       <c r="AH84" s="7"/>
       <c r="AI84" s="7"/>
+      <c r="AJ84" s="7"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
@@ -6113,6 +6201,7 @@
       <c r="AG85" s="7"/>
       <c r="AH85" s="7"/>
       <c r="AI85" s="7"/>
+      <c r="AJ85" s="7"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
@@ -6174,6 +6263,7 @@
       <c r="AG86" s="7"/>
       <c r="AH86" s="7"/>
       <c r="AI86" s="7"/>
+      <c r="AJ86" s="7"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
@@ -6230,6 +6320,7 @@
       <c r="AG87" s="7"/>
       <c r="AH87" s="7"/>
       <c r="AI87" s="7"/>
+      <c r="AJ87" s="7"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
@@ -6286,6 +6377,7 @@
       <c r="AG88" s="7"/>
       <c r="AH88" s="7"/>
       <c r="AI88" s="7"/>
+      <c r="AJ88" s="7"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
@@ -6342,6 +6434,7 @@
       <c r="AG89" s="7"/>
       <c r="AH89" s="7"/>
       <c r="AI89" s="7"/>
+      <c r="AJ89" s="7"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
@@ -6427,6 +6520,7 @@
       <c r="AG90" s="7"/>
       <c r="AH90" s="7"/>
       <c r="AI90" s="7"/>
+      <c r="AJ90" s="7"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
@@ -6483,6 +6577,7 @@
       <c r="AG91" s="7"/>
       <c r="AH91" s="7"/>
       <c r="AI91" s="7"/>
+      <c r="AJ91" s="7"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
@@ -6575,6 +6670,7 @@
       <c r="AG92" s="7"/>
       <c r="AH92" s="7"/>
       <c r="AI92" s="7"/>
+      <c r="AJ92" s="7"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
@@ -6672,6 +6768,7 @@
       <c r="AG93" s="7"/>
       <c r="AH93" s="7"/>
       <c r="AI93" s="7"/>
+      <c r="AJ93" s="7"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
@@ -6733,6 +6830,7 @@
       <c r="AG94" s="7"/>
       <c r="AH94" s="7"/>
       <c r="AI94" s="7"/>
+      <c r="AJ94" s="7"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
@@ -6794,6 +6892,7 @@
       <c r="AG95" s="7"/>
       <c r="AH95" s="7"/>
       <c r="AI95" s="7"/>
+      <c r="AJ95" s="7"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
@@ -6874,6 +6973,7 @@
       <c r="AG96" s="7"/>
       <c r="AH96" s="7"/>
       <c r="AI96" s="7"/>
+      <c r="AJ96" s="7"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="inlineStr">
@@ -6930,6 +7030,7 @@
       <c r="AG97" s="7"/>
       <c r="AH97" s="7"/>
       <c r="AI97" s="7"/>
+      <c r="AJ97" s="7"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
@@ -6986,6 +7087,7 @@
       <c r="AG98" s="7"/>
       <c r="AH98" s="7"/>
       <c r="AI98" s="7"/>
+      <c r="AJ98" s="7"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
@@ -7042,6 +7144,7 @@
       <c r="AG99" s="7"/>
       <c r="AH99" s="7"/>
       <c r="AI99" s="7"/>
+      <c r="AJ99" s="7"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
@@ -7107,6 +7210,7 @@
       <c r="AG100" s="7"/>
       <c r="AH100" s="7"/>
       <c r="AI100" s="7"/>
+      <c r="AJ100" s="7"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
@@ -7163,6 +7267,7 @@
       <c r="AG101" s="7"/>
       <c r="AH101" s="7"/>
       <c r="AI101" s="7"/>
+      <c r="AJ101" s="7"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
@@ -7219,6 +7324,7 @@
       <c r="AG102" s="7"/>
       <c r="AH102" s="7"/>
       <c r="AI102" s="7"/>
+      <c r="AJ102" s="7"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="inlineStr">
@@ -7275,6 +7381,7 @@
       <c r="AG103" s="7"/>
       <c r="AH103" s="7"/>
       <c r="AI103" s="7"/>
+      <c r="AJ103" s="7"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="inlineStr">
@@ -7336,6 +7443,7 @@
       <c r="AG104" s="7"/>
       <c r="AH104" s="7"/>
       <c r="AI104" s="7"/>
+      <c r="AJ104" s="7"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
@@ -7392,6 +7500,7 @@
       <c r="AG105" s="7"/>
       <c r="AH105" s="7"/>
       <c r="AI105" s="7"/>
+      <c r="AJ105" s="7"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
@@ -7448,6 +7557,7 @@
       <c r="AG106" s="7"/>
       <c r="AH106" s="7"/>
       <c r="AI106" s="7"/>
+      <c r="AJ106" s="7"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
@@ -7504,6 +7614,7 @@
       <c r="AG107" s="7"/>
       <c r="AH107" s="7"/>
       <c r="AI107" s="7"/>
+      <c r="AJ107" s="7"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
@@ -7564,6 +7675,7 @@
       <c r="AG108" s="7"/>
       <c r="AH108" s="7"/>
       <c r="AI108" s="7"/>
+      <c r="AJ108" s="7"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="inlineStr">
@@ -7629,6 +7741,7 @@
       <c r="AG109" s="7"/>
       <c r="AH109" s="7"/>
       <c r="AI109" s="7"/>
+      <c r="AJ109" s="7"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
@@ -7702,6 +7815,7 @@
       <c r="AG110" s="7"/>
       <c r="AH110" s="7"/>
       <c r="AI110" s="7"/>
+      <c r="AJ110" s="7"/>
     </row>
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
@@ -7778,6 +7892,7 @@
       <c r="AG111" s="7"/>
       <c r="AH111" s="7"/>
       <c r="AI111" s="7"/>
+      <c r="AJ111" s="7"/>
     </row>
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
@@ -7851,6 +7966,7 @@
       <c r="AG112" s="7"/>
       <c r="AH112" s="7"/>
       <c r="AI112" s="7"/>
+      <c r="AJ112" s="7"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
@@ -7916,6 +8032,7 @@
       <c r="AG113" s="7"/>
       <c r="AH113" s="7"/>
       <c r="AI113" s="7"/>
+      <c r="AJ113" s="7"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="inlineStr">
@@ -7997,6 +8114,7 @@
       <c r="AG114" s="7"/>
       <c r="AH114" s="7"/>
       <c r="AI114" s="7"/>
+      <c r="AJ114" s="7"/>
     </row>
     <row r="115">
       <c r="A115" s="7" t="inlineStr">
@@ -8070,6 +8188,7 @@
       <c r="AG115" s="7"/>
       <c r="AH115" s="7"/>
       <c r="AI115" s="7"/>
+      <c r="AJ115" s="7"/>
     </row>
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
@@ -8151,6 +8270,7 @@
         </is>
       </c>
       <c r="AI116" s="7"/>
+      <c r="AJ116" s="7"/>
     </row>
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
@@ -8228,6 +8348,7 @@
       <c r="AG117" s="7"/>
       <c r="AH117" s="7"/>
       <c r="AI117" s="7"/>
+      <c r="AJ117" s="7"/>
     </row>
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
@@ -8305,6 +8426,7 @@
       <c r="AG118" s="7"/>
       <c r="AH118" s="7"/>
       <c r="AI118" s="7"/>
+      <c r="AJ118" s="7"/>
     </row>
     <row r="119">
       <c r="A119" s="7" t="inlineStr">
@@ -8378,6 +8500,7 @@
       <c r="AG119" s="7"/>
       <c r="AH119" s="7"/>
       <c r="AI119" s="7"/>
+      <c r="AJ119" s="7"/>
     </row>
     <row r="120">
       <c r="A120" s="7" t="inlineStr">
@@ -8443,6 +8566,7 @@
       <c r="AG120" s="7"/>
       <c r="AH120" s="7"/>
       <c r="AI120" s="7"/>
+      <c r="AJ120" s="7"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="inlineStr">
@@ -8520,6 +8644,7 @@
       <c r="AG121" s="7"/>
       <c r="AH121" s="7"/>
       <c r="AI121" s="7"/>
+      <c r="AJ121" s="7"/>
     </row>
     <row r="122">
       <c r="A122" s="7" t="inlineStr">
@@ -8597,6 +8722,7 @@
       <c r="AG122" s="7"/>
       <c r="AH122" s="7"/>
       <c r="AI122" s="7"/>
+      <c r="AJ122" s="7"/>
     </row>
     <row r="123">
       <c r="A123" s="7" t="inlineStr">
@@ -8662,6 +8788,7 @@
       <c r="AG123" s="7"/>
       <c r="AH123" s="7"/>
       <c r="AI123" s="7"/>
+      <c r="AJ123" s="7"/>
     </row>
     <row r="124">
       <c r="A124" s="7" t="inlineStr">
@@ -8735,6 +8862,7 @@
       <c r="AG124" s="7"/>
       <c r="AH124" s="7"/>
       <c r="AI124" s="7"/>
+      <c r="AJ124" s="7"/>
     </row>
     <row r="125">
       <c r="A125" s="7" t="inlineStr">
@@ -8800,6 +8928,7 @@
       <c r="AG125" s="7"/>
       <c r="AH125" s="7"/>
       <c r="AI125" s="7"/>
+      <c r="AJ125" s="7"/>
     </row>
     <row r="126">
       <c r="A126" s="7" t="inlineStr">
@@ -8865,6 +8994,7 @@
       <c r="AG126" s="7"/>
       <c r="AH126" s="7"/>
       <c r="AI126" s="7"/>
+      <c r="AJ126" s="7"/>
     </row>
     <row r="127">
       <c r="A127" s="7" t="inlineStr">
@@ -8934,6 +9064,7 @@
       <c r="AG127" s="7"/>
       <c r="AH127" s="7"/>
       <c r="AI127" s="7"/>
+      <c r="AJ127" s="7"/>
     </row>
     <row r="128">
       <c r="A128" s="7" t="inlineStr">
@@ -9003,6 +9134,7 @@
       <c r="AG128" s="7"/>
       <c r="AH128" s="7"/>
       <c r="AI128" s="7"/>
+      <c r="AJ128" s="7"/>
     </row>
     <row r="129">
       <c r="A129" s="7" t="inlineStr">
@@ -9072,6 +9204,7 @@
       <c r="AG129" s="7"/>
       <c r="AH129" s="7"/>
       <c r="AI129" s="7"/>
+      <c r="AJ129" s="7"/>
     </row>
     <row r="130">
       <c r="A130" s="7" t="inlineStr">
@@ -9137,6 +9270,7 @@
       <c r="AG130" s="7"/>
       <c r="AH130" s="7"/>
       <c r="AI130" s="7"/>
+      <c r="AJ130" s="7"/>
     </row>
     <row r="131">
       <c r="A131" s="7" t="inlineStr">
@@ -9210,6 +9344,7 @@
       <c r="AG131" s="7"/>
       <c r="AH131" s="7"/>
       <c r="AI131" s="7"/>
+      <c r="AJ131" s="7"/>
     </row>
     <row r="132">
       <c r="A132" s="7" t="inlineStr">
@@ -9287,6 +9422,7 @@
       <c r="AG132" s="7"/>
       <c r="AH132" s="7"/>
       <c r="AI132" s="7"/>
+      <c r="AJ132" s="7"/>
     </row>
     <row r="133">
       <c r="A133" s="7" t="inlineStr">
@@ -9364,6 +9500,7 @@
       <c r="AG133" s="7"/>
       <c r="AH133" s="7"/>
       <c r="AI133" s="7"/>
+      <c r="AJ133" s="7"/>
     </row>
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
@@ -9437,6 +9574,7 @@
       <c r="AG134" s="7"/>
       <c r="AH134" s="7"/>
       <c r="AI134" s="7"/>
+      <c r="AJ134" s="7"/>
     </row>
     <row r="135">
       <c r="A135" s="7" t="inlineStr">
@@ -9510,6 +9648,7 @@
       <c r="AG135" s="7"/>
       <c r="AH135" s="7"/>
       <c r="AI135" s="7"/>
+      <c r="AJ135" s="7"/>
     </row>
     <row r="136">
       <c r="A136" s="7" t="inlineStr">
@@ -9583,6 +9722,7 @@
       <c r="AG136" s="7"/>
       <c r="AH136" s="7"/>
       <c r="AI136" s="7"/>
+      <c r="AJ136" s="7"/>
     </row>
     <row r="137">
       <c r="A137" s="7" t="inlineStr">
@@ -9652,6 +9792,7 @@
       <c r="AG137" s="7"/>
       <c r="AH137" s="7"/>
       <c r="AI137" s="7"/>
+      <c r="AJ137" s="7"/>
     </row>
     <row r="138">
       <c r="A138" s="7" t="inlineStr">
@@ -9721,6 +9862,7 @@
       <c r="AG138" s="7"/>
       <c r="AH138" s="7"/>
       <c r="AI138" s="7"/>
+      <c r="AJ138" s="7"/>
     </row>
     <row r="139">
       <c r="A139" s="7" t="inlineStr">
@@ -9790,6 +9932,7 @@
       <c r="AG139" s="7"/>
       <c r="AH139" s="7"/>
       <c r="AI139" s="7"/>
+      <c r="AJ139" s="7"/>
     </row>
     <row r="140">
       <c r="A140" s="7" t="inlineStr">
@@ -9855,6 +9998,7 @@
       <c r="AG140" s="7"/>
       <c r="AH140" s="7"/>
       <c r="AI140" s="7"/>
+      <c r="AJ140" s="7"/>
     </row>
     <row r="141">
       <c r="A141" s="7" t="inlineStr">
@@ -9932,6 +10076,7 @@
       <c r="AG141" s="7"/>
       <c r="AH141" s="7"/>
       <c r="AI141" s="7"/>
+      <c r="AJ141" s="7"/>
     </row>
     <row r="142">
       <c r="A142" s="7" t="inlineStr">
@@ -9997,6 +10142,7 @@
       <c r="AG142" s="7"/>
       <c r="AH142" s="7"/>
       <c r="AI142" s="7"/>
+      <c r="AJ142" s="7"/>
     </row>
     <row r="143">
       <c r="A143" s="7" t="inlineStr">
@@ -10062,6 +10208,7 @@
       <c r="AG143" s="7"/>
       <c r="AH143" s="7"/>
       <c r="AI143" s="7"/>
+      <c r="AJ143" s="7"/>
     </row>
     <row r="144">
       <c r="A144" s="7" t="inlineStr">
@@ -10127,6 +10274,7 @@
       <c r="AG144" s="7"/>
       <c r="AH144" s="7"/>
       <c r="AI144" s="7"/>
+      <c r="AJ144" s="7"/>
     </row>
     <row r="145">
       <c r="A145" s="7" t="inlineStr">
@@ -10208,6 +10356,7 @@
       <c r="AG145" s="7"/>
       <c r="AH145" s="7"/>
       <c r="AI145" s="7"/>
+      <c r="AJ145" s="7"/>
     </row>
     <row r="146">
       <c r="A146" s="7" t="inlineStr">
@@ -10277,6 +10426,7 @@
       <c r="AG146" s="7"/>
       <c r="AH146" s="7"/>
       <c r="AI146" s="7"/>
+      <c r="AJ146" s="7"/>
     </row>
     <row r="147">
       <c r="A147" s="7" t="inlineStr">
@@ -10358,6 +10508,7 @@
       <c r="AG147" s="7"/>
       <c r="AH147" s="7"/>
       <c r="AI147" s="7"/>
+      <c r="AJ147" s="7"/>
     </row>
     <row r="148">
       <c r="A148" s="7" t="inlineStr">
@@ -10423,6 +10574,7 @@
       <c r="AG148" s="7"/>
       <c r="AH148" s="7"/>
       <c r="AI148" s="7"/>
+      <c r="AJ148" s="7"/>
     </row>
     <row r="149">
       <c r="A149" s="7" t="inlineStr">
@@ -10496,6 +10648,7 @@
       <c r="AG149" s="7"/>
       <c r="AH149" s="7"/>
       <c r="AI149" s="7"/>
+      <c r="AJ149" s="7"/>
     </row>
     <row r="150">
       <c r="A150" s="7" t="inlineStr">
@@ -10573,6 +10726,7 @@
       <c r="AG150" s="7"/>
       <c r="AH150" s="7"/>
       <c r="AI150" s="7"/>
+      <c r="AJ150" s="7"/>
     </row>
     <row r="151">
       <c r="A151" s="7" t="inlineStr">
@@ -10642,6 +10796,7 @@
       <c r="AG151" s="7"/>
       <c r="AH151" s="7"/>
       <c r="AI151" s="7"/>
+      <c r="AJ151" s="7"/>
     </row>
     <row r="152">
       <c r="A152" s="7" t="inlineStr">
@@ -10715,6 +10870,7 @@
       <c r="AG152" s="7"/>
       <c r="AH152" s="7"/>
       <c r="AI152" s="7"/>
+      <c r="AJ152" s="7"/>
     </row>
     <row r="153">
       <c r="A153" s="7" t="inlineStr">
@@ -10788,6 +10944,7 @@
       <c r="AG153" s="7"/>
       <c r="AH153" s="7"/>
       <c r="AI153" s="7"/>
+      <c r="AJ153" s="7"/>
     </row>
     <row r="154">
       <c r="A154" s="7" t="inlineStr">
@@ -10849,6 +11006,7 @@
       <c r="AG154" s="7"/>
       <c r="AH154" s="7"/>
       <c r="AI154" s="7"/>
+      <c r="AJ154" s="7"/>
     </row>
     <row r="155">
       <c r="A155" s="7" t="inlineStr">
@@ -10914,6 +11072,7 @@
       <c r="AG155" s="7"/>
       <c r="AH155" s="7"/>
       <c r="AI155" s="7"/>
+      <c r="AJ155" s="7"/>
     </row>
     <row r="156">
       <c r="A156" s="7" t="inlineStr">
@@ -10983,6 +11142,7 @@
       <c r="AG156" s="7"/>
       <c r="AH156" s="7"/>
       <c r="AI156" s="7"/>
+      <c r="AJ156" s="7"/>
     </row>
     <row r="157">
       <c r="A157" s="7" t="inlineStr">
@@ -11048,6 +11208,7 @@
       <c r="AG157" s="7"/>
       <c r="AH157" s="7"/>
       <c r="AI157" s="7"/>
+      <c r="AJ157" s="7"/>
     </row>
     <row r="158">
       <c r="A158" s="7" t="inlineStr">
@@ -11113,6 +11274,7 @@
       <c r="AG158" s="7"/>
       <c r="AH158" s="7"/>
       <c r="AI158" s="7"/>
+      <c r="AJ158" s="7"/>
     </row>
     <row r="159">
       <c r="A159" s="7" t="inlineStr">
@@ -11178,6 +11340,7 @@
       <c r="AG159" s="7"/>
       <c r="AH159" s="7"/>
       <c r="AI159" s="7"/>
+      <c r="AJ159" s="7"/>
     </row>
     <row r="160">
       <c r="A160" s="7" t="inlineStr">
@@ -11243,6 +11406,7 @@
       <c r="AG160" s="7"/>
       <c r="AH160" s="7"/>
       <c r="AI160" s="7"/>
+      <c r="AJ160" s="7"/>
     </row>
     <row r="161">
       <c r="A161" s="7" t="inlineStr">
@@ -11312,6 +11476,7 @@
       <c r="AG161" s="7"/>
       <c r="AH161" s="7"/>
       <c r="AI161" s="7"/>
+      <c r="AJ161" s="7"/>
     </row>
     <row r="162">
       <c r="A162" s="7" t="inlineStr">
@@ -11377,6 +11542,7 @@
       <c r="AG162" s="7"/>
       <c r="AH162" s="7"/>
       <c r="AI162" s="7"/>
+      <c r="AJ162" s="7"/>
     </row>
     <row r="163">
       <c r="A163" s="7" t="inlineStr">
@@ -11442,6 +11608,7 @@
       <c r="AG163" s="7"/>
       <c r="AH163" s="7"/>
       <c r="AI163" s="7"/>
+      <c r="AJ163" s="7"/>
     </row>
     <row r="164">
       <c r="A164" s="7" t="inlineStr">
@@ -11507,6 +11674,7 @@
       <c r="AG164" s="7"/>
       <c r="AH164" s="7"/>
       <c r="AI164" s="7"/>
+      <c r="AJ164" s="7"/>
     </row>
     <row r="165">
       <c r="A165" s="7" t="inlineStr">
@@ -11572,6 +11740,7 @@
       <c r="AG165" s="7"/>
       <c r="AH165" s="7"/>
       <c r="AI165" s="7"/>
+      <c r="AJ165" s="7"/>
     </row>
     <row r="166">
       <c r="A166" s="7" t="inlineStr">
@@ -11641,6 +11810,7 @@
       <c r="AG166" s="7"/>
       <c r="AH166" s="7"/>
       <c r="AI166" s="7"/>
+      <c r="AJ166" s="7"/>
     </row>
     <row r="167">
       <c r="A167" s="7" t="inlineStr">
@@ -11706,6 +11876,7 @@
       <c r="AG167" s="7"/>
       <c r="AH167" s="7"/>
       <c r="AI167" s="7"/>
+      <c r="AJ167" s="7"/>
     </row>
     <row r="168">
       <c r="A168" s="7" t="inlineStr">
@@ -11771,6 +11942,7 @@
       <c r="AG168" s="7"/>
       <c r="AH168" s="7"/>
       <c r="AI168" s="7"/>
+      <c r="AJ168" s="7"/>
     </row>
     <row r="169">
       <c r="A169" s="7" t="inlineStr">
@@ -11836,6 +12008,7 @@
       <c r="AG169" s="7"/>
       <c r="AH169" s="7"/>
       <c r="AI169" s="7"/>
+      <c r="AJ169" s="7"/>
     </row>
     <row r="170">
       <c r="A170" s="7" t="inlineStr">
@@ -11905,6 +12078,7 @@
       <c r="AG170" s="7"/>
       <c r="AH170" s="7"/>
       <c r="AI170" s="7"/>
+      <c r="AJ170" s="7"/>
     </row>
     <row r="171">
       <c r="A171" s="7" t="inlineStr">
@@ -11966,6 +12140,7 @@
       <c r="AG171" s="7"/>
       <c r="AH171" s="7"/>
       <c r="AI171" s="7"/>
+      <c r="AJ171" s="7"/>
     </row>
     <row r="172">
       <c r="A172" s="7" t="inlineStr">
@@ -12027,6 +12202,7 @@
       <c r="AG172" s="7"/>
       <c r="AH172" s="7"/>
       <c r="AI172" s="7"/>
+      <c r="AJ172" s="7"/>
     </row>
     <row r="173">
       <c r="A173" s="7" t="inlineStr">
@@ -12096,6 +12272,7 @@
       <c r="AG173" s="7"/>
       <c r="AH173" s="7"/>
       <c r="AI173" s="7"/>
+      <c r="AJ173" s="7"/>
     </row>
     <row r="174">
       <c r="A174" s="7" t="inlineStr">
@@ -12161,6 +12338,7 @@
       <c r="AG174" s="7"/>
       <c r="AH174" s="7"/>
       <c r="AI174" s="7"/>
+      <c r="AJ174" s="7"/>
     </row>
     <row r="175">
       <c r="A175" s="7" t="inlineStr">
@@ -12230,6 +12408,7 @@
       <c r="AG175" s="7"/>
       <c r="AH175" s="7"/>
       <c r="AI175" s="7"/>
+      <c r="AJ175" s="7"/>
     </row>
     <row r="176">
       <c r="A176" s="7" t="inlineStr">
@@ -12295,6 +12474,7 @@
       <c r="AG176" s="7"/>
       <c r="AH176" s="7"/>
       <c r="AI176" s="7"/>
+      <c r="AJ176" s="7"/>
     </row>
     <row r="177">
       <c r="A177" s="7" t="inlineStr">
@@ -12360,6 +12540,7 @@
       <c r="AG177" s="7"/>
       <c r="AH177" s="7"/>
       <c r="AI177" s="7"/>
+      <c r="AJ177" s="7"/>
     </row>
     <row r="178">
       <c r="A178" s="7" t="inlineStr">
@@ -12425,6 +12606,7 @@
       <c r="AG178" s="7"/>
       <c r="AH178" s="7"/>
       <c r="AI178" s="7"/>
+      <c r="AJ178" s="7"/>
     </row>
     <row r="179">
       <c r="A179" s="7" t="inlineStr">
@@ -12490,6 +12672,7 @@
       <c r="AG179" s="7"/>
       <c r="AH179" s="7"/>
       <c r="AI179" s="7"/>
+      <c r="AJ179" s="7"/>
     </row>
     <row r="180">
       <c r="A180" s="7" t="inlineStr">
@@ -12555,6 +12738,7 @@
       <c r="AG180" s="7"/>
       <c r="AH180" s="7"/>
       <c r="AI180" s="7"/>
+      <c r="AJ180" s="7"/>
     </row>
     <row r="181">
       <c r="A181" s="7" t="inlineStr">
@@ -12620,6 +12804,7 @@
       </c>
       <c r="AH181" s="7"/>
       <c r="AI181" s="7"/>
+      <c r="AJ181" s="7"/>
     </row>
     <row r="182">
       <c r="A182" s="7" t="inlineStr">
@@ -12685,6 +12870,7 @@
       </c>
       <c r="AH182" s="7"/>
       <c r="AI182" s="7"/>
+      <c r="AJ182" s="7"/>
     </row>
     <row r="183">
       <c r="A183" s="7" t="inlineStr">
@@ -12750,6 +12936,7 @@
         </is>
       </c>
       <c r="AI183" s="7"/>
+      <c r="AJ183" s="7"/>
     </row>
     <row r="184">
       <c r="A184" s="7" t="inlineStr">
@@ -12811,6 +12998,7 @@
       <c r="AG184" s="7"/>
       <c r="AH184" s="7"/>
       <c r="AI184" s="7"/>
+      <c r="AJ184" s="7"/>
     </row>
     <row r="185">
       <c r="A185" s="7" t="inlineStr">
@@ -12876,6 +13064,7 @@
         </is>
       </c>
       <c r="AI185" s="7"/>
+      <c r="AJ185" s="7"/>
     </row>
     <row r="186">
       <c r="A186" s="7" t="inlineStr">
@@ -12941,6 +13130,7 @@
         </is>
       </c>
       <c r="AI186" s="7"/>
+      <c r="AJ186" s="7"/>
     </row>
     <row r="187">
       <c r="A187" s="7" t="inlineStr">
@@ -13006,6 +13196,7 @@
         </is>
       </c>
       <c r="AI187" s="7"/>
+      <c r="AJ187" s="7"/>
     </row>
     <row r="188">
       <c r="A188" s="7" t="inlineStr">
@@ -13071,6 +13262,7 @@
         </is>
       </c>
       <c r="AI188" s="7"/>
+      <c r="AJ188" s="7"/>
     </row>
     <row r="189">
       <c r="A189" s="7" t="inlineStr">
@@ -13136,6 +13328,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AJ189" s="7"/>
     </row>
     <row r="190">
       <c r="A190" s="7" t="inlineStr">
@@ -13201,6 +13394,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AJ190" s="7"/>
     </row>
     <row r="191">
       <c r="A191" s="7" t="inlineStr">
@@ -13230,7 +13424,7 @@
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t xml:space="preserve">#186 · 10-19 17:xx 조건별(8123): ③ 전력 부족 = 에너지 둘 지움 → 「⚠ 전력 부족 — 수요가 공급을 넘었다」 · 되놓음 → 사라짐 ✓ / ⑤ 고철 부족 = 변환기 연속 설치(약 30) → 18 에서 「⚠ 고철 부족」 · 20 되자 사라짐 ✓ / ① 미연결 = 성립 안 함(런타임 GlobalCause 가 Power·Heat·None 만 냄 · Blocked·NoInput 은 진단에만) / ② 생산 정지 · ④ 마운트 빔 = 화면 미성립(S1 파밍 · 운반로 두 칸 끊고 약 2분 · 적 희소로 마운트 안 빔) / 조립 화면에서는 띠가 팔레트 밑에 깔려 안 보임(그리기 순서) — 전투 화면에서만 보임</t>
+          <t xml:space="preserve">#186 · 10-19 17:xx 조건별(8123): ③ 전력 부족 = 에너지 둘 지움 → 「⚠ 전력 부족 — 수요가 공급을 넘었다」 · 되놓음 → 사라짐 ✓ / ⑤ 고철 부족 = 변환기 연속 설치(약 30) → 18 에서 「⚠ 고철 부족」 · 20 되자 사라짐 ✓ / ① 미연결 = 성립 안 함(런타임 GlobalCause 가 Power·Heat·None 만 냄 · Blocked·NoInput 은 진단에만) / ② 생산 정지 · ④ 마운트 빔 = 화면 미성립(S1 파밍 · 운반로 두 칸 끊고 약 2분 · 적 희소로 마운트 안 빔) / 조립 화면에서는 띠가 팔레트 밑에 깔려 안 보임(그리기 순서) — 전투 화면에서만 보임 · 10-19 #187 확인 중 ② 생산 정지 · ④ 마운트 빔도 화면 성립 — 「처음부터」 직후 튜토리얼 판(고스트 빈 칸)에서 「생산 정지 … 외 1건」 · 고스트 채우면 사라짐</t>
         </is>
       </c>
       <c r="G191" s="7"/>
@@ -13266,6 +13460,77 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AJ191" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_184</t>
+        </is>
+      </c>
+      <c r="B192" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C192" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">탄약 소진 아이콘</t>
+        </is>
+      </c>
+      <c r="D192" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">머리 위</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t xml:space="preserve">싸우는 로봇 마운트가 비면 주황 탄약 소진 아이콘(「물류 마크」)이 로봇 머리 위에 뜨고 HP · 쉴드 막대 · 회피 눈금과 겹치지 않으며, 재공급되면 사라지는가?</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#187 · 틈 0.1 ⚠️ 가정</t>
+        </is>
+      </c>
+      <c r="G192" s="7"/>
+      <c r="H192" s="7"/>
+      <c r="I192" s="7"/>
+      <c r="J192" s="7"/>
+      <c r="K192" s="7"/>
+      <c r="L192" s="7"/>
+      <c r="M192" s="7"/>
+      <c r="N192" s="7"/>
+      <c r="O192" s="7"/>
+      <c r="P192" s="7"/>
+      <c r="Q192" s="7"/>
+      <c r="R192" s="7"/>
+      <c r="S192" s="7"/>
+      <c r="T192" s="7"/>
+      <c r="U192" s="7"/>
+      <c r="V192" s="7"/>
+      <c r="W192" s="7"/>
+      <c r="X192" s="7"/>
+      <c r="Y192" s="7"/>
+      <c r="Z192" s="7"/>
+      <c r="AA192" s="7"/>
+      <c r="AB192" s="7"/>
+      <c r="AC192" s="7"/>
+      <c r="AD192" s="7"/>
+      <c r="AE192" s="7"/>
+      <c r="AF192" s="7"/>
+      <c r="AG192" s="7"/>
+      <c r="AH192" s="7"/>
+      <c r="AI192" s="7"/>
+      <c r="AJ192" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="26">
@@ -13294,9 +13559,9 @@
     <mergeCell ref="B92:B99"/>
     <mergeCell ref="B100:B106"/>
     <mergeCell ref="B107:B111"/>
-    <mergeCell ref="G7:AI7"/>
+    <mergeCell ref="G7:AJ7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:AI191">
+  <conditionalFormatting sqref="G9:AJ192">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
docs: QA AK열(cae560d · CID_185~194) · 촬영 가이드 8133 후보(#188~#196 · 컷 영향)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -192,8 +192,9 @@
     <col min="34" max="34" width="12" customWidth="1"/>
     <col min="35" max="35" width="12" customWidth="1"/>
     <col min="36" max="36" width="12" customWidth="1"/>
-    <col min="37" max="37" width="11" customWidth="1"/>
+    <col min="37" max="37" width="12" customWidth="1"/>
     <col min="38" max="38" width="11" customWidth="1"/>
+    <col min="39" max="39" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -456,6 +457,11 @@
       <c r="AJ6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">video-261019d 후보(8133 · 새 사본 · 8132 동결) · #187 탄약 소진 아이콘 머리 위 ‖ 10-19 코드 세션 재확인(8123 · 캔버스 캡처): 「처음부터」 → 튜토리얼 판(마운트 0/40 · 고스트 빈 칸) = 주황 「물류 마크」가 로봇 머리 위 · HP · 쉴드 막대 · 회피 눈금과 겹침 0 · 같은 화면에 띠 「⚠ 생산 정지 — 만드는 것이 없다 외 1건」(② · ④) → 조립에서 고스트 채움(조립 화면 위 전투 인셋에도 머리 위) → 30초 뒤 마운트 차오름 = 아이콘 · 띠 사라짐 · ⚠️ 로봇 B · 합체 몸은 화면 미확인(몸 윗변을 그려진 사각에서 읽는 같은 길) · 576×1024 · 1024×768 창 미확인(인앱 프레임 하나) · 8133 복사 17:37:00 · CID_184 새 항목)</t>
+        </is>
+      </c>
+      <c r="AK6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">video-261019d 후보 갈아엎음(8133 · 19:00:23) · #188~#196(플랜 §98-47) ‖ 10-19 코드 세션 재확인(8123 · 인앱 · 새 저장 「처음부터」 자연 진행): S1 승리 = 「강화 재료 +30」 · [스테이지로][다음 스테이지로](다시 도전 없음) → 스테이지로 = 「통과함」 흐림 → S2 T4 → 승리 +33 → S3 파밍 주제 「마운트 강화」 · 막 「조립에서 마운트를 탭해 강화해보세요」 → 보드 시야 A 마운트 · 안내 → 팝오버 「강화 재료 63/50」 → 강화 = 13/50 → ⚠️ S3 파밍 강화 뒤에도 약 35초에 파괴(HP 970 → 100/30초) → S2 로 밀림 · S3 도전 승리 +37 → S4 해금 → (페이지 새로고침 뒤) S4 도전 = 합체 막 「합체 버튼을 눌러 합체해보세요」 → 합체 = 막 해제 → S4 승리(보상 줄 없음) → S5 알림 「복합 가공소가 열렸습니다」 · 주제 「폭발탄」 · 막 → A 판 ① 안내 · 변환기 조합표 발전재료 선택 ✓ → S5 파밍 파괴로 S4 로 밀려 ②~⑤ 화면 미확인 · #192 BGM(소리 0) · #195 B 강화(S6 미도달) 화면 미확인 = 시험이 든다 · ⚠️ 새로고침 뒤 HUD 전투력 0(8132 동결 빌드도 같음 · 기존) · CID_185~194 새 항목)</t>
         </is>
       </c>
     </row>
@@ -516,14 +522,15 @@
       <c r="AH7" s="2"/>
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
-      <c r="AK7" s="2" t="inlineStr">
+      <c r="AK7" s="2"/>
+      <c r="AL7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">버전</t>
         </is>
       </c>
-      <c r="AL7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">caf9133</t>
+      <c r="AM7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cae560d</t>
         </is>
       </c>
     </row>
@@ -698,11 +705,16 @@
       </c>
       <c r="AK8" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">cae560d</t>
+        </is>
+      </c>
+      <c r="AL8" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">PASSrate</t>
         </is>
       </c>
-      <c r="AL8" s="7">
-        <f>COUNTIF(AJ9:AJ192,"Pass")</f>
+      <c r="AM8" s="7">
+        <f>COUNTIF(AK9:AK202,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -802,13 +814,14 @@
       <c r="AH9" s="7"/>
       <c r="AI9" s="7"/>
       <c r="AJ9" s="7"/>
-      <c r="AK9" s="2" t="inlineStr">
+      <c r="AK9" s="7"/>
+      <c r="AL9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FAILrate</t>
         </is>
       </c>
-      <c r="AL9" s="7">
-        <f>COUNTIF(AJ9:AJ192,"Fail")+COUNTIF(AJ9:AJ192,"Broken")</f>
+      <c r="AM9" s="7">
+        <f>COUNTIF(AK9:AK202,"Fail")+COUNTIF(AK9:AK202,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -872,13 +885,14 @@
       <c r="AH10" s="7"/>
       <c r="AI10" s="7"/>
       <c r="AJ10" s="7"/>
-      <c r="AK10" s="2" t="inlineStr">
+      <c r="AK10" s="7"/>
+      <c r="AL10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">N/A</t>
         </is>
       </c>
-      <c r="AL10" s="7">
-        <f>COUNTIF(AJ9:AJ192,"N/A")</f>
+      <c r="AM10" s="7">
+        <f>COUNTIF(AK9:AK202,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -942,13 +956,14 @@
       <c r="AH11" s="7"/>
       <c r="AI11" s="7"/>
       <c r="AJ11" s="7"/>
-      <c r="AK11" s="2" t="inlineStr">
+      <c r="AK11" s="7"/>
+      <c r="AL11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">전체 개수</t>
         </is>
       </c>
-      <c r="AL11" s="7">
-        <v>184</v>
+      <c r="AM11" s="7">
+        <v>194</v>
       </c>
     </row>
     <row r="12">
@@ -1012,13 +1027,14 @@
       <c r="AH12" s="7"/>
       <c r="AI12" s="7"/>
       <c r="AJ12" s="7"/>
-      <c r="AK12" s="2" t="inlineStr">
+      <c r="AK12" s="7"/>
+      <c r="AL12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">진행율</t>
         </is>
       </c>
-      <c r="AL12" s="7">
-        <f>TEXT((COUNTA(AJ9:AJ192))/184,"0.00%")</f>
+      <c r="AM12" s="7">
+        <f>TEXT((COUNTA(AK9:AK202))/194,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -1086,6 +1102,7 @@
       <c r="AH13" s="7"/>
       <c r="AI13" s="7"/>
       <c r="AJ13" s="7"/>
+      <c r="AK13" s="7"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -1143,6 +1160,7 @@
       <c r="AH14" s="7"/>
       <c r="AI14" s="7"/>
       <c r="AJ14" s="7"/>
+      <c r="AK14" s="7"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -1236,6 +1254,7 @@
       <c r="AH15" s="7"/>
       <c r="AI15" s="7"/>
       <c r="AJ15" s="7"/>
+      <c r="AK15" s="7"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -1329,6 +1348,7 @@
       <c r="AH16" s="7"/>
       <c r="AI16" s="7"/>
       <c r="AJ16" s="7"/>
+      <c r="AK16" s="7"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -1427,6 +1447,7 @@
       <c r="AH17" s="7"/>
       <c r="AI17" s="7"/>
       <c r="AJ17" s="7"/>
+      <c r="AK17" s="7"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -1489,6 +1510,7 @@
       <c r="AH18" s="7"/>
       <c r="AI18" s="7"/>
       <c r="AJ18" s="7"/>
+      <c r="AK18" s="7"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -1546,6 +1568,7 @@
       <c r="AH19" s="7"/>
       <c r="AI19" s="7"/>
       <c r="AJ19" s="7"/>
+      <c r="AK19" s="7"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1603,6 +1626,7 @@
       <c r="AH20" s="7"/>
       <c r="AI20" s="7"/>
       <c r="AJ20" s="7"/>
+      <c r="AK20" s="7"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1696,6 +1720,7 @@
       <c r="AH21" s="7"/>
       <c r="AI21" s="7"/>
       <c r="AJ21" s="7"/>
+      <c r="AK21" s="7"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1782,6 +1807,7 @@
       <c r="AH22" s="7"/>
       <c r="AI22" s="7"/>
       <c r="AJ22" s="7"/>
+      <c r="AK22" s="7"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -1847,6 +1873,7 @@
       <c r="AH23" s="7"/>
       <c r="AI23" s="7"/>
       <c r="AJ23" s="7"/>
+      <c r="AK23" s="7"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -1904,6 +1931,7 @@
       <c r="AH24" s="7"/>
       <c r="AI24" s="7"/>
       <c r="AJ24" s="7"/>
+      <c r="AK24" s="7"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -1961,6 +1989,7 @@
       <c r="AH25" s="7"/>
       <c r="AI25" s="7"/>
       <c r="AJ25" s="7"/>
+      <c r="AK25" s="7"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -2047,6 +2076,7 @@
       <c r="AH26" s="7"/>
       <c r="AI26" s="7"/>
       <c r="AJ26" s="7"/>
+      <c r="AK26" s="7"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -2108,6 +2138,7 @@
       <c r="AH27" s="7"/>
       <c r="AI27" s="7"/>
       <c r="AJ27" s="7"/>
+      <c r="AK27" s="7"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -2178,6 +2209,7 @@
       <c r="AH28" s="7"/>
       <c r="AI28" s="7"/>
       <c r="AJ28" s="7"/>
+      <c r="AK28" s="7"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -2243,6 +2275,7 @@
       <c r="AH29" s="7"/>
       <c r="AI29" s="7"/>
       <c r="AJ29" s="7"/>
+      <c r="AK29" s="7"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -2332,6 +2365,7 @@
       <c r="AH30" s="7"/>
       <c r="AI30" s="7"/>
       <c r="AJ30" s="7"/>
+      <c r="AK30" s="7"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -2426,6 +2460,7 @@
       <c r="AH31" s="7"/>
       <c r="AI31" s="7"/>
       <c r="AJ31" s="7"/>
+      <c r="AK31" s="7"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -2507,6 +2542,7 @@
       <c r="AH32" s="7"/>
       <c r="AI32" s="7"/>
       <c r="AJ32" s="7"/>
+      <c r="AK32" s="7"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -2596,6 +2632,7 @@
       <c r="AH33" s="7"/>
       <c r="AI33" s="7"/>
       <c r="AJ33" s="7"/>
+      <c r="AK33" s="7"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -2685,6 +2722,7 @@
       <c r="AH34" s="7"/>
       <c r="AI34" s="7"/>
       <c r="AJ34" s="7"/>
+      <c r="AK34" s="7"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -2783,6 +2821,7 @@
       <c r="AH35" s="7"/>
       <c r="AI35" s="7"/>
       <c r="AJ35" s="7"/>
+      <c r="AK35" s="7"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -2856,6 +2895,7 @@
       <c r="AH36" s="7"/>
       <c r="AI36" s="7"/>
       <c r="AJ36" s="7"/>
+      <c r="AK36" s="7"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -2913,6 +2953,7 @@
       <c r="AH37" s="7"/>
       <c r="AI37" s="7"/>
       <c r="AJ37" s="7"/>
+      <c r="AK37" s="7"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -2991,6 +3032,7 @@
       <c r="AH38" s="7"/>
       <c r="AI38" s="7"/>
       <c r="AJ38" s="7"/>
+      <c r="AK38" s="7"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -3080,6 +3122,7 @@
       <c r="AH39" s="7"/>
       <c r="AI39" s="7"/>
       <c r="AJ39" s="7"/>
+      <c r="AK39" s="7"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -3170,6 +3213,7 @@
       <c r="AH40" s="7"/>
       <c r="AI40" s="7"/>
       <c r="AJ40" s="7"/>
+      <c r="AK40" s="7"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -3255,6 +3299,7 @@
       <c r="AH41" s="7"/>
       <c r="AI41" s="7"/>
       <c r="AJ41" s="7"/>
+      <c r="AK41" s="7"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -3324,6 +3369,7 @@
       <c r="AH42" s="7"/>
       <c r="AI42" s="7"/>
       <c r="AJ42" s="7"/>
+      <c r="AK42" s="7"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -3413,6 +3459,7 @@
       <c r="AH43" s="7"/>
       <c r="AI43" s="7"/>
       <c r="AJ43" s="7"/>
+      <c r="AK43" s="7"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -3475,6 +3522,7 @@
       <c r="AH44" s="7"/>
       <c r="AI44" s="7"/>
       <c r="AJ44" s="7"/>
+      <c r="AK44" s="7"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -3560,6 +3608,7 @@
       <c r="AH45" s="7"/>
       <c r="AI45" s="7"/>
       <c r="AJ45" s="7"/>
+      <c r="AK45" s="7"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -3645,6 +3694,7 @@
       <c r="AH46" s="7"/>
       <c r="AI46" s="7"/>
       <c r="AJ46" s="7"/>
+      <c r="AK46" s="7"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -3707,6 +3757,7 @@
       <c r="AH47" s="7"/>
       <c r="AI47" s="7"/>
       <c r="AJ47" s="7"/>
+      <c r="AK47" s="7"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -3764,6 +3815,7 @@
       <c r="AH48" s="7"/>
       <c r="AI48" s="7"/>
       <c r="AJ48" s="7"/>
+      <c r="AK48" s="7"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -3821,6 +3873,7 @@
       <c r="AH49" s="7"/>
       <c r="AI49" s="7"/>
       <c r="AJ49" s="7"/>
+      <c r="AK49" s="7"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -3902,6 +3955,7 @@
       <c r="AH50" s="7"/>
       <c r="AI50" s="7"/>
       <c r="AJ50" s="7"/>
+      <c r="AK50" s="7"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -3983,6 +4037,7 @@
       <c r="AH51" s="7"/>
       <c r="AI51" s="7"/>
       <c r="AJ51" s="7"/>
+      <c r="AK51" s="7"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -4045,6 +4100,7 @@
       <c r="AH52" s="7"/>
       <c r="AI52" s="7"/>
       <c r="AJ52" s="7"/>
+      <c r="AK52" s="7"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -4107,6 +4163,7 @@
       <c r="AH53" s="7"/>
       <c r="AI53" s="7"/>
       <c r="AJ53" s="7"/>
+      <c r="AK53" s="7"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -4164,6 +4221,7 @@
       <c r="AH54" s="7"/>
       <c r="AI54" s="7"/>
       <c r="AJ54" s="7"/>
+      <c r="AK54" s="7"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -4257,6 +4315,7 @@
       <c r="AH55" s="7"/>
       <c r="AI55" s="7"/>
       <c r="AJ55" s="7"/>
+      <c r="AK55" s="7"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -4330,6 +4389,7 @@
       <c r="AH56" s="7"/>
       <c r="AI56" s="7"/>
       <c r="AJ56" s="7"/>
+      <c r="AK56" s="7"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -4412,6 +4472,7 @@
       <c r="AH57" s="7"/>
       <c r="AI57" s="7"/>
       <c r="AJ57" s="7"/>
+      <c r="AK57" s="7"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -4502,6 +4563,7 @@
       <c r="AH58" s="7"/>
       <c r="AI58" s="7"/>
       <c r="AJ58" s="7"/>
+      <c r="AK58" s="7"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -4559,6 +4621,7 @@
       <c r="AH59" s="7"/>
       <c r="AI59" s="7"/>
       <c r="AJ59" s="7"/>
+      <c r="AK59" s="7"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -4616,6 +4679,7 @@
       <c r="AH60" s="7"/>
       <c r="AI60" s="7"/>
       <c r="AJ60" s="7"/>
+      <c r="AK60" s="7"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -4685,6 +4749,7 @@
       <c r="AH61" s="7"/>
       <c r="AI61" s="7"/>
       <c r="AJ61" s="7"/>
+      <c r="AK61" s="7"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -4762,6 +4827,7 @@
       <c r="AH62" s="7"/>
       <c r="AI62" s="7"/>
       <c r="AJ62" s="7"/>
+      <c r="AK62" s="7"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -4831,6 +4897,7 @@
       <c r="AH63" s="7"/>
       <c r="AI63" s="7"/>
       <c r="AJ63" s="7"/>
+      <c r="AK63" s="7"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -4888,6 +4955,7 @@
       <c r="AH64" s="7"/>
       <c r="AI64" s="7"/>
       <c r="AJ64" s="7"/>
+      <c r="AK64" s="7"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -4950,6 +5018,7 @@
       <c r="AH65" s="7"/>
       <c r="AI65" s="7"/>
       <c r="AJ65" s="7"/>
+      <c r="AK65" s="7"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
@@ -5019,6 +5088,7 @@
       <c r="AH66" s="7"/>
       <c r="AI66" s="7"/>
       <c r="AJ66" s="7"/>
+      <c r="AK66" s="7"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -5076,6 +5146,7 @@
       <c r="AH67" s="7"/>
       <c r="AI67" s="7"/>
       <c r="AJ67" s="7"/>
+      <c r="AK67" s="7"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
@@ -5137,6 +5208,7 @@
       <c r="AH68" s="7"/>
       <c r="AI68" s="7"/>
       <c r="AJ68" s="7"/>
+      <c r="AK68" s="7"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -5230,6 +5302,7 @@
       <c r="AH69" s="7"/>
       <c r="AI69" s="7"/>
       <c r="AJ69" s="7"/>
+      <c r="AK69" s="7"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
@@ -5287,6 +5360,7 @@
       <c r="AH70" s="7"/>
       <c r="AI70" s="7"/>
       <c r="AJ70" s="7"/>
+      <c r="AK70" s="7"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -5349,6 +5423,7 @@
       <c r="AH71" s="7"/>
       <c r="AI71" s="7"/>
       <c r="AJ71" s="7"/>
+      <c r="AK71" s="7"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
@@ -5422,6 +5497,7 @@
       <c r="AH72" s="7"/>
       <c r="AI72" s="7"/>
       <c r="AJ72" s="7"/>
+      <c r="AK72" s="7"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
@@ -5484,6 +5560,7 @@
       <c r="AH73" s="7"/>
       <c r="AI73" s="7"/>
       <c r="AJ73" s="7"/>
+      <c r="AK73" s="7"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -5541,6 +5618,7 @@
       <c r="AH74" s="7"/>
       <c r="AI74" s="7"/>
       <c r="AJ74" s="7"/>
+      <c r="AK74" s="7"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -5598,6 +5676,7 @@
       <c r="AH75" s="7"/>
       <c r="AI75" s="7"/>
       <c r="AJ75" s="7"/>
+      <c r="AK75" s="7"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -5655,6 +5734,7 @@
       <c r="AH76" s="7"/>
       <c r="AI76" s="7"/>
       <c r="AJ76" s="7"/>
+      <c r="AK76" s="7"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -5716,6 +5796,7 @@
       <c r="AH77" s="7"/>
       <c r="AI77" s="7"/>
       <c r="AJ77" s="7"/>
+      <c r="AK77" s="7"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
@@ -5773,6 +5854,7 @@
       <c r="AH78" s="7"/>
       <c r="AI78" s="7"/>
       <c r="AJ78" s="7"/>
+      <c r="AK78" s="7"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -5835,6 +5917,7 @@
       <c r="AH79" s="7"/>
       <c r="AI79" s="7"/>
       <c r="AJ79" s="7"/>
+      <c r="AK79" s="7"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
@@ -5908,6 +5991,7 @@
       <c r="AH80" s="7"/>
       <c r="AI80" s="7"/>
       <c r="AJ80" s="7"/>
+      <c r="AK80" s="7"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
@@ -5969,6 +6053,7 @@
       <c r="AH81" s="7"/>
       <c r="AI81" s="7"/>
       <c r="AJ81" s="7"/>
+      <c r="AK81" s="7"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
@@ -6026,6 +6111,7 @@
       <c r="AH82" s="7"/>
       <c r="AI82" s="7"/>
       <c r="AJ82" s="7"/>
+      <c r="AK82" s="7"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
@@ -6088,6 +6174,7 @@
       <c r="AH83" s="7"/>
       <c r="AI83" s="7"/>
       <c r="AJ83" s="7"/>
+      <c r="AK83" s="7"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
@@ -6145,6 +6232,7 @@
       <c r="AH84" s="7"/>
       <c r="AI84" s="7"/>
       <c r="AJ84" s="7"/>
+      <c r="AK84" s="7"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
@@ -6202,6 +6290,7 @@
       <c r="AH85" s="7"/>
       <c r="AI85" s="7"/>
       <c r="AJ85" s="7"/>
+      <c r="AK85" s="7"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
@@ -6264,6 +6353,7 @@
       <c r="AH86" s="7"/>
       <c r="AI86" s="7"/>
       <c r="AJ86" s="7"/>
+      <c r="AK86" s="7"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
@@ -6321,6 +6411,7 @@
       <c r="AH87" s="7"/>
       <c r="AI87" s="7"/>
       <c r="AJ87" s="7"/>
+      <c r="AK87" s="7"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
@@ -6378,6 +6469,7 @@
       <c r="AH88" s="7"/>
       <c r="AI88" s="7"/>
       <c r="AJ88" s="7"/>
+      <c r="AK88" s="7"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
@@ -6435,6 +6527,7 @@
       <c r="AH89" s="7"/>
       <c r="AI89" s="7"/>
       <c r="AJ89" s="7"/>
+      <c r="AK89" s="7"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
@@ -6521,6 +6614,7 @@
       <c r="AH90" s="7"/>
       <c r="AI90" s="7"/>
       <c r="AJ90" s="7"/>
+      <c r="AK90" s="7"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
@@ -6578,6 +6672,7 @@
       <c r="AH91" s="7"/>
       <c r="AI91" s="7"/>
       <c r="AJ91" s="7"/>
+      <c r="AK91" s="7"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
@@ -6671,6 +6766,7 @@
       <c r="AH92" s="7"/>
       <c r="AI92" s="7"/>
       <c r="AJ92" s="7"/>
+      <c r="AK92" s="7"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
@@ -6769,6 +6865,7 @@
       <c r="AH93" s="7"/>
       <c r="AI93" s="7"/>
       <c r="AJ93" s="7"/>
+      <c r="AK93" s="7"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
@@ -6831,6 +6928,7 @@
       <c r="AH94" s="7"/>
       <c r="AI94" s="7"/>
       <c r="AJ94" s="7"/>
+      <c r="AK94" s="7"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
@@ -6893,6 +6991,7 @@
       <c r="AH95" s="7"/>
       <c r="AI95" s="7"/>
       <c r="AJ95" s="7"/>
+      <c r="AK95" s="7"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
@@ -6974,6 +7073,7 @@
       <c r="AH96" s="7"/>
       <c r="AI96" s="7"/>
       <c r="AJ96" s="7"/>
+      <c r="AK96" s="7"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="inlineStr">
@@ -7031,6 +7131,7 @@
       <c r="AH97" s="7"/>
       <c r="AI97" s="7"/>
       <c r="AJ97" s="7"/>
+      <c r="AK97" s="7"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
@@ -7088,6 +7189,7 @@
       <c r="AH98" s="7"/>
       <c r="AI98" s="7"/>
       <c r="AJ98" s="7"/>
+      <c r="AK98" s="7"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
@@ -7145,6 +7247,7 @@
       <c r="AH99" s="7"/>
       <c r="AI99" s="7"/>
       <c r="AJ99" s="7"/>
+      <c r="AK99" s="7"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
@@ -7211,6 +7314,7 @@
       <c r="AH100" s="7"/>
       <c r="AI100" s="7"/>
       <c r="AJ100" s="7"/>
+      <c r="AK100" s="7"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
@@ -7268,6 +7372,7 @@
       <c r="AH101" s="7"/>
       <c r="AI101" s="7"/>
       <c r="AJ101" s="7"/>
+      <c r="AK101" s="7"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
@@ -7325,6 +7430,7 @@
       <c r="AH102" s="7"/>
       <c r="AI102" s="7"/>
       <c r="AJ102" s="7"/>
+      <c r="AK102" s="7"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="inlineStr">
@@ -7382,6 +7488,7 @@
       <c r="AH103" s="7"/>
       <c r="AI103" s="7"/>
       <c r="AJ103" s="7"/>
+      <c r="AK103" s="7"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="inlineStr">
@@ -7444,6 +7551,7 @@
       <c r="AH104" s="7"/>
       <c r="AI104" s="7"/>
       <c r="AJ104" s="7"/>
+      <c r="AK104" s="7"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
@@ -7501,6 +7609,7 @@
       <c r="AH105" s="7"/>
       <c r="AI105" s="7"/>
       <c r="AJ105" s="7"/>
+      <c r="AK105" s="7"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
@@ -7558,6 +7667,7 @@
       <c r="AH106" s="7"/>
       <c r="AI106" s="7"/>
       <c r="AJ106" s="7"/>
+      <c r="AK106" s="7"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
@@ -7615,6 +7725,7 @@
       <c r="AH107" s="7"/>
       <c r="AI107" s="7"/>
       <c r="AJ107" s="7"/>
+      <c r="AK107" s="7"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
@@ -7676,6 +7787,7 @@
       <c r="AH108" s="7"/>
       <c r="AI108" s="7"/>
       <c r="AJ108" s="7"/>
+      <c r="AK108" s="7"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="inlineStr">
@@ -7742,6 +7854,7 @@
       <c r="AH109" s="7"/>
       <c r="AI109" s="7"/>
       <c r="AJ109" s="7"/>
+      <c r="AK109" s="7"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
@@ -7816,6 +7929,7 @@
       <c r="AH110" s="7"/>
       <c r="AI110" s="7"/>
       <c r="AJ110" s="7"/>
+      <c r="AK110" s="7"/>
     </row>
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
@@ -7893,6 +8007,7 @@
       <c r="AH111" s="7"/>
       <c r="AI111" s="7"/>
       <c r="AJ111" s="7"/>
+      <c r="AK111" s="7"/>
     </row>
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
@@ -7967,6 +8082,7 @@
       <c r="AH112" s="7"/>
       <c r="AI112" s="7"/>
       <c r="AJ112" s="7"/>
+      <c r="AK112" s="7"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
@@ -8033,6 +8149,7 @@
       <c r="AH113" s="7"/>
       <c r="AI113" s="7"/>
       <c r="AJ113" s="7"/>
+      <c r="AK113" s="7"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="inlineStr">
@@ -8115,6 +8232,7 @@
       <c r="AH114" s="7"/>
       <c r="AI114" s="7"/>
       <c r="AJ114" s="7"/>
+      <c r="AK114" s="7"/>
     </row>
     <row r="115">
       <c r="A115" s="7" t="inlineStr">
@@ -8189,6 +8307,7 @@
       <c r="AH115" s="7"/>
       <c r="AI115" s="7"/>
       <c r="AJ115" s="7"/>
+      <c r="AK115" s="7"/>
     </row>
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
@@ -8271,6 +8390,7 @@
       </c>
       <c r="AI116" s="7"/>
       <c r="AJ116" s="7"/>
+      <c r="AK116" s="7"/>
     </row>
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
@@ -8349,6 +8469,7 @@
       <c r="AH117" s="7"/>
       <c r="AI117" s="7"/>
       <c r="AJ117" s="7"/>
+      <c r="AK117" s="7"/>
     </row>
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
@@ -8427,6 +8548,7 @@
       <c r="AH118" s="7"/>
       <c r="AI118" s="7"/>
       <c r="AJ118" s="7"/>
+      <c r="AK118" s="7"/>
     </row>
     <row r="119">
       <c r="A119" s="7" t="inlineStr">
@@ -8501,6 +8623,7 @@
       <c r="AH119" s="7"/>
       <c r="AI119" s="7"/>
       <c r="AJ119" s="7"/>
+      <c r="AK119" s="7"/>
     </row>
     <row r="120">
       <c r="A120" s="7" t="inlineStr">
@@ -8567,6 +8690,7 @@
       <c r="AH120" s="7"/>
       <c r="AI120" s="7"/>
       <c r="AJ120" s="7"/>
+      <c r="AK120" s="7"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="inlineStr">
@@ -8645,6 +8769,7 @@
       <c r="AH121" s="7"/>
       <c r="AI121" s="7"/>
       <c r="AJ121" s="7"/>
+      <c r="AK121" s="7"/>
     </row>
     <row r="122">
       <c r="A122" s="7" t="inlineStr">
@@ -8723,6 +8848,7 @@
       <c r="AH122" s="7"/>
       <c r="AI122" s="7"/>
       <c r="AJ122" s="7"/>
+      <c r="AK122" s="7"/>
     </row>
     <row r="123">
       <c r="A123" s="7" t="inlineStr">
@@ -8789,6 +8915,7 @@
       <c r="AH123" s="7"/>
       <c r="AI123" s="7"/>
       <c r="AJ123" s="7"/>
+      <c r="AK123" s="7"/>
     </row>
     <row r="124">
       <c r="A124" s="7" t="inlineStr">
@@ -8863,6 +8990,7 @@
       <c r="AH124" s="7"/>
       <c r="AI124" s="7"/>
       <c r="AJ124" s="7"/>
+      <c r="AK124" s="7"/>
     </row>
     <row r="125">
       <c r="A125" s="7" t="inlineStr">
@@ -8929,6 +9057,7 @@
       <c r="AH125" s="7"/>
       <c r="AI125" s="7"/>
       <c r="AJ125" s="7"/>
+      <c r="AK125" s="7"/>
     </row>
     <row r="126">
       <c r="A126" s="7" t="inlineStr">
@@ -8995,6 +9124,7 @@
       <c r="AH126" s="7"/>
       <c r="AI126" s="7"/>
       <c r="AJ126" s="7"/>
+      <c r="AK126" s="7"/>
     </row>
     <row r="127">
       <c r="A127" s="7" t="inlineStr">
@@ -9065,6 +9195,7 @@
       <c r="AH127" s="7"/>
       <c r="AI127" s="7"/>
       <c r="AJ127" s="7"/>
+      <c r="AK127" s="7"/>
     </row>
     <row r="128">
       <c r="A128" s="7" t="inlineStr">
@@ -9135,6 +9266,7 @@
       <c r="AH128" s="7"/>
       <c r="AI128" s="7"/>
       <c r="AJ128" s="7"/>
+      <c r="AK128" s="7"/>
     </row>
     <row r="129">
       <c r="A129" s="7" t="inlineStr">
@@ -9205,6 +9337,7 @@
       <c r="AH129" s="7"/>
       <c r="AI129" s="7"/>
       <c r="AJ129" s="7"/>
+      <c r="AK129" s="7"/>
     </row>
     <row r="130">
       <c r="A130" s="7" t="inlineStr">
@@ -9271,6 +9404,7 @@
       <c r="AH130" s="7"/>
       <c r="AI130" s="7"/>
       <c r="AJ130" s="7"/>
+      <c r="AK130" s="7"/>
     </row>
     <row r="131">
       <c r="A131" s="7" t="inlineStr">
@@ -9345,6 +9479,7 @@
       <c r="AH131" s="7"/>
       <c r="AI131" s="7"/>
       <c r="AJ131" s="7"/>
+      <c r="AK131" s="7"/>
     </row>
     <row r="132">
       <c r="A132" s="7" t="inlineStr">
@@ -9423,6 +9558,7 @@
       <c r="AH132" s="7"/>
       <c r="AI132" s="7"/>
       <c r="AJ132" s="7"/>
+      <c r="AK132" s="7"/>
     </row>
     <row r="133">
       <c r="A133" s="7" t="inlineStr">
@@ -9501,6 +9637,7 @@
       <c r="AH133" s="7"/>
       <c r="AI133" s="7"/>
       <c r="AJ133" s="7"/>
+      <c r="AK133" s="7"/>
     </row>
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
@@ -9575,6 +9712,7 @@
       <c r="AH134" s="7"/>
       <c r="AI134" s="7"/>
       <c r="AJ134" s="7"/>
+      <c r="AK134" s="7"/>
     </row>
     <row r="135">
       <c r="A135" s="7" t="inlineStr">
@@ -9649,6 +9787,7 @@
       <c r="AH135" s="7"/>
       <c r="AI135" s="7"/>
       <c r="AJ135" s="7"/>
+      <c r="AK135" s="7"/>
     </row>
     <row r="136">
       <c r="A136" s="7" t="inlineStr">
@@ -9723,6 +9862,7 @@
       <c r="AH136" s="7"/>
       <c r="AI136" s="7"/>
       <c r="AJ136" s="7"/>
+      <c r="AK136" s="7"/>
     </row>
     <row r="137">
       <c r="A137" s="7" t="inlineStr">
@@ -9793,6 +9933,7 @@
       <c r="AH137" s="7"/>
       <c r="AI137" s="7"/>
       <c r="AJ137" s="7"/>
+      <c r="AK137" s="7"/>
     </row>
     <row r="138">
       <c r="A138" s="7" t="inlineStr">
@@ -9863,6 +10004,7 @@
       <c r="AH138" s="7"/>
       <c r="AI138" s="7"/>
       <c r="AJ138" s="7"/>
+      <c r="AK138" s="7"/>
     </row>
     <row r="139">
       <c r="A139" s="7" t="inlineStr">
@@ -9933,6 +10075,7 @@
       <c r="AH139" s="7"/>
       <c r="AI139" s="7"/>
       <c r="AJ139" s="7"/>
+      <c r="AK139" s="7"/>
     </row>
     <row r="140">
       <c r="A140" s="7" t="inlineStr">
@@ -9999,6 +10142,7 @@
       <c r="AH140" s="7"/>
       <c r="AI140" s="7"/>
       <c r="AJ140" s="7"/>
+      <c r="AK140" s="7"/>
     </row>
     <row r="141">
       <c r="A141" s="7" t="inlineStr">
@@ -10077,6 +10221,7 @@
       <c r="AH141" s="7"/>
       <c r="AI141" s="7"/>
       <c r="AJ141" s="7"/>
+      <c r="AK141" s="7"/>
     </row>
     <row r="142">
       <c r="A142" s="7" t="inlineStr">
@@ -10143,6 +10288,7 @@
       <c r="AH142" s="7"/>
       <c r="AI142" s="7"/>
       <c r="AJ142" s="7"/>
+      <c r="AK142" s="7"/>
     </row>
     <row r="143">
       <c r="A143" s="7" t="inlineStr">
@@ -10209,6 +10355,7 @@
       <c r="AH143" s="7"/>
       <c r="AI143" s="7"/>
       <c r="AJ143" s="7"/>
+      <c r="AK143" s="7"/>
     </row>
     <row r="144">
       <c r="A144" s="7" t="inlineStr">
@@ -10275,6 +10422,7 @@
       <c r="AH144" s="7"/>
       <c r="AI144" s="7"/>
       <c r="AJ144" s="7"/>
+      <c r="AK144" s="7"/>
     </row>
     <row r="145">
       <c r="A145" s="7" t="inlineStr">
@@ -10357,6 +10505,7 @@
       <c r="AH145" s="7"/>
       <c r="AI145" s="7"/>
       <c r="AJ145" s="7"/>
+      <c r="AK145" s="7"/>
     </row>
     <row r="146">
       <c r="A146" s="7" t="inlineStr">
@@ -10427,6 +10576,7 @@
       <c r="AH146" s="7"/>
       <c r="AI146" s="7"/>
       <c r="AJ146" s="7"/>
+      <c r="AK146" s="7"/>
     </row>
     <row r="147">
       <c r="A147" s="7" t="inlineStr">
@@ -10509,6 +10659,7 @@
       <c r="AH147" s="7"/>
       <c r="AI147" s="7"/>
       <c r="AJ147" s="7"/>
+      <c r="AK147" s="7"/>
     </row>
     <row r="148">
       <c r="A148" s="7" t="inlineStr">
@@ -10575,6 +10726,7 @@
       <c r="AH148" s="7"/>
       <c r="AI148" s="7"/>
       <c r="AJ148" s="7"/>
+      <c r="AK148" s="7"/>
     </row>
     <row r="149">
       <c r="A149" s="7" t="inlineStr">
@@ -10649,6 +10801,7 @@
       <c r="AH149" s="7"/>
       <c r="AI149" s="7"/>
       <c r="AJ149" s="7"/>
+      <c r="AK149" s="7"/>
     </row>
     <row r="150">
       <c r="A150" s="7" t="inlineStr">
@@ -10727,6 +10880,7 @@
       <c r="AH150" s="7"/>
       <c r="AI150" s="7"/>
       <c r="AJ150" s="7"/>
+      <c r="AK150" s="7"/>
     </row>
     <row r="151">
       <c r="A151" s="7" t="inlineStr">
@@ -10797,6 +10951,7 @@
       <c r="AH151" s="7"/>
       <c r="AI151" s="7"/>
       <c r="AJ151" s="7"/>
+      <c r="AK151" s="7"/>
     </row>
     <row r="152">
       <c r="A152" s="7" t="inlineStr">
@@ -10871,6 +11026,7 @@
       <c r="AH152" s="7"/>
       <c r="AI152" s="7"/>
       <c r="AJ152" s="7"/>
+      <c r="AK152" s="7"/>
     </row>
     <row r="153">
       <c r="A153" s="7" t="inlineStr">
@@ -10945,6 +11101,7 @@
       <c r="AH153" s="7"/>
       <c r="AI153" s="7"/>
       <c r="AJ153" s="7"/>
+      <c r="AK153" s="7"/>
     </row>
     <row r="154">
       <c r="A154" s="7" t="inlineStr">
@@ -11007,6 +11164,7 @@
       <c r="AH154" s="7"/>
       <c r="AI154" s="7"/>
       <c r="AJ154" s="7"/>
+      <c r="AK154" s="7"/>
     </row>
     <row r="155">
       <c r="A155" s="7" t="inlineStr">
@@ -11073,6 +11231,7 @@
       <c r="AH155" s="7"/>
       <c r="AI155" s="7"/>
       <c r="AJ155" s="7"/>
+      <c r="AK155" s="7"/>
     </row>
     <row r="156">
       <c r="A156" s="7" t="inlineStr">
@@ -11143,6 +11302,7 @@
       <c r="AH156" s="7"/>
       <c r="AI156" s="7"/>
       <c r="AJ156" s="7"/>
+      <c r="AK156" s="7"/>
     </row>
     <row r="157">
       <c r="A157" s="7" t="inlineStr">
@@ -11209,6 +11369,7 @@
       <c r="AH157" s="7"/>
       <c r="AI157" s="7"/>
       <c r="AJ157" s="7"/>
+      <c r="AK157" s="7"/>
     </row>
     <row r="158">
       <c r="A158" s="7" t="inlineStr">
@@ -11275,6 +11436,7 @@
       <c r="AH158" s="7"/>
       <c r="AI158" s="7"/>
       <c r="AJ158" s="7"/>
+      <c r="AK158" s="7"/>
     </row>
     <row r="159">
       <c r="A159" s="7" t="inlineStr">
@@ -11341,6 +11503,7 @@
       <c r="AH159" s="7"/>
       <c r="AI159" s="7"/>
       <c r="AJ159" s="7"/>
+      <c r="AK159" s="7"/>
     </row>
     <row r="160">
       <c r="A160" s="7" t="inlineStr">
@@ -11407,6 +11570,7 @@
       <c r="AH160" s="7"/>
       <c r="AI160" s="7"/>
       <c r="AJ160" s="7"/>
+      <c r="AK160" s="7"/>
     </row>
     <row r="161">
       <c r="A161" s="7" t="inlineStr">
@@ -11477,6 +11641,7 @@
       <c r="AH161" s="7"/>
       <c r="AI161" s="7"/>
       <c r="AJ161" s="7"/>
+      <c r="AK161" s="7"/>
     </row>
     <row r="162">
       <c r="A162" s="7" t="inlineStr">
@@ -11543,6 +11708,7 @@
       <c r="AH162" s="7"/>
       <c r="AI162" s="7"/>
       <c r="AJ162" s="7"/>
+      <c r="AK162" s="7"/>
     </row>
     <row r="163">
       <c r="A163" s="7" t="inlineStr">
@@ -11609,6 +11775,7 @@
       <c r="AH163" s="7"/>
       <c r="AI163" s="7"/>
       <c r="AJ163" s="7"/>
+      <c r="AK163" s="7"/>
     </row>
     <row r="164">
       <c r="A164" s="7" t="inlineStr">
@@ -11675,6 +11842,7 @@
       <c r="AH164" s="7"/>
       <c r="AI164" s="7"/>
       <c r="AJ164" s="7"/>
+      <c r="AK164" s="7"/>
     </row>
     <row r="165">
       <c r="A165" s="7" t="inlineStr">
@@ -11741,6 +11909,7 @@
       <c r="AH165" s="7"/>
       <c r="AI165" s="7"/>
       <c r="AJ165" s="7"/>
+      <c r="AK165" s="7"/>
     </row>
     <row r="166">
       <c r="A166" s="7" t="inlineStr">
@@ -11811,6 +11980,7 @@
       <c r="AH166" s="7"/>
       <c r="AI166" s="7"/>
       <c r="AJ166" s="7"/>
+      <c r="AK166" s="7"/>
     </row>
     <row r="167">
       <c r="A167" s="7" t="inlineStr">
@@ -11877,6 +12047,7 @@
       <c r="AH167" s="7"/>
       <c r="AI167" s="7"/>
       <c r="AJ167" s="7"/>
+      <c r="AK167" s="7"/>
     </row>
     <row r="168">
       <c r="A168" s="7" t="inlineStr">
@@ -11943,6 +12114,7 @@
       <c r="AH168" s="7"/>
       <c r="AI168" s="7"/>
       <c r="AJ168" s="7"/>
+      <c r="AK168" s="7"/>
     </row>
     <row r="169">
       <c r="A169" s="7" t="inlineStr">
@@ -12009,6 +12181,7 @@
       <c r="AH169" s="7"/>
       <c r="AI169" s="7"/>
       <c r="AJ169" s="7"/>
+      <c r="AK169" s="7"/>
     </row>
     <row r="170">
       <c r="A170" s="7" t="inlineStr">
@@ -12079,6 +12252,7 @@
       <c r="AH170" s="7"/>
       <c r="AI170" s="7"/>
       <c r="AJ170" s="7"/>
+      <c r="AK170" s="7"/>
     </row>
     <row r="171">
       <c r="A171" s="7" t="inlineStr">
@@ -12141,6 +12315,7 @@
       <c r="AH171" s="7"/>
       <c r="AI171" s="7"/>
       <c r="AJ171" s="7"/>
+      <c r="AK171" s="7"/>
     </row>
     <row r="172">
       <c r="A172" s="7" t="inlineStr">
@@ -12203,6 +12378,7 @@
       <c r="AH172" s="7"/>
       <c r="AI172" s="7"/>
       <c r="AJ172" s="7"/>
+      <c r="AK172" s="7"/>
     </row>
     <row r="173">
       <c r="A173" s="7" t="inlineStr">
@@ -12273,6 +12449,7 @@
       <c r="AH173" s="7"/>
       <c r="AI173" s="7"/>
       <c r="AJ173" s="7"/>
+      <c r="AK173" s="7"/>
     </row>
     <row r="174">
       <c r="A174" s="7" t="inlineStr">
@@ -12339,6 +12516,7 @@
       <c r="AH174" s="7"/>
       <c r="AI174" s="7"/>
       <c r="AJ174" s="7"/>
+      <c r="AK174" s="7"/>
     </row>
     <row r="175">
       <c r="A175" s="7" t="inlineStr">
@@ -12409,6 +12587,7 @@
       <c r="AH175" s="7"/>
       <c r="AI175" s="7"/>
       <c r="AJ175" s="7"/>
+      <c r="AK175" s="7"/>
     </row>
     <row r="176">
       <c r="A176" s="7" t="inlineStr">
@@ -12475,6 +12654,7 @@
       <c r="AH176" s="7"/>
       <c r="AI176" s="7"/>
       <c r="AJ176" s="7"/>
+      <c r="AK176" s="7"/>
     </row>
     <row r="177">
       <c r="A177" s="7" t="inlineStr">
@@ -12541,6 +12721,7 @@
       <c r="AH177" s="7"/>
       <c r="AI177" s="7"/>
       <c r="AJ177" s="7"/>
+      <c r="AK177" s="7"/>
     </row>
     <row r="178">
       <c r="A178" s="7" t="inlineStr">
@@ -12607,6 +12788,7 @@
       <c r="AH178" s="7"/>
       <c r="AI178" s="7"/>
       <c r="AJ178" s="7"/>
+      <c r="AK178" s="7"/>
     </row>
     <row r="179">
       <c r="A179" s="7" t="inlineStr">
@@ -12673,6 +12855,7 @@
       <c r="AH179" s="7"/>
       <c r="AI179" s="7"/>
       <c r="AJ179" s="7"/>
+      <c r="AK179" s="7"/>
     </row>
     <row r="180">
       <c r="A180" s="7" t="inlineStr">
@@ -12739,6 +12922,7 @@
       <c r="AH180" s="7"/>
       <c r="AI180" s="7"/>
       <c r="AJ180" s="7"/>
+      <c r="AK180" s="7"/>
     </row>
     <row r="181">
       <c r="A181" s="7" t="inlineStr">
@@ -12805,6 +12989,7 @@
       <c r="AH181" s="7"/>
       <c r="AI181" s="7"/>
       <c r="AJ181" s="7"/>
+      <c r="AK181" s="7"/>
     </row>
     <row r="182">
       <c r="A182" s="7" t="inlineStr">
@@ -12871,6 +13056,7 @@
       <c r="AH182" s="7"/>
       <c r="AI182" s="7"/>
       <c r="AJ182" s="7"/>
+      <c r="AK182" s="7"/>
     </row>
     <row r="183">
       <c r="A183" s="7" t="inlineStr">
@@ -12900,7 +13086,7 @@
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t xml:space="preserve">#182 · 문구 ⚠️ 가정</t>
+          <t xml:space="preserve">#182 · 문구 ⚠️ 가정 · 10-19 #188 로 S3 파밍으로 옮김(CID_185)</t>
         </is>
       </c>
       <c r="G183" s="7"/>
@@ -12937,6 +13123,7 @@
       </c>
       <c r="AI183" s="7"/>
       <c r="AJ183" s="7"/>
+      <c r="AK183" s="7"/>
     </row>
     <row r="184">
       <c r="A184" s="7" t="inlineStr">
@@ -12999,6 +13186,7 @@
       <c r="AH184" s="7"/>
       <c r="AI184" s="7"/>
       <c r="AJ184" s="7"/>
+      <c r="AK184" s="7"/>
     </row>
     <row r="185">
       <c r="A185" s="7" t="inlineStr">
@@ -13065,6 +13253,7 @@
       </c>
       <c r="AI185" s="7"/>
       <c r="AJ185" s="7"/>
+      <c r="AK185" s="7"/>
     </row>
     <row r="186">
       <c r="A186" s="7" t="inlineStr">
@@ -13131,6 +13320,7 @@
       </c>
       <c r="AI186" s="7"/>
       <c r="AJ186" s="7"/>
+      <c r="AK186" s="7"/>
     </row>
     <row r="187">
       <c r="A187" s="7" t="inlineStr">
@@ -13197,6 +13387,7 @@
       </c>
       <c r="AI187" s="7"/>
       <c r="AJ187" s="7"/>
+      <c r="AK187" s="7"/>
     </row>
     <row r="188">
       <c r="A188" s="7" t="inlineStr">
@@ -13263,6 +13454,7 @@
       </c>
       <c r="AI188" s="7"/>
       <c r="AJ188" s="7"/>
+      <c r="AK188" s="7"/>
     </row>
     <row r="189">
       <c r="A189" s="7" t="inlineStr">
@@ -13329,6 +13521,7 @@
         </is>
       </c>
       <c r="AJ189" s="7"/>
+      <c r="AK189" s="7"/>
     </row>
     <row r="190">
       <c r="A190" s="7" t="inlineStr">
@@ -13395,6 +13588,7 @@
         </is>
       </c>
       <c r="AJ190" s="7"/>
+      <c r="AK190" s="7"/>
     </row>
     <row r="191">
       <c r="A191" s="7" t="inlineStr">
@@ -13465,6 +13659,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AK191" s="7"/>
     </row>
     <row r="192">
       <c r="A192" s="7" t="inlineStr">
@@ -13531,6 +13726,665 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AK192" s="7"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_185</t>
+        </is>
+      </c>
+      <c r="B193" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼</t>
+        </is>
+      </c>
+      <c r="C193" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 강화 안내</t>
+        </is>
+      </c>
+      <c r="D193" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">막 · 해제</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 파밍(튜토리얼 마침 · 재료 ≥ 50 · 고철 ≥ 300)에서 강화 막 → 보드 A 마운트 → 팝오버 강화 → 막 해제가 되는가? (B 해금 조건 없음)</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#188 · 🗑️ S4</t>
+        </is>
+      </c>
+      <c r="G193" s="7"/>
+      <c r="H193" s="7"/>
+      <c r="I193" s="7"/>
+      <c r="J193" s="7"/>
+      <c r="K193" s="7"/>
+      <c r="L193" s="7"/>
+      <c r="M193" s="7"/>
+      <c r="N193" s="7"/>
+      <c r="O193" s="7"/>
+      <c r="P193" s="7"/>
+      <c r="Q193" s="7"/>
+      <c r="R193" s="7"/>
+      <c r="S193" s="7"/>
+      <c r="T193" s="7"/>
+      <c r="U193" s="7"/>
+      <c r="V193" s="7"/>
+      <c r="W193" s="7"/>
+      <c r="X193" s="7"/>
+      <c r="Y193" s="7"/>
+      <c r="Z193" s="7"/>
+      <c r="AA193" s="7"/>
+      <c r="AB193" s="7"/>
+      <c r="AC193" s="7"/>
+      <c r="AD193" s="7"/>
+      <c r="AE193" s="7"/>
+      <c r="AF193" s="7"/>
+      <c r="AG193" s="7"/>
+      <c r="AH193" s="7"/>
+      <c r="AI193" s="7"/>
+      <c r="AJ193" s="7"/>
+      <c r="AK193" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_186</t>
+        </is>
+      </c>
+      <c r="B194" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼</t>
+        </is>
+      </c>
+      <c r="C194" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 합체 강제</t>
+        </is>
+      </c>
+      <c r="D194" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">막 · 해제</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 첫 도전에서 게이지가 차면 막 + 합체 원형만 밝음 + 「합체 버튼을 눌러 합체해보세요」 → 합체 누르면 해제되는가?</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#189 · 문구 ⚠️ 가정</t>
+        </is>
+      </c>
+      <c r="G194" s="7"/>
+      <c r="H194" s="7"/>
+      <c r="I194" s="7"/>
+      <c r="J194" s="7"/>
+      <c r="K194" s="7"/>
+      <c r="L194" s="7"/>
+      <c r="M194" s="7"/>
+      <c r="N194" s="7"/>
+      <c r="O194" s="7"/>
+      <c r="P194" s="7"/>
+      <c r="Q194" s="7"/>
+      <c r="R194" s="7"/>
+      <c r="S194" s="7"/>
+      <c r="T194" s="7"/>
+      <c r="U194" s="7"/>
+      <c r="V194" s="7"/>
+      <c r="W194" s="7"/>
+      <c r="X194" s="7"/>
+      <c r="Y194" s="7"/>
+      <c r="Z194" s="7"/>
+      <c r="AA194" s="7"/>
+      <c r="AB194" s="7"/>
+      <c r="AC194" s="7"/>
+      <c r="AD194" s="7"/>
+      <c r="AE194" s="7"/>
+      <c r="AF194" s="7"/>
+      <c r="AG194" s="7"/>
+      <c r="AH194" s="7"/>
+      <c r="AI194" s="7"/>
+      <c r="AJ194" s="7"/>
+      <c r="AK194" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_187</t>
+        </is>
+      </c>
+      <c r="B195" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼</t>
+        </is>
+      </c>
+      <c r="C195" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S5 폭발탄</t>
+        </is>
+      </c>
+      <c r="D195" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">알림 · 막 · 첫 걸음</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S5 파밍 첫 진입에 「복합 가공소가 열렸습니다」 알림 → 막 「▼ 조립」 → A 판 변환기 (6,7) 안내 · 조합표 「발전재료」 선택이 되는가?</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#190</t>
+        </is>
+      </c>
+      <c r="G195" s="7"/>
+      <c r="H195" s="7"/>
+      <c r="I195" s="7"/>
+      <c r="J195" s="7"/>
+      <c r="K195" s="7"/>
+      <c r="L195" s="7"/>
+      <c r="M195" s="7"/>
+      <c r="N195" s="7"/>
+      <c r="O195" s="7"/>
+      <c r="P195" s="7"/>
+      <c r="Q195" s="7"/>
+      <c r="R195" s="7"/>
+      <c r="S195" s="7"/>
+      <c r="T195" s="7"/>
+      <c r="U195" s="7"/>
+      <c r="V195" s="7"/>
+      <c r="W195" s="7"/>
+      <c r="X195" s="7"/>
+      <c r="Y195" s="7"/>
+      <c r="Z195" s="7"/>
+      <c r="AA195" s="7"/>
+      <c r="AB195" s="7"/>
+      <c r="AC195" s="7"/>
+      <c r="AD195" s="7"/>
+      <c r="AE195" s="7"/>
+      <c r="AF195" s="7"/>
+      <c r="AG195" s="7"/>
+      <c r="AH195" s="7"/>
+      <c r="AI195" s="7"/>
+      <c r="AJ195" s="7"/>
+      <c r="AK195" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_188</t>
+        </is>
+      </c>
+      <c r="B196" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼</t>
+        </is>
+      </c>
+      <c r="C196" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S5 폭발탄</t>
+        </is>
+      </c>
+      <c r="D196" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">다섯 걸음 끝</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(7,7) 탭 = 벨트 · 분류기 고르고 (8,8) 탭 · 복합 가공소 고르고 (8,7) 탭(90°) · 조합표 「폭발탄」 → 안내 해제 · 폭발탄이 마운트 A 에 닿는가? (팔레트는 그 걸음 것만)</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#190 · 끝 = 구조 판정(구현 판단)</t>
+        </is>
+      </c>
+      <c r="G196" s="7"/>
+      <c r="H196" s="7"/>
+      <c r="I196" s="7"/>
+      <c r="J196" s="7"/>
+      <c r="K196" s="7"/>
+      <c r="L196" s="7"/>
+      <c r="M196" s="7"/>
+      <c r="N196" s="7"/>
+      <c r="O196" s="7"/>
+      <c r="P196" s="7"/>
+      <c r="Q196" s="7"/>
+      <c r="R196" s="7"/>
+      <c r="S196" s="7"/>
+      <c r="T196" s="7"/>
+      <c r="U196" s="7"/>
+      <c r="V196" s="7"/>
+      <c r="W196" s="7"/>
+      <c r="X196" s="7"/>
+      <c r="Y196" s="7"/>
+      <c r="Z196" s="7"/>
+      <c r="AA196" s="7"/>
+      <c r="AB196" s="7"/>
+      <c r="AC196" s="7"/>
+      <c r="AD196" s="7"/>
+      <c r="AE196" s="7"/>
+      <c r="AF196" s="7"/>
+      <c r="AG196" s="7"/>
+      <c r="AH196" s="7"/>
+      <c r="AI196" s="7"/>
+      <c r="AJ196" s="7"/>
+      <c r="AK196" s="7"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_189</t>
+        </is>
+      </c>
+      <c r="B197" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">스테이지</t>
+        </is>
+      </c>
+      <c r="C197" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">주제</t>
+        </is>
+      </c>
+      <c r="D197" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3~S6</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t xml:space="preserve">스테이지 카드 주제가 S3 마운트 강화 · S4 로봇 B 해금 · 합체 · S5 폭발탄 · S6 자유 플레이 · 보스 인가?</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#191 · S6 화면 미확인</t>
+        </is>
+      </c>
+      <c r="G197" s="7"/>
+      <c r="H197" s="7"/>
+      <c r="I197" s="7"/>
+      <c r="J197" s="7"/>
+      <c r="K197" s="7"/>
+      <c r="L197" s="7"/>
+      <c r="M197" s="7"/>
+      <c r="N197" s="7"/>
+      <c r="O197" s="7"/>
+      <c r="P197" s="7"/>
+      <c r="Q197" s="7"/>
+      <c r="R197" s="7"/>
+      <c r="S197" s="7"/>
+      <c r="T197" s="7"/>
+      <c r="U197" s="7"/>
+      <c r="V197" s="7"/>
+      <c r="W197" s="7"/>
+      <c r="X197" s="7"/>
+      <c r="Y197" s="7"/>
+      <c r="Z197" s="7"/>
+      <c r="AA197" s="7"/>
+      <c r="AB197" s="7"/>
+      <c r="AC197" s="7"/>
+      <c r="AD197" s="7"/>
+      <c r="AE197" s="7"/>
+      <c r="AF197" s="7"/>
+      <c r="AG197" s="7"/>
+      <c r="AH197" s="7"/>
+      <c r="AI197" s="7"/>
+      <c r="AJ197" s="7"/>
+      <c r="AK197" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_190</t>
+        </is>
+      </c>
+      <c r="B198" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">사운드</t>
+        </is>
+      </c>
+      <c r="C198" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BGM</t>
+        </is>
+      </c>
+      <c r="D198" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S6 파밍</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S6 파밍 층은 기본 곡 · 도전 층만 보스 곡이고 전환 때 바뀌는가?</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#192</t>
+        </is>
+      </c>
+      <c r="G198" s="7"/>
+      <c r="H198" s="7"/>
+      <c r="I198" s="7"/>
+      <c r="J198" s="7"/>
+      <c r="K198" s="7"/>
+      <c r="L198" s="7"/>
+      <c r="M198" s="7"/>
+      <c r="N198" s="7"/>
+      <c r="O198" s="7"/>
+      <c r="P198" s="7"/>
+      <c r="Q198" s="7"/>
+      <c r="R198" s="7"/>
+      <c r="S198" s="7"/>
+      <c r="T198" s="7"/>
+      <c r="U198" s="7"/>
+      <c r="V198" s="7"/>
+      <c r="W198" s="7"/>
+      <c r="X198" s="7"/>
+      <c r="Y198" s="7"/>
+      <c r="Z198" s="7"/>
+      <c r="AA198" s="7"/>
+      <c r="AB198" s="7"/>
+      <c r="AC198" s="7"/>
+      <c r="AD198" s="7"/>
+      <c r="AE198" s="7"/>
+      <c r="AF198" s="7"/>
+      <c r="AG198" s="7"/>
+      <c r="AH198" s="7"/>
+      <c r="AI198" s="7"/>
+      <c r="AJ198" s="7"/>
+      <c r="AK198" s="7"/>
+    </row>
+    <row r="199">
+      <c r="A199" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_191</t>
+        </is>
+      </c>
+      <c r="B199" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C199" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도전 단추</t>
+        </is>
+      </c>
+      <c r="D199" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">통과함</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t xml:space="preserve">통과한 판의 「도전」이 「통과함」으로 흐려 눌리지 않고, 승리 결과 화면에 [다시 도전]이 없는가? (실패 때는 있음 · 바로가기 판은 도전 가능)</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#193</t>
+        </is>
+      </c>
+      <c r="G199" s="7"/>
+      <c r="H199" s="7"/>
+      <c r="I199" s="7"/>
+      <c r="J199" s="7"/>
+      <c r="K199" s="7"/>
+      <c r="L199" s="7"/>
+      <c r="M199" s="7"/>
+      <c r="N199" s="7"/>
+      <c r="O199" s="7"/>
+      <c r="P199" s="7"/>
+      <c r="Q199" s="7"/>
+      <c r="R199" s="7"/>
+      <c r="S199" s="7"/>
+      <c r="T199" s="7"/>
+      <c r="U199" s="7"/>
+      <c r="V199" s="7"/>
+      <c r="W199" s="7"/>
+      <c r="X199" s="7"/>
+      <c r="Y199" s="7"/>
+      <c r="Z199" s="7"/>
+      <c r="AA199" s="7"/>
+      <c r="AB199" s="7"/>
+      <c r="AC199" s="7"/>
+      <c r="AD199" s="7"/>
+      <c r="AE199" s="7"/>
+      <c r="AF199" s="7"/>
+      <c r="AG199" s="7"/>
+      <c r="AH199" s="7"/>
+      <c r="AI199" s="7"/>
+      <c r="AJ199" s="7"/>
+      <c r="AK199" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_192</t>
+        </is>
+      </c>
+      <c r="B200" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C200" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">결과 화면</t>
+        </is>
+      </c>
+      <c r="D200" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">강화 재료 +N</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t xml:space="preserve">최초 통과 승리 결과 화면에 「강화 재료 +N」(S1 30 · S2 33 · S3 37)이 뜨고, 보상 0 판은 안 뜨는가?</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#194</t>
+        </is>
+      </c>
+      <c r="G200" s="7"/>
+      <c r="H200" s="7"/>
+      <c r="I200" s="7"/>
+      <c r="J200" s="7"/>
+      <c r="K200" s="7"/>
+      <c r="L200" s="7"/>
+      <c r="M200" s="7"/>
+      <c r="N200" s="7"/>
+      <c r="O200" s="7"/>
+      <c r="P200" s="7"/>
+      <c r="Q200" s="7"/>
+      <c r="R200" s="7"/>
+      <c r="S200" s="7"/>
+      <c r="T200" s="7"/>
+      <c r="U200" s="7"/>
+      <c r="V200" s="7"/>
+      <c r="W200" s="7"/>
+      <c r="X200" s="7"/>
+      <c r="Y200" s="7"/>
+      <c r="Z200" s="7"/>
+      <c r="AA200" s="7"/>
+      <c r="AB200" s="7"/>
+      <c r="AC200" s="7"/>
+      <c r="AD200" s="7"/>
+      <c r="AE200" s="7"/>
+      <c r="AF200" s="7"/>
+      <c r="AG200" s="7"/>
+      <c r="AH200" s="7"/>
+      <c r="AI200" s="7"/>
+      <c r="AJ200" s="7"/>
+      <c r="AK200" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_193</t>
+        </is>
+      </c>
+      <c r="B201" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">조립</t>
+        </is>
+      </c>
+      <c r="C201" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">마운트 팝오버</t>
+        </is>
+      </c>
+      <c r="D201" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">로봇 B 강화</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S6 파밍에서 B 강화 막 → 조립(B 판) → B 마운트 칸 안내 → 팝오버 강화(재료 50 · 고철 300) → B 계수 ×1.45 · A 표식과 따로인가?</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#195</t>
+        </is>
+      </c>
+      <c r="G201" s="7"/>
+      <c r="H201" s="7"/>
+      <c r="I201" s="7"/>
+      <c r="J201" s="7"/>
+      <c r="K201" s="7"/>
+      <c r="L201" s="7"/>
+      <c r="M201" s="7"/>
+      <c r="N201" s="7"/>
+      <c r="O201" s="7"/>
+      <c r="P201" s="7"/>
+      <c r="Q201" s="7"/>
+      <c r="R201" s="7"/>
+      <c r="S201" s="7"/>
+      <c r="T201" s="7"/>
+      <c r="U201" s="7"/>
+      <c r="V201" s="7"/>
+      <c r="W201" s="7"/>
+      <c r="X201" s="7"/>
+      <c r="Y201" s="7"/>
+      <c r="Z201" s="7"/>
+      <c r="AA201" s="7"/>
+      <c r="AB201" s="7"/>
+      <c r="AC201" s="7"/>
+      <c r="AD201" s="7"/>
+      <c r="AE201" s="7"/>
+      <c r="AF201" s="7"/>
+      <c r="AG201" s="7"/>
+      <c r="AH201" s="7"/>
+      <c r="AI201" s="7"/>
+      <c r="AJ201" s="7"/>
+      <c r="AK201" s="7"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_194</t>
+        </is>
+      </c>
+      <c r="B202" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">조립</t>
+        </is>
+      </c>
+      <c r="C202" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">마운트 팝오버</t>
+        </is>
+      </c>
+      <c r="D202" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">강화 비용 50</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t xml:space="preserve">마운트 팝오버가 「강화 재료 n/50」이고 50 이면 강화되는가?</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#196</t>
+        </is>
+      </c>
+      <c r="G202" s="7"/>
+      <c r="H202" s="7"/>
+      <c r="I202" s="7"/>
+      <c r="J202" s="7"/>
+      <c r="K202" s="7"/>
+      <c r="L202" s="7"/>
+      <c r="M202" s="7"/>
+      <c r="N202" s="7"/>
+      <c r="O202" s="7"/>
+      <c r="P202" s="7"/>
+      <c r="Q202" s="7"/>
+      <c r="R202" s="7"/>
+      <c r="S202" s="7"/>
+      <c r="T202" s="7"/>
+      <c r="U202" s="7"/>
+      <c r="V202" s="7"/>
+      <c r="W202" s="7"/>
+      <c r="X202" s="7"/>
+      <c r="Y202" s="7"/>
+      <c r="Z202" s="7"/>
+      <c r="AA202" s="7"/>
+      <c r="AB202" s="7"/>
+      <c r="AC202" s="7"/>
+      <c r="AD202" s="7"/>
+      <c r="AE202" s="7"/>
+      <c r="AF202" s="7"/>
+      <c r="AG202" s="7"/>
+      <c r="AH202" s="7"/>
+      <c r="AI202" s="7"/>
+      <c r="AJ202" s="7"/>
+      <c r="AK202" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="26">
@@ -13559,9 +14413,9 @@
     <mergeCell ref="B92:B99"/>
     <mergeCell ref="B100:B106"/>
     <mergeCell ref="B107:B111"/>
-    <mergeCell ref="G7:AJ7"/>
+    <mergeCell ref="G7:AK7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:AJ192">
+  <conditionalFormatting sqref="G9:AK202">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
docs: QA AL열(4a6f983 · CID_195 #197) · 가이드 8133 후보 4a6f983 · B 판 새로고침 리셋 경고
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -193,8 +193,9 @@
     <col min="35" max="35" width="12" customWidth="1"/>
     <col min="36" max="36" width="12" customWidth="1"/>
     <col min="37" max="37" width="12" customWidth="1"/>
-    <col min="38" max="38" width="11" customWidth="1"/>
+    <col min="38" max="38" width="12" customWidth="1"/>
     <col min="39" max="39" width="11" customWidth="1"/>
+    <col min="40" max="40" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -462,6 +463,11 @@
       <c r="AK6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">video-261019d 후보 갈아엎음(8133 · 19:00:23) · #188~#196(플랜 §98-47) ‖ 10-19 코드 세션 재확인(8123 · 인앱 · 새 저장 「처음부터」 자연 진행): S1 승리 = 「강화 재료 +30」 · [스테이지로][다음 스테이지로](다시 도전 없음) → 스테이지로 = 「통과함」 흐림 → S2 T4 → 승리 +33 → S3 파밍 주제 「마운트 강화」 · 막 「조립에서 마운트를 탭해 강화해보세요」 → 보드 시야 A 마운트 · 안내 → 팝오버 「강화 재료 63/50」 → 강화 = 13/50 → ⚠️ S3 파밍 강화 뒤에도 약 35초에 파괴(HP 970 → 100/30초) → S2 로 밀림 · S3 도전 승리 +37 → S4 해금 → (페이지 새로고침 뒤) S4 도전 = 합체 막 「합체 버튼을 눌러 합체해보세요」 → 합체 = 막 해제 → S4 승리(보상 줄 없음) → S5 알림 「복합 가공소가 열렸습니다」 · 주제 「폭발탄」 · 막 → A 판 ① 안내 · 변환기 조합표 발전재료 선택 ✓ → S5 파밍 파괴로 S4 로 밀려 ②~⑤ 화면 미확인 · #192 BGM(소리 0) · #195 B 강화(S6 미도달) 화면 미확인 = 시험이 든다 · ⚠️ 새로고침 뒤 HUD 전투력 0(8132 동결 빌드도 같음 · 기존) · CID_185~194 새 항목)</t>
+        </is>
+      </c>
+      <c r="AL6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8133 갈아엎음(19:16:23) · #197 보드 저장 주인 칸 결함 수정 ‖ 10-19 코드 세션 재확인(8123): 「처음부터」 → 바로가기 S5(A 프리셋) → 조립 → 로봇 B 탭 → 전투로 → 20초 → 새로고침 → 조립 A 판 = 프리셋 그대로(복합 가공소 (8,7) · 변환기 (6,7) 발전재료 · (7,7) 벨트) ✅ · 고치기 전 재현 = 새로고침 뒤 콘솔 「저장된 보드(RobotA)를 버린다 — 저장 0x0」 → 시작 보드 · 전투력 0(8132 도 같음) · ⚠️ 콘솔 버퍼가 앞 판 경고를 들고 있어 경고 유무로는 못 가름 — 판 모양으로 확인 · CID_195 새 항목</t>
         </is>
       </c>
     </row>
@@ -523,14 +529,15 @@
       <c r="AI7" s="2"/>
       <c r="AJ7" s="2"/>
       <c r="AK7" s="2"/>
-      <c r="AL7" s="2" t="inlineStr">
+      <c r="AL7" s="2"/>
+      <c r="AM7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">버전</t>
         </is>
       </c>
-      <c r="AM7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">cae560d</t>
+      <c r="AN7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4a6f983</t>
         </is>
       </c>
     </row>
@@ -710,11 +717,16 @@
       </c>
       <c r="AL8" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">4a6f983</t>
+        </is>
+      </c>
+      <c r="AM8" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">PASSrate</t>
         </is>
       </c>
-      <c r="AM8" s="7">
-        <f>COUNTIF(AK9:AK202,"Pass")</f>
+      <c r="AN8" s="7">
+        <f>COUNTIF(AL9:AL203,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -815,13 +827,14 @@
       <c r="AI9" s="7"/>
       <c r="AJ9" s="7"/>
       <c r="AK9" s="7"/>
-      <c r="AL9" s="2" t="inlineStr">
+      <c r="AL9" s="7"/>
+      <c r="AM9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FAILrate</t>
         </is>
       </c>
-      <c r="AM9" s="7">
-        <f>COUNTIF(AK9:AK202,"Fail")+COUNTIF(AK9:AK202,"Broken")</f>
+      <c r="AN9" s="7">
+        <f>COUNTIF(AL9:AL203,"Fail")+COUNTIF(AL9:AL203,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -886,13 +899,14 @@
       <c r="AI10" s="7"/>
       <c r="AJ10" s="7"/>
       <c r="AK10" s="7"/>
-      <c r="AL10" s="2" t="inlineStr">
+      <c r="AL10" s="7"/>
+      <c r="AM10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">N/A</t>
         </is>
       </c>
-      <c r="AM10" s="7">
-        <f>COUNTIF(AK9:AK202,"N/A")</f>
+      <c r="AN10" s="7">
+        <f>COUNTIF(AL9:AL203,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -957,13 +971,14 @@
       <c r="AI11" s="7"/>
       <c r="AJ11" s="7"/>
       <c r="AK11" s="7"/>
-      <c r="AL11" s="2" t="inlineStr">
+      <c r="AL11" s="7"/>
+      <c r="AM11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">전체 개수</t>
         </is>
       </c>
-      <c r="AM11" s="7">
-        <v>194</v>
+      <c r="AN11" s="7">
+        <v>195</v>
       </c>
     </row>
     <row r="12">
@@ -1028,13 +1043,14 @@
       <c r="AI12" s="7"/>
       <c r="AJ12" s="7"/>
       <c r="AK12" s="7"/>
-      <c r="AL12" s="2" t="inlineStr">
+      <c r="AL12" s="7"/>
+      <c r="AM12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">진행율</t>
         </is>
       </c>
-      <c r="AM12" s="7">
-        <f>TEXT((COUNTA(AK9:AK202))/194,"0.00%")</f>
+      <c r="AN12" s="7">
+        <f>TEXT((COUNTA(AL9:AL203))/195,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -1103,6 +1119,7 @@
       <c r="AI13" s="7"/>
       <c r="AJ13" s="7"/>
       <c r="AK13" s="7"/>
+      <c r="AL13" s="7"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -1161,6 +1178,7 @@
       <c r="AI14" s="7"/>
       <c r="AJ14" s="7"/>
       <c r="AK14" s="7"/>
+      <c r="AL14" s="7"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -1255,6 +1273,7 @@
       <c r="AI15" s="7"/>
       <c r="AJ15" s="7"/>
       <c r="AK15" s="7"/>
+      <c r="AL15" s="7"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -1349,6 +1368,7 @@
       <c r="AI16" s="7"/>
       <c r="AJ16" s="7"/>
       <c r="AK16" s="7"/>
+      <c r="AL16" s="7"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -1448,6 +1468,7 @@
       <c r="AI17" s="7"/>
       <c r="AJ17" s="7"/>
       <c r="AK17" s="7"/>
+      <c r="AL17" s="7"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -1511,6 +1532,7 @@
       <c r="AI18" s="7"/>
       <c r="AJ18" s="7"/>
       <c r="AK18" s="7"/>
+      <c r="AL18" s="7"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -1569,6 +1591,7 @@
       <c r="AI19" s="7"/>
       <c r="AJ19" s="7"/>
       <c r="AK19" s="7"/>
+      <c r="AL19" s="7"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1627,6 +1650,7 @@
       <c r="AI20" s="7"/>
       <c r="AJ20" s="7"/>
       <c r="AK20" s="7"/>
+      <c r="AL20" s="7"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1721,6 +1745,7 @@
       <c r="AI21" s="7"/>
       <c r="AJ21" s="7"/>
       <c r="AK21" s="7"/>
+      <c r="AL21" s="7"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1808,6 +1833,7 @@
       <c r="AI22" s="7"/>
       <c r="AJ22" s="7"/>
       <c r="AK22" s="7"/>
+      <c r="AL22" s="7"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -1874,6 +1900,7 @@
       <c r="AI23" s="7"/>
       <c r="AJ23" s="7"/>
       <c r="AK23" s="7"/>
+      <c r="AL23" s="7"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -1932,6 +1959,7 @@
       <c r="AI24" s="7"/>
       <c r="AJ24" s="7"/>
       <c r="AK24" s="7"/>
+      <c r="AL24" s="7"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -1990,6 +2018,7 @@
       <c r="AI25" s="7"/>
       <c r="AJ25" s="7"/>
       <c r="AK25" s="7"/>
+      <c r="AL25" s="7"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -2077,6 +2106,7 @@
       <c r="AI26" s="7"/>
       <c r="AJ26" s="7"/>
       <c r="AK26" s="7"/>
+      <c r="AL26" s="7"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -2139,6 +2169,7 @@
       <c r="AI27" s="7"/>
       <c r="AJ27" s="7"/>
       <c r="AK27" s="7"/>
+      <c r="AL27" s="7"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -2210,6 +2241,7 @@
       <c r="AI28" s="7"/>
       <c r="AJ28" s="7"/>
       <c r="AK28" s="7"/>
+      <c r="AL28" s="7"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -2276,6 +2308,7 @@
       <c r="AI29" s="7"/>
       <c r="AJ29" s="7"/>
       <c r="AK29" s="7"/>
+      <c r="AL29" s="7"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -2366,6 +2399,7 @@
       <c r="AI30" s="7"/>
       <c r="AJ30" s="7"/>
       <c r="AK30" s="7"/>
+      <c r="AL30" s="7"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -2461,6 +2495,7 @@
       <c r="AI31" s="7"/>
       <c r="AJ31" s="7"/>
       <c r="AK31" s="7"/>
+      <c r="AL31" s="7"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -2543,6 +2578,7 @@
       <c r="AI32" s="7"/>
       <c r="AJ32" s="7"/>
       <c r="AK32" s="7"/>
+      <c r="AL32" s="7"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -2633,6 +2669,7 @@
       <c r="AI33" s="7"/>
       <c r="AJ33" s="7"/>
       <c r="AK33" s="7"/>
+      <c r="AL33" s="7"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -2723,6 +2760,7 @@
       <c r="AI34" s="7"/>
       <c r="AJ34" s="7"/>
       <c r="AK34" s="7"/>
+      <c r="AL34" s="7"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -2822,6 +2860,7 @@
       <c r="AI35" s="7"/>
       <c r="AJ35" s="7"/>
       <c r="AK35" s="7"/>
+      <c r="AL35" s="7"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -2896,6 +2935,7 @@
       <c r="AI36" s="7"/>
       <c r="AJ36" s="7"/>
       <c r="AK36" s="7"/>
+      <c r="AL36" s="7"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -2954,6 +2994,7 @@
       <c r="AI37" s="7"/>
       <c r="AJ37" s="7"/>
       <c r="AK37" s="7"/>
+      <c r="AL37" s="7"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -3033,6 +3074,7 @@
       <c r="AI38" s="7"/>
       <c r="AJ38" s="7"/>
       <c r="AK38" s="7"/>
+      <c r="AL38" s="7"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -3123,6 +3165,7 @@
       <c r="AI39" s="7"/>
       <c r="AJ39" s="7"/>
       <c r="AK39" s="7"/>
+      <c r="AL39" s="7"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -3214,6 +3257,7 @@
       <c r="AI40" s="7"/>
       <c r="AJ40" s="7"/>
       <c r="AK40" s="7"/>
+      <c r="AL40" s="7"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -3300,6 +3344,7 @@
       <c r="AI41" s="7"/>
       <c r="AJ41" s="7"/>
       <c r="AK41" s="7"/>
+      <c r="AL41" s="7"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -3370,6 +3415,7 @@
       <c r="AI42" s="7"/>
       <c r="AJ42" s="7"/>
       <c r="AK42" s="7"/>
+      <c r="AL42" s="7"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -3460,6 +3506,7 @@
       <c r="AI43" s="7"/>
       <c r="AJ43" s="7"/>
       <c r="AK43" s="7"/>
+      <c r="AL43" s="7"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -3523,6 +3570,7 @@
       <c r="AI44" s="7"/>
       <c r="AJ44" s="7"/>
       <c r="AK44" s="7"/>
+      <c r="AL44" s="7"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -3609,6 +3657,7 @@
       <c r="AI45" s="7"/>
       <c r="AJ45" s="7"/>
       <c r="AK45" s="7"/>
+      <c r="AL45" s="7"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -3695,6 +3744,7 @@
       <c r="AI46" s="7"/>
       <c r="AJ46" s="7"/>
       <c r="AK46" s="7"/>
+      <c r="AL46" s="7"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -3758,6 +3808,7 @@
       <c r="AI47" s="7"/>
       <c r="AJ47" s="7"/>
       <c r="AK47" s="7"/>
+      <c r="AL47" s="7"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -3816,6 +3867,7 @@
       <c r="AI48" s="7"/>
       <c r="AJ48" s="7"/>
       <c r="AK48" s="7"/>
+      <c r="AL48" s="7"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -3874,6 +3926,7 @@
       <c r="AI49" s="7"/>
       <c r="AJ49" s="7"/>
       <c r="AK49" s="7"/>
+      <c r="AL49" s="7"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -3956,6 +4009,7 @@
       <c r="AI50" s="7"/>
       <c r="AJ50" s="7"/>
       <c r="AK50" s="7"/>
+      <c r="AL50" s="7"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -4038,6 +4092,7 @@
       <c r="AI51" s="7"/>
       <c r="AJ51" s="7"/>
       <c r="AK51" s="7"/>
+      <c r="AL51" s="7"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -4101,6 +4156,7 @@
       <c r="AI52" s="7"/>
       <c r="AJ52" s="7"/>
       <c r="AK52" s="7"/>
+      <c r="AL52" s="7"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -4164,6 +4220,7 @@
       <c r="AI53" s="7"/>
       <c r="AJ53" s="7"/>
       <c r="AK53" s="7"/>
+      <c r="AL53" s="7"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -4222,6 +4279,7 @@
       <c r="AI54" s="7"/>
       <c r="AJ54" s="7"/>
       <c r="AK54" s="7"/>
+      <c r="AL54" s="7"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -4316,6 +4374,7 @@
       <c r="AI55" s="7"/>
       <c r="AJ55" s="7"/>
       <c r="AK55" s="7"/>
+      <c r="AL55" s="7"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -4390,6 +4449,7 @@
       <c r="AI56" s="7"/>
       <c r="AJ56" s="7"/>
       <c r="AK56" s="7"/>
+      <c r="AL56" s="7"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -4473,6 +4533,7 @@
       <c r="AI57" s="7"/>
       <c r="AJ57" s="7"/>
       <c r="AK57" s="7"/>
+      <c r="AL57" s="7"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -4564,6 +4625,7 @@
       <c r="AI58" s="7"/>
       <c r="AJ58" s="7"/>
       <c r="AK58" s="7"/>
+      <c r="AL58" s="7"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -4622,6 +4684,7 @@
       <c r="AI59" s="7"/>
       <c r="AJ59" s="7"/>
       <c r="AK59" s="7"/>
+      <c r="AL59" s="7"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -4680,6 +4743,7 @@
       <c r="AI60" s="7"/>
       <c r="AJ60" s="7"/>
       <c r="AK60" s="7"/>
+      <c r="AL60" s="7"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -4750,6 +4814,7 @@
       <c r="AI61" s="7"/>
       <c r="AJ61" s="7"/>
       <c r="AK61" s="7"/>
+      <c r="AL61" s="7"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -4828,6 +4893,7 @@
       <c r="AI62" s="7"/>
       <c r="AJ62" s="7"/>
       <c r="AK62" s="7"/>
+      <c r="AL62" s="7"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -4898,6 +4964,7 @@
       <c r="AI63" s="7"/>
       <c r="AJ63" s="7"/>
       <c r="AK63" s="7"/>
+      <c r="AL63" s="7"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -4956,6 +5023,7 @@
       <c r="AI64" s="7"/>
       <c r="AJ64" s="7"/>
       <c r="AK64" s="7"/>
+      <c r="AL64" s="7"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -5019,6 +5087,7 @@
       <c r="AI65" s="7"/>
       <c r="AJ65" s="7"/>
       <c r="AK65" s="7"/>
+      <c r="AL65" s="7"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
@@ -5089,6 +5158,7 @@
       <c r="AI66" s="7"/>
       <c r="AJ66" s="7"/>
       <c r="AK66" s="7"/>
+      <c r="AL66" s="7"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -5147,6 +5217,7 @@
       <c r="AI67" s="7"/>
       <c r="AJ67" s="7"/>
       <c r="AK67" s="7"/>
+      <c r="AL67" s="7"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
@@ -5209,6 +5280,7 @@
       <c r="AI68" s="7"/>
       <c r="AJ68" s="7"/>
       <c r="AK68" s="7"/>
+      <c r="AL68" s="7"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -5303,6 +5375,7 @@
       <c r="AI69" s="7"/>
       <c r="AJ69" s="7"/>
       <c r="AK69" s="7"/>
+      <c r="AL69" s="7"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
@@ -5361,6 +5434,7 @@
       <c r="AI70" s="7"/>
       <c r="AJ70" s="7"/>
       <c r="AK70" s="7"/>
+      <c r="AL70" s="7"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -5424,6 +5498,7 @@
       <c r="AI71" s="7"/>
       <c r="AJ71" s="7"/>
       <c r="AK71" s="7"/>
+      <c r="AL71" s="7"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
@@ -5498,6 +5573,7 @@
       <c r="AI72" s="7"/>
       <c r="AJ72" s="7"/>
       <c r="AK72" s="7"/>
+      <c r="AL72" s="7"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
@@ -5561,6 +5637,7 @@
       <c r="AI73" s="7"/>
       <c r="AJ73" s="7"/>
       <c r="AK73" s="7"/>
+      <c r="AL73" s="7"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -5619,6 +5696,7 @@
       <c r="AI74" s="7"/>
       <c r="AJ74" s="7"/>
       <c r="AK74" s="7"/>
+      <c r="AL74" s="7"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -5677,6 +5755,7 @@
       <c r="AI75" s="7"/>
       <c r="AJ75" s="7"/>
       <c r="AK75" s="7"/>
+      <c r="AL75" s="7"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -5735,6 +5814,7 @@
       <c r="AI76" s="7"/>
       <c r="AJ76" s="7"/>
       <c r="AK76" s="7"/>
+      <c r="AL76" s="7"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -5797,6 +5877,7 @@
       <c r="AI77" s="7"/>
       <c r="AJ77" s="7"/>
       <c r="AK77" s="7"/>
+      <c r="AL77" s="7"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
@@ -5855,6 +5936,7 @@
       <c r="AI78" s="7"/>
       <c r="AJ78" s="7"/>
       <c r="AK78" s="7"/>
+      <c r="AL78" s="7"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -5918,6 +6000,7 @@
       <c r="AI79" s="7"/>
       <c r="AJ79" s="7"/>
       <c r="AK79" s="7"/>
+      <c r="AL79" s="7"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
@@ -5992,6 +6075,7 @@
       <c r="AI80" s="7"/>
       <c r="AJ80" s="7"/>
       <c r="AK80" s="7"/>
+      <c r="AL80" s="7"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
@@ -6054,6 +6138,7 @@
       <c r="AI81" s="7"/>
       <c r="AJ81" s="7"/>
       <c r="AK81" s="7"/>
+      <c r="AL81" s="7"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
@@ -6112,6 +6197,7 @@
       <c r="AI82" s="7"/>
       <c r="AJ82" s="7"/>
       <c r="AK82" s="7"/>
+      <c r="AL82" s="7"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
@@ -6175,6 +6261,7 @@
       <c r="AI83" s="7"/>
       <c r="AJ83" s="7"/>
       <c r="AK83" s="7"/>
+      <c r="AL83" s="7"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
@@ -6233,6 +6320,7 @@
       <c r="AI84" s="7"/>
       <c r="AJ84" s="7"/>
       <c r="AK84" s="7"/>
+      <c r="AL84" s="7"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
@@ -6291,6 +6379,7 @@
       <c r="AI85" s="7"/>
       <c r="AJ85" s="7"/>
       <c r="AK85" s="7"/>
+      <c r="AL85" s="7"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
@@ -6354,6 +6443,7 @@
       <c r="AI86" s="7"/>
       <c r="AJ86" s="7"/>
       <c r="AK86" s="7"/>
+      <c r="AL86" s="7"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
@@ -6412,6 +6502,7 @@
       <c r="AI87" s="7"/>
       <c r="AJ87" s="7"/>
       <c r="AK87" s="7"/>
+      <c r="AL87" s="7"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
@@ -6470,6 +6561,7 @@
       <c r="AI88" s="7"/>
       <c r="AJ88" s="7"/>
       <c r="AK88" s="7"/>
+      <c r="AL88" s="7"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
@@ -6528,6 +6620,7 @@
       <c r="AI89" s="7"/>
       <c r="AJ89" s="7"/>
       <c r="AK89" s="7"/>
+      <c r="AL89" s="7"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
@@ -6615,6 +6708,7 @@
       <c r="AI90" s="7"/>
       <c r="AJ90" s="7"/>
       <c r="AK90" s="7"/>
+      <c r="AL90" s="7"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
@@ -6673,6 +6767,7 @@
       <c r="AI91" s="7"/>
       <c r="AJ91" s="7"/>
       <c r="AK91" s="7"/>
+      <c r="AL91" s="7"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
@@ -6767,6 +6862,7 @@
       <c r="AI92" s="7"/>
       <c r="AJ92" s="7"/>
       <c r="AK92" s="7"/>
+      <c r="AL92" s="7"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
@@ -6866,6 +6962,7 @@
       <c r="AI93" s="7"/>
       <c r="AJ93" s="7"/>
       <c r="AK93" s="7"/>
+      <c r="AL93" s="7"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
@@ -6929,6 +7026,7 @@
       <c r="AI94" s="7"/>
       <c r="AJ94" s="7"/>
       <c r="AK94" s="7"/>
+      <c r="AL94" s="7"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
@@ -6992,6 +7090,7 @@
       <c r="AI95" s="7"/>
       <c r="AJ95" s="7"/>
       <c r="AK95" s="7"/>
+      <c r="AL95" s="7"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
@@ -7074,6 +7173,7 @@
       <c r="AI96" s="7"/>
       <c r="AJ96" s="7"/>
       <c r="AK96" s="7"/>
+      <c r="AL96" s="7"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="inlineStr">
@@ -7132,6 +7232,7 @@
       <c r="AI97" s="7"/>
       <c r="AJ97" s="7"/>
       <c r="AK97" s="7"/>
+      <c r="AL97" s="7"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
@@ -7190,6 +7291,7 @@
       <c r="AI98" s="7"/>
       <c r="AJ98" s="7"/>
       <c r="AK98" s="7"/>
+      <c r="AL98" s="7"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
@@ -7248,6 +7350,7 @@
       <c r="AI99" s="7"/>
       <c r="AJ99" s="7"/>
       <c r="AK99" s="7"/>
+      <c r="AL99" s="7"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
@@ -7315,6 +7418,7 @@
       <c r="AI100" s="7"/>
       <c r="AJ100" s="7"/>
       <c r="AK100" s="7"/>
+      <c r="AL100" s="7"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
@@ -7373,6 +7477,7 @@
       <c r="AI101" s="7"/>
       <c r="AJ101" s="7"/>
       <c r="AK101" s="7"/>
+      <c r="AL101" s="7"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
@@ -7431,6 +7536,7 @@
       <c r="AI102" s="7"/>
       <c r="AJ102" s="7"/>
       <c r="AK102" s="7"/>
+      <c r="AL102" s="7"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="inlineStr">
@@ -7489,6 +7595,7 @@
       <c r="AI103" s="7"/>
       <c r="AJ103" s="7"/>
       <c r="AK103" s="7"/>
+      <c r="AL103" s="7"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="inlineStr">
@@ -7552,6 +7659,7 @@
       <c r="AI104" s="7"/>
       <c r="AJ104" s="7"/>
       <c r="AK104" s="7"/>
+      <c r="AL104" s="7"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
@@ -7610,6 +7718,7 @@
       <c r="AI105" s="7"/>
       <c r="AJ105" s="7"/>
       <c r="AK105" s="7"/>
+      <c r="AL105" s="7"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
@@ -7668,6 +7777,7 @@
       <c r="AI106" s="7"/>
       <c r="AJ106" s="7"/>
       <c r="AK106" s="7"/>
+      <c r="AL106" s="7"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
@@ -7726,6 +7836,7 @@
       <c r="AI107" s="7"/>
       <c r="AJ107" s="7"/>
       <c r="AK107" s="7"/>
+      <c r="AL107" s="7"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
@@ -7788,6 +7899,7 @@
       <c r="AI108" s="7"/>
       <c r="AJ108" s="7"/>
       <c r="AK108" s="7"/>
+      <c r="AL108" s="7"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="inlineStr">
@@ -7855,6 +7967,7 @@
       <c r="AI109" s="7"/>
       <c r="AJ109" s="7"/>
       <c r="AK109" s="7"/>
+      <c r="AL109" s="7"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
@@ -7930,6 +8043,7 @@
       <c r="AI110" s="7"/>
       <c r="AJ110" s="7"/>
       <c r="AK110" s="7"/>
+      <c r="AL110" s="7"/>
     </row>
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
@@ -8008,6 +8122,7 @@
       <c r="AI111" s="7"/>
       <c r="AJ111" s="7"/>
       <c r="AK111" s="7"/>
+      <c r="AL111" s="7"/>
     </row>
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
@@ -8083,6 +8198,7 @@
       <c r="AI112" s="7"/>
       <c r="AJ112" s="7"/>
       <c r="AK112" s="7"/>
+      <c r="AL112" s="7"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
@@ -8150,6 +8266,7 @@
       <c r="AI113" s="7"/>
       <c r="AJ113" s="7"/>
       <c r="AK113" s="7"/>
+      <c r="AL113" s="7"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="inlineStr">
@@ -8233,6 +8350,7 @@
       <c r="AI114" s="7"/>
       <c r="AJ114" s="7"/>
       <c r="AK114" s="7"/>
+      <c r="AL114" s="7"/>
     </row>
     <row r="115">
       <c r="A115" s="7" t="inlineStr">
@@ -8308,6 +8426,7 @@
       <c r="AI115" s="7"/>
       <c r="AJ115" s="7"/>
       <c r="AK115" s="7"/>
+      <c r="AL115" s="7"/>
     </row>
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
@@ -8391,6 +8510,7 @@
       <c r="AI116" s="7"/>
       <c r="AJ116" s="7"/>
       <c r="AK116" s="7"/>
+      <c r="AL116" s="7"/>
     </row>
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
@@ -8470,6 +8590,7 @@
       <c r="AI117" s="7"/>
       <c r="AJ117" s="7"/>
       <c r="AK117" s="7"/>
+      <c r="AL117" s="7"/>
     </row>
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
@@ -8549,6 +8670,7 @@
       <c r="AI118" s="7"/>
       <c r="AJ118" s="7"/>
       <c r="AK118" s="7"/>
+      <c r="AL118" s="7"/>
     </row>
     <row r="119">
       <c r="A119" s="7" t="inlineStr">
@@ -8624,6 +8746,7 @@
       <c r="AI119" s="7"/>
       <c r="AJ119" s="7"/>
       <c r="AK119" s="7"/>
+      <c r="AL119" s="7"/>
     </row>
     <row r="120">
       <c r="A120" s="7" t="inlineStr">
@@ -8691,6 +8814,7 @@
       <c r="AI120" s="7"/>
       <c r="AJ120" s="7"/>
       <c r="AK120" s="7"/>
+      <c r="AL120" s="7"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="inlineStr">
@@ -8770,6 +8894,7 @@
       <c r="AI121" s="7"/>
       <c r="AJ121" s="7"/>
       <c r="AK121" s="7"/>
+      <c r="AL121" s="7"/>
     </row>
     <row r="122">
       <c r="A122" s="7" t="inlineStr">
@@ -8849,6 +8974,7 @@
       <c r="AI122" s="7"/>
       <c r="AJ122" s="7"/>
       <c r="AK122" s="7"/>
+      <c r="AL122" s="7"/>
     </row>
     <row r="123">
       <c r="A123" s="7" t="inlineStr">
@@ -8916,6 +9042,7 @@
       <c r="AI123" s="7"/>
       <c r="AJ123" s="7"/>
       <c r="AK123" s="7"/>
+      <c r="AL123" s="7"/>
     </row>
     <row r="124">
       <c r="A124" s="7" t="inlineStr">
@@ -8991,6 +9118,7 @@
       <c r="AI124" s="7"/>
       <c r="AJ124" s="7"/>
       <c r="AK124" s="7"/>
+      <c r="AL124" s="7"/>
     </row>
     <row r="125">
       <c r="A125" s="7" t="inlineStr">
@@ -9058,6 +9186,7 @@
       <c r="AI125" s="7"/>
       <c r="AJ125" s="7"/>
       <c r="AK125" s="7"/>
+      <c r="AL125" s="7"/>
     </row>
     <row r="126">
       <c r="A126" s="7" t="inlineStr">
@@ -9125,6 +9254,7 @@
       <c r="AI126" s="7"/>
       <c r="AJ126" s="7"/>
       <c r="AK126" s="7"/>
+      <c r="AL126" s="7"/>
     </row>
     <row r="127">
       <c r="A127" s="7" t="inlineStr">
@@ -9196,6 +9326,7 @@
       <c r="AI127" s="7"/>
       <c r="AJ127" s="7"/>
       <c r="AK127" s="7"/>
+      <c r="AL127" s="7"/>
     </row>
     <row r="128">
       <c r="A128" s="7" t="inlineStr">
@@ -9267,6 +9398,7 @@
       <c r="AI128" s="7"/>
       <c r="AJ128" s="7"/>
       <c r="AK128" s="7"/>
+      <c r="AL128" s="7"/>
     </row>
     <row r="129">
       <c r="A129" s="7" t="inlineStr">
@@ -9338,6 +9470,7 @@
       <c r="AI129" s="7"/>
       <c r="AJ129" s="7"/>
       <c r="AK129" s="7"/>
+      <c r="AL129" s="7"/>
     </row>
     <row r="130">
       <c r="A130" s="7" t="inlineStr">
@@ -9405,6 +9538,7 @@
       <c r="AI130" s="7"/>
       <c r="AJ130" s="7"/>
       <c r="AK130" s="7"/>
+      <c r="AL130" s="7"/>
     </row>
     <row r="131">
       <c r="A131" s="7" t="inlineStr">
@@ -9480,6 +9614,7 @@
       <c r="AI131" s="7"/>
       <c r="AJ131" s="7"/>
       <c r="AK131" s="7"/>
+      <c r="AL131" s="7"/>
     </row>
     <row r="132">
       <c r="A132" s="7" t="inlineStr">
@@ -9559,6 +9694,7 @@
       <c r="AI132" s="7"/>
       <c r="AJ132" s="7"/>
       <c r="AK132" s="7"/>
+      <c r="AL132" s="7"/>
     </row>
     <row r="133">
       <c r="A133" s="7" t="inlineStr">
@@ -9638,6 +9774,7 @@
       <c r="AI133" s="7"/>
       <c r="AJ133" s="7"/>
       <c r="AK133" s="7"/>
+      <c r="AL133" s="7"/>
     </row>
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
@@ -9713,6 +9850,7 @@
       <c r="AI134" s="7"/>
       <c r="AJ134" s="7"/>
       <c r="AK134" s="7"/>
+      <c r="AL134" s="7"/>
     </row>
     <row r="135">
       <c r="A135" s="7" t="inlineStr">
@@ -9788,6 +9926,7 @@
       <c r="AI135" s="7"/>
       <c r="AJ135" s="7"/>
       <c r="AK135" s="7"/>
+      <c r="AL135" s="7"/>
     </row>
     <row r="136">
       <c r="A136" s="7" t="inlineStr">
@@ -9863,6 +10002,7 @@
       <c r="AI136" s="7"/>
       <c r="AJ136" s="7"/>
       <c r="AK136" s="7"/>
+      <c r="AL136" s="7"/>
     </row>
     <row r="137">
       <c r="A137" s="7" t="inlineStr">
@@ -9934,6 +10074,7 @@
       <c r="AI137" s="7"/>
       <c r="AJ137" s="7"/>
       <c r="AK137" s="7"/>
+      <c r="AL137" s="7"/>
     </row>
     <row r="138">
       <c r="A138" s="7" t="inlineStr">
@@ -10005,6 +10146,7 @@
       <c r="AI138" s="7"/>
       <c r="AJ138" s="7"/>
       <c r="AK138" s="7"/>
+      <c r="AL138" s="7"/>
     </row>
     <row r="139">
       <c r="A139" s="7" t="inlineStr">
@@ -10076,6 +10218,7 @@
       <c r="AI139" s="7"/>
       <c r="AJ139" s="7"/>
       <c r="AK139" s="7"/>
+      <c r="AL139" s="7"/>
     </row>
     <row r="140">
       <c r="A140" s="7" t="inlineStr">
@@ -10143,6 +10286,7 @@
       <c r="AI140" s="7"/>
       <c r="AJ140" s="7"/>
       <c r="AK140" s="7"/>
+      <c r="AL140" s="7"/>
     </row>
     <row r="141">
       <c r="A141" s="7" t="inlineStr">
@@ -10222,6 +10366,7 @@
       <c r="AI141" s="7"/>
       <c r="AJ141" s="7"/>
       <c r="AK141" s="7"/>
+      <c r="AL141" s="7"/>
     </row>
     <row r="142">
       <c r="A142" s="7" t="inlineStr">
@@ -10289,6 +10434,7 @@
       <c r="AI142" s="7"/>
       <c r="AJ142" s="7"/>
       <c r="AK142" s="7"/>
+      <c r="AL142" s="7"/>
     </row>
     <row r="143">
       <c r="A143" s="7" t="inlineStr">
@@ -10356,6 +10502,7 @@
       <c r="AI143" s="7"/>
       <c r="AJ143" s="7"/>
       <c r="AK143" s="7"/>
+      <c r="AL143" s="7"/>
     </row>
     <row r="144">
       <c r="A144" s="7" t="inlineStr">
@@ -10423,6 +10570,7 @@
       <c r="AI144" s="7"/>
       <c r="AJ144" s="7"/>
       <c r="AK144" s="7"/>
+      <c r="AL144" s="7"/>
     </row>
     <row r="145">
       <c r="A145" s="7" t="inlineStr">
@@ -10506,6 +10654,7 @@
       <c r="AI145" s="7"/>
       <c r="AJ145" s="7"/>
       <c r="AK145" s="7"/>
+      <c r="AL145" s="7"/>
     </row>
     <row r="146">
       <c r="A146" s="7" t="inlineStr">
@@ -10577,6 +10726,7 @@
       <c r="AI146" s="7"/>
       <c r="AJ146" s="7"/>
       <c r="AK146" s="7"/>
+      <c r="AL146" s="7"/>
     </row>
     <row r="147">
       <c r="A147" s="7" t="inlineStr">
@@ -10660,6 +10810,7 @@
       <c r="AI147" s="7"/>
       <c r="AJ147" s="7"/>
       <c r="AK147" s="7"/>
+      <c r="AL147" s="7"/>
     </row>
     <row r="148">
       <c r="A148" s="7" t="inlineStr">
@@ -10727,6 +10878,7 @@
       <c r="AI148" s="7"/>
       <c r="AJ148" s="7"/>
       <c r="AK148" s="7"/>
+      <c r="AL148" s="7"/>
     </row>
     <row r="149">
       <c r="A149" s="7" t="inlineStr">
@@ -10802,6 +10954,7 @@
       <c r="AI149" s="7"/>
       <c r="AJ149" s="7"/>
       <c r="AK149" s="7"/>
+      <c r="AL149" s="7"/>
     </row>
     <row r="150">
       <c r="A150" s="7" t="inlineStr">
@@ -10881,6 +11034,7 @@
       <c r="AI150" s="7"/>
       <c r="AJ150" s="7"/>
       <c r="AK150" s="7"/>
+      <c r="AL150" s="7"/>
     </row>
     <row r="151">
       <c r="A151" s="7" t="inlineStr">
@@ -10952,6 +11106,7 @@
       <c r="AI151" s="7"/>
       <c r="AJ151" s="7"/>
       <c r="AK151" s="7"/>
+      <c r="AL151" s="7"/>
     </row>
     <row r="152">
       <c r="A152" s="7" t="inlineStr">
@@ -11027,6 +11182,7 @@
       <c r="AI152" s="7"/>
       <c r="AJ152" s="7"/>
       <c r="AK152" s="7"/>
+      <c r="AL152" s="7"/>
     </row>
     <row r="153">
       <c r="A153" s="7" t="inlineStr">
@@ -11102,6 +11258,7 @@
       <c r="AI153" s="7"/>
       <c r="AJ153" s="7"/>
       <c r="AK153" s="7"/>
+      <c r="AL153" s="7"/>
     </row>
     <row r="154">
       <c r="A154" s="7" t="inlineStr">
@@ -11165,6 +11322,7 @@
       <c r="AI154" s="7"/>
       <c r="AJ154" s="7"/>
       <c r="AK154" s="7"/>
+      <c r="AL154" s="7"/>
     </row>
     <row r="155">
       <c r="A155" s="7" t="inlineStr">
@@ -11232,6 +11390,7 @@
       <c r="AI155" s="7"/>
       <c r="AJ155" s="7"/>
       <c r="AK155" s="7"/>
+      <c r="AL155" s="7"/>
     </row>
     <row r="156">
       <c r="A156" s="7" t="inlineStr">
@@ -11303,6 +11462,7 @@
       <c r="AI156" s="7"/>
       <c r="AJ156" s="7"/>
       <c r="AK156" s="7"/>
+      <c r="AL156" s="7"/>
     </row>
     <row r="157">
       <c r="A157" s="7" t="inlineStr">
@@ -11370,6 +11530,7 @@
       <c r="AI157" s="7"/>
       <c r="AJ157" s="7"/>
       <c r="AK157" s="7"/>
+      <c r="AL157" s="7"/>
     </row>
     <row r="158">
       <c r="A158" s="7" t="inlineStr">
@@ -11437,6 +11598,7 @@
       <c r="AI158" s="7"/>
       <c r="AJ158" s="7"/>
       <c r="AK158" s="7"/>
+      <c r="AL158" s="7"/>
     </row>
     <row r="159">
       <c r="A159" s="7" t="inlineStr">
@@ -11504,6 +11666,7 @@
       <c r="AI159" s="7"/>
       <c r="AJ159" s="7"/>
       <c r="AK159" s="7"/>
+      <c r="AL159" s="7"/>
     </row>
     <row r="160">
       <c r="A160" s="7" t="inlineStr">
@@ -11571,6 +11734,7 @@
       <c r="AI160" s="7"/>
       <c r="AJ160" s="7"/>
       <c r="AK160" s="7"/>
+      <c r="AL160" s="7"/>
     </row>
     <row r="161">
       <c r="A161" s="7" t="inlineStr">
@@ -11642,6 +11806,7 @@
       <c r="AI161" s="7"/>
       <c r="AJ161" s="7"/>
       <c r="AK161" s="7"/>
+      <c r="AL161" s="7"/>
     </row>
     <row r="162">
       <c r="A162" s="7" t="inlineStr">
@@ -11709,6 +11874,7 @@
       <c r="AI162" s="7"/>
       <c r="AJ162" s="7"/>
       <c r="AK162" s="7"/>
+      <c r="AL162" s="7"/>
     </row>
     <row r="163">
       <c r="A163" s="7" t="inlineStr">
@@ -11776,6 +11942,7 @@
       <c r="AI163" s="7"/>
       <c r="AJ163" s="7"/>
       <c r="AK163" s="7"/>
+      <c r="AL163" s="7"/>
     </row>
     <row r="164">
       <c r="A164" s="7" t="inlineStr">
@@ -11843,6 +12010,7 @@
       <c r="AI164" s="7"/>
       <c r="AJ164" s="7"/>
       <c r="AK164" s="7"/>
+      <c r="AL164" s="7"/>
     </row>
     <row r="165">
       <c r="A165" s="7" t="inlineStr">
@@ -11910,6 +12078,7 @@
       <c r="AI165" s="7"/>
       <c r="AJ165" s="7"/>
       <c r="AK165" s="7"/>
+      <c r="AL165" s="7"/>
     </row>
     <row r="166">
       <c r="A166" s="7" t="inlineStr">
@@ -11981,6 +12150,7 @@
       <c r="AI166" s="7"/>
       <c r="AJ166" s="7"/>
       <c r="AK166" s="7"/>
+      <c r="AL166" s="7"/>
     </row>
     <row r="167">
       <c r="A167" s="7" t="inlineStr">
@@ -12048,6 +12218,7 @@
       <c r="AI167" s="7"/>
       <c r="AJ167" s="7"/>
       <c r="AK167" s="7"/>
+      <c r="AL167" s="7"/>
     </row>
     <row r="168">
       <c r="A168" s="7" t="inlineStr">
@@ -12115,6 +12286,7 @@
       <c r="AI168" s="7"/>
       <c r="AJ168" s="7"/>
       <c r="AK168" s="7"/>
+      <c r="AL168" s="7"/>
     </row>
     <row r="169">
       <c r="A169" s="7" t="inlineStr">
@@ -12182,6 +12354,7 @@
       <c r="AI169" s="7"/>
       <c r="AJ169" s="7"/>
       <c r="AK169" s="7"/>
+      <c r="AL169" s="7"/>
     </row>
     <row r="170">
       <c r="A170" s="7" t="inlineStr">
@@ -12253,6 +12426,7 @@
       <c r="AI170" s="7"/>
       <c r="AJ170" s="7"/>
       <c r="AK170" s="7"/>
+      <c r="AL170" s="7"/>
     </row>
     <row r="171">
       <c r="A171" s="7" t="inlineStr">
@@ -12316,6 +12490,7 @@
       <c r="AI171" s="7"/>
       <c r="AJ171" s="7"/>
       <c r="AK171" s="7"/>
+      <c r="AL171" s="7"/>
     </row>
     <row r="172">
       <c r="A172" s="7" t="inlineStr">
@@ -12379,6 +12554,7 @@
       <c r="AI172" s="7"/>
       <c r="AJ172" s="7"/>
       <c r="AK172" s="7"/>
+      <c r="AL172" s="7"/>
     </row>
     <row r="173">
       <c r="A173" s="7" t="inlineStr">
@@ -12450,6 +12626,7 @@
       <c r="AI173" s="7"/>
       <c r="AJ173" s="7"/>
       <c r="AK173" s="7"/>
+      <c r="AL173" s="7"/>
     </row>
     <row r="174">
       <c r="A174" s="7" t="inlineStr">
@@ -12517,6 +12694,7 @@
       <c r="AI174" s="7"/>
       <c r="AJ174" s="7"/>
       <c r="AK174" s="7"/>
+      <c r="AL174" s="7"/>
     </row>
     <row r="175">
       <c r="A175" s="7" t="inlineStr">
@@ -12588,6 +12766,7 @@
       <c r="AI175" s="7"/>
       <c r="AJ175" s="7"/>
       <c r="AK175" s="7"/>
+      <c r="AL175" s="7"/>
     </row>
     <row r="176">
       <c r="A176" s="7" t="inlineStr">
@@ -12655,6 +12834,7 @@
       <c r="AI176" s="7"/>
       <c r="AJ176" s="7"/>
       <c r="AK176" s="7"/>
+      <c r="AL176" s="7"/>
     </row>
     <row r="177">
       <c r="A177" s="7" t="inlineStr">
@@ -12722,6 +12902,7 @@
       <c r="AI177" s="7"/>
       <c r="AJ177" s="7"/>
       <c r="AK177" s="7"/>
+      <c r="AL177" s="7"/>
     </row>
     <row r="178">
       <c r="A178" s="7" t="inlineStr">
@@ -12789,6 +12970,7 @@
       <c r="AI178" s="7"/>
       <c r="AJ178" s="7"/>
       <c r="AK178" s="7"/>
+      <c r="AL178" s="7"/>
     </row>
     <row r="179">
       <c r="A179" s="7" t="inlineStr">
@@ -12856,6 +13038,7 @@
       <c r="AI179" s="7"/>
       <c r="AJ179" s="7"/>
       <c r="AK179" s="7"/>
+      <c r="AL179" s="7"/>
     </row>
     <row r="180">
       <c r="A180" s="7" t="inlineStr">
@@ -12923,6 +13106,7 @@
       <c r="AI180" s="7"/>
       <c r="AJ180" s="7"/>
       <c r="AK180" s="7"/>
+      <c r="AL180" s="7"/>
     </row>
     <row r="181">
       <c r="A181" s="7" t="inlineStr">
@@ -12990,6 +13174,7 @@
       <c r="AI181" s="7"/>
       <c r="AJ181" s="7"/>
       <c r="AK181" s="7"/>
+      <c r="AL181" s="7"/>
     </row>
     <row r="182">
       <c r="A182" s="7" t="inlineStr">
@@ -13057,6 +13242,7 @@
       <c r="AI182" s="7"/>
       <c r="AJ182" s="7"/>
       <c r="AK182" s="7"/>
+      <c r="AL182" s="7"/>
     </row>
     <row r="183">
       <c r="A183" s="7" t="inlineStr">
@@ -13124,6 +13310,7 @@
       <c r="AI183" s="7"/>
       <c r="AJ183" s="7"/>
       <c r="AK183" s="7"/>
+      <c r="AL183" s="7"/>
     </row>
     <row r="184">
       <c r="A184" s="7" t="inlineStr">
@@ -13187,6 +13374,7 @@
       <c r="AI184" s="7"/>
       <c r="AJ184" s="7"/>
       <c r="AK184" s="7"/>
+      <c r="AL184" s="7"/>
     </row>
     <row r="185">
       <c r="A185" s="7" t="inlineStr">
@@ -13254,6 +13442,7 @@
       <c r="AI185" s="7"/>
       <c r="AJ185" s="7"/>
       <c r="AK185" s="7"/>
+      <c r="AL185" s="7"/>
     </row>
     <row r="186">
       <c r="A186" s="7" t="inlineStr">
@@ -13321,6 +13510,7 @@
       <c r="AI186" s="7"/>
       <c r="AJ186" s="7"/>
       <c r="AK186" s="7"/>
+      <c r="AL186" s="7"/>
     </row>
     <row r="187">
       <c r="A187" s="7" t="inlineStr">
@@ -13388,6 +13578,7 @@
       <c r="AI187" s="7"/>
       <c r="AJ187" s="7"/>
       <c r="AK187" s="7"/>
+      <c r="AL187" s="7"/>
     </row>
     <row r="188">
       <c r="A188" s="7" t="inlineStr">
@@ -13455,6 +13646,7 @@
       <c r="AI188" s="7"/>
       <c r="AJ188" s="7"/>
       <c r="AK188" s="7"/>
+      <c r="AL188" s="7"/>
     </row>
     <row r="189">
       <c r="A189" s="7" t="inlineStr">
@@ -13522,6 +13714,7 @@
       </c>
       <c r="AJ189" s="7"/>
       <c r="AK189" s="7"/>
+      <c r="AL189" s="7"/>
     </row>
     <row r="190">
       <c r="A190" s="7" t="inlineStr">
@@ -13589,6 +13782,7 @@
       </c>
       <c r="AJ190" s="7"/>
       <c r="AK190" s="7"/>
+      <c r="AL190" s="7"/>
     </row>
     <row r="191">
       <c r="A191" s="7" t="inlineStr">
@@ -13660,6 +13854,7 @@
         </is>
       </c>
       <c r="AK191" s="7"/>
+      <c r="AL191" s="7"/>
     </row>
     <row r="192">
       <c r="A192" s="7" t="inlineStr">
@@ -13727,6 +13922,7 @@
         </is>
       </c>
       <c r="AK192" s="7"/>
+      <c r="AL192" s="7"/>
     </row>
     <row r="193">
       <c r="A193" s="7" t="inlineStr">
@@ -13794,6 +13990,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AL193" s="7"/>
     </row>
     <row r="194">
       <c r="A194" s="7" t="inlineStr">
@@ -13861,6 +14058,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AL194" s="7"/>
     </row>
     <row r="195">
       <c r="A195" s="7" t="inlineStr">
@@ -13928,6 +14126,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AL195" s="7"/>
     </row>
     <row r="196">
       <c r="A196" s="7" t="inlineStr">
@@ -13991,6 +14190,7 @@
       <c r="AI196" s="7"/>
       <c r="AJ196" s="7"/>
       <c r="AK196" s="7"/>
+      <c r="AL196" s="7"/>
     </row>
     <row r="197">
       <c r="A197" s="7" t="inlineStr">
@@ -14058,6 +14258,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AL197" s="7"/>
     </row>
     <row r="198">
       <c r="A198" s="7" t="inlineStr">
@@ -14121,6 +14322,7 @@
       <c r="AI198" s="7"/>
       <c r="AJ198" s="7"/>
       <c r="AK198" s="7"/>
+      <c r="AL198" s="7"/>
     </row>
     <row r="199">
       <c r="A199" s="7" t="inlineStr">
@@ -14188,6 +14390,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AL199" s="7"/>
     </row>
     <row r="200">
       <c r="A200" s="7" t="inlineStr">
@@ -14255,6 +14458,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AL200" s="7"/>
     </row>
     <row r="201">
       <c r="A201" s="7" t="inlineStr">
@@ -14318,6 +14522,7 @@
       <c r="AI201" s="7"/>
       <c r="AJ201" s="7"/>
       <c r="AK201" s="7"/>
+      <c r="AL201" s="7"/>
     </row>
     <row r="202">
       <c r="A202" s="7" t="inlineStr">
@@ -14385,6 +14590,75 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AL202" s="7"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_195</t>
+        </is>
+      </c>
+      <c r="B203" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">저장</t>
+        </is>
+      </c>
+      <c r="C203" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">보드 저장</t>
+        </is>
+      </c>
+      <c r="D203" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B 편집 뒤 새로고침</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t xml:space="preserve">로봇 B 판을 연(편집한) 뒤 새로고침해도 로봇 A 판이 그대로 돌아오고 전투력이 정상인가? (시작 보드로 리셋 · 전투력 0 아님)</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#197 · 8132 이하 결함</t>
+        </is>
+      </c>
+      <c r="G203" s="7"/>
+      <c r="H203" s="7"/>
+      <c r="I203" s="7"/>
+      <c r="J203" s="7"/>
+      <c r="K203" s="7"/>
+      <c r="L203" s="7"/>
+      <c r="M203" s="7"/>
+      <c r="N203" s="7"/>
+      <c r="O203" s="7"/>
+      <c r="P203" s="7"/>
+      <c r="Q203" s="7"/>
+      <c r="R203" s="7"/>
+      <c r="S203" s="7"/>
+      <c r="T203" s="7"/>
+      <c r="U203" s="7"/>
+      <c r="V203" s="7"/>
+      <c r="W203" s="7"/>
+      <c r="X203" s="7"/>
+      <c r="Y203" s="7"/>
+      <c r="Z203" s="7"/>
+      <c r="AA203" s="7"/>
+      <c r="AB203" s="7"/>
+      <c r="AC203" s="7"/>
+      <c r="AD203" s="7"/>
+      <c r="AE203" s="7"/>
+      <c r="AF203" s="7"/>
+      <c r="AG203" s="7"/>
+      <c r="AH203" s="7"/>
+      <c r="AI203" s="7"/>
+      <c r="AJ203" s="7"/>
+      <c r="AK203" s="7"/>
+      <c r="AL203" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="26">
@@ -14413,9 +14687,9 @@
     <mergeCell ref="B92:B99"/>
     <mergeCell ref="B100:B106"/>
     <mergeCell ref="B107:B111"/>
-    <mergeCell ref="G7:AK7"/>
+    <mergeCell ref="G7:AL7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:AK202">
+  <conditionalFormatting sqref="G9:AL203">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
docs: QA AM열 — 사용자 육안(8133 4a6f983 · 20:4x) Pass 7 기입 · CID_196~200 신설(Fail 5 · #198 #200 #201 · S6 시간 초과)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="AO8" s="7">
-        <f>COUNTIF(AM9:AM203,"Pass")</f>
+        <f>COUNTIF(AM9:AM208,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="AO9" s="7">
-        <f>COUNTIF(AM9:AM203,"Fail")+COUNTIF(AM9:AM203,"Broken")</f>
+        <f>COUNTIF(AM9:AM208,"Fail")+COUNTIF(AM9:AM208,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -920,7 +920,7 @@
         </is>
       </c>
       <c r="AO10" s="7">
-        <f>COUNTIF(AM9:AM203,"N/A")</f>
+        <f>COUNTIF(AM9:AM208,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -993,7 +993,7 @@
         </is>
       </c>
       <c r="AO11" s="7">
-        <v>195</v>
+        <v>200</v>
       </c>
     </row>
     <row r="12">
@@ -1066,7 +1066,7 @@
         </is>
       </c>
       <c r="AO12" s="7">
-        <f>TEXT((COUNTA(AM9:AM203))/195,"0.00%")</f>
+        <f>TEXT((COUNTA(AM9:AM208))/200,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -11368,7 +11368,7 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t xml:space="preserve">#161 · 화면 승리 00:04 남음 · #164 → 15000(10-17 · 화면 남은 00:26 / 00:23)</t>
+          <t xml:space="preserve">#161 · 화면 승리 00:04 남음 · #164 → 15000(10-17 · 화면 남은 00:26 / 00:23) · 10-19 사용자 육안(8133 4a6f983 · 20:4x) — 합체 뒤 S6 도전 클리어</t>
         </is>
       </c>
       <c r="G153" s="7"/>
@@ -11415,7 +11415,11 @@
       <c r="AJ153" s="7"/>
       <c r="AK153" s="7"/>
       <c r="AL153" s="7"/>
-      <c r="AM153" s="7"/>
+      <c r="AM153" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="7" t="inlineStr">
@@ -12277,7 +12281,7 @@
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t xml:space="preserve">#173 · 🗑️ 구 「S4 통과 = 해금」(#84)</t>
+          <t xml:space="preserve">#173 · 🗑️ 구 「S4 통과 = 해금」(#84) · 10-19 사용자 육안(8133 4a6f983 · 20:4x)</t>
         </is>
       </c>
       <c r="G166" s="7"/>
@@ -12320,7 +12324,11 @@
       <c r="AJ166" s="7"/>
       <c r="AK166" s="7"/>
       <c r="AL166" s="7"/>
-      <c r="AM166" s="7"/>
+      <c r="AM166" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="7" t="inlineStr">
@@ -12350,7 +12358,7 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t xml:space="preserve">#173 · 문구 가정</t>
+          <t xml:space="preserve">#173 · 문구 가정 · 10-19 사용자 육안(8133 4a6f983 · 20:4x) — 해금 막 · 골드 50</t>
         </is>
       </c>
       <c r="G167" s="7"/>
@@ -12389,7 +12397,11 @@
       <c r="AJ167" s="7"/>
       <c r="AK167" s="7"/>
       <c r="AL167" s="7"/>
-      <c r="AM167" s="7"/>
+      <c r="AM167" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="7" t="inlineStr">
@@ -14241,7 +14253,7 @@
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t xml:space="preserve">#189 · 문구 ⚠️ 가정</t>
+          <t xml:space="preserve">#189 · 문구 ⚠️ 가정 · 10-19 사용자 육안(8133 4a6f983 · 20:4x) — 합체 막</t>
         </is>
       </c>
       <c r="G194" s="7"/>
@@ -14387,7 +14399,7 @@
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t xml:space="preserve">#190 · 끝 = 구조 판정(구현 판단)</t>
+          <t xml:space="preserve">#190 · 끝 = 구조 판정(구현 판단) · 10-19 사용자 육안(8133 4a6f983 · 20:4x) — 폭발탄 걸음 ①~⑤ 끝까지</t>
         </is>
       </c>
       <c r="G196" s="7"/>
@@ -14422,7 +14434,11 @@
       <c r="AJ196" s="7"/>
       <c r="AK196" s="7"/>
       <c r="AL196" s="7"/>
-      <c r="AM196" s="7"/>
+      <c r="AM196" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="7" t="inlineStr">
@@ -14525,7 +14541,7 @@
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t xml:space="preserve">#192</t>
+          <t xml:space="preserve">#192 · 10-19 사용자 육안(8133 4a6f983 · 20:4x) — S6 파밍 기본 BGM(도전 보스 곡은 미언급)</t>
         </is>
       </c>
       <c r="G198" s="7"/>
@@ -14560,7 +14576,11 @@
       <c r="AJ198" s="7"/>
       <c r="AK198" s="7"/>
       <c r="AL198" s="7"/>
-      <c r="AM198" s="7"/>
+      <c r="AM198" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="7" t="inlineStr">
@@ -14874,7 +14894,7 @@
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t xml:space="preserve">#197 · 8132 이하 결함</t>
+          <t xml:space="preserve">#197 · 8132 이하 결함 · 10-19 사용자 육안(8133 4a6f983 · 20:4x) — 새로고침 뒤 보드 유지</t>
         </is>
       </c>
       <c r="G203" s="7"/>
@@ -14913,7 +14933,356 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
-      <c r="AM203" s="7"/>
+      <c r="AM203" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_196</t>
+        </is>
+      </c>
+      <c r="B204" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">경제</t>
+        </is>
+      </c>
+      <c r="C204" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">바로가기 점프</t>
+        </is>
+      </c>
+      <c r="D204" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">강화 재료 지급</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t xml:space="preserve">바로가기 S3 점프에서 강화 재료 63 이 지갑에 들어와 S3 강화 막이 서는가? (점프 판 앞 보상까지만 · 중복 지급 없음)</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#198 · 4a6f983 사용자 육안 = 재료 0(Fail) → e86eb9a 에서 고침</t>
+        </is>
+      </c>
+      <c r="G204" s="7"/>
+      <c r="H204" s="7"/>
+      <c r="I204" s="7"/>
+      <c r="J204" s="7"/>
+      <c r="K204" s="7"/>
+      <c r="L204" s="7"/>
+      <c r="M204" s="7"/>
+      <c r="N204" s="7"/>
+      <c r="O204" s="7"/>
+      <c r="P204" s="7"/>
+      <c r="Q204" s="7"/>
+      <c r="R204" s="7"/>
+      <c r="S204" s="7"/>
+      <c r="T204" s="7"/>
+      <c r="U204" s="7"/>
+      <c r="V204" s="7"/>
+      <c r="W204" s="7"/>
+      <c r="X204" s="7"/>
+      <c r="Y204" s="7"/>
+      <c r="Z204" s="7"/>
+      <c r="AA204" s="7"/>
+      <c r="AB204" s="7"/>
+      <c r="AC204" s="7"/>
+      <c r="AD204" s="7"/>
+      <c r="AE204" s="7"/>
+      <c r="AF204" s="7"/>
+      <c r="AG204" s="7"/>
+      <c r="AH204" s="7"/>
+      <c r="AI204" s="7"/>
+      <c r="AJ204" s="7"/>
+      <c r="AK204" s="7"/>
+      <c r="AL204" s="7"/>
+      <c r="AM204" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_197</t>
+        </is>
+      </c>
+      <c r="B205" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">경제</t>
+        </is>
+      </c>
+      <c r="C205" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">바로가기 점프</t>
+        </is>
+      </c>
+      <c r="D205" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S6 B 강화</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t xml:space="preserve">바로가기 S6 점프에서 A 는 자동 ×1.45 · B 는 재료 50 이 들어와 B 강화 막에서 직접 강화할 수 있는가?</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#198 · 4a6f983 사용자 육안 = A·B 강화 불가(B 재료 0/50) Fail → e86eb9a</t>
+        </is>
+      </c>
+      <c r="G205" s="7"/>
+      <c r="H205" s="7"/>
+      <c r="I205" s="7"/>
+      <c r="J205" s="7"/>
+      <c r="K205" s="7"/>
+      <c r="L205" s="7"/>
+      <c r="M205" s="7"/>
+      <c r="N205" s="7"/>
+      <c r="O205" s="7"/>
+      <c r="P205" s="7"/>
+      <c r="Q205" s="7"/>
+      <c r="R205" s="7"/>
+      <c r="S205" s="7"/>
+      <c r="T205" s="7"/>
+      <c r="U205" s="7"/>
+      <c r="V205" s="7"/>
+      <c r="W205" s="7"/>
+      <c r="X205" s="7"/>
+      <c r="Y205" s="7"/>
+      <c r="Z205" s="7"/>
+      <c r="AA205" s="7"/>
+      <c r="AB205" s="7"/>
+      <c r="AC205" s="7"/>
+      <c r="AD205" s="7"/>
+      <c r="AE205" s="7"/>
+      <c r="AF205" s="7"/>
+      <c r="AG205" s="7"/>
+      <c r="AH205" s="7"/>
+      <c r="AI205" s="7"/>
+      <c r="AJ205" s="7"/>
+      <c r="AK205" s="7"/>
+      <c r="AL205" s="7"/>
+      <c r="AM205" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_198</t>
+        </is>
+      </c>
+      <c r="B206" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UI</t>
+        </is>
+      </c>
+      <c r="C206" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도전 시작 창</t>
+        </is>
+      </c>
+      <c r="D206" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">단추 자리</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도전 시작 창이 [취소] 왼쪽 · [도전 시작] 오른쪽인가? (T3 창은 [도전 시작] 하나)</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#200 · 4a6f983 = 반대 자리(사용자 확정으로 바꿈) → e86eb9a</t>
+        </is>
+      </c>
+      <c r="G206" s="7"/>
+      <c r="H206" s="7"/>
+      <c r="I206" s="7"/>
+      <c r="J206" s="7"/>
+      <c r="K206" s="7"/>
+      <c r="L206" s="7"/>
+      <c r="M206" s="7"/>
+      <c r="N206" s="7"/>
+      <c r="O206" s="7"/>
+      <c r="P206" s="7"/>
+      <c r="Q206" s="7"/>
+      <c r="R206" s="7"/>
+      <c r="S206" s="7"/>
+      <c r="T206" s="7"/>
+      <c r="U206" s="7"/>
+      <c r="V206" s="7"/>
+      <c r="W206" s="7"/>
+      <c r="X206" s="7"/>
+      <c r="Y206" s="7"/>
+      <c r="Z206" s="7"/>
+      <c r="AA206" s="7"/>
+      <c r="AB206" s="7"/>
+      <c r="AC206" s="7"/>
+      <c r="AD206" s="7"/>
+      <c r="AE206" s="7"/>
+      <c r="AF206" s="7"/>
+      <c r="AG206" s="7"/>
+      <c r="AH206" s="7"/>
+      <c r="AI206" s="7"/>
+      <c r="AJ206" s="7"/>
+      <c r="AK206" s="7"/>
+      <c r="AL206" s="7"/>
+      <c r="AM206" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_199</t>
+        </is>
+      </c>
+      <c r="B207" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C207" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도전 배지</t>
+        </is>
+      </c>
+      <c r="D207" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">요구치 0 판</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S5 · S6 처럼 요구치가 0 인 판의 도전 배지가 「목표: {주제}」만이고 「전투력 0 넘기기」가 안 뜨는가?</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#201 결함 · 4a6f983 사용자 육안 S6 「전투력 0 넘기기」 Fail → e86eb9a</t>
+        </is>
+      </c>
+      <c r="G207" s="7"/>
+      <c r="H207" s="7"/>
+      <c r="I207" s="7"/>
+      <c r="J207" s="7"/>
+      <c r="K207" s="7"/>
+      <c r="L207" s="7"/>
+      <c r="M207" s="7"/>
+      <c r="N207" s="7"/>
+      <c r="O207" s="7"/>
+      <c r="P207" s="7"/>
+      <c r="Q207" s="7"/>
+      <c r="R207" s="7"/>
+      <c r="S207" s="7"/>
+      <c r="T207" s="7"/>
+      <c r="U207" s="7"/>
+      <c r="V207" s="7"/>
+      <c r="W207" s="7"/>
+      <c r="X207" s="7"/>
+      <c r="Y207" s="7"/>
+      <c r="Z207" s="7"/>
+      <c r="AA207" s="7"/>
+      <c r="AB207" s="7"/>
+      <c r="AC207" s="7"/>
+      <c r="AD207" s="7"/>
+      <c r="AE207" s="7"/>
+      <c r="AF207" s="7"/>
+      <c r="AG207" s="7"/>
+      <c r="AH207" s="7"/>
+      <c r="AI207" s="7"/>
+      <c r="AJ207" s="7"/>
+      <c r="AK207" s="7"/>
+      <c r="AL207" s="7"/>
+      <c r="AM207" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_200</t>
+        </is>
+      </c>
+      <c r="B208" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C208" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S6 도전</t>
+        </is>
+      </c>
+      <c r="D208" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">자연 진행 보스</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t xml:space="preserve">자연 진행 S6 도전(합체 · 강화)에서 60초 안에 보스를 잡는가?</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4a6f983 사용자 육안 = 시간 초과(보스 ≈30%) · 조건 = 옛 저장(#197 전 A 판 리셋 · HUD 전투력 0) — 새 저장으로 재확인 자리</t>
+        </is>
+      </c>
+      <c r="G208" s="7"/>
+      <c r="H208" s="7"/>
+      <c r="I208" s="7"/>
+      <c r="J208" s="7"/>
+      <c r="K208" s="7"/>
+      <c r="L208" s="7"/>
+      <c r="M208" s="7"/>
+      <c r="N208" s="7"/>
+      <c r="O208" s="7"/>
+      <c r="P208" s="7"/>
+      <c r="Q208" s="7"/>
+      <c r="R208" s="7"/>
+      <c r="S208" s="7"/>
+      <c r="T208" s="7"/>
+      <c r="U208" s="7"/>
+      <c r="V208" s="7"/>
+      <c r="W208" s="7"/>
+      <c r="X208" s="7"/>
+      <c r="Y208" s="7"/>
+      <c r="Z208" s="7"/>
+      <c r="AA208" s="7"/>
+      <c r="AB208" s="7"/>
+      <c r="AC208" s="7"/>
+      <c r="AD208" s="7"/>
+      <c r="AE208" s="7"/>
+      <c r="AF208" s="7"/>
+      <c r="AG208" s="7"/>
+      <c r="AH208" s="7"/>
+      <c r="AI208" s="7"/>
+      <c r="AJ208" s="7"/>
+      <c r="AK208" s="7"/>
+      <c r="AL208" s="7"/>
+      <c r="AM208" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="26">
@@ -14944,7 +15313,7 @@
     <mergeCell ref="B107:B111"/>
     <mergeCell ref="G7:AM7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:AM203">
+  <conditionalFormatting sqref="G9:AM208">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
docs: QA AN열(e86eb9a · CID_196·197·201) · 가이드 8133 후보 e86eb9a
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -195,8 +195,9 @@
     <col min="37" max="37" width="12" customWidth="1"/>
     <col min="38" max="38" width="12" customWidth="1"/>
     <col min="39" max="39" width="12" customWidth="1"/>
-    <col min="40" max="40" width="11" customWidth="1"/>
+    <col min="40" max="40" width="12" customWidth="1"/>
     <col min="41" max="41" width="11" customWidth="1"/>
+    <col min="42" max="42" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -474,6 +475,11 @@
       <c r="AM6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">10-19 19:3x 사용자 지시 「8133 신규 기능 직접 플레이 테스트 · 볼륨 전부 끔」 ‖ 8133(4a6f983) 인앱 · 소리 셋 0% 확인 · 「처음부터」 자연 진행: T1 노드 단추 흐림(채운 뒤에도) · 머리 위 탄약 소진 아이콘 · 벨트 채움 → S1 T3 → 배지 「전투력 18 넘기기」 → 승리 「강화 재료 +30」 · [다시 도전] 없음 → S2 알림 「…모듈이 열렸습니다」 → T4 모듈 = 노랑 테두리 · 안내 줄 「생산량 모듈 · [고철] 30」 · 붙임 「-30」 떠오름 · 전투력 19→24 → S2 승리 +33 → S3 파밍 주제 「마운트 강화」 · 막 → 조립 시야 A 마운트 · 안내 → 팝오버 「63/50 · 582/300」 → 강화 = 13/50 · 고철 −300 → S3 도전(인앱 저속: 실시간 42초 = 게임 16초 · 자연 통과 시간 못 잼) → 전멸 → S4 파밍 해금 막 → 해금(골드 −50) · 태그 링 하늘색 → S4 도전 = 합체 막 · 태그 눌러도 무반응 · 합체 = 해제 · 「합체 화력 34→60 · 버스트 101」 → 승리(보상 줄 없음) → S5 알림 「복합 가공소가 열렸습니다」 · 주제 「폭발탄」 → Auto 끔 → 조립 A 판 ① 안내 → ⛔ 인앱 창 렌더/누름 좌표 불일치로 보드 칸 탭이 엉뚱한 칸(보호막)에 먹음 · 합성 이벤트는 보드(입력 시스템)에 안 닿음 → ②~⑤ · S6 B 강화 · 보스 · BGM 전환 · 새로고침 유지 = 이번 판 못 봄(도구 한계 · 결함 아님) · 상태 띠 숨김 = 문제 0 판에서 띠 없음 ✅</t>
+        </is>
+      </c>
+      <c r="AN6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8133 갈아엎음(21:02:57) · #198 점프 재료 · #199 팝오버 Lv · #200 창 단추 · #201 요구치 0 목표 줄 ‖ 10-19 코드 세션 재확인(8123): 「처음부터」 → 바로가기 S3 = 강화 막 섬(재료 ≥ 50) → 팝오버 「강화 Lv 1 · ×1.00 · 강화 재료 63/50 · 312/300 · [강화 (재료 50 · 고철 300)]」 ✅ · 바로가기 S6 = 주제 「자유 플레이 · 보스」 · 화면 흐림 막(B 강화 막 — 문구는 창 밖) ✅ · 강화 누름 · B 팝오버 · S6 배지 · 창 단추 자리 = 인앱 누름 어긋남으로 못 봄(시험이 든다) · ⚠️ 바로가기 S3 직후 HUD 전투력 0 한동안(관찰)</t>
         </is>
       </c>
     </row>
@@ -537,14 +543,15 @@
       <c r="AK7" s="2"/>
       <c r="AL7" s="2"/>
       <c r="AM7" s="2"/>
-      <c r="AN7" s="2" t="inlineStr">
+      <c r="AN7" s="2"/>
+      <c r="AO7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">버전</t>
         </is>
       </c>
-      <c r="AO7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4a6f983</t>
+      <c r="AP7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">e86eb9a</t>
         </is>
       </c>
     </row>
@@ -734,11 +741,16 @@
       </c>
       <c r="AN8" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">e86eb9a</t>
+        </is>
+      </c>
+      <c r="AO8" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">PASSrate</t>
         </is>
       </c>
-      <c r="AO8" s="7">
-        <f>COUNTIF(AM9:AM208,"Pass")</f>
+      <c r="AP8" s="7">
+        <f>COUNTIF(AN9:AN209,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -841,13 +853,14 @@
       <c r="AK9" s="7"/>
       <c r="AL9" s="7"/>
       <c r="AM9" s="7"/>
-      <c r="AN9" s="2" t="inlineStr">
+      <c r="AN9" s="7"/>
+      <c r="AO9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FAILrate</t>
         </is>
       </c>
-      <c r="AO9" s="7">
-        <f>COUNTIF(AM9:AM208,"Fail")+COUNTIF(AM9:AM208,"Broken")</f>
+      <c r="AP9" s="7">
+        <f>COUNTIF(AN9:AN209,"Fail")+COUNTIF(AN9:AN209,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -914,13 +927,14 @@
       <c r="AK10" s="7"/>
       <c r="AL10" s="7"/>
       <c r="AM10" s="7"/>
-      <c r="AN10" s="2" t="inlineStr">
+      <c r="AN10" s="7"/>
+      <c r="AO10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">N/A</t>
         </is>
       </c>
-      <c r="AO10" s="7">
-        <f>COUNTIF(AM9:AM208,"N/A")</f>
+      <c r="AP10" s="7">
+        <f>COUNTIF(AN9:AN209,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -987,13 +1001,14 @@
       <c r="AK11" s="7"/>
       <c r="AL11" s="7"/>
       <c r="AM11" s="7"/>
-      <c r="AN11" s="2" t="inlineStr">
+      <c r="AN11" s="7"/>
+      <c r="AO11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">전체 개수</t>
         </is>
       </c>
-      <c r="AO11" s="7">
-        <v>200</v>
+      <c r="AP11" s="7">
+        <v>201</v>
       </c>
     </row>
     <row r="12">
@@ -1060,13 +1075,14 @@
       <c r="AK12" s="7"/>
       <c r="AL12" s="7"/>
       <c r="AM12" s="7"/>
-      <c r="AN12" s="2" t="inlineStr">
+      <c r="AN12" s="7"/>
+      <c r="AO12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">진행율</t>
         </is>
       </c>
-      <c r="AO12" s="7">
-        <f>TEXT((COUNTA(AM9:AM208))/200,"0.00%")</f>
+      <c r="AP12" s="7">
+        <f>TEXT((COUNTA(AN9:AN209))/201,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -1137,6 +1153,7 @@
       <c r="AK13" s="7"/>
       <c r="AL13" s="7"/>
       <c r="AM13" s="7"/>
+      <c r="AN13" s="7"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -1197,6 +1214,7 @@
       <c r="AK14" s="7"/>
       <c r="AL14" s="7"/>
       <c r="AM14" s="7"/>
+      <c r="AN14" s="7"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -1293,6 +1311,7 @@
       <c r="AK15" s="7"/>
       <c r="AL15" s="7"/>
       <c r="AM15" s="7"/>
+      <c r="AN15" s="7"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -1389,6 +1408,7 @@
       <c r="AK16" s="7"/>
       <c r="AL16" s="7"/>
       <c r="AM16" s="7"/>
+      <c r="AN16" s="7"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -1490,6 +1510,7 @@
       <c r="AK17" s="7"/>
       <c r="AL17" s="7"/>
       <c r="AM17" s="7"/>
+      <c r="AN17" s="7"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -1555,6 +1576,7 @@
       <c r="AK18" s="7"/>
       <c r="AL18" s="7"/>
       <c r="AM18" s="7"/>
+      <c r="AN18" s="7"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -1615,6 +1637,7 @@
       <c r="AK19" s="7"/>
       <c r="AL19" s="7"/>
       <c r="AM19" s="7"/>
+      <c r="AN19" s="7"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1675,6 +1698,7 @@
       <c r="AK20" s="7"/>
       <c r="AL20" s="7"/>
       <c r="AM20" s="7"/>
+      <c r="AN20" s="7"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1771,6 +1795,7 @@
       <c r="AK21" s="7"/>
       <c r="AL21" s="7"/>
       <c r="AM21" s="7"/>
+      <c r="AN21" s="7"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1860,6 +1885,7 @@
       <c r="AK22" s="7"/>
       <c r="AL22" s="7"/>
       <c r="AM22" s="7"/>
+      <c r="AN22" s="7"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -1928,6 +1954,7 @@
       <c r="AK23" s="7"/>
       <c r="AL23" s="7"/>
       <c r="AM23" s="7"/>
+      <c r="AN23" s="7"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -1988,6 +2015,7 @@
       <c r="AK24" s="7"/>
       <c r="AL24" s="7"/>
       <c r="AM24" s="7"/>
+      <c r="AN24" s="7"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -2048,6 +2076,7 @@
       <c r="AK25" s="7"/>
       <c r="AL25" s="7"/>
       <c r="AM25" s="7"/>
+      <c r="AN25" s="7"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -2137,6 +2166,7 @@
       <c r="AK26" s="7"/>
       <c r="AL26" s="7"/>
       <c r="AM26" s="7"/>
+      <c r="AN26" s="7"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -2201,6 +2231,7 @@
       <c r="AK27" s="7"/>
       <c r="AL27" s="7"/>
       <c r="AM27" s="7"/>
+      <c r="AN27" s="7"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -2274,6 +2305,7 @@
       <c r="AK28" s="7"/>
       <c r="AL28" s="7"/>
       <c r="AM28" s="7"/>
+      <c r="AN28" s="7"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -2342,6 +2374,7 @@
       <c r="AK29" s="7"/>
       <c r="AL29" s="7"/>
       <c r="AM29" s="7"/>
+      <c r="AN29" s="7"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -2434,6 +2467,7 @@
       <c r="AK30" s="7"/>
       <c r="AL30" s="7"/>
       <c r="AM30" s="7"/>
+      <c r="AN30" s="7"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -2531,6 +2565,7 @@
       <c r="AK31" s="7"/>
       <c r="AL31" s="7"/>
       <c r="AM31" s="7"/>
+      <c r="AN31" s="7"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -2615,6 +2650,7 @@
       <c r="AK32" s="7"/>
       <c r="AL32" s="7"/>
       <c r="AM32" s="7"/>
+      <c r="AN32" s="7"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -2707,6 +2743,7 @@
       <c r="AK33" s="7"/>
       <c r="AL33" s="7"/>
       <c r="AM33" s="7"/>
+      <c r="AN33" s="7"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -2799,6 +2836,7 @@
       <c r="AK34" s="7"/>
       <c r="AL34" s="7"/>
       <c r="AM34" s="7"/>
+      <c r="AN34" s="7"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -2900,6 +2938,7 @@
       <c r="AK35" s="7"/>
       <c r="AL35" s="7"/>
       <c r="AM35" s="7"/>
+      <c r="AN35" s="7"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -2976,6 +3015,7 @@
       <c r="AK36" s="7"/>
       <c r="AL36" s="7"/>
       <c r="AM36" s="7"/>
+      <c r="AN36" s="7"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -3036,6 +3076,7 @@
       <c r="AK37" s="7"/>
       <c r="AL37" s="7"/>
       <c r="AM37" s="7"/>
+      <c r="AN37" s="7"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -3117,6 +3158,7 @@
       <c r="AK38" s="7"/>
       <c r="AL38" s="7"/>
       <c r="AM38" s="7"/>
+      <c r="AN38" s="7"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -3209,6 +3251,7 @@
       <c r="AK39" s="7"/>
       <c r="AL39" s="7"/>
       <c r="AM39" s="7"/>
+      <c r="AN39" s="7"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -3302,6 +3345,7 @@
       <c r="AK40" s="7"/>
       <c r="AL40" s="7"/>
       <c r="AM40" s="7"/>
+      <c r="AN40" s="7"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -3390,6 +3434,7 @@
       <c r="AK41" s="7"/>
       <c r="AL41" s="7"/>
       <c r="AM41" s="7"/>
+      <c r="AN41" s="7"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -3462,6 +3507,7 @@
       <c r="AK42" s="7"/>
       <c r="AL42" s="7"/>
       <c r="AM42" s="7"/>
+      <c r="AN42" s="7"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -3554,6 +3600,7 @@
       <c r="AK43" s="7"/>
       <c r="AL43" s="7"/>
       <c r="AM43" s="7"/>
+      <c r="AN43" s="7"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -3619,6 +3666,7 @@
       <c r="AK44" s="7"/>
       <c r="AL44" s="7"/>
       <c r="AM44" s="7"/>
+      <c r="AN44" s="7"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -3707,6 +3755,7 @@
       <c r="AK45" s="7"/>
       <c r="AL45" s="7"/>
       <c r="AM45" s="7"/>
+      <c r="AN45" s="7"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -3795,6 +3844,7 @@
       <c r="AK46" s="7"/>
       <c r="AL46" s="7"/>
       <c r="AM46" s="7"/>
+      <c r="AN46" s="7"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -3860,6 +3910,7 @@
       <c r="AK47" s="7"/>
       <c r="AL47" s="7"/>
       <c r="AM47" s="7"/>
+      <c r="AN47" s="7"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -3920,6 +3971,7 @@
       <c r="AK48" s="7"/>
       <c r="AL48" s="7"/>
       <c r="AM48" s="7"/>
+      <c r="AN48" s="7"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -3980,6 +4032,7 @@
       <c r="AK49" s="7"/>
       <c r="AL49" s="7"/>
       <c r="AM49" s="7"/>
+      <c r="AN49" s="7"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -4064,6 +4117,7 @@
       <c r="AK50" s="7"/>
       <c r="AL50" s="7"/>
       <c r="AM50" s="7"/>
+      <c r="AN50" s="7"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -4148,6 +4202,7 @@
       <c r="AK51" s="7"/>
       <c r="AL51" s="7"/>
       <c r="AM51" s="7"/>
+      <c r="AN51" s="7"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -4213,6 +4268,7 @@
       <c r="AK52" s="7"/>
       <c r="AL52" s="7"/>
       <c r="AM52" s="7"/>
+      <c r="AN52" s="7"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -4278,6 +4334,7 @@
       <c r="AK53" s="7"/>
       <c r="AL53" s="7"/>
       <c r="AM53" s="7"/>
+      <c r="AN53" s="7"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -4338,6 +4395,7 @@
       <c r="AK54" s="7"/>
       <c r="AL54" s="7"/>
       <c r="AM54" s="7"/>
+      <c r="AN54" s="7"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -4434,6 +4492,7 @@
       <c r="AK55" s="7"/>
       <c r="AL55" s="7"/>
       <c r="AM55" s="7"/>
+      <c r="AN55" s="7"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -4510,6 +4569,7 @@
       <c r="AK56" s="7"/>
       <c r="AL56" s="7"/>
       <c r="AM56" s="7"/>
+      <c r="AN56" s="7"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -4595,6 +4655,7 @@
       <c r="AK57" s="7"/>
       <c r="AL57" s="7"/>
       <c r="AM57" s="7"/>
+      <c r="AN57" s="7"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -4688,6 +4749,7 @@
       <c r="AK58" s="7"/>
       <c r="AL58" s="7"/>
       <c r="AM58" s="7"/>
+      <c r="AN58" s="7"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -4748,6 +4810,7 @@
       <c r="AK59" s="7"/>
       <c r="AL59" s="7"/>
       <c r="AM59" s="7"/>
+      <c r="AN59" s="7"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -4808,6 +4871,7 @@
       <c r="AK60" s="7"/>
       <c r="AL60" s="7"/>
       <c r="AM60" s="7"/>
+      <c r="AN60" s="7"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -4880,6 +4944,7 @@
       <c r="AK61" s="7"/>
       <c r="AL61" s="7"/>
       <c r="AM61" s="7"/>
+      <c r="AN61" s="7"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -4960,6 +5025,7 @@
       <c r="AK62" s="7"/>
       <c r="AL62" s="7"/>
       <c r="AM62" s="7"/>
+      <c r="AN62" s="7"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -5032,6 +5098,7 @@
       <c r="AK63" s="7"/>
       <c r="AL63" s="7"/>
       <c r="AM63" s="7"/>
+      <c r="AN63" s="7"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -5092,6 +5159,7 @@
       <c r="AK64" s="7"/>
       <c r="AL64" s="7"/>
       <c r="AM64" s="7"/>
+      <c r="AN64" s="7"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -5157,6 +5225,7 @@
       <c r="AK65" s="7"/>
       <c r="AL65" s="7"/>
       <c r="AM65" s="7"/>
+      <c r="AN65" s="7"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
@@ -5229,6 +5298,7 @@
       <c r="AK66" s="7"/>
       <c r="AL66" s="7"/>
       <c r="AM66" s="7"/>
+      <c r="AN66" s="7"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -5289,6 +5359,7 @@
       <c r="AK67" s="7"/>
       <c r="AL67" s="7"/>
       <c r="AM67" s="7"/>
+      <c r="AN67" s="7"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
@@ -5353,6 +5424,7 @@
       <c r="AK68" s="7"/>
       <c r="AL68" s="7"/>
       <c r="AM68" s="7"/>
+      <c r="AN68" s="7"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -5449,6 +5521,7 @@
       <c r="AK69" s="7"/>
       <c r="AL69" s="7"/>
       <c r="AM69" s="7"/>
+      <c r="AN69" s="7"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
@@ -5509,6 +5582,7 @@
       <c r="AK70" s="7"/>
       <c r="AL70" s="7"/>
       <c r="AM70" s="7"/>
+      <c r="AN70" s="7"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -5574,6 +5648,7 @@
       <c r="AK71" s="7"/>
       <c r="AL71" s="7"/>
       <c r="AM71" s="7"/>
+      <c r="AN71" s="7"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
@@ -5650,6 +5725,7 @@
       <c r="AK72" s="7"/>
       <c r="AL72" s="7"/>
       <c r="AM72" s="7"/>
+      <c r="AN72" s="7"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
@@ -5715,6 +5791,7 @@
       <c r="AK73" s="7"/>
       <c r="AL73" s="7"/>
       <c r="AM73" s="7"/>
+      <c r="AN73" s="7"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -5775,6 +5852,7 @@
       <c r="AK74" s="7"/>
       <c r="AL74" s="7"/>
       <c r="AM74" s="7"/>
+      <c r="AN74" s="7"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -5835,6 +5913,7 @@
       <c r="AK75" s="7"/>
       <c r="AL75" s="7"/>
       <c r="AM75" s="7"/>
+      <c r="AN75" s="7"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -5895,6 +5974,7 @@
       <c r="AK76" s="7"/>
       <c r="AL76" s="7"/>
       <c r="AM76" s="7"/>
+      <c r="AN76" s="7"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -5959,6 +6039,7 @@
       <c r="AK77" s="7"/>
       <c r="AL77" s="7"/>
       <c r="AM77" s="7"/>
+      <c r="AN77" s="7"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
@@ -6019,6 +6100,7 @@
       <c r="AK78" s="7"/>
       <c r="AL78" s="7"/>
       <c r="AM78" s="7"/>
+      <c r="AN78" s="7"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -6084,6 +6166,7 @@
       <c r="AK79" s="7"/>
       <c r="AL79" s="7"/>
       <c r="AM79" s="7"/>
+      <c r="AN79" s="7"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
@@ -6160,6 +6243,7 @@
       <c r="AK80" s="7"/>
       <c r="AL80" s="7"/>
       <c r="AM80" s="7"/>
+      <c r="AN80" s="7"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
@@ -6224,6 +6308,7 @@
       <c r="AK81" s="7"/>
       <c r="AL81" s="7"/>
       <c r="AM81" s="7"/>
+      <c r="AN81" s="7"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
@@ -6284,6 +6369,7 @@
       <c r="AK82" s="7"/>
       <c r="AL82" s="7"/>
       <c r="AM82" s="7"/>
+      <c r="AN82" s="7"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
@@ -6349,6 +6435,7 @@
       <c r="AK83" s="7"/>
       <c r="AL83" s="7"/>
       <c r="AM83" s="7"/>
+      <c r="AN83" s="7"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
@@ -6409,6 +6496,7 @@
       <c r="AK84" s="7"/>
       <c r="AL84" s="7"/>
       <c r="AM84" s="7"/>
+      <c r="AN84" s="7"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
@@ -6469,6 +6557,7 @@
       <c r="AK85" s="7"/>
       <c r="AL85" s="7"/>
       <c r="AM85" s="7"/>
+      <c r="AN85" s="7"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
@@ -6534,6 +6623,7 @@
       <c r="AK86" s="7"/>
       <c r="AL86" s="7"/>
       <c r="AM86" s="7"/>
+      <c r="AN86" s="7"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
@@ -6594,6 +6684,7 @@
       <c r="AK87" s="7"/>
       <c r="AL87" s="7"/>
       <c r="AM87" s="7"/>
+      <c r="AN87" s="7"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
@@ -6654,6 +6745,7 @@
       <c r="AK88" s="7"/>
       <c r="AL88" s="7"/>
       <c r="AM88" s="7"/>
+      <c r="AN88" s="7"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
@@ -6714,6 +6806,7 @@
       <c r="AK89" s="7"/>
       <c r="AL89" s="7"/>
       <c r="AM89" s="7"/>
+      <c r="AN89" s="7"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
@@ -6803,6 +6896,7 @@
       <c r="AK90" s="7"/>
       <c r="AL90" s="7"/>
       <c r="AM90" s="7"/>
+      <c r="AN90" s="7"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
@@ -6863,6 +6957,7 @@
       <c r="AK91" s="7"/>
       <c r="AL91" s="7"/>
       <c r="AM91" s="7"/>
+      <c r="AN91" s="7"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
@@ -6959,6 +7054,7 @@
       <c r="AK92" s="7"/>
       <c r="AL92" s="7"/>
       <c r="AM92" s="7"/>
+      <c r="AN92" s="7"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
@@ -7060,6 +7156,7 @@
       <c r="AK93" s="7"/>
       <c r="AL93" s="7"/>
       <c r="AM93" s="7"/>
+      <c r="AN93" s="7"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
@@ -7125,6 +7222,7 @@
       <c r="AK94" s="7"/>
       <c r="AL94" s="7"/>
       <c r="AM94" s="7"/>
+      <c r="AN94" s="7"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
@@ -7190,6 +7288,7 @@
       <c r="AK95" s="7"/>
       <c r="AL95" s="7"/>
       <c r="AM95" s="7"/>
+      <c r="AN95" s="7"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
@@ -7274,6 +7373,7 @@
       <c r="AK96" s="7"/>
       <c r="AL96" s="7"/>
       <c r="AM96" s="7"/>
+      <c r="AN96" s="7"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="inlineStr">
@@ -7334,6 +7434,7 @@
       <c r="AK97" s="7"/>
       <c r="AL97" s="7"/>
       <c r="AM97" s="7"/>
+      <c r="AN97" s="7"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
@@ -7394,6 +7495,7 @@
       <c r="AK98" s="7"/>
       <c r="AL98" s="7"/>
       <c r="AM98" s="7"/>
+      <c r="AN98" s="7"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
@@ -7454,6 +7556,7 @@
       <c r="AK99" s="7"/>
       <c r="AL99" s="7"/>
       <c r="AM99" s="7"/>
+      <c r="AN99" s="7"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
@@ -7523,6 +7626,7 @@
       <c r="AK100" s="7"/>
       <c r="AL100" s="7"/>
       <c r="AM100" s="7"/>
+      <c r="AN100" s="7"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
@@ -7583,6 +7687,7 @@
       <c r="AK101" s="7"/>
       <c r="AL101" s="7"/>
       <c r="AM101" s="7"/>
+      <c r="AN101" s="7"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
@@ -7643,6 +7748,7 @@
       <c r="AK102" s="7"/>
       <c r="AL102" s="7"/>
       <c r="AM102" s="7"/>
+      <c r="AN102" s="7"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="inlineStr">
@@ -7703,6 +7809,7 @@
       <c r="AK103" s="7"/>
       <c r="AL103" s="7"/>
       <c r="AM103" s="7"/>
+      <c r="AN103" s="7"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="inlineStr">
@@ -7768,6 +7875,7 @@
       <c r="AK104" s="7"/>
       <c r="AL104" s="7"/>
       <c r="AM104" s="7"/>
+      <c r="AN104" s="7"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
@@ -7828,6 +7936,7 @@
       <c r="AK105" s="7"/>
       <c r="AL105" s="7"/>
       <c r="AM105" s="7"/>
+      <c r="AN105" s="7"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
@@ -7888,6 +7997,7 @@
       <c r="AK106" s="7"/>
       <c r="AL106" s="7"/>
       <c r="AM106" s="7"/>
+      <c r="AN106" s="7"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
@@ -7948,6 +8058,7 @@
       <c r="AK107" s="7"/>
       <c r="AL107" s="7"/>
       <c r="AM107" s="7"/>
+      <c r="AN107" s="7"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
@@ -8012,6 +8123,7 @@
       <c r="AK108" s="7"/>
       <c r="AL108" s="7"/>
       <c r="AM108" s="7"/>
+      <c r="AN108" s="7"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="inlineStr">
@@ -8081,6 +8193,7 @@
       <c r="AK109" s="7"/>
       <c r="AL109" s="7"/>
       <c r="AM109" s="7"/>
+      <c r="AN109" s="7"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
@@ -8158,6 +8271,7 @@
       <c r="AK110" s="7"/>
       <c r="AL110" s="7"/>
       <c r="AM110" s="7"/>
+      <c r="AN110" s="7"/>
     </row>
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
@@ -8238,6 +8352,7 @@
       <c r="AK111" s="7"/>
       <c r="AL111" s="7"/>
       <c r="AM111" s="7"/>
+      <c r="AN111" s="7"/>
     </row>
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
@@ -8315,6 +8430,7 @@
       <c r="AK112" s="7"/>
       <c r="AL112" s="7"/>
       <c r="AM112" s="7"/>
+      <c r="AN112" s="7"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
@@ -8384,6 +8500,7 @@
       <c r="AK113" s="7"/>
       <c r="AL113" s="7"/>
       <c r="AM113" s="7"/>
+      <c r="AN113" s="7"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="inlineStr">
@@ -8469,6 +8586,7 @@
       <c r="AK114" s="7"/>
       <c r="AL114" s="7"/>
       <c r="AM114" s="7"/>
+      <c r="AN114" s="7"/>
     </row>
     <row r="115">
       <c r="A115" s="7" t="inlineStr">
@@ -8546,6 +8664,7 @@
       <c r="AK115" s="7"/>
       <c r="AL115" s="7"/>
       <c r="AM115" s="7"/>
+      <c r="AN115" s="7"/>
     </row>
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
@@ -8631,6 +8750,7 @@
       <c r="AK116" s="7"/>
       <c r="AL116" s="7"/>
       <c r="AM116" s="7"/>
+      <c r="AN116" s="7"/>
     </row>
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
@@ -8712,6 +8832,7 @@
       <c r="AK117" s="7"/>
       <c r="AL117" s="7"/>
       <c r="AM117" s="7"/>
+      <c r="AN117" s="7"/>
     </row>
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
@@ -8793,6 +8914,7 @@
       <c r="AK118" s="7"/>
       <c r="AL118" s="7"/>
       <c r="AM118" s="7"/>
+      <c r="AN118" s="7"/>
     </row>
     <row r="119">
       <c r="A119" s="7" t="inlineStr">
@@ -8870,6 +8992,7 @@
       <c r="AK119" s="7"/>
       <c r="AL119" s="7"/>
       <c r="AM119" s="7"/>
+      <c r="AN119" s="7"/>
     </row>
     <row r="120">
       <c r="A120" s="7" t="inlineStr">
@@ -8939,6 +9062,7 @@
       <c r="AK120" s="7"/>
       <c r="AL120" s="7"/>
       <c r="AM120" s="7"/>
+      <c r="AN120" s="7"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="inlineStr">
@@ -9020,6 +9144,7 @@
       <c r="AK121" s="7"/>
       <c r="AL121" s="7"/>
       <c r="AM121" s="7"/>
+      <c r="AN121" s="7"/>
     </row>
     <row r="122">
       <c r="A122" s="7" t="inlineStr">
@@ -9101,6 +9226,7 @@
       <c r="AK122" s="7"/>
       <c r="AL122" s="7"/>
       <c r="AM122" s="7"/>
+      <c r="AN122" s="7"/>
     </row>
     <row r="123">
       <c r="A123" s="7" t="inlineStr">
@@ -9170,6 +9296,7 @@
       <c r="AK123" s="7"/>
       <c r="AL123" s="7"/>
       <c r="AM123" s="7"/>
+      <c r="AN123" s="7"/>
     </row>
     <row r="124">
       <c r="A124" s="7" t="inlineStr">
@@ -9247,6 +9374,7 @@
       <c r="AK124" s="7"/>
       <c r="AL124" s="7"/>
       <c r="AM124" s="7"/>
+      <c r="AN124" s="7"/>
     </row>
     <row r="125">
       <c r="A125" s="7" t="inlineStr">
@@ -9316,6 +9444,7 @@
       <c r="AK125" s="7"/>
       <c r="AL125" s="7"/>
       <c r="AM125" s="7"/>
+      <c r="AN125" s="7"/>
     </row>
     <row r="126">
       <c r="A126" s="7" t="inlineStr">
@@ -9385,6 +9514,7 @@
       <c r="AK126" s="7"/>
       <c r="AL126" s="7"/>
       <c r="AM126" s="7"/>
+      <c r="AN126" s="7"/>
     </row>
     <row r="127">
       <c r="A127" s="7" t="inlineStr">
@@ -9458,6 +9588,7 @@
       <c r="AK127" s="7"/>
       <c r="AL127" s="7"/>
       <c r="AM127" s="7"/>
+      <c r="AN127" s="7"/>
     </row>
     <row r="128">
       <c r="A128" s="7" t="inlineStr">
@@ -9531,6 +9662,7 @@
       <c r="AK128" s="7"/>
       <c r="AL128" s="7"/>
       <c r="AM128" s="7"/>
+      <c r="AN128" s="7"/>
     </row>
     <row r="129">
       <c r="A129" s="7" t="inlineStr">
@@ -9604,6 +9736,7 @@
       <c r="AK129" s="7"/>
       <c r="AL129" s="7"/>
       <c r="AM129" s="7"/>
+      <c r="AN129" s="7"/>
     </row>
     <row r="130">
       <c r="A130" s="7" t="inlineStr">
@@ -9673,6 +9806,7 @@
       <c r="AK130" s="7"/>
       <c r="AL130" s="7"/>
       <c r="AM130" s="7"/>
+      <c r="AN130" s="7"/>
     </row>
     <row r="131">
       <c r="A131" s="7" t="inlineStr">
@@ -9750,6 +9884,7 @@
       <c r="AK131" s="7"/>
       <c r="AL131" s="7"/>
       <c r="AM131" s="7"/>
+      <c r="AN131" s="7"/>
     </row>
     <row r="132">
       <c r="A132" s="7" t="inlineStr">
@@ -9831,6 +9966,7 @@
       <c r="AK132" s="7"/>
       <c r="AL132" s="7"/>
       <c r="AM132" s="7"/>
+      <c r="AN132" s="7"/>
     </row>
     <row r="133">
       <c r="A133" s="7" t="inlineStr">
@@ -9912,6 +10048,7 @@
       <c r="AK133" s="7"/>
       <c r="AL133" s="7"/>
       <c r="AM133" s="7"/>
+      <c r="AN133" s="7"/>
     </row>
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
@@ -9989,6 +10126,7 @@
       <c r="AK134" s="7"/>
       <c r="AL134" s="7"/>
       <c r="AM134" s="7"/>
+      <c r="AN134" s="7"/>
     </row>
     <row r="135">
       <c r="A135" s="7" t="inlineStr">
@@ -10066,6 +10204,7 @@
       <c r="AK135" s="7"/>
       <c r="AL135" s="7"/>
       <c r="AM135" s="7"/>
+      <c r="AN135" s="7"/>
     </row>
     <row r="136">
       <c r="A136" s="7" t="inlineStr">
@@ -10143,6 +10282,7 @@
       <c r="AK136" s="7"/>
       <c r="AL136" s="7"/>
       <c r="AM136" s="7"/>
+      <c r="AN136" s="7"/>
     </row>
     <row r="137">
       <c r="A137" s="7" t="inlineStr">
@@ -10216,6 +10356,7 @@
       <c r="AK137" s="7"/>
       <c r="AL137" s="7"/>
       <c r="AM137" s="7"/>
+      <c r="AN137" s="7"/>
     </row>
     <row r="138">
       <c r="A138" s="7" t="inlineStr">
@@ -10289,6 +10430,7 @@
       <c r="AK138" s="7"/>
       <c r="AL138" s="7"/>
       <c r="AM138" s="7"/>
+      <c r="AN138" s="7"/>
     </row>
     <row r="139">
       <c r="A139" s="7" t="inlineStr">
@@ -10362,6 +10504,7 @@
       <c r="AK139" s="7"/>
       <c r="AL139" s="7"/>
       <c r="AM139" s="7"/>
+      <c r="AN139" s="7"/>
     </row>
     <row r="140">
       <c r="A140" s="7" t="inlineStr">
@@ -10431,6 +10574,7 @@
       <c r="AK140" s="7"/>
       <c r="AL140" s="7"/>
       <c r="AM140" s="7"/>
+      <c r="AN140" s="7"/>
     </row>
     <row r="141">
       <c r="A141" s="7" t="inlineStr">
@@ -10512,6 +10656,7 @@
       <c r="AK141" s="7"/>
       <c r="AL141" s="7"/>
       <c r="AM141" s="7"/>
+      <c r="AN141" s="7"/>
     </row>
     <row r="142">
       <c r="A142" s="7" t="inlineStr">
@@ -10581,6 +10726,7 @@
       <c r="AK142" s="7"/>
       <c r="AL142" s="7"/>
       <c r="AM142" s="7"/>
+      <c r="AN142" s="7"/>
     </row>
     <row r="143">
       <c r="A143" s="7" t="inlineStr">
@@ -10650,6 +10796,7 @@
       <c r="AK143" s="7"/>
       <c r="AL143" s="7"/>
       <c r="AM143" s="7"/>
+      <c r="AN143" s="7"/>
     </row>
     <row r="144">
       <c r="A144" s="7" t="inlineStr">
@@ -10719,6 +10866,7 @@
       <c r="AK144" s="7"/>
       <c r="AL144" s="7"/>
       <c r="AM144" s="7"/>
+      <c r="AN144" s="7"/>
     </row>
     <row r="145">
       <c r="A145" s="7" t="inlineStr">
@@ -10804,6 +10952,7 @@
       <c r="AK145" s="7"/>
       <c r="AL145" s="7"/>
       <c r="AM145" s="7"/>
+      <c r="AN145" s="7"/>
     </row>
     <row r="146">
       <c r="A146" s="7" t="inlineStr">
@@ -10877,6 +11026,7 @@
       <c r="AK146" s="7"/>
       <c r="AL146" s="7"/>
       <c r="AM146" s="7"/>
+      <c r="AN146" s="7"/>
     </row>
     <row r="147">
       <c r="A147" s="7" t="inlineStr">
@@ -10962,6 +11112,7 @@
       <c r="AK147" s="7"/>
       <c r="AL147" s="7"/>
       <c r="AM147" s="7"/>
+      <c r="AN147" s="7"/>
     </row>
     <row r="148">
       <c r="A148" s="7" t="inlineStr">
@@ -11031,6 +11182,7 @@
       <c r="AK148" s="7"/>
       <c r="AL148" s="7"/>
       <c r="AM148" s="7"/>
+      <c r="AN148" s="7"/>
     </row>
     <row r="149">
       <c r="A149" s="7" t="inlineStr">
@@ -11108,6 +11260,7 @@
       <c r="AK149" s="7"/>
       <c r="AL149" s="7"/>
       <c r="AM149" s="7"/>
+      <c r="AN149" s="7"/>
     </row>
     <row r="150">
       <c r="A150" s="7" t="inlineStr">
@@ -11189,6 +11342,7 @@
       <c r="AK150" s="7"/>
       <c r="AL150" s="7"/>
       <c r="AM150" s="7"/>
+      <c r="AN150" s="7"/>
     </row>
     <row r="151">
       <c r="A151" s="7" t="inlineStr">
@@ -11262,6 +11416,7 @@
       <c r="AK151" s="7"/>
       <c r="AL151" s="7"/>
       <c r="AM151" s="7"/>
+      <c r="AN151" s="7"/>
     </row>
     <row r="152">
       <c r="A152" s="7" t="inlineStr">
@@ -11339,6 +11494,7 @@
       <c r="AK152" s="7"/>
       <c r="AL152" s="7"/>
       <c r="AM152" s="7"/>
+      <c r="AN152" s="7"/>
     </row>
     <row r="153">
       <c r="A153" s="7" t="inlineStr">
@@ -11420,6 +11576,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AN153" s="7"/>
     </row>
     <row r="154">
       <c r="A154" s="7" t="inlineStr">
@@ -11485,6 +11642,7 @@
       <c r="AK154" s="7"/>
       <c r="AL154" s="7"/>
       <c r="AM154" s="7"/>
+      <c r="AN154" s="7"/>
     </row>
     <row r="155">
       <c r="A155" s="7" t="inlineStr">
@@ -11554,6 +11712,7 @@
       <c r="AK155" s="7"/>
       <c r="AL155" s="7"/>
       <c r="AM155" s="7"/>
+      <c r="AN155" s="7"/>
     </row>
     <row r="156">
       <c r="A156" s="7" t="inlineStr">
@@ -11627,6 +11786,7 @@
       <c r="AK156" s="7"/>
       <c r="AL156" s="7"/>
       <c r="AM156" s="7"/>
+      <c r="AN156" s="7"/>
     </row>
     <row r="157">
       <c r="A157" s="7" t="inlineStr">
@@ -11696,6 +11856,7 @@
       <c r="AK157" s="7"/>
       <c r="AL157" s="7"/>
       <c r="AM157" s="7"/>
+      <c r="AN157" s="7"/>
     </row>
     <row r="158">
       <c r="A158" s="7" t="inlineStr">
@@ -11765,6 +11926,7 @@
       <c r="AK158" s="7"/>
       <c r="AL158" s="7"/>
       <c r="AM158" s="7"/>
+      <c r="AN158" s="7"/>
     </row>
     <row r="159">
       <c r="A159" s="7" t="inlineStr">
@@ -11834,6 +11996,7 @@
       <c r="AK159" s="7"/>
       <c r="AL159" s="7"/>
       <c r="AM159" s="7"/>
+      <c r="AN159" s="7"/>
     </row>
     <row r="160">
       <c r="A160" s="7" t="inlineStr">
@@ -11903,6 +12066,7 @@
       <c r="AK160" s="7"/>
       <c r="AL160" s="7"/>
       <c r="AM160" s="7"/>
+      <c r="AN160" s="7"/>
     </row>
     <row r="161">
       <c r="A161" s="7" t="inlineStr">
@@ -11976,6 +12140,7 @@
       <c r="AK161" s="7"/>
       <c r="AL161" s="7"/>
       <c r="AM161" s="7"/>
+      <c r="AN161" s="7"/>
     </row>
     <row r="162">
       <c r="A162" s="7" t="inlineStr">
@@ -12045,6 +12210,7 @@
       <c r="AK162" s="7"/>
       <c r="AL162" s="7"/>
       <c r="AM162" s="7"/>
+      <c r="AN162" s="7"/>
     </row>
     <row r="163">
       <c r="A163" s="7" t="inlineStr">
@@ -12114,6 +12280,7 @@
       <c r="AK163" s="7"/>
       <c r="AL163" s="7"/>
       <c r="AM163" s="7"/>
+      <c r="AN163" s="7"/>
     </row>
     <row r="164">
       <c r="A164" s="7" t="inlineStr">
@@ -12183,6 +12350,7 @@
       <c r="AK164" s="7"/>
       <c r="AL164" s="7"/>
       <c r="AM164" s="7"/>
+      <c r="AN164" s="7"/>
     </row>
     <row r="165">
       <c r="A165" s="7" t="inlineStr">
@@ -12252,6 +12420,7 @@
       <c r="AK165" s="7"/>
       <c r="AL165" s="7"/>
       <c r="AM165" s="7"/>
+      <c r="AN165" s="7"/>
     </row>
     <row r="166">
       <c r="A166" s="7" t="inlineStr">
@@ -12329,6 +12498,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AN166" s="7"/>
     </row>
     <row r="167">
       <c r="A167" s="7" t="inlineStr">
@@ -12402,6 +12572,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AN167" s="7"/>
     </row>
     <row r="168">
       <c r="A168" s="7" t="inlineStr">
@@ -12471,6 +12642,7 @@
       <c r="AK168" s="7"/>
       <c r="AL168" s="7"/>
       <c r="AM168" s="7"/>
+      <c r="AN168" s="7"/>
     </row>
     <row r="169">
       <c r="A169" s="7" t="inlineStr">
@@ -12540,6 +12712,7 @@
       <c r="AK169" s="7"/>
       <c r="AL169" s="7"/>
       <c r="AM169" s="7"/>
+      <c r="AN169" s="7"/>
     </row>
     <row r="170">
       <c r="A170" s="7" t="inlineStr">
@@ -12613,6 +12786,7 @@
       <c r="AK170" s="7"/>
       <c r="AL170" s="7"/>
       <c r="AM170" s="7"/>
+      <c r="AN170" s="7"/>
     </row>
     <row r="171">
       <c r="A171" s="7" t="inlineStr">
@@ -12678,6 +12852,7 @@
       <c r="AK171" s="7"/>
       <c r="AL171" s="7"/>
       <c r="AM171" s="7"/>
+      <c r="AN171" s="7"/>
     </row>
     <row r="172">
       <c r="A172" s="7" t="inlineStr">
@@ -12743,6 +12918,7 @@
       <c r="AK172" s="7"/>
       <c r="AL172" s="7"/>
       <c r="AM172" s="7"/>
+      <c r="AN172" s="7"/>
     </row>
     <row r="173">
       <c r="A173" s="7" t="inlineStr">
@@ -12816,6 +12992,7 @@
       <c r="AK173" s="7"/>
       <c r="AL173" s="7"/>
       <c r="AM173" s="7"/>
+      <c r="AN173" s="7"/>
     </row>
     <row r="174">
       <c r="A174" s="7" t="inlineStr">
@@ -12885,6 +13062,7 @@
       <c r="AK174" s="7"/>
       <c r="AL174" s="7"/>
       <c r="AM174" s="7"/>
+      <c r="AN174" s="7"/>
     </row>
     <row r="175">
       <c r="A175" s="7" t="inlineStr">
@@ -12958,6 +13136,7 @@
       <c r="AK175" s="7"/>
       <c r="AL175" s="7"/>
       <c r="AM175" s="7"/>
+      <c r="AN175" s="7"/>
     </row>
     <row r="176">
       <c r="A176" s="7" t="inlineStr">
@@ -13027,6 +13206,7 @@
       <c r="AK176" s="7"/>
       <c r="AL176" s="7"/>
       <c r="AM176" s="7"/>
+      <c r="AN176" s="7"/>
     </row>
     <row r="177">
       <c r="A177" s="7" t="inlineStr">
@@ -13096,6 +13276,7 @@
       <c r="AK177" s="7"/>
       <c r="AL177" s="7"/>
       <c r="AM177" s="7"/>
+      <c r="AN177" s="7"/>
     </row>
     <row r="178">
       <c r="A178" s="7" t="inlineStr">
@@ -13165,6 +13346,7 @@
       <c r="AK178" s="7"/>
       <c r="AL178" s="7"/>
       <c r="AM178" s="7"/>
+      <c r="AN178" s="7"/>
     </row>
     <row r="179">
       <c r="A179" s="7" t="inlineStr">
@@ -13234,6 +13416,7 @@
       <c r="AK179" s="7"/>
       <c r="AL179" s="7"/>
       <c r="AM179" s="7"/>
+      <c r="AN179" s="7"/>
     </row>
     <row r="180">
       <c r="A180" s="7" t="inlineStr">
@@ -13303,6 +13486,7 @@
       <c r="AK180" s="7"/>
       <c r="AL180" s="7"/>
       <c r="AM180" s="7"/>
+      <c r="AN180" s="7"/>
     </row>
     <row r="181">
       <c r="A181" s="7" t="inlineStr">
@@ -13372,6 +13556,7 @@
       <c r="AK181" s="7"/>
       <c r="AL181" s="7"/>
       <c r="AM181" s="7"/>
+      <c r="AN181" s="7"/>
     </row>
     <row r="182">
       <c r="A182" s="7" t="inlineStr">
@@ -13441,6 +13626,7 @@
       <c r="AK182" s="7"/>
       <c r="AL182" s="7"/>
       <c r="AM182" s="7"/>
+      <c r="AN182" s="7"/>
     </row>
     <row r="183">
       <c r="A183" s="7" t="inlineStr">
@@ -13510,6 +13696,7 @@
       <c r="AK183" s="7"/>
       <c r="AL183" s="7"/>
       <c r="AM183" s="7"/>
+      <c r="AN183" s="7"/>
     </row>
     <row r="184">
       <c r="A184" s="7" t="inlineStr">
@@ -13575,6 +13762,7 @@
       <c r="AK184" s="7"/>
       <c r="AL184" s="7"/>
       <c r="AM184" s="7"/>
+      <c r="AN184" s="7"/>
     </row>
     <row r="185">
       <c r="A185" s="7" t="inlineStr">
@@ -13644,6 +13832,7 @@
       <c r="AK185" s="7"/>
       <c r="AL185" s="7"/>
       <c r="AM185" s="7"/>
+      <c r="AN185" s="7"/>
     </row>
     <row r="186">
       <c r="A186" s="7" t="inlineStr">
@@ -13713,6 +13902,7 @@
       <c r="AK186" s="7"/>
       <c r="AL186" s="7"/>
       <c r="AM186" s="7"/>
+      <c r="AN186" s="7"/>
     </row>
     <row r="187">
       <c r="A187" s="7" t="inlineStr">
@@ -13786,6 +13976,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AN187" s="7"/>
     </row>
     <row r="188">
       <c r="A188" s="7" t="inlineStr">
@@ -13859,6 +14050,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AN188" s="7"/>
     </row>
     <row r="189">
       <c r="A189" s="7" t="inlineStr">
@@ -13932,6 +14124,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AN189" s="7"/>
     </row>
     <row r="190">
       <c r="A190" s="7" t="inlineStr">
@@ -14005,6 +14198,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AN190" s="7"/>
     </row>
     <row r="191">
       <c r="A191" s="7" t="inlineStr">
@@ -14078,6 +14272,7 @@
       <c r="AK191" s="7"/>
       <c r="AL191" s="7"/>
       <c r="AM191" s="7"/>
+      <c r="AN191" s="7"/>
     </row>
     <row r="192">
       <c r="A192" s="7" t="inlineStr">
@@ -14151,6 +14346,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AN192" s="7"/>
     </row>
     <row r="193">
       <c r="A193" s="7" t="inlineStr">
@@ -14224,6 +14420,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AN193" s="7"/>
     </row>
     <row r="194">
       <c r="A194" s="7" t="inlineStr">
@@ -14297,6 +14494,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AN194" s="7"/>
     </row>
     <row r="195">
       <c r="A195" s="7" t="inlineStr">
@@ -14370,6 +14568,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AN195" s="7"/>
     </row>
     <row r="196">
       <c r="A196" s="7" t="inlineStr">
@@ -14439,6 +14638,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AN196" s="7"/>
     </row>
     <row r="197">
       <c r="A197" s="7" t="inlineStr">
@@ -14512,6 +14712,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AN197" s="7"/>
     </row>
     <row r="198">
       <c r="A198" s="7" t="inlineStr">
@@ -14581,6 +14782,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AN198" s="7"/>
     </row>
     <row r="199">
       <c r="A199" s="7" t="inlineStr">
@@ -14654,6 +14856,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AN199" s="7"/>
     </row>
     <row r="200">
       <c r="A200" s="7" t="inlineStr">
@@ -14727,6 +14930,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AN200" s="7"/>
     </row>
     <row r="201">
       <c r="A201" s="7" t="inlineStr">
@@ -14792,6 +14996,7 @@
       <c r="AK201" s="7"/>
       <c r="AL201" s="7"/>
       <c r="AM201" s="7"/>
+      <c r="AN201" s="7"/>
     </row>
     <row r="202">
       <c r="A202" s="7" t="inlineStr">
@@ -14865,6 +15070,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AN202" s="7"/>
     </row>
     <row r="203">
       <c r="A203" s="7" t="inlineStr">
@@ -14938,6 +15144,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AN203" s="7"/>
     </row>
     <row r="204">
       <c r="A204" s="7" t="inlineStr">
@@ -15007,6 +15214,11 @@
           <t xml:space="preserve">Fail</t>
         </is>
       </c>
+      <c r="AN204" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="7" t="inlineStr">
@@ -15076,6 +15288,11 @@
           <t xml:space="preserve">Fail</t>
         </is>
       </c>
+      <c r="AN205" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="7" t="inlineStr">
@@ -15145,6 +15362,7 @@
           <t xml:space="preserve">Fail</t>
         </is>
       </c>
+      <c r="AN206" s="7"/>
     </row>
     <row r="207">
       <c r="A207" s="7" t="inlineStr">
@@ -15214,6 +15432,7 @@
           <t xml:space="preserve">Fail</t>
         </is>
       </c>
+      <c r="AN207" s="7"/>
     </row>
     <row r="208">
       <c r="A208" s="7" t="inlineStr">
@@ -15283,6 +15502,77 @@
           <t xml:space="preserve">Fail</t>
         </is>
       </c>
+      <c r="AN208" s="7"/>
+    </row>
+    <row r="209">
+      <c r="A209" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_201</t>
+        </is>
+      </c>
+      <c r="B209" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">조립</t>
+        </is>
+      </c>
+      <c r="C209" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">마운트 팝오버</t>
+        </is>
+      </c>
+      <c r="D209" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lv 줄 · 단추</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t xml:space="preserve">마운트 팝오버에 「강화 Lv 1 · ×1.00」(강화 뒤 Lv 2 · ×1.45) 줄이 있고 단추가 「강화 (재료 50 · 고철 300)」 · 강화 뒤 「강화 완료」(흐림)인가?</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#199 · 꼴 ⚠️ 가정 · 고철은 글자(아이콘 아님 · 구현 판단)</t>
+        </is>
+      </c>
+      <c r="G209" s="7"/>
+      <c r="H209" s="7"/>
+      <c r="I209" s="7"/>
+      <c r="J209" s="7"/>
+      <c r="K209" s="7"/>
+      <c r="L209" s="7"/>
+      <c r="M209" s="7"/>
+      <c r="N209" s="7"/>
+      <c r="O209" s="7"/>
+      <c r="P209" s="7"/>
+      <c r="Q209" s="7"/>
+      <c r="R209" s="7"/>
+      <c r="S209" s="7"/>
+      <c r="T209" s="7"/>
+      <c r="U209" s="7"/>
+      <c r="V209" s="7"/>
+      <c r="W209" s="7"/>
+      <c r="X209" s="7"/>
+      <c r="Y209" s="7"/>
+      <c r="Z209" s="7"/>
+      <c r="AA209" s="7"/>
+      <c r="AB209" s="7"/>
+      <c r="AC209" s="7"/>
+      <c r="AD209" s="7"/>
+      <c r="AE209" s="7"/>
+      <c r="AF209" s="7"/>
+      <c r="AG209" s="7"/>
+      <c r="AH209" s="7"/>
+      <c r="AI209" s="7"/>
+      <c r="AJ209" s="7"/>
+      <c r="AK209" s="7"/>
+      <c r="AL209" s="7"/>
+      <c r="AM209" s="7"/>
+      <c r="AN209" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="26">
@@ -15311,9 +15601,9 @@
     <mergeCell ref="B92:B99"/>
     <mergeCell ref="B100:B106"/>
     <mergeCell ref="B107:B111"/>
-    <mergeCell ref="G7:AM7"/>
+    <mergeCell ref="G7:AN7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:AM208">
+  <conditionalFormatting sqref="G9:AN209">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
docs: QA AO열(6fb2f5e · CID_202 #203) · 가이드 8133 후보 6fb2f5e
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -196,8 +196,9 @@
     <col min="38" max="38" width="12" customWidth="1"/>
     <col min="39" max="39" width="12" customWidth="1"/>
     <col min="40" max="40" width="12" customWidth="1"/>
-    <col min="41" max="41" width="11" customWidth="1"/>
+    <col min="41" max="41" width="12" customWidth="1"/>
     <col min="42" max="42" width="11" customWidth="1"/>
+    <col min="43" max="43" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -480,6 +481,11 @@
       <c r="AN6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">8133 갈아엎음(21:02:57) · #198 점프 재료 · #199 팝오버 Lv · #200 창 단추 · #201 요구치 0 목표 줄 ‖ 10-19 코드 세션 재확인(8123): 「처음부터」 → 바로가기 S3 = 강화 막 섬(재료 ≥ 50) → 팝오버 「강화 Lv 1 · ×1.00 · 강화 재료 63/50 · 312/300 · [강화 (재료 50 · 고철 300)]」 ✅ · 바로가기 S6 = 주제 「자유 플레이 · 보스」 · 화면 흐림 막(B 강화 막 — 문구는 창 밖) ✅ · 강화 누름 · B 팝오버 · S6 배지 · 창 단추 자리 = 인앱 누름 어긋남으로 못 봄(시험이 든다) · ⚠️ 바로가기 S3 직후 HUD 전투력 0 한동안(관찰)</t>
+        </is>
+      </c>
+      <c r="AO6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8133 갈아엎음(21:33:11) · #202 팝오버 「Lv · 피해량 ×」 · #203 튜토리얼 막 동안 전투 정지 ‖ 10-19 사용자 육안(e86eb9a · 21:2x) = 팝오버 Lv 줄 · 창 [취소] 왼쪽 · S6 B 강화 ✅ / 코드 세션(8123): 바로가기 S3 = 강화 막 동안 적 · 리젠 00:10 정지 · 바로가기 S6 = B 막 동안 쿨다운 5.0s · 게이지 0% · 리젠 정지(Auto 태그 안 나감) ✅ · 정지 중 HUD 전투력 = 보드 예상 출력(첫 판 390 명목값 멈춤 → 0 → 예상 출력으로 고침 · 구현 판단) · S1 T3 정지 · 강화 뒤 재개 = 화면 미확인(시험)</t>
         </is>
       </c>
     </row>
@@ -544,14 +550,15 @@
       <c r="AL7" s="2"/>
       <c r="AM7" s="2"/>
       <c r="AN7" s="2"/>
-      <c r="AO7" s="2" t="inlineStr">
+      <c r="AO7" s="2"/>
+      <c r="AP7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">버전</t>
         </is>
       </c>
-      <c r="AP7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">e86eb9a</t>
+      <c r="AQ7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6fb2f5e</t>
         </is>
       </c>
     </row>
@@ -746,11 +753,16 @@
       </c>
       <c r="AO8" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">6fb2f5e</t>
+        </is>
+      </c>
+      <c r="AP8" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">PASSrate</t>
         </is>
       </c>
-      <c r="AP8" s="7">
-        <f>COUNTIF(AN9:AN209,"Pass")</f>
+      <c r="AQ8" s="7">
+        <f>COUNTIF(AO9:AO210,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -854,13 +866,14 @@
       <c r="AL9" s="7"/>
       <c r="AM9" s="7"/>
       <c r="AN9" s="7"/>
-      <c r="AO9" s="2" t="inlineStr">
+      <c r="AO9" s="7"/>
+      <c r="AP9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FAILrate</t>
         </is>
       </c>
-      <c r="AP9" s="7">
-        <f>COUNTIF(AN9:AN209,"Fail")+COUNTIF(AN9:AN209,"Broken")</f>
+      <c r="AQ9" s="7">
+        <f>COUNTIF(AO9:AO210,"Fail")+COUNTIF(AO9:AO210,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -928,13 +941,14 @@
       <c r="AL10" s="7"/>
       <c r="AM10" s="7"/>
       <c r="AN10" s="7"/>
-      <c r="AO10" s="2" t="inlineStr">
+      <c r="AO10" s="7"/>
+      <c r="AP10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">N/A</t>
         </is>
       </c>
-      <c r="AP10" s="7">
-        <f>COUNTIF(AN9:AN209,"N/A")</f>
+      <c r="AQ10" s="7">
+        <f>COUNTIF(AO9:AO210,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -1002,13 +1016,14 @@
       <c r="AL11" s="7"/>
       <c r="AM11" s="7"/>
       <c r="AN11" s="7"/>
-      <c r="AO11" s="2" t="inlineStr">
+      <c r="AO11" s="7"/>
+      <c r="AP11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">전체 개수</t>
         </is>
       </c>
-      <c r="AP11" s="7">
-        <v>201</v>
+      <c r="AQ11" s="7">
+        <v>202</v>
       </c>
     </row>
     <row r="12">
@@ -1076,13 +1091,14 @@
       <c r="AL12" s="7"/>
       <c r="AM12" s="7"/>
       <c r="AN12" s="7"/>
-      <c r="AO12" s="2" t="inlineStr">
+      <c r="AO12" s="7"/>
+      <c r="AP12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">진행율</t>
         </is>
       </c>
-      <c r="AP12" s="7">
-        <f>TEXT((COUNTA(AN9:AN209))/201,"0.00%")</f>
+      <c r="AQ12" s="7">
+        <f>TEXT((COUNTA(AO9:AO210))/202,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -1154,6 +1170,7 @@
       <c r="AL13" s="7"/>
       <c r="AM13" s="7"/>
       <c r="AN13" s="7"/>
+      <c r="AO13" s="7"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -1215,6 +1232,7 @@
       <c r="AL14" s="7"/>
       <c r="AM14" s="7"/>
       <c r="AN14" s="7"/>
+      <c r="AO14" s="7"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -1312,6 +1330,7 @@
       <c r="AL15" s="7"/>
       <c r="AM15" s="7"/>
       <c r="AN15" s="7"/>
+      <c r="AO15" s="7"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -1409,6 +1428,7 @@
       <c r="AL16" s="7"/>
       <c r="AM16" s="7"/>
       <c r="AN16" s="7"/>
+      <c r="AO16" s="7"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -1511,6 +1531,7 @@
       <c r="AL17" s="7"/>
       <c r="AM17" s="7"/>
       <c r="AN17" s="7"/>
+      <c r="AO17" s="7"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -1577,6 +1598,7 @@
       <c r="AL18" s="7"/>
       <c r="AM18" s="7"/>
       <c r="AN18" s="7"/>
+      <c r="AO18" s="7"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -1638,6 +1660,7 @@
       <c r="AL19" s="7"/>
       <c r="AM19" s="7"/>
       <c r="AN19" s="7"/>
+      <c r="AO19" s="7"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1699,6 +1722,7 @@
       <c r="AL20" s="7"/>
       <c r="AM20" s="7"/>
       <c r="AN20" s="7"/>
+      <c r="AO20" s="7"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1796,6 +1820,7 @@
       <c r="AL21" s="7"/>
       <c r="AM21" s="7"/>
       <c r="AN21" s="7"/>
+      <c r="AO21" s="7"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1886,6 +1911,7 @@
       <c r="AL22" s="7"/>
       <c r="AM22" s="7"/>
       <c r="AN22" s="7"/>
+      <c r="AO22" s="7"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -1955,6 +1981,7 @@
       <c r="AL23" s="7"/>
       <c r="AM23" s="7"/>
       <c r="AN23" s="7"/>
+      <c r="AO23" s="7"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -2016,6 +2043,7 @@
       <c r="AL24" s="7"/>
       <c r="AM24" s="7"/>
       <c r="AN24" s="7"/>
+      <c r="AO24" s="7"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -2077,6 +2105,7 @@
       <c r="AL25" s="7"/>
       <c r="AM25" s="7"/>
       <c r="AN25" s="7"/>
+      <c r="AO25" s="7"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -2167,6 +2196,7 @@
       <c r="AL26" s="7"/>
       <c r="AM26" s="7"/>
       <c r="AN26" s="7"/>
+      <c r="AO26" s="7"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -2232,6 +2262,7 @@
       <c r="AL27" s="7"/>
       <c r="AM27" s="7"/>
       <c r="AN27" s="7"/>
+      <c r="AO27" s="7"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -2306,6 +2337,7 @@
       <c r="AL28" s="7"/>
       <c r="AM28" s="7"/>
       <c r="AN28" s="7"/>
+      <c r="AO28" s="7"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -2375,6 +2407,7 @@
       <c r="AL29" s="7"/>
       <c r="AM29" s="7"/>
       <c r="AN29" s="7"/>
+      <c r="AO29" s="7"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -2468,6 +2501,7 @@
       <c r="AL30" s="7"/>
       <c r="AM30" s="7"/>
       <c r="AN30" s="7"/>
+      <c r="AO30" s="7"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -2566,6 +2600,7 @@
       <c r="AL31" s="7"/>
       <c r="AM31" s="7"/>
       <c r="AN31" s="7"/>
+      <c r="AO31" s="7"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -2651,6 +2686,7 @@
       <c r="AL32" s="7"/>
       <c r="AM32" s="7"/>
       <c r="AN32" s="7"/>
+      <c r="AO32" s="7"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -2744,6 +2780,7 @@
       <c r="AL33" s="7"/>
       <c r="AM33" s="7"/>
       <c r="AN33" s="7"/>
+      <c r="AO33" s="7"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -2837,6 +2874,7 @@
       <c r="AL34" s="7"/>
       <c r="AM34" s="7"/>
       <c r="AN34" s="7"/>
+      <c r="AO34" s="7"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -2939,6 +2977,7 @@
       <c r="AL35" s="7"/>
       <c r="AM35" s="7"/>
       <c r="AN35" s="7"/>
+      <c r="AO35" s="7"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -3016,6 +3055,7 @@
       <c r="AL36" s="7"/>
       <c r="AM36" s="7"/>
       <c r="AN36" s="7"/>
+      <c r="AO36" s="7"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -3077,6 +3117,7 @@
       <c r="AL37" s="7"/>
       <c r="AM37" s="7"/>
       <c r="AN37" s="7"/>
+      <c r="AO37" s="7"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -3159,6 +3200,7 @@
       <c r="AL38" s="7"/>
       <c r="AM38" s="7"/>
       <c r="AN38" s="7"/>
+      <c r="AO38" s="7"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -3252,6 +3294,7 @@
       <c r="AL39" s="7"/>
       <c r="AM39" s="7"/>
       <c r="AN39" s="7"/>
+      <c r="AO39" s="7"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -3346,6 +3389,7 @@
       <c r="AL40" s="7"/>
       <c r="AM40" s="7"/>
       <c r="AN40" s="7"/>
+      <c r="AO40" s="7"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -3435,6 +3479,7 @@
       <c r="AL41" s="7"/>
       <c r="AM41" s="7"/>
       <c r="AN41" s="7"/>
+      <c r="AO41" s="7"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -3508,6 +3553,7 @@
       <c r="AL42" s="7"/>
       <c r="AM42" s="7"/>
       <c r="AN42" s="7"/>
+      <c r="AO42" s="7"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -3601,6 +3647,7 @@
       <c r="AL43" s="7"/>
       <c r="AM43" s="7"/>
       <c r="AN43" s="7"/>
+      <c r="AO43" s="7"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -3667,6 +3714,7 @@
       <c r="AL44" s="7"/>
       <c r="AM44" s="7"/>
       <c r="AN44" s="7"/>
+      <c r="AO44" s="7"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -3756,6 +3804,7 @@
       <c r="AL45" s="7"/>
       <c r="AM45" s="7"/>
       <c r="AN45" s="7"/>
+      <c r="AO45" s="7"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -3845,6 +3894,7 @@
       <c r="AL46" s="7"/>
       <c r="AM46" s="7"/>
       <c r="AN46" s="7"/>
+      <c r="AO46" s="7"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -3911,6 +3961,7 @@
       <c r="AL47" s="7"/>
       <c r="AM47" s="7"/>
       <c r="AN47" s="7"/>
+      <c r="AO47" s="7"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -3972,6 +4023,7 @@
       <c r="AL48" s="7"/>
       <c r="AM48" s="7"/>
       <c r="AN48" s="7"/>
+      <c r="AO48" s="7"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -4033,6 +4085,7 @@
       <c r="AL49" s="7"/>
       <c r="AM49" s="7"/>
       <c r="AN49" s="7"/>
+      <c r="AO49" s="7"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -4118,6 +4171,7 @@
       <c r="AL50" s="7"/>
       <c r="AM50" s="7"/>
       <c r="AN50" s="7"/>
+      <c r="AO50" s="7"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -4203,6 +4257,7 @@
       <c r="AL51" s="7"/>
       <c r="AM51" s="7"/>
       <c r="AN51" s="7"/>
+      <c r="AO51" s="7"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -4269,6 +4324,7 @@
       <c r="AL52" s="7"/>
       <c r="AM52" s="7"/>
       <c r="AN52" s="7"/>
+      <c r="AO52" s="7"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -4335,6 +4391,7 @@
       <c r="AL53" s="7"/>
       <c r="AM53" s="7"/>
       <c r="AN53" s="7"/>
+      <c r="AO53" s="7"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -4396,6 +4453,7 @@
       <c r="AL54" s="7"/>
       <c r="AM54" s="7"/>
       <c r="AN54" s="7"/>
+      <c r="AO54" s="7"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -4493,6 +4551,7 @@
       <c r="AL55" s="7"/>
       <c r="AM55" s="7"/>
       <c r="AN55" s="7"/>
+      <c r="AO55" s="7"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -4570,6 +4629,7 @@
       <c r="AL56" s="7"/>
       <c r="AM56" s="7"/>
       <c r="AN56" s="7"/>
+      <c r="AO56" s="7"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -4656,6 +4716,7 @@
       <c r="AL57" s="7"/>
       <c r="AM57" s="7"/>
       <c r="AN57" s="7"/>
+      <c r="AO57" s="7"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -4750,6 +4811,7 @@
       <c r="AL58" s="7"/>
       <c r="AM58" s="7"/>
       <c r="AN58" s="7"/>
+      <c r="AO58" s="7"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -4811,6 +4873,7 @@
       <c r="AL59" s="7"/>
       <c r="AM59" s="7"/>
       <c r="AN59" s="7"/>
+      <c r="AO59" s="7"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -4872,6 +4935,7 @@
       <c r="AL60" s="7"/>
       <c r="AM60" s="7"/>
       <c r="AN60" s="7"/>
+      <c r="AO60" s="7"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -4945,6 +5009,7 @@
       <c r="AL61" s="7"/>
       <c r="AM61" s="7"/>
       <c r="AN61" s="7"/>
+      <c r="AO61" s="7"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -5026,6 +5091,7 @@
       <c r="AL62" s="7"/>
       <c r="AM62" s="7"/>
       <c r="AN62" s="7"/>
+      <c r="AO62" s="7"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -5099,6 +5165,7 @@
       <c r="AL63" s="7"/>
       <c r="AM63" s="7"/>
       <c r="AN63" s="7"/>
+      <c r="AO63" s="7"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -5160,6 +5227,7 @@
       <c r="AL64" s="7"/>
       <c r="AM64" s="7"/>
       <c r="AN64" s="7"/>
+      <c r="AO64" s="7"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -5226,6 +5294,7 @@
       <c r="AL65" s="7"/>
       <c r="AM65" s="7"/>
       <c r="AN65" s="7"/>
+      <c r="AO65" s="7"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
@@ -5299,6 +5368,7 @@
       <c r="AL66" s="7"/>
       <c r="AM66" s="7"/>
       <c r="AN66" s="7"/>
+      <c r="AO66" s="7"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -5360,6 +5430,7 @@
       <c r="AL67" s="7"/>
       <c r="AM67" s="7"/>
       <c r="AN67" s="7"/>
+      <c r="AO67" s="7"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
@@ -5425,6 +5496,7 @@
       <c r="AL68" s="7"/>
       <c r="AM68" s="7"/>
       <c r="AN68" s="7"/>
+      <c r="AO68" s="7"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -5522,6 +5594,7 @@
       <c r="AL69" s="7"/>
       <c r="AM69" s="7"/>
       <c r="AN69" s="7"/>
+      <c r="AO69" s="7"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
@@ -5583,6 +5656,7 @@
       <c r="AL70" s="7"/>
       <c r="AM70" s="7"/>
       <c r="AN70" s="7"/>
+      <c r="AO70" s="7"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -5649,6 +5723,7 @@
       <c r="AL71" s="7"/>
       <c r="AM71" s="7"/>
       <c r="AN71" s="7"/>
+      <c r="AO71" s="7"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
@@ -5726,6 +5801,7 @@
       <c r="AL72" s="7"/>
       <c r="AM72" s="7"/>
       <c r="AN72" s="7"/>
+      <c r="AO72" s="7"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
@@ -5792,6 +5868,7 @@
       <c r="AL73" s="7"/>
       <c r="AM73" s="7"/>
       <c r="AN73" s="7"/>
+      <c r="AO73" s="7"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -5853,6 +5930,7 @@
       <c r="AL74" s="7"/>
       <c r="AM74" s="7"/>
       <c r="AN74" s="7"/>
+      <c r="AO74" s="7"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -5914,6 +5992,7 @@
       <c r="AL75" s="7"/>
       <c r="AM75" s="7"/>
       <c r="AN75" s="7"/>
+      <c r="AO75" s="7"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -5975,6 +6054,7 @@
       <c r="AL76" s="7"/>
       <c r="AM76" s="7"/>
       <c r="AN76" s="7"/>
+      <c r="AO76" s="7"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -6040,6 +6120,7 @@
       <c r="AL77" s="7"/>
       <c r="AM77" s="7"/>
       <c r="AN77" s="7"/>
+      <c r="AO77" s="7"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
@@ -6101,6 +6182,7 @@
       <c r="AL78" s="7"/>
       <c r="AM78" s="7"/>
       <c r="AN78" s="7"/>
+      <c r="AO78" s="7"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -6167,6 +6249,7 @@
       <c r="AL79" s="7"/>
       <c r="AM79" s="7"/>
       <c r="AN79" s="7"/>
+      <c r="AO79" s="7"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
@@ -6244,6 +6327,7 @@
       <c r="AL80" s="7"/>
       <c r="AM80" s="7"/>
       <c r="AN80" s="7"/>
+      <c r="AO80" s="7"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
@@ -6309,6 +6393,7 @@
       <c r="AL81" s="7"/>
       <c r="AM81" s="7"/>
       <c r="AN81" s="7"/>
+      <c r="AO81" s="7"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
@@ -6370,6 +6455,7 @@
       <c r="AL82" s="7"/>
       <c r="AM82" s="7"/>
       <c r="AN82" s="7"/>
+      <c r="AO82" s="7"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
@@ -6436,6 +6522,7 @@
       <c r="AL83" s="7"/>
       <c r="AM83" s="7"/>
       <c r="AN83" s="7"/>
+      <c r="AO83" s="7"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
@@ -6497,6 +6584,7 @@
       <c r="AL84" s="7"/>
       <c r="AM84" s="7"/>
       <c r="AN84" s="7"/>
+      <c r="AO84" s="7"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
@@ -6558,6 +6646,7 @@
       <c r="AL85" s="7"/>
       <c r="AM85" s="7"/>
       <c r="AN85" s="7"/>
+      <c r="AO85" s="7"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
@@ -6624,6 +6713,7 @@
       <c r="AL86" s="7"/>
       <c r="AM86" s="7"/>
       <c r="AN86" s="7"/>
+      <c r="AO86" s="7"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
@@ -6685,6 +6775,7 @@
       <c r="AL87" s="7"/>
       <c r="AM87" s="7"/>
       <c r="AN87" s="7"/>
+      <c r="AO87" s="7"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
@@ -6746,6 +6837,7 @@
       <c r="AL88" s="7"/>
       <c r="AM88" s="7"/>
       <c r="AN88" s="7"/>
+      <c r="AO88" s="7"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
@@ -6807,6 +6899,7 @@
       <c r="AL89" s="7"/>
       <c r="AM89" s="7"/>
       <c r="AN89" s="7"/>
+      <c r="AO89" s="7"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
@@ -6897,6 +6990,7 @@
       <c r="AL90" s="7"/>
       <c r="AM90" s="7"/>
       <c r="AN90" s="7"/>
+      <c r="AO90" s="7"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
@@ -6958,6 +7052,7 @@
       <c r="AL91" s="7"/>
       <c r="AM91" s="7"/>
       <c r="AN91" s="7"/>
+      <c r="AO91" s="7"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
@@ -7055,6 +7150,7 @@
       <c r="AL92" s="7"/>
       <c r="AM92" s="7"/>
       <c r="AN92" s="7"/>
+      <c r="AO92" s="7"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
@@ -7157,6 +7253,7 @@
       <c r="AL93" s="7"/>
       <c r="AM93" s="7"/>
       <c r="AN93" s="7"/>
+      <c r="AO93" s="7"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
@@ -7223,6 +7320,7 @@
       <c r="AL94" s="7"/>
       <c r="AM94" s="7"/>
       <c r="AN94" s="7"/>
+      <c r="AO94" s="7"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
@@ -7289,6 +7387,7 @@
       <c r="AL95" s="7"/>
       <c r="AM95" s="7"/>
       <c r="AN95" s="7"/>
+      <c r="AO95" s="7"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
@@ -7374,6 +7473,7 @@
       <c r="AL96" s="7"/>
       <c r="AM96" s="7"/>
       <c r="AN96" s="7"/>
+      <c r="AO96" s="7"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="inlineStr">
@@ -7435,6 +7535,7 @@
       <c r="AL97" s="7"/>
       <c r="AM97" s="7"/>
       <c r="AN97" s="7"/>
+      <c r="AO97" s="7"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
@@ -7496,6 +7597,7 @@
       <c r="AL98" s="7"/>
       <c r="AM98" s="7"/>
       <c r="AN98" s="7"/>
+      <c r="AO98" s="7"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
@@ -7557,6 +7659,7 @@
       <c r="AL99" s="7"/>
       <c r="AM99" s="7"/>
       <c r="AN99" s="7"/>
+      <c r="AO99" s="7"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
@@ -7627,6 +7730,7 @@
       <c r="AL100" s="7"/>
       <c r="AM100" s="7"/>
       <c r="AN100" s="7"/>
+      <c r="AO100" s="7"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
@@ -7688,6 +7792,7 @@
       <c r="AL101" s="7"/>
       <c r="AM101" s="7"/>
       <c r="AN101" s="7"/>
+      <c r="AO101" s="7"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
@@ -7749,6 +7854,7 @@
       <c r="AL102" s="7"/>
       <c r="AM102" s="7"/>
       <c r="AN102" s="7"/>
+      <c r="AO102" s="7"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="inlineStr">
@@ -7810,6 +7916,7 @@
       <c r="AL103" s="7"/>
       <c r="AM103" s="7"/>
       <c r="AN103" s="7"/>
+      <c r="AO103" s="7"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="inlineStr">
@@ -7876,6 +7983,7 @@
       <c r="AL104" s="7"/>
       <c r="AM104" s="7"/>
       <c r="AN104" s="7"/>
+      <c r="AO104" s="7"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
@@ -7937,6 +8045,7 @@
       <c r="AL105" s="7"/>
       <c r="AM105" s="7"/>
       <c r="AN105" s="7"/>
+      <c r="AO105" s="7"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
@@ -7998,6 +8107,7 @@
       <c r="AL106" s="7"/>
       <c r="AM106" s="7"/>
       <c r="AN106" s="7"/>
+      <c r="AO106" s="7"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
@@ -8059,6 +8169,7 @@
       <c r="AL107" s="7"/>
       <c r="AM107" s="7"/>
       <c r="AN107" s="7"/>
+      <c r="AO107" s="7"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
@@ -8124,6 +8235,7 @@
       <c r="AL108" s="7"/>
       <c r="AM108" s="7"/>
       <c r="AN108" s="7"/>
+      <c r="AO108" s="7"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="inlineStr">
@@ -8194,6 +8306,7 @@
       <c r="AL109" s="7"/>
       <c r="AM109" s="7"/>
       <c r="AN109" s="7"/>
+      <c r="AO109" s="7"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
@@ -8272,6 +8385,7 @@
       <c r="AL110" s="7"/>
       <c r="AM110" s="7"/>
       <c r="AN110" s="7"/>
+      <c r="AO110" s="7"/>
     </row>
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
@@ -8353,6 +8467,7 @@
       <c r="AL111" s="7"/>
       <c r="AM111" s="7"/>
       <c r="AN111" s="7"/>
+      <c r="AO111" s="7"/>
     </row>
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
@@ -8431,6 +8546,7 @@
       <c r="AL112" s="7"/>
       <c r="AM112" s="7"/>
       <c r="AN112" s="7"/>
+      <c r="AO112" s="7"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
@@ -8501,6 +8617,7 @@
       <c r="AL113" s="7"/>
       <c r="AM113" s="7"/>
       <c r="AN113" s="7"/>
+      <c r="AO113" s="7"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="inlineStr">
@@ -8587,6 +8704,7 @@
       <c r="AL114" s="7"/>
       <c r="AM114" s="7"/>
       <c r="AN114" s="7"/>
+      <c r="AO114" s="7"/>
     </row>
     <row r="115">
       <c r="A115" s="7" t="inlineStr">
@@ -8665,6 +8783,7 @@
       <c r="AL115" s="7"/>
       <c r="AM115" s="7"/>
       <c r="AN115" s="7"/>
+      <c r="AO115" s="7"/>
     </row>
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
@@ -8751,6 +8870,7 @@
       <c r="AL116" s="7"/>
       <c r="AM116" s="7"/>
       <c r="AN116" s="7"/>
+      <c r="AO116" s="7"/>
     </row>
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
@@ -8833,6 +8953,7 @@
       <c r="AL117" s="7"/>
       <c r="AM117" s="7"/>
       <c r="AN117" s="7"/>
+      <c r="AO117" s="7"/>
     </row>
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
@@ -8915,6 +9036,7 @@
       <c r="AL118" s="7"/>
       <c r="AM118" s="7"/>
       <c r="AN118" s="7"/>
+      <c r="AO118" s="7"/>
     </row>
     <row r="119">
       <c r="A119" s="7" t="inlineStr">
@@ -8993,6 +9115,7 @@
       <c r="AL119" s="7"/>
       <c r="AM119" s="7"/>
       <c r="AN119" s="7"/>
+      <c r="AO119" s="7"/>
     </row>
     <row r="120">
       <c r="A120" s="7" t="inlineStr">
@@ -9063,6 +9186,7 @@
       <c r="AL120" s="7"/>
       <c r="AM120" s="7"/>
       <c r="AN120" s="7"/>
+      <c r="AO120" s="7"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="inlineStr">
@@ -9145,6 +9269,7 @@
       <c r="AL121" s="7"/>
       <c r="AM121" s="7"/>
       <c r="AN121" s="7"/>
+      <c r="AO121" s="7"/>
     </row>
     <row r="122">
       <c r="A122" s="7" t="inlineStr">
@@ -9227,6 +9352,7 @@
       <c r="AL122" s="7"/>
       <c r="AM122" s="7"/>
       <c r="AN122" s="7"/>
+      <c r="AO122" s="7"/>
     </row>
     <row r="123">
       <c r="A123" s="7" t="inlineStr">
@@ -9297,6 +9423,7 @@
       <c r="AL123" s="7"/>
       <c r="AM123" s="7"/>
       <c r="AN123" s="7"/>
+      <c r="AO123" s="7"/>
     </row>
     <row r="124">
       <c r="A124" s="7" t="inlineStr">
@@ -9375,6 +9502,7 @@
       <c r="AL124" s="7"/>
       <c r="AM124" s="7"/>
       <c r="AN124" s="7"/>
+      <c r="AO124" s="7"/>
     </row>
     <row r="125">
       <c r="A125" s="7" t="inlineStr">
@@ -9445,6 +9573,7 @@
       <c r="AL125" s="7"/>
       <c r="AM125" s="7"/>
       <c r="AN125" s="7"/>
+      <c r="AO125" s="7"/>
     </row>
     <row r="126">
       <c r="A126" s="7" t="inlineStr">
@@ -9515,6 +9644,7 @@
       <c r="AL126" s="7"/>
       <c r="AM126" s="7"/>
       <c r="AN126" s="7"/>
+      <c r="AO126" s="7"/>
     </row>
     <row r="127">
       <c r="A127" s="7" t="inlineStr">
@@ -9589,6 +9719,7 @@
       <c r="AL127" s="7"/>
       <c r="AM127" s="7"/>
       <c r="AN127" s="7"/>
+      <c r="AO127" s="7"/>
     </row>
     <row r="128">
       <c r="A128" s="7" t="inlineStr">
@@ -9663,6 +9794,7 @@
       <c r="AL128" s="7"/>
       <c r="AM128" s="7"/>
       <c r="AN128" s="7"/>
+      <c r="AO128" s="7"/>
     </row>
     <row r="129">
       <c r="A129" s="7" t="inlineStr">
@@ -9737,6 +9869,7 @@
       <c r="AL129" s="7"/>
       <c r="AM129" s="7"/>
       <c r="AN129" s="7"/>
+      <c r="AO129" s="7"/>
     </row>
     <row r="130">
       <c r="A130" s="7" t="inlineStr">
@@ -9807,6 +9940,7 @@
       <c r="AL130" s="7"/>
       <c r="AM130" s="7"/>
       <c r="AN130" s="7"/>
+      <c r="AO130" s="7"/>
     </row>
     <row r="131">
       <c r="A131" s="7" t="inlineStr">
@@ -9885,6 +10019,7 @@
       <c r="AL131" s="7"/>
       <c r="AM131" s="7"/>
       <c r="AN131" s="7"/>
+      <c r="AO131" s="7"/>
     </row>
     <row r="132">
       <c r="A132" s="7" t="inlineStr">
@@ -9967,6 +10102,7 @@
       <c r="AL132" s="7"/>
       <c r="AM132" s="7"/>
       <c r="AN132" s="7"/>
+      <c r="AO132" s="7"/>
     </row>
     <row r="133">
       <c r="A133" s="7" t="inlineStr">
@@ -10049,6 +10185,7 @@
       <c r="AL133" s="7"/>
       <c r="AM133" s="7"/>
       <c r="AN133" s="7"/>
+      <c r="AO133" s="7"/>
     </row>
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
@@ -10127,6 +10264,7 @@
       <c r="AL134" s="7"/>
       <c r="AM134" s="7"/>
       <c r="AN134" s="7"/>
+      <c r="AO134" s="7"/>
     </row>
     <row r="135">
       <c r="A135" s="7" t="inlineStr">
@@ -10205,6 +10343,7 @@
       <c r="AL135" s="7"/>
       <c r="AM135" s="7"/>
       <c r="AN135" s="7"/>
+      <c r="AO135" s="7"/>
     </row>
     <row r="136">
       <c r="A136" s="7" t="inlineStr">
@@ -10283,6 +10422,7 @@
       <c r="AL136" s="7"/>
       <c r="AM136" s="7"/>
       <c r="AN136" s="7"/>
+      <c r="AO136" s="7"/>
     </row>
     <row r="137">
       <c r="A137" s="7" t="inlineStr">
@@ -10357,6 +10497,7 @@
       <c r="AL137" s="7"/>
       <c r="AM137" s="7"/>
       <c r="AN137" s="7"/>
+      <c r="AO137" s="7"/>
     </row>
     <row r="138">
       <c r="A138" s="7" t="inlineStr">
@@ -10431,6 +10572,7 @@
       <c r="AL138" s="7"/>
       <c r="AM138" s="7"/>
       <c r="AN138" s="7"/>
+      <c r="AO138" s="7"/>
     </row>
     <row r="139">
       <c r="A139" s="7" t="inlineStr">
@@ -10505,6 +10647,7 @@
       <c r="AL139" s="7"/>
       <c r="AM139" s="7"/>
       <c r="AN139" s="7"/>
+      <c r="AO139" s="7"/>
     </row>
     <row r="140">
       <c r="A140" s="7" t="inlineStr">
@@ -10575,6 +10718,7 @@
       <c r="AL140" s="7"/>
       <c r="AM140" s="7"/>
       <c r="AN140" s="7"/>
+      <c r="AO140" s="7"/>
     </row>
     <row r="141">
       <c r="A141" s="7" t="inlineStr">
@@ -10657,6 +10801,7 @@
       <c r="AL141" s="7"/>
       <c r="AM141" s="7"/>
       <c r="AN141" s="7"/>
+      <c r="AO141" s="7"/>
     </row>
     <row r="142">
       <c r="A142" s="7" t="inlineStr">
@@ -10727,6 +10872,7 @@
       <c r="AL142" s="7"/>
       <c r="AM142" s="7"/>
       <c r="AN142" s="7"/>
+      <c r="AO142" s="7"/>
     </row>
     <row r="143">
       <c r="A143" s="7" t="inlineStr">
@@ -10797,6 +10943,7 @@
       <c r="AL143" s="7"/>
       <c r="AM143" s="7"/>
       <c r="AN143" s="7"/>
+      <c r="AO143" s="7"/>
     </row>
     <row r="144">
       <c r="A144" s="7" t="inlineStr">
@@ -10867,6 +11014,7 @@
       <c r="AL144" s="7"/>
       <c r="AM144" s="7"/>
       <c r="AN144" s="7"/>
+      <c r="AO144" s="7"/>
     </row>
     <row r="145">
       <c r="A145" s="7" t="inlineStr">
@@ -10953,6 +11101,7 @@
       <c r="AL145" s="7"/>
       <c r="AM145" s="7"/>
       <c r="AN145" s="7"/>
+      <c r="AO145" s="7"/>
     </row>
     <row r="146">
       <c r="A146" s="7" t="inlineStr">
@@ -11027,6 +11176,7 @@
       <c r="AL146" s="7"/>
       <c r="AM146" s="7"/>
       <c r="AN146" s="7"/>
+      <c r="AO146" s="7"/>
     </row>
     <row r="147">
       <c r="A147" s="7" t="inlineStr">
@@ -11113,6 +11263,7 @@
       <c r="AL147" s="7"/>
       <c r="AM147" s="7"/>
       <c r="AN147" s="7"/>
+      <c r="AO147" s="7"/>
     </row>
     <row r="148">
       <c r="A148" s="7" t="inlineStr">
@@ -11183,6 +11334,7 @@
       <c r="AL148" s="7"/>
       <c r="AM148" s="7"/>
       <c r="AN148" s="7"/>
+      <c r="AO148" s="7"/>
     </row>
     <row r="149">
       <c r="A149" s="7" t="inlineStr">
@@ -11261,6 +11413,7 @@
       <c r="AL149" s="7"/>
       <c r="AM149" s="7"/>
       <c r="AN149" s="7"/>
+      <c r="AO149" s="7"/>
     </row>
     <row r="150">
       <c r="A150" s="7" t="inlineStr">
@@ -11343,6 +11496,7 @@
       <c r="AL150" s="7"/>
       <c r="AM150" s="7"/>
       <c r="AN150" s="7"/>
+      <c r="AO150" s="7"/>
     </row>
     <row r="151">
       <c r="A151" s="7" t="inlineStr">
@@ -11417,6 +11571,7 @@
       <c r="AL151" s="7"/>
       <c r="AM151" s="7"/>
       <c r="AN151" s="7"/>
+      <c r="AO151" s="7"/>
     </row>
     <row r="152">
       <c r="A152" s="7" t="inlineStr">
@@ -11495,6 +11650,7 @@
       <c r="AL152" s="7"/>
       <c r="AM152" s="7"/>
       <c r="AN152" s="7"/>
+      <c r="AO152" s="7"/>
     </row>
     <row r="153">
       <c r="A153" s="7" t="inlineStr">
@@ -11577,6 +11733,7 @@
         </is>
       </c>
       <c r="AN153" s="7"/>
+      <c r="AO153" s="7"/>
     </row>
     <row r="154">
       <c r="A154" s="7" t="inlineStr">
@@ -11643,6 +11800,7 @@
       <c r="AL154" s="7"/>
       <c r="AM154" s="7"/>
       <c r="AN154" s="7"/>
+      <c r="AO154" s="7"/>
     </row>
     <row r="155">
       <c r="A155" s="7" t="inlineStr">
@@ -11713,6 +11871,7 @@
       <c r="AL155" s="7"/>
       <c r="AM155" s="7"/>
       <c r="AN155" s="7"/>
+      <c r="AO155" s="7"/>
     </row>
     <row r="156">
       <c r="A156" s="7" t="inlineStr">
@@ -11787,6 +11946,7 @@
       <c r="AL156" s="7"/>
       <c r="AM156" s="7"/>
       <c r="AN156" s="7"/>
+      <c r="AO156" s="7"/>
     </row>
     <row r="157">
       <c r="A157" s="7" t="inlineStr">
@@ -11857,6 +12017,7 @@
       <c r="AL157" s="7"/>
       <c r="AM157" s="7"/>
       <c r="AN157" s="7"/>
+      <c r="AO157" s="7"/>
     </row>
     <row r="158">
       <c r="A158" s="7" t="inlineStr">
@@ -11927,6 +12088,7 @@
       <c r="AL158" s="7"/>
       <c r="AM158" s="7"/>
       <c r="AN158" s="7"/>
+      <c r="AO158" s="7"/>
     </row>
     <row r="159">
       <c r="A159" s="7" t="inlineStr">
@@ -11997,6 +12159,7 @@
       <c r="AL159" s="7"/>
       <c r="AM159" s="7"/>
       <c r="AN159" s="7"/>
+      <c r="AO159" s="7"/>
     </row>
     <row r="160">
       <c r="A160" s="7" t="inlineStr">
@@ -12067,6 +12230,7 @@
       <c r="AL160" s="7"/>
       <c r="AM160" s="7"/>
       <c r="AN160" s="7"/>
+      <c r="AO160" s="7"/>
     </row>
     <row r="161">
       <c r="A161" s="7" t="inlineStr">
@@ -12141,6 +12305,7 @@
       <c r="AL161" s="7"/>
       <c r="AM161" s="7"/>
       <c r="AN161" s="7"/>
+      <c r="AO161" s="7"/>
     </row>
     <row r="162">
       <c r="A162" s="7" t="inlineStr">
@@ -12211,6 +12376,7 @@
       <c r="AL162" s="7"/>
       <c r="AM162" s="7"/>
       <c r="AN162" s="7"/>
+      <c r="AO162" s="7"/>
     </row>
     <row r="163">
       <c r="A163" s="7" t="inlineStr">
@@ -12281,6 +12447,7 @@
       <c r="AL163" s="7"/>
       <c r="AM163" s="7"/>
       <c r="AN163" s="7"/>
+      <c r="AO163" s="7"/>
     </row>
     <row r="164">
       <c r="A164" s="7" t="inlineStr">
@@ -12351,6 +12518,7 @@
       <c r="AL164" s="7"/>
       <c r="AM164" s="7"/>
       <c r="AN164" s="7"/>
+      <c r="AO164" s="7"/>
     </row>
     <row r="165">
       <c r="A165" s="7" t="inlineStr">
@@ -12421,6 +12589,7 @@
       <c r="AL165" s="7"/>
       <c r="AM165" s="7"/>
       <c r="AN165" s="7"/>
+      <c r="AO165" s="7"/>
     </row>
     <row r="166">
       <c r="A166" s="7" t="inlineStr">
@@ -12499,6 +12668,7 @@
         </is>
       </c>
       <c r="AN166" s="7"/>
+      <c r="AO166" s="7"/>
     </row>
     <row r="167">
       <c r="A167" s="7" t="inlineStr">
@@ -12573,6 +12743,7 @@
         </is>
       </c>
       <c r="AN167" s="7"/>
+      <c r="AO167" s="7"/>
     </row>
     <row r="168">
       <c r="A168" s="7" t="inlineStr">
@@ -12643,6 +12814,7 @@
       <c r="AL168" s="7"/>
       <c r="AM168" s="7"/>
       <c r="AN168" s="7"/>
+      <c r="AO168" s="7"/>
     </row>
     <row r="169">
       <c r="A169" s="7" t="inlineStr">
@@ -12713,6 +12885,7 @@
       <c r="AL169" s="7"/>
       <c r="AM169" s="7"/>
       <c r="AN169" s="7"/>
+      <c r="AO169" s="7"/>
     </row>
     <row r="170">
       <c r="A170" s="7" t="inlineStr">
@@ -12787,6 +12960,7 @@
       <c r="AL170" s="7"/>
       <c r="AM170" s="7"/>
       <c r="AN170" s="7"/>
+      <c r="AO170" s="7"/>
     </row>
     <row r="171">
       <c r="A171" s="7" t="inlineStr">
@@ -12853,6 +13027,7 @@
       <c r="AL171" s="7"/>
       <c r="AM171" s="7"/>
       <c r="AN171" s="7"/>
+      <c r="AO171" s="7"/>
     </row>
     <row r="172">
       <c r="A172" s="7" t="inlineStr">
@@ -12919,6 +13094,7 @@
       <c r="AL172" s="7"/>
       <c r="AM172" s="7"/>
       <c r="AN172" s="7"/>
+      <c r="AO172" s="7"/>
     </row>
     <row r="173">
       <c r="A173" s="7" t="inlineStr">
@@ -12993,6 +13169,7 @@
       <c r="AL173" s="7"/>
       <c r="AM173" s="7"/>
       <c r="AN173" s="7"/>
+      <c r="AO173" s="7"/>
     </row>
     <row r="174">
       <c r="A174" s="7" t="inlineStr">
@@ -13063,6 +13240,7 @@
       <c r="AL174" s="7"/>
       <c r="AM174" s="7"/>
       <c r="AN174" s="7"/>
+      <c r="AO174" s="7"/>
     </row>
     <row r="175">
       <c r="A175" s="7" t="inlineStr">
@@ -13137,6 +13315,7 @@
       <c r="AL175" s="7"/>
       <c r="AM175" s="7"/>
       <c r="AN175" s="7"/>
+      <c r="AO175" s="7"/>
     </row>
     <row r="176">
       <c r="A176" s="7" t="inlineStr">
@@ -13207,6 +13386,7 @@
       <c r="AL176" s="7"/>
       <c r="AM176" s="7"/>
       <c r="AN176" s="7"/>
+      <c r="AO176" s="7"/>
     </row>
     <row r="177">
       <c r="A177" s="7" t="inlineStr">
@@ -13277,6 +13457,7 @@
       <c r="AL177" s="7"/>
       <c r="AM177" s="7"/>
       <c r="AN177" s="7"/>
+      <c r="AO177" s="7"/>
     </row>
     <row r="178">
       <c r="A178" s="7" t="inlineStr">
@@ -13347,6 +13528,7 @@
       <c r="AL178" s="7"/>
       <c r="AM178" s="7"/>
       <c r="AN178" s="7"/>
+      <c r="AO178" s="7"/>
     </row>
     <row r="179">
       <c r="A179" s="7" t="inlineStr">
@@ -13417,6 +13599,7 @@
       <c r="AL179" s="7"/>
       <c r="AM179" s="7"/>
       <c r="AN179" s="7"/>
+      <c r="AO179" s="7"/>
     </row>
     <row r="180">
       <c r="A180" s="7" t="inlineStr">
@@ -13487,6 +13670,7 @@
       <c r="AL180" s="7"/>
       <c r="AM180" s="7"/>
       <c r="AN180" s="7"/>
+      <c r="AO180" s="7"/>
     </row>
     <row r="181">
       <c r="A181" s="7" t="inlineStr">
@@ -13557,6 +13741,7 @@
       <c r="AL181" s="7"/>
       <c r="AM181" s="7"/>
       <c r="AN181" s="7"/>
+      <c r="AO181" s="7"/>
     </row>
     <row r="182">
       <c r="A182" s="7" t="inlineStr">
@@ -13627,6 +13812,7 @@
       <c r="AL182" s="7"/>
       <c r="AM182" s="7"/>
       <c r="AN182" s="7"/>
+      <c r="AO182" s="7"/>
     </row>
     <row r="183">
       <c r="A183" s="7" t="inlineStr">
@@ -13697,6 +13883,7 @@
       <c r="AL183" s="7"/>
       <c r="AM183" s="7"/>
       <c r="AN183" s="7"/>
+      <c r="AO183" s="7"/>
     </row>
     <row r="184">
       <c r="A184" s="7" t="inlineStr">
@@ -13763,6 +13950,7 @@
       <c r="AL184" s="7"/>
       <c r="AM184" s="7"/>
       <c r="AN184" s="7"/>
+      <c r="AO184" s="7"/>
     </row>
     <row r="185">
       <c r="A185" s="7" t="inlineStr">
@@ -13833,6 +14021,7 @@
       <c r="AL185" s="7"/>
       <c r="AM185" s="7"/>
       <c r="AN185" s="7"/>
+      <c r="AO185" s="7"/>
     </row>
     <row r="186">
       <c r="A186" s="7" t="inlineStr">
@@ -13903,6 +14092,7 @@
       <c r="AL186" s="7"/>
       <c r="AM186" s="7"/>
       <c r="AN186" s="7"/>
+      <c r="AO186" s="7"/>
     </row>
     <row r="187">
       <c r="A187" s="7" t="inlineStr">
@@ -13977,6 +14167,7 @@
         </is>
       </c>
       <c r="AN187" s="7"/>
+      <c r="AO187" s="7"/>
     </row>
     <row r="188">
       <c r="A188" s="7" t="inlineStr">
@@ -14051,6 +14242,7 @@
         </is>
       </c>
       <c r="AN188" s="7"/>
+      <c r="AO188" s="7"/>
     </row>
     <row r="189">
       <c r="A189" s="7" t="inlineStr">
@@ -14125,6 +14317,7 @@
         </is>
       </c>
       <c r="AN189" s="7"/>
+      <c r="AO189" s="7"/>
     </row>
     <row r="190">
       <c r="A190" s="7" t="inlineStr">
@@ -14199,6 +14392,7 @@
         </is>
       </c>
       <c r="AN190" s="7"/>
+      <c r="AO190" s="7"/>
     </row>
     <row r="191">
       <c r="A191" s="7" t="inlineStr">
@@ -14273,6 +14467,7 @@
       <c r="AL191" s="7"/>
       <c r="AM191" s="7"/>
       <c r="AN191" s="7"/>
+      <c r="AO191" s="7"/>
     </row>
     <row r="192">
       <c r="A192" s="7" t="inlineStr">
@@ -14347,6 +14542,7 @@
         </is>
       </c>
       <c r="AN192" s="7"/>
+      <c r="AO192" s="7"/>
     </row>
     <row r="193">
       <c r="A193" s="7" t="inlineStr">
@@ -14421,6 +14617,7 @@
         </is>
       </c>
       <c r="AN193" s="7"/>
+      <c r="AO193" s="7"/>
     </row>
     <row r="194">
       <c r="A194" s="7" t="inlineStr">
@@ -14495,6 +14692,7 @@
         </is>
       </c>
       <c r="AN194" s="7"/>
+      <c r="AO194" s="7"/>
     </row>
     <row r="195">
       <c r="A195" s="7" t="inlineStr">
@@ -14569,6 +14767,7 @@
         </is>
       </c>
       <c r="AN195" s="7"/>
+      <c r="AO195" s="7"/>
     </row>
     <row r="196">
       <c r="A196" s="7" t="inlineStr">
@@ -14639,6 +14838,7 @@
         </is>
       </c>
       <c r="AN196" s="7"/>
+      <c r="AO196" s="7"/>
     </row>
     <row r="197">
       <c r="A197" s="7" t="inlineStr">
@@ -14713,6 +14913,7 @@
         </is>
       </c>
       <c r="AN197" s="7"/>
+      <c r="AO197" s="7"/>
     </row>
     <row r="198">
       <c r="A198" s="7" t="inlineStr">
@@ -14783,6 +14984,7 @@
         </is>
       </c>
       <c r="AN198" s="7"/>
+      <c r="AO198" s="7"/>
     </row>
     <row r="199">
       <c r="A199" s="7" t="inlineStr">
@@ -14857,6 +15059,7 @@
         </is>
       </c>
       <c r="AN199" s="7"/>
+      <c r="AO199" s="7"/>
     </row>
     <row r="200">
       <c r="A200" s="7" t="inlineStr">
@@ -14931,6 +15134,7 @@
         </is>
       </c>
       <c r="AN200" s="7"/>
+      <c r="AO200" s="7"/>
     </row>
     <row r="201">
       <c r="A201" s="7" t="inlineStr">
@@ -14997,6 +15201,7 @@
       <c r="AL201" s="7"/>
       <c r="AM201" s="7"/>
       <c r="AN201" s="7"/>
+      <c r="AO201" s="7"/>
     </row>
     <row r="202">
       <c r="A202" s="7" t="inlineStr">
@@ -15071,6 +15276,7 @@
         </is>
       </c>
       <c r="AN202" s="7"/>
+      <c r="AO202" s="7"/>
     </row>
     <row r="203">
       <c r="A203" s="7" t="inlineStr">
@@ -15145,6 +15351,7 @@
         </is>
       </c>
       <c r="AN203" s="7"/>
+      <c r="AO203" s="7"/>
     </row>
     <row r="204">
       <c r="A204" s="7" t="inlineStr">
@@ -15219,6 +15426,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AO204" s="7"/>
     </row>
     <row r="205">
       <c r="A205" s="7" t="inlineStr">
@@ -15293,6 +15501,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AO205" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="7" t="inlineStr">
@@ -15363,6 +15576,11 @@
         </is>
       </c>
       <c r="AN206" s="7"/>
+      <c r="AO206" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="7" t="inlineStr">
@@ -15433,6 +15651,7 @@
         </is>
       </c>
       <c r="AN207" s="7"/>
+      <c r="AO207" s="7"/>
     </row>
     <row r="208">
       <c r="A208" s="7" t="inlineStr">
@@ -15503,6 +15722,7 @@
         </is>
       </c>
       <c r="AN208" s="7"/>
+      <c r="AO208" s="7"/>
     </row>
     <row r="209">
       <c r="A209" s="7" t="inlineStr">
@@ -15532,7 +15752,7 @@
       </c>
       <c r="F209" t="inlineStr">
         <is>
-          <t xml:space="preserve">#199 · 꼴 ⚠️ 가정 · 고철은 글자(아이콘 아님 · 구현 판단)</t>
+          <t xml:space="preserve">#199 · 꼴 ⚠️ 가정 · 고철은 글자(아이콘 아님 · 구현 판단) · 10-19 #202 로 「Lv 1 · 피해량 ×1.00」 꼴</t>
         </is>
       </c>
       <c r="G209" s="7"/>
@@ -15573,6 +15793,82 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AO209" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_202</t>
+        </is>
+      </c>
+      <c r="B210" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼</t>
+        </is>
+      </c>
+      <c r="C210" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투 정지</t>
+        </is>
+      </c>
+      <c r="D210" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S1 · S3 · S6 막</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S1 T3 막(안내 창까지) · S3 강화 막 · S6 B 강화 막이 선 동안 적 · 발사 · 태그 Auto · 합체 게이지 · 리젠 시계가 멈추고(물류 보드는 계속), 막이 걷히면 이어서 도는가? S2 T4 · S4 · S5 막은 안 멈추는가?</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#203 · 범위 = 사용자 「S1 S3 S6」 · 물류 계속 ⚠️ 가정</t>
+        </is>
+      </c>
+      <c r="G210" s="7"/>
+      <c r="H210" s="7"/>
+      <c r="I210" s="7"/>
+      <c r="J210" s="7"/>
+      <c r="K210" s="7"/>
+      <c r="L210" s="7"/>
+      <c r="M210" s="7"/>
+      <c r="N210" s="7"/>
+      <c r="O210" s="7"/>
+      <c r="P210" s="7"/>
+      <c r="Q210" s="7"/>
+      <c r="R210" s="7"/>
+      <c r="S210" s="7"/>
+      <c r="T210" s="7"/>
+      <c r="U210" s="7"/>
+      <c r="V210" s="7"/>
+      <c r="W210" s="7"/>
+      <c r="X210" s="7"/>
+      <c r="Y210" s="7"/>
+      <c r="Z210" s="7"/>
+      <c r="AA210" s="7"/>
+      <c r="AB210" s="7"/>
+      <c r="AC210" s="7"/>
+      <c r="AD210" s="7"/>
+      <c r="AE210" s="7"/>
+      <c r="AF210" s="7"/>
+      <c r="AG210" s="7"/>
+      <c r="AH210" s="7"/>
+      <c r="AI210" s="7"/>
+      <c r="AJ210" s="7"/>
+      <c r="AK210" s="7"/>
+      <c r="AL210" s="7"/>
+      <c r="AM210" s="7"/>
+      <c r="AN210" s="7"/>
+      <c r="AO210" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="26">
@@ -15601,9 +15897,9 @@
     <mergeCell ref="B92:B99"/>
     <mergeCell ref="B100:B106"/>
     <mergeCell ref="B107:B111"/>
-    <mergeCell ref="G7:AN7"/>
+    <mergeCell ref="G7:AO7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:AN209">
+  <conditionalFormatting sqref="G9:AO210">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
docs: QA AP열(109e859 · CID_203 #204) · 가이드 8133 후보 109e859
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -197,8 +197,9 @@
     <col min="39" max="39" width="12" customWidth="1"/>
     <col min="40" max="40" width="12" customWidth="1"/>
     <col min="41" max="41" width="12" customWidth="1"/>
-    <col min="42" max="42" width="11" customWidth="1"/>
+    <col min="42" max="42" width="12" customWidth="1"/>
     <col min="43" max="43" width="11" customWidth="1"/>
+    <col min="44" max="44" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -486,6 +487,11 @@
       <c r="AO6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">8133 갈아엎음(21:33:11) · #202 팝오버 「Lv · 피해량 ×」 · #203 튜토리얼 막 동안 전투 정지 ‖ 10-19 사용자 육안(e86eb9a · 21:2x) = 팝오버 Lv 줄 · 창 [취소] 왼쪽 · S6 B 강화 ✅ / 코드 세션(8123): 바로가기 S3 = 강화 막 동안 적 · 리젠 00:10 정지 · 바로가기 S6 = B 막 동안 쿨다운 5.0s · 게이지 0% · 리젠 정지(Auto 태그 안 나감) ✅ · 정지 중 HUD 전투력 = 보드 예상 출력(첫 판 390 명목값 멈춤 → 0 → 예상 출력으로 고침 · 구현 판단) · S1 T3 정지 · 강화 뒤 재개 = 화면 미확인(시험)</t>
+        </is>
+      </c>
+      <c r="AP6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8133 갈아엎음(22:03:24) · #204 S3 파밍 장갑 hp 600→300 · S4 파밍 정원 18→10(8·1·1) ‖ 하네스: 전투 12줄 불변 · 파밍 A 단독 S3 생존 HP 바닥 593 · S4 생존 723 · 두 로봇(S5 · S6) 생존(표 Docs/261019_farm_tag.md) / 화면(8133 사용자 저장): 바로가기 S4 파밍 「맵 7/10」 ✅ · S3 화면 생존 = 미확인(육안 자리)</t>
         </is>
       </c>
     </row>
@@ -551,14 +557,15 @@
       <c r="AM7" s="2"/>
       <c r="AN7" s="2"/>
       <c r="AO7" s="2"/>
-      <c r="AP7" s="2" t="inlineStr">
+      <c r="AP7" s="2"/>
+      <c r="AQ7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">버전</t>
         </is>
       </c>
-      <c r="AQ7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6fb2f5e</t>
+      <c r="AR7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">109e859</t>
         </is>
       </c>
     </row>
@@ -758,11 +765,16 @@
       </c>
       <c r="AP8" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">109e859</t>
+        </is>
+      </c>
+      <c r="AQ8" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">PASSrate</t>
         </is>
       </c>
-      <c r="AQ8" s="7">
-        <f>COUNTIF(AO9:AO210,"Pass")</f>
+      <c r="AR8" s="7">
+        <f>COUNTIF(AP9:AP211,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -867,13 +879,14 @@
       <c r="AM9" s="7"/>
       <c r="AN9" s="7"/>
       <c r="AO9" s="7"/>
-      <c r="AP9" s="2" t="inlineStr">
+      <c r="AP9" s="7"/>
+      <c r="AQ9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FAILrate</t>
         </is>
       </c>
-      <c r="AQ9" s="7">
-        <f>COUNTIF(AO9:AO210,"Fail")+COUNTIF(AO9:AO210,"Broken")</f>
+      <c r="AR9" s="7">
+        <f>COUNTIF(AP9:AP211,"Fail")+COUNTIF(AP9:AP211,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -942,13 +955,14 @@
       <c r="AM10" s="7"/>
       <c r="AN10" s="7"/>
       <c r="AO10" s="7"/>
-      <c r="AP10" s="2" t="inlineStr">
+      <c r="AP10" s="7"/>
+      <c r="AQ10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">N/A</t>
         </is>
       </c>
-      <c r="AQ10" s="7">
-        <f>COUNTIF(AO9:AO210,"N/A")</f>
+      <c r="AR10" s="7">
+        <f>COUNTIF(AP9:AP211,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -1017,13 +1031,14 @@
       <c r="AM11" s="7"/>
       <c r="AN11" s="7"/>
       <c r="AO11" s="7"/>
-      <c r="AP11" s="2" t="inlineStr">
+      <c r="AP11" s="7"/>
+      <c r="AQ11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">전체 개수</t>
         </is>
       </c>
-      <c r="AQ11" s="7">
-        <v>202</v>
+      <c r="AR11" s="7">
+        <v>203</v>
       </c>
     </row>
     <row r="12">
@@ -1092,13 +1107,14 @@
       <c r="AM12" s="7"/>
       <c r="AN12" s="7"/>
       <c r="AO12" s="7"/>
-      <c r="AP12" s="2" t="inlineStr">
+      <c r="AP12" s="7"/>
+      <c r="AQ12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">진행율</t>
         </is>
       </c>
-      <c r="AQ12" s="7">
-        <f>TEXT((COUNTA(AO9:AO210))/202,"0.00%")</f>
+      <c r="AR12" s="7">
+        <f>TEXT((COUNTA(AP9:AP211))/203,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -1171,6 +1187,7 @@
       <c r="AM13" s="7"/>
       <c r="AN13" s="7"/>
       <c r="AO13" s="7"/>
+      <c r="AP13" s="7"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -1233,6 +1250,7 @@
       <c r="AM14" s="7"/>
       <c r="AN14" s="7"/>
       <c r="AO14" s="7"/>
+      <c r="AP14" s="7"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -1331,6 +1349,7 @@
       <c r="AM15" s="7"/>
       <c r="AN15" s="7"/>
       <c r="AO15" s="7"/>
+      <c r="AP15" s="7"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -1429,6 +1448,7 @@
       <c r="AM16" s="7"/>
       <c r="AN16" s="7"/>
       <c r="AO16" s="7"/>
+      <c r="AP16" s="7"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -1532,6 +1552,7 @@
       <c r="AM17" s="7"/>
       <c r="AN17" s="7"/>
       <c r="AO17" s="7"/>
+      <c r="AP17" s="7"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -1599,6 +1620,7 @@
       <c r="AM18" s="7"/>
       <c r="AN18" s="7"/>
       <c r="AO18" s="7"/>
+      <c r="AP18" s="7"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -1661,6 +1683,7 @@
       <c r="AM19" s="7"/>
       <c r="AN19" s="7"/>
       <c r="AO19" s="7"/>
+      <c r="AP19" s="7"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1723,6 +1746,7 @@
       <c r="AM20" s="7"/>
       <c r="AN20" s="7"/>
       <c r="AO20" s="7"/>
+      <c r="AP20" s="7"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1821,6 +1845,7 @@
       <c r="AM21" s="7"/>
       <c r="AN21" s="7"/>
       <c r="AO21" s="7"/>
+      <c r="AP21" s="7"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1912,6 +1937,7 @@
       <c r="AM22" s="7"/>
       <c r="AN22" s="7"/>
       <c r="AO22" s="7"/>
+      <c r="AP22" s="7"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -1982,6 +2008,7 @@
       <c r="AM23" s="7"/>
       <c r="AN23" s="7"/>
       <c r="AO23" s="7"/>
+      <c r="AP23" s="7"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -2044,6 +2071,7 @@
       <c r="AM24" s="7"/>
       <c r="AN24" s="7"/>
       <c r="AO24" s="7"/>
+      <c r="AP24" s="7"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -2106,6 +2134,7 @@
       <c r="AM25" s="7"/>
       <c r="AN25" s="7"/>
       <c r="AO25" s="7"/>
+      <c r="AP25" s="7"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -2197,6 +2226,7 @@
       <c r="AM26" s="7"/>
       <c r="AN26" s="7"/>
       <c r="AO26" s="7"/>
+      <c r="AP26" s="7"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -2263,6 +2293,7 @@
       <c r="AM27" s="7"/>
       <c r="AN27" s="7"/>
       <c r="AO27" s="7"/>
+      <c r="AP27" s="7"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -2338,6 +2369,7 @@
       <c r="AM28" s="7"/>
       <c r="AN28" s="7"/>
       <c r="AO28" s="7"/>
+      <c r="AP28" s="7"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -2408,6 +2440,7 @@
       <c r="AM29" s="7"/>
       <c r="AN29" s="7"/>
       <c r="AO29" s="7"/>
+      <c r="AP29" s="7"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -2502,6 +2535,7 @@
       <c r="AM30" s="7"/>
       <c r="AN30" s="7"/>
       <c r="AO30" s="7"/>
+      <c r="AP30" s="7"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -2601,6 +2635,7 @@
       <c r="AM31" s="7"/>
       <c r="AN31" s="7"/>
       <c r="AO31" s="7"/>
+      <c r="AP31" s="7"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -2687,6 +2722,7 @@
       <c r="AM32" s="7"/>
       <c r="AN32" s="7"/>
       <c r="AO32" s="7"/>
+      <c r="AP32" s="7"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -2781,6 +2817,7 @@
       <c r="AM33" s="7"/>
       <c r="AN33" s="7"/>
       <c r="AO33" s="7"/>
+      <c r="AP33" s="7"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -2875,6 +2912,7 @@
       <c r="AM34" s="7"/>
       <c r="AN34" s="7"/>
       <c r="AO34" s="7"/>
+      <c r="AP34" s="7"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -2978,6 +3016,7 @@
       <c r="AM35" s="7"/>
       <c r="AN35" s="7"/>
       <c r="AO35" s="7"/>
+      <c r="AP35" s="7"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -3056,6 +3095,7 @@
       <c r="AM36" s="7"/>
       <c r="AN36" s="7"/>
       <c r="AO36" s="7"/>
+      <c r="AP36" s="7"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -3118,6 +3158,7 @@
       <c r="AM37" s="7"/>
       <c r="AN37" s="7"/>
       <c r="AO37" s="7"/>
+      <c r="AP37" s="7"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -3201,6 +3242,7 @@
       <c r="AM38" s="7"/>
       <c r="AN38" s="7"/>
       <c r="AO38" s="7"/>
+      <c r="AP38" s="7"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -3295,6 +3337,7 @@
       <c r="AM39" s="7"/>
       <c r="AN39" s="7"/>
       <c r="AO39" s="7"/>
+      <c r="AP39" s="7"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -3390,6 +3433,7 @@
       <c r="AM40" s="7"/>
       <c r="AN40" s="7"/>
       <c r="AO40" s="7"/>
+      <c r="AP40" s="7"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -3480,6 +3524,7 @@
       <c r="AM41" s="7"/>
       <c r="AN41" s="7"/>
       <c r="AO41" s="7"/>
+      <c r="AP41" s="7"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -3554,6 +3599,7 @@
       <c r="AM42" s="7"/>
       <c r="AN42" s="7"/>
       <c r="AO42" s="7"/>
+      <c r="AP42" s="7"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -3648,6 +3694,7 @@
       <c r="AM43" s="7"/>
       <c r="AN43" s="7"/>
       <c r="AO43" s="7"/>
+      <c r="AP43" s="7"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -3715,6 +3762,7 @@
       <c r="AM44" s="7"/>
       <c r="AN44" s="7"/>
       <c r="AO44" s="7"/>
+      <c r="AP44" s="7"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -3805,6 +3853,7 @@
       <c r="AM45" s="7"/>
       <c r="AN45" s="7"/>
       <c r="AO45" s="7"/>
+      <c r="AP45" s="7"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -3895,6 +3944,7 @@
       <c r="AM46" s="7"/>
       <c r="AN46" s="7"/>
       <c r="AO46" s="7"/>
+      <c r="AP46" s="7"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -3962,6 +4012,7 @@
       <c r="AM47" s="7"/>
       <c r="AN47" s="7"/>
       <c r="AO47" s="7"/>
+      <c r="AP47" s="7"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -4024,6 +4075,7 @@
       <c r="AM48" s="7"/>
       <c r="AN48" s="7"/>
       <c r="AO48" s="7"/>
+      <c r="AP48" s="7"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -4086,6 +4138,7 @@
       <c r="AM49" s="7"/>
       <c r="AN49" s="7"/>
       <c r="AO49" s="7"/>
+      <c r="AP49" s="7"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -4172,6 +4225,7 @@
       <c r="AM50" s="7"/>
       <c r="AN50" s="7"/>
       <c r="AO50" s="7"/>
+      <c r="AP50" s="7"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -4258,6 +4312,7 @@
       <c r="AM51" s="7"/>
       <c r="AN51" s="7"/>
       <c r="AO51" s="7"/>
+      <c r="AP51" s="7"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -4325,6 +4380,7 @@
       <c r="AM52" s="7"/>
       <c r="AN52" s="7"/>
       <c r="AO52" s="7"/>
+      <c r="AP52" s="7"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -4392,6 +4448,7 @@
       <c r="AM53" s="7"/>
       <c r="AN53" s="7"/>
       <c r="AO53" s="7"/>
+      <c r="AP53" s="7"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -4454,6 +4511,7 @@
       <c r="AM54" s="7"/>
       <c r="AN54" s="7"/>
       <c r="AO54" s="7"/>
+      <c r="AP54" s="7"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -4552,6 +4610,7 @@
       <c r="AM55" s="7"/>
       <c r="AN55" s="7"/>
       <c r="AO55" s="7"/>
+      <c r="AP55" s="7"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -4630,6 +4689,7 @@
       <c r="AM56" s="7"/>
       <c r="AN56" s="7"/>
       <c r="AO56" s="7"/>
+      <c r="AP56" s="7"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -4717,6 +4777,7 @@
       <c r="AM57" s="7"/>
       <c r="AN57" s="7"/>
       <c r="AO57" s="7"/>
+      <c r="AP57" s="7"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -4812,6 +4873,7 @@
       <c r="AM58" s="7"/>
       <c r="AN58" s="7"/>
       <c r="AO58" s="7"/>
+      <c r="AP58" s="7"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -4874,6 +4936,7 @@
       <c r="AM59" s="7"/>
       <c r="AN59" s="7"/>
       <c r="AO59" s="7"/>
+      <c r="AP59" s="7"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -4936,6 +4999,7 @@
       <c r="AM60" s="7"/>
       <c r="AN60" s="7"/>
       <c r="AO60" s="7"/>
+      <c r="AP60" s="7"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -5010,6 +5074,7 @@
       <c r="AM61" s="7"/>
       <c r="AN61" s="7"/>
       <c r="AO61" s="7"/>
+      <c r="AP61" s="7"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -5092,6 +5157,7 @@
       <c r="AM62" s="7"/>
       <c r="AN62" s="7"/>
       <c r="AO62" s="7"/>
+      <c r="AP62" s="7"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -5166,6 +5232,7 @@
       <c r="AM63" s="7"/>
       <c r="AN63" s="7"/>
       <c r="AO63" s="7"/>
+      <c r="AP63" s="7"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -5228,6 +5295,7 @@
       <c r="AM64" s="7"/>
       <c r="AN64" s="7"/>
       <c r="AO64" s="7"/>
+      <c r="AP64" s="7"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -5295,6 +5363,7 @@
       <c r="AM65" s="7"/>
       <c r="AN65" s="7"/>
       <c r="AO65" s="7"/>
+      <c r="AP65" s="7"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
@@ -5369,6 +5438,7 @@
       <c r="AM66" s="7"/>
       <c r="AN66" s="7"/>
       <c r="AO66" s="7"/>
+      <c r="AP66" s="7"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -5431,6 +5501,7 @@
       <c r="AM67" s="7"/>
       <c r="AN67" s="7"/>
       <c r="AO67" s="7"/>
+      <c r="AP67" s="7"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
@@ -5497,6 +5568,7 @@
       <c r="AM68" s="7"/>
       <c r="AN68" s="7"/>
       <c r="AO68" s="7"/>
+      <c r="AP68" s="7"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -5595,6 +5667,7 @@
       <c r="AM69" s="7"/>
       <c r="AN69" s="7"/>
       <c r="AO69" s="7"/>
+      <c r="AP69" s="7"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
@@ -5657,6 +5730,7 @@
       <c r="AM70" s="7"/>
       <c r="AN70" s="7"/>
       <c r="AO70" s="7"/>
+      <c r="AP70" s="7"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -5724,6 +5798,7 @@
       <c r="AM71" s="7"/>
       <c r="AN71" s="7"/>
       <c r="AO71" s="7"/>
+      <c r="AP71" s="7"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
@@ -5802,6 +5877,7 @@
       <c r="AM72" s="7"/>
       <c r="AN72" s="7"/>
       <c r="AO72" s="7"/>
+      <c r="AP72" s="7"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
@@ -5869,6 +5945,7 @@
       <c r="AM73" s="7"/>
       <c r="AN73" s="7"/>
       <c r="AO73" s="7"/>
+      <c r="AP73" s="7"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -5931,6 +6008,7 @@
       <c r="AM74" s="7"/>
       <c r="AN74" s="7"/>
       <c r="AO74" s="7"/>
+      <c r="AP74" s="7"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -5993,6 +6071,7 @@
       <c r="AM75" s="7"/>
       <c r="AN75" s="7"/>
       <c r="AO75" s="7"/>
+      <c r="AP75" s="7"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -6055,6 +6134,7 @@
       <c r="AM76" s="7"/>
       <c r="AN76" s="7"/>
       <c r="AO76" s="7"/>
+      <c r="AP76" s="7"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -6121,6 +6201,7 @@
       <c r="AM77" s="7"/>
       <c r="AN77" s="7"/>
       <c r="AO77" s="7"/>
+      <c r="AP77" s="7"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
@@ -6183,6 +6264,7 @@
       <c r="AM78" s="7"/>
       <c r="AN78" s="7"/>
       <c r="AO78" s="7"/>
+      <c r="AP78" s="7"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -6250,6 +6332,7 @@
       <c r="AM79" s="7"/>
       <c r="AN79" s="7"/>
       <c r="AO79" s="7"/>
+      <c r="AP79" s="7"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
@@ -6328,6 +6411,7 @@
       <c r="AM80" s="7"/>
       <c r="AN80" s="7"/>
       <c r="AO80" s="7"/>
+      <c r="AP80" s="7"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
@@ -6394,6 +6478,7 @@
       <c r="AM81" s="7"/>
       <c r="AN81" s="7"/>
       <c r="AO81" s="7"/>
+      <c r="AP81" s="7"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
@@ -6456,6 +6541,7 @@
       <c r="AM82" s="7"/>
       <c r="AN82" s="7"/>
       <c r="AO82" s="7"/>
+      <c r="AP82" s="7"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
@@ -6523,6 +6609,7 @@
       <c r="AM83" s="7"/>
       <c r="AN83" s="7"/>
       <c r="AO83" s="7"/>
+      <c r="AP83" s="7"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
@@ -6585,6 +6672,7 @@
       <c r="AM84" s="7"/>
       <c r="AN84" s="7"/>
       <c r="AO84" s="7"/>
+      <c r="AP84" s="7"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
@@ -6647,6 +6735,7 @@
       <c r="AM85" s="7"/>
       <c r="AN85" s="7"/>
       <c r="AO85" s="7"/>
+      <c r="AP85" s="7"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
@@ -6714,6 +6803,7 @@
       <c r="AM86" s="7"/>
       <c r="AN86" s="7"/>
       <c r="AO86" s="7"/>
+      <c r="AP86" s="7"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
@@ -6776,6 +6866,7 @@
       <c r="AM87" s="7"/>
       <c r="AN87" s="7"/>
       <c r="AO87" s="7"/>
+      <c r="AP87" s="7"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
@@ -6838,6 +6929,7 @@
       <c r="AM88" s="7"/>
       <c r="AN88" s="7"/>
       <c r="AO88" s="7"/>
+      <c r="AP88" s="7"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
@@ -6900,6 +6992,7 @@
       <c r="AM89" s="7"/>
       <c r="AN89" s="7"/>
       <c r="AO89" s="7"/>
+      <c r="AP89" s="7"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
@@ -6991,6 +7084,7 @@
       <c r="AM90" s="7"/>
       <c r="AN90" s="7"/>
       <c r="AO90" s="7"/>
+      <c r="AP90" s="7"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
@@ -7053,6 +7147,7 @@
       <c r="AM91" s="7"/>
       <c r="AN91" s="7"/>
       <c r="AO91" s="7"/>
+      <c r="AP91" s="7"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
@@ -7151,6 +7246,7 @@
       <c r="AM92" s="7"/>
       <c r="AN92" s="7"/>
       <c r="AO92" s="7"/>
+      <c r="AP92" s="7"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
@@ -7254,6 +7350,7 @@
       <c r="AM93" s="7"/>
       <c r="AN93" s="7"/>
       <c r="AO93" s="7"/>
+      <c r="AP93" s="7"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
@@ -7321,6 +7418,7 @@
       <c r="AM94" s="7"/>
       <c r="AN94" s="7"/>
       <c r="AO94" s="7"/>
+      <c r="AP94" s="7"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
@@ -7388,6 +7486,7 @@
       <c r="AM95" s="7"/>
       <c r="AN95" s="7"/>
       <c r="AO95" s="7"/>
+      <c r="AP95" s="7"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
@@ -7474,6 +7573,7 @@
       <c r="AM96" s="7"/>
       <c r="AN96" s="7"/>
       <c r="AO96" s="7"/>
+      <c r="AP96" s="7"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="inlineStr">
@@ -7536,6 +7636,7 @@
       <c r="AM97" s="7"/>
       <c r="AN97" s="7"/>
       <c r="AO97" s="7"/>
+      <c r="AP97" s="7"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
@@ -7598,6 +7699,7 @@
       <c r="AM98" s="7"/>
       <c r="AN98" s="7"/>
       <c r="AO98" s="7"/>
+      <c r="AP98" s="7"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
@@ -7660,6 +7762,7 @@
       <c r="AM99" s="7"/>
       <c r="AN99" s="7"/>
       <c r="AO99" s="7"/>
+      <c r="AP99" s="7"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
@@ -7731,6 +7834,7 @@
       <c r="AM100" s="7"/>
       <c r="AN100" s="7"/>
       <c r="AO100" s="7"/>
+      <c r="AP100" s="7"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
@@ -7793,6 +7897,7 @@
       <c r="AM101" s="7"/>
       <c r="AN101" s="7"/>
       <c r="AO101" s="7"/>
+      <c r="AP101" s="7"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
@@ -7855,6 +7960,7 @@
       <c r="AM102" s="7"/>
       <c r="AN102" s="7"/>
       <c r="AO102" s="7"/>
+      <c r="AP102" s="7"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="inlineStr">
@@ -7917,6 +8023,7 @@
       <c r="AM103" s="7"/>
       <c r="AN103" s="7"/>
       <c r="AO103" s="7"/>
+      <c r="AP103" s="7"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="inlineStr">
@@ -7984,6 +8091,7 @@
       <c r="AM104" s="7"/>
       <c r="AN104" s="7"/>
       <c r="AO104" s="7"/>
+      <c r="AP104" s="7"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
@@ -8046,6 +8154,7 @@
       <c r="AM105" s="7"/>
       <c r="AN105" s="7"/>
       <c r="AO105" s="7"/>
+      <c r="AP105" s="7"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
@@ -8108,6 +8217,7 @@
       <c r="AM106" s="7"/>
       <c r="AN106" s="7"/>
       <c r="AO106" s="7"/>
+      <c r="AP106" s="7"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
@@ -8170,6 +8280,7 @@
       <c r="AM107" s="7"/>
       <c r="AN107" s="7"/>
       <c r="AO107" s="7"/>
+      <c r="AP107" s="7"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
@@ -8236,6 +8347,7 @@
       <c r="AM108" s="7"/>
       <c r="AN108" s="7"/>
       <c r="AO108" s="7"/>
+      <c r="AP108" s="7"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="inlineStr">
@@ -8307,6 +8419,7 @@
       <c r="AM109" s="7"/>
       <c r="AN109" s="7"/>
       <c r="AO109" s="7"/>
+      <c r="AP109" s="7"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
@@ -8386,6 +8499,7 @@
       <c r="AM110" s="7"/>
       <c r="AN110" s="7"/>
       <c r="AO110" s="7"/>
+      <c r="AP110" s="7"/>
     </row>
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
@@ -8468,6 +8582,7 @@
       <c r="AM111" s="7"/>
       <c r="AN111" s="7"/>
       <c r="AO111" s="7"/>
+      <c r="AP111" s="7"/>
     </row>
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
@@ -8547,6 +8662,7 @@
       <c r="AM112" s="7"/>
       <c r="AN112" s="7"/>
       <c r="AO112" s="7"/>
+      <c r="AP112" s="7"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
@@ -8618,6 +8734,7 @@
       <c r="AM113" s="7"/>
       <c r="AN113" s="7"/>
       <c r="AO113" s="7"/>
+      <c r="AP113" s="7"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="inlineStr">
@@ -8705,6 +8822,7 @@
       <c r="AM114" s="7"/>
       <c r="AN114" s="7"/>
       <c r="AO114" s="7"/>
+      <c r="AP114" s="7"/>
     </row>
     <row r="115">
       <c r="A115" s="7" t="inlineStr">
@@ -8784,6 +8902,7 @@
       <c r="AM115" s="7"/>
       <c r="AN115" s="7"/>
       <c r="AO115" s="7"/>
+      <c r="AP115" s="7"/>
     </row>
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
@@ -8871,6 +8990,7 @@
       <c r="AM116" s="7"/>
       <c r="AN116" s="7"/>
       <c r="AO116" s="7"/>
+      <c r="AP116" s="7"/>
     </row>
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
@@ -8954,6 +9074,7 @@
       <c r="AM117" s="7"/>
       <c r="AN117" s="7"/>
       <c r="AO117" s="7"/>
+      <c r="AP117" s="7"/>
     </row>
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
@@ -9037,6 +9158,7 @@
       <c r="AM118" s="7"/>
       <c r="AN118" s="7"/>
       <c r="AO118" s="7"/>
+      <c r="AP118" s="7"/>
     </row>
     <row r="119">
       <c r="A119" s="7" t="inlineStr">
@@ -9116,6 +9238,7 @@
       <c r="AM119" s="7"/>
       <c r="AN119" s="7"/>
       <c r="AO119" s="7"/>
+      <c r="AP119" s="7"/>
     </row>
     <row r="120">
       <c r="A120" s="7" t="inlineStr">
@@ -9187,6 +9310,7 @@
       <c r="AM120" s="7"/>
       <c r="AN120" s="7"/>
       <c r="AO120" s="7"/>
+      <c r="AP120" s="7"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="inlineStr">
@@ -9270,6 +9394,7 @@
       <c r="AM121" s="7"/>
       <c r="AN121" s="7"/>
       <c r="AO121" s="7"/>
+      <c r="AP121" s="7"/>
     </row>
     <row r="122">
       <c r="A122" s="7" t="inlineStr">
@@ -9353,6 +9478,7 @@
       <c r="AM122" s="7"/>
       <c r="AN122" s="7"/>
       <c r="AO122" s="7"/>
+      <c r="AP122" s="7"/>
     </row>
     <row r="123">
       <c r="A123" s="7" t="inlineStr">
@@ -9424,6 +9550,7 @@
       <c r="AM123" s="7"/>
       <c r="AN123" s="7"/>
       <c r="AO123" s="7"/>
+      <c r="AP123" s="7"/>
     </row>
     <row r="124">
       <c r="A124" s="7" t="inlineStr">
@@ -9503,6 +9630,7 @@
       <c r="AM124" s="7"/>
       <c r="AN124" s="7"/>
       <c r="AO124" s="7"/>
+      <c r="AP124" s="7"/>
     </row>
     <row r="125">
       <c r="A125" s="7" t="inlineStr">
@@ -9574,6 +9702,7 @@
       <c r="AM125" s="7"/>
       <c r="AN125" s="7"/>
       <c r="AO125" s="7"/>
+      <c r="AP125" s="7"/>
     </row>
     <row r="126">
       <c r="A126" s="7" t="inlineStr">
@@ -9645,6 +9774,7 @@
       <c r="AM126" s="7"/>
       <c r="AN126" s="7"/>
       <c r="AO126" s="7"/>
+      <c r="AP126" s="7"/>
     </row>
     <row r="127">
       <c r="A127" s="7" t="inlineStr">
@@ -9720,6 +9850,7 @@
       <c r="AM127" s="7"/>
       <c r="AN127" s="7"/>
       <c r="AO127" s="7"/>
+      <c r="AP127" s="7"/>
     </row>
     <row r="128">
       <c r="A128" s="7" t="inlineStr">
@@ -9795,6 +9926,7 @@
       <c r="AM128" s="7"/>
       <c r="AN128" s="7"/>
       <c r="AO128" s="7"/>
+      <c r="AP128" s="7"/>
     </row>
     <row r="129">
       <c r="A129" s="7" t="inlineStr">
@@ -9870,6 +10002,7 @@
       <c r="AM129" s="7"/>
       <c r="AN129" s="7"/>
       <c r="AO129" s="7"/>
+      <c r="AP129" s="7"/>
     </row>
     <row r="130">
       <c r="A130" s="7" t="inlineStr">
@@ -9941,6 +10074,7 @@
       <c r="AM130" s="7"/>
       <c r="AN130" s="7"/>
       <c r="AO130" s="7"/>
+      <c r="AP130" s="7"/>
     </row>
     <row r="131">
       <c r="A131" s="7" t="inlineStr">
@@ -10020,6 +10154,7 @@
       <c r="AM131" s="7"/>
       <c r="AN131" s="7"/>
       <c r="AO131" s="7"/>
+      <c r="AP131" s="7"/>
     </row>
     <row r="132">
       <c r="A132" s="7" t="inlineStr">
@@ -10103,6 +10238,7 @@
       <c r="AM132" s="7"/>
       <c r="AN132" s="7"/>
       <c r="AO132" s="7"/>
+      <c r="AP132" s="7"/>
     </row>
     <row r="133">
       <c r="A133" s="7" t="inlineStr">
@@ -10186,6 +10322,7 @@
       <c r="AM133" s="7"/>
       <c r="AN133" s="7"/>
       <c r="AO133" s="7"/>
+      <c r="AP133" s="7"/>
     </row>
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
@@ -10265,6 +10402,7 @@
       <c r="AM134" s="7"/>
       <c r="AN134" s="7"/>
       <c r="AO134" s="7"/>
+      <c r="AP134" s="7"/>
     </row>
     <row r="135">
       <c r="A135" s="7" t="inlineStr">
@@ -10344,6 +10482,7 @@
       <c r="AM135" s="7"/>
       <c r="AN135" s="7"/>
       <c r="AO135" s="7"/>
+      <c r="AP135" s="7"/>
     </row>
     <row r="136">
       <c r="A136" s="7" t="inlineStr">
@@ -10423,6 +10562,7 @@
       <c r="AM136" s="7"/>
       <c r="AN136" s="7"/>
       <c r="AO136" s="7"/>
+      <c r="AP136" s="7"/>
     </row>
     <row r="137">
       <c r="A137" s="7" t="inlineStr">
@@ -10498,6 +10638,7 @@
       <c r="AM137" s="7"/>
       <c r="AN137" s="7"/>
       <c r="AO137" s="7"/>
+      <c r="AP137" s="7"/>
     </row>
     <row r="138">
       <c r="A138" s="7" t="inlineStr">
@@ -10573,6 +10714,7 @@
       <c r="AM138" s="7"/>
       <c r="AN138" s="7"/>
       <c r="AO138" s="7"/>
+      <c r="AP138" s="7"/>
     </row>
     <row r="139">
       <c r="A139" s="7" t="inlineStr">
@@ -10648,6 +10790,7 @@
       <c r="AM139" s="7"/>
       <c r="AN139" s="7"/>
       <c r="AO139" s="7"/>
+      <c r="AP139" s="7"/>
     </row>
     <row r="140">
       <c r="A140" s="7" t="inlineStr">
@@ -10719,6 +10862,7 @@
       <c r="AM140" s="7"/>
       <c r="AN140" s="7"/>
       <c r="AO140" s="7"/>
+      <c r="AP140" s="7"/>
     </row>
     <row r="141">
       <c r="A141" s="7" t="inlineStr">
@@ -10802,6 +10946,7 @@
       <c r="AM141" s="7"/>
       <c r="AN141" s="7"/>
       <c r="AO141" s="7"/>
+      <c r="AP141" s="7"/>
     </row>
     <row r="142">
       <c r="A142" s="7" t="inlineStr">
@@ -10873,6 +11018,7 @@
       <c r="AM142" s="7"/>
       <c r="AN142" s="7"/>
       <c r="AO142" s="7"/>
+      <c r="AP142" s="7"/>
     </row>
     <row r="143">
       <c r="A143" s="7" t="inlineStr">
@@ -10944,6 +11090,7 @@
       <c r="AM143" s="7"/>
       <c r="AN143" s="7"/>
       <c r="AO143" s="7"/>
+      <c r="AP143" s="7"/>
     </row>
     <row r="144">
       <c r="A144" s="7" t="inlineStr">
@@ -11015,6 +11162,7 @@
       <c r="AM144" s="7"/>
       <c r="AN144" s="7"/>
       <c r="AO144" s="7"/>
+      <c r="AP144" s="7"/>
     </row>
     <row r="145">
       <c r="A145" s="7" t="inlineStr">
@@ -11102,6 +11250,7 @@
       <c r="AM145" s="7"/>
       <c r="AN145" s="7"/>
       <c r="AO145" s="7"/>
+      <c r="AP145" s="7"/>
     </row>
     <row r="146">
       <c r="A146" s="7" t="inlineStr">
@@ -11177,6 +11326,7 @@
       <c r="AM146" s="7"/>
       <c r="AN146" s="7"/>
       <c r="AO146" s="7"/>
+      <c r="AP146" s="7"/>
     </row>
     <row r="147">
       <c r="A147" s="7" t="inlineStr">
@@ -11264,6 +11414,7 @@
       <c r="AM147" s="7"/>
       <c r="AN147" s="7"/>
       <c r="AO147" s="7"/>
+      <c r="AP147" s="7"/>
     </row>
     <row r="148">
       <c r="A148" s="7" t="inlineStr">
@@ -11335,6 +11486,7 @@
       <c r="AM148" s="7"/>
       <c r="AN148" s="7"/>
       <c r="AO148" s="7"/>
+      <c r="AP148" s="7"/>
     </row>
     <row r="149">
       <c r="A149" s="7" t="inlineStr">
@@ -11414,6 +11566,7 @@
       <c r="AM149" s="7"/>
       <c r="AN149" s="7"/>
       <c r="AO149" s="7"/>
+      <c r="AP149" s="7"/>
     </row>
     <row r="150">
       <c r="A150" s="7" t="inlineStr">
@@ -11497,6 +11650,7 @@
       <c r="AM150" s="7"/>
       <c r="AN150" s="7"/>
       <c r="AO150" s="7"/>
+      <c r="AP150" s="7"/>
     </row>
     <row r="151">
       <c r="A151" s="7" t="inlineStr">
@@ -11572,6 +11726,7 @@
       <c r="AM151" s="7"/>
       <c r="AN151" s="7"/>
       <c r="AO151" s="7"/>
+      <c r="AP151" s="7"/>
     </row>
     <row r="152">
       <c r="A152" s="7" t="inlineStr">
@@ -11651,6 +11806,7 @@
       <c r="AM152" s="7"/>
       <c r="AN152" s="7"/>
       <c r="AO152" s="7"/>
+      <c r="AP152" s="7"/>
     </row>
     <row r="153">
       <c r="A153" s="7" t="inlineStr">
@@ -11734,6 +11890,7 @@
       </c>
       <c r="AN153" s="7"/>
       <c r="AO153" s="7"/>
+      <c r="AP153" s="7"/>
     </row>
     <row r="154">
       <c r="A154" s="7" t="inlineStr">
@@ -11801,6 +11958,7 @@
       <c r="AM154" s="7"/>
       <c r="AN154" s="7"/>
       <c r="AO154" s="7"/>
+      <c r="AP154" s="7"/>
     </row>
     <row r="155">
       <c r="A155" s="7" t="inlineStr">
@@ -11872,6 +12030,7 @@
       <c r="AM155" s="7"/>
       <c r="AN155" s="7"/>
       <c r="AO155" s="7"/>
+      <c r="AP155" s="7"/>
     </row>
     <row r="156">
       <c r="A156" s="7" t="inlineStr">
@@ -11947,6 +12106,7 @@
       <c r="AM156" s="7"/>
       <c r="AN156" s="7"/>
       <c r="AO156" s="7"/>
+      <c r="AP156" s="7"/>
     </row>
     <row r="157">
       <c r="A157" s="7" t="inlineStr">
@@ -12018,6 +12178,7 @@
       <c r="AM157" s="7"/>
       <c r="AN157" s="7"/>
       <c r="AO157" s="7"/>
+      <c r="AP157" s="7"/>
     </row>
     <row r="158">
       <c r="A158" s="7" t="inlineStr">
@@ -12089,6 +12250,7 @@
       <c r="AM158" s="7"/>
       <c r="AN158" s="7"/>
       <c r="AO158" s="7"/>
+      <c r="AP158" s="7"/>
     </row>
     <row r="159">
       <c r="A159" s="7" t="inlineStr">
@@ -12160,6 +12322,7 @@
       <c r="AM159" s="7"/>
       <c r="AN159" s="7"/>
       <c r="AO159" s="7"/>
+      <c r="AP159" s="7"/>
     </row>
     <row r="160">
       <c r="A160" s="7" t="inlineStr">
@@ -12231,6 +12394,7 @@
       <c r="AM160" s="7"/>
       <c r="AN160" s="7"/>
       <c r="AO160" s="7"/>
+      <c r="AP160" s="7"/>
     </row>
     <row r="161">
       <c r="A161" s="7" t="inlineStr">
@@ -12306,6 +12470,7 @@
       <c r="AM161" s="7"/>
       <c r="AN161" s="7"/>
       <c r="AO161" s="7"/>
+      <c r="AP161" s="7"/>
     </row>
     <row r="162">
       <c r="A162" s="7" t="inlineStr">
@@ -12377,6 +12542,7 @@
       <c r="AM162" s="7"/>
       <c r="AN162" s="7"/>
       <c r="AO162" s="7"/>
+      <c r="AP162" s="7"/>
     </row>
     <row r="163">
       <c r="A163" s="7" t="inlineStr">
@@ -12448,6 +12614,7 @@
       <c r="AM163" s="7"/>
       <c r="AN163" s="7"/>
       <c r="AO163" s="7"/>
+      <c r="AP163" s="7"/>
     </row>
     <row r="164">
       <c r="A164" s="7" t="inlineStr">
@@ -12519,6 +12686,7 @@
       <c r="AM164" s="7"/>
       <c r="AN164" s="7"/>
       <c r="AO164" s="7"/>
+      <c r="AP164" s="7"/>
     </row>
     <row r="165">
       <c r="A165" s="7" t="inlineStr">
@@ -12590,6 +12758,7 @@
       <c r="AM165" s="7"/>
       <c r="AN165" s="7"/>
       <c r="AO165" s="7"/>
+      <c r="AP165" s="7"/>
     </row>
     <row r="166">
       <c r="A166" s="7" t="inlineStr">
@@ -12669,6 +12838,7 @@
       </c>
       <c r="AN166" s="7"/>
       <c r="AO166" s="7"/>
+      <c r="AP166" s="7"/>
     </row>
     <row r="167">
       <c r="A167" s="7" t="inlineStr">
@@ -12744,6 +12914,7 @@
       </c>
       <c r="AN167" s="7"/>
       <c r="AO167" s="7"/>
+      <c r="AP167" s="7"/>
     </row>
     <row r="168">
       <c r="A168" s="7" t="inlineStr">
@@ -12815,6 +12986,7 @@
       <c r="AM168" s="7"/>
       <c r="AN168" s="7"/>
       <c r="AO168" s="7"/>
+      <c r="AP168" s="7"/>
     </row>
     <row r="169">
       <c r="A169" s="7" t="inlineStr">
@@ -12886,6 +13058,7 @@
       <c r="AM169" s="7"/>
       <c r="AN169" s="7"/>
       <c r="AO169" s="7"/>
+      <c r="AP169" s="7"/>
     </row>
     <row r="170">
       <c r="A170" s="7" t="inlineStr">
@@ -12961,6 +13134,7 @@
       <c r="AM170" s="7"/>
       <c r="AN170" s="7"/>
       <c r="AO170" s="7"/>
+      <c r="AP170" s="7"/>
     </row>
     <row r="171">
       <c r="A171" s="7" t="inlineStr">
@@ -13028,6 +13202,7 @@
       <c r="AM171" s="7"/>
       <c r="AN171" s="7"/>
       <c r="AO171" s="7"/>
+      <c r="AP171" s="7"/>
     </row>
     <row r="172">
       <c r="A172" s="7" t="inlineStr">
@@ -13095,6 +13270,7 @@
       <c r="AM172" s="7"/>
       <c r="AN172" s="7"/>
       <c r="AO172" s="7"/>
+      <c r="AP172" s="7"/>
     </row>
     <row r="173">
       <c r="A173" s="7" t="inlineStr">
@@ -13170,6 +13346,7 @@
       <c r="AM173" s="7"/>
       <c r="AN173" s="7"/>
       <c r="AO173" s="7"/>
+      <c r="AP173" s="7"/>
     </row>
     <row r="174">
       <c r="A174" s="7" t="inlineStr">
@@ -13241,6 +13418,7 @@
       <c r="AM174" s="7"/>
       <c r="AN174" s="7"/>
       <c r="AO174" s="7"/>
+      <c r="AP174" s="7"/>
     </row>
     <row r="175">
       <c r="A175" s="7" t="inlineStr">
@@ -13316,6 +13494,7 @@
       <c r="AM175" s="7"/>
       <c r="AN175" s="7"/>
       <c r="AO175" s="7"/>
+      <c r="AP175" s="7"/>
     </row>
     <row r="176">
       <c r="A176" s="7" t="inlineStr">
@@ -13387,6 +13566,7 @@
       <c r="AM176" s="7"/>
       <c r="AN176" s="7"/>
       <c r="AO176" s="7"/>
+      <c r="AP176" s="7"/>
     </row>
     <row r="177">
       <c r="A177" s="7" t="inlineStr">
@@ -13458,6 +13638,7 @@
       <c r="AM177" s="7"/>
       <c r="AN177" s="7"/>
       <c r="AO177" s="7"/>
+      <c r="AP177" s="7"/>
     </row>
     <row r="178">
       <c r="A178" s="7" t="inlineStr">
@@ -13529,6 +13710,7 @@
       <c r="AM178" s="7"/>
       <c r="AN178" s="7"/>
       <c r="AO178" s="7"/>
+      <c r="AP178" s="7"/>
     </row>
     <row r="179">
       <c r="A179" s="7" t="inlineStr">
@@ -13600,6 +13782,7 @@
       <c r="AM179" s="7"/>
       <c r="AN179" s="7"/>
       <c r="AO179" s="7"/>
+      <c r="AP179" s="7"/>
     </row>
     <row r="180">
       <c r="A180" s="7" t="inlineStr">
@@ -13671,6 +13854,7 @@
       <c r="AM180" s="7"/>
       <c r="AN180" s="7"/>
       <c r="AO180" s="7"/>
+      <c r="AP180" s="7"/>
     </row>
     <row r="181">
       <c r="A181" s="7" t="inlineStr">
@@ -13742,6 +13926,7 @@
       <c r="AM181" s="7"/>
       <c r="AN181" s="7"/>
       <c r="AO181" s="7"/>
+      <c r="AP181" s="7"/>
     </row>
     <row r="182">
       <c r="A182" s="7" t="inlineStr">
@@ -13813,6 +13998,7 @@
       <c r="AM182" s="7"/>
       <c r="AN182" s="7"/>
       <c r="AO182" s="7"/>
+      <c r="AP182" s="7"/>
     </row>
     <row r="183">
       <c r="A183" s="7" t="inlineStr">
@@ -13884,6 +14070,7 @@
       <c r="AM183" s="7"/>
       <c r="AN183" s="7"/>
       <c r="AO183" s="7"/>
+      <c r="AP183" s="7"/>
     </row>
     <row r="184">
       <c r="A184" s="7" t="inlineStr">
@@ -13951,6 +14138,7 @@
       <c r="AM184" s="7"/>
       <c r="AN184" s="7"/>
       <c r="AO184" s="7"/>
+      <c r="AP184" s="7"/>
     </row>
     <row r="185">
       <c r="A185" s="7" t="inlineStr">
@@ -14022,6 +14210,7 @@
       <c r="AM185" s="7"/>
       <c r="AN185" s="7"/>
       <c r="AO185" s="7"/>
+      <c r="AP185" s="7"/>
     </row>
     <row r="186">
       <c r="A186" s="7" t="inlineStr">
@@ -14093,6 +14282,7 @@
       <c r="AM186" s="7"/>
       <c r="AN186" s="7"/>
       <c r="AO186" s="7"/>
+      <c r="AP186" s="7"/>
     </row>
     <row r="187">
       <c r="A187" s="7" t="inlineStr">
@@ -14168,6 +14358,7 @@
       </c>
       <c r="AN187" s="7"/>
       <c r="AO187" s="7"/>
+      <c r="AP187" s="7"/>
     </row>
     <row r="188">
       <c r="A188" s="7" t="inlineStr">
@@ -14243,6 +14434,7 @@
       </c>
       <c r="AN188" s="7"/>
       <c r="AO188" s="7"/>
+      <c r="AP188" s="7"/>
     </row>
     <row r="189">
       <c r="A189" s="7" t="inlineStr">
@@ -14318,6 +14510,7 @@
       </c>
       <c r="AN189" s="7"/>
       <c r="AO189" s="7"/>
+      <c r="AP189" s="7"/>
     </row>
     <row r="190">
       <c r="A190" s="7" t="inlineStr">
@@ -14393,6 +14586,7 @@
       </c>
       <c r="AN190" s="7"/>
       <c r="AO190" s="7"/>
+      <c r="AP190" s="7"/>
     </row>
     <row r="191">
       <c r="A191" s="7" t="inlineStr">
@@ -14468,6 +14662,7 @@
       <c r="AM191" s="7"/>
       <c r="AN191" s="7"/>
       <c r="AO191" s="7"/>
+      <c r="AP191" s="7"/>
     </row>
     <row r="192">
       <c r="A192" s="7" t="inlineStr">
@@ -14543,6 +14738,7 @@
       </c>
       <c r="AN192" s="7"/>
       <c r="AO192" s="7"/>
+      <c r="AP192" s="7"/>
     </row>
     <row r="193">
       <c r="A193" s="7" t="inlineStr">
@@ -14618,6 +14814,7 @@
       </c>
       <c r="AN193" s="7"/>
       <c r="AO193" s="7"/>
+      <c r="AP193" s="7"/>
     </row>
     <row r="194">
       <c r="A194" s="7" t="inlineStr">
@@ -14693,6 +14890,7 @@
       </c>
       <c r="AN194" s="7"/>
       <c r="AO194" s="7"/>
+      <c r="AP194" s="7"/>
     </row>
     <row r="195">
       <c r="A195" s="7" t="inlineStr">
@@ -14768,6 +14966,7 @@
       </c>
       <c r="AN195" s="7"/>
       <c r="AO195" s="7"/>
+      <c r="AP195" s="7"/>
     </row>
     <row r="196">
       <c r="A196" s="7" t="inlineStr">
@@ -14839,6 +15038,7 @@
       </c>
       <c r="AN196" s="7"/>
       <c r="AO196" s="7"/>
+      <c r="AP196" s="7"/>
     </row>
     <row r="197">
       <c r="A197" s="7" t="inlineStr">
@@ -14914,6 +15114,7 @@
       </c>
       <c r="AN197" s="7"/>
       <c r="AO197" s="7"/>
+      <c r="AP197" s="7"/>
     </row>
     <row r="198">
       <c r="A198" s="7" t="inlineStr">
@@ -14985,6 +15186,7 @@
       </c>
       <c r="AN198" s="7"/>
       <c r="AO198" s="7"/>
+      <c r="AP198" s="7"/>
     </row>
     <row r="199">
       <c r="A199" s="7" t="inlineStr">
@@ -15060,6 +15262,7 @@
       </c>
       <c r="AN199" s="7"/>
       <c r="AO199" s="7"/>
+      <c r="AP199" s="7"/>
     </row>
     <row r="200">
       <c r="A200" s="7" t="inlineStr">
@@ -15135,6 +15338,7 @@
       </c>
       <c r="AN200" s="7"/>
       <c r="AO200" s="7"/>
+      <c r="AP200" s="7"/>
     </row>
     <row r="201">
       <c r="A201" s="7" t="inlineStr">
@@ -15202,6 +15406,7 @@
       <c r="AM201" s="7"/>
       <c r="AN201" s="7"/>
       <c r="AO201" s="7"/>
+      <c r="AP201" s="7"/>
     </row>
     <row r="202">
       <c r="A202" s="7" t="inlineStr">
@@ -15277,6 +15482,7 @@
       </c>
       <c r="AN202" s="7"/>
       <c r="AO202" s="7"/>
+      <c r="AP202" s="7"/>
     </row>
     <row r="203">
       <c r="A203" s="7" t="inlineStr">
@@ -15352,6 +15558,7 @@
       </c>
       <c r="AN203" s="7"/>
       <c r="AO203" s="7"/>
+      <c r="AP203" s="7"/>
     </row>
     <row r="204">
       <c r="A204" s="7" t="inlineStr">
@@ -15427,6 +15634,7 @@
         </is>
       </c>
       <c r="AO204" s="7"/>
+      <c r="AP204" s="7"/>
     </row>
     <row r="205">
       <c r="A205" s="7" t="inlineStr">
@@ -15506,6 +15714,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AP205" s="7"/>
     </row>
     <row r="206">
       <c r="A206" s="7" t="inlineStr">
@@ -15581,6 +15790,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AP206" s="7"/>
     </row>
     <row r="207">
       <c r="A207" s="7" t="inlineStr">
@@ -15652,6 +15862,7 @@
       </c>
       <c r="AN207" s="7"/>
       <c r="AO207" s="7"/>
+      <c r="AP207" s="7"/>
     </row>
     <row r="208">
       <c r="A208" s="7" t="inlineStr">
@@ -15723,6 +15934,7 @@
       </c>
       <c r="AN208" s="7"/>
       <c r="AO208" s="7"/>
+      <c r="AP208" s="7"/>
     </row>
     <row r="209">
       <c r="A209" s="7" t="inlineStr">
@@ -15798,6 +16010,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AP209" s="7"/>
     </row>
     <row r="210">
       <c r="A210" s="7" t="inlineStr">
@@ -15869,6 +16082,79 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AP210" s="7"/>
+    </row>
+    <row r="211">
+      <c r="A211" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_203</t>
+        </is>
+      </c>
+      <c r="B211" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">파밍</t>
+        </is>
+      </c>
+      <c r="C211" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 · S4 난이도</t>
+        </is>
+      </c>
+      <c r="D211" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#204 값</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 파밍(장갑 hp 300) · S4 파밍(정원 10 = 보병 8 · 포격 1 · 장갑 1)을 강화한 시작 보드로 60초 넘게 버티는가?</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#204 · S4 비율 ⚠️ 플랜 어림 · 하네스 생존(593 · 723)</t>
+        </is>
+      </c>
+      <c r="G211" s="7"/>
+      <c r="H211" s="7"/>
+      <c r="I211" s="7"/>
+      <c r="J211" s="7"/>
+      <c r="K211" s="7"/>
+      <c r="L211" s="7"/>
+      <c r="M211" s="7"/>
+      <c r="N211" s="7"/>
+      <c r="O211" s="7"/>
+      <c r="P211" s="7"/>
+      <c r="Q211" s="7"/>
+      <c r="R211" s="7"/>
+      <c r="S211" s="7"/>
+      <c r="T211" s="7"/>
+      <c r="U211" s="7"/>
+      <c r="V211" s="7"/>
+      <c r="W211" s="7"/>
+      <c r="X211" s="7"/>
+      <c r="Y211" s="7"/>
+      <c r="Z211" s="7"/>
+      <c r="AA211" s="7"/>
+      <c r="AB211" s="7"/>
+      <c r="AC211" s="7"/>
+      <c r="AD211" s="7"/>
+      <c r="AE211" s="7"/>
+      <c r="AF211" s="7"/>
+      <c r="AG211" s="7"/>
+      <c r="AH211" s="7"/>
+      <c r="AI211" s="7"/>
+      <c r="AJ211" s="7"/>
+      <c r="AK211" s="7"/>
+      <c r="AL211" s="7"/>
+      <c r="AM211" s="7"/>
+      <c r="AN211" s="7"/>
+      <c r="AO211" s="7"/>
+      <c r="AP211" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="26">
@@ -15897,9 +16183,9 @@
     <mergeCell ref="B92:B99"/>
     <mergeCell ref="B100:B106"/>
     <mergeCell ref="B107:B111"/>
-    <mergeCell ref="G7:AO7"/>
+    <mergeCell ref="G7:AP7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:AO210">
+  <conditionalFormatting sqref="G9:AP211">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
QA AQ: 8133 109e859 전체 플레이 한 바퀴 (Pass 15 · Fail 4 · CID_204~207)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -198,8 +198,9 @@
     <col min="40" max="40" width="12" customWidth="1"/>
     <col min="41" max="41" width="12" customWidth="1"/>
     <col min="42" max="42" width="12" customWidth="1"/>
-    <col min="43" max="43" width="11" customWidth="1"/>
+    <col min="43" max="43" width="12" customWidth="1"/>
     <col min="44" max="44" width="11" customWidth="1"/>
+    <col min="45" max="45" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -492,6 +493,11 @@
       <c r="AP6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">8133 갈아엎음(22:03:24) · #204 S3 파밍 장갑 hp 600→300 · S4 파밍 정원 18→10(8·1·1) ‖ 하네스: 전투 12줄 불변 · 파밍 A 단독 S3 생존 HP 바닥 593 · S4 생존 723 · 두 로봇(S5 · S6) 생존(표 Docs/261019_farm_tag.md) / 화면(8133 사용자 저장): 바로가기 S4 파밍 「맵 7/10」 ✅ · S3 화면 생존 = 미확인(육안 자리)</t>
+        </is>
+      </c>
+      <c r="AQ6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8133 109e859 전체 플레이 한 바퀴(코드 세션 · 인앱 브라우저 · 소리 0) — 자연 진행 S1→S5(파괴 → S4) → 바로가기 S6 · 새로고침 · 처음부터 → 바로가기 S3 · S5. 빈 칸 = 못 봄(까닭은 F). 새 결함 = CID_204~207.</t>
         </is>
       </c>
     </row>
@@ -558,12 +564,13 @@
       <c r="AN7" s="2"/>
       <c r="AO7" s="2"/>
       <c r="AP7" s="2"/>
-      <c r="AQ7" s="2" t="inlineStr">
+      <c r="AQ7" s="2"/>
+      <c r="AR7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">버전</t>
         </is>
       </c>
-      <c r="AR7" s="7" t="inlineStr">
+      <c r="AS7" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">109e859</t>
         </is>
@@ -770,11 +777,16 @@
       </c>
       <c r="AQ8" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">109e859</t>
+        </is>
+      </c>
+      <c r="AR8" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">PASSrate</t>
         </is>
       </c>
-      <c r="AR8" s="7">
-        <f>COUNTIF(AP9:AP211,"Pass")</f>
+      <c r="AS8" s="7">
+        <f>COUNTIF(AQ9:AQ215,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -880,13 +892,14 @@
       <c r="AN9" s="7"/>
       <c r="AO9" s="7"/>
       <c r="AP9" s="7"/>
-      <c r="AQ9" s="2" t="inlineStr">
+      <c r="AQ9" s="7"/>
+      <c r="AR9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FAILrate</t>
         </is>
       </c>
-      <c r="AR9" s="7">
-        <f>COUNTIF(AP9:AP211,"Fail")+COUNTIF(AP9:AP211,"Broken")</f>
+      <c r="AS9" s="7">
+        <f>COUNTIF(AQ9:AQ215,"Fail")+COUNTIF(AQ9:AQ215,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -956,13 +969,14 @@
       <c r="AN10" s="7"/>
       <c r="AO10" s="7"/>
       <c r="AP10" s="7"/>
-      <c r="AQ10" s="2" t="inlineStr">
+      <c r="AQ10" s="7"/>
+      <c r="AR10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">N/A</t>
         </is>
       </c>
-      <c r="AR10" s="7">
-        <f>COUNTIF(AP9:AP211,"N/A")</f>
+      <c r="AS10" s="7">
+        <f>COUNTIF(AQ9:AQ215,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -1032,13 +1046,14 @@
       <c r="AN11" s="7"/>
       <c r="AO11" s="7"/>
       <c r="AP11" s="7"/>
-      <c r="AQ11" s="2" t="inlineStr">
+      <c r="AQ11" s="7"/>
+      <c r="AR11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">전체 개수</t>
         </is>
       </c>
-      <c r="AR11" s="7">
-        <v>203</v>
+      <c r="AS11" s="7">
+        <v>207</v>
       </c>
     </row>
     <row r="12">
@@ -1108,13 +1123,14 @@
       <c r="AN12" s="7"/>
       <c r="AO12" s="7"/>
       <c r="AP12" s="7"/>
-      <c r="AQ12" s="2" t="inlineStr">
+      <c r="AQ12" s="7"/>
+      <c r="AR12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">진행율</t>
         </is>
       </c>
-      <c r="AR12" s="7">
-        <f>TEXT((COUNTA(AP9:AP211))/203,"0.00%")</f>
+      <c r="AS12" s="7">
+        <f>TEXT((COUNTA(AQ9:AQ215))/207,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -1188,6 +1204,7 @@
       <c r="AN13" s="7"/>
       <c r="AO13" s="7"/>
       <c r="AP13" s="7"/>
+      <c r="AQ13" s="7"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -1251,6 +1268,7 @@
       <c r="AN14" s="7"/>
       <c r="AO14" s="7"/>
       <c r="AP14" s="7"/>
+      <c r="AQ14" s="7"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -1350,6 +1368,7 @@
       <c r="AN15" s="7"/>
       <c r="AO15" s="7"/>
       <c r="AP15" s="7"/>
+      <c r="AQ15" s="7"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -1449,6 +1468,7 @@
       <c r="AN16" s="7"/>
       <c r="AO16" s="7"/>
       <c r="AP16" s="7"/>
+      <c r="AQ16" s="7"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -1553,6 +1573,7 @@
       <c r="AN17" s="7"/>
       <c r="AO17" s="7"/>
       <c r="AP17" s="7"/>
+      <c r="AQ17" s="7"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -1621,6 +1642,7 @@
       <c r="AN18" s="7"/>
       <c r="AO18" s="7"/>
       <c r="AP18" s="7"/>
+      <c r="AQ18" s="7"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -1684,6 +1706,7 @@
       <c r="AN19" s="7"/>
       <c r="AO19" s="7"/>
       <c r="AP19" s="7"/>
+      <c r="AQ19" s="7"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1747,6 +1770,7 @@
       <c r="AN20" s="7"/>
       <c r="AO20" s="7"/>
       <c r="AP20" s="7"/>
+      <c r="AQ20" s="7"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1846,6 +1870,7 @@
       <c r="AN21" s="7"/>
       <c r="AO21" s="7"/>
       <c r="AP21" s="7"/>
+      <c r="AQ21" s="7"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1938,6 +1963,7 @@
       <c r="AN22" s="7"/>
       <c r="AO22" s="7"/>
       <c r="AP22" s="7"/>
+      <c r="AQ22" s="7"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -2009,6 +2035,7 @@
       <c r="AN23" s="7"/>
       <c r="AO23" s="7"/>
       <c r="AP23" s="7"/>
+      <c r="AQ23" s="7"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -2072,6 +2099,7 @@
       <c r="AN24" s="7"/>
       <c r="AO24" s="7"/>
       <c r="AP24" s="7"/>
+      <c r="AQ24" s="7"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -2135,6 +2163,7 @@
       <c r="AN25" s="7"/>
       <c r="AO25" s="7"/>
       <c r="AP25" s="7"/>
+      <c r="AQ25" s="7"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -2227,6 +2256,7 @@
       <c r="AN26" s="7"/>
       <c r="AO26" s="7"/>
       <c r="AP26" s="7"/>
+      <c r="AQ26" s="7"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -2294,6 +2324,7 @@
       <c r="AN27" s="7"/>
       <c r="AO27" s="7"/>
       <c r="AP27" s="7"/>
+      <c r="AQ27" s="7"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -2370,6 +2401,7 @@
       <c r="AN28" s="7"/>
       <c r="AO28" s="7"/>
       <c r="AP28" s="7"/>
+      <c r="AQ28" s="7"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -2441,6 +2473,7 @@
       <c r="AN29" s="7"/>
       <c r="AO29" s="7"/>
       <c r="AP29" s="7"/>
+      <c r="AQ29" s="7"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -2536,6 +2569,7 @@
       <c r="AN30" s="7"/>
       <c r="AO30" s="7"/>
       <c r="AP30" s="7"/>
+      <c r="AQ30" s="7"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -2636,6 +2670,7 @@
       <c r="AN31" s="7"/>
       <c r="AO31" s="7"/>
       <c r="AP31" s="7"/>
+      <c r="AQ31" s="7"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -2723,6 +2758,7 @@
       <c r="AN32" s="7"/>
       <c r="AO32" s="7"/>
       <c r="AP32" s="7"/>
+      <c r="AQ32" s="7"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -2818,6 +2854,7 @@
       <c r="AN33" s="7"/>
       <c r="AO33" s="7"/>
       <c r="AP33" s="7"/>
+      <c r="AQ33" s="7"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -2913,6 +2950,7 @@
       <c r="AN34" s="7"/>
       <c r="AO34" s="7"/>
       <c r="AP34" s="7"/>
+      <c r="AQ34" s="7"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -3017,6 +3055,7 @@
       <c r="AN35" s="7"/>
       <c r="AO35" s="7"/>
       <c r="AP35" s="7"/>
+      <c r="AQ35" s="7"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -3096,6 +3135,7 @@
       <c r="AN36" s="7"/>
       <c r="AO36" s="7"/>
       <c r="AP36" s="7"/>
+      <c r="AQ36" s="7"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -3159,6 +3199,7 @@
       <c r="AN37" s="7"/>
       <c r="AO37" s="7"/>
       <c r="AP37" s="7"/>
+      <c r="AQ37" s="7"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -3243,6 +3284,7 @@
       <c r="AN38" s="7"/>
       <c r="AO38" s="7"/>
       <c r="AP38" s="7"/>
+      <c r="AQ38" s="7"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -3338,6 +3380,7 @@
       <c r="AN39" s="7"/>
       <c r="AO39" s="7"/>
       <c r="AP39" s="7"/>
+      <c r="AQ39" s="7"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -3434,6 +3477,7 @@
       <c r="AN40" s="7"/>
       <c r="AO40" s="7"/>
       <c r="AP40" s="7"/>
+      <c r="AQ40" s="7"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -3525,6 +3569,7 @@
       <c r="AN41" s="7"/>
       <c r="AO41" s="7"/>
       <c r="AP41" s="7"/>
+      <c r="AQ41" s="7"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -3600,6 +3645,7 @@
       <c r="AN42" s="7"/>
       <c r="AO42" s="7"/>
       <c r="AP42" s="7"/>
+      <c r="AQ42" s="7"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -3695,6 +3741,7 @@
       <c r="AN43" s="7"/>
       <c r="AO43" s="7"/>
       <c r="AP43" s="7"/>
+      <c r="AQ43" s="7"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -3763,6 +3810,7 @@
       <c r="AN44" s="7"/>
       <c r="AO44" s="7"/>
       <c r="AP44" s="7"/>
+      <c r="AQ44" s="7"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -3854,6 +3902,7 @@
       <c r="AN45" s="7"/>
       <c r="AO45" s="7"/>
       <c r="AP45" s="7"/>
+      <c r="AQ45" s="7"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -3945,6 +3994,7 @@
       <c r="AN46" s="7"/>
       <c r="AO46" s="7"/>
       <c r="AP46" s="7"/>
+      <c r="AQ46" s="7"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -4013,6 +4063,7 @@
       <c r="AN47" s="7"/>
       <c r="AO47" s="7"/>
       <c r="AP47" s="7"/>
+      <c r="AQ47" s="7"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -4076,6 +4127,7 @@
       <c r="AN48" s="7"/>
       <c r="AO48" s="7"/>
       <c r="AP48" s="7"/>
+      <c r="AQ48" s="7"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -4139,6 +4191,7 @@
       <c r="AN49" s="7"/>
       <c r="AO49" s="7"/>
       <c r="AP49" s="7"/>
+      <c r="AQ49" s="7"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -4226,6 +4279,7 @@
       <c r="AN50" s="7"/>
       <c r="AO50" s="7"/>
       <c r="AP50" s="7"/>
+      <c r="AQ50" s="7"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -4313,6 +4367,7 @@
       <c r="AN51" s="7"/>
       <c r="AO51" s="7"/>
       <c r="AP51" s="7"/>
+      <c r="AQ51" s="7"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -4381,6 +4436,7 @@
       <c r="AN52" s="7"/>
       <c r="AO52" s="7"/>
       <c r="AP52" s="7"/>
+      <c r="AQ52" s="7"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -4449,6 +4505,7 @@
       <c r="AN53" s="7"/>
       <c r="AO53" s="7"/>
       <c r="AP53" s="7"/>
+      <c r="AQ53" s="7"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -4512,6 +4569,7 @@
       <c r="AN54" s="7"/>
       <c r="AO54" s="7"/>
       <c r="AP54" s="7"/>
+      <c r="AQ54" s="7"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -4611,6 +4669,7 @@
       <c r="AN55" s="7"/>
       <c r="AO55" s="7"/>
       <c r="AP55" s="7"/>
+      <c r="AQ55" s="7"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -4690,6 +4749,7 @@
       <c r="AN56" s="7"/>
       <c r="AO56" s="7"/>
       <c r="AP56" s="7"/>
+      <c r="AQ56" s="7"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -4778,6 +4838,7 @@
       <c r="AN57" s="7"/>
       <c r="AO57" s="7"/>
       <c r="AP57" s="7"/>
+      <c r="AQ57" s="7"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -4874,6 +4935,7 @@
       <c r="AN58" s="7"/>
       <c r="AO58" s="7"/>
       <c r="AP58" s="7"/>
+      <c r="AQ58" s="7"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -4937,6 +4999,7 @@
       <c r="AN59" s="7"/>
       <c r="AO59" s="7"/>
       <c r="AP59" s="7"/>
+      <c r="AQ59" s="7"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -5000,6 +5063,7 @@
       <c r="AN60" s="7"/>
       <c r="AO60" s="7"/>
       <c r="AP60" s="7"/>
+      <c r="AQ60" s="7"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -5075,6 +5139,7 @@
       <c r="AN61" s="7"/>
       <c r="AO61" s="7"/>
       <c r="AP61" s="7"/>
+      <c r="AQ61" s="7"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -5158,6 +5223,7 @@
       <c r="AN62" s="7"/>
       <c r="AO62" s="7"/>
       <c r="AP62" s="7"/>
+      <c r="AQ62" s="7"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -5233,6 +5299,7 @@
       <c r="AN63" s="7"/>
       <c r="AO63" s="7"/>
       <c r="AP63" s="7"/>
+      <c r="AQ63" s="7"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -5296,6 +5363,7 @@
       <c r="AN64" s="7"/>
       <c r="AO64" s="7"/>
       <c r="AP64" s="7"/>
+      <c r="AQ64" s="7"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -5364,6 +5432,7 @@
       <c r="AN65" s="7"/>
       <c r="AO65" s="7"/>
       <c r="AP65" s="7"/>
+      <c r="AQ65" s="7"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
@@ -5439,6 +5508,7 @@
       <c r="AN66" s="7"/>
       <c r="AO66" s="7"/>
       <c r="AP66" s="7"/>
+      <c r="AQ66" s="7"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -5502,6 +5572,7 @@
       <c r="AN67" s="7"/>
       <c r="AO67" s="7"/>
       <c r="AP67" s="7"/>
+      <c r="AQ67" s="7"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
@@ -5569,6 +5640,7 @@
       <c r="AN68" s="7"/>
       <c r="AO68" s="7"/>
       <c r="AP68" s="7"/>
+      <c r="AQ68" s="7"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -5668,6 +5740,7 @@
       <c r="AN69" s="7"/>
       <c r="AO69" s="7"/>
       <c r="AP69" s="7"/>
+      <c r="AQ69" s="7"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
@@ -5731,6 +5804,7 @@
       <c r="AN70" s="7"/>
       <c r="AO70" s="7"/>
       <c r="AP70" s="7"/>
+      <c r="AQ70" s="7"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -5799,6 +5873,7 @@
       <c r="AN71" s="7"/>
       <c r="AO71" s="7"/>
       <c r="AP71" s="7"/>
+      <c r="AQ71" s="7"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
@@ -5878,6 +5953,7 @@
       <c r="AN72" s="7"/>
       <c r="AO72" s="7"/>
       <c r="AP72" s="7"/>
+      <c r="AQ72" s="7"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
@@ -5946,6 +6022,7 @@
       <c r="AN73" s="7"/>
       <c r="AO73" s="7"/>
       <c r="AP73" s="7"/>
+      <c r="AQ73" s="7"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -6009,6 +6086,7 @@
       <c r="AN74" s="7"/>
       <c r="AO74" s="7"/>
       <c r="AP74" s="7"/>
+      <c r="AQ74" s="7"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -6072,6 +6150,7 @@
       <c r="AN75" s="7"/>
       <c r="AO75" s="7"/>
       <c r="AP75" s="7"/>
+      <c r="AQ75" s="7"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -6135,6 +6214,7 @@
       <c r="AN76" s="7"/>
       <c r="AO76" s="7"/>
       <c r="AP76" s="7"/>
+      <c r="AQ76" s="7"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -6202,6 +6282,7 @@
       <c r="AN77" s="7"/>
       <c r="AO77" s="7"/>
       <c r="AP77" s="7"/>
+      <c r="AQ77" s="7"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
@@ -6265,6 +6346,7 @@
       <c r="AN78" s="7"/>
       <c r="AO78" s="7"/>
       <c r="AP78" s="7"/>
+      <c r="AQ78" s="7"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -6333,6 +6415,7 @@
       <c r="AN79" s="7"/>
       <c r="AO79" s="7"/>
       <c r="AP79" s="7"/>
+      <c r="AQ79" s="7"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
@@ -6412,6 +6495,7 @@
       <c r="AN80" s="7"/>
       <c r="AO80" s="7"/>
       <c r="AP80" s="7"/>
+      <c r="AQ80" s="7"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
@@ -6479,6 +6563,7 @@
       <c r="AN81" s="7"/>
       <c r="AO81" s="7"/>
       <c r="AP81" s="7"/>
+      <c r="AQ81" s="7"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
@@ -6542,6 +6627,7 @@
       <c r="AN82" s="7"/>
       <c r="AO82" s="7"/>
       <c r="AP82" s="7"/>
+      <c r="AQ82" s="7"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
@@ -6610,6 +6696,7 @@
       <c r="AN83" s="7"/>
       <c r="AO83" s="7"/>
       <c r="AP83" s="7"/>
+      <c r="AQ83" s="7"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
@@ -6673,6 +6760,7 @@
       <c r="AN84" s="7"/>
       <c r="AO84" s="7"/>
       <c r="AP84" s="7"/>
+      <c r="AQ84" s="7"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
@@ -6736,6 +6824,7 @@
       <c r="AN85" s="7"/>
       <c r="AO85" s="7"/>
       <c r="AP85" s="7"/>
+      <c r="AQ85" s="7"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
@@ -6804,6 +6893,7 @@
       <c r="AN86" s="7"/>
       <c r="AO86" s="7"/>
       <c r="AP86" s="7"/>
+      <c r="AQ86" s="7"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
@@ -6867,6 +6957,7 @@
       <c r="AN87" s="7"/>
       <c r="AO87" s="7"/>
       <c r="AP87" s="7"/>
+      <c r="AQ87" s="7"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
@@ -6930,6 +7021,7 @@
       <c r="AN88" s="7"/>
       <c r="AO88" s="7"/>
       <c r="AP88" s="7"/>
+      <c r="AQ88" s="7"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
@@ -6993,6 +7085,7 @@
       <c r="AN89" s="7"/>
       <c r="AO89" s="7"/>
       <c r="AP89" s="7"/>
+      <c r="AQ89" s="7"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
@@ -7085,6 +7178,7 @@
       <c r="AN90" s="7"/>
       <c r="AO90" s="7"/>
       <c r="AP90" s="7"/>
+      <c r="AQ90" s="7"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
@@ -7148,6 +7242,7 @@
       <c r="AN91" s="7"/>
       <c r="AO91" s="7"/>
       <c r="AP91" s="7"/>
+      <c r="AQ91" s="7"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
@@ -7247,6 +7342,7 @@
       <c r="AN92" s="7"/>
       <c r="AO92" s="7"/>
       <c r="AP92" s="7"/>
+      <c r="AQ92" s="7"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
@@ -7351,6 +7447,7 @@
       <c r="AN93" s="7"/>
       <c r="AO93" s="7"/>
       <c r="AP93" s="7"/>
+      <c r="AQ93" s="7"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
@@ -7419,6 +7516,7 @@
       <c r="AN94" s="7"/>
       <c r="AO94" s="7"/>
       <c r="AP94" s="7"/>
+      <c r="AQ94" s="7"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
@@ -7487,6 +7585,7 @@
       <c r="AN95" s="7"/>
       <c r="AO95" s="7"/>
       <c r="AP95" s="7"/>
+      <c r="AQ95" s="7"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
@@ -7574,6 +7673,7 @@
       <c r="AN96" s="7"/>
       <c r="AO96" s="7"/>
       <c r="AP96" s="7"/>
+      <c r="AQ96" s="7"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="inlineStr">
@@ -7637,6 +7737,7 @@
       <c r="AN97" s="7"/>
       <c r="AO97" s="7"/>
       <c r="AP97" s="7"/>
+      <c r="AQ97" s="7"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
@@ -7700,6 +7801,7 @@
       <c r="AN98" s="7"/>
       <c r="AO98" s="7"/>
       <c r="AP98" s="7"/>
+      <c r="AQ98" s="7"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
@@ -7763,6 +7865,7 @@
       <c r="AN99" s="7"/>
       <c r="AO99" s="7"/>
       <c r="AP99" s="7"/>
+      <c r="AQ99" s="7"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
@@ -7835,6 +7938,7 @@
       <c r="AN100" s="7"/>
       <c r="AO100" s="7"/>
       <c r="AP100" s="7"/>
+      <c r="AQ100" s="7"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
@@ -7898,6 +8002,7 @@
       <c r="AN101" s="7"/>
       <c r="AO101" s="7"/>
       <c r="AP101" s="7"/>
+      <c r="AQ101" s="7"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
@@ -7961,6 +8066,7 @@
       <c r="AN102" s="7"/>
       <c r="AO102" s="7"/>
       <c r="AP102" s="7"/>
+      <c r="AQ102" s="7"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="inlineStr">
@@ -8024,6 +8130,7 @@
       <c r="AN103" s="7"/>
       <c r="AO103" s="7"/>
       <c r="AP103" s="7"/>
+      <c r="AQ103" s="7"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="inlineStr">
@@ -8092,6 +8199,7 @@
       <c r="AN104" s="7"/>
       <c r="AO104" s="7"/>
       <c r="AP104" s="7"/>
+      <c r="AQ104" s="7"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
@@ -8155,6 +8263,7 @@
       <c r="AN105" s="7"/>
       <c r="AO105" s="7"/>
       <c r="AP105" s="7"/>
+      <c r="AQ105" s="7"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
@@ -8218,6 +8327,7 @@
       <c r="AN106" s="7"/>
       <c r="AO106" s="7"/>
       <c r="AP106" s="7"/>
+      <c r="AQ106" s="7"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
@@ -8281,6 +8391,7 @@
       <c r="AN107" s="7"/>
       <c r="AO107" s="7"/>
       <c r="AP107" s="7"/>
+      <c r="AQ107" s="7"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
@@ -8348,6 +8459,7 @@
       <c r="AN108" s="7"/>
       <c r="AO108" s="7"/>
       <c r="AP108" s="7"/>
+      <c r="AQ108" s="7"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="inlineStr">
@@ -8420,6 +8532,7 @@
       <c r="AN109" s="7"/>
       <c r="AO109" s="7"/>
       <c r="AP109" s="7"/>
+      <c r="AQ109" s="7"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
@@ -8500,6 +8613,7 @@
       <c r="AN110" s="7"/>
       <c r="AO110" s="7"/>
       <c r="AP110" s="7"/>
+      <c r="AQ110" s="7"/>
     </row>
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
@@ -8583,6 +8697,7 @@
       <c r="AN111" s="7"/>
       <c r="AO111" s="7"/>
       <c r="AP111" s="7"/>
+      <c r="AQ111" s="7"/>
     </row>
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
@@ -8663,6 +8778,7 @@
       <c r="AN112" s="7"/>
       <c r="AO112" s="7"/>
       <c r="AP112" s="7"/>
+      <c r="AQ112" s="7"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
@@ -8735,6 +8851,7 @@
       <c r="AN113" s="7"/>
       <c r="AO113" s="7"/>
       <c r="AP113" s="7"/>
+      <c r="AQ113" s="7"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="inlineStr">
@@ -8823,6 +8940,7 @@
       <c r="AN114" s="7"/>
       <c r="AO114" s="7"/>
       <c r="AP114" s="7"/>
+      <c r="AQ114" s="7"/>
     </row>
     <row r="115">
       <c r="A115" s="7" t="inlineStr">
@@ -8903,6 +9021,7 @@
       <c r="AN115" s="7"/>
       <c r="AO115" s="7"/>
       <c r="AP115" s="7"/>
+      <c r="AQ115" s="7"/>
     </row>
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
@@ -8991,6 +9110,7 @@
       <c r="AN116" s="7"/>
       <c r="AO116" s="7"/>
       <c r="AP116" s="7"/>
+      <c r="AQ116" s="7"/>
     </row>
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
@@ -9075,6 +9195,7 @@
       <c r="AN117" s="7"/>
       <c r="AO117" s="7"/>
       <c r="AP117" s="7"/>
+      <c r="AQ117" s="7"/>
     </row>
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
@@ -9159,6 +9280,7 @@
       <c r="AN118" s="7"/>
       <c r="AO118" s="7"/>
       <c r="AP118" s="7"/>
+      <c r="AQ118" s="7"/>
     </row>
     <row r="119">
       <c r="A119" s="7" t="inlineStr">
@@ -9239,6 +9361,7 @@
       <c r="AN119" s="7"/>
       <c r="AO119" s="7"/>
       <c r="AP119" s="7"/>
+      <c r="AQ119" s="7"/>
     </row>
     <row r="120">
       <c r="A120" s="7" t="inlineStr">
@@ -9311,6 +9434,7 @@
       <c r="AN120" s="7"/>
       <c r="AO120" s="7"/>
       <c r="AP120" s="7"/>
+      <c r="AQ120" s="7"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="inlineStr">
@@ -9395,6 +9519,7 @@
       <c r="AN121" s="7"/>
       <c r="AO121" s="7"/>
       <c r="AP121" s="7"/>
+      <c r="AQ121" s="7"/>
     </row>
     <row r="122">
       <c r="A122" s="7" t="inlineStr">
@@ -9479,6 +9604,7 @@
       <c r="AN122" s="7"/>
       <c r="AO122" s="7"/>
       <c r="AP122" s="7"/>
+      <c r="AQ122" s="7"/>
     </row>
     <row r="123">
       <c r="A123" s="7" t="inlineStr">
@@ -9551,6 +9677,7 @@
       <c r="AN123" s="7"/>
       <c r="AO123" s="7"/>
       <c r="AP123" s="7"/>
+      <c r="AQ123" s="7"/>
     </row>
     <row r="124">
       <c r="A124" s="7" t="inlineStr">
@@ -9631,6 +9758,7 @@
       <c r="AN124" s="7"/>
       <c r="AO124" s="7"/>
       <c r="AP124" s="7"/>
+      <c r="AQ124" s="7"/>
     </row>
     <row r="125">
       <c r="A125" s="7" t="inlineStr">
@@ -9703,6 +9831,7 @@
       <c r="AN125" s="7"/>
       <c r="AO125" s="7"/>
       <c r="AP125" s="7"/>
+      <c r="AQ125" s="7"/>
     </row>
     <row r="126">
       <c r="A126" s="7" t="inlineStr">
@@ -9775,6 +9904,7 @@
       <c r="AN126" s="7"/>
       <c r="AO126" s="7"/>
       <c r="AP126" s="7"/>
+      <c r="AQ126" s="7"/>
     </row>
     <row r="127">
       <c r="A127" s="7" t="inlineStr">
@@ -9851,6 +9981,7 @@
       <c r="AN127" s="7"/>
       <c r="AO127" s="7"/>
       <c r="AP127" s="7"/>
+      <c r="AQ127" s="7"/>
     </row>
     <row r="128">
       <c r="A128" s="7" t="inlineStr">
@@ -9927,6 +10058,7 @@
       <c r="AN128" s="7"/>
       <c r="AO128" s="7"/>
       <c r="AP128" s="7"/>
+      <c r="AQ128" s="7"/>
     </row>
     <row r="129">
       <c r="A129" s="7" t="inlineStr">
@@ -10003,6 +10135,7 @@
       <c r="AN129" s="7"/>
       <c r="AO129" s="7"/>
       <c r="AP129" s="7"/>
+      <c r="AQ129" s="7"/>
     </row>
     <row r="130">
       <c r="A130" s="7" t="inlineStr">
@@ -10075,6 +10208,7 @@
       <c r="AN130" s="7"/>
       <c r="AO130" s="7"/>
       <c r="AP130" s="7"/>
+      <c r="AQ130" s="7"/>
     </row>
     <row r="131">
       <c r="A131" s="7" t="inlineStr">
@@ -10155,6 +10289,7 @@
       <c r="AN131" s="7"/>
       <c r="AO131" s="7"/>
       <c r="AP131" s="7"/>
+      <c r="AQ131" s="7"/>
     </row>
     <row r="132">
       <c r="A132" s="7" t="inlineStr">
@@ -10239,6 +10374,7 @@
       <c r="AN132" s="7"/>
       <c r="AO132" s="7"/>
       <c r="AP132" s="7"/>
+      <c r="AQ132" s="7"/>
     </row>
     <row r="133">
       <c r="A133" s="7" t="inlineStr">
@@ -10323,6 +10459,7 @@
       <c r="AN133" s="7"/>
       <c r="AO133" s="7"/>
       <c r="AP133" s="7"/>
+      <c r="AQ133" s="7"/>
     </row>
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
@@ -10403,6 +10540,7 @@
       <c r="AN134" s="7"/>
       <c r="AO134" s="7"/>
       <c r="AP134" s="7"/>
+      <c r="AQ134" s="7"/>
     </row>
     <row r="135">
       <c r="A135" s="7" t="inlineStr">
@@ -10483,6 +10621,7 @@
       <c r="AN135" s="7"/>
       <c r="AO135" s="7"/>
       <c r="AP135" s="7"/>
+      <c r="AQ135" s="7"/>
     </row>
     <row r="136">
       <c r="A136" s="7" t="inlineStr">
@@ -10563,6 +10702,7 @@
       <c r="AN136" s="7"/>
       <c r="AO136" s="7"/>
       <c r="AP136" s="7"/>
+      <c r="AQ136" s="7"/>
     </row>
     <row r="137">
       <c r="A137" s="7" t="inlineStr">
@@ -10639,6 +10779,7 @@
       <c r="AN137" s="7"/>
       <c r="AO137" s="7"/>
       <c r="AP137" s="7"/>
+      <c r="AQ137" s="7"/>
     </row>
     <row r="138">
       <c r="A138" s="7" t="inlineStr">
@@ -10715,6 +10856,7 @@
       <c r="AN138" s="7"/>
       <c r="AO138" s="7"/>
       <c r="AP138" s="7"/>
+      <c r="AQ138" s="7"/>
     </row>
     <row r="139">
       <c r="A139" s="7" t="inlineStr">
@@ -10791,6 +10933,7 @@
       <c r="AN139" s="7"/>
       <c r="AO139" s="7"/>
       <c r="AP139" s="7"/>
+      <c r="AQ139" s="7"/>
     </row>
     <row r="140">
       <c r="A140" s="7" t="inlineStr">
@@ -10863,6 +11006,7 @@
       <c r="AN140" s="7"/>
       <c r="AO140" s="7"/>
       <c r="AP140" s="7"/>
+      <c r="AQ140" s="7"/>
     </row>
     <row r="141">
       <c r="A141" s="7" t="inlineStr">
@@ -10947,6 +11091,7 @@
       <c r="AN141" s="7"/>
       <c r="AO141" s="7"/>
       <c r="AP141" s="7"/>
+      <c r="AQ141" s="7"/>
     </row>
     <row r="142">
       <c r="A142" s="7" t="inlineStr">
@@ -11019,6 +11164,7 @@
       <c r="AN142" s="7"/>
       <c r="AO142" s="7"/>
       <c r="AP142" s="7"/>
+      <c r="AQ142" s="7"/>
     </row>
     <row r="143">
       <c r="A143" s="7" t="inlineStr">
@@ -11091,6 +11237,7 @@
       <c r="AN143" s="7"/>
       <c r="AO143" s="7"/>
       <c r="AP143" s="7"/>
+      <c r="AQ143" s="7"/>
     </row>
     <row r="144">
       <c r="A144" s="7" t="inlineStr">
@@ -11163,6 +11310,7 @@
       <c r="AN144" s="7"/>
       <c r="AO144" s="7"/>
       <c r="AP144" s="7"/>
+      <c r="AQ144" s="7"/>
     </row>
     <row r="145">
       <c r="A145" s="7" t="inlineStr">
@@ -11251,6 +11399,7 @@
       <c r="AN145" s="7"/>
       <c r="AO145" s="7"/>
       <c r="AP145" s="7"/>
+      <c r="AQ145" s="7"/>
     </row>
     <row r="146">
       <c r="A146" s="7" t="inlineStr">
@@ -11327,6 +11476,7 @@
       <c r="AN146" s="7"/>
       <c r="AO146" s="7"/>
       <c r="AP146" s="7"/>
+      <c r="AQ146" s="7"/>
     </row>
     <row r="147">
       <c r="A147" s="7" t="inlineStr">
@@ -11415,6 +11565,7 @@
       <c r="AN147" s="7"/>
       <c r="AO147" s="7"/>
       <c r="AP147" s="7"/>
+      <c r="AQ147" s="7"/>
     </row>
     <row r="148">
       <c r="A148" s="7" t="inlineStr">
@@ -11487,6 +11638,7 @@
       <c r="AN148" s="7"/>
       <c r="AO148" s="7"/>
       <c r="AP148" s="7"/>
+      <c r="AQ148" s="7"/>
     </row>
     <row r="149">
       <c r="A149" s="7" t="inlineStr">
@@ -11567,6 +11719,7 @@
       <c r="AN149" s="7"/>
       <c r="AO149" s="7"/>
       <c r="AP149" s="7"/>
+      <c r="AQ149" s="7"/>
     </row>
     <row r="150">
       <c r="A150" s="7" t="inlineStr">
@@ -11651,6 +11804,7 @@
       <c r="AN150" s="7"/>
       <c r="AO150" s="7"/>
       <c r="AP150" s="7"/>
+      <c r="AQ150" s="7"/>
     </row>
     <row r="151">
       <c r="A151" s="7" t="inlineStr">
@@ -11727,6 +11881,7 @@
       <c r="AN151" s="7"/>
       <c r="AO151" s="7"/>
       <c r="AP151" s="7"/>
+      <c r="AQ151" s="7"/>
     </row>
     <row r="152">
       <c r="A152" s="7" t="inlineStr">
@@ -11807,6 +11962,7 @@
       <c r="AN152" s="7"/>
       <c r="AO152" s="7"/>
       <c r="AP152" s="7"/>
+      <c r="AQ152" s="7"/>
     </row>
     <row r="153">
       <c r="A153" s="7" t="inlineStr">
@@ -11891,6 +12047,7 @@
       <c r="AN153" s="7"/>
       <c r="AO153" s="7"/>
       <c r="AP153" s="7"/>
+      <c r="AQ153" s="7"/>
     </row>
     <row r="154">
       <c r="A154" s="7" t="inlineStr">
@@ -11959,6 +12116,7 @@
       <c r="AN154" s="7"/>
       <c r="AO154" s="7"/>
       <c r="AP154" s="7"/>
+      <c r="AQ154" s="7"/>
     </row>
     <row r="155">
       <c r="A155" s="7" t="inlineStr">
@@ -12031,6 +12189,7 @@
       <c r="AN155" s="7"/>
       <c r="AO155" s="7"/>
       <c r="AP155" s="7"/>
+      <c r="AQ155" s="7"/>
     </row>
     <row r="156">
       <c r="A156" s="7" t="inlineStr">
@@ -12107,6 +12266,7 @@
       <c r="AN156" s="7"/>
       <c r="AO156" s="7"/>
       <c r="AP156" s="7"/>
+      <c r="AQ156" s="7"/>
     </row>
     <row r="157">
       <c r="A157" s="7" t="inlineStr">
@@ -12179,6 +12339,7 @@
       <c r="AN157" s="7"/>
       <c r="AO157" s="7"/>
       <c r="AP157" s="7"/>
+      <c r="AQ157" s="7"/>
     </row>
     <row r="158">
       <c r="A158" s="7" t="inlineStr">
@@ -12251,6 +12412,7 @@
       <c r="AN158" s="7"/>
       <c r="AO158" s="7"/>
       <c r="AP158" s="7"/>
+      <c r="AQ158" s="7"/>
     </row>
     <row r="159">
       <c r="A159" s="7" t="inlineStr">
@@ -12323,6 +12485,7 @@
       <c r="AN159" s="7"/>
       <c r="AO159" s="7"/>
       <c r="AP159" s="7"/>
+      <c r="AQ159" s="7"/>
     </row>
     <row r="160">
       <c r="A160" s="7" t="inlineStr">
@@ -12395,6 +12558,7 @@
       <c r="AN160" s="7"/>
       <c r="AO160" s="7"/>
       <c r="AP160" s="7"/>
+      <c r="AQ160" s="7"/>
     </row>
     <row r="161">
       <c r="A161" s="7" t="inlineStr">
@@ -12471,6 +12635,7 @@
       <c r="AN161" s="7"/>
       <c r="AO161" s="7"/>
       <c r="AP161" s="7"/>
+      <c r="AQ161" s="7"/>
     </row>
     <row r="162">
       <c r="A162" s="7" t="inlineStr">
@@ -12543,6 +12708,7 @@
       <c r="AN162" s="7"/>
       <c r="AO162" s="7"/>
       <c r="AP162" s="7"/>
+      <c r="AQ162" s="7"/>
     </row>
     <row r="163">
       <c r="A163" s="7" t="inlineStr">
@@ -12615,6 +12781,7 @@
       <c r="AN163" s="7"/>
       <c r="AO163" s="7"/>
       <c r="AP163" s="7"/>
+      <c r="AQ163" s="7"/>
     </row>
     <row r="164">
       <c r="A164" s="7" t="inlineStr">
@@ -12687,6 +12854,7 @@
       <c r="AN164" s="7"/>
       <c r="AO164" s="7"/>
       <c r="AP164" s="7"/>
+      <c r="AQ164" s="7"/>
     </row>
     <row r="165">
       <c r="A165" s="7" t="inlineStr">
@@ -12759,6 +12927,7 @@
       <c r="AN165" s="7"/>
       <c r="AO165" s="7"/>
       <c r="AP165" s="7"/>
+      <c r="AQ165" s="7"/>
     </row>
     <row r="166">
       <c r="A166" s="7" t="inlineStr">
@@ -12839,6 +13008,7 @@
       <c r="AN166" s="7"/>
       <c r="AO166" s="7"/>
       <c r="AP166" s="7"/>
+      <c r="AQ166" s="7"/>
     </row>
     <row r="167">
       <c r="A167" s="7" t="inlineStr">
@@ -12915,6 +13085,7 @@
       <c r="AN167" s="7"/>
       <c r="AO167" s="7"/>
       <c r="AP167" s="7"/>
+      <c r="AQ167" s="7"/>
     </row>
     <row r="168">
       <c r="A168" s="7" t="inlineStr">
@@ -12987,6 +13158,7 @@
       <c r="AN168" s="7"/>
       <c r="AO168" s="7"/>
       <c r="AP168" s="7"/>
+      <c r="AQ168" s="7"/>
     </row>
     <row r="169">
       <c r="A169" s="7" t="inlineStr">
@@ -13059,6 +13231,7 @@
       <c r="AN169" s="7"/>
       <c r="AO169" s="7"/>
       <c r="AP169" s="7"/>
+      <c r="AQ169" s="7"/>
     </row>
     <row r="170">
       <c r="A170" s="7" t="inlineStr">
@@ -13135,6 +13308,7 @@
       <c r="AN170" s="7"/>
       <c r="AO170" s="7"/>
       <c r="AP170" s="7"/>
+      <c r="AQ170" s="7"/>
     </row>
     <row r="171">
       <c r="A171" s="7" t="inlineStr">
@@ -13203,6 +13377,7 @@
       <c r="AN171" s="7"/>
       <c r="AO171" s="7"/>
       <c r="AP171" s="7"/>
+      <c r="AQ171" s="7"/>
     </row>
     <row r="172">
       <c r="A172" s="7" t="inlineStr">
@@ -13271,6 +13446,7 @@
       <c r="AN172" s="7"/>
       <c r="AO172" s="7"/>
       <c r="AP172" s="7"/>
+      <c r="AQ172" s="7"/>
     </row>
     <row r="173">
       <c r="A173" s="7" t="inlineStr">
@@ -13347,6 +13523,7 @@
       <c r="AN173" s="7"/>
       <c r="AO173" s="7"/>
       <c r="AP173" s="7"/>
+      <c r="AQ173" s="7"/>
     </row>
     <row r="174">
       <c r="A174" s="7" t="inlineStr">
@@ -13419,6 +13596,7 @@
       <c r="AN174" s="7"/>
       <c r="AO174" s="7"/>
       <c r="AP174" s="7"/>
+      <c r="AQ174" s="7"/>
     </row>
     <row r="175">
       <c r="A175" s="7" t="inlineStr">
@@ -13495,6 +13673,7 @@
       <c r="AN175" s="7"/>
       <c r="AO175" s="7"/>
       <c r="AP175" s="7"/>
+      <c r="AQ175" s="7"/>
     </row>
     <row r="176">
       <c r="A176" s="7" t="inlineStr">
@@ -13567,6 +13746,7 @@
       <c r="AN176" s="7"/>
       <c r="AO176" s="7"/>
       <c r="AP176" s="7"/>
+      <c r="AQ176" s="7"/>
     </row>
     <row r="177">
       <c r="A177" s="7" t="inlineStr">
@@ -13639,6 +13819,7 @@
       <c r="AN177" s="7"/>
       <c r="AO177" s="7"/>
       <c r="AP177" s="7"/>
+      <c r="AQ177" s="7"/>
     </row>
     <row r="178">
       <c r="A178" s="7" t="inlineStr">
@@ -13711,6 +13892,7 @@
       <c r="AN178" s="7"/>
       <c r="AO178" s="7"/>
       <c r="AP178" s="7"/>
+      <c r="AQ178" s="7"/>
     </row>
     <row r="179">
       <c r="A179" s="7" t="inlineStr">
@@ -13783,6 +13965,7 @@
       <c r="AN179" s="7"/>
       <c r="AO179" s="7"/>
       <c r="AP179" s="7"/>
+      <c r="AQ179" s="7"/>
     </row>
     <row r="180">
       <c r="A180" s="7" t="inlineStr">
@@ -13855,6 +14038,7 @@
       <c r="AN180" s="7"/>
       <c r="AO180" s="7"/>
       <c r="AP180" s="7"/>
+      <c r="AQ180" s="7"/>
     </row>
     <row r="181">
       <c r="A181" s="7" t="inlineStr">
@@ -13927,6 +14111,7 @@
       <c r="AN181" s="7"/>
       <c r="AO181" s="7"/>
       <c r="AP181" s="7"/>
+      <c r="AQ181" s="7"/>
     </row>
     <row r="182">
       <c r="A182" s="7" t="inlineStr">
@@ -13999,6 +14184,7 @@
       <c r="AN182" s="7"/>
       <c r="AO182" s="7"/>
       <c r="AP182" s="7"/>
+      <c r="AQ182" s="7"/>
     </row>
     <row r="183">
       <c r="A183" s="7" t="inlineStr">
@@ -14071,6 +14257,7 @@
       <c r="AN183" s="7"/>
       <c r="AO183" s="7"/>
       <c r="AP183" s="7"/>
+      <c r="AQ183" s="7"/>
     </row>
     <row r="184">
       <c r="A184" s="7" t="inlineStr">
@@ -14139,6 +14326,7 @@
       <c r="AN184" s="7"/>
       <c r="AO184" s="7"/>
       <c r="AP184" s="7"/>
+      <c r="AQ184" s="7"/>
     </row>
     <row r="185">
       <c r="A185" s="7" t="inlineStr">
@@ -14211,6 +14399,7 @@
       <c r="AN185" s="7"/>
       <c r="AO185" s="7"/>
       <c r="AP185" s="7"/>
+      <c r="AQ185" s="7"/>
     </row>
     <row r="186">
       <c r="A186" s="7" t="inlineStr">
@@ -14283,6 +14472,7 @@
       <c r="AN186" s="7"/>
       <c r="AO186" s="7"/>
       <c r="AP186" s="7"/>
+      <c r="AQ186" s="7"/>
     </row>
     <row r="187">
       <c r="A187" s="7" t="inlineStr">
@@ -14359,6 +14549,7 @@
       <c r="AN187" s="7"/>
       <c r="AO187" s="7"/>
       <c r="AP187" s="7"/>
+      <c r="AQ187" s="7"/>
     </row>
     <row r="188">
       <c r="A188" s="7" t="inlineStr">
@@ -14435,6 +14626,7 @@
       <c r="AN188" s="7"/>
       <c r="AO188" s="7"/>
       <c r="AP188" s="7"/>
+      <c r="AQ188" s="7"/>
     </row>
     <row r="189">
       <c r="A189" s="7" t="inlineStr">
@@ -14511,6 +14703,7 @@
       <c r="AN189" s="7"/>
       <c r="AO189" s="7"/>
       <c r="AP189" s="7"/>
+      <c r="AQ189" s="7"/>
     </row>
     <row r="190">
       <c r="A190" s="7" t="inlineStr">
@@ -14587,6 +14780,7 @@
       <c r="AN190" s="7"/>
       <c r="AO190" s="7"/>
       <c r="AP190" s="7"/>
+      <c r="AQ190" s="7"/>
     </row>
     <row r="191">
       <c r="A191" s="7" t="inlineStr">
@@ -14663,6 +14857,7 @@
       <c r="AN191" s="7"/>
       <c r="AO191" s="7"/>
       <c r="AP191" s="7"/>
+      <c r="AQ191" s="7"/>
     </row>
     <row r="192">
       <c r="A192" s="7" t="inlineStr">
@@ -14739,6 +14934,7 @@
       <c r="AN192" s="7"/>
       <c r="AO192" s="7"/>
       <c r="AP192" s="7"/>
+      <c r="AQ192" s="7"/>
     </row>
     <row r="193">
       <c r="A193" s="7" t="inlineStr">
@@ -14815,6 +15011,11 @@
       <c r="AN193" s="7"/>
       <c r="AO193" s="7"/>
       <c r="AP193" s="7"/>
+      <c r="AQ193" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="7" t="inlineStr">
@@ -14891,6 +15092,11 @@
       <c r="AN194" s="7"/>
       <c r="AO194" s="7"/>
       <c r="AP194" s="7"/>
+      <c r="AQ194" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="7" t="inlineStr">
@@ -14920,7 +15126,7 @@
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t xml:space="preserve">#190</t>
+          <t xml:space="preserve">#190 · AQ 109e859 — 알림 「복합 가공소가 열렸습니다」 · 1걸음(변환기 → 발전재료) Pass · 조건 = Auto 끔(CID_204)</t>
         </is>
       </c>
       <c r="G195" s="7"/>
@@ -14967,6 +15173,11 @@
       <c r="AN195" s="7"/>
       <c r="AO195" s="7"/>
       <c r="AP195" s="7"/>
+      <c r="AQ195" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="7" t="inlineStr">
@@ -14996,7 +15207,7 @@
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t xml:space="preserve">#190 · 끝 = 구조 판정(구현 판단) · 10-19 사용자 육안(8133 4a6f983 · 20:4x) — 폭발탄 걸음 ①~⑤ 끝까지</t>
+          <t xml:space="preserve">#190 · 끝 = 구조 판정(구현 판단) · 10-19 사용자 육안(8133 4a6f983 · 20:4x) — 폭발탄 걸음 ①~⑤ 끝까지 · AQ 못 봄 — 2걸음(벨트 덮어쓰기) Pass · 3걸음부터 인앱 창 캡처가 캔버스 y≤771 만 보여 팔레트(분류기) 못 고름 · 바로가기 S5 는 막 안 섬(CID_205)</t>
         </is>
       </c>
       <c r="G196" s="7"/>
@@ -15039,6 +15250,7 @@
       <c r="AN196" s="7"/>
       <c r="AO196" s="7"/>
       <c r="AP196" s="7"/>
+      <c r="AQ196" s="7"/>
     </row>
     <row r="197">
       <c r="A197" s="7" t="inlineStr">
@@ -15068,7 +15280,7 @@
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t xml:space="preserve">#191 · S6 화면 미확인</t>
+          <t xml:space="preserve">#191 · S6 화면 미확인 · AQ — S3 · S4 · S5 · S6 파밍/도전 배지 주제 확인</t>
         </is>
       </c>
       <c r="G197" s="7"/>
@@ -15115,6 +15327,11 @@
       <c r="AN197" s="7"/>
       <c r="AO197" s="7"/>
       <c r="AP197" s="7"/>
+      <c r="AQ197" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="7" t="inlineStr">
@@ -15187,6 +15404,7 @@
       <c r="AN198" s="7"/>
       <c r="AO198" s="7"/>
       <c r="AP198" s="7"/>
+      <c r="AQ198" s="7"/>
     </row>
     <row r="199">
       <c r="A199" s="7" t="inlineStr">
@@ -15216,7 +15434,7 @@
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t xml:space="preserve">#193</t>
+          <t xml:space="preserve">#193 · AQ — S4 「통과함」 · 승리 화면 [스테이지로][다음 스테이지로]</t>
         </is>
       </c>
       <c r="G199" s="7"/>
@@ -15263,6 +15481,11 @@
       <c r="AN199" s="7"/>
       <c r="AO199" s="7"/>
       <c r="AP199" s="7"/>
+      <c r="AQ199" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="7" t="inlineStr">
@@ -15292,7 +15515,7 @@
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t xml:space="preserve">#194</t>
+          <t xml:space="preserve">#194 · AQ — S1 「강화 재료 +30」 · S4 승리(보상 0) 안 뜸</t>
         </is>
       </c>
       <c r="G200" s="7"/>
@@ -15339,6 +15562,11 @@
       <c r="AN200" s="7"/>
       <c r="AO200" s="7"/>
       <c r="AP200" s="7"/>
+      <c r="AQ200" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="7" t="inlineStr">
@@ -15368,7 +15596,7 @@
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t xml:space="preserve">#195</t>
+          <t xml:space="preserve">#195 · AQ — S6 정지 · 「로봇 B 마운트를 탭한 뒤 강화를 누르세요」 · 재료 50/50 → 0/50 · Lv 2 · 피해량 ×1.45 · 강화 완료</t>
         </is>
       </c>
       <c r="G201" s="7"/>
@@ -15407,6 +15635,11 @@
       <c r="AN201" s="7"/>
       <c r="AO201" s="7"/>
       <c r="AP201" s="7"/>
+      <c r="AQ201" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="7" t="inlineStr">
@@ -15483,6 +15716,11 @@
       <c r="AN202" s="7"/>
       <c r="AO202" s="7"/>
       <c r="AP202" s="7"/>
+      <c r="AQ202" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="7" t="inlineStr">
@@ -15512,7 +15750,7 @@
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t xml:space="preserve">#197 · 8132 이하 결함 · 10-19 사용자 육안(8133 4a6f983 · 20:4x) — 새로고침 뒤 보드 유지</t>
+          <t xml:space="preserve">#197 · 8132 이하 결함 · 10-19 사용자 육안(8133 4a6f983 · 20:4x) — 새로고침 뒤 보드 유지 · AQ — A 판(폭발탄 1·2걸음 흔적) 그대로 · 단 시작 판 S1(CID_207)</t>
         </is>
       </c>
       <c r="G203" s="7"/>
@@ -15559,6 +15797,11 @@
       <c r="AN203" s="7"/>
       <c r="AO203" s="7"/>
       <c r="AP203" s="7"/>
+      <c r="AQ203" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="7" t="inlineStr">
@@ -15588,7 +15831,7 @@
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t xml:space="preserve">#198 · 4a6f983 사용자 육안 = 재료 0(Fail) → e86eb9a 에서 고침</t>
+          <t xml:space="preserve">#198 · 4a6f983 사용자 육안 = 재료 0(Fail) → e86eb9a 에서 고침 · AQ — 처음부터 → S3 점프: 재료 63/50 · 고철 300/300 · 막 · 정지</t>
         </is>
       </c>
       <c r="G204" s="7"/>
@@ -15635,6 +15878,11 @@
       </c>
       <c r="AO204" s="7"/>
       <c r="AP204" s="7"/>
+      <c r="AQ204" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="7" t="inlineStr">
@@ -15664,7 +15912,7 @@
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t xml:space="preserve">#198 · 4a6f983 사용자 육안 = A·B 강화 불가(B 재료 0/50) Fail → e86eb9a</t>
+          <t xml:space="preserve">#198 · 4a6f983 사용자 육안 = A·B 강화 불가(B 재료 0/50) Fail → e86eb9a · AQ — 자연 진행(A 강화) 뒤 S6 점프: B 재료 50/50 · B 막에서 직접 강화</t>
         </is>
       </c>
       <c r="G205" s="7"/>
@@ -15715,6 +15963,11 @@
         </is>
       </c>
       <c r="AP205" s="7"/>
+      <c r="AQ205" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="7" t="inlineStr">
@@ -15791,6 +16044,11 @@
         </is>
       </c>
       <c r="AP206" s="7"/>
+      <c r="AQ206" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="7" t="inlineStr">
@@ -15820,7 +16078,7 @@
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t xml:space="preserve">#201 결함 · 4a6f983 사용자 육안 S6 「전투력 0 넘기기」 Fail → e86eb9a</t>
+          <t xml:space="preserve">#201 결함 · 4a6f983 사용자 육안 S6 「전투력 0 넘기기」 Fail → e86eb9a · AQ — S6 「목표: 자유 플레이 · 보스」 · S5 도전 배지는 못 봄</t>
         </is>
       </c>
       <c r="G207" s="7"/>
@@ -15863,6 +16121,11 @@
       <c r="AN207" s="7"/>
       <c r="AO207" s="7"/>
       <c r="AP207" s="7"/>
+      <c r="AQ207" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="7" t="inlineStr">
@@ -15892,7 +16155,7 @@
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t xml:space="preserve">4a6f983 사용자 육안 = 시간 초과(보스 ≈30%) · 조건 = 옛 저장(#197 전 A 판 리셋 · HUD 전투력 0) — 새 저장으로 재확인 자리</t>
+          <t xml:space="preserve">4a6f983 사용자 육안 = 시간 초과(보스 ≈30%) · 조건 = 옛 저장(#197 전 A 판 리셋 · HUD 전투력 0) — 새 저장으로 재확인 자리 · AQ Fail — 시간 초과 · 보스 ≈40% 남음. 조건 = A 판이 폭발탄 1·2걸음만 된 채(라인 끊김) → 마운트 탄 0/200 · HUD 전투력 3→0 · 합체 1회</t>
         </is>
       </c>
       <c r="G208" s="7"/>
@@ -15935,6 +16198,11 @@
       <c r="AN208" s="7"/>
       <c r="AO208" s="7"/>
       <c r="AP208" s="7"/>
+      <c r="AQ208" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="7" t="inlineStr">
@@ -16011,6 +16279,11 @@
         </is>
       </c>
       <c r="AP209" s="7"/>
+      <c r="AQ209" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="7" t="inlineStr">
@@ -16040,7 +16313,7 @@
       </c>
       <c r="F210" t="inlineStr">
         <is>
-          <t xml:space="preserve">#203 · 범위 = 사용자 「S1 S3 S6」 · 물류 계속 ⚠️ 가정</t>
+          <t xml:space="preserve">#203 · 범위 = 사용자 「S1 S3 S6」 · 물류 계속 ⚠️ 가정 · AQ — S1 T3 · S3 강화 · S6 B 강화 셋 다 정지(리젠 고정 · 적 정지) → 해제 뒤 재개</t>
         </is>
       </c>
       <c r="G210" s="7"/>
@@ -16083,6 +16356,11 @@
         </is>
       </c>
       <c r="AP210" s="7"/>
+      <c r="AQ210" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="7" t="inlineStr">
@@ -16112,7 +16390,7 @@
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t xml:space="preserve">#204 · S4 비율 ⚠️ 플랜 어림 · 하네스 생존(593 · 723)</t>
+          <t xml:space="preserve">#204 · S4 비율 ⚠️ 플랜 어림 · 하네스 생존(593 · 723) · AQ 경계 — S3 파밍 약 55~65초 뒤 파괴(하네스는 생존 593) · S4 파밍 「맵 9~10/10」 HP 983 유지 ✅</t>
         </is>
       </c>
       <c r="G211" s="7"/>
@@ -16155,6 +16433,295 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AQ211" s="7"/>
+    </row>
+    <row r="212">
+      <c r="A212" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_204</t>
+        </is>
+      </c>
+      <c r="B212" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼</t>
+        </is>
+      </c>
+      <c r="C212" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S5 폭발탄</t>
+        </is>
+      </c>
+      <c r="D212" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Auto 태그 중</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Auto 태그가 켜진 채 S5 폭발탄 막에서 조립을 열면, 교대 때마다 보드가 B 판으로 따라가도 안내 · 잠금이 유지되는가(B 판 탭이 보통 조작으로 새지 않는가)?</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AQ 코드 세션 실측 — 교대마다 보드가 B 판으로 바뀌어(FollowActiveRobotTab) 안내가 사라지고, B 판 변환기 탭에 생산량 모듈이 붙어 고철 −30. Auto 끄면 A 판 고정 · 1·2걸음 정상</t>
+        </is>
+      </c>
+      <c r="G212" s="7"/>
+      <c r="H212" s="7"/>
+      <c r="I212" s="7"/>
+      <c r="J212" s="7"/>
+      <c r="K212" s="7"/>
+      <c r="L212" s="7"/>
+      <c r="M212" s="7"/>
+      <c r="N212" s="7"/>
+      <c r="O212" s="7"/>
+      <c r="P212" s="7"/>
+      <c r="Q212" s="7"/>
+      <c r="R212" s="7"/>
+      <c r="S212" s="7"/>
+      <c r="T212" s="7"/>
+      <c r="U212" s="7"/>
+      <c r="V212" s="7"/>
+      <c r="W212" s="7"/>
+      <c r="X212" s="7"/>
+      <c r="Y212" s="7"/>
+      <c r="Z212" s="7"/>
+      <c r="AA212" s="7"/>
+      <c r="AB212" s="7"/>
+      <c r="AC212" s="7"/>
+      <c r="AD212" s="7"/>
+      <c r="AE212" s="7"/>
+      <c r="AF212" s="7"/>
+      <c r="AG212" s="7"/>
+      <c r="AH212" s="7"/>
+      <c r="AI212" s="7"/>
+      <c r="AJ212" s="7"/>
+      <c r="AK212" s="7"/>
+      <c r="AL212" s="7"/>
+      <c r="AM212" s="7"/>
+      <c r="AN212" s="7"/>
+      <c r="AO212" s="7"/>
+      <c r="AP212" s="7"/>
+      <c r="AQ212" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_205</t>
+        </is>
+      </c>
+      <c r="B213" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼</t>
+        </is>
+      </c>
+      <c r="C213" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S5 폭발탄</t>
+        </is>
+      </c>
+      <c r="D213" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">바로가기 점프</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t xml:space="preserve">바로가기 S5 점프(튜토리얼 안 마친 새 저장)에서도 폭발탄 막이 서는가? (#198 이 A · B 강화 막은 튜토리얼 마침 조건을 걷었다)</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AQ — 「처음부터」 → 바로가기 S5 = 막 안 섬 · 「도전」 밝음. ExplosiveTutorialRule.IsActive 가 tutorialCleared 요구(판정 요청 · 의도인지)</t>
+        </is>
+      </c>
+      <c r="G213" s="7"/>
+      <c r="H213" s="7"/>
+      <c r="I213" s="7"/>
+      <c r="J213" s="7"/>
+      <c r="K213" s="7"/>
+      <c r="L213" s="7"/>
+      <c r="M213" s="7"/>
+      <c r="N213" s="7"/>
+      <c r="O213" s="7"/>
+      <c r="P213" s="7"/>
+      <c r="Q213" s="7"/>
+      <c r="R213" s="7"/>
+      <c r="S213" s="7"/>
+      <c r="T213" s="7"/>
+      <c r="U213" s="7"/>
+      <c r="V213" s="7"/>
+      <c r="W213" s="7"/>
+      <c r="X213" s="7"/>
+      <c r="Y213" s="7"/>
+      <c r="Z213" s="7"/>
+      <c r="AA213" s="7"/>
+      <c r="AB213" s="7"/>
+      <c r="AC213" s="7"/>
+      <c r="AD213" s="7"/>
+      <c r="AE213" s="7"/>
+      <c r="AF213" s="7"/>
+      <c r="AG213" s="7"/>
+      <c r="AH213" s="7"/>
+      <c r="AI213" s="7"/>
+      <c r="AJ213" s="7"/>
+      <c r="AK213" s="7"/>
+      <c r="AL213" s="7"/>
+      <c r="AM213" s="7"/>
+      <c r="AN213" s="7"/>
+      <c r="AO213" s="7"/>
+      <c r="AP213" s="7"/>
+      <c r="AQ213" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_206</t>
+        </is>
+      </c>
+      <c r="B214" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">파밍</t>
+        </is>
+      </c>
+      <c r="C214" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S5 파밍</t>
+        </is>
+      </c>
+      <c r="D214" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">생존</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t xml:space="preserve">자연 진행으로 S5 파밍에 든 뒤(A 강화 · B 미강화 · Auto 태그 · A 판 = 시작 보드 + M) 60초 넘게 버티는가?</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AQ — 약 60초(게임) 만에 파괴 → S4 로 내려감. 마운트 탄 0~2/200 · HP 1000→299→0. 폭발탄 막 진행 중(1걸음 전후)</t>
+        </is>
+      </c>
+      <c r="G214" s="7"/>
+      <c r="H214" s="7"/>
+      <c r="I214" s="7"/>
+      <c r="J214" s="7"/>
+      <c r="K214" s="7"/>
+      <c r="L214" s="7"/>
+      <c r="M214" s="7"/>
+      <c r="N214" s="7"/>
+      <c r="O214" s="7"/>
+      <c r="P214" s="7"/>
+      <c r="Q214" s="7"/>
+      <c r="R214" s="7"/>
+      <c r="S214" s="7"/>
+      <c r="T214" s="7"/>
+      <c r="U214" s="7"/>
+      <c r="V214" s="7"/>
+      <c r="W214" s="7"/>
+      <c r="X214" s="7"/>
+      <c r="Y214" s="7"/>
+      <c r="Z214" s="7"/>
+      <c r="AA214" s="7"/>
+      <c r="AB214" s="7"/>
+      <c r="AC214" s="7"/>
+      <c r="AD214" s="7"/>
+      <c r="AE214" s="7"/>
+      <c r="AF214" s="7"/>
+      <c r="AG214" s="7"/>
+      <c r="AH214" s="7"/>
+      <c r="AI214" s="7"/>
+      <c r="AJ214" s="7"/>
+      <c r="AK214" s="7"/>
+      <c r="AL214" s="7"/>
+      <c r="AM214" s="7"/>
+      <c r="AN214" s="7"/>
+      <c r="AO214" s="7"/>
+      <c r="AP214" s="7"/>
+      <c r="AQ214" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_207</t>
+        </is>
+      </c>
+      <c r="B215" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">저장</t>
+        </is>
+      </c>
+      <c r="C215" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">새로고침</t>
+        </is>
+      </c>
+      <c r="D215" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">판 복귀</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S6 파밍(바로가기 점프 · 직전 자연 진행 S4) 중 새로고침하면 마지막 판으로 돌아오는가?</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AQ — S1 파밍으로 돌아옴(지갑 · 보드는 유지). 의도(점프는 저장 안 함 등)인지 판정 요청</t>
+        </is>
+      </c>
+      <c r="G215" s="7"/>
+      <c r="H215" s="7"/>
+      <c r="I215" s="7"/>
+      <c r="J215" s="7"/>
+      <c r="K215" s="7"/>
+      <c r="L215" s="7"/>
+      <c r="M215" s="7"/>
+      <c r="N215" s="7"/>
+      <c r="O215" s="7"/>
+      <c r="P215" s="7"/>
+      <c r="Q215" s="7"/>
+      <c r="R215" s="7"/>
+      <c r="S215" s="7"/>
+      <c r="T215" s="7"/>
+      <c r="U215" s="7"/>
+      <c r="V215" s="7"/>
+      <c r="W215" s="7"/>
+      <c r="X215" s="7"/>
+      <c r="Y215" s="7"/>
+      <c r="Z215" s="7"/>
+      <c r="AA215" s="7"/>
+      <c r="AB215" s="7"/>
+      <c r="AC215" s="7"/>
+      <c r="AD215" s="7"/>
+      <c r="AE215" s="7"/>
+      <c r="AF215" s="7"/>
+      <c r="AG215" s="7"/>
+      <c r="AH215" s="7"/>
+      <c r="AI215" s="7"/>
+      <c r="AJ215" s="7"/>
+      <c r="AK215" s="7"/>
+      <c r="AL215" s="7"/>
+      <c r="AM215" s="7"/>
+      <c r="AN215" s="7"/>
+      <c r="AO215" s="7"/>
+      <c r="AP215" s="7"/>
+      <c r="AQ215" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="26">
@@ -16183,9 +16750,9 @@
     <mergeCell ref="B92:B99"/>
     <mergeCell ref="B100:B106"/>
     <mergeCell ref="B107:B111"/>
-    <mergeCell ref="G7:AP7"/>
+    <mergeCell ref="G7:AQ7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:AP211">
+  <conditionalFormatting sqref="G9:AQ215">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
QA AQ 정정: CID_200 · CID_195 조건(S6 점프 = 폭발탄 프리셋 판)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -15750,7 +15750,7 @@
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t xml:space="preserve">#197 · 8132 이하 결함 · 10-19 사용자 육안(8133 4a6f983 · 20:4x) — 새로고침 뒤 보드 유지 · AQ — A 판(폭발탄 1·2걸음 흔적) 그대로 · 단 시작 판 S1(CID_207)</t>
+          <t xml:space="preserve">#197 · 8132 이하 결함 · 10-19 사용자 육안(8133 4a6f983 · 20:4x) — 새로고침 뒤 보드 유지 · AQ — A 판(S6 점프가 세운 폭발탄 프리셋 · 🗑️ 「1·2걸음 흔적」 정정) 그대로 · 단 시작 판 S1(CID_207)</t>
         </is>
       </c>
       <c r="G203" s="7"/>
@@ -16155,7 +16155,7 @@
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t xml:space="preserve">4a6f983 사용자 육안 = 시간 초과(보스 ≈30%) · 조건 = 옛 저장(#197 전 A 판 리셋 · HUD 전투력 0) — 새 저장으로 재확인 자리 · AQ Fail — 시간 초과 · 보스 ≈40% 남음. 조건 = A 판이 폭발탄 1·2걸음만 된 채(라인 끊김) → 마운트 탄 0/200 · HUD 전투력 3→0 · 합체 1회</t>
+          <t xml:space="preserve">4a6f983 사용자 육안 = 시간 초과(보스 ≈30%) · 조건 = 옛 저장(#197 전 A 판 리셋 · HUD 전투력 0) — 새 저장으로 재확인 자리 · AQ Fail — 시간 초과 · 보스 ≈40% 남음. 🗑️(정정) 「A 판이 폭발탄 1·2걸음만 된 채」는 틀림 — 바로가기 S6 점프가 #167 폭발탄 프리셋으로 A 판을 덮었다(새로고침 뒤 복합 가공소 확인). 조건 = 바로가기 S6 · A 판 폭발탄 프리셋 · A·B 강화 · 마운트 탄 0/200 · HUD 전투력 3→0 · 합체 1회</t>
         </is>
       </c>
       <c r="G208" s="7"/>

</xml_diff>

<commit_message>
QA AR(7635b57 보이는 창 재확인 · Pass 8 · Fail 2 · N/A 1 · CID_208~215) · 촬영 가이드 7635b57
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -199,8 +199,9 @@
     <col min="41" max="41" width="12" customWidth="1"/>
     <col min="42" max="42" width="12" customWidth="1"/>
     <col min="43" max="43" width="12" customWidth="1"/>
-    <col min="44" max="44" width="11" customWidth="1"/>
+    <col min="44" max="44" width="12" customWidth="1"/>
     <col min="45" max="45" width="11" customWidth="1"/>
+    <col min="46" max="46" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -498,6 +499,11 @@
       <c r="AQ6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">8133 109e859 전체 플레이 한 바퀴(코드 세션 · 인앱 브라우저 · 소리 0) — 자연 진행 S1→S5(파괴 → S4) → 바로가기 S6 · 새로고침 · 처음부터 → 바로가기 S3 · S5. 빈 칸 = 못 봄(까닭은 F). 새 결함 = CID_204~207.</t>
+        </is>
+      </c>
+      <c r="AR6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8133 7635b57 갈아엎음(23:02) · #206 첫 스폰 띠 ×1.3 · #207 튜토리얼 국면 전부 정지+스폰 보류 · #208 S3 장갑 0 · #209 복구 · 모듈 풀림 · CID_204 탭 고정 ‖ 보이는 창(인앱 브라우저 · 소리 0) 재확인 — 남은 저장 → S1 T3 · S2 T4 · S3 파밍 / 처음부터 → 바로가기 S3 · S6 길. 자연 진행 S4 해금 · S4 합체 막 · S5 폭발탄은 못 봄(T1 벨트 끌기가 인앱 브라우저에서 안 먹음). 시험 1675/1669/0/6 · 전투 12줄 = S3 두 줄만.</t>
         </is>
       </c>
     </row>
@@ -565,14 +571,15 @@
       <c r="AO7" s="2"/>
       <c r="AP7" s="2"/>
       <c r="AQ7" s="2"/>
-      <c r="AR7" s="2" t="inlineStr">
+      <c r="AR7" s="2"/>
+      <c r="AS7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">버전</t>
         </is>
       </c>
-      <c r="AS7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">109e859</t>
+      <c r="AT7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7635b57</t>
         </is>
       </c>
     </row>
@@ -782,11 +789,16 @@
       </c>
       <c r="AR8" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">7635b57</t>
+        </is>
+      </c>
+      <c r="AS8" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">PASSrate</t>
         </is>
       </c>
-      <c r="AS8" s="7">
-        <f>COUNTIF(AQ9:AQ215,"Pass")</f>
+      <c r="AT8" s="7">
+        <f>COUNTIF(AR9:AR223,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -893,13 +905,14 @@
       <c r="AO9" s="7"/>
       <c r="AP9" s="7"/>
       <c r="AQ9" s="7"/>
-      <c r="AR9" s="2" t="inlineStr">
+      <c r="AR9" s="7"/>
+      <c r="AS9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FAILrate</t>
         </is>
       </c>
-      <c r="AS9" s="7">
-        <f>COUNTIF(AQ9:AQ215,"Fail")+COUNTIF(AQ9:AQ215,"Broken")</f>
+      <c r="AT9" s="7">
+        <f>COUNTIF(AR9:AR223,"Fail")+COUNTIF(AR9:AR223,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -970,13 +983,14 @@
       <c r="AO10" s="7"/>
       <c r="AP10" s="7"/>
       <c r="AQ10" s="7"/>
-      <c r="AR10" s="2" t="inlineStr">
+      <c r="AR10" s="7"/>
+      <c r="AS10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">N/A</t>
         </is>
       </c>
-      <c r="AS10" s="7">
-        <f>COUNTIF(AQ9:AQ215,"N/A")</f>
+      <c r="AT10" s="7">
+        <f>COUNTIF(AR9:AR223,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -1047,13 +1061,14 @@
       <c r="AO11" s="7"/>
       <c r="AP11" s="7"/>
       <c r="AQ11" s="7"/>
-      <c r="AR11" s="2" t="inlineStr">
+      <c r="AR11" s="7"/>
+      <c r="AS11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">전체 개수</t>
         </is>
       </c>
-      <c r="AS11" s="7">
-        <v>207</v>
+      <c r="AT11" s="7">
+        <v>215</v>
       </c>
     </row>
     <row r="12">
@@ -1124,13 +1139,14 @@
       <c r="AO12" s="7"/>
       <c r="AP12" s="7"/>
       <c r="AQ12" s="7"/>
-      <c r="AR12" s="2" t="inlineStr">
+      <c r="AR12" s="7"/>
+      <c r="AS12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">진행율</t>
         </is>
       </c>
-      <c r="AS12" s="7">
-        <f>TEXT((COUNTA(AQ9:AQ215))/207,"0.00%")</f>
+      <c r="AT12" s="7">
+        <f>TEXT((COUNTA(AR9:AR223))/215,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -1205,6 +1221,7 @@
       <c r="AO13" s="7"/>
       <c r="AP13" s="7"/>
       <c r="AQ13" s="7"/>
+      <c r="AR13" s="7"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -1269,6 +1286,7 @@
       <c r="AO14" s="7"/>
       <c r="AP14" s="7"/>
       <c r="AQ14" s="7"/>
+      <c r="AR14" s="7"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -1369,6 +1387,7 @@
       <c r="AO15" s="7"/>
       <c r="AP15" s="7"/>
       <c r="AQ15" s="7"/>
+      <c r="AR15" s="7"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -1469,6 +1488,7 @@
       <c r="AO16" s="7"/>
       <c r="AP16" s="7"/>
       <c r="AQ16" s="7"/>
+      <c r="AR16" s="7"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -1574,6 +1594,7 @@
       <c r="AO17" s="7"/>
       <c r="AP17" s="7"/>
       <c r="AQ17" s="7"/>
+      <c r="AR17" s="7"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -1643,6 +1664,7 @@
       <c r="AO18" s="7"/>
       <c r="AP18" s="7"/>
       <c r="AQ18" s="7"/>
+      <c r="AR18" s="7"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -1707,6 +1729,7 @@
       <c r="AO19" s="7"/>
       <c r="AP19" s="7"/>
       <c r="AQ19" s="7"/>
+      <c r="AR19" s="7"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1771,6 +1794,7 @@
       <c r="AO20" s="7"/>
       <c r="AP20" s="7"/>
       <c r="AQ20" s="7"/>
+      <c r="AR20" s="7"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1871,6 +1895,7 @@
       <c r="AO21" s="7"/>
       <c r="AP21" s="7"/>
       <c r="AQ21" s="7"/>
+      <c r="AR21" s="7"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1964,6 +1989,7 @@
       <c r="AO22" s="7"/>
       <c r="AP22" s="7"/>
       <c r="AQ22" s="7"/>
+      <c r="AR22" s="7"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -2036,6 +2062,7 @@
       <c r="AO23" s="7"/>
       <c r="AP23" s="7"/>
       <c r="AQ23" s="7"/>
+      <c r="AR23" s="7"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -2100,6 +2127,7 @@
       <c r="AO24" s="7"/>
       <c r="AP24" s="7"/>
       <c r="AQ24" s="7"/>
+      <c r="AR24" s="7"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -2164,6 +2192,7 @@
       <c r="AO25" s="7"/>
       <c r="AP25" s="7"/>
       <c r="AQ25" s="7"/>
+      <c r="AR25" s="7"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -2257,6 +2286,7 @@
       <c r="AO26" s="7"/>
       <c r="AP26" s="7"/>
       <c r="AQ26" s="7"/>
+      <c r="AR26" s="7"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -2325,6 +2355,7 @@
       <c r="AO27" s="7"/>
       <c r="AP27" s="7"/>
       <c r="AQ27" s="7"/>
+      <c r="AR27" s="7"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -2402,6 +2433,7 @@
       <c r="AO28" s="7"/>
       <c r="AP28" s="7"/>
       <c r="AQ28" s="7"/>
+      <c r="AR28" s="7"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -2474,6 +2506,7 @@
       <c r="AO29" s="7"/>
       <c r="AP29" s="7"/>
       <c r="AQ29" s="7"/>
+      <c r="AR29" s="7"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -2570,6 +2603,7 @@
       <c r="AO30" s="7"/>
       <c r="AP30" s="7"/>
       <c r="AQ30" s="7"/>
+      <c r="AR30" s="7"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -2671,6 +2705,7 @@
       <c r="AO31" s="7"/>
       <c r="AP31" s="7"/>
       <c r="AQ31" s="7"/>
+      <c r="AR31" s="7"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -2759,6 +2794,7 @@
       <c r="AO32" s="7"/>
       <c r="AP32" s="7"/>
       <c r="AQ32" s="7"/>
+      <c r="AR32" s="7"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -2855,6 +2891,7 @@
       <c r="AO33" s="7"/>
       <c r="AP33" s="7"/>
       <c r="AQ33" s="7"/>
+      <c r="AR33" s="7"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -2951,6 +2988,7 @@
       <c r="AO34" s="7"/>
       <c r="AP34" s="7"/>
       <c r="AQ34" s="7"/>
+      <c r="AR34" s="7"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -3056,6 +3094,7 @@
       <c r="AO35" s="7"/>
       <c r="AP35" s="7"/>
       <c r="AQ35" s="7"/>
+      <c r="AR35" s="7"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -3136,6 +3175,7 @@
       <c r="AO36" s="7"/>
       <c r="AP36" s="7"/>
       <c r="AQ36" s="7"/>
+      <c r="AR36" s="7"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -3200,6 +3240,7 @@
       <c r="AO37" s="7"/>
       <c r="AP37" s="7"/>
       <c r="AQ37" s="7"/>
+      <c r="AR37" s="7"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -3285,6 +3326,7 @@
       <c r="AO38" s="7"/>
       <c r="AP38" s="7"/>
       <c r="AQ38" s="7"/>
+      <c r="AR38" s="7"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -3381,6 +3423,7 @@
       <c r="AO39" s="7"/>
       <c r="AP39" s="7"/>
       <c r="AQ39" s="7"/>
+      <c r="AR39" s="7"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -3478,6 +3521,7 @@
       <c r="AO40" s="7"/>
       <c r="AP40" s="7"/>
       <c r="AQ40" s="7"/>
+      <c r="AR40" s="7"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -3570,6 +3614,7 @@
       <c r="AO41" s="7"/>
       <c r="AP41" s="7"/>
       <c r="AQ41" s="7"/>
+      <c r="AR41" s="7"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -3646,6 +3691,7 @@
       <c r="AO42" s="7"/>
       <c r="AP42" s="7"/>
       <c r="AQ42" s="7"/>
+      <c r="AR42" s="7"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -3742,6 +3788,7 @@
       <c r="AO43" s="7"/>
       <c r="AP43" s="7"/>
       <c r="AQ43" s="7"/>
+      <c r="AR43" s="7"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -3811,6 +3858,7 @@
       <c r="AO44" s="7"/>
       <c r="AP44" s="7"/>
       <c r="AQ44" s="7"/>
+      <c r="AR44" s="7"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -3903,6 +3951,7 @@
       <c r="AO45" s="7"/>
       <c r="AP45" s="7"/>
       <c r="AQ45" s="7"/>
+      <c r="AR45" s="7"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -3995,6 +4044,7 @@
       <c r="AO46" s="7"/>
       <c r="AP46" s="7"/>
       <c r="AQ46" s="7"/>
+      <c r="AR46" s="7"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -4064,6 +4114,7 @@
       <c r="AO47" s="7"/>
       <c r="AP47" s="7"/>
       <c r="AQ47" s="7"/>
+      <c r="AR47" s="7"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -4128,6 +4179,7 @@
       <c r="AO48" s="7"/>
       <c r="AP48" s="7"/>
       <c r="AQ48" s="7"/>
+      <c r="AR48" s="7"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -4192,6 +4244,7 @@
       <c r="AO49" s="7"/>
       <c r="AP49" s="7"/>
       <c r="AQ49" s="7"/>
+      <c r="AR49" s="7"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -4280,6 +4333,7 @@
       <c r="AO50" s="7"/>
       <c r="AP50" s="7"/>
       <c r="AQ50" s="7"/>
+      <c r="AR50" s="7"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -4368,6 +4422,7 @@
       <c r="AO51" s="7"/>
       <c r="AP51" s="7"/>
       <c r="AQ51" s="7"/>
+      <c r="AR51" s="7"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -4437,6 +4492,7 @@
       <c r="AO52" s="7"/>
       <c r="AP52" s="7"/>
       <c r="AQ52" s="7"/>
+      <c r="AR52" s="7"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -4506,6 +4562,7 @@
       <c r="AO53" s="7"/>
       <c r="AP53" s="7"/>
       <c r="AQ53" s="7"/>
+      <c r="AR53" s="7"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -4570,6 +4627,7 @@
       <c r="AO54" s="7"/>
       <c r="AP54" s="7"/>
       <c r="AQ54" s="7"/>
+      <c r="AR54" s="7"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -4670,6 +4728,7 @@
       <c r="AO55" s="7"/>
       <c r="AP55" s="7"/>
       <c r="AQ55" s="7"/>
+      <c r="AR55" s="7"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -4750,6 +4809,7 @@
       <c r="AO56" s="7"/>
       <c r="AP56" s="7"/>
       <c r="AQ56" s="7"/>
+      <c r="AR56" s="7"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -4839,6 +4899,7 @@
       <c r="AO57" s="7"/>
       <c r="AP57" s="7"/>
       <c r="AQ57" s="7"/>
+      <c r="AR57" s="7"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -4936,6 +4997,7 @@
       <c r="AO58" s="7"/>
       <c r="AP58" s="7"/>
       <c r="AQ58" s="7"/>
+      <c r="AR58" s="7"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -5000,6 +5062,7 @@
       <c r="AO59" s="7"/>
       <c r="AP59" s="7"/>
       <c r="AQ59" s="7"/>
+      <c r="AR59" s="7"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -5064,6 +5127,7 @@
       <c r="AO60" s="7"/>
       <c r="AP60" s="7"/>
       <c r="AQ60" s="7"/>
+      <c r="AR60" s="7"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -5140,6 +5204,7 @@
       <c r="AO61" s="7"/>
       <c r="AP61" s="7"/>
       <c r="AQ61" s="7"/>
+      <c r="AR61" s="7"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -5224,6 +5289,7 @@
       <c r="AO62" s="7"/>
       <c r="AP62" s="7"/>
       <c r="AQ62" s="7"/>
+      <c r="AR62" s="7"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -5300,6 +5366,7 @@
       <c r="AO63" s="7"/>
       <c r="AP63" s="7"/>
       <c r="AQ63" s="7"/>
+      <c r="AR63" s="7"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -5364,6 +5431,7 @@
       <c r="AO64" s="7"/>
       <c r="AP64" s="7"/>
       <c r="AQ64" s="7"/>
+      <c r="AR64" s="7"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -5433,6 +5501,7 @@
       <c r="AO65" s="7"/>
       <c r="AP65" s="7"/>
       <c r="AQ65" s="7"/>
+      <c r="AR65" s="7"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
@@ -5509,6 +5578,7 @@
       <c r="AO66" s="7"/>
       <c r="AP66" s="7"/>
       <c r="AQ66" s="7"/>
+      <c r="AR66" s="7"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -5573,6 +5643,7 @@
       <c r="AO67" s="7"/>
       <c r="AP67" s="7"/>
       <c r="AQ67" s="7"/>
+      <c r="AR67" s="7"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
@@ -5641,6 +5712,7 @@
       <c r="AO68" s="7"/>
       <c r="AP68" s="7"/>
       <c r="AQ68" s="7"/>
+      <c r="AR68" s="7"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -5741,6 +5813,7 @@
       <c r="AO69" s="7"/>
       <c r="AP69" s="7"/>
       <c r="AQ69" s="7"/>
+      <c r="AR69" s="7"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
@@ -5805,6 +5878,7 @@
       <c r="AO70" s="7"/>
       <c r="AP70" s="7"/>
       <c r="AQ70" s="7"/>
+      <c r="AR70" s="7"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -5874,6 +5948,7 @@
       <c r="AO71" s="7"/>
       <c r="AP71" s="7"/>
       <c r="AQ71" s="7"/>
+      <c r="AR71" s="7"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
@@ -5954,6 +6029,7 @@
       <c r="AO72" s="7"/>
       <c r="AP72" s="7"/>
       <c r="AQ72" s="7"/>
+      <c r="AR72" s="7"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
@@ -6023,6 +6099,7 @@
       <c r="AO73" s="7"/>
       <c r="AP73" s="7"/>
       <c r="AQ73" s="7"/>
+      <c r="AR73" s="7"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -6087,6 +6164,7 @@
       <c r="AO74" s="7"/>
       <c r="AP74" s="7"/>
       <c r="AQ74" s="7"/>
+      <c r="AR74" s="7"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -6151,6 +6229,7 @@
       <c r="AO75" s="7"/>
       <c r="AP75" s="7"/>
       <c r="AQ75" s="7"/>
+      <c r="AR75" s="7"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -6215,6 +6294,7 @@
       <c r="AO76" s="7"/>
       <c r="AP76" s="7"/>
       <c r="AQ76" s="7"/>
+      <c r="AR76" s="7"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -6283,6 +6363,7 @@
       <c r="AO77" s="7"/>
       <c r="AP77" s="7"/>
       <c r="AQ77" s="7"/>
+      <c r="AR77" s="7"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
@@ -6347,6 +6428,7 @@
       <c r="AO78" s="7"/>
       <c r="AP78" s="7"/>
       <c r="AQ78" s="7"/>
+      <c r="AR78" s="7"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -6416,6 +6498,7 @@
       <c r="AO79" s="7"/>
       <c r="AP79" s="7"/>
       <c r="AQ79" s="7"/>
+      <c r="AR79" s="7"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
@@ -6496,6 +6579,7 @@
       <c r="AO80" s="7"/>
       <c r="AP80" s="7"/>
       <c r="AQ80" s="7"/>
+      <c r="AR80" s="7"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
@@ -6564,6 +6648,7 @@
       <c r="AO81" s="7"/>
       <c r="AP81" s="7"/>
       <c r="AQ81" s="7"/>
+      <c r="AR81" s="7"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
@@ -6628,6 +6713,7 @@
       <c r="AO82" s="7"/>
       <c r="AP82" s="7"/>
       <c r="AQ82" s="7"/>
+      <c r="AR82" s="7"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
@@ -6697,6 +6783,7 @@
       <c r="AO83" s="7"/>
       <c r="AP83" s="7"/>
       <c r="AQ83" s="7"/>
+      <c r="AR83" s="7"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
@@ -6761,6 +6848,7 @@
       <c r="AO84" s="7"/>
       <c r="AP84" s="7"/>
       <c r="AQ84" s="7"/>
+      <c r="AR84" s="7"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
@@ -6825,6 +6913,7 @@
       <c r="AO85" s="7"/>
       <c r="AP85" s="7"/>
       <c r="AQ85" s="7"/>
+      <c r="AR85" s="7"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
@@ -6894,6 +6983,7 @@
       <c r="AO86" s="7"/>
       <c r="AP86" s="7"/>
       <c r="AQ86" s="7"/>
+      <c r="AR86" s="7"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
@@ -6958,6 +7048,7 @@
       <c r="AO87" s="7"/>
       <c r="AP87" s="7"/>
       <c r="AQ87" s="7"/>
+      <c r="AR87" s="7"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
@@ -7022,6 +7113,7 @@
       <c r="AO88" s="7"/>
       <c r="AP88" s="7"/>
       <c r="AQ88" s="7"/>
+      <c r="AR88" s="7"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
@@ -7086,6 +7178,7 @@
       <c r="AO89" s="7"/>
       <c r="AP89" s="7"/>
       <c r="AQ89" s="7"/>
+      <c r="AR89" s="7"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
@@ -7179,6 +7272,7 @@
       <c r="AO90" s="7"/>
       <c r="AP90" s="7"/>
       <c r="AQ90" s="7"/>
+      <c r="AR90" s="7"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
@@ -7243,6 +7337,7 @@
       <c r="AO91" s="7"/>
       <c r="AP91" s="7"/>
       <c r="AQ91" s="7"/>
+      <c r="AR91" s="7"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
@@ -7343,6 +7438,7 @@
       <c r="AO92" s="7"/>
       <c r="AP92" s="7"/>
       <c r="AQ92" s="7"/>
+      <c r="AR92" s="7"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
@@ -7448,6 +7544,7 @@
       <c r="AO93" s="7"/>
       <c r="AP93" s="7"/>
       <c r="AQ93" s="7"/>
+      <c r="AR93" s="7"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
@@ -7517,6 +7614,7 @@
       <c r="AO94" s="7"/>
       <c r="AP94" s="7"/>
       <c r="AQ94" s="7"/>
+      <c r="AR94" s="7"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
@@ -7586,6 +7684,7 @@
       <c r="AO95" s="7"/>
       <c r="AP95" s="7"/>
       <c r="AQ95" s="7"/>
+      <c r="AR95" s="7"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
@@ -7674,6 +7773,7 @@
       <c r="AO96" s="7"/>
       <c r="AP96" s="7"/>
       <c r="AQ96" s="7"/>
+      <c r="AR96" s="7"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="inlineStr">
@@ -7738,6 +7838,7 @@
       <c r="AO97" s="7"/>
       <c r="AP97" s="7"/>
       <c r="AQ97" s="7"/>
+      <c r="AR97" s="7"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
@@ -7802,6 +7903,7 @@
       <c r="AO98" s="7"/>
       <c r="AP98" s="7"/>
       <c r="AQ98" s="7"/>
+      <c r="AR98" s="7"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
@@ -7866,6 +7968,7 @@
       <c r="AO99" s="7"/>
       <c r="AP99" s="7"/>
       <c r="AQ99" s="7"/>
+      <c r="AR99" s="7"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
@@ -7939,6 +8042,7 @@
       <c r="AO100" s="7"/>
       <c r="AP100" s="7"/>
       <c r="AQ100" s="7"/>
+      <c r="AR100" s="7"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
@@ -8003,6 +8107,7 @@
       <c r="AO101" s="7"/>
       <c r="AP101" s="7"/>
       <c r="AQ101" s="7"/>
+      <c r="AR101" s="7"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
@@ -8067,6 +8172,7 @@
       <c r="AO102" s="7"/>
       <c r="AP102" s="7"/>
       <c r="AQ102" s="7"/>
+      <c r="AR102" s="7"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="inlineStr">
@@ -8131,6 +8237,7 @@
       <c r="AO103" s="7"/>
       <c r="AP103" s="7"/>
       <c r="AQ103" s="7"/>
+      <c r="AR103" s="7"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="inlineStr">
@@ -8200,6 +8307,7 @@
       <c r="AO104" s="7"/>
       <c r="AP104" s="7"/>
       <c r="AQ104" s="7"/>
+      <c r="AR104" s="7"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
@@ -8264,6 +8372,7 @@
       <c r="AO105" s="7"/>
       <c r="AP105" s="7"/>
       <c r="AQ105" s="7"/>
+      <c r="AR105" s="7"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
@@ -8328,6 +8437,7 @@
       <c r="AO106" s="7"/>
       <c r="AP106" s="7"/>
       <c r="AQ106" s="7"/>
+      <c r="AR106" s="7"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
@@ -8392,6 +8502,7 @@
       <c r="AO107" s="7"/>
       <c r="AP107" s="7"/>
       <c r="AQ107" s="7"/>
+      <c r="AR107" s="7"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
@@ -8460,6 +8571,7 @@
       <c r="AO108" s="7"/>
       <c r="AP108" s="7"/>
       <c r="AQ108" s="7"/>
+      <c r="AR108" s="7"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="inlineStr">
@@ -8533,6 +8645,7 @@
       <c r="AO109" s="7"/>
       <c r="AP109" s="7"/>
       <c r="AQ109" s="7"/>
+      <c r="AR109" s="7"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
@@ -8614,6 +8727,7 @@
       <c r="AO110" s="7"/>
       <c r="AP110" s="7"/>
       <c r="AQ110" s="7"/>
+      <c r="AR110" s="7"/>
     </row>
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
@@ -8698,6 +8812,7 @@
       <c r="AO111" s="7"/>
       <c r="AP111" s="7"/>
       <c r="AQ111" s="7"/>
+      <c r="AR111" s="7"/>
     </row>
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
@@ -8779,6 +8894,7 @@
       <c r="AO112" s="7"/>
       <c r="AP112" s="7"/>
       <c r="AQ112" s="7"/>
+      <c r="AR112" s="7"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
@@ -8852,6 +8968,7 @@
       <c r="AO113" s="7"/>
       <c r="AP113" s="7"/>
       <c r="AQ113" s="7"/>
+      <c r="AR113" s="7"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="inlineStr">
@@ -8941,6 +9058,7 @@
       <c r="AO114" s="7"/>
       <c r="AP114" s="7"/>
       <c r="AQ114" s="7"/>
+      <c r="AR114" s="7"/>
     </row>
     <row r="115">
       <c r="A115" s="7" t="inlineStr">
@@ -9022,6 +9140,7 @@
       <c r="AO115" s="7"/>
       <c r="AP115" s="7"/>
       <c r="AQ115" s="7"/>
+      <c r="AR115" s="7"/>
     </row>
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
@@ -9111,6 +9230,7 @@
       <c r="AO116" s="7"/>
       <c r="AP116" s="7"/>
       <c r="AQ116" s="7"/>
+      <c r="AR116" s="7"/>
     </row>
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
@@ -9196,6 +9316,7 @@
       <c r="AO117" s="7"/>
       <c r="AP117" s="7"/>
       <c r="AQ117" s="7"/>
+      <c r="AR117" s="7"/>
     </row>
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
@@ -9281,6 +9402,7 @@
       <c r="AO118" s="7"/>
       <c r="AP118" s="7"/>
       <c r="AQ118" s="7"/>
+      <c r="AR118" s="7"/>
     </row>
     <row r="119">
       <c r="A119" s="7" t="inlineStr">
@@ -9362,6 +9484,7 @@
       <c r="AO119" s="7"/>
       <c r="AP119" s="7"/>
       <c r="AQ119" s="7"/>
+      <c r="AR119" s="7"/>
     </row>
     <row r="120">
       <c r="A120" s="7" t="inlineStr">
@@ -9435,6 +9558,7 @@
       <c r="AO120" s="7"/>
       <c r="AP120" s="7"/>
       <c r="AQ120" s="7"/>
+      <c r="AR120" s="7"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="inlineStr">
@@ -9520,6 +9644,7 @@
       <c r="AO121" s="7"/>
       <c r="AP121" s="7"/>
       <c r="AQ121" s="7"/>
+      <c r="AR121" s="7"/>
     </row>
     <row r="122">
       <c r="A122" s="7" t="inlineStr">
@@ -9605,6 +9730,7 @@
       <c r="AO122" s="7"/>
       <c r="AP122" s="7"/>
       <c r="AQ122" s="7"/>
+      <c r="AR122" s="7"/>
     </row>
     <row r="123">
       <c r="A123" s="7" t="inlineStr">
@@ -9678,6 +9804,7 @@
       <c r="AO123" s="7"/>
       <c r="AP123" s="7"/>
       <c r="AQ123" s="7"/>
+      <c r="AR123" s="7"/>
     </row>
     <row r="124">
       <c r="A124" s="7" t="inlineStr">
@@ -9759,6 +9886,7 @@
       <c r="AO124" s="7"/>
       <c r="AP124" s="7"/>
       <c r="AQ124" s="7"/>
+      <c r="AR124" s="7"/>
     </row>
     <row r="125">
       <c r="A125" s="7" t="inlineStr">
@@ -9832,6 +9960,7 @@
       <c r="AO125" s="7"/>
       <c r="AP125" s="7"/>
       <c r="AQ125" s="7"/>
+      <c r="AR125" s="7"/>
     </row>
     <row r="126">
       <c r="A126" s="7" t="inlineStr">
@@ -9905,6 +10034,7 @@
       <c r="AO126" s="7"/>
       <c r="AP126" s="7"/>
       <c r="AQ126" s="7"/>
+      <c r="AR126" s="7"/>
     </row>
     <row r="127">
       <c r="A127" s="7" t="inlineStr">
@@ -9982,6 +10112,7 @@
       <c r="AO127" s="7"/>
       <c r="AP127" s="7"/>
       <c r="AQ127" s="7"/>
+      <c r="AR127" s="7"/>
     </row>
     <row r="128">
       <c r="A128" s="7" t="inlineStr">
@@ -10059,6 +10190,7 @@
       <c r="AO128" s="7"/>
       <c r="AP128" s="7"/>
       <c r="AQ128" s="7"/>
+      <c r="AR128" s="7"/>
     </row>
     <row r="129">
       <c r="A129" s="7" t="inlineStr">
@@ -10136,6 +10268,7 @@
       <c r="AO129" s="7"/>
       <c r="AP129" s="7"/>
       <c r="AQ129" s="7"/>
+      <c r="AR129" s="7"/>
     </row>
     <row r="130">
       <c r="A130" s="7" t="inlineStr">
@@ -10209,6 +10342,7 @@
       <c r="AO130" s="7"/>
       <c r="AP130" s="7"/>
       <c r="AQ130" s="7"/>
+      <c r="AR130" s="7"/>
     </row>
     <row r="131">
       <c r="A131" s="7" t="inlineStr">
@@ -10290,6 +10424,7 @@
       <c r="AO131" s="7"/>
       <c r="AP131" s="7"/>
       <c r="AQ131" s="7"/>
+      <c r="AR131" s="7"/>
     </row>
     <row r="132">
       <c r="A132" s="7" t="inlineStr">
@@ -10375,6 +10510,7 @@
       <c r="AO132" s="7"/>
       <c r="AP132" s="7"/>
       <c r="AQ132" s="7"/>
+      <c r="AR132" s="7"/>
     </row>
     <row r="133">
       <c r="A133" s="7" t="inlineStr">
@@ -10460,6 +10596,7 @@
       <c r="AO133" s="7"/>
       <c r="AP133" s="7"/>
       <c r="AQ133" s="7"/>
+      <c r="AR133" s="7"/>
     </row>
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
@@ -10541,6 +10678,7 @@
       <c r="AO134" s="7"/>
       <c r="AP134" s="7"/>
       <c r="AQ134" s="7"/>
+      <c r="AR134" s="7"/>
     </row>
     <row r="135">
       <c r="A135" s="7" t="inlineStr">
@@ -10622,6 +10760,7 @@
       <c r="AO135" s="7"/>
       <c r="AP135" s="7"/>
       <c r="AQ135" s="7"/>
+      <c r="AR135" s="7"/>
     </row>
     <row r="136">
       <c r="A136" s="7" t="inlineStr">
@@ -10703,6 +10842,7 @@
       <c r="AO136" s="7"/>
       <c r="AP136" s="7"/>
       <c r="AQ136" s="7"/>
+      <c r="AR136" s="7"/>
     </row>
     <row r="137">
       <c r="A137" s="7" t="inlineStr">
@@ -10780,6 +10920,7 @@
       <c r="AO137" s="7"/>
       <c r="AP137" s="7"/>
       <c r="AQ137" s="7"/>
+      <c r="AR137" s="7"/>
     </row>
     <row r="138">
       <c r="A138" s="7" t="inlineStr">
@@ -10857,6 +10998,7 @@
       <c r="AO138" s="7"/>
       <c r="AP138" s="7"/>
       <c r="AQ138" s="7"/>
+      <c r="AR138" s="7"/>
     </row>
     <row r="139">
       <c r="A139" s="7" t="inlineStr">
@@ -10934,6 +11076,7 @@
       <c r="AO139" s="7"/>
       <c r="AP139" s="7"/>
       <c r="AQ139" s="7"/>
+      <c r="AR139" s="7"/>
     </row>
     <row r="140">
       <c r="A140" s="7" t="inlineStr">
@@ -11007,6 +11150,7 @@
       <c r="AO140" s="7"/>
       <c r="AP140" s="7"/>
       <c r="AQ140" s="7"/>
+      <c r="AR140" s="7"/>
     </row>
     <row r="141">
       <c r="A141" s="7" t="inlineStr">
@@ -11092,6 +11236,7 @@
       <c r="AO141" s="7"/>
       <c r="AP141" s="7"/>
       <c r="AQ141" s="7"/>
+      <c r="AR141" s="7"/>
     </row>
     <row r="142">
       <c r="A142" s="7" t="inlineStr">
@@ -11165,6 +11310,7 @@
       <c r="AO142" s="7"/>
       <c r="AP142" s="7"/>
       <c r="AQ142" s="7"/>
+      <c r="AR142" s="7"/>
     </row>
     <row r="143">
       <c r="A143" s="7" t="inlineStr">
@@ -11238,6 +11384,7 @@
       <c r="AO143" s="7"/>
       <c r="AP143" s="7"/>
       <c r="AQ143" s="7"/>
+      <c r="AR143" s="7"/>
     </row>
     <row r="144">
       <c r="A144" s="7" t="inlineStr">
@@ -11311,6 +11458,7 @@
       <c r="AO144" s="7"/>
       <c r="AP144" s="7"/>
       <c r="AQ144" s="7"/>
+      <c r="AR144" s="7"/>
     </row>
     <row r="145">
       <c r="A145" s="7" t="inlineStr">
@@ -11400,6 +11548,7 @@
       <c r="AO145" s="7"/>
       <c r="AP145" s="7"/>
       <c r="AQ145" s="7"/>
+      <c r="AR145" s="7"/>
     </row>
     <row r="146">
       <c r="A146" s="7" t="inlineStr">
@@ -11477,6 +11626,7 @@
       <c r="AO146" s="7"/>
       <c r="AP146" s="7"/>
       <c r="AQ146" s="7"/>
+      <c r="AR146" s="7"/>
     </row>
     <row r="147">
       <c r="A147" s="7" t="inlineStr">
@@ -11566,6 +11716,7 @@
       <c r="AO147" s="7"/>
       <c r="AP147" s="7"/>
       <c r="AQ147" s="7"/>
+      <c r="AR147" s="7"/>
     </row>
     <row r="148">
       <c r="A148" s="7" t="inlineStr">
@@ -11639,6 +11790,7 @@
       <c r="AO148" s="7"/>
       <c r="AP148" s="7"/>
       <c r="AQ148" s="7"/>
+      <c r="AR148" s="7"/>
     </row>
     <row r="149">
       <c r="A149" s="7" t="inlineStr">
@@ -11720,6 +11872,7 @@
       <c r="AO149" s="7"/>
       <c r="AP149" s="7"/>
       <c r="AQ149" s="7"/>
+      <c r="AR149" s="7"/>
     </row>
     <row r="150">
       <c r="A150" s="7" t="inlineStr">
@@ -11805,6 +11958,7 @@
       <c r="AO150" s="7"/>
       <c r="AP150" s="7"/>
       <c r="AQ150" s="7"/>
+      <c r="AR150" s="7"/>
     </row>
     <row r="151">
       <c r="A151" s="7" t="inlineStr">
@@ -11882,6 +12036,7 @@
       <c r="AO151" s="7"/>
       <c r="AP151" s="7"/>
       <c r="AQ151" s="7"/>
+      <c r="AR151" s="7"/>
     </row>
     <row r="152">
       <c r="A152" s="7" t="inlineStr">
@@ -11963,6 +12118,7 @@
       <c r="AO152" s="7"/>
       <c r="AP152" s="7"/>
       <c r="AQ152" s="7"/>
+      <c r="AR152" s="7"/>
     </row>
     <row r="153">
       <c r="A153" s="7" t="inlineStr">
@@ -12048,6 +12204,7 @@
       <c r="AO153" s="7"/>
       <c r="AP153" s="7"/>
       <c r="AQ153" s="7"/>
+      <c r="AR153" s="7"/>
     </row>
     <row r="154">
       <c r="A154" s="7" t="inlineStr">
@@ -12117,6 +12274,7 @@
       <c r="AO154" s="7"/>
       <c r="AP154" s="7"/>
       <c r="AQ154" s="7"/>
+      <c r="AR154" s="7"/>
     </row>
     <row r="155">
       <c r="A155" s="7" t="inlineStr">
@@ -12190,6 +12348,7 @@
       <c r="AO155" s="7"/>
       <c r="AP155" s="7"/>
       <c r="AQ155" s="7"/>
+      <c r="AR155" s="7"/>
     </row>
     <row r="156">
       <c r="A156" s="7" t="inlineStr">
@@ -12267,6 +12426,7 @@
       <c r="AO156" s="7"/>
       <c r="AP156" s="7"/>
       <c r="AQ156" s="7"/>
+      <c r="AR156" s="7"/>
     </row>
     <row r="157">
       <c r="A157" s="7" t="inlineStr">
@@ -12340,6 +12500,7 @@
       <c r="AO157" s="7"/>
       <c r="AP157" s="7"/>
       <c r="AQ157" s="7"/>
+      <c r="AR157" s="7"/>
     </row>
     <row r="158">
       <c r="A158" s="7" t="inlineStr">
@@ -12413,6 +12574,7 @@
       <c r="AO158" s="7"/>
       <c r="AP158" s="7"/>
       <c r="AQ158" s="7"/>
+      <c r="AR158" s="7"/>
     </row>
     <row r="159">
       <c r="A159" s="7" t="inlineStr">
@@ -12486,6 +12648,7 @@
       <c r="AO159" s="7"/>
       <c r="AP159" s="7"/>
       <c r="AQ159" s="7"/>
+      <c r="AR159" s="7"/>
     </row>
     <row r="160">
       <c r="A160" s="7" t="inlineStr">
@@ -12559,6 +12722,7 @@
       <c r="AO160" s="7"/>
       <c r="AP160" s="7"/>
       <c r="AQ160" s="7"/>
+      <c r="AR160" s="7"/>
     </row>
     <row r="161">
       <c r="A161" s="7" t="inlineStr">
@@ -12636,6 +12800,7 @@
       <c r="AO161" s="7"/>
       <c r="AP161" s="7"/>
       <c r="AQ161" s="7"/>
+      <c r="AR161" s="7"/>
     </row>
     <row r="162">
       <c r="A162" s="7" t="inlineStr">
@@ -12709,6 +12874,7 @@
       <c r="AO162" s="7"/>
       <c r="AP162" s="7"/>
       <c r="AQ162" s="7"/>
+      <c r="AR162" s="7"/>
     </row>
     <row r="163">
       <c r="A163" s="7" t="inlineStr">
@@ -12782,6 +12948,7 @@
       <c r="AO163" s="7"/>
       <c r="AP163" s="7"/>
       <c r="AQ163" s="7"/>
+      <c r="AR163" s="7"/>
     </row>
     <row r="164">
       <c r="A164" s="7" t="inlineStr">
@@ -12855,6 +13022,7 @@
       <c r="AO164" s="7"/>
       <c r="AP164" s="7"/>
       <c r="AQ164" s="7"/>
+      <c r="AR164" s="7"/>
     </row>
     <row r="165">
       <c r="A165" s="7" t="inlineStr">
@@ -12928,6 +13096,7 @@
       <c r="AO165" s="7"/>
       <c r="AP165" s="7"/>
       <c r="AQ165" s="7"/>
+      <c r="AR165" s="7"/>
     </row>
     <row r="166">
       <c r="A166" s="7" t="inlineStr">
@@ -13009,6 +13178,7 @@
       <c r="AO166" s="7"/>
       <c r="AP166" s="7"/>
       <c r="AQ166" s="7"/>
+      <c r="AR166" s="7"/>
     </row>
     <row r="167">
       <c r="A167" s="7" t="inlineStr">
@@ -13086,6 +13256,7 @@
       <c r="AO167" s="7"/>
       <c r="AP167" s="7"/>
       <c r="AQ167" s="7"/>
+      <c r="AR167" s="7"/>
     </row>
     <row r="168">
       <c r="A168" s="7" t="inlineStr">
@@ -13159,6 +13330,7 @@
       <c r="AO168" s="7"/>
       <c r="AP168" s="7"/>
       <c r="AQ168" s="7"/>
+      <c r="AR168" s="7"/>
     </row>
     <row r="169">
       <c r="A169" s="7" t="inlineStr">
@@ -13232,6 +13404,7 @@
       <c r="AO169" s="7"/>
       <c r="AP169" s="7"/>
       <c r="AQ169" s="7"/>
+      <c r="AR169" s="7"/>
     </row>
     <row r="170">
       <c r="A170" s="7" t="inlineStr">
@@ -13309,6 +13482,7 @@
       <c r="AO170" s="7"/>
       <c r="AP170" s="7"/>
       <c r="AQ170" s="7"/>
+      <c r="AR170" s="7"/>
     </row>
     <row r="171">
       <c r="A171" s="7" t="inlineStr">
@@ -13378,6 +13552,7 @@
       <c r="AO171" s="7"/>
       <c r="AP171" s="7"/>
       <c r="AQ171" s="7"/>
+      <c r="AR171" s="7"/>
     </row>
     <row r="172">
       <c r="A172" s="7" t="inlineStr">
@@ -13447,6 +13622,7 @@
       <c r="AO172" s="7"/>
       <c r="AP172" s="7"/>
       <c r="AQ172" s="7"/>
+      <c r="AR172" s="7"/>
     </row>
     <row r="173">
       <c r="A173" s="7" t="inlineStr">
@@ -13524,6 +13700,7 @@
       <c r="AO173" s="7"/>
       <c r="AP173" s="7"/>
       <c r="AQ173" s="7"/>
+      <c r="AR173" s="7"/>
     </row>
     <row r="174">
       <c r="A174" s="7" t="inlineStr">
@@ -13597,6 +13774,7 @@
       <c r="AO174" s="7"/>
       <c r="AP174" s="7"/>
       <c r="AQ174" s="7"/>
+      <c r="AR174" s="7"/>
     </row>
     <row r="175">
       <c r="A175" s="7" t="inlineStr">
@@ -13674,6 +13852,7 @@
       <c r="AO175" s="7"/>
       <c r="AP175" s="7"/>
       <c r="AQ175" s="7"/>
+      <c r="AR175" s="7"/>
     </row>
     <row r="176">
       <c r="A176" s="7" t="inlineStr">
@@ -13747,6 +13926,7 @@
       <c r="AO176" s="7"/>
       <c r="AP176" s="7"/>
       <c r="AQ176" s="7"/>
+      <c r="AR176" s="7"/>
     </row>
     <row r="177">
       <c r="A177" s="7" t="inlineStr">
@@ -13820,6 +14000,7 @@
       <c r="AO177" s="7"/>
       <c r="AP177" s="7"/>
       <c r="AQ177" s="7"/>
+      <c r="AR177" s="7"/>
     </row>
     <row r="178">
       <c r="A178" s="7" t="inlineStr">
@@ -13893,6 +14074,7 @@
       <c r="AO178" s="7"/>
       <c r="AP178" s="7"/>
       <c r="AQ178" s="7"/>
+      <c r="AR178" s="7"/>
     </row>
     <row r="179">
       <c r="A179" s="7" t="inlineStr">
@@ -13966,6 +14148,7 @@
       <c r="AO179" s="7"/>
       <c r="AP179" s="7"/>
       <c r="AQ179" s="7"/>
+      <c r="AR179" s="7"/>
     </row>
     <row r="180">
       <c r="A180" s="7" t="inlineStr">
@@ -14039,6 +14222,7 @@
       <c r="AO180" s="7"/>
       <c r="AP180" s="7"/>
       <c r="AQ180" s="7"/>
+      <c r="AR180" s="7"/>
     </row>
     <row r="181">
       <c r="A181" s="7" t="inlineStr">
@@ -14112,6 +14296,7 @@
       <c r="AO181" s="7"/>
       <c r="AP181" s="7"/>
       <c r="AQ181" s="7"/>
+      <c r="AR181" s="7"/>
     </row>
     <row r="182">
       <c r="A182" s="7" t="inlineStr">
@@ -14185,6 +14370,7 @@
       <c r="AO182" s="7"/>
       <c r="AP182" s="7"/>
       <c r="AQ182" s="7"/>
+      <c r="AR182" s="7"/>
     </row>
     <row r="183">
       <c r="A183" s="7" t="inlineStr">
@@ -14258,6 +14444,7 @@
       <c r="AO183" s="7"/>
       <c r="AP183" s="7"/>
       <c r="AQ183" s="7"/>
+      <c r="AR183" s="7"/>
     </row>
     <row r="184">
       <c r="A184" s="7" t="inlineStr">
@@ -14327,6 +14514,7 @@
       <c r="AO184" s="7"/>
       <c r="AP184" s="7"/>
       <c r="AQ184" s="7"/>
+      <c r="AR184" s="7"/>
     </row>
     <row r="185">
       <c r="A185" s="7" t="inlineStr">
@@ -14400,6 +14588,7 @@
       <c r="AO185" s="7"/>
       <c r="AP185" s="7"/>
       <c r="AQ185" s="7"/>
+      <c r="AR185" s="7"/>
     </row>
     <row r="186">
       <c r="A186" s="7" t="inlineStr">
@@ -14473,6 +14662,7 @@
       <c r="AO186" s="7"/>
       <c r="AP186" s="7"/>
       <c r="AQ186" s="7"/>
+      <c r="AR186" s="7"/>
     </row>
     <row r="187">
       <c r="A187" s="7" t="inlineStr">
@@ -14550,6 +14740,7 @@
       <c r="AO187" s="7"/>
       <c r="AP187" s="7"/>
       <c r="AQ187" s="7"/>
+      <c r="AR187" s="7"/>
     </row>
     <row r="188">
       <c r="A188" s="7" t="inlineStr">
@@ -14627,6 +14818,7 @@
       <c r="AO188" s="7"/>
       <c r="AP188" s="7"/>
       <c r="AQ188" s="7"/>
+      <c r="AR188" s="7"/>
     </row>
     <row r="189">
       <c r="A189" s="7" t="inlineStr">
@@ -14704,6 +14896,7 @@
       <c r="AO189" s="7"/>
       <c r="AP189" s="7"/>
       <c r="AQ189" s="7"/>
+      <c r="AR189" s="7"/>
     </row>
     <row r="190">
       <c r="A190" s="7" t="inlineStr">
@@ -14781,6 +14974,7 @@
       <c r="AO190" s="7"/>
       <c r="AP190" s="7"/>
       <c r="AQ190" s="7"/>
+      <c r="AR190" s="7"/>
     </row>
     <row r="191">
       <c r="A191" s="7" t="inlineStr">
@@ -14858,6 +15052,7 @@
       <c r="AO191" s="7"/>
       <c r="AP191" s="7"/>
       <c r="AQ191" s="7"/>
+      <c r="AR191" s="7"/>
     </row>
     <row r="192">
       <c r="A192" s="7" t="inlineStr">
@@ -14935,6 +15130,7 @@
       <c r="AO192" s="7"/>
       <c r="AP192" s="7"/>
       <c r="AQ192" s="7"/>
+      <c r="AR192" s="7"/>
     </row>
     <row r="193">
       <c r="A193" s="7" t="inlineStr">
@@ -15016,6 +15212,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AR193" s="7"/>
     </row>
     <row r="194">
       <c r="A194" s="7" t="inlineStr">
@@ -15097,6 +15294,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AR194" s="7"/>
     </row>
     <row r="195">
       <c r="A195" s="7" t="inlineStr">
@@ -15178,6 +15376,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AR195" s="7"/>
     </row>
     <row r="196">
       <c r="A196" s="7" t="inlineStr">
@@ -15251,6 +15450,7 @@
       <c r="AO196" s="7"/>
       <c r="AP196" s="7"/>
       <c r="AQ196" s="7"/>
+      <c r="AR196" s="7"/>
     </row>
     <row r="197">
       <c r="A197" s="7" t="inlineStr">
@@ -15332,6 +15532,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AR197" s="7"/>
     </row>
     <row r="198">
       <c r="A198" s="7" t="inlineStr">
@@ -15405,6 +15606,7 @@
       <c r="AO198" s="7"/>
       <c r="AP198" s="7"/>
       <c r="AQ198" s="7"/>
+      <c r="AR198" s="7"/>
     </row>
     <row r="199">
       <c r="A199" s="7" t="inlineStr">
@@ -15486,6 +15688,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AR199" s="7"/>
     </row>
     <row r="200">
       <c r="A200" s="7" t="inlineStr">
@@ -15567,6 +15770,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AR200" s="7"/>
     </row>
     <row r="201">
       <c r="A201" s="7" t="inlineStr">
@@ -15640,6 +15844,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AR201" s="7"/>
     </row>
     <row r="202">
       <c r="A202" s="7" t="inlineStr">
@@ -15721,6 +15926,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AR202" s="7"/>
     </row>
     <row r="203">
       <c r="A203" s="7" t="inlineStr">
@@ -15802,6 +16008,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AR203" s="7"/>
     </row>
     <row r="204">
       <c r="A204" s="7" t="inlineStr">
@@ -15831,7 +16038,7 @@
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t xml:space="preserve">#198 · 4a6f983 사용자 육안 = 재료 0(Fail) → e86eb9a 에서 고침 · AQ — 처음부터 → S3 점프: 재료 63/50 · 고철 300/300 · 막 · 정지</t>
+          <t xml:space="preserve">#198 · 4a6f983 사용자 육안 = 재료 0(Fail) → e86eb9a 에서 고침 · AQ — 처음부터 → S3 점프: 재료 63/50 · 고철 300/300 · 막 · 정지 · AR — 처음부터 → S3 점프: 재료 63/50 · 고철 300/300 · 막 동안 적 0</t>
         </is>
       </c>
       <c r="G204" s="7"/>
@@ -15883,6 +16090,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AR204" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="7" t="inlineStr">
@@ -15968,6 +16180,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AR205" s="7"/>
     </row>
     <row r="206">
       <c r="A206" s="7" t="inlineStr">
@@ -16049,6 +16262,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AR206" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="7" t="inlineStr">
@@ -16126,6 +16344,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AR207" s="7"/>
     </row>
     <row r="208">
       <c r="A208" s="7" t="inlineStr">
@@ -16155,7 +16374,7 @@
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t xml:space="preserve">4a6f983 사용자 육안 = 시간 초과(보스 ≈30%) · 조건 = 옛 저장(#197 전 A 판 리셋 · HUD 전투력 0) — 새 저장으로 재확인 자리 · AQ Fail — 시간 초과 · 보스 ≈40% 남음. 🗑️(정정) 「A 판이 폭발탄 1·2걸음만 된 채」는 틀림 — 바로가기 S6 점프가 #167 폭발탄 프리셋으로 A 판을 덮었다(새로고침 뒤 복합 가공소 확인). 조건 = 바로가기 S6 · A 판 폭발탄 프리셋 · A·B 강화 · 마운트 탄 0/200 · HUD 전투력 3→0 · 합체 1회</t>
+          <t xml:space="preserve">4a6f983 사용자 육안 = 시간 초과(보스 ≈30%) · 조건 = 옛 저장(#197 전 A 판 리셋 · HUD 전투력 0) — 새 저장으로 재확인 자리 · AQ Fail — 시간 초과 · 보스 ≈40% 남음. 🗑️(정정) 「A 판이 폭발탄 1·2걸음만 된 채」는 틀림 — 바로가기 S6 점프가 #167 폭발탄 프리셋으로 A 판을 덮었다(새로고침 뒤 복합 가공소 확인). 조건 = 바로가기 S6 · A 판 폭발탄 프리셋 · A·B 강화 · 마운트 탄 0/200 · HUD 전투력 3→0 · 합체 1회 · AR Pass(보이는 창) — 처음부터 → S6 → B 막 강화 → 도전(A 1/40 · B 31/40 · 게이지 100%) → 즉시 합체 → 승리 남은 00:41. AQ Fail 은 숨긴 창(배경 탭) 조건</t>
         </is>
       </c>
       <c r="G208" s="7"/>
@@ -16201,6 +16420,11 @@
       <c r="AQ208" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
+      <c r="AR208" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
         </is>
       </c>
     </row>
@@ -16284,6 +16508,11 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AR209" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="7" t="inlineStr">
@@ -16313,7 +16542,7 @@
       </c>
       <c r="F210" t="inlineStr">
         <is>
-          <t xml:space="preserve">#203 · 범위 = 사용자 「S1 S3 S6」 · 물류 계속 ⚠️ 가정 · AQ — S1 T3 · S3 강화 · S6 B 강화 셋 다 정지(리젠 고정 · 적 정지) → 해제 뒤 재개</t>
+          <t xml:space="preserve">#203 · 범위 = 사용자 「S1 S3 S6」 · 물류 계속 ⚠️ 가정 · AQ — S1 T3 · S3 강화 · S6 B 강화 셋 다 정지(리젠 고정 · 적 정지) → 해제 뒤 재개 · AR — #207 로 확장(스폰 보류까지) · CID_209 참조</t>
         </is>
       </c>
       <c r="G210" s="7"/>
@@ -16357,6 +16586,11 @@
       </c>
       <c r="AP210" s="7"/>
       <c r="AQ210" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+      <c r="AR210" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Pass</t>
         </is>
@@ -16434,6 +16668,7 @@
         </is>
       </c>
       <c r="AQ211" s="7"/>
+      <c r="AR211" s="7"/>
     </row>
     <row r="212">
       <c r="A212" s="7" t="inlineStr">
@@ -16463,7 +16698,7 @@
       </c>
       <c r="F212" t="inlineStr">
         <is>
-          <t xml:space="preserve">AQ 코드 세션 실측 — 교대마다 보드가 B 판으로 바뀌어(FollowActiveRobotTab) 안내가 사라지고, B 판 변환기 탭에 생산량 모듈이 붙어 고철 −30. Auto 끄면 A 판 고정 · 1·2걸음 정상</t>
+          <t xml:space="preserve">AQ 코드 세션 실측 — 교대마다 보드가 B 판으로 바뀌어(FollowActiveRobotTab) 안내가 사라지고, B 판 변환기 탭에 생산량 모듈이 붙어 고철 −30. Auto 끄면 A 판 고정 · 1·2걸음 정상 · AR — S6 조립 진입 = B 판 ✅ · S5 Auto 교대 고정은 못 봄(자연 S5 못 감)</t>
         </is>
       </c>
       <c r="G212" s="7"/>
@@ -16507,6 +16742,7 @@
           <t xml:space="preserve">Fail</t>
         </is>
       </c>
+      <c r="AR212" s="7"/>
     </row>
     <row r="213">
       <c r="A213" s="7" t="inlineStr">
@@ -16536,7 +16772,7 @@
       </c>
       <c r="F213" t="inlineStr">
         <is>
-          <t xml:space="preserve">AQ — 「처음부터」 → 바로가기 S5 = 막 안 섬 · 「도전」 밝음. ExplosiveTutorialRule.IsActive 가 tutorialCleared 요구(판정 요청 · 의도인지)</t>
+          <t xml:space="preserve">AQ — 「처음부터」 → 바로가기 S5 = 막 안 섬 · 「도전」 밝음. ExplosiveTutorialRule.IsActive 가 tutorialCleared 요구(판정 요청 · 의도인지) · AR N/A — 「의도」로 닫음(#209 사용자) · 점프 S5 = 폭발탄 프리셋(다섯 칸 완성) → 막 안 섬이 맞다</t>
         </is>
       </c>
       <c r="G213" s="7"/>
@@ -16580,6 +16816,11 @@
           <t xml:space="preserve">Fail</t>
         </is>
       </c>
+      <c r="AR213" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N/A</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="7" t="inlineStr">
@@ -16609,7 +16850,7 @@
       </c>
       <c r="F214" t="inlineStr">
         <is>
-          <t xml:space="preserve">AQ — 약 60초(게임) 만에 파괴 → S4 로 내려감. 마운트 탄 0~2/200 · HP 1000→299→0. 폭발탄 막 진행 중(1걸음 전후)</t>
+          <t xml:space="preserve">AQ — 약 60초(게임) 만에 파괴 → S4 로 내려감. 마운트 탄 0~2/200 · HP 1000→299→0. 폭발탄 막 진행 중(1걸음 전후) · AR 못 봄 — #207 확장(S5 막 동안 정지)로 닫힐 가능성 · 자연 S5 못 감</t>
         </is>
       </c>
       <c r="G214" s="7"/>
@@ -16653,6 +16894,7 @@
           <t xml:space="preserve">Fail</t>
         </is>
       </c>
+      <c r="AR214" s="7"/>
     </row>
     <row r="215">
       <c r="A215" s="7" t="inlineStr">
@@ -16722,6 +16964,587 @@
       <c r="AO215" s="7"/>
       <c r="AP215" s="7"/>
       <c r="AQ215" s="7"/>
+      <c r="AR215" s="7"/>
+    </row>
+    <row r="216">
+      <c r="A216" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_208</t>
+        </is>
+      </c>
+      <c r="B216" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">파밍</t>
+        </is>
+      </c>
+      <c r="C216" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">첫 스폰</t>
+        </is>
+      </c>
+      <c r="D216" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">띠 ×1.3</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">파밍 층이 새로 설 때(진입 · 파괴 뒤 밀림 · 점프 · 도전 뒤 복귀) 첫 묶음만 스폰 띠 ×1.3 바깥에서 걸어 들어오고, 그 뒤 리필은 종전 띠인가?</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#206 · 값 1.3 = 사용자 확정(표 행 없음 · 상수) · AR 못 봄(화면에서 거리 못 잼) · 시험 FarmFirstSpawnRuleTests</t>
+        </is>
+      </c>
+      <c r="G216" s="7"/>
+      <c r="H216" s="7"/>
+      <c r="I216" s="7"/>
+      <c r="J216" s="7"/>
+      <c r="K216" s="7"/>
+      <c r="L216" s="7"/>
+      <c r="M216" s="7"/>
+      <c r="N216" s="7"/>
+      <c r="O216" s="7"/>
+      <c r="P216" s="7"/>
+      <c r="Q216" s="7"/>
+      <c r="R216" s="7"/>
+      <c r="S216" s="7"/>
+      <c r="T216" s="7"/>
+      <c r="U216" s="7"/>
+      <c r="V216" s="7"/>
+      <c r="W216" s="7"/>
+      <c r="X216" s="7"/>
+      <c r="Y216" s="7"/>
+      <c r="Z216" s="7"/>
+      <c r="AA216" s="7"/>
+      <c r="AB216" s="7"/>
+      <c r="AC216" s="7"/>
+      <c r="AD216" s="7"/>
+      <c r="AE216" s="7"/>
+      <c r="AF216" s="7"/>
+      <c r="AG216" s="7"/>
+      <c r="AH216" s="7"/>
+      <c r="AI216" s="7"/>
+      <c r="AJ216" s="7"/>
+      <c r="AK216" s="7"/>
+      <c r="AL216" s="7"/>
+      <c r="AM216" s="7"/>
+      <c r="AN216" s="7"/>
+      <c r="AO216" s="7"/>
+      <c r="AP216" s="7"/>
+      <c r="AQ216" s="7"/>
+      <c r="AR216" s="7"/>
+    </row>
+    <row r="217">
+      <c r="A217" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_209</t>
+        </is>
+      </c>
+      <c r="B217" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼</t>
+        </is>
+      </c>
+      <c r="C217" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">막 중 스폰 보류</t>
+        </is>
+      </c>
+      <c r="D217" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S1 · S2 · S3 · S6</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t xml:space="preserve">파밍 튜토리얼 막(S1 T3 · S2 T4 · S3 강화 · S6 B 강화) 동안 적이 0 으로 서고 리젠 시계가 멈추며, 막이 끝나면 첫 스폰이 나오는가?</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#207 · AR 실측: S1 「맵 0/13 · 00:10」 · S2 「0/10」 → 모듈 붙이자 스폰 · 바로가기 S3 「0/17」 → 강화 뒤 스폰 · S6 「0/10」 → B 강화 뒤 「리젠 00:08」</t>
+        </is>
+      </c>
+      <c r="G217" s="7"/>
+      <c r="H217" s="7"/>
+      <c r="I217" s="7"/>
+      <c r="J217" s="7"/>
+      <c r="K217" s="7"/>
+      <c r="L217" s="7"/>
+      <c r="M217" s="7"/>
+      <c r="N217" s="7"/>
+      <c r="O217" s="7"/>
+      <c r="P217" s="7"/>
+      <c r="Q217" s="7"/>
+      <c r="R217" s="7"/>
+      <c r="S217" s="7"/>
+      <c r="T217" s="7"/>
+      <c r="U217" s="7"/>
+      <c r="V217" s="7"/>
+      <c r="W217" s="7"/>
+      <c r="X217" s="7"/>
+      <c r="Y217" s="7"/>
+      <c r="Z217" s="7"/>
+      <c r="AA217" s="7"/>
+      <c r="AB217" s="7"/>
+      <c r="AC217" s="7"/>
+      <c r="AD217" s="7"/>
+      <c r="AE217" s="7"/>
+      <c r="AF217" s="7"/>
+      <c r="AG217" s="7"/>
+      <c r="AH217" s="7"/>
+      <c r="AI217" s="7"/>
+      <c r="AJ217" s="7"/>
+      <c r="AK217" s="7"/>
+      <c r="AL217" s="7"/>
+      <c r="AM217" s="7"/>
+      <c r="AN217" s="7"/>
+      <c r="AO217" s="7"/>
+      <c r="AP217" s="7"/>
+      <c r="AQ217" s="7"/>
+      <c r="AR217" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_210</t>
+        </is>
+      </c>
+      <c r="B218" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼</t>
+        </is>
+      </c>
+      <c r="C218" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">막 중 정지(확장)</t>
+        </is>
+      </c>
+      <c r="D218" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 · S5 · 도전 S4</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 해금 막 · S5 폭발탄(알림 · 막 · 보드 걸음 ①~⑤) 동안 정지 + 스폰 보류, 도전 층 S4 합체 막 동안 정지(남은 시간 멈춤 · 합체 누르면 재개)인가?</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#207 확장(23:4x) · AR 못 봄 — 자연 진행 필요(T1 벨트 끌기가 인앱 브라우저 합성 끌기로 안 먹음) · 바로가기는 이 막들을 안 세움 · 시험 PauseRule 7갈래</t>
+        </is>
+      </c>
+      <c r="G218" s="7"/>
+      <c r="H218" s="7"/>
+      <c r="I218" s="7"/>
+      <c r="J218" s="7"/>
+      <c r="K218" s="7"/>
+      <c r="L218" s="7"/>
+      <c r="M218" s="7"/>
+      <c r="N218" s="7"/>
+      <c r="O218" s="7"/>
+      <c r="P218" s="7"/>
+      <c r="Q218" s="7"/>
+      <c r="R218" s="7"/>
+      <c r="S218" s="7"/>
+      <c r="T218" s="7"/>
+      <c r="U218" s="7"/>
+      <c r="V218" s="7"/>
+      <c r="W218" s="7"/>
+      <c r="X218" s="7"/>
+      <c r="Y218" s="7"/>
+      <c r="Z218" s="7"/>
+      <c r="AA218" s="7"/>
+      <c r="AB218" s="7"/>
+      <c r="AC218" s="7"/>
+      <c r="AD218" s="7"/>
+      <c r="AE218" s="7"/>
+      <c r="AF218" s="7"/>
+      <c r="AG218" s="7"/>
+      <c r="AH218" s="7"/>
+      <c r="AI218" s="7"/>
+      <c r="AJ218" s="7"/>
+      <c r="AK218" s="7"/>
+      <c r="AL218" s="7"/>
+      <c r="AM218" s="7"/>
+      <c r="AN218" s="7"/>
+      <c r="AO218" s="7"/>
+      <c r="AP218" s="7"/>
+      <c r="AQ218" s="7"/>
+      <c r="AR218" s="7"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_211</t>
+        </is>
+      </c>
+      <c r="B219" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C219" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 장갑 0</t>
+        </is>
+      </c>
+      <c r="D219" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">파밍 · 도전</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S3 파밍(보병 15 · 포격 2)과 도전(보병 26 · 포격 4)에 장갑이 안 나오고 강화 뒤 파밍을 버티며 도전을 60초 안에 넘는가?</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#208 · 하네스 도전 Win 43.9 / 24.9초 · 파밍 바닥 989 · AR 화면 S3 파밍 35초+ HP 1000/1000</t>
+        </is>
+      </c>
+      <c r="G219" s="7"/>
+      <c r="H219" s="7"/>
+      <c r="I219" s="7"/>
+      <c r="J219" s="7"/>
+      <c r="K219" s="7"/>
+      <c r="L219" s="7"/>
+      <c r="M219" s="7"/>
+      <c r="N219" s="7"/>
+      <c r="O219" s="7"/>
+      <c r="P219" s="7"/>
+      <c r="Q219" s="7"/>
+      <c r="R219" s="7"/>
+      <c r="S219" s="7"/>
+      <c r="T219" s="7"/>
+      <c r="U219" s="7"/>
+      <c r="V219" s="7"/>
+      <c r="W219" s="7"/>
+      <c r="X219" s="7"/>
+      <c r="Y219" s="7"/>
+      <c r="Z219" s="7"/>
+      <c r="AA219" s="7"/>
+      <c r="AB219" s="7"/>
+      <c r="AC219" s="7"/>
+      <c r="AD219" s="7"/>
+      <c r="AE219" s="7"/>
+      <c r="AF219" s="7"/>
+      <c r="AG219" s="7"/>
+      <c r="AH219" s="7"/>
+      <c r="AI219" s="7"/>
+      <c r="AJ219" s="7"/>
+      <c r="AK219" s="7"/>
+      <c r="AL219" s="7"/>
+      <c r="AM219" s="7"/>
+      <c r="AN219" s="7"/>
+      <c r="AO219" s="7"/>
+      <c r="AP219" s="7"/>
+      <c r="AQ219" s="7"/>
+      <c r="AR219" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_212</t>
+        </is>
+      </c>
+      <c r="B220" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">저장</t>
+        </is>
+      </c>
+      <c r="C220" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">옛 저장 복구</t>
+        </is>
+      </c>
+      <c r="D220" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A 운반로 칸</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#197 전 옛 저장(A 판 운반로 칸 빔 · 튜토리얼 마침)을 불러오면 그 칸이 채워져 전투력이 서는가?</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#209 · AR 못 봄(옛 손상 저장 없음) · 시험 SaveRepairRuleTests</t>
+        </is>
+      </c>
+      <c r="G220" s="7"/>
+      <c r="H220" s="7"/>
+      <c r="I220" s="7"/>
+      <c r="J220" s="7"/>
+      <c r="K220" s="7"/>
+      <c r="L220" s="7"/>
+      <c r="M220" s="7"/>
+      <c r="N220" s="7"/>
+      <c r="O220" s="7"/>
+      <c r="P220" s="7"/>
+      <c r="Q220" s="7"/>
+      <c r="R220" s="7"/>
+      <c r="S220" s="7"/>
+      <c r="T220" s="7"/>
+      <c r="U220" s="7"/>
+      <c r="V220" s="7"/>
+      <c r="W220" s="7"/>
+      <c r="X220" s="7"/>
+      <c r="Y220" s="7"/>
+      <c r="Z220" s="7"/>
+      <c r="AA220" s="7"/>
+      <c r="AB220" s="7"/>
+      <c r="AC220" s="7"/>
+      <c r="AD220" s="7"/>
+      <c r="AE220" s="7"/>
+      <c r="AF220" s="7"/>
+      <c r="AG220" s="7"/>
+      <c r="AH220" s="7"/>
+      <c r="AI220" s="7"/>
+      <c r="AJ220" s="7"/>
+      <c r="AK220" s="7"/>
+      <c r="AL220" s="7"/>
+      <c r="AM220" s="7"/>
+      <c r="AN220" s="7"/>
+      <c r="AO220" s="7"/>
+      <c r="AP220" s="7"/>
+      <c r="AQ220" s="7"/>
+      <c r="AR220" s="7"/>
+    </row>
+    <row r="221">
+      <c r="A221" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_213</t>
+        </is>
+      </c>
+      <c r="B221" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UI</t>
+        </is>
+      </c>
+      <c r="C221" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">모듈 선택</t>
+        </is>
+      </c>
+      <c r="D221" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">붙이면 풀림</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t xml:space="preserve">모듈을 고르고 노드에 붙이면 고르기가 풀리는가?(노드 #175 ⓔ 와 같게)</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#209 · AR 실측: S2 T4 붙인 뒤 안내 줄이 기본 문구로</t>
+        </is>
+      </c>
+      <c r="G221" s="7"/>
+      <c r="H221" s="7"/>
+      <c r="I221" s="7"/>
+      <c r="J221" s="7"/>
+      <c r="K221" s="7"/>
+      <c r="L221" s="7"/>
+      <c r="M221" s="7"/>
+      <c r="N221" s="7"/>
+      <c r="O221" s="7"/>
+      <c r="P221" s="7"/>
+      <c r="Q221" s="7"/>
+      <c r="R221" s="7"/>
+      <c r="S221" s="7"/>
+      <c r="T221" s="7"/>
+      <c r="U221" s="7"/>
+      <c r="V221" s="7"/>
+      <c r="W221" s="7"/>
+      <c r="X221" s="7"/>
+      <c r="Y221" s="7"/>
+      <c r="Z221" s="7"/>
+      <c r="AA221" s="7"/>
+      <c r="AB221" s="7"/>
+      <c r="AC221" s="7"/>
+      <c r="AD221" s="7"/>
+      <c r="AE221" s="7"/>
+      <c r="AF221" s="7"/>
+      <c r="AG221" s="7"/>
+      <c r="AH221" s="7"/>
+      <c r="AI221" s="7"/>
+      <c r="AJ221" s="7"/>
+      <c r="AK221" s="7"/>
+      <c r="AL221" s="7"/>
+      <c r="AM221" s="7"/>
+      <c r="AN221" s="7"/>
+      <c r="AO221" s="7"/>
+      <c r="AP221" s="7"/>
+      <c r="AQ221" s="7"/>
+      <c r="AR221" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_214</t>
+        </is>
+      </c>
+      <c r="B222" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼</t>
+        </is>
+      </c>
+      <c r="C222" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S6 B 막 시야</t>
+        </is>
+      </c>
+      <c r="D222" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B 마운트 칸</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t xml:space="preserve">처음부터 → 바로가기 S6 → 조립에 들어가면 B 판 B 마운트 칸이 화면 안에 보이는가?</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AR Fail — B 판이 열리고 안내 「로봇 B 마운트를 탭한 뒤 강화를 누르세요」는 섰으나 B 마운트 칸이 보드 위쪽 화면 밖 · 줌아웃 한계라 이동 모드로 끌어 내려야 보임. 그 뒤 탭 · 강화는 정상</t>
+        </is>
+      </c>
+      <c r="G222" s="7"/>
+      <c r="H222" s="7"/>
+      <c r="I222" s="7"/>
+      <c r="J222" s="7"/>
+      <c r="K222" s="7"/>
+      <c r="L222" s="7"/>
+      <c r="M222" s="7"/>
+      <c r="N222" s="7"/>
+      <c r="O222" s="7"/>
+      <c r="P222" s="7"/>
+      <c r="Q222" s="7"/>
+      <c r="R222" s="7"/>
+      <c r="S222" s="7"/>
+      <c r="T222" s="7"/>
+      <c r="U222" s="7"/>
+      <c r="V222" s="7"/>
+      <c r="W222" s="7"/>
+      <c r="X222" s="7"/>
+      <c r="Y222" s="7"/>
+      <c r="Z222" s="7"/>
+      <c r="AA222" s="7"/>
+      <c r="AB222" s="7"/>
+      <c r="AC222" s="7"/>
+      <c r="AD222" s="7"/>
+      <c r="AE222" s="7"/>
+      <c r="AF222" s="7"/>
+      <c r="AG222" s="7"/>
+      <c r="AH222" s="7"/>
+      <c r="AI222" s="7"/>
+      <c r="AJ222" s="7"/>
+      <c r="AK222" s="7"/>
+      <c r="AL222" s="7"/>
+      <c r="AM222" s="7"/>
+      <c r="AN222" s="7"/>
+      <c r="AO222" s="7"/>
+      <c r="AP222" s="7"/>
+      <c r="AQ222" s="7"/>
+      <c r="AR222" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_215</t>
+        </is>
+      </c>
+      <c r="B223" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UI</t>
+        </is>
+      </c>
+      <c r="C223" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">처음부터 뒤 마일스톤</t>
+        </is>
+      </c>
+      <c r="D223" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">표시</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">「처음부터」 직후 튜토리얼 마일스톤이 [ ] 끊긴 자리를 잇는다 · (0/40) 으로 다시 서는가?</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AR Fail(경미) — 처음부터 직후 [v] 로 남고 판은 빈 칸(고스트) · 새로고침하면 [ ] 로 바로 섬</t>
+        </is>
+      </c>
+      <c r="G223" s="7"/>
+      <c r="H223" s="7"/>
+      <c r="I223" s="7"/>
+      <c r="J223" s="7"/>
+      <c r="K223" s="7"/>
+      <c r="L223" s="7"/>
+      <c r="M223" s="7"/>
+      <c r="N223" s="7"/>
+      <c r="O223" s="7"/>
+      <c r="P223" s="7"/>
+      <c r="Q223" s="7"/>
+      <c r="R223" s="7"/>
+      <c r="S223" s="7"/>
+      <c r="T223" s="7"/>
+      <c r="U223" s="7"/>
+      <c r="V223" s="7"/>
+      <c r="W223" s="7"/>
+      <c r="X223" s="7"/>
+      <c r="Y223" s="7"/>
+      <c r="Z223" s="7"/>
+      <c r="AA223" s="7"/>
+      <c r="AB223" s="7"/>
+      <c r="AC223" s="7"/>
+      <c r="AD223" s="7"/>
+      <c r="AE223" s="7"/>
+      <c r="AF223" s="7"/>
+      <c r="AG223" s="7"/>
+      <c r="AH223" s="7"/>
+      <c r="AI223" s="7"/>
+      <c r="AJ223" s="7"/>
+      <c r="AK223" s="7"/>
+      <c r="AL223" s="7"/>
+      <c r="AM223" s="7"/>
+      <c r="AN223" s="7"/>
+      <c r="AO223" s="7"/>
+      <c r="AP223" s="7"/>
+      <c r="AQ223" s="7"/>
+      <c r="AR223" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="26">
@@ -16750,9 +17573,9 @@
     <mergeCell ref="B92:B99"/>
     <mergeCell ref="B100:B106"/>
     <mergeCell ref="B107:B111"/>
-    <mergeCell ref="G7:AQ7"/>
+    <mergeCell ref="G7:AR7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:AQ215">
+  <conditionalFormatting sqref="G9:AR223">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
QA AS(8b54a82 · CID_214 Pass) · 촬영 가이드 8b54a82
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -200,8 +200,9 @@
     <col min="42" max="42" width="12" customWidth="1"/>
     <col min="43" max="43" width="12" customWidth="1"/>
     <col min="44" max="44" width="12" customWidth="1"/>
-    <col min="45" max="45" width="11" customWidth="1"/>
+    <col min="45" max="45" width="12" customWidth="1"/>
     <col min="46" max="46" width="11" customWidth="1"/>
+    <col min="47" max="47" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -504,6 +505,11 @@
       <c r="AR6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">8133 7635b57 갈아엎음(23:02) · #206 첫 스폰 띠 ×1.3 · #207 튜토리얼 국면 전부 정지+스폰 보류 · #208 S3 장갑 0 · #209 복구 · 모듈 풀림 · CID_204 탭 고정 ‖ 보이는 창(인앱 브라우저 · 소리 0) 재확인 — 남은 저장 → S1 T3 · S2 T4 · S3 파밍 / 처음부터 → 바로가기 S3 · S6 길. 자연 진행 S4 해금 · S4 합체 막 · S5 폭발탄은 못 봄(T1 벨트 끌기가 인앱 브라우저에서 안 먹음). 시험 1675/1669/0/6 · 전투 12줄 = S3 두 줄만.</t>
+        </is>
+      </c>
+      <c r="AS6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8133 8b54a82 갈아엎음(23:23) · CID_214 튜토리얼 시야 이동을 조립 카메라가 선 뒤로(A·B 강화 · S5 폭발탄 같은 규칙) ‖ 보이는 창 재확인: 처음부터 → 바로가기 S6 → 조립 = B 마운트 칸 화면 안 + 안내 → 탭 → 강화 ✅ · 시험 1679/1673/0/6 · 전투 12줄 불변. 나머지 칸 = AR 그대로(이 빌드에서 안 다시 봄).</t>
         </is>
       </c>
     </row>
@@ -572,14 +578,15 @@
       <c r="AP7" s="2"/>
       <c r="AQ7" s="2"/>
       <c r="AR7" s="2"/>
-      <c r="AS7" s="2" t="inlineStr">
+      <c r="AS7" s="2"/>
+      <c r="AT7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">버전</t>
         </is>
       </c>
-      <c r="AT7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">7635b57</t>
+      <c r="AU7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8b54a82</t>
         </is>
       </c>
     </row>
@@ -794,11 +801,16 @@
       </c>
       <c r="AS8" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">8b54a82</t>
+        </is>
+      </c>
+      <c r="AT8" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">PASSrate</t>
         </is>
       </c>
-      <c r="AT8" s="7">
-        <f>COUNTIF(AR9:AR223,"Pass")</f>
+      <c r="AU8" s="7">
+        <f>COUNTIF(AS9:AS223,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -906,13 +918,14 @@
       <c r="AP9" s="7"/>
       <c r="AQ9" s="7"/>
       <c r="AR9" s="7"/>
-      <c r="AS9" s="2" t="inlineStr">
+      <c r="AS9" s="7"/>
+      <c r="AT9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FAILrate</t>
         </is>
       </c>
-      <c r="AT9" s="7">
-        <f>COUNTIF(AR9:AR223,"Fail")+COUNTIF(AR9:AR223,"Broken")</f>
+      <c r="AU9" s="7">
+        <f>COUNTIF(AS9:AS223,"Fail")+COUNTIF(AS9:AS223,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -984,13 +997,14 @@
       <c r="AP10" s="7"/>
       <c r="AQ10" s="7"/>
       <c r="AR10" s="7"/>
-      <c r="AS10" s="2" t="inlineStr">
+      <c r="AS10" s="7"/>
+      <c r="AT10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">N/A</t>
         </is>
       </c>
-      <c r="AT10" s="7">
-        <f>COUNTIF(AR9:AR223,"N/A")</f>
+      <c r="AU10" s="7">
+        <f>COUNTIF(AS9:AS223,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -1062,12 +1076,13 @@
       <c r="AP11" s="7"/>
       <c r="AQ11" s="7"/>
       <c r="AR11" s="7"/>
-      <c r="AS11" s="2" t="inlineStr">
+      <c r="AS11" s="7"/>
+      <c r="AT11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">전체 개수</t>
         </is>
       </c>
-      <c r="AT11" s="7">
+      <c r="AU11" s="7">
         <v>215</v>
       </c>
     </row>
@@ -1140,13 +1155,14 @@
       <c r="AP12" s="7"/>
       <c r="AQ12" s="7"/>
       <c r="AR12" s="7"/>
-      <c r="AS12" s="2" t="inlineStr">
+      <c r="AS12" s="7"/>
+      <c r="AT12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">진행율</t>
         </is>
       </c>
-      <c r="AT12" s="7">
-        <f>TEXT((COUNTA(AR9:AR223))/215,"0.00%")</f>
+      <c r="AU12" s="7">
+        <f>TEXT((COUNTA(AS9:AS223))/215,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -1222,6 +1238,7 @@
       <c r="AP13" s="7"/>
       <c r="AQ13" s="7"/>
       <c r="AR13" s="7"/>
+      <c r="AS13" s="7"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -1287,6 +1304,7 @@
       <c r="AP14" s="7"/>
       <c r="AQ14" s="7"/>
       <c r="AR14" s="7"/>
+      <c r="AS14" s="7"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -1388,6 +1406,7 @@
       <c r="AP15" s="7"/>
       <c r="AQ15" s="7"/>
       <c r="AR15" s="7"/>
+      <c r="AS15" s="7"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -1489,6 +1508,7 @@
       <c r="AP16" s="7"/>
       <c r="AQ16" s="7"/>
       <c r="AR16" s="7"/>
+      <c r="AS16" s="7"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -1595,6 +1615,7 @@
       <c r="AP17" s="7"/>
       <c r="AQ17" s="7"/>
       <c r="AR17" s="7"/>
+      <c r="AS17" s="7"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -1665,6 +1686,7 @@
       <c r="AP18" s="7"/>
       <c r="AQ18" s="7"/>
       <c r="AR18" s="7"/>
+      <c r="AS18" s="7"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -1730,6 +1752,7 @@
       <c r="AP19" s="7"/>
       <c r="AQ19" s="7"/>
       <c r="AR19" s="7"/>
+      <c r="AS19" s="7"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1795,6 +1818,7 @@
       <c r="AP20" s="7"/>
       <c r="AQ20" s="7"/>
       <c r="AR20" s="7"/>
+      <c r="AS20" s="7"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1896,6 +1920,7 @@
       <c r="AP21" s="7"/>
       <c r="AQ21" s="7"/>
       <c r="AR21" s="7"/>
+      <c r="AS21" s="7"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1990,6 +2015,7 @@
       <c r="AP22" s="7"/>
       <c r="AQ22" s="7"/>
       <c r="AR22" s="7"/>
+      <c r="AS22" s="7"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -2063,6 +2089,7 @@
       <c r="AP23" s="7"/>
       <c r="AQ23" s="7"/>
       <c r="AR23" s="7"/>
+      <c r="AS23" s="7"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -2128,6 +2155,7 @@
       <c r="AP24" s="7"/>
       <c r="AQ24" s="7"/>
       <c r="AR24" s="7"/>
+      <c r="AS24" s="7"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -2193,6 +2221,7 @@
       <c r="AP25" s="7"/>
       <c r="AQ25" s="7"/>
       <c r="AR25" s="7"/>
+      <c r="AS25" s="7"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -2287,6 +2316,7 @@
       <c r="AP26" s="7"/>
       <c r="AQ26" s="7"/>
       <c r="AR26" s="7"/>
+      <c r="AS26" s="7"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -2356,6 +2386,7 @@
       <c r="AP27" s="7"/>
       <c r="AQ27" s="7"/>
       <c r="AR27" s="7"/>
+      <c r="AS27" s="7"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -2434,6 +2465,7 @@
       <c r="AP28" s="7"/>
       <c r="AQ28" s="7"/>
       <c r="AR28" s="7"/>
+      <c r="AS28" s="7"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -2507,6 +2539,7 @@
       <c r="AP29" s="7"/>
       <c r="AQ29" s="7"/>
       <c r="AR29" s="7"/>
+      <c r="AS29" s="7"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -2604,6 +2637,7 @@
       <c r="AP30" s="7"/>
       <c r="AQ30" s="7"/>
       <c r="AR30" s="7"/>
+      <c r="AS30" s="7"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -2706,6 +2740,7 @@
       <c r="AP31" s="7"/>
       <c r="AQ31" s="7"/>
       <c r="AR31" s="7"/>
+      <c r="AS31" s="7"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -2795,6 +2830,7 @@
       <c r="AP32" s="7"/>
       <c r="AQ32" s="7"/>
       <c r="AR32" s="7"/>
+      <c r="AS32" s="7"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -2892,6 +2928,7 @@
       <c r="AP33" s="7"/>
       <c r="AQ33" s="7"/>
       <c r="AR33" s="7"/>
+      <c r="AS33" s="7"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -2989,6 +3026,7 @@
       <c r="AP34" s="7"/>
       <c r="AQ34" s="7"/>
       <c r="AR34" s="7"/>
+      <c r="AS34" s="7"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -3095,6 +3133,7 @@
       <c r="AP35" s="7"/>
       <c r="AQ35" s="7"/>
       <c r="AR35" s="7"/>
+      <c r="AS35" s="7"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -3176,6 +3215,7 @@
       <c r="AP36" s="7"/>
       <c r="AQ36" s="7"/>
       <c r="AR36" s="7"/>
+      <c r="AS36" s="7"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -3241,6 +3281,7 @@
       <c r="AP37" s="7"/>
       <c r="AQ37" s="7"/>
       <c r="AR37" s="7"/>
+      <c r="AS37" s="7"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -3327,6 +3368,7 @@
       <c r="AP38" s="7"/>
       <c r="AQ38" s="7"/>
       <c r="AR38" s="7"/>
+      <c r="AS38" s="7"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -3424,6 +3466,7 @@
       <c r="AP39" s="7"/>
       <c r="AQ39" s="7"/>
       <c r="AR39" s="7"/>
+      <c r="AS39" s="7"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -3522,6 +3565,7 @@
       <c r="AP40" s="7"/>
       <c r="AQ40" s="7"/>
       <c r="AR40" s="7"/>
+      <c r="AS40" s="7"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -3615,6 +3659,7 @@
       <c r="AP41" s="7"/>
       <c r="AQ41" s="7"/>
       <c r="AR41" s="7"/>
+      <c r="AS41" s="7"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -3692,6 +3737,7 @@
       <c r="AP42" s="7"/>
       <c r="AQ42" s="7"/>
       <c r="AR42" s="7"/>
+      <c r="AS42" s="7"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -3789,6 +3835,7 @@
       <c r="AP43" s="7"/>
       <c r="AQ43" s="7"/>
       <c r="AR43" s="7"/>
+      <c r="AS43" s="7"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -3859,6 +3906,7 @@
       <c r="AP44" s="7"/>
       <c r="AQ44" s="7"/>
       <c r="AR44" s="7"/>
+      <c r="AS44" s="7"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -3952,6 +4000,7 @@
       <c r="AP45" s="7"/>
       <c r="AQ45" s="7"/>
       <c r="AR45" s="7"/>
+      <c r="AS45" s="7"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -4045,6 +4094,7 @@
       <c r="AP46" s="7"/>
       <c r="AQ46" s="7"/>
       <c r="AR46" s="7"/>
+      <c r="AS46" s="7"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -4115,6 +4165,7 @@
       <c r="AP47" s="7"/>
       <c r="AQ47" s="7"/>
       <c r="AR47" s="7"/>
+      <c r="AS47" s="7"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -4180,6 +4231,7 @@
       <c r="AP48" s="7"/>
       <c r="AQ48" s="7"/>
       <c r="AR48" s="7"/>
+      <c r="AS48" s="7"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -4245,6 +4297,7 @@
       <c r="AP49" s="7"/>
       <c r="AQ49" s="7"/>
       <c r="AR49" s="7"/>
+      <c r="AS49" s="7"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -4334,6 +4387,7 @@
       <c r="AP50" s="7"/>
       <c r="AQ50" s="7"/>
       <c r="AR50" s="7"/>
+      <c r="AS50" s="7"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -4423,6 +4477,7 @@
       <c r="AP51" s="7"/>
       <c r="AQ51" s="7"/>
       <c r="AR51" s="7"/>
+      <c r="AS51" s="7"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -4493,6 +4548,7 @@
       <c r="AP52" s="7"/>
       <c r="AQ52" s="7"/>
       <c r="AR52" s="7"/>
+      <c r="AS52" s="7"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -4563,6 +4619,7 @@
       <c r="AP53" s="7"/>
       <c r="AQ53" s="7"/>
       <c r="AR53" s="7"/>
+      <c r="AS53" s="7"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -4628,6 +4685,7 @@
       <c r="AP54" s="7"/>
       <c r="AQ54" s="7"/>
       <c r="AR54" s="7"/>
+      <c r="AS54" s="7"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -4729,6 +4787,7 @@
       <c r="AP55" s="7"/>
       <c r="AQ55" s="7"/>
       <c r="AR55" s="7"/>
+      <c r="AS55" s="7"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -4810,6 +4869,7 @@
       <c r="AP56" s="7"/>
       <c r="AQ56" s="7"/>
       <c r="AR56" s="7"/>
+      <c r="AS56" s="7"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -4900,6 +4960,7 @@
       <c r="AP57" s="7"/>
       <c r="AQ57" s="7"/>
       <c r="AR57" s="7"/>
+      <c r="AS57" s="7"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -4998,6 +5059,7 @@
       <c r="AP58" s="7"/>
       <c r="AQ58" s="7"/>
       <c r="AR58" s="7"/>
+      <c r="AS58" s="7"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -5063,6 +5125,7 @@
       <c r="AP59" s="7"/>
       <c r="AQ59" s="7"/>
       <c r="AR59" s="7"/>
+      <c r="AS59" s="7"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -5128,6 +5191,7 @@
       <c r="AP60" s="7"/>
       <c r="AQ60" s="7"/>
       <c r="AR60" s="7"/>
+      <c r="AS60" s="7"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -5205,6 +5269,7 @@
       <c r="AP61" s="7"/>
       <c r="AQ61" s="7"/>
       <c r="AR61" s="7"/>
+      <c r="AS61" s="7"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -5290,6 +5355,7 @@
       <c r="AP62" s="7"/>
       <c r="AQ62" s="7"/>
       <c r="AR62" s="7"/>
+      <c r="AS62" s="7"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -5367,6 +5433,7 @@
       <c r="AP63" s="7"/>
       <c r="AQ63" s="7"/>
       <c r="AR63" s="7"/>
+      <c r="AS63" s="7"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -5432,6 +5499,7 @@
       <c r="AP64" s="7"/>
       <c r="AQ64" s="7"/>
       <c r="AR64" s="7"/>
+      <c r="AS64" s="7"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -5502,6 +5570,7 @@
       <c r="AP65" s="7"/>
       <c r="AQ65" s="7"/>
       <c r="AR65" s="7"/>
+      <c r="AS65" s="7"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
@@ -5579,6 +5648,7 @@
       <c r="AP66" s="7"/>
       <c r="AQ66" s="7"/>
       <c r="AR66" s="7"/>
+      <c r="AS66" s="7"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -5644,6 +5714,7 @@
       <c r="AP67" s="7"/>
       <c r="AQ67" s="7"/>
       <c r="AR67" s="7"/>
+      <c r="AS67" s="7"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
@@ -5713,6 +5784,7 @@
       <c r="AP68" s="7"/>
       <c r="AQ68" s="7"/>
       <c r="AR68" s="7"/>
+      <c r="AS68" s="7"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -5814,6 +5886,7 @@
       <c r="AP69" s="7"/>
       <c r="AQ69" s="7"/>
       <c r="AR69" s="7"/>
+      <c r="AS69" s="7"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
@@ -5879,6 +5952,7 @@
       <c r="AP70" s="7"/>
       <c r="AQ70" s="7"/>
       <c r="AR70" s="7"/>
+      <c r="AS70" s="7"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -5949,6 +6023,7 @@
       <c r="AP71" s="7"/>
       <c r="AQ71" s="7"/>
       <c r="AR71" s="7"/>
+      <c r="AS71" s="7"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
@@ -6030,6 +6105,7 @@
       <c r="AP72" s="7"/>
       <c r="AQ72" s="7"/>
       <c r="AR72" s="7"/>
+      <c r="AS72" s="7"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
@@ -6100,6 +6176,7 @@
       <c r="AP73" s="7"/>
       <c r="AQ73" s="7"/>
       <c r="AR73" s="7"/>
+      <c r="AS73" s="7"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -6165,6 +6242,7 @@
       <c r="AP74" s="7"/>
       <c r="AQ74" s="7"/>
       <c r="AR74" s="7"/>
+      <c r="AS74" s="7"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -6230,6 +6308,7 @@
       <c r="AP75" s="7"/>
       <c r="AQ75" s="7"/>
       <c r="AR75" s="7"/>
+      <c r="AS75" s="7"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -6295,6 +6374,7 @@
       <c r="AP76" s="7"/>
       <c r="AQ76" s="7"/>
       <c r="AR76" s="7"/>
+      <c r="AS76" s="7"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -6364,6 +6444,7 @@
       <c r="AP77" s="7"/>
       <c r="AQ77" s="7"/>
       <c r="AR77" s="7"/>
+      <c r="AS77" s="7"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
@@ -6429,6 +6510,7 @@
       <c r="AP78" s="7"/>
       <c r="AQ78" s="7"/>
       <c r="AR78" s="7"/>
+      <c r="AS78" s="7"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -6499,6 +6581,7 @@
       <c r="AP79" s="7"/>
       <c r="AQ79" s="7"/>
       <c r="AR79" s="7"/>
+      <c r="AS79" s="7"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
@@ -6580,6 +6663,7 @@
       <c r="AP80" s="7"/>
       <c r="AQ80" s="7"/>
       <c r="AR80" s="7"/>
+      <c r="AS80" s="7"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
@@ -6649,6 +6733,7 @@
       <c r="AP81" s="7"/>
       <c r="AQ81" s="7"/>
       <c r="AR81" s="7"/>
+      <c r="AS81" s="7"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
@@ -6714,6 +6799,7 @@
       <c r="AP82" s="7"/>
       <c r="AQ82" s="7"/>
       <c r="AR82" s="7"/>
+      <c r="AS82" s="7"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
@@ -6784,6 +6870,7 @@
       <c r="AP83" s="7"/>
       <c r="AQ83" s="7"/>
       <c r="AR83" s="7"/>
+      <c r="AS83" s="7"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
@@ -6849,6 +6936,7 @@
       <c r="AP84" s="7"/>
       <c r="AQ84" s="7"/>
       <c r="AR84" s="7"/>
+      <c r="AS84" s="7"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
@@ -6914,6 +7002,7 @@
       <c r="AP85" s="7"/>
       <c r="AQ85" s="7"/>
       <c r="AR85" s="7"/>
+      <c r="AS85" s="7"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
@@ -6984,6 +7073,7 @@
       <c r="AP86" s="7"/>
       <c r="AQ86" s="7"/>
       <c r="AR86" s="7"/>
+      <c r="AS86" s="7"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
@@ -7049,6 +7139,7 @@
       <c r="AP87" s="7"/>
       <c r="AQ87" s="7"/>
       <c r="AR87" s="7"/>
+      <c r="AS87" s="7"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
@@ -7114,6 +7205,7 @@
       <c r="AP88" s="7"/>
       <c r="AQ88" s="7"/>
       <c r="AR88" s="7"/>
+      <c r="AS88" s="7"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
@@ -7179,6 +7271,7 @@
       <c r="AP89" s="7"/>
       <c r="AQ89" s="7"/>
       <c r="AR89" s="7"/>
+      <c r="AS89" s="7"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
@@ -7273,6 +7366,7 @@
       <c r="AP90" s="7"/>
       <c r="AQ90" s="7"/>
       <c r="AR90" s="7"/>
+      <c r="AS90" s="7"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
@@ -7338,6 +7432,7 @@
       <c r="AP91" s="7"/>
       <c r="AQ91" s="7"/>
       <c r="AR91" s="7"/>
+      <c r="AS91" s="7"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
@@ -7439,6 +7534,7 @@
       <c r="AP92" s="7"/>
       <c r="AQ92" s="7"/>
       <c r="AR92" s="7"/>
+      <c r="AS92" s="7"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
@@ -7545,6 +7641,7 @@
       <c r="AP93" s="7"/>
       <c r="AQ93" s="7"/>
       <c r="AR93" s="7"/>
+      <c r="AS93" s="7"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
@@ -7615,6 +7712,7 @@
       <c r="AP94" s="7"/>
       <c r="AQ94" s="7"/>
       <c r="AR94" s="7"/>
+      <c r="AS94" s="7"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
@@ -7685,6 +7783,7 @@
       <c r="AP95" s="7"/>
       <c r="AQ95" s="7"/>
       <c r="AR95" s="7"/>
+      <c r="AS95" s="7"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
@@ -7774,6 +7873,7 @@
       <c r="AP96" s="7"/>
       <c r="AQ96" s="7"/>
       <c r="AR96" s="7"/>
+      <c r="AS96" s="7"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="inlineStr">
@@ -7839,6 +7939,7 @@
       <c r="AP97" s="7"/>
       <c r="AQ97" s="7"/>
       <c r="AR97" s="7"/>
+      <c r="AS97" s="7"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
@@ -7904,6 +8005,7 @@
       <c r="AP98" s="7"/>
       <c r="AQ98" s="7"/>
       <c r="AR98" s="7"/>
+      <c r="AS98" s="7"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
@@ -7969,6 +8071,7 @@
       <c r="AP99" s="7"/>
       <c r="AQ99" s="7"/>
       <c r="AR99" s="7"/>
+      <c r="AS99" s="7"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
@@ -8043,6 +8146,7 @@
       <c r="AP100" s="7"/>
       <c r="AQ100" s="7"/>
       <c r="AR100" s="7"/>
+      <c r="AS100" s="7"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
@@ -8108,6 +8212,7 @@
       <c r="AP101" s="7"/>
       <c r="AQ101" s="7"/>
       <c r="AR101" s="7"/>
+      <c r="AS101" s="7"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
@@ -8173,6 +8278,7 @@
       <c r="AP102" s="7"/>
       <c r="AQ102" s="7"/>
       <c r="AR102" s="7"/>
+      <c r="AS102" s="7"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="inlineStr">
@@ -8238,6 +8344,7 @@
       <c r="AP103" s="7"/>
       <c r="AQ103" s="7"/>
       <c r="AR103" s="7"/>
+      <c r="AS103" s="7"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="inlineStr">
@@ -8308,6 +8415,7 @@
       <c r="AP104" s="7"/>
       <c r="AQ104" s="7"/>
       <c r="AR104" s="7"/>
+      <c r="AS104" s="7"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
@@ -8373,6 +8481,7 @@
       <c r="AP105" s="7"/>
       <c r="AQ105" s="7"/>
       <c r="AR105" s="7"/>
+      <c r="AS105" s="7"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
@@ -8438,6 +8547,7 @@
       <c r="AP106" s="7"/>
       <c r="AQ106" s="7"/>
       <c r="AR106" s="7"/>
+      <c r="AS106" s="7"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
@@ -8503,6 +8613,7 @@
       <c r="AP107" s="7"/>
       <c r="AQ107" s="7"/>
       <c r="AR107" s="7"/>
+      <c r="AS107" s="7"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
@@ -8572,6 +8683,7 @@
       <c r="AP108" s="7"/>
       <c r="AQ108" s="7"/>
       <c r="AR108" s="7"/>
+      <c r="AS108" s="7"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="inlineStr">
@@ -8646,6 +8758,7 @@
       <c r="AP109" s="7"/>
       <c r="AQ109" s="7"/>
       <c r="AR109" s="7"/>
+      <c r="AS109" s="7"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
@@ -8728,6 +8841,7 @@
       <c r="AP110" s="7"/>
       <c r="AQ110" s="7"/>
       <c r="AR110" s="7"/>
+      <c r="AS110" s="7"/>
     </row>
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
@@ -8813,6 +8927,7 @@
       <c r="AP111" s="7"/>
       <c r="AQ111" s="7"/>
       <c r="AR111" s="7"/>
+      <c r="AS111" s="7"/>
     </row>
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
@@ -8895,6 +9010,7 @@
       <c r="AP112" s="7"/>
       <c r="AQ112" s="7"/>
       <c r="AR112" s="7"/>
+      <c r="AS112" s="7"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
@@ -8969,6 +9085,7 @@
       <c r="AP113" s="7"/>
       <c r="AQ113" s="7"/>
       <c r="AR113" s="7"/>
+      <c r="AS113" s="7"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="inlineStr">
@@ -9059,6 +9176,7 @@
       <c r="AP114" s="7"/>
       <c r="AQ114" s="7"/>
       <c r="AR114" s="7"/>
+      <c r="AS114" s="7"/>
     </row>
     <row r="115">
       <c r="A115" s="7" t="inlineStr">
@@ -9141,6 +9259,7 @@
       <c r="AP115" s="7"/>
       <c r="AQ115" s="7"/>
       <c r="AR115" s="7"/>
+      <c r="AS115" s="7"/>
     </row>
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
@@ -9231,6 +9350,7 @@
       <c r="AP116" s="7"/>
       <c r="AQ116" s="7"/>
       <c r="AR116" s="7"/>
+      <c r="AS116" s="7"/>
     </row>
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
@@ -9317,6 +9437,7 @@
       <c r="AP117" s="7"/>
       <c r="AQ117" s="7"/>
       <c r="AR117" s="7"/>
+      <c r="AS117" s="7"/>
     </row>
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
@@ -9403,6 +9524,7 @@
       <c r="AP118" s="7"/>
       <c r="AQ118" s="7"/>
       <c r="AR118" s="7"/>
+      <c r="AS118" s="7"/>
     </row>
     <row r="119">
       <c r="A119" s="7" t="inlineStr">
@@ -9485,6 +9607,7 @@
       <c r="AP119" s="7"/>
       <c r="AQ119" s="7"/>
       <c r="AR119" s="7"/>
+      <c r="AS119" s="7"/>
     </row>
     <row r="120">
       <c r="A120" s="7" t="inlineStr">
@@ -9559,6 +9682,7 @@
       <c r="AP120" s="7"/>
       <c r="AQ120" s="7"/>
       <c r="AR120" s="7"/>
+      <c r="AS120" s="7"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="inlineStr">
@@ -9645,6 +9769,7 @@
       <c r="AP121" s="7"/>
       <c r="AQ121" s="7"/>
       <c r="AR121" s="7"/>
+      <c r="AS121" s="7"/>
     </row>
     <row r="122">
       <c r="A122" s="7" t="inlineStr">
@@ -9731,6 +9856,7 @@
       <c r="AP122" s="7"/>
       <c r="AQ122" s="7"/>
       <c r="AR122" s="7"/>
+      <c r="AS122" s="7"/>
     </row>
     <row r="123">
       <c r="A123" s="7" t="inlineStr">
@@ -9805,6 +9931,7 @@
       <c r="AP123" s="7"/>
       <c r="AQ123" s="7"/>
       <c r="AR123" s="7"/>
+      <c r="AS123" s="7"/>
     </row>
     <row r="124">
       <c r="A124" s="7" t="inlineStr">
@@ -9887,6 +10014,7 @@
       <c r="AP124" s="7"/>
       <c r="AQ124" s="7"/>
       <c r="AR124" s="7"/>
+      <c r="AS124" s="7"/>
     </row>
     <row r="125">
       <c r="A125" s="7" t="inlineStr">
@@ -9961,6 +10089,7 @@
       <c r="AP125" s="7"/>
       <c r="AQ125" s="7"/>
       <c r="AR125" s="7"/>
+      <c r="AS125" s="7"/>
     </row>
     <row r="126">
       <c r="A126" s="7" t="inlineStr">
@@ -10035,6 +10164,7 @@
       <c r="AP126" s="7"/>
       <c r="AQ126" s="7"/>
       <c r="AR126" s="7"/>
+      <c r="AS126" s="7"/>
     </row>
     <row r="127">
       <c r="A127" s="7" t="inlineStr">
@@ -10113,6 +10243,7 @@
       <c r="AP127" s="7"/>
       <c r="AQ127" s="7"/>
       <c r="AR127" s="7"/>
+      <c r="AS127" s="7"/>
     </row>
     <row r="128">
       <c r="A128" s="7" t="inlineStr">
@@ -10191,6 +10322,7 @@
       <c r="AP128" s="7"/>
       <c r="AQ128" s="7"/>
       <c r="AR128" s="7"/>
+      <c r="AS128" s="7"/>
     </row>
     <row r="129">
       <c r="A129" s="7" t="inlineStr">
@@ -10269,6 +10401,7 @@
       <c r="AP129" s="7"/>
       <c r="AQ129" s="7"/>
       <c r="AR129" s="7"/>
+      <c r="AS129" s="7"/>
     </row>
     <row r="130">
       <c r="A130" s="7" t="inlineStr">
@@ -10343,6 +10476,7 @@
       <c r="AP130" s="7"/>
       <c r="AQ130" s="7"/>
       <c r="AR130" s="7"/>
+      <c r="AS130" s="7"/>
     </row>
     <row r="131">
       <c r="A131" s="7" t="inlineStr">
@@ -10425,6 +10559,7 @@
       <c r="AP131" s="7"/>
       <c r="AQ131" s="7"/>
       <c r="AR131" s="7"/>
+      <c r="AS131" s="7"/>
     </row>
     <row r="132">
       <c r="A132" s="7" t="inlineStr">
@@ -10511,6 +10646,7 @@
       <c r="AP132" s="7"/>
       <c r="AQ132" s="7"/>
       <c r="AR132" s="7"/>
+      <c r="AS132" s="7"/>
     </row>
     <row r="133">
       <c r="A133" s="7" t="inlineStr">
@@ -10597,6 +10733,7 @@
       <c r="AP133" s="7"/>
       <c r="AQ133" s="7"/>
       <c r="AR133" s="7"/>
+      <c r="AS133" s="7"/>
     </row>
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
@@ -10679,6 +10816,7 @@
       <c r="AP134" s="7"/>
       <c r="AQ134" s="7"/>
       <c r="AR134" s="7"/>
+      <c r="AS134" s="7"/>
     </row>
     <row r="135">
       <c r="A135" s="7" t="inlineStr">
@@ -10761,6 +10899,7 @@
       <c r="AP135" s="7"/>
       <c r="AQ135" s="7"/>
       <c r="AR135" s="7"/>
+      <c r="AS135" s="7"/>
     </row>
     <row r="136">
       <c r="A136" s="7" t="inlineStr">
@@ -10843,6 +10982,7 @@
       <c r="AP136" s="7"/>
       <c r="AQ136" s="7"/>
       <c r="AR136" s="7"/>
+      <c r="AS136" s="7"/>
     </row>
     <row r="137">
       <c r="A137" s="7" t="inlineStr">
@@ -10921,6 +11061,7 @@
       <c r="AP137" s="7"/>
       <c r="AQ137" s="7"/>
       <c r="AR137" s="7"/>
+      <c r="AS137" s="7"/>
     </row>
     <row r="138">
       <c r="A138" s="7" t="inlineStr">
@@ -10999,6 +11140,7 @@
       <c r="AP138" s="7"/>
       <c r="AQ138" s="7"/>
       <c r="AR138" s="7"/>
+      <c r="AS138" s="7"/>
     </row>
     <row r="139">
       <c r="A139" s="7" t="inlineStr">
@@ -11077,6 +11219,7 @@
       <c r="AP139" s="7"/>
       <c r="AQ139" s="7"/>
       <c r="AR139" s="7"/>
+      <c r="AS139" s="7"/>
     </row>
     <row r="140">
       <c r="A140" s="7" t="inlineStr">
@@ -11151,6 +11294,7 @@
       <c r="AP140" s="7"/>
       <c r="AQ140" s="7"/>
       <c r="AR140" s="7"/>
+      <c r="AS140" s="7"/>
     </row>
     <row r="141">
       <c r="A141" s="7" t="inlineStr">
@@ -11237,6 +11381,7 @@
       <c r="AP141" s="7"/>
       <c r="AQ141" s="7"/>
       <c r="AR141" s="7"/>
+      <c r="AS141" s="7"/>
     </row>
     <row r="142">
       <c r="A142" s="7" t="inlineStr">
@@ -11311,6 +11456,7 @@
       <c r="AP142" s="7"/>
       <c r="AQ142" s="7"/>
       <c r="AR142" s="7"/>
+      <c r="AS142" s="7"/>
     </row>
     <row r="143">
       <c r="A143" s="7" t="inlineStr">
@@ -11385,6 +11531,7 @@
       <c r="AP143" s="7"/>
       <c r="AQ143" s="7"/>
       <c r="AR143" s="7"/>
+      <c r="AS143" s="7"/>
     </row>
     <row r="144">
       <c r="A144" s="7" t="inlineStr">
@@ -11459,6 +11606,7 @@
       <c r="AP144" s="7"/>
       <c r="AQ144" s="7"/>
       <c r="AR144" s="7"/>
+      <c r="AS144" s="7"/>
     </row>
     <row r="145">
       <c r="A145" s="7" t="inlineStr">
@@ -11549,6 +11697,7 @@
       <c r="AP145" s="7"/>
       <c r="AQ145" s="7"/>
       <c r="AR145" s="7"/>
+      <c r="AS145" s="7"/>
     </row>
     <row r="146">
       <c r="A146" s="7" t="inlineStr">
@@ -11627,6 +11776,7 @@
       <c r="AP146" s="7"/>
       <c r="AQ146" s="7"/>
       <c r="AR146" s="7"/>
+      <c r="AS146" s="7"/>
     </row>
     <row r="147">
       <c r="A147" s="7" t="inlineStr">
@@ -11717,6 +11867,7 @@
       <c r="AP147" s="7"/>
       <c r="AQ147" s="7"/>
       <c r="AR147" s="7"/>
+      <c r="AS147" s="7"/>
     </row>
     <row r="148">
       <c r="A148" s="7" t="inlineStr">
@@ -11791,6 +11942,7 @@
       <c r="AP148" s="7"/>
       <c r="AQ148" s="7"/>
       <c r="AR148" s="7"/>
+      <c r="AS148" s="7"/>
     </row>
     <row r="149">
       <c r="A149" s="7" t="inlineStr">
@@ -11873,6 +12025,7 @@
       <c r="AP149" s="7"/>
       <c r="AQ149" s="7"/>
       <c r="AR149" s="7"/>
+      <c r="AS149" s="7"/>
     </row>
     <row r="150">
       <c r="A150" s="7" t="inlineStr">
@@ -11959,6 +12112,7 @@
       <c r="AP150" s="7"/>
       <c r="AQ150" s="7"/>
       <c r="AR150" s="7"/>
+      <c r="AS150" s="7"/>
     </row>
     <row r="151">
       <c r="A151" s="7" t="inlineStr">
@@ -12037,6 +12191,7 @@
       <c r="AP151" s="7"/>
       <c r="AQ151" s="7"/>
       <c r="AR151" s="7"/>
+      <c r="AS151" s="7"/>
     </row>
     <row r="152">
       <c r="A152" s="7" t="inlineStr">
@@ -12119,6 +12274,7 @@
       <c r="AP152" s="7"/>
       <c r="AQ152" s="7"/>
       <c r="AR152" s="7"/>
+      <c r="AS152" s="7"/>
     </row>
     <row r="153">
       <c r="A153" s="7" t="inlineStr">
@@ -12205,6 +12361,7 @@
       <c r="AP153" s="7"/>
       <c r="AQ153" s="7"/>
       <c r="AR153" s="7"/>
+      <c r="AS153" s="7"/>
     </row>
     <row r="154">
       <c r="A154" s="7" t="inlineStr">
@@ -12275,6 +12432,7 @@
       <c r="AP154" s="7"/>
       <c r="AQ154" s="7"/>
       <c r="AR154" s="7"/>
+      <c r="AS154" s="7"/>
     </row>
     <row r="155">
       <c r="A155" s="7" t="inlineStr">
@@ -12349,6 +12507,7 @@
       <c r="AP155" s="7"/>
       <c r="AQ155" s="7"/>
       <c r="AR155" s="7"/>
+      <c r="AS155" s="7"/>
     </row>
     <row r="156">
       <c r="A156" s="7" t="inlineStr">
@@ -12427,6 +12586,7 @@
       <c r="AP156" s="7"/>
       <c r="AQ156" s="7"/>
       <c r="AR156" s="7"/>
+      <c r="AS156" s="7"/>
     </row>
     <row r="157">
       <c r="A157" s="7" t="inlineStr">
@@ -12501,6 +12661,7 @@
       <c r="AP157" s="7"/>
       <c r="AQ157" s="7"/>
       <c r="AR157" s="7"/>
+      <c r="AS157" s="7"/>
     </row>
     <row r="158">
       <c r="A158" s="7" t="inlineStr">
@@ -12575,6 +12736,7 @@
       <c r="AP158" s="7"/>
       <c r="AQ158" s="7"/>
       <c r="AR158" s="7"/>
+      <c r="AS158" s="7"/>
     </row>
     <row r="159">
       <c r="A159" s="7" t="inlineStr">
@@ -12649,6 +12811,7 @@
       <c r="AP159" s="7"/>
       <c r="AQ159" s="7"/>
       <c r="AR159" s="7"/>
+      <c r="AS159" s="7"/>
     </row>
     <row r="160">
       <c r="A160" s="7" t="inlineStr">
@@ -12723,6 +12886,7 @@
       <c r="AP160" s="7"/>
       <c r="AQ160" s="7"/>
       <c r="AR160" s="7"/>
+      <c r="AS160" s="7"/>
     </row>
     <row r="161">
       <c r="A161" s="7" t="inlineStr">
@@ -12801,6 +12965,7 @@
       <c r="AP161" s="7"/>
       <c r="AQ161" s="7"/>
       <c r="AR161" s="7"/>
+      <c r="AS161" s="7"/>
     </row>
     <row r="162">
       <c r="A162" s="7" t="inlineStr">
@@ -12875,6 +13040,7 @@
       <c r="AP162" s="7"/>
       <c r="AQ162" s="7"/>
       <c r="AR162" s="7"/>
+      <c r="AS162" s="7"/>
     </row>
     <row r="163">
       <c r="A163" s="7" t="inlineStr">
@@ -12949,6 +13115,7 @@
       <c r="AP163" s="7"/>
       <c r="AQ163" s="7"/>
       <c r="AR163" s="7"/>
+      <c r="AS163" s="7"/>
     </row>
     <row r="164">
       <c r="A164" s="7" t="inlineStr">
@@ -13023,6 +13190,7 @@
       <c r="AP164" s="7"/>
       <c r="AQ164" s="7"/>
       <c r="AR164" s="7"/>
+      <c r="AS164" s="7"/>
     </row>
     <row r="165">
       <c r="A165" s="7" t="inlineStr">
@@ -13097,6 +13265,7 @@
       <c r="AP165" s="7"/>
       <c r="AQ165" s="7"/>
       <c r="AR165" s="7"/>
+      <c r="AS165" s="7"/>
     </row>
     <row r="166">
       <c r="A166" s="7" t="inlineStr">
@@ -13179,6 +13348,7 @@
       <c r="AP166" s="7"/>
       <c r="AQ166" s="7"/>
       <c r="AR166" s="7"/>
+      <c r="AS166" s="7"/>
     </row>
     <row r="167">
       <c r="A167" s="7" t="inlineStr">
@@ -13257,6 +13427,7 @@
       <c r="AP167" s="7"/>
       <c r="AQ167" s="7"/>
       <c r="AR167" s="7"/>
+      <c r="AS167" s="7"/>
     </row>
     <row r="168">
       <c r="A168" s="7" t="inlineStr">
@@ -13331,6 +13502,7 @@
       <c r="AP168" s="7"/>
       <c r="AQ168" s="7"/>
       <c r="AR168" s="7"/>
+      <c r="AS168" s="7"/>
     </row>
     <row r="169">
       <c r="A169" s="7" t="inlineStr">
@@ -13405,6 +13577,7 @@
       <c r="AP169" s="7"/>
       <c r="AQ169" s="7"/>
       <c r="AR169" s="7"/>
+      <c r="AS169" s="7"/>
     </row>
     <row r="170">
       <c r="A170" s="7" t="inlineStr">
@@ -13483,6 +13656,7 @@
       <c r="AP170" s="7"/>
       <c r="AQ170" s="7"/>
       <c r="AR170" s="7"/>
+      <c r="AS170" s="7"/>
     </row>
     <row r="171">
       <c r="A171" s="7" t="inlineStr">
@@ -13553,6 +13727,7 @@
       <c r="AP171" s="7"/>
       <c r="AQ171" s="7"/>
       <c r="AR171" s="7"/>
+      <c r="AS171" s="7"/>
     </row>
     <row r="172">
       <c r="A172" s="7" t="inlineStr">
@@ -13623,6 +13798,7 @@
       <c r="AP172" s="7"/>
       <c r="AQ172" s="7"/>
       <c r="AR172" s="7"/>
+      <c r="AS172" s="7"/>
     </row>
     <row r="173">
       <c r="A173" s="7" t="inlineStr">
@@ -13701,6 +13877,7 @@
       <c r="AP173" s="7"/>
       <c r="AQ173" s="7"/>
       <c r="AR173" s="7"/>
+      <c r="AS173" s="7"/>
     </row>
     <row r="174">
       <c r="A174" s="7" t="inlineStr">
@@ -13775,6 +13952,7 @@
       <c r="AP174" s="7"/>
       <c r="AQ174" s="7"/>
       <c r="AR174" s="7"/>
+      <c r="AS174" s="7"/>
     </row>
     <row r="175">
       <c r="A175" s="7" t="inlineStr">
@@ -13853,6 +14031,7 @@
       <c r="AP175" s="7"/>
       <c r="AQ175" s="7"/>
       <c r="AR175" s="7"/>
+      <c r="AS175" s="7"/>
     </row>
     <row r="176">
       <c r="A176" s="7" t="inlineStr">
@@ -13927,6 +14106,7 @@
       <c r="AP176" s="7"/>
       <c r="AQ176" s="7"/>
       <c r="AR176" s="7"/>
+      <c r="AS176" s="7"/>
     </row>
     <row r="177">
       <c r="A177" s="7" t="inlineStr">
@@ -14001,6 +14181,7 @@
       <c r="AP177" s="7"/>
       <c r="AQ177" s="7"/>
       <c r="AR177" s="7"/>
+      <c r="AS177" s="7"/>
     </row>
     <row r="178">
       <c r="A178" s="7" t="inlineStr">
@@ -14075,6 +14256,7 @@
       <c r="AP178" s="7"/>
       <c r="AQ178" s="7"/>
       <c r="AR178" s="7"/>
+      <c r="AS178" s="7"/>
     </row>
     <row r="179">
       <c r="A179" s="7" t="inlineStr">
@@ -14149,6 +14331,7 @@
       <c r="AP179" s="7"/>
       <c r="AQ179" s="7"/>
       <c r="AR179" s="7"/>
+      <c r="AS179" s="7"/>
     </row>
     <row r="180">
       <c r="A180" s="7" t="inlineStr">
@@ -14223,6 +14406,7 @@
       <c r="AP180" s="7"/>
       <c r="AQ180" s="7"/>
       <c r="AR180" s="7"/>
+      <c r="AS180" s="7"/>
     </row>
     <row r="181">
       <c r="A181" s="7" t="inlineStr">
@@ -14297,6 +14481,7 @@
       <c r="AP181" s="7"/>
       <c r="AQ181" s="7"/>
       <c r="AR181" s="7"/>
+      <c r="AS181" s="7"/>
     </row>
     <row r="182">
       <c r="A182" s="7" t="inlineStr">
@@ -14371,6 +14556,7 @@
       <c r="AP182" s="7"/>
       <c r="AQ182" s="7"/>
       <c r="AR182" s="7"/>
+      <c r="AS182" s="7"/>
     </row>
     <row r="183">
       <c r="A183" s="7" t="inlineStr">
@@ -14445,6 +14631,7 @@
       <c r="AP183" s="7"/>
       <c r="AQ183" s="7"/>
       <c r="AR183" s="7"/>
+      <c r="AS183" s="7"/>
     </row>
     <row r="184">
       <c r="A184" s="7" t="inlineStr">
@@ -14515,6 +14702,7 @@
       <c r="AP184" s="7"/>
       <c r="AQ184" s="7"/>
       <c r="AR184" s="7"/>
+      <c r="AS184" s="7"/>
     </row>
     <row r="185">
       <c r="A185" s="7" t="inlineStr">
@@ -14589,6 +14777,7 @@
       <c r="AP185" s="7"/>
       <c r="AQ185" s="7"/>
       <c r="AR185" s="7"/>
+      <c r="AS185" s="7"/>
     </row>
     <row r="186">
       <c r="A186" s="7" t="inlineStr">
@@ -14663,6 +14852,7 @@
       <c r="AP186" s="7"/>
       <c r="AQ186" s="7"/>
       <c r="AR186" s="7"/>
+      <c r="AS186" s="7"/>
     </row>
     <row r="187">
       <c r="A187" s="7" t="inlineStr">
@@ -14741,6 +14931,7 @@
       <c r="AP187" s="7"/>
       <c r="AQ187" s="7"/>
       <c r="AR187" s="7"/>
+      <c r="AS187" s="7"/>
     </row>
     <row r="188">
       <c r="A188" s="7" t="inlineStr">
@@ -14819,6 +15010,7 @@
       <c r="AP188" s="7"/>
       <c r="AQ188" s="7"/>
       <c r="AR188" s="7"/>
+      <c r="AS188" s="7"/>
     </row>
     <row r="189">
       <c r="A189" s="7" t="inlineStr">
@@ -14897,6 +15089,7 @@
       <c r="AP189" s="7"/>
       <c r="AQ189" s="7"/>
       <c r="AR189" s="7"/>
+      <c r="AS189" s="7"/>
     </row>
     <row r="190">
       <c r="A190" s="7" t="inlineStr">
@@ -14975,6 +15168,7 @@
       <c r="AP190" s="7"/>
       <c r="AQ190" s="7"/>
       <c r="AR190" s="7"/>
+      <c r="AS190" s="7"/>
     </row>
     <row r="191">
       <c r="A191" s="7" t="inlineStr">
@@ -15053,6 +15247,7 @@
       <c r="AP191" s="7"/>
       <c r="AQ191" s="7"/>
       <c r="AR191" s="7"/>
+      <c r="AS191" s="7"/>
     </row>
     <row r="192">
       <c r="A192" s="7" t="inlineStr">
@@ -15131,6 +15326,7 @@
       <c r="AP192" s="7"/>
       <c r="AQ192" s="7"/>
       <c r="AR192" s="7"/>
+      <c r="AS192" s="7"/>
     </row>
     <row r="193">
       <c r="A193" s="7" t="inlineStr">
@@ -15213,6 +15409,7 @@
         </is>
       </c>
       <c r="AR193" s="7"/>
+      <c r="AS193" s="7"/>
     </row>
     <row r="194">
       <c r="A194" s="7" t="inlineStr">
@@ -15295,6 +15492,7 @@
         </is>
       </c>
       <c r="AR194" s="7"/>
+      <c r="AS194" s="7"/>
     </row>
     <row r="195">
       <c r="A195" s="7" t="inlineStr">
@@ -15377,6 +15575,7 @@
         </is>
       </c>
       <c r="AR195" s="7"/>
+      <c r="AS195" s="7"/>
     </row>
     <row r="196">
       <c r="A196" s="7" t="inlineStr">
@@ -15451,6 +15650,7 @@
       <c r="AP196" s="7"/>
       <c r="AQ196" s="7"/>
       <c r="AR196" s="7"/>
+      <c r="AS196" s="7"/>
     </row>
     <row r="197">
       <c r="A197" s="7" t="inlineStr">
@@ -15533,6 +15733,7 @@
         </is>
       </c>
       <c r="AR197" s="7"/>
+      <c r="AS197" s="7"/>
     </row>
     <row r="198">
       <c r="A198" s="7" t="inlineStr">
@@ -15607,6 +15808,7 @@
       <c r="AP198" s="7"/>
       <c r="AQ198" s="7"/>
       <c r="AR198" s="7"/>
+      <c r="AS198" s="7"/>
     </row>
     <row r="199">
       <c r="A199" s="7" t="inlineStr">
@@ -15689,6 +15891,7 @@
         </is>
       </c>
       <c r="AR199" s="7"/>
+      <c r="AS199" s="7"/>
     </row>
     <row r="200">
       <c r="A200" s="7" t="inlineStr">
@@ -15771,6 +15974,7 @@
         </is>
       </c>
       <c r="AR200" s="7"/>
+      <c r="AS200" s="7"/>
     </row>
     <row r="201">
       <c r="A201" s="7" t="inlineStr">
@@ -15845,6 +16049,7 @@
         </is>
       </c>
       <c r="AR201" s="7"/>
+      <c r="AS201" s="7"/>
     </row>
     <row r="202">
       <c r="A202" s="7" t="inlineStr">
@@ -15927,6 +16132,7 @@
         </is>
       </c>
       <c r="AR202" s="7"/>
+      <c r="AS202" s="7"/>
     </row>
     <row r="203">
       <c r="A203" s="7" t="inlineStr">
@@ -16009,6 +16215,7 @@
         </is>
       </c>
       <c r="AR203" s="7"/>
+      <c r="AS203" s="7"/>
     </row>
     <row r="204">
       <c r="A204" s="7" t="inlineStr">
@@ -16095,6 +16302,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AS204" s="7"/>
     </row>
     <row r="205">
       <c r="A205" s="7" t="inlineStr">
@@ -16181,6 +16389,7 @@
         </is>
       </c>
       <c r="AR205" s="7"/>
+      <c r="AS205" s="7"/>
     </row>
     <row r="206">
       <c r="A206" s="7" t="inlineStr">
@@ -16267,6 +16476,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AS206" s="7"/>
     </row>
     <row r="207">
       <c r="A207" s="7" t="inlineStr">
@@ -16345,6 +16555,7 @@
         </is>
       </c>
       <c r="AR207" s="7"/>
+      <c r="AS207" s="7"/>
     </row>
     <row r="208">
       <c r="A208" s="7" t="inlineStr">
@@ -16427,6 +16638,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AS208" s="7"/>
     </row>
     <row r="209">
       <c r="A209" s="7" t="inlineStr">
@@ -16513,6 +16725,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AS209" s="7"/>
     </row>
     <row r="210">
       <c r="A210" s="7" t="inlineStr">
@@ -16595,6 +16808,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AS210" s="7"/>
     </row>
     <row r="211">
       <c r="A211" s="7" t="inlineStr">
@@ -16669,6 +16883,7 @@
       </c>
       <c r="AQ211" s="7"/>
       <c r="AR211" s="7"/>
+      <c r="AS211" s="7"/>
     </row>
     <row r="212">
       <c r="A212" s="7" t="inlineStr">
@@ -16743,6 +16958,7 @@
         </is>
       </c>
       <c r="AR212" s="7"/>
+      <c r="AS212" s="7"/>
     </row>
     <row r="213">
       <c r="A213" s="7" t="inlineStr">
@@ -16821,6 +17037,7 @@
           <t xml:space="preserve">N/A</t>
         </is>
       </c>
+      <c r="AS213" s="7"/>
     </row>
     <row r="214">
       <c r="A214" s="7" t="inlineStr">
@@ -16895,6 +17112,7 @@
         </is>
       </c>
       <c r="AR214" s="7"/>
+      <c r="AS214" s="7"/>
     </row>
     <row r="215">
       <c r="A215" s="7" t="inlineStr">
@@ -16965,6 +17183,7 @@
       <c r="AP215" s="7"/>
       <c r="AQ215" s="7"/>
       <c r="AR215" s="7"/>
+      <c r="AS215" s="7"/>
     </row>
     <row r="216">
       <c r="A216" s="7" t="inlineStr">
@@ -17035,6 +17254,7 @@
       <c r="AP216" s="7"/>
       <c r="AQ216" s="7"/>
       <c r="AR216" s="7"/>
+      <c r="AS216" s="7"/>
     </row>
     <row r="217">
       <c r="A217" s="7" t="inlineStr">
@@ -17109,6 +17329,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AS217" s="7"/>
     </row>
     <row r="218">
       <c r="A218" s="7" t="inlineStr">
@@ -17179,6 +17400,7 @@
       <c r="AP218" s="7"/>
       <c r="AQ218" s="7"/>
       <c r="AR218" s="7"/>
+      <c r="AS218" s="7"/>
     </row>
     <row r="219">
       <c r="A219" s="7" t="inlineStr">
@@ -17253,6 +17475,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AS219" s="7"/>
     </row>
     <row r="220">
       <c r="A220" s="7" t="inlineStr">
@@ -17323,6 +17546,7 @@
       <c r="AP220" s="7"/>
       <c r="AQ220" s="7"/>
       <c r="AR220" s="7"/>
+      <c r="AS220" s="7"/>
     </row>
     <row r="221">
       <c r="A221" s="7" t="inlineStr">
@@ -17397,6 +17621,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AS221" s="7"/>
     </row>
     <row r="222">
       <c r="A222" s="7" t="inlineStr">
@@ -17426,7 +17651,7 @@
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t xml:space="preserve">AR Fail — B 판이 열리고 안내 「로봇 B 마운트를 탭한 뒤 강화를 누르세요」는 섰으나 B 마운트 칸이 보드 위쪽 화면 밖 · 줌아웃 한계라 이동 모드로 끌어 내려야 보임. 그 뒤 탭 · 강화는 정상</t>
+          <t xml:space="preserve">AR Fail — B 판이 열리고 안내 「로봇 B 마운트를 탭한 뒤 강화를 누르세요」는 섰으나 B 마운트 칸이 보드 위쪽 화면 밖 · 줌아웃 한계라 이동 모드로 끌어 내려야 보임. 그 뒤 탭 · 강화는 정상 · AS Pass — 원인 = FocusCell 이 들어간 첫 프레임(카메라 미끄러짐 중)에 한 번 → 카메라가 선 뒤로 옮김(BoardFocusRule) · 8b54a82 처음부터 → S6 → 조립: B 마운트 칸 화면 가운데 · 탭 → 팝오버 → 강화 완료</t>
         </is>
       </c>
       <c r="G222" s="7"/>
@@ -17471,6 +17696,11 @@
           <t xml:space="preserve">Fail</t>
         </is>
       </c>
+      <c r="AS222" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="7" t="inlineStr">
@@ -17500,7 +17730,7 @@
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t xml:space="preserve">AR Fail(경미) — 처음부터 직후 [v] 로 남고 판은 빈 칸(고스트) · 새로고침하면 [ ] 로 바로 섬</t>
+          <t xml:space="preserve">AR Fail(경미) — 처음부터 직후 [v] 로 남고 판은 빈 칸(고스트) · 새로고침하면 [ ] 로 바로 섬 · AS — 태그 뒤 결함 후보 목록(플랜)</t>
         </is>
       </c>
       <c r="G223" s="7"/>
@@ -17545,6 +17775,7 @@
           <t xml:space="preserve">Fail</t>
         </is>
       </c>
+      <c r="AS223" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="26">
@@ -17573,9 +17804,9 @@
     <mergeCell ref="B92:B99"/>
     <mergeCell ref="B100:B106"/>
     <mergeCell ref="B107:B111"/>
-    <mergeCell ref="G7:AR7"/>
+    <mergeCell ref="G7:AS7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:AR223">
+  <conditionalFormatting sqref="G9:AS223">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
QA AT(5d04f2f · CID_216~222)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -201,8 +201,9 @@
     <col min="43" max="43" width="12" customWidth="1"/>
     <col min="44" max="44" width="12" customWidth="1"/>
     <col min="45" max="45" width="12" customWidth="1"/>
-    <col min="46" max="46" width="11" customWidth="1"/>
+    <col min="46" max="46" width="12" customWidth="1"/>
     <col min="47" max="47" width="11" customWidth="1"/>
+    <col min="48" max="48" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -510,6 +511,11 @@
       <c r="AS6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">8133 8b54a82 갈아엎음(23:23) · CID_214 튜토리얼 시야 이동을 조립 카메라가 선 뒤로(A·B 강화 · S5 폭발탄 같은 규칙) ‖ 보이는 창 재확인: 처음부터 → 바로가기 S6 → 조립 = B 마운트 칸 화면 안 + 안내 → 탭 → 강화 ✅ · 시험 1679/1673/0/6 · 전투 12줄 불변. 나머지 칸 = AR 그대로(이 빌드에서 안 다시 봄).</t>
+        </is>
+      </c>
+      <c r="AT6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8133 5d04f2f 갈아엎음(10-20 00:04) · 사용자 육안(10-19 23:4x · 8b54a82) 결함 ①③④⑤ + #210 · #211 · #212 ‖ 보이는 창 재확인 일부. 시험 1684/1678/0/6 · 전투 12줄 불변.</t>
         </is>
       </c>
     </row>
@@ -579,14 +585,15 @@
       <c r="AQ7" s="2"/>
       <c r="AR7" s="2"/>
       <c r="AS7" s="2"/>
-      <c r="AT7" s="2" t="inlineStr">
+      <c r="AT7" s="2"/>
+      <c r="AU7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">버전</t>
         </is>
       </c>
-      <c r="AU7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8b54a82</t>
+      <c r="AV7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5d04f2f</t>
         </is>
       </c>
     </row>
@@ -806,11 +813,16 @@
       </c>
       <c r="AT8" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">5d04f2f</t>
+        </is>
+      </c>
+      <c r="AU8" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">PASSrate</t>
         </is>
       </c>
-      <c r="AU8" s="7">
-        <f>COUNTIF(AS9:AS223,"Pass")</f>
+      <c r="AV8" s="7">
+        <f>COUNTIF(AT9:AT230,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -919,13 +931,14 @@
       <c r="AQ9" s="7"/>
       <c r="AR9" s="7"/>
       <c r="AS9" s="7"/>
-      <c r="AT9" s="2" t="inlineStr">
+      <c r="AT9" s="7"/>
+      <c r="AU9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FAILrate</t>
         </is>
       </c>
-      <c r="AU9" s="7">
-        <f>COUNTIF(AS9:AS223,"Fail")+COUNTIF(AS9:AS223,"Broken")</f>
+      <c r="AV9" s="7">
+        <f>COUNTIF(AT9:AT230,"Fail")+COUNTIF(AT9:AT230,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -998,13 +1011,14 @@
       <c r="AQ10" s="7"/>
       <c r="AR10" s="7"/>
       <c r="AS10" s="7"/>
-      <c r="AT10" s="2" t="inlineStr">
+      <c r="AT10" s="7"/>
+      <c r="AU10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">N/A</t>
         </is>
       </c>
-      <c r="AU10" s="7">
-        <f>COUNTIF(AS9:AS223,"N/A")</f>
+      <c r="AV10" s="7">
+        <f>COUNTIF(AT9:AT230,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -1077,13 +1091,14 @@
       <c r="AQ11" s="7"/>
       <c r="AR11" s="7"/>
       <c r="AS11" s="7"/>
-      <c r="AT11" s="2" t="inlineStr">
+      <c r="AT11" s="7"/>
+      <c r="AU11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">전체 개수</t>
         </is>
       </c>
-      <c r="AU11" s="7">
-        <v>215</v>
+      <c r="AV11" s="7">
+        <v>222</v>
       </c>
     </row>
     <row r="12">
@@ -1156,13 +1171,14 @@
       <c r="AQ12" s="7"/>
       <c r="AR12" s="7"/>
       <c r="AS12" s="7"/>
-      <c r="AT12" s="2" t="inlineStr">
+      <c r="AT12" s="7"/>
+      <c r="AU12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">진행율</t>
         </is>
       </c>
-      <c r="AU12" s="7">
-        <f>TEXT((COUNTA(AS9:AS223))/215,"0.00%")</f>
+      <c r="AV12" s="7">
+        <f>TEXT((COUNTA(AT9:AT230))/222,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -1239,6 +1255,7 @@
       <c r="AQ13" s="7"/>
       <c r="AR13" s="7"/>
       <c r="AS13" s="7"/>
+      <c r="AT13" s="7"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -1305,6 +1322,7 @@
       <c r="AQ14" s="7"/>
       <c r="AR14" s="7"/>
       <c r="AS14" s="7"/>
+      <c r="AT14" s="7"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -1407,6 +1425,7 @@
       <c r="AQ15" s="7"/>
       <c r="AR15" s="7"/>
       <c r="AS15" s="7"/>
+      <c r="AT15" s="7"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -1509,6 +1528,7 @@
       <c r="AQ16" s="7"/>
       <c r="AR16" s="7"/>
       <c r="AS16" s="7"/>
+      <c r="AT16" s="7"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -1616,6 +1636,7 @@
       <c r="AQ17" s="7"/>
       <c r="AR17" s="7"/>
       <c r="AS17" s="7"/>
+      <c r="AT17" s="7"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -1687,6 +1708,7 @@
       <c r="AQ18" s="7"/>
       <c r="AR18" s="7"/>
       <c r="AS18" s="7"/>
+      <c r="AT18" s="7"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -1753,6 +1775,7 @@
       <c r="AQ19" s="7"/>
       <c r="AR19" s="7"/>
       <c r="AS19" s="7"/>
+      <c r="AT19" s="7"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1819,6 +1842,7 @@
       <c r="AQ20" s="7"/>
       <c r="AR20" s="7"/>
       <c r="AS20" s="7"/>
+      <c r="AT20" s="7"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1921,6 +1945,7 @@
       <c r="AQ21" s="7"/>
       <c r="AR21" s="7"/>
       <c r="AS21" s="7"/>
+      <c r="AT21" s="7"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -2016,6 +2041,7 @@
       <c r="AQ22" s="7"/>
       <c r="AR22" s="7"/>
       <c r="AS22" s="7"/>
+      <c r="AT22" s="7"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -2090,6 +2116,7 @@
       <c r="AQ23" s="7"/>
       <c r="AR23" s="7"/>
       <c r="AS23" s="7"/>
+      <c r="AT23" s="7"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -2156,6 +2183,7 @@
       <c r="AQ24" s="7"/>
       <c r="AR24" s="7"/>
       <c r="AS24" s="7"/>
+      <c r="AT24" s="7"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -2222,6 +2250,7 @@
       <c r="AQ25" s="7"/>
       <c r="AR25" s="7"/>
       <c r="AS25" s="7"/>
+      <c r="AT25" s="7"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -2317,6 +2346,7 @@
       <c r="AQ26" s="7"/>
       <c r="AR26" s="7"/>
       <c r="AS26" s="7"/>
+      <c r="AT26" s="7"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -2387,6 +2417,7 @@
       <c r="AQ27" s="7"/>
       <c r="AR27" s="7"/>
       <c r="AS27" s="7"/>
+      <c r="AT27" s="7"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -2466,6 +2497,7 @@
       <c r="AQ28" s="7"/>
       <c r="AR28" s="7"/>
       <c r="AS28" s="7"/>
+      <c r="AT28" s="7"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -2540,6 +2572,7 @@
       <c r="AQ29" s="7"/>
       <c r="AR29" s="7"/>
       <c r="AS29" s="7"/>
+      <c r="AT29" s="7"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -2638,6 +2671,7 @@
       <c r="AQ30" s="7"/>
       <c r="AR30" s="7"/>
       <c r="AS30" s="7"/>
+      <c r="AT30" s="7"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -2741,6 +2775,7 @@
       <c r="AQ31" s="7"/>
       <c r="AR31" s="7"/>
       <c r="AS31" s="7"/>
+      <c r="AT31" s="7"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -2831,6 +2866,7 @@
       <c r="AQ32" s="7"/>
       <c r="AR32" s="7"/>
       <c r="AS32" s="7"/>
+      <c r="AT32" s="7"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -2929,6 +2965,7 @@
       <c r="AQ33" s="7"/>
       <c r="AR33" s="7"/>
       <c r="AS33" s="7"/>
+      <c r="AT33" s="7"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -3027,6 +3064,7 @@
       <c r="AQ34" s="7"/>
       <c r="AR34" s="7"/>
       <c r="AS34" s="7"/>
+      <c r="AT34" s="7"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -3134,6 +3172,7 @@
       <c r="AQ35" s="7"/>
       <c r="AR35" s="7"/>
       <c r="AS35" s="7"/>
+      <c r="AT35" s="7"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -3216,6 +3255,7 @@
       <c r="AQ36" s="7"/>
       <c r="AR36" s="7"/>
       <c r="AS36" s="7"/>
+      <c r="AT36" s="7"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -3282,6 +3322,7 @@
       <c r="AQ37" s="7"/>
       <c r="AR37" s="7"/>
       <c r="AS37" s="7"/>
+      <c r="AT37" s="7"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -3369,6 +3410,7 @@
       <c r="AQ38" s="7"/>
       <c r="AR38" s="7"/>
       <c r="AS38" s="7"/>
+      <c r="AT38" s="7"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -3467,6 +3509,7 @@
       <c r="AQ39" s="7"/>
       <c r="AR39" s="7"/>
       <c r="AS39" s="7"/>
+      <c r="AT39" s="7"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -3566,6 +3609,7 @@
       <c r="AQ40" s="7"/>
       <c r="AR40" s="7"/>
       <c r="AS40" s="7"/>
+      <c r="AT40" s="7"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -3660,6 +3704,7 @@
       <c r="AQ41" s="7"/>
       <c r="AR41" s="7"/>
       <c r="AS41" s="7"/>
+      <c r="AT41" s="7"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -3738,6 +3783,7 @@
       <c r="AQ42" s="7"/>
       <c r="AR42" s="7"/>
       <c r="AS42" s="7"/>
+      <c r="AT42" s="7"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -3836,6 +3882,7 @@
       <c r="AQ43" s="7"/>
       <c r="AR43" s="7"/>
       <c r="AS43" s="7"/>
+      <c r="AT43" s="7"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -3907,6 +3954,7 @@
       <c r="AQ44" s="7"/>
       <c r="AR44" s="7"/>
       <c r="AS44" s="7"/>
+      <c r="AT44" s="7"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -4001,6 +4049,7 @@
       <c r="AQ45" s="7"/>
       <c r="AR45" s="7"/>
       <c r="AS45" s="7"/>
+      <c r="AT45" s="7"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -4095,6 +4144,7 @@
       <c r="AQ46" s="7"/>
       <c r="AR46" s="7"/>
       <c r="AS46" s="7"/>
+      <c r="AT46" s="7"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -4166,6 +4216,7 @@
       <c r="AQ47" s="7"/>
       <c r="AR47" s="7"/>
       <c r="AS47" s="7"/>
+      <c r="AT47" s="7"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -4232,6 +4283,7 @@
       <c r="AQ48" s="7"/>
       <c r="AR48" s="7"/>
       <c r="AS48" s="7"/>
+      <c r="AT48" s="7"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -4298,6 +4350,7 @@
       <c r="AQ49" s="7"/>
       <c r="AR49" s="7"/>
       <c r="AS49" s="7"/>
+      <c r="AT49" s="7"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -4388,6 +4441,7 @@
       <c r="AQ50" s="7"/>
       <c r="AR50" s="7"/>
       <c r="AS50" s="7"/>
+      <c r="AT50" s="7"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -4478,6 +4532,7 @@
       <c r="AQ51" s="7"/>
       <c r="AR51" s="7"/>
       <c r="AS51" s="7"/>
+      <c r="AT51" s="7"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -4549,6 +4604,7 @@
       <c r="AQ52" s="7"/>
       <c r="AR52" s="7"/>
       <c r="AS52" s="7"/>
+      <c r="AT52" s="7"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -4620,6 +4676,7 @@
       <c r="AQ53" s="7"/>
       <c r="AR53" s="7"/>
       <c r="AS53" s="7"/>
+      <c r="AT53" s="7"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -4686,6 +4743,7 @@
       <c r="AQ54" s="7"/>
       <c r="AR54" s="7"/>
       <c r="AS54" s="7"/>
+      <c r="AT54" s="7"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -4788,6 +4846,7 @@
       <c r="AQ55" s="7"/>
       <c r="AR55" s="7"/>
       <c r="AS55" s="7"/>
+      <c r="AT55" s="7"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -4870,6 +4929,7 @@
       <c r="AQ56" s="7"/>
       <c r="AR56" s="7"/>
       <c r="AS56" s="7"/>
+      <c r="AT56" s="7"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -4961,6 +5021,7 @@
       <c r="AQ57" s="7"/>
       <c r="AR57" s="7"/>
       <c r="AS57" s="7"/>
+      <c r="AT57" s="7"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -5060,6 +5121,7 @@
       <c r="AQ58" s="7"/>
       <c r="AR58" s="7"/>
       <c r="AS58" s="7"/>
+      <c r="AT58" s="7"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -5126,6 +5188,7 @@
       <c r="AQ59" s="7"/>
       <c r="AR59" s="7"/>
       <c r="AS59" s="7"/>
+      <c r="AT59" s="7"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -5192,6 +5255,7 @@
       <c r="AQ60" s="7"/>
       <c r="AR60" s="7"/>
       <c r="AS60" s="7"/>
+      <c r="AT60" s="7"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -5270,6 +5334,7 @@
       <c r="AQ61" s="7"/>
       <c r="AR61" s="7"/>
       <c r="AS61" s="7"/>
+      <c r="AT61" s="7"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -5356,6 +5421,7 @@
       <c r="AQ62" s="7"/>
       <c r="AR62" s="7"/>
       <c r="AS62" s="7"/>
+      <c r="AT62" s="7"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -5434,6 +5500,7 @@
       <c r="AQ63" s="7"/>
       <c r="AR63" s="7"/>
       <c r="AS63" s="7"/>
+      <c r="AT63" s="7"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -5500,6 +5567,7 @@
       <c r="AQ64" s="7"/>
       <c r="AR64" s="7"/>
       <c r="AS64" s="7"/>
+      <c r="AT64" s="7"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -5571,6 +5639,7 @@
       <c r="AQ65" s="7"/>
       <c r="AR65" s="7"/>
       <c r="AS65" s="7"/>
+      <c r="AT65" s="7"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
@@ -5649,6 +5718,7 @@
       <c r="AQ66" s="7"/>
       <c r="AR66" s="7"/>
       <c r="AS66" s="7"/>
+      <c r="AT66" s="7"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -5715,6 +5785,7 @@
       <c r="AQ67" s="7"/>
       <c r="AR67" s="7"/>
       <c r="AS67" s="7"/>
+      <c r="AT67" s="7"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
@@ -5785,6 +5856,7 @@
       <c r="AQ68" s="7"/>
       <c r="AR68" s="7"/>
       <c r="AS68" s="7"/>
+      <c r="AT68" s="7"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -5887,6 +5959,7 @@
       <c r="AQ69" s="7"/>
       <c r="AR69" s="7"/>
       <c r="AS69" s="7"/>
+      <c r="AT69" s="7"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
@@ -5953,6 +6026,7 @@
       <c r="AQ70" s="7"/>
       <c r="AR70" s="7"/>
       <c r="AS70" s="7"/>
+      <c r="AT70" s="7"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -6024,6 +6098,7 @@
       <c r="AQ71" s="7"/>
       <c r="AR71" s="7"/>
       <c r="AS71" s="7"/>
+      <c r="AT71" s="7"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
@@ -6106,6 +6181,7 @@
       <c r="AQ72" s="7"/>
       <c r="AR72" s="7"/>
       <c r="AS72" s="7"/>
+      <c r="AT72" s="7"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
@@ -6177,6 +6253,7 @@
       <c r="AQ73" s="7"/>
       <c r="AR73" s="7"/>
       <c r="AS73" s="7"/>
+      <c r="AT73" s="7"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -6243,6 +6320,7 @@
       <c r="AQ74" s="7"/>
       <c r="AR74" s="7"/>
       <c r="AS74" s="7"/>
+      <c r="AT74" s="7"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -6309,6 +6387,7 @@
       <c r="AQ75" s="7"/>
       <c r="AR75" s="7"/>
       <c r="AS75" s="7"/>
+      <c r="AT75" s="7"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -6375,6 +6454,7 @@
       <c r="AQ76" s="7"/>
       <c r="AR76" s="7"/>
       <c r="AS76" s="7"/>
+      <c r="AT76" s="7"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -6445,6 +6525,7 @@
       <c r="AQ77" s="7"/>
       <c r="AR77" s="7"/>
       <c r="AS77" s="7"/>
+      <c r="AT77" s="7"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
@@ -6511,6 +6592,7 @@
       <c r="AQ78" s="7"/>
       <c r="AR78" s="7"/>
       <c r="AS78" s="7"/>
+      <c r="AT78" s="7"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -6582,6 +6664,7 @@
       <c r="AQ79" s="7"/>
       <c r="AR79" s="7"/>
       <c r="AS79" s="7"/>
+      <c r="AT79" s="7"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
@@ -6664,6 +6747,7 @@
       <c r="AQ80" s="7"/>
       <c r="AR80" s="7"/>
       <c r="AS80" s="7"/>
+      <c r="AT80" s="7"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
@@ -6734,6 +6818,7 @@
       <c r="AQ81" s="7"/>
       <c r="AR81" s="7"/>
       <c r="AS81" s="7"/>
+      <c r="AT81" s="7"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
@@ -6800,6 +6885,7 @@
       <c r="AQ82" s="7"/>
       <c r="AR82" s="7"/>
       <c r="AS82" s="7"/>
+      <c r="AT82" s="7"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
@@ -6871,6 +6957,7 @@
       <c r="AQ83" s="7"/>
       <c r="AR83" s="7"/>
       <c r="AS83" s="7"/>
+      <c r="AT83" s="7"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
@@ -6937,6 +7024,7 @@
       <c r="AQ84" s="7"/>
       <c r="AR84" s="7"/>
       <c r="AS84" s="7"/>
+      <c r="AT84" s="7"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
@@ -7003,6 +7091,7 @@
       <c r="AQ85" s="7"/>
       <c r="AR85" s="7"/>
       <c r="AS85" s="7"/>
+      <c r="AT85" s="7"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
@@ -7074,6 +7163,7 @@
       <c r="AQ86" s="7"/>
       <c r="AR86" s="7"/>
       <c r="AS86" s="7"/>
+      <c r="AT86" s="7"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
@@ -7140,6 +7230,7 @@
       <c r="AQ87" s="7"/>
       <c r="AR87" s="7"/>
       <c r="AS87" s="7"/>
+      <c r="AT87" s="7"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
@@ -7206,6 +7297,7 @@
       <c r="AQ88" s="7"/>
       <c r="AR88" s="7"/>
       <c r="AS88" s="7"/>
+      <c r="AT88" s="7"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
@@ -7272,6 +7364,7 @@
       <c r="AQ89" s="7"/>
       <c r="AR89" s="7"/>
       <c r="AS89" s="7"/>
+      <c r="AT89" s="7"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
@@ -7367,6 +7460,7 @@
       <c r="AQ90" s="7"/>
       <c r="AR90" s="7"/>
       <c r="AS90" s="7"/>
+      <c r="AT90" s="7"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
@@ -7433,6 +7527,7 @@
       <c r="AQ91" s="7"/>
       <c r="AR91" s="7"/>
       <c r="AS91" s="7"/>
+      <c r="AT91" s="7"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
@@ -7535,6 +7630,7 @@
       <c r="AQ92" s="7"/>
       <c r="AR92" s="7"/>
       <c r="AS92" s="7"/>
+      <c r="AT92" s="7"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
@@ -7642,6 +7738,7 @@
       <c r="AQ93" s="7"/>
       <c r="AR93" s="7"/>
       <c r="AS93" s="7"/>
+      <c r="AT93" s="7"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
@@ -7713,6 +7810,7 @@
       <c r="AQ94" s="7"/>
       <c r="AR94" s="7"/>
       <c r="AS94" s="7"/>
+      <c r="AT94" s="7"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
@@ -7784,6 +7882,7 @@
       <c r="AQ95" s="7"/>
       <c r="AR95" s="7"/>
       <c r="AS95" s="7"/>
+      <c r="AT95" s="7"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
@@ -7874,6 +7973,7 @@
       <c r="AQ96" s="7"/>
       <c r="AR96" s="7"/>
       <c r="AS96" s="7"/>
+      <c r="AT96" s="7"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="inlineStr">
@@ -7940,6 +8040,7 @@
       <c r="AQ97" s="7"/>
       <c r="AR97" s="7"/>
       <c r="AS97" s="7"/>
+      <c r="AT97" s="7"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
@@ -8006,6 +8107,7 @@
       <c r="AQ98" s="7"/>
       <c r="AR98" s="7"/>
       <c r="AS98" s="7"/>
+      <c r="AT98" s="7"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
@@ -8072,6 +8174,7 @@
       <c r="AQ99" s="7"/>
       <c r="AR99" s="7"/>
       <c r="AS99" s="7"/>
+      <c r="AT99" s="7"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
@@ -8147,6 +8250,7 @@
       <c r="AQ100" s="7"/>
       <c r="AR100" s="7"/>
       <c r="AS100" s="7"/>
+      <c r="AT100" s="7"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
@@ -8213,6 +8317,7 @@
       <c r="AQ101" s="7"/>
       <c r="AR101" s="7"/>
       <c r="AS101" s="7"/>
+      <c r="AT101" s="7"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
@@ -8279,6 +8384,7 @@
       <c r="AQ102" s="7"/>
       <c r="AR102" s="7"/>
       <c r="AS102" s="7"/>
+      <c r="AT102" s="7"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="inlineStr">
@@ -8345,6 +8451,7 @@
       <c r="AQ103" s="7"/>
       <c r="AR103" s="7"/>
       <c r="AS103" s="7"/>
+      <c r="AT103" s="7"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="inlineStr">
@@ -8416,6 +8523,7 @@
       <c r="AQ104" s="7"/>
       <c r="AR104" s="7"/>
       <c r="AS104" s="7"/>
+      <c r="AT104" s="7"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
@@ -8482,6 +8590,7 @@
       <c r="AQ105" s="7"/>
       <c r="AR105" s="7"/>
       <c r="AS105" s="7"/>
+      <c r="AT105" s="7"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
@@ -8548,6 +8657,7 @@
       <c r="AQ106" s="7"/>
       <c r="AR106" s="7"/>
       <c r="AS106" s="7"/>
+      <c r="AT106" s="7"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
@@ -8614,6 +8724,7 @@
       <c r="AQ107" s="7"/>
       <c r="AR107" s="7"/>
       <c r="AS107" s="7"/>
+      <c r="AT107" s="7"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
@@ -8684,6 +8795,7 @@
       <c r="AQ108" s="7"/>
       <c r="AR108" s="7"/>
       <c r="AS108" s="7"/>
+      <c r="AT108" s="7"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="inlineStr">
@@ -8759,6 +8871,7 @@
       <c r="AQ109" s="7"/>
       <c r="AR109" s="7"/>
       <c r="AS109" s="7"/>
+      <c r="AT109" s="7"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
@@ -8842,6 +8955,7 @@
       <c r="AQ110" s="7"/>
       <c r="AR110" s="7"/>
       <c r="AS110" s="7"/>
+      <c r="AT110" s="7"/>
     </row>
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
@@ -8928,6 +9042,7 @@
       <c r="AQ111" s="7"/>
       <c r="AR111" s="7"/>
       <c r="AS111" s="7"/>
+      <c r="AT111" s="7"/>
     </row>
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
@@ -9011,6 +9126,7 @@
       <c r="AQ112" s="7"/>
       <c r="AR112" s="7"/>
       <c r="AS112" s="7"/>
+      <c r="AT112" s="7"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
@@ -9086,6 +9202,7 @@
       <c r="AQ113" s="7"/>
       <c r="AR113" s="7"/>
       <c r="AS113" s="7"/>
+      <c r="AT113" s="7"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="inlineStr">
@@ -9177,6 +9294,7 @@
       <c r="AQ114" s="7"/>
       <c r="AR114" s="7"/>
       <c r="AS114" s="7"/>
+      <c r="AT114" s="7"/>
     </row>
     <row r="115">
       <c r="A115" s="7" t="inlineStr">
@@ -9260,6 +9378,7 @@
       <c r="AQ115" s="7"/>
       <c r="AR115" s="7"/>
       <c r="AS115" s="7"/>
+      <c r="AT115" s="7"/>
     </row>
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
@@ -9351,6 +9470,7 @@
       <c r="AQ116" s="7"/>
       <c r="AR116" s="7"/>
       <c r="AS116" s="7"/>
+      <c r="AT116" s="7"/>
     </row>
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
@@ -9438,6 +9558,7 @@
       <c r="AQ117" s="7"/>
       <c r="AR117" s="7"/>
       <c r="AS117" s="7"/>
+      <c r="AT117" s="7"/>
     </row>
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
@@ -9525,6 +9646,7 @@
       <c r="AQ118" s="7"/>
       <c r="AR118" s="7"/>
       <c r="AS118" s="7"/>
+      <c r="AT118" s="7"/>
     </row>
     <row r="119">
       <c r="A119" s="7" t="inlineStr">
@@ -9608,6 +9730,7 @@
       <c r="AQ119" s="7"/>
       <c r="AR119" s="7"/>
       <c r="AS119" s="7"/>
+      <c r="AT119" s="7"/>
     </row>
     <row r="120">
       <c r="A120" s="7" t="inlineStr">
@@ -9683,6 +9806,7 @@
       <c r="AQ120" s="7"/>
       <c r="AR120" s="7"/>
       <c r="AS120" s="7"/>
+      <c r="AT120" s="7"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="inlineStr">
@@ -9770,6 +9894,7 @@
       <c r="AQ121" s="7"/>
       <c r="AR121" s="7"/>
       <c r="AS121" s="7"/>
+      <c r="AT121" s="7"/>
     </row>
     <row r="122">
       <c r="A122" s="7" t="inlineStr">
@@ -9857,6 +9982,7 @@
       <c r="AQ122" s="7"/>
       <c r="AR122" s="7"/>
       <c r="AS122" s="7"/>
+      <c r="AT122" s="7"/>
     </row>
     <row r="123">
       <c r="A123" s="7" t="inlineStr">
@@ -9932,6 +10058,7 @@
       <c r="AQ123" s="7"/>
       <c r="AR123" s="7"/>
       <c r="AS123" s="7"/>
+      <c r="AT123" s="7"/>
     </row>
     <row r="124">
       <c r="A124" s="7" t="inlineStr">
@@ -10015,6 +10142,7 @@
       <c r="AQ124" s="7"/>
       <c r="AR124" s="7"/>
       <c r="AS124" s="7"/>
+      <c r="AT124" s="7"/>
     </row>
     <row r="125">
       <c r="A125" s="7" t="inlineStr">
@@ -10090,6 +10218,7 @@
       <c r="AQ125" s="7"/>
       <c r="AR125" s="7"/>
       <c r="AS125" s="7"/>
+      <c r="AT125" s="7"/>
     </row>
     <row r="126">
       <c r="A126" s="7" t="inlineStr">
@@ -10165,6 +10294,7 @@
       <c r="AQ126" s="7"/>
       <c r="AR126" s="7"/>
       <c r="AS126" s="7"/>
+      <c r="AT126" s="7"/>
     </row>
     <row r="127">
       <c r="A127" s="7" t="inlineStr">
@@ -10244,6 +10374,7 @@
       <c r="AQ127" s="7"/>
       <c r="AR127" s="7"/>
       <c r="AS127" s="7"/>
+      <c r="AT127" s="7"/>
     </row>
     <row r="128">
       <c r="A128" s="7" t="inlineStr">
@@ -10323,6 +10454,7 @@
       <c r="AQ128" s="7"/>
       <c r="AR128" s="7"/>
       <c r="AS128" s="7"/>
+      <c r="AT128" s="7"/>
     </row>
     <row r="129">
       <c r="A129" s="7" t="inlineStr">
@@ -10402,6 +10534,7 @@
       <c r="AQ129" s="7"/>
       <c r="AR129" s="7"/>
       <c r="AS129" s="7"/>
+      <c r="AT129" s="7"/>
     </row>
     <row r="130">
       <c r="A130" s="7" t="inlineStr">
@@ -10477,6 +10610,7 @@
       <c r="AQ130" s="7"/>
       <c r="AR130" s="7"/>
       <c r="AS130" s="7"/>
+      <c r="AT130" s="7"/>
     </row>
     <row r="131">
       <c r="A131" s="7" t="inlineStr">
@@ -10560,6 +10694,7 @@
       <c r="AQ131" s="7"/>
       <c r="AR131" s="7"/>
       <c r="AS131" s="7"/>
+      <c r="AT131" s="7"/>
     </row>
     <row r="132">
       <c r="A132" s="7" t="inlineStr">
@@ -10647,6 +10782,7 @@
       <c r="AQ132" s="7"/>
       <c r="AR132" s="7"/>
       <c r="AS132" s="7"/>
+      <c r="AT132" s="7"/>
     </row>
     <row r="133">
       <c r="A133" s="7" t="inlineStr">
@@ -10734,6 +10870,7 @@
       <c r="AQ133" s="7"/>
       <c r="AR133" s="7"/>
       <c r="AS133" s="7"/>
+      <c r="AT133" s="7"/>
     </row>
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
@@ -10817,6 +10954,7 @@
       <c r="AQ134" s="7"/>
       <c r="AR134" s="7"/>
       <c r="AS134" s="7"/>
+      <c r="AT134" s="7"/>
     </row>
     <row r="135">
       <c r="A135" s="7" t="inlineStr">
@@ -10900,6 +11038,7 @@
       <c r="AQ135" s="7"/>
       <c r="AR135" s="7"/>
       <c r="AS135" s="7"/>
+      <c r="AT135" s="7"/>
     </row>
     <row r="136">
       <c r="A136" s="7" t="inlineStr">
@@ -10983,6 +11122,7 @@
       <c r="AQ136" s="7"/>
       <c r="AR136" s="7"/>
       <c r="AS136" s="7"/>
+      <c r="AT136" s="7"/>
     </row>
     <row r="137">
       <c r="A137" s="7" t="inlineStr">
@@ -11062,6 +11202,7 @@
       <c r="AQ137" s="7"/>
       <c r="AR137" s="7"/>
       <c r="AS137" s="7"/>
+      <c r="AT137" s="7"/>
     </row>
     <row r="138">
       <c r="A138" s="7" t="inlineStr">
@@ -11141,6 +11282,7 @@
       <c r="AQ138" s="7"/>
       <c r="AR138" s="7"/>
       <c r="AS138" s="7"/>
+      <c r="AT138" s="7"/>
     </row>
     <row r="139">
       <c r="A139" s="7" t="inlineStr">
@@ -11220,6 +11362,7 @@
       <c r="AQ139" s="7"/>
       <c r="AR139" s="7"/>
       <c r="AS139" s="7"/>
+      <c r="AT139" s="7"/>
     </row>
     <row r="140">
       <c r="A140" s="7" t="inlineStr">
@@ -11295,6 +11438,7 @@
       <c r="AQ140" s="7"/>
       <c r="AR140" s="7"/>
       <c r="AS140" s="7"/>
+      <c r="AT140" s="7"/>
     </row>
     <row r="141">
       <c r="A141" s="7" t="inlineStr">
@@ -11382,6 +11526,7 @@
       <c r="AQ141" s="7"/>
       <c r="AR141" s="7"/>
       <c r="AS141" s="7"/>
+      <c r="AT141" s="7"/>
     </row>
     <row r="142">
       <c r="A142" s="7" t="inlineStr">
@@ -11457,6 +11602,7 @@
       <c r="AQ142" s="7"/>
       <c r="AR142" s="7"/>
       <c r="AS142" s="7"/>
+      <c r="AT142" s="7"/>
     </row>
     <row r="143">
       <c r="A143" s="7" t="inlineStr">
@@ -11532,6 +11678,7 @@
       <c r="AQ143" s="7"/>
       <c r="AR143" s="7"/>
       <c r="AS143" s="7"/>
+      <c r="AT143" s="7"/>
     </row>
     <row r="144">
       <c r="A144" s="7" t="inlineStr">
@@ -11607,6 +11754,7 @@
       <c r="AQ144" s="7"/>
       <c r="AR144" s="7"/>
       <c r="AS144" s="7"/>
+      <c r="AT144" s="7"/>
     </row>
     <row r="145">
       <c r="A145" s="7" t="inlineStr">
@@ -11698,6 +11846,7 @@
       <c r="AQ145" s="7"/>
       <c r="AR145" s="7"/>
       <c r="AS145" s="7"/>
+      <c r="AT145" s="7"/>
     </row>
     <row r="146">
       <c r="A146" s="7" t="inlineStr">
@@ -11777,6 +11926,7 @@
       <c r="AQ146" s="7"/>
       <c r="AR146" s="7"/>
       <c r="AS146" s="7"/>
+      <c r="AT146" s="7"/>
     </row>
     <row r="147">
       <c r="A147" s="7" t="inlineStr">
@@ -11868,6 +12018,7 @@
       <c r="AQ147" s="7"/>
       <c r="AR147" s="7"/>
       <c r="AS147" s="7"/>
+      <c r="AT147" s="7"/>
     </row>
     <row r="148">
       <c r="A148" s="7" t="inlineStr">
@@ -11943,6 +12094,7 @@
       <c r="AQ148" s="7"/>
       <c r="AR148" s="7"/>
       <c r="AS148" s="7"/>
+      <c r="AT148" s="7"/>
     </row>
     <row r="149">
       <c r="A149" s="7" t="inlineStr">
@@ -12026,6 +12178,7 @@
       <c r="AQ149" s="7"/>
       <c r="AR149" s="7"/>
       <c r="AS149" s="7"/>
+      <c r="AT149" s="7"/>
     </row>
     <row r="150">
       <c r="A150" s="7" t="inlineStr">
@@ -12113,6 +12266,7 @@
       <c r="AQ150" s="7"/>
       <c r="AR150" s="7"/>
       <c r="AS150" s="7"/>
+      <c r="AT150" s="7"/>
     </row>
     <row r="151">
       <c r="A151" s="7" t="inlineStr">
@@ -12192,6 +12346,7 @@
       <c r="AQ151" s="7"/>
       <c r="AR151" s="7"/>
       <c r="AS151" s="7"/>
+      <c r="AT151" s="7"/>
     </row>
     <row r="152">
       <c r="A152" s="7" t="inlineStr">
@@ -12275,6 +12430,7 @@
       <c r="AQ152" s="7"/>
       <c r="AR152" s="7"/>
       <c r="AS152" s="7"/>
+      <c r="AT152" s="7"/>
     </row>
     <row r="153">
       <c r="A153" s="7" t="inlineStr">
@@ -12362,6 +12518,7 @@
       <c r="AQ153" s="7"/>
       <c r="AR153" s="7"/>
       <c r="AS153" s="7"/>
+      <c r="AT153" s="7"/>
     </row>
     <row r="154">
       <c r="A154" s="7" t="inlineStr">
@@ -12433,6 +12590,7 @@
       <c r="AQ154" s="7"/>
       <c r="AR154" s="7"/>
       <c r="AS154" s="7"/>
+      <c r="AT154" s="7"/>
     </row>
     <row r="155">
       <c r="A155" s="7" t="inlineStr">
@@ -12508,6 +12666,7 @@
       <c r="AQ155" s="7"/>
       <c r="AR155" s="7"/>
       <c r="AS155" s="7"/>
+      <c r="AT155" s="7"/>
     </row>
     <row r="156">
       <c r="A156" s="7" t="inlineStr">
@@ -12587,6 +12746,7 @@
       <c r="AQ156" s="7"/>
       <c r="AR156" s="7"/>
       <c r="AS156" s="7"/>
+      <c r="AT156" s="7"/>
     </row>
     <row r="157">
       <c r="A157" s="7" t="inlineStr">
@@ -12662,6 +12822,7 @@
       <c r="AQ157" s="7"/>
       <c r="AR157" s="7"/>
       <c r="AS157" s="7"/>
+      <c r="AT157" s="7"/>
     </row>
     <row r="158">
       <c r="A158" s="7" t="inlineStr">
@@ -12737,6 +12898,7 @@
       <c r="AQ158" s="7"/>
       <c r="AR158" s="7"/>
       <c r="AS158" s="7"/>
+      <c r="AT158" s="7"/>
     </row>
     <row r="159">
       <c r="A159" s="7" t="inlineStr">
@@ -12812,6 +12974,7 @@
       <c r="AQ159" s="7"/>
       <c r="AR159" s="7"/>
       <c r="AS159" s="7"/>
+      <c r="AT159" s="7"/>
     </row>
     <row r="160">
       <c r="A160" s="7" t="inlineStr">
@@ -12887,6 +13050,7 @@
       <c r="AQ160" s="7"/>
       <c r="AR160" s="7"/>
       <c r="AS160" s="7"/>
+      <c r="AT160" s="7"/>
     </row>
     <row r="161">
       <c r="A161" s="7" t="inlineStr">
@@ -12966,6 +13130,7 @@
       <c r="AQ161" s="7"/>
       <c r="AR161" s="7"/>
       <c r="AS161" s="7"/>
+      <c r="AT161" s="7"/>
     </row>
     <row r="162">
       <c r="A162" s="7" t="inlineStr">
@@ -13041,6 +13206,7 @@
       <c r="AQ162" s="7"/>
       <c r="AR162" s="7"/>
       <c r="AS162" s="7"/>
+      <c r="AT162" s="7"/>
     </row>
     <row r="163">
       <c r="A163" s="7" t="inlineStr">
@@ -13116,6 +13282,7 @@
       <c r="AQ163" s="7"/>
       <c r="AR163" s="7"/>
       <c r="AS163" s="7"/>
+      <c r="AT163" s="7"/>
     </row>
     <row r="164">
       <c r="A164" s="7" t="inlineStr">
@@ -13191,6 +13358,7 @@
       <c r="AQ164" s="7"/>
       <c r="AR164" s="7"/>
       <c r="AS164" s="7"/>
+      <c r="AT164" s="7"/>
     </row>
     <row r="165">
       <c r="A165" s="7" t="inlineStr">
@@ -13266,6 +13434,7 @@
       <c r="AQ165" s="7"/>
       <c r="AR165" s="7"/>
       <c r="AS165" s="7"/>
+      <c r="AT165" s="7"/>
     </row>
     <row r="166">
       <c r="A166" s="7" t="inlineStr">
@@ -13349,6 +13518,7 @@
       <c r="AQ166" s="7"/>
       <c r="AR166" s="7"/>
       <c r="AS166" s="7"/>
+      <c r="AT166" s="7"/>
     </row>
     <row r="167">
       <c r="A167" s="7" t="inlineStr">
@@ -13428,6 +13598,7 @@
       <c r="AQ167" s="7"/>
       <c r="AR167" s="7"/>
       <c r="AS167" s="7"/>
+      <c r="AT167" s="7"/>
     </row>
     <row r="168">
       <c r="A168" s="7" t="inlineStr">
@@ -13503,6 +13674,7 @@
       <c r="AQ168" s="7"/>
       <c r="AR168" s="7"/>
       <c r="AS168" s="7"/>
+      <c r="AT168" s="7"/>
     </row>
     <row r="169">
       <c r="A169" s="7" t="inlineStr">
@@ -13578,6 +13750,7 @@
       <c r="AQ169" s="7"/>
       <c r="AR169" s="7"/>
       <c r="AS169" s="7"/>
+      <c r="AT169" s="7"/>
     </row>
     <row r="170">
       <c r="A170" s="7" t="inlineStr">
@@ -13657,6 +13830,7 @@
       <c r="AQ170" s="7"/>
       <c r="AR170" s="7"/>
       <c r="AS170" s="7"/>
+      <c r="AT170" s="7"/>
     </row>
     <row r="171">
       <c r="A171" s="7" t="inlineStr">
@@ -13728,6 +13902,7 @@
       <c r="AQ171" s="7"/>
       <c r="AR171" s="7"/>
       <c r="AS171" s="7"/>
+      <c r="AT171" s="7"/>
     </row>
     <row r="172">
       <c r="A172" s="7" t="inlineStr">
@@ -13799,6 +13974,7 @@
       <c r="AQ172" s="7"/>
       <c r="AR172" s="7"/>
       <c r="AS172" s="7"/>
+      <c r="AT172" s="7"/>
     </row>
     <row r="173">
       <c r="A173" s="7" t="inlineStr">
@@ -13878,6 +14054,7 @@
       <c r="AQ173" s="7"/>
       <c r="AR173" s="7"/>
       <c r="AS173" s="7"/>
+      <c r="AT173" s="7"/>
     </row>
     <row r="174">
       <c r="A174" s="7" t="inlineStr">
@@ -13953,6 +14130,7 @@
       <c r="AQ174" s="7"/>
       <c r="AR174" s="7"/>
       <c r="AS174" s="7"/>
+      <c r="AT174" s="7"/>
     </row>
     <row r="175">
       <c r="A175" s="7" t="inlineStr">
@@ -14032,6 +14210,7 @@
       <c r="AQ175" s="7"/>
       <c r="AR175" s="7"/>
       <c r="AS175" s="7"/>
+      <c r="AT175" s="7"/>
     </row>
     <row r="176">
       <c r="A176" s="7" t="inlineStr">
@@ -14107,6 +14286,7 @@
       <c r="AQ176" s="7"/>
       <c r="AR176" s="7"/>
       <c r="AS176" s="7"/>
+      <c r="AT176" s="7"/>
     </row>
     <row r="177">
       <c r="A177" s="7" t="inlineStr">
@@ -14182,6 +14362,7 @@
       <c r="AQ177" s="7"/>
       <c r="AR177" s="7"/>
       <c r="AS177" s="7"/>
+      <c r="AT177" s="7"/>
     </row>
     <row r="178">
       <c r="A178" s="7" t="inlineStr">
@@ -14257,6 +14438,7 @@
       <c r="AQ178" s="7"/>
       <c r="AR178" s="7"/>
       <c r="AS178" s="7"/>
+      <c r="AT178" s="7"/>
     </row>
     <row r="179">
       <c r="A179" s="7" t="inlineStr">
@@ -14332,6 +14514,7 @@
       <c r="AQ179" s="7"/>
       <c r="AR179" s="7"/>
       <c r="AS179" s="7"/>
+      <c r="AT179" s="7"/>
     </row>
     <row r="180">
       <c r="A180" s="7" t="inlineStr">
@@ -14407,6 +14590,7 @@
       <c r="AQ180" s="7"/>
       <c r="AR180" s="7"/>
       <c r="AS180" s="7"/>
+      <c r="AT180" s="7"/>
     </row>
     <row r="181">
       <c r="A181" s="7" t="inlineStr">
@@ -14482,6 +14666,7 @@
       <c r="AQ181" s="7"/>
       <c r="AR181" s="7"/>
       <c r="AS181" s="7"/>
+      <c r="AT181" s="7"/>
     </row>
     <row r="182">
       <c r="A182" s="7" t="inlineStr">
@@ -14557,6 +14742,7 @@
       <c r="AQ182" s="7"/>
       <c r="AR182" s="7"/>
       <c r="AS182" s="7"/>
+      <c r="AT182" s="7"/>
     </row>
     <row r="183">
       <c r="A183" s="7" t="inlineStr">
@@ -14632,6 +14818,7 @@
       <c r="AQ183" s="7"/>
       <c r="AR183" s="7"/>
       <c r="AS183" s="7"/>
+      <c r="AT183" s="7"/>
     </row>
     <row r="184">
       <c r="A184" s="7" t="inlineStr">
@@ -14703,6 +14890,7 @@
       <c r="AQ184" s="7"/>
       <c r="AR184" s="7"/>
       <c r="AS184" s="7"/>
+      <c r="AT184" s="7"/>
     </row>
     <row r="185">
       <c r="A185" s="7" t="inlineStr">
@@ -14778,6 +14966,7 @@
       <c r="AQ185" s="7"/>
       <c r="AR185" s="7"/>
       <c r="AS185" s="7"/>
+      <c r="AT185" s="7"/>
     </row>
     <row r="186">
       <c r="A186" s="7" t="inlineStr">
@@ -14853,6 +15042,7 @@
       <c r="AQ186" s="7"/>
       <c r="AR186" s="7"/>
       <c r="AS186" s="7"/>
+      <c r="AT186" s="7"/>
     </row>
     <row r="187">
       <c r="A187" s="7" t="inlineStr">
@@ -14932,6 +15122,7 @@
       <c r="AQ187" s="7"/>
       <c r="AR187" s="7"/>
       <c r="AS187" s="7"/>
+      <c r="AT187" s="7"/>
     </row>
     <row r="188">
       <c r="A188" s="7" t="inlineStr">
@@ -15011,6 +15202,7 @@
       <c r="AQ188" s="7"/>
       <c r="AR188" s="7"/>
       <c r="AS188" s="7"/>
+      <c r="AT188" s="7"/>
     </row>
     <row r="189">
       <c r="A189" s="7" t="inlineStr">
@@ -15090,6 +15282,7 @@
       <c r="AQ189" s="7"/>
       <c r="AR189" s="7"/>
       <c r="AS189" s="7"/>
+      <c r="AT189" s="7"/>
     </row>
     <row r="190">
       <c r="A190" s="7" t="inlineStr">
@@ -15169,6 +15362,7 @@
       <c r="AQ190" s="7"/>
       <c r="AR190" s="7"/>
       <c r="AS190" s="7"/>
+      <c r="AT190" s="7"/>
     </row>
     <row r="191">
       <c r="A191" s="7" t="inlineStr">
@@ -15248,6 +15442,7 @@
       <c r="AQ191" s="7"/>
       <c r="AR191" s="7"/>
       <c r="AS191" s="7"/>
+      <c r="AT191" s="7"/>
     </row>
     <row r="192">
       <c r="A192" s="7" t="inlineStr">
@@ -15327,6 +15522,7 @@
       <c r="AQ192" s="7"/>
       <c r="AR192" s="7"/>
       <c r="AS192" s="7"/>
+      <c r="AT192" s="7"/>
     </row>
     <row r="193">
       <c r="A193" s="7" t="inlineStr">
@@ -15410,6 +15606,7 @@
       </c>
       <c r="AR193" s="7"/>
       <c r="AS193" s="7"/>
+      <c r="AT193" s="7"/>
     </row>
     <row r="194">
       <c r="A194" s="7" t="inlineStr">
@@ -15493,6 +15690,7 @@
       </c>
       <c r="AR194" s="7"/>
       <c r="AS194" s="7"/>
+      <c r="AT194" s="7"/>
     </row>
     <row r="195">
       <c r="A195" s="7" t="inlineStr">
@@ -15576,6 +15774,7 @@
       </c>
       <c r="AR195" s="7"/>
       <c r="AS195" s="7"/>
+      <c r="AT195" s="7"/>
     </row>
     <row r="196">
       <c r="A196" s="7" t="inlineStr">
@@ -15651,6 +15850,7 @@
       <c r="AQ196" s="7"/>
       <c r="AR196" s="7"/>
       <c r="AS196" s="7"/>
+      <c r="AT196" s="7"/>
     </row>
     <row r="197">
       <c r="A197" s="7" t="inlineStr">
@@ -15734,6 +15934,7 @@
       </c>
       <c r="AR197" s="7"/>
       <c r="AS197" s="7"/>
+      <c r="AT197" s="7"/>
     </row>
     <row r="198">
       <c r="A198" s="7" t="inlineStr">
@@ -15809,6 +16010,7 @@
       <c r="AQ198" s="7"/>
       <c r="AR198" s="7"/>
       <c r="AS198" s="7"/>
+      <c r="AT198" s="7"/>
     </row>
     <row r="199">
       <c r="A199" s="7" t="inlineStr">
@@ -15892,6 +16094,7 @@
       </c>
       <c r="AR199" s="7"/>
       <c r="AS199" s="7"/>
+      <c r="AT199" s="7"/>
     </row>
     <row r="200">
       <c r="A200" s="7" t="inlineStr">
@@ -15975,6 +16178,7 @@
       </c>
       <c r="AR200" s="7"/>
       <c r="AS200" s="7"/>
+      <c r="AT200" s="7"/>
     </row>
     <row r="201">
       <c r="A201" s="7" t="inlineStr">
@@ -16050,6 +16254,7 @@
       </c>
       <c r="AR201" s="7"/>
       <c r="AS201" s="7"/>
+      <c r="AT201" s="7"/>
     </row>
     <row r="202">
       <c r="A202" s="7" t="inlineStr">
@@ -16133,6 +16338,7 @@
       </c>
       <c r="AR202" s="7"/>
       <c r="AS202" s="7"/>
+      <c r="AT202" s="7"/>
     </row>
     <row r="203">
       <c r="A203" s="7" t="inlineStr">
@@ -16216,6 +16422,7 @@
       </c>
       <c r="AR203" s="7"/>
       <c r="AS203" s="7"/>
+      <c r="AT203" s="7"/>
     </row>
     <row r="204">
       <c r="A204" s="7" t="inlineStr">
@@ -16303,6 +16510,7 @@
         </is>
       </c>
       <c r="AS204" s="7"/>
+      <c r="AT204" s="7"/>
     </row>
     <row r="205">
       <c r="A205" s="7" t="inlineStr">
@@ -16390,6 +16598,7 @@
       </c>
       <c r="AR205" s="7"/>
       <c r="AS205" s="7"/>
+      <c r="AT205" s="7"/>
     </row>
     <row r="206">
       <c r="A206" s="7" t="inlineStr">
@@ -16477,6 +16686,7 @@
         </is>
       </c>
       <c r="AS206" s="7"/>
+      <c r="AT206" s="7"/>
     </row>
     <row r="207">
       <c r="A207" s="7" t="inlineStr">
@@ -16556,6 +16766,7 @@
       </c>
       <c r="AR207" s="7"/>
       <c r="AS207" s="7"/>
+      <c r="AT207" s="7"/>
     </row>
     <row r="208">
       <c r="A208" s="7" t="inlineStr">
@@ -16639,6 +16850,7 @@
         </is>
       </c>
       <c r="AS208" s="7"/>
+      <c r="AT208" s="7"/>
     </row>
     <row r="209">
       <c r="A209" s="7" t="inlineStr">
@@ -16726,6 +16938,7 @@
         </is>
       </c>
       <c r="AS209" s="7"/>
+      <c r="AT209" s="7"/>
     </row>
     <row r="210">
       <c r="A210" s="7" t="inlineStr">
@@ -16809,6 +17022,7 @@
         </is>
       </c>
       <c r="AS210" s="7"/>
+      <c r="AT210" s="7"/>
     </row>
     <row r="211">
       <c r="A211" s="7" t="inlineStr">
@@ -16884,6 +17098,7 @@
       <c r="AQ211" s="7"/>
       <c r="AR211" s="7"/>
       <c r="AS211" s="7"/>
+      <c r="AT211" s="7"/>
     </row>
     <row r="212">
       <c r="A212" s="7" t="inlineStr">
@@ -16959,6 +17174,7 @@
       </c>
       <c r="AR212" s="7"/>
       <c r="AS212" s="7"/>
+      <c r="AT212" s="7"/>
     </row>
     <row r="213">
       <c r="A213" s="7" t="inlineStr">
@@ -17038,6 +17254,7 @@
         </is>
       </c>
       <c r="AS213" s="7"/>
+      <c r="AT213" s="7"/>
     </row>
     <row r="214">
       <c r="A214" s="7" t="inlineStr">
@@ -17113,6 +17330,7 @@
       </c>
       <c r="AR214" s="7"/>
       <c r="AS214" s="7"/>
+      <c r="AT214" s="7"/>
     </row>
     <row r="215">
       <c r="A215" s="7" t="inlineStr">
@@ -17184,6 +17402,7 @@
       <c r="AQ215" s="7"/>
       <c r="AR215" s="7"/>
       <c r="AS215" s="7"/>
+      <c r="AT215" s="7"/>
     </row>
     <row r="216">
       <c r="A216" s="7" t="inlineStr">
@@ -17255,6 +17474,7 @@
       <c r="AQ216" s="7"/>
       <c r="AR216" s="7"/>
       <c r="AS216" s="7"/>
+      <c r="AT216" s="7"/>
     </row>
     <row r="217">
       <c r="A217" s="7" t="inlineStr">
@@ -17330,6 +17550,7 @@
         </is>
       </c>
       <c r="AS217" s="7"/>
+      <c r="AT217" s="7"/>
     </row>
     <row r="218">
       <c r="A218" s="7" t="inlineStr">
@@ -17401,6 +17622,7 @@
       <c r="AQ218" s="7"/>
       <c r="AR218" s="7"/>
       <c r="AS218" s="7"/>
+      <c r="AT218" s="7"/>
     </row>
     <row r="219">
       <c r="A219" s="7" t="inlineStr">
@@ -17476,6 +17698,7 @@
         </is>
       </c>
       <c r="AS219" s="7"/>
+      <c r="AT219" s="7"/>
     </row>
     <row r="220">
       <c r="A220" s="7" t="inlineStr">
@@ -17547,6 +17770,7 @@
       <c r="AQ220" s="7"/>
       <c r="AR220" s="7"/>
       <c r="AS220" s="7"/>
+      <c r="AT220" s="7"/>
     </row>
     <row r="221">
       <c r="A221" s="7" t="inlineStr">
@@ -17622,6 +17846,7 @@
         </is>
       </c>
       <c r="AS221" s="7"/>
+      <c r="AT221" s="7"/>
     </row>
     <row r="222">
       <c r="A222" s="7" t="inlineStr">
@@ -17701,6 +17926,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AT222" s="7"/>
     </row>
     <row r="223">
       <c r="A223" s="7" t="inlineStr">
@@ -17776,6 +18002,523 @@
         </is>
       </c>
       <c r="AS223" s="7"/>
+      <c r="AT223" s="7"/>
+    </row>
+    <row r="224">
+      <c r="A224" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_216</t>
+        </is>
+      </c>
+      <c r="B224" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">화면</t>
+        </is>
+      </c>
+      <c r="C224" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">바닥 덮임</t>
+        </is>
+      </c>
+      <c r="D224" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">정지 중</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼 막(정지) 중 · 판 전환 직후에도 전투 바닥이 화면을 다 덮는가?(하단 띠 · 왼쪽 빈 구역 없음)</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t xml:space="preserve">결함 ① · 원인 = #203/#207 정지 goto 가 바닥 따라가기를 건너뜀 → LateUpdate · AT 실측: 처음부터 → 바로가기 S3 막 중 전폭 덮임(28 의 왼쪽 빈 구역 없음) · 세로 큰 창 하단 띠는 인앱 창 높이로 못 봄</t>
+        </is>
+      </c>
+      <c r="G224" s="7"/>
+      <c r="H224" s="7"/>
+      <c r="I224" s="7"/>
+      <c r="J224" s="7"/>
+      <c r="K224" s="7"/>
+      <c r="L224" s="7"/>
+      <c r="M224" s="7"/>
+      <c r="N224" s="7"/>
+      <c r="O224" s="7"/>
+      <c r="P224" s="7"/>
+      <c r="Q224" s="7"/>
+      <c r="R224" s="7"/>
+      <c r="S224" s="7"/>
+      <c r="T224" s="7"/>
+      <c r="U224" s="7"/>
+      <c r="V224" s="7"/>
+      <c r="W224" s="7"/>
+      <c r="X224" s="7"/>
+      <c r="Y224" s="7"/>
+      <c r="Z224" s="7"/>
+      <c r="AA224" s="7"/>
+      <c r="AB224" s="7"/>
+      <c r="AC224" s="7"/>
+      <c r="AD224" s="7"/>
+      <c r="AE224" s="7"/>
+      <c r="AF224" s="7"/>
+      <c r="AG224" s="7"/>
+      <c r="AH224" s="7"/>
+      <c r="AI224" s="7"/>
+      <c r="AJ224" s="7"/>
+      <c r="AK224" s="7"/>
+      <c r="AL224" s="7"/>
+      <c r="AM224" s="7"/>
+      <c r="AN224" s="7"/>
+      <c r="AO224" s="7"/>
+      <c r="AP224" s="7"/>
+      <c r="AQ224" s="7"/>
+      <c r="AR224" s="7"/>
+      <c r="AS224" s="7"/>
+      <c r="AT224" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_217</t>
+        </is>
+      </c>
+      <c r="B225" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C225" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">합체 수치</t>
+        </is>
+      </c>
+      <c r="D225" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 합체 막</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 첫 도전 합체 막에서 합체하면 「화력 n → m」이 0 이 아닌가?</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t xml:space="preserve">결함 ③ · 원인 = 도전 시작부터 정지 → RefreshFireRate 안 돎 → 발사 줄 빔 · 정지 중에도 배분 · AT 못 봄(자연 진행 필요)</t>
+        </is>
+      </c>
+      <c r="G225" s="7"/>
+      <c r="H225" s="7"/>
+      <c r="I225" s="7"/>
+      <c r="J225" s="7"/>
+      <c r="K225" s="7"/>
+      <c r="L225" s="7"/>
+      <c r="M225" s="7"/>
+      <c r="N225" s="7"/>
+      <c r="O225" s="7"/>
+      <c r="P225" s="7"/>
+      <c r="Q225" s="7"/>
+      <c r="R225" s="7"/>
+      <c r="S225" s="7"/>
+      <c r="T225" s="7"/>
+      <c r="U225" s="7"/>
+      <c r="V225" s="7"/>
+      <c r="W225" s="7"/>
+      <c r="X225" s="7"/>
+      <c r="Y225" s="7"/>
+      <c r="Z225" s="7"/>
+      <c r="AA225" s="7"/>
+      <c r="AB225" s="7"/>
+      <c r="AC225" s="7"/>
+      <c r="AD225" s="7"/>
+      <c r="AE225" s="7"/>
+      <c r="AF225" s="7"/>
+      <c r="AG225" s="7"/>
+      <c r="AH225" s="7"/>
+      <c r="AI225" s="7"/>
+      <c r="AJ225" s="7"/>
+      <c r="AK225" s="7"/>
+      <c r="AL225" s="7"/>
+      <c r="AM225" s="7"/>
+      <c r="AN225" s="7"/>
+      <c r="AO225" s="7"/>
+      <c r="AP225" s="7"/>
+      <c r="AQ225" s="7"/>
+      <c r="AR225" s="7"/>
+      <c r="AS225" s="7"/>
+      <c r="AT225" s="7"/>
+    </row>
+    <row r="226">
+      <c r="A226" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_218</t>
+        </is>
+      </c>
+      <c r="B226" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C226" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도전 추격</t>
+        </is>
+      </c>
+      <c r="D226" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B 혼자</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 도전에서 B 가 나섰고 드론 재고 · 필드 드론이 0 이면 남은 적에게 걸어가 깨우는가(멈춰 시간 초과 없음)?</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t xml:space="preserve">결함 ④ (b) · 원인 = 잠든 적(깨움 6)이 9.2 안이면 멈춤 + B 는 칠 수단 0 · 첫 고침(2fff44d)은 SetFireLines 가 B 에 A 줄을 써 안 걸림(실측 멈춤) → 5d04f2f 보정 · AT: B 혼자(Auto 끔) 남은 23→11→10→7 진행 뒤 시간 초과(B 드론만 화력) — 「완전 정지」는 안 보였으나 확정 못 함</t>
+        </is>
+      </c>
+      <c r="G226" s="7"/>
+      <c r="H226" s="7"/>
+      <c r="I226" s="7"/>
+      <c r="J226" s="7"/>
+      <c r="K226" s="7"/>
+      <c r="L226" s="7"/>
+      <c r="M226" s="7"/>
+      <c r="N226" s="7"/>
+      <c r="O226" s="7"/>
+      <c r="P226" s="7"/>
+      <c r="Q226" s="7"/>
+      <c r="R226" s="7"/>
+      <c r="S226" s="7"/>
+      <c r="T226" s="7"/>
+      <c r="U226" s="7"/>
+      <c r="V226" s="7"/>
+      <c r="W226" s="7"/>
+      <c r="X226" s="7"/>
+      <c r="Y226" s="7"/>
+      <c r="Z226" s="7"/>
+      <c r="AA226" s="7"/>
+      <c r="AB226" s="7"/>
+      <c r="AC226" s="7"/>
+      <c r="AD226" s="7"/>
+      <c r="AE226" s="7"/>
+      <c r="AF226" s="7"/>
+      <c r="AG226" s="7"/>
+      <c r="AH226" s="7"/>
+      <c r="AI226" s="7"/>
+      <c r="AJ226" s="7"/>
+      <c r="AK226" s="7"/>
+      <c r="AL226" s="7"/>
+      <c r="AM226" s="7"/>
+      <c r="AN226" s="7"/>
+      <c r="AO226" s="7"/>
+      <c r="AP226" s="7"/>
+      <c r="AQ226" s="7"/>
+      <c r="AR226" s="7"/>
+      <c r="AS226" s="7"/>
+      <c r="AT226" s="7"/>
+    </row>
+    <row r="227">
+      <c r="A227" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_219</t>
+        </is>
+      </c>
+      <c r="B227" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">연출</t>
+        </is>
+      </c>
+      <c r="C227" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">태그 스킬 고리</t>
+        </is>
+      </c>
+      <c r="D227" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">승리 뒤</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S6 보스를 태그 스킬로 처치한 뒤 고리 파동이 한 번만 지나가고 화면을 덮지 않는가?</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t xml:space="preserve">결함 ⑤ · 원인 = 끝난 판 Tick 이 이번 틱 사건을 안 비워 프레임마다 고리 재생성 · 고침 + 시험 AfterWin_TickClearsThisTickEvents · AT 화면 재현 못 함</t>
+        </is>
+      </c>
+      <c r="G227" s="7"/>
+      <c r="H227" s="7"/>
+      <c r="I227" s="7"/>
+      <c r="J227" s="7"/>
+      <c r="K227" s="7"/>
+      <c r="L227" s="7"/>
+      <c r="M227" s="7"/>
+      <c r="N227" s="7"/>
+      <c r="O227" s="7"/>
+      <c r="P227" s="7"/>
+      <c r="Q227" s="7"/>
+      <c r="R227" s="7"/>
+      <c r="S227" s="7"/>
+      <c r="T227" s="7"/>
+      <c r="U227" s="7"/>
+      <c r="V227" s="7"/>
+      <c r="W227" s="7"/>
+      <c r="X227" s="7"/>
+      <c r="Y227" s="7"/>
+      <c r="Z227" s="7"/>
+      <c r="AA227" s="7"/>
+      <c r="AB227" s="7"/>
+      <c r="AC227" s="7"/>
+      <c r="AD227" s="7"/>
+      <c r="AE227" s="7"/>
+      <c r="AF227" s="7"/>
+      <c r="AG227" s="7"/>
+      <c r="AH227" s="7"/>
+      <c r="AI227" s="7"/>
+      <c r="AJ227" s="7"/>
+      <c r="AK227" s="7"/>
+      <c r="AL227" s="7"/>
+      <c r="AM227" s="7"/>
+      <c r="AN227" s="7"/>
+      <c r="AO227" s="7"/>
+      <c r="AP227" s="7"/>
+      <c r="AQ227" s="7"/>
+      <c r="AR227" s="7"/>
+      <c r="AS227" s="7"/>
+      <c r="AT227" s="7"/>
+    </row>
+    <row r="228">
+      <c r="A228" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_220</t>
+        </is>
+      </c>
+      <c r="B228" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼</t>
+        </is>
+      </c>
+      <c r="C228" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">누를 곳 테두리</t>
+        </is>
+      </c>
+      <c r="D228" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#210</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼 국면마다 눌러야 할 자리(보드 칸 · 탭 · 단추 · 조합표 행 · 강화 · 도전 · 조립 · 해금 · 합체)에 노란 테두리가 서는가?</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#210 · AT 실측: S3 마운트 칸 · T1 빈 칸 테두리 ✅ · 강화 단추 · 합체 원형은 46d56cd 에서 단추 뒤로 옮김(그 뒤 화면 못 봄) · S5 · T4 · 탭은 못 봄</t>
+        </is>
+      </c>
+      <c r="G228" s="7"/>
+      <c r="H228" s="7"/>
+      <c r="I228" s="7"/>
+      <c r="J228" s="7"/>
+      <c r="K228" s="7"/>
+      <c r="L228" s="7"/>
+      <c r="M228" s="7"/>
+      <c r="N228" s="7"/>
+      <c r="O228" s="7"/>
+      <c r="P228" s="7"/>
+      <c r="Q228" s="7"/>
+      <c r="R228" s="7"/>
+      <c r="S228" s="7"/>
+      <c r="T228" s="7"/>
+      <c r="U228" s="7"/>
+      <c r="V228" s="7"/>
+      <c r="W228" s="7"/>
+      <c r="X228" s="7"/>
+      <c r="Y228" s="7"/>
+      <c r="Z228" s="7"/>
+      <c r="AA228" s="7"/>
+      <c r="AB228" s="7"/>
+      <c r="AC228" s="7"/>
+      <c r="AD228" s="7"/>
+      <c r="AE228" s="7"/>
+      <c r="AF228" s="7"/>
+      <c r="AG228" s="7"/>
+      <c r="AH228" s="7"/>
+      <c r="AI228" s="7"/>
+      <c r="AJ228" s="7"/>
+      <c r="AK228" s="7"/>
+      <c r="AL228" s="7"/>
+      <c r="AM228" s="7"/>
+      <c r="AN228" s="7"/>
+      <c r="AO228" s="7"/>
+      <c r="AP228" s="7"/>
+      <c r="AQ228" s="7"/>
+      <c r="AR228" s="7"/>
+      <c r="AS228" s="7"/>
+      <c r="AT228" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_221</t>
+        </is>
+      </c>
+      <c r="B229" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UI</t>
+        </is>
+      </c>
+      <c r="C229" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">팔레트 세로 휠</t>
+        </is>
+      </c>
+      <c r="D229" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#211</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t xml:space="preserve">팔레트 단추 줄에 세로 스크롤 막대가 없고 가로로만 밀리는가?</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#211 · 단추 변에서 가로 바 높이 빼기 + 세로 막대 GUIStyle.none · AT 화면 캡처가 팔레트를 못 담아 못 봄</t>
+        </is>
+      </c>
+      <c r="G229" s="7"/>
+      <c r="H229" s="7"/>
+      <c r="I229" s="7"/>
+      <c r="J229" s="7"/>
+      <c r="K229" s="7"/>
+      <c r="L229" s="7"/>
+      <c r="M229" s="7"/>
+      <c r="N229" s="7"/>
+      <c r="O229" s="7"/>
+      <c r="P229" s="7"/>
+      <c r="Q229" s="7"/>
+      <c r="R229" s="7"/>
+      <c r="S229" s="7"/>
+      <c r="T229" s="7"/>
+      <c r="U229" s="7"/>
+      <c r="V229" s="7"/>
+      <c r="W229" s="7"/>
+      <c r="X229" s="7"/>
+      <c r="Y229" s="7"/>
+      <c r="Z229" s="7"/>
+      <c r="AA229" s="7"/>
+      <c r="AB229" s="7"/>
+      <c r="AC229" s="7"/>
+      <c r="AD229" s="7"/>
+      <c r="AE229" s="7"/>
+      <c r="AF229" s="7"/>
+      <c r="AG229" s="7"/>
+      <c r="AH229" s="7"/>
+      <c r="AI229" s="7"/>
+      <c r="AJ229" s="7"/>
+      <c r="AK229" s="7"/>
+      <c r="AL229" s="7"/>
+      <c r="AM229" s="7"/>
+      <c r="AN229" s="7"/>
+      <c r="AO229" s="7"/>
+      <c r="AP229" s="7"/>
+      <c r="AQ229" s="7"/>
+      <c r="AR229" s="7"/>
+      <c r="AS229" s="7"/>
+      <c r="AT229" s="7"/>
+    </row>
+    <row r="230">
+      <c r="A230" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_222</t>
+        </is>
+      </c>
+      <c r="B230" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UI</t>
+        </is>
+      </c>
+      <c r="C230" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">메인 메뉴 문구</t>
+        </is>
+      </c>
+      <c r="D230" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#212</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t xml:space="preserve">「게임 시작」 아래에 「플레이 시, BGM 및 사운드가 자동 재생이 진행되니, 이 점 유의해주시면 감사하겠습니다.」가 보이는가?</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#212 · AT 실측: 단추 폭 안 세 줄로 보임 ✅</t>
+        </is>
+      </c>
+      <c r="G230" s="7"/>
+      <c r="H230" s="7"/>
+      <c r="I230" s="7"/>
+      <c r="J230" s="7"/>
+      <c r="K230" s="7"/>
+      <c r="L230" s="7"/>
+      <c r="M230" s="7"/>
+      <c r="N230" s="7"/>
+      <c r="O230" s="7"/>
+      <c r="P230" s="7"/>
+      <c r="Q230" s="7"/>
+      <c r="R230" s="7"/>
+      <c r="S230" s="7"/>
+      <c r="T230" s="7"/>
+      <c r="U230" s="7"/>
+      <c r="V230" s="7"/>
+      <c r="W230" s="7"/>
+      <c r="X230" s="7"/>
+      <c r="Y230" s="7"/>
+      <c r="Z230" s="7"/>
+      <c r="AA230" s="7"/>
+      <c r="AB230" s="7"/>
+      <c r="AC230" s="7"/>
+      <c r="AD230" s="7"/>
+      <c r="AE230" s="7"/>
+      <c r="AF230" s="7"/>
+      <c r="AG230" s="7"/>
+      <c r="AH230" s="7"/>
+      <c r="AI230" s="7"/>
+      <c r="AJ230" s="7"/>
+      <c r="AK230" s="7"/>
+      <c r="AL230" s="7"/>
+      <c r="AM230" s="7"/>
+      <c r="AN230" s="7"/>
+      <c r="AO230" s="7"/>
+      <c r="AP230" s="7"/>
+      <c r="AQ230" s="7"/>
+      <c r="AR230" s="7"/>
+      <c r="AS230" s="7"/>
+      <c r="AT230" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="26">
@@ -17804,9 +18547,9 @@
     <mergeCell ref="B92:B99"/>
     <mergeCell ref="B100:B106"/>
     <mergeCell ref="B107:B111"/>
-    <mergeCell ref="G7:AS7"/>
+    <mergeCell ref="G7:AT7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:AS223">
+  <conditionalFormatting sqref="G9:AT230">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
QA AU(22d9191 · CID_231~236)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -202,8 +202,9 @@
     <col min="44" max="44" width="12" customWidth="1"/>
     <col min="45" max="45" width="12" customWidth="1"/>
     <col min="46" max="46" width="12" customWidth="1"/>
-    <col min="47" max="47" width="11" customWidth="1"/>
+    <col min="47" max="47" width="12" customWidth="1"/>
     <col min="48" max="48" width="11" customWidth="1"/>
+    <col min="49" max="49" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -516,6 +517,11 @@
       <c r="AT6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">8133 5d04f2f 갈아엎음(10-20 00:04) · 사용자 육안(10-19 23:4x · 8b54a82) 결함 ①③④⑤ + #210 · #211 · #212 ‖ 보이는 창 재확인 일부. 시험 1684/1678/0/6 · 전투 12줄 불변.</t>
+        </is>
+      </c>
+      <c r="AU6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8133 22d9191 갈아엎음(10-20 11:20) · 사용자 육안(10-20 아침) #213~#218 · 결함 ⑨ 가름 ‖ 시험 1691/1685/0/6 · 전투 12줄 = #217 로 네 줄 바뀜(S2 전 LoseTimeout 53/55 · 판정 요청) · 프리셋 표 불변.</t>
         </is>
       </c>
     </row>
@@ -586,14 +592,15 @@
       <c r="AR7" s="2"/>
       <c r="AS7" s="2"/>
       <c r="AT7" s="2"/>
-      <c r="AU7" s="2" t="inlineStr">
+      <c r="AU7" s="2"/>
+      <c r="AV7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">버전</t>
         </is>
       </c>
-      <c r="AV7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5d04f2f</t>
+      <c r="AW7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">22d9191</t>
         </is>
       </c>
     </row>
@@ -818,11 +825,16 @@
       </c>
       <c r="AU8" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">22d9191</t>
+        </is>
+      </c>
+      <c r="AV8" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">PASSrate</t>
         </is>
       </c>
-      <c r="AV8" s="7">
-        <f>COUNTIF(AT9:AT230,"Pass")</f>
+      <c r="AW8" s="7">
+        <f>COUNTIF(AU9:AU236,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -932,13 +944,14 @@
       <c r="AR9" s="7"/>
       <c r="AS9" s="7"/>
       <c r="AT9" s="7"/>
-      <c r="AU9" s="2" t="inlineStr">
+      <c r="AU9" s="7"/>
+      <c r="AV9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FAILrate</t>
         </is>
       </c>
-      <c r="AV9" s="7">
-        <f>COUNTIF(AT9:AT230,"Fail")+COUNTIF(AT9:AT230,"Broken")</f>
+      <c r="AW9" s="7">
+        <f>COUNTIF(AU9:AU236,"Fail")+COUNTIF(AU9:AU236,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -1012,13 +1025,14 @@
       <c r="AR10" s="7"/>
       <c r="AS10" s="7"/>
       <c r="AT10" s="7"/>
-      <c r="AU10" s="2" t="inlineStr">
+      <c r="AU10" s="7"/>
+      <c r="AV10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">N/A</t>
         </is>
       </c>
-      <c r="AV10" s="7">
-        <f>COUNTIF(AT9:AT230,"N/A")</f>
+      <c r="AW10" s="7">
+        <f>COUNTIF(AU9:AU236,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -1092,13 +1106,14 @@
       <c r="AR11" s="7"/>
       <c r="AS11" s="7"/>
       <c r="AT11" s="7"/>
-      <c r="AU11" s="2" t="inlineStr">
+      <c r="AU11" s="7"/>
+      <c r="AV11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">전체 개수</t>
         </is>
       </c>
-      <c r="AV11" s="7">
-        <v>222</v>
+      <c r="AW11" s="7">
+        <v>228</v>
       </c>
     </row>
     <row r="12">
@@ -1172,13 +1187,14 @@
       <c r="AR12" s="7"/>
       <c r="AS12" s="7"/>
       <c r="AT12" s="7"/>
-      <c r="AU12" s="2" t="inlineStr">
+      <c r="AU12" s="7"/>
+      <c r="AV12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">진행율</t>
         </is>
       </c>
-      <c r="AV12" s="7">
-        <f>TEXT((COUNTA(AT9:AT230))/222,"0.00%")</f>
+      <c r="AW12" s="7">
+        <f>TEXT((COUNTA(AU9:AU236))/228,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -1256,6 +1272,7 @@
       <c r="AR13" s="7"/>
       <c r="AS13" s="7"/>
       <c r="AT13" s="7"/>
+      <c r="AU13" s="7"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -1323,6 +1340,7 @@
       <c r="AR14" s="7"/>
       <c r="AS14" s="7"/>
       <c r="AT14" s="7"/>
+      <c r="AU14" s="7"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -1426,6 +1444,7 @@
       <c r="AR15" s="7"/>
       <c r="AS15" s="7"/>
       <c r="AT15" s="7"/>
+      <c r="AU15" s="7"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -1529,6 +1548,7 @@
       <c r="AR16" s="7"/>
       <c r="AS16" s="7"/>
       <c r="AT16" s="7"/>
+      <c r="AU16" s="7"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -1637,6 +1657,7 @@
       <c r="AR17" s="7"/>
       <c r="AS17" s="7"/>
       <c r="AT17" s="7"/>
+      <c r="AU17" s="7"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -1709,6 +1730,7 @@
       <c r="AR18" s="7"/>
       <c r="AS18" s="7"/>
       <c r="AT18" s="7"/>
+      <c r="AU18" s="7"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -1776,6 +1798,7 @@
       <c r="AR19" s="7"/>
       <c r="AS19" s="7"/>
       <c r="AT19" s="7"/>
+      <c r="AU19" s="7"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1843,6 +1866,7 @@
       <c r="AR20" s="7"/>
       <c r="AS20" s="7"/>
       <c r="AT20" s="7"/>
+      <c r="AU20" s="7"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1946,6 +1970,7 @@
       <c r="AR21" s="7"/>
       <c r="AS21" s="7"/>
       <c r="AT21" s="7"/>
+      <c r="AU21" s="7"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -2042,6 +2067,7 @@
       <c r="AR22" s="7"/>
       <c r="AS22" s="7"/>
       <c r="AT22" s="7"/>
+      <c r="AU22" s="7"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -2117,6 +2143,7 @@
       <c r="AR23" s="7"/>
       <c r="AS23" s="7"/>
       <c r="AT23" s="7"/>
+      <c r="AU23" s="7"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -2184,6 +2211,7 @@
       <c r="AR24" s="7"/>
       <c r="AS24" s="7"/>
       <c r="AT24" s="7"/>
+      <c r="AU24" s="7"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -2251,6 +2279,7 @@
       <c r="AR25" s="7"/>
       <c r="AS25" s="7"/>
       <c r="AT25" s="7"/>
+      <c r="AU25" s="7"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -2347,6 +2376,7 @@
       <c r="AR26" s="7"/>
       <c r="AS26" s="7"/>
       <c r="AT26" s="7"/>
+      <c r="AU26" s="7"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -2418,6 +2448,7 @@
       <c r="AR27" s="7"/>
       <c r="AS27" s="7"/>
       <c r="AT27" s="7"/>
+      <c r="AU27" s="7"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -2498,6 +2529,7 @@
       <c r="AR28" s="7"/>
       <c r="AS28" s="7"/>
       <c r="AT28" s="7"/>
+      <c r="AU28" s="7"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -2573,6 +2605,7 @@
       <c r="AR29" s="7"/>
       <c r="AS29" s="7"/>
       <c r="AT29" s="7"/>
+      <c r="AU29" s="7"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -2672,6 +2705,7 @@
       <c r="AR30" s="7"/>
       <c r="AS30" s="7"/>
       <c r="AT30" s="7"/>
+      <c r="AU30" s="7"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -2776,6 +2810,7 @@
       <c r="AR31" s="7"/>
       <c r="AS31" s="7"/>
       <c r="AT31" s="7"/>
+      <c r="AU31" s="7"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -2867,6 +2902,7 @@
       <c r="AR32" s="7"/>
       <c r="AS32" s="7"/>
       <c r="AT32" s="7"/>
+      <c r="AU32" s="7"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -2966,6 +3002,7 @@
       <c r="AR33" s="7"/>
       <c r="AS33" s="7"/>
       <c r="AT33" s="7"/>
+      <c r="AU33" s="7"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -3065,6 +3102,7 @@
       <c r="AR34" s="7"/>
       <c r="AS34" s="7"/>
       <c r="AT34" s="7"/>
+      <c r="AU34" s="7"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -3173,6 +3211,7 @@
       <c r="AR35" s="7"/>
       <c r="AS35" s="7"/>
       <c r="AT35" s="7"/>
+      <c r="AU35" s="7"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -3256,6 +3295,7 @@
       <c r="AR36" s="7"/>
       <c r="AS36" s="7"/>
       <c r="AT36" s="7"/>
+      <c r="AU36" s="7"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -3323,6 +3363,7 @@
       <c r="AR37" s="7"/>
       <c r="AS37" s="7"/>
       <c r="AT37" s="7"/>
+      <c r="AU37" s="7"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -3411,6 +3452,7 @@
       <c r="AR38" s="7"/>
       <c r="AS38" s="7"/>
       <c r="AT38" s="7"/>
+      <c r="AU38" s="7"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -3510,6 +3552,7 @@
       <c r="AR39" s="7"/>
       <c r="AS39" s="7"/>
       <c r="AT39" s="7"/>
+      <c r="AU39" s="7"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -3610,6 +3653,7 @@
       <c r="AR40" s="7"/>
       <c r="AS40" s="7"/>
       <c r="AT40" s="7"/>
+      <c r="AU40" s="7"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -3705,6 +3749,7 @@
       <c r="AR41" s="7"/>
       <c r="AS41" s="7"/>
       <c r="AT41" s="7"/>
+      <c r="AU41" s="7"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -3784,6 +3829,7 @@
       <c r="AR42" s="7"/>
       <c r="AS42" s="7"/>
       <c r="AT42" s="7"/>
+      <c r="AU42" s="7"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -3883,6 +3929,7 @@
       <c r="AR43" s="7"/>
       <c r="AS43" s="7"/>
       <c r="AT43" s="7"/>
+      <c r="AU43" s="7"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -3955,6 +4002,7 @@
       <c r="AR44" s="7"/>
       <c r="AS44" s="7"/>
       <c r="AT44" s="7"/>
+      <c r="AU44" s="7"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -4050,6 +4098,7 @@
       <c r="AR45" s="7"/>
       <c r="AS45" s="7"/>
       <c r="AT45" s="7"/>
+      <c r="AU45" s="7"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -4145,6 +4194,7 @@
       <c r="AR46" s="7"/>
       <c r="AS46" s="7"/>
       <c r="AT46" s="7"/>
+      <c r="AU46" s="7"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -4217,6 +4267,7 @@
       <c r="AR47" s="7"/>
       <c r="AS47" s="7"/>
       <c r="AT47" s="7"/>
+      <c r="AU47" s="7"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -4284,6 +4335,7 @@
       <c r="AR48" s="7"/>
       <c r="AS48" s="7"/>
       <c r="AT48" s="7"/>
+      <c r="AU48" s="7"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -4351,6 +4403,7 @@
       <c r="AR49" s="7"/>
       <c r="AS49" s="7"/>
       <c r="AT49" s="7"/>
+      <c r="AU49" s="7"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -4442,6 +4495,7 @@
       <c r="AR50" s="7"/>
       <c r="AS50" s="7"/>
       <c r="AT50" s="7"/>
+      <c r="AU50" s="7"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -4533,6 +4587,7 @@
       <c r="AR51" s="7"/>
       <c r="AS51" s="7"/>
       <c r="AT51" s="7"/>
+      <c r="AU51" s="7"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -4605,6 +4660,7 @@
       <c r="AR52" s="7"/>
       <c r="AS52" s="7"/>
       <c r="AT52" s="7"/>
+      <c r="AU52" s="7"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -4677,6 +4733,7 @@
       <c r="AR53" s="7"/>
       <c r="AS53" s="7"/>
       <c r="AT53" s="7"/>
+      <c r="AU53" s="7"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -4744,6 +4801,7 @@
       <c r="AR54" s="7"/>
       <c r="AS54" s="7"/>
       <c r="AT54" s="7"/>
+      <c r="AU54" s="7"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -4847,6 +4905,7 @@
       <c r="AR55" s="7"/>
       <c r="AS55" s="7"/>
       <c r="AT55" s="7"/>
+      <c r="AU55" s="7"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -4930,6 +4989,7 @@
       <c r="AR56" s="7"/>
       <c r="AS56" s="7"/>
       <c r="AT56" s="7"/>
+      <c r="AU56" s="7"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -5022,6 +5082,7 @@
       <c r="AR57" s="7"/>
       <c r="AS57" s="7"/>
       <c r="AT57" s="7"/>
+      <c r="AU57" s="7"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -5122,6 +5183,7 @@
       <c r="AR58" s="7"/>
       <c r="AS58" s="7"/>
       <c r="AT58" s="7"/>
+      <c r="AU58" s="7"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -5189,6 +5251,7 @@
       <c r="AR59" s="7"/>
       <c r="AS59" s="7"/>
       <c r="AT59" s="7"/>
+      <c r="AU59" s="7"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -5256,6 +5319,7 @@
       <c r="AR60" s="7"/>
       <c r="AS60" s="7"/>
       <c r="AT60" s="7"/>
+      <c r="AU60" s="7"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -5335,6 +5399,7 @@
       <c r="AR61" s="7"/>
       <c r="AS61" s="7"/>
       <c r="AT61" s="7"/>
+      <c r="AU61" s="7"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -5422,6 +5487,7 @@
       <c r="AR62" s="7"/>
       <c r="AS62" s="7"/>
       <c r="AT62" s="7"/>
+      <c r="AU62" s="7"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -5501,6 +5567,7 @@
       <c r="AR63" s="7"/>
       <c r="AS63" s="7"/>
       <c r="AT63" s="7"/>
+      <c r="AU63" s="7"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -5568,6 +5635,7 @@
       <c r="AR64" s="7"/>
       <c r="AS64" s="7"/>
       <c r="AT64" s="7"/>
+      <c r="AU64" s="7"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -5640,6 +5708,7 @@
       <c r="AR65" s="7"/>
       <c r="AS65" s="7"/>
       <c r="AT65" s="7"/>
+      <c r="AU65" s="7"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
@@ -5719,6 +5788,7 @@
       <c r="AR66" s="7"/>
       <c r="AS66" s="7"/>
       <c r="AT66" s="7"/>
+      <c r="AU66" s="7"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -5786,6 +5856,7 @@
       <c r="AR67" s="7"/>
       <c r="AS67" s="7"/>
       <c r="AT67" s="7"/>
+      <c r="AU67" s="7"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
@@ -5857,6 +5928,7 @@
       <c r="AR68" s="7"/>
       <c r="AS68" s="7"/>
       <c r="AT68" s="7"/>
+      <c r="AU68" s="7"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -5960,6 +6032,7 @@
       <c r="AR69" s="7"/>
       <c r="AS69" s="7"/>
       <c r="AT69" s="7"/>
+      <c r="AU69" s="7"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
@@ -6027,6 +6100,7 @@
       <c r="AR70" s="7"/>
       <c r="AS70" s="7"/>
       <c r="AT70" s="7"/>
+      <c r="AU70" s="7"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -6099,6 +6173,7 @@
       <c r="AR71" s="7"/>
       <c r="AS71" s="7"/>
       <c r="AT71" s="7"/>
+      <c r="AU71" s="7"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
@@ -6182,6 +6257,7 @@
       <c r="AR72" s="7"/>
       <c r="AS72" s="7"/>
       <c r="AT72" s="7"/>
+      <c r="AU72" s="7"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
@@ -6254,6 +6330,7 @@
       <c r="AR73" s="7"/>
       <c r="AS73" s="7"/>
       <c r="AT73" s="7"/>
+      <c r="AU73" s="7"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -6321,6 +6398,7 @@
       <c r="AR74" s="7"/>
       <c r="AS74" s="7"/>
       <c r="AT74" s="7"/>
+      <c r="AU74" s="7"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -6388,6 +6466,7 @@
       <c r="AR75" s="7"/>
       <c r="AS75" s="7"/>
       <c r="AT75" s="7"/>
+      <c r="AU75" s="7"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -6455,6 +6534,7 @@
       <c r="AR76" s="7"/>
       <c r="AS76" s="7"/>
       <c r="AT76" s="7"/>
+      <c r="AU76" s="7"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -6526,6 +6606,7 @@
       <c r="AR77" s="7"/>
       <c r="AS77" s="7"/>
       <c r="AT77" s="7"/>
+      <c r="AU77" s="7"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
@@ -6593,6 +6674,7 @@
       <c r="AR78" s="7"/>
       <c r="AS78" s="7"/>
       <c r="AT78" s="7"/>
+      <c r="AU78" s="7"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -6665,6 +6747,7 @@
       <c r="AR79" s="7"/>
       <c r="AS79" s="7"/>
       <c r="AT79" s="7"/>
+      <c r="AU79" s="7"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
@@ -6748,6 +6831,7 @@
       <c r="AR80" s="7"/>
       <c r="AS80" s="7"/>
       <c r="AT80" s="7"/>
+      <c r="AU80" s="7"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
@@ -6819,6 +6903,7 @@
       <c r="AR81" s="7"/>
       <c r="AS81" s="7"/>
       <c r="AT81" s="7"/>
+      <c r="AU81" s="7"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
@@ -6886,6 +6971,7 @@
       <c r="AR82" s="7"/>
       <c r="AS82" s="7"/>
       <c r="AT82" s="7"/>
+      <c r="AU82" s="7"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
@@ -6958,6 +7044,7 @@
       <c r="AR83" s="7"/>
       <c r="AS83" s="7"/>
       <c r="AT83" s="7"/>
+      <c r="AU83" s="7"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
@@ -7025,6 +7112,7 @@
       <c r="AR84" s="7"/>
       <c r="AS84" s="7"/>
       <c r="AT84" s="7"/>
+      <c r="AU84" s="7"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
@@ -7092,6 +7180,7 @@
       <c r="AR85" s="7"/>
       <c r="AS85" s="7"/>
       <c r="AT85" s="7"/>
+      <c r="AU85" s="7"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
@@ -7164,6 +7253,7 @@
       <c r="AR86" s="7"/>
       <c r="AS86" s="7"/>
       <c r="AT86" s="7"/>
+      <c r="AU86" s="7"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
@@ -7231,6 +7321,7 @@
       <c r="AR87" s="7"/>
       <c r="AS87" s="7"/>
       <c r="AT87" s="7"/>
+      <c r="AU87" s="7"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
@@ -7298,6 +7389,7 @@
       <c r="AR88" s="7"/>
       <c r="AS88" s="7"/>
       <c r="AT88" s="7"/>
+      <c r="AU88" s="7"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
@@ -7365,6 +7457,7 @@
       <c r="AR89" s="7"/>
       <c r="AS89" s="7"/>
       <c r="AT89" s="7"/>
+      <c r="AU89" s="7"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
@@ -7461,6 +7554,7 @@
       <c r="AR90" s="7"/>
       <c r="AS90" s="7"/>
       <c r="AT90" s="7"/>
+      <c r="AU90" s="7"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
@@ -7528,6 +7622,7 @@
       <c r="AR91" s="7"/>
       <c r="AS91" s="7"/>
       <c r="AT91" s="7"/>
+      <c r="AU91" s="7"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
@@ -7631,6 +7726,7 @@
       <c r="AR92" s="7"/>
       <c r="AS92" s="7"/>
       <c r="AT92" s="7"/>
+      <c r="AU92" s="7"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
@@ -7739,6 +7835,7 @@
       <c r="AR93" s="7"/>
       <c r="AS93" s="7"/>
       <c r="AT93" s="7"/>
+      <c r="AU93" s="7"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
@@ -7811,6 +7908,7 @@
       <c r="AR94" s="7"/>
       <c r="AS94" s="7"/>
       <c r="AT94" s="7"/>
+      <c r="AU94" s="7"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
@@ -7883,6 +7981,7 @@
       <c r="AR95" s="7"/>
       <c r="AS95" s="7"/>
       <c r="AT95" s="7"/>
+      <c r="AU95" s="7"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
@@ -7974,6 +8073,7 @@
       <c r="AR96" s="7"/>
       <c r="AS96" s="7"/>
       <c r="AT96" s="7"/>
+      <c r="AU96" s="7"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="inlineStr">
@@ -8041,6 +8141,7 @@
       <c r="AR97" s="7"/>
       <c r="AS97" s="7"/>
       <c r="AT97" s="7"/>
+      <c r="AU97" s="7"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
@@ -8108,6 +8209,7 @@
       <c r="AR98" s="7"/>
       <c r="AS98" s="7"/>
       <c r="AT98" s="7"/>
+      <c r="AU98" s="7"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
@@ -8175,6 +8277,7 @@
       <c r="AR99" s="7"/>
       <c r="AS99" s="7"/>
       <c r="AT99" s="7"/>
+      <c r="AU99" s="7"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
@@ -8251,6 +8354,7 @@
       <c r="AR100" s="7"/>
       <c r="AS100" s="7"/>
       <c r="AT100" s="7"/>
+      <c r="AU100" s="7"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
@@ -8318,6 +8422,7 @@
       <c r="AR101" s="7"/>
       <c r="AS101" s="7"/>
       <c r="AT101" s="7"/>
+      <c r="AU101" s="7"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
@@ -8385,6 +8490,7 @@
       <c r="AR102" s="7"/>
       <c r="AS102" s="7"/>
       <c r="AT102" s="7"/>
+      <c r="AU102" s="7"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="inlineStr">
@@ -8452,6 +8558,7 @@
       <c r="AR103" s="7"/>
       <c r="AS103" s="7"/>
       <c r="AT103" s="7"/>
+      <c r="AU103" s="7"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="inlineStr">
@@ -8524,6 +8631,7 @@
       <c r="AR104" s="7"/>
       <c r="AS104" s="7"/>
       <c r="AT104" s="7"/>
+      <c r="AU104" s="7"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
@@ -8591,6 +8699,7 @@
       <c r="AR105" s="7"/>
       <c r="AS105" s="7"/>
       <c r="AT105" s="7"/>
+      <c r="AU105" s="7"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
@@ -8658,6 +8767,7 @@
       <c r="AR106" s="7"/>
       <c r="AS106" s="7"/>
       <c r="AT106" s="7"/>
+      <c r="AU106" s="7"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
@@ -8725,6 +8835,7 @@
       <c r="AR107" s="7"/>
       <c r="AS107" s="7"/>
       <c r="AT107" s="7"/>
+      <c r="AU107" s="7"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
@@ -8796,6 +8907,7 @@
       <c r="AR108" s="7"/>
       <c r="AS108" s="7"/>
       <c r="AT108" s="7"/>
+      <c r="AU108" s="7"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="inlineStr">
@@ -8872,6 +8984,7 @@
       <c r="AR109" s="7"/>
       <c r="AS109" s="7"/>
       <c r="AT109" s="7"/>
+      <c r="AU109" s="7"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
@@ -8956,6 +9069,7 @@
       <c r="AR110" s="7"/>
       <c r="AS110" s="7"/>
       <c r="AT110" s="7"/>
+      <c r="AU110" s="7"/>
     </row>
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
@@ -9043,6 +9157,7 @@
       <c r="AR111" s="7"/>
       <c r="AS111" s="7"/>
       <c r="AT111" s="7"/>
+      <c r="AU111" s="7"/>
     </row>
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
@@ -9127,6 +9242,7 @@
       <c r="AR112" s="7"/>
       <c r="AS112" s="7"/>
       <c r="AT112" s="7"/>
+      <c r="AU112" s="7"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
@@ -9203,6 +9319,7 @@
       <c r="AR113" s="7"/>
       <c r="AS113" s="7"/>
       <c r="AT113" s="7"/>
+      <c r="AU113" s="7"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="inlineStr">
@@ -9295,6 +9412,7 @@
       <c r="AR114" s="7"/>
       <c r="AS114" s="7"/>
       <c r="AT114" s="7"/>
+      <c r="AU114" s="7"/>
     </row>
     <row r="115">
       <c r="A115" s="7" t="inlineStr">
@@ -9379,6 +9497,7 @@
       <c r="AR115" s="7"/>
       <c r="AS115" s="7"/>
       <c r="AT115" s="7"/>
+      <c r="AU115" s="7"/>
     </row>
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
@@ -9471,6 +9590,7 @@
       <c r="AR116" s="7"/>
       <c r="AS116" s="7"/>
       <c r="AT116" s="7"/>
+      <c r="AU116" s="7"/>
     </row>
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
@@ -9559,6 +9679,7 @@
       <c r="AR117" s="7"/>
       <c r="AS117" s="7"/>
       <c r="AT117" s="7"/>
+      <c r="AU117" s="7"/>
     </row>
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
@@ -9647,6 +9768,7 @@
       <c r="AR118" s="7"/>
       <c r="AS118" s="7"/>
       <c r="AT118" s="7"/>
+      <c r="AU118" s="7"/>
     </row>
     <row r="119">
       <c r="A119" s="7" t="inlineStr">
@@ -9731,6 +9853,7 @@
       <c r="AR119" s="7"/>
       <c r="AS119" s="7"/>
       <c r="AT119" s="7"/>
+      <c r="AU119" s="7"/>
     </row>
     <row r="120">
       <c r="A120" s="7" t="inlineStr">
@@ -9807,6 +9930,7 @@
       <c r="AR120" s="7"/>
       <c r="AS120" s="7"/>
       <c r="AT120" s="7"/>
+      <c r="AU120" s="7"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="inlineStr">
@@ -9895,6 +10019,7 @@
       <c r="AR121" s="7"/>
       <c r="AS121" s="7"/>
       <c r="AT121" s="7"/>
+      <c r="AU121" s="7"/>
     </row>
     <row r="122">
       <c r="A122" s="7" t="inlineStr">
@@ -9983,6 +10108,7 @@
       <c r="AR122" s="7"/>
       <c r="AS122" s="7"/>
       <c r="AT122" s="7"/>
+      <c r="AU122" s="7"/>
     </row>
     <row r="123">
       <c r="A123" s="7" t="inlineStr">
@@ -10059,6 +10185,7 @@
       <c r="AR123" s="7"/>
       <c r="AS123" s="7"/>
       <c r="AT123" s="7"/>
+      <c r="AU123" s="7"/>
     </row>
     <row r="124">
       <c r="A124" s="7" t="inlineStr">
@@ -10143,6 +10270,7 @@
       <c r="AR124" s="7"/>
       <c r="AS124" s="7"/>
       <c r="AT124" s="7"/>
+      <c r="AU124" s="7"/>
     </row>
     <row r="125">
       <c r="A125" s="7" t="inlineStr">
@@ -10219,6 +10347,7 @@
       <c r="AR125" s="7"/>
       <c r="AS125" s="7"/>
       <c r="AT125" s="7"/>
+      <c r="AU125" s="7"/>
     </row>
     <row r="126">
       <c r="A126" s="7" t="inlineStr">
@@ -10295,6 +10424,7 @@
       <c r="AR126" s="7"/>
       <c r="AS126" s="7"/>
       <c r="AT126" s="7"/>
+      <c r="AU126" s="7"/>
     </row>
     <row r="127">
       <c r="A127" s="7" t="inlineStr">
@@ -10375,6 +10505,7 @@
       <c r="AR127" s="7"/>
       <c r="AS127" s="7"/>
       <c r="AT127" s="7"/>
+      <c r="AU127" s="7"/>
     </row>
     <row r="128">
       <c r="A128" s="7" t="inlineStr">
@@ -10455,6 +10586,7 @@
       <c r="AR128" s="7"/>
       <c r="AS128" s="7"/>
       <c r="AT128" s="7"/>
+      <c r="AU128" s="7"/>
     </row>
     <row r="129">
       <c r="A129" s="7" t="inlineStr">
@@ -10535,6 +10667,7 @@
       <c r="AR129" s="7"/>
       <c r="AS129" s="7"/>
       <c r="AT129" s="7"/>
+      <c r="AU129" s="7"/>
     </row>
     <row r="130">
       <c r="A130" s="7" t="inlineStr">
@@ -10611,6 +10744,7 @@
       <c r="AR130" s="7"/>
       <c r="AS130" s="7"/>
       <c r="AT130" s="7"/>
+      <c r="AU130" s="7"/>
     </row>
     <row r="131">
       <c r="A131" s="7" t="inlineStr">
@@ -10695,6 +10829,7 @@
       <c r="AR131" s="7"/>
       <c r="AS131" s="7"/>
       <c r="AT131" s="7"/>
+      <c r="AU131" s="7"/>
     </row>
     <row r="132">
       <c r="A132" s="7" t="inlineStr">
@@ -10783,6 +10918,7 @@
       <c r="AR132" s="7"/>
       <c r="AS132" s="7"/>
       <c r="AT132" s="7"/>
+      <c r="AU132" s="7"/>
     </row>
     <row r="133">
       <c r="A133" s="7" t="inlineStr">
@@ -10871,6 +11007,7 @@
       <c r="AR133" s="7"/>
       <c r="AS133" s="7"/>
       <c r="AT133" s="7"/>
+      <c r="AU133" s="7"/>
     </row>
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
@@ -10955,6 +11092,7 @@
       <c r="AR134" s="7"/>
       <c r="AS134" s="7"/>
       <c r="AT134" s="7"/>
+      <c r="AU134" s="7"/>
     </row>
     <row r="135">
       <c r="A135" s="7" t="inlineStr">
@@ -11039,6 +11177,7 @@
       <c r="AR135" s="7"/>
       <c r="AS135" s="7"/>
       <c r="AT135" s="7"/>
+      <c r="AU135" s="7"/>
     </row>
     <row r="136">
       <c r="A136" s="7" t="inlineStr">
@@ -11123,6 +11262,7 @@
       <c r="AR136" s="7"/>
       <c r="AS136" s="7"/>
       <c r="AT136" s="7"/>
+      <c r="AU136" s="7"/>
     </row>
     <row r="137">
       <c r="A137" s="7" t="inlineStr">
@@ -11203,6 +11343,7 @@
       <c r="AR137" s="7"/>
       <c r="AS137" s="7"/>
       <c r="AT137" s="7"/>
+      <c r="AU137" s="7"/>
     </row>
     <row r="138">
       <c r="A138" s="7" t="inlineStr">
@@ -11283,6 +11424,7 @@
       <c r="AR138" s="7"/>
       <c r="AS138" s="7"/>
       <c r="AT138" s="7"/>
+      <c r="AU138" s="7"/>
     </row>
     <row r="139">
       <c r="A139" s="7" t="inlineStr">
@@ -11363,6 +11505,7 @@
       <c r="AR139" s="7"/>
       <c r="AS139" s="7"/>
       <c r="AT139" s="7"/>
+      <c r="AU139" s="7"/>
     </row>
     <row r="140">
       <c r="A140" s="7" t="inlineStr">
@@ -11439,6 +11582,7 @@
       <c r="AR140" s="7"/>
       <c r="AS140" s="7"/>
       <c r="AT140" s="7"/>
+      <c r="AU140" s="7"/>
     </row>
     <row r="141">
       <c r="A141" s="7" t="inlineStr">
@@ -11527,6 +11671,7 @@
       <c r="AR141" s="7"/>
       <c r="AS141" s="7"/>
       <c r="AT141" s="7"/>
+      <c r="AU141" s="7"/>
     </row>
     <row r="142">
       <c r="A142" s="7" t="inlineStr">
@@ -11603,6 +11748,7 @@
       <c r="AR142" s="7"/>
       <c r="AS142" s="7"/>
       <c r="AT142" s="7"/>
+      <c r="AU142" s="7"/>
     </row>
     <row r="143">
       <c r="A143" s="7" t="inlineStr">
@@ -11679,6 +11825,7 @@
       <c r="AR143" s="7"/>
       <c r="AS143" s="7"/>
       <c r="AT143" s="7"/>
+      <c r="AU143" s="7"/>
     </row>
     <row r="144">
       <c r="A144" s="7" t="inlineStr">
@@ -11755,6 +11902,7 @@
       <c r="AR144" s="7"/>
       <c r="AS144" s="7"/>
       <c r="AT144" s="7"/>
+      <c r="AU144" s="7"/>
     </row>
     <row r="145">
       <c r="A145" s="7" t="inlineStr">
@@ -11847,6 +11995,7 @@
       <c r="AR145" s="7"/>
       <c r="AS145" s="7"/>
       <c r="AT145" s="7"/>
+      <c r="AU145" s="7"/>
     </row>
     <row r="146">
       <c r="A146" s="7" t="inlineStr">
@@ -11927,6 +12076,7 @@
       <c r="AR146" s="7"/>
       <c r="AS146" s="7"/>
       <c r="AT146" s="7"/>
+      <c r="AU146" s="7"/>
     </row>
     <row r="147">
       <c r="A147" s="7" t="inlineStr">
@@ -12019,6 +12169,7 @@
       <c r="AR147" s="7"/>
       <c r="AS147" s="7"/>
       <c r="AT147" s="7"/>
+      <c r="AU147" s="7"/>
     </row>
     <row r="148">
       <c r="A148" s="7" t="inlineStr">
@@ -12095,6 +12246,7 @@
       <c r="AR148" s="7"/>
       <c r="AS148" s="7"/>
       <c r="AT148" s="7"/>
+      <c r="AU148" s="7"/>
     </row>
     <row r="149">
       <c r="A149" s="7" t="inlineStr">
@@ -12179,6 +12331,7 @@
       <c r="AR149" s="7"/>
       <c r="AS149" s="7"/>
       <c r="AT149" s="7"/>
+      <c r="AU149" s="7"/>
     </row>
     <row r="150">
       <c r="A150" s="7" t="inlineStr">
@@ -12267,6 +12420,7 @@
       <c r="AR150" s="7"/>
       <c r="AS150" s="7"/>
       <c r="AT150" s="7"/>
+      <c r="AU150" s="7"/>
     </row>
     <row r="151">
       <c r="A151" s="7" t="inlineStr">
@@ -12347,6 +12501,7 @@
       <c r="AR151" s="7"/>
       <c r="AS151" s="7"/>
       <c r="AT151" s="7"/>
+      <c r="AU151" s="7"/>
     </row>
     <row r="152">
       <c r="A152" s="7" t="inlineStr">
@@ -12431,6 +12586,7 @@
       <c r="AR152" s="7"/>
       <c r="AS152" s="7"/>
       <c r="AT152" s="7"/>
+      <c r="AU152" s="7"/>
     </row>
     <row r="153">
       <c r="A153" s="7" t="inlineStr">
@@ -12519,6 +12675,7 @@
       <c r="AR153" s="7"/>
       <c r="AS153" s="7"/>
       <c r="AT153" s="7"/>
+      <c r="AU153" s="7"/>
     </row>
     <row r="154">
       <c r="A154" s="7" t="inlineStr">
@@ -12591,6 +12748,7 @@
       <c r="AR154" s="7"/>
       <c r="AS154" s="7"/>
       <c r="AT154" s="7"/>
+      <c r="AU154" s="7"/>
     </row>
     <row r="155">
       <c r="A155" s="7" t="inlineStr">
@@ -12667,6 +12825,7 @@
       <c r="AR155" s="7"/>
       <c r="AS155" s="7"/>
       <c r="AT155" s="7"/>
+      <c r="AU155" s="7"/>
     </row>
     <row r="156">
       <c r="A156" s="7" t="inlineStr">
@@ -12747,6 +12906,7 @@
       <c r="AR156" s="7"/>
       <c r="AS156" s="7"/>
       <c r="AT156" s="7"/>
+      <c r="AU156" s="7"/>
     </row>
     <row r="157">
       <c r="A157" s="7" t="inlineStr">
@@ -12823,6 +12983,7 @@
       <c r="AR157" s="7"/>
       <c r="AS157" s="7"/>
       <c r="AT157" s="7"/>
+      <c r="AU157" s="7"/>
     </row>
     <row r="158">
       <c r="A158" s="7" t="inlineStr">
@@ -12899,6 +13060,7 @@
       <c r="AR158" s="7"/>
       <c r="AS158" s="7"/>
       <c r="AT158" s="7"/>
+      <c r="AU158" s="7"/>
     </row>
     <row r="159">
       <c r="A159" s="7" t="inlineStr">
@@ -12975,6 +13137,7 @@
       <c r="AR159" s="7"/>
       <c r="AS159" s="7"/>
       <c r="AT159" s="7"/>
+      <c r="AU159" s="7"/>
     </row>
     <row r="160">
       <c r="A160" s="7" t="inlineStr">
@@ -13051,6 +13214,7 @@
       <c r="AR160" s="7"/>
       <c r="AS160" s="7"/>
       <c r="AT160" s="7"/>
+      <c r="AU160" s="7"/>
     </row>
     <row r="161">
       <c r="A161" s="7" t="inlineStr">
@@ -13131,6 +13295,7 @@
       <c r="AR161" s="7"/>
       <c r="AS161" s="7"/>
       <c r="AT161" s="7"/>
+      <c r="AU161" s="7"/>
     </row>
     <row r="162">
       <c r="A162" s="7" t="inlineStr">
@@ -13207,6 +13372,7 @@
       <c r="AR162" s="7"/>
       <c r="AS162" s="7"/>
       <c r="AT162" s="7"/>
+      <c r="AU162" s="7"/>
     </row>
     <row r="163">
       <c r="A163" s="7" t="inlineStr">
@@ -13283,6 +13449,7 @@
       <c r="AR163" s="7"/>
       <c r="AS163" s="7"/>
       <c r="AT163" s="7"/>
+      <c r="AU163" s="7"/>
     </row>
     <row r="164">
       <c r="A164" s="7" t="inlineStr">
@@ -13359,6 +13526,7 @@
       <c r="AR164" s="7"/>
       <c r="AS164" s="7"/>
       <c r="AT164" s="7"/>
+      <c r="AU164" s="7"/>
     </row>
     <row r="165">
       <c r="A165" s="7" t="inlineStr">
@@ -13435,6 +13603,7 @@
       <c r="AR165" s="7"/>
       <c r="AS165" s="7"/>
       <c r="AT165" s="7"/>
+      <c r="AU165" s="7"/>
     </row>
     <row r="166">
       <c r="A166" s="7" t="inlineStr">
@@ -13519,6 +13688,7 @@
       <c r="AR166" s="7"/>
       <c r="AS166" s="7"/>
       <c r="AT166" s="7"/>
+      <c r="AU166" s="7"/>
     </row>
     <row r="167">
       <c r="A167" s="7" t="inlineStr">
@@ -13599,6 +13769,7 @@
       <c r="AR167" s="7"/>
       <c r="AS167" s="7"/>
       <c r="AT167" s="7"/>
+      <c r="AU167" s="7"/>
     </row>
     <row r="168">
       <c r="A168" s="7" t="inlineStr">
@@ -13675,6 +13846,7 @@
       <c r="AR168" s="7"/>
       <c r="AS168" s="7"/>
       <c r="AT168" s="7"/>
+      <c r="AU168" s="7"/>
     </row>
     <row r="169">
       <c r="A169" s="7" t="inlineStr">
@@ -13751,6 +13923,7 @@
       <c r="AR169" s="7"/>
       <c r="AS169" s="7"/>
       <c r="AT169" s="7"/>
+      <c r="AU169" s="7"/>
     </row>
     <row r="170">
       <c r="A170" s="7" t="inlineStr">
@@ -13831,6 +14004,7 @@
       <c r="AR170" s="7"/>
       <c r="AS170" s="7"/>
       <c r="AT170" s="7"/>
+      <c r="AU170" s="7"/>
     </row>
     <row r="171">
       <c r="A171" s="7" t="inlineStr">
@@ -13903,6 +14077,7 @@
       <c r="AR171" s="7"/>
       <c r="AS171" s="7"/>
       <c r="AT171" s="7"/>
+      <c r="AU171" s="7"/>
     </row>
     <row r="172">
       <c r="A172" s="7" t="inlineStr">
@@ -13975,6 +14150,7 @@
       <c r="AR172" s="7"/>
       <c r="AS172" s="7"/>
       <c r="AT172" s="7"/>
+      <c r="AU172" s="7"/>
     </row>
     <row r="173">
       <c r="A173" s="7" t="inlineStr">
@@ -14055,6 +14231,7 @@
       <c r="AR173" s="7"/>
       <c r="AS173" s="7"/>
       <c r="AT173" s="7"/>
+      <c r="AU173" s="7"/>
     </row>
     <row r="174">
       <c r="A174" s="7" t="inlineStr">
@@ -14131,6 +14308,7 @@
       <c r="AR174" s="7"/>
       <c r="AS174" s="7"/>
       <c r="AT174" s="7"/>
+      <c r="AU174" s="7"/>
     </row>
     <row r="175">
       <c r="A175" s="7" t="inlineStr">
@@ -14211,6 +14389,7 @@
       <c r="AR175" s="7"/>
       <c r="AS175" s="7"/>
       <c r="AT175" s="7"/>
+      <c r="AU175" s="7"/>
     </row>
     <row r="176">
       <c r="A176" s="7" t="inlineStr">
@@ -14287,6 +14466,7 @@
       <c r="AR176" s="7"/>
       <c r="AS176" s="7"/>
       <c r="AT176" s="7"/>
+      <c r="AU176" s="7"/>
     </row>
     <row r="177">
       <c r="A177" s="7" t="inlineStr">
@@ -14363,6 +14543,7 @@
       <c r="AR177" s="7"/>
       <c r="AS177" s="7"/>
       <c r="AT177" s="7"/>
+      <c r="AU177" s="7"/>
     </row>
     <row r="178">
       <c r="A178" s="7" t="inlineStr">
@@ -14439,6 +14620,7 @@
       <c r="AR178" s="7"/>
       <c r="AS178" s="7"/>
       <c r="AT178" s="7"/>
+      <c r="AU178" s="7"/>
     </row>
     <row r="179">
       <c r="A179" s="7" t="inlineStr">
@@ -14515,6 +14697,7 @@
       <c r="AR179" s="7"/>
       <c r="AS179" s="7"/>
       <c r="AT179" s="7"/>
+      <c r="AU179" s="7"/>
     </row>
     <row r="180">
       <c r="A180" s="7" t="inlineStr">
@@ -14591,6 +14774,7 @@
       <c r="AR180" s="7"/>
       <c r="AS180" s="7"/>
       <c r="AT180" s="7"/>
+      <c r="AU180" s="7"/>
     </row>
     <row r="181">
       <c r="A181" s="7" t="inlineStr">
@@ -14667,6 +14851,7 @@
       <c r="AR181" s="7"/>
       <c r="AS181" s="7"/>
       <c r="AT181" s="7"/>
+      <c r="AU181" s="7"/>
     </row>
     <row r="182">
       <c r="A182" s="7" t="inlineStr">
@@ -14743,6 +14928,7 @@
       <c r="AR182" s="7"/>
       <c r="AS182" s="7"/>
       <c r="AT182" s="7"/>
+      <c r="AU182" s="7"/>
     </row>
     <row r="183">
       <c r="A183" s="7" t="inlineStr">
@@ -14819,6 +15005,7 @@
       <c r="AR183" s="7"/>
       <c r="AS183" s="7"/>
       <c r="AT183" s="7"/>
+      <c r="AU183" s="7"/>
     </row>
     <row r="184">
       <c r="A184" s="7" t="inlineStr">
@@ -14891,6 +15078,7 @@
       <c r="AR184" s="7"/>
       <c r="AS184" s="7"/>
       <c r="AT184" s="7"/>
+      <c r="AU184" s="7"/>
     </row>
     <row r="185">
       <c r="A185" s="7" t="inlineStr">
@@ -14967,6 +15155,7 @@
       <c r="AR185" s="7"/>
       <c r="AS185" s="7"/>
       <c r="AT185" s="7"/>
+      <c r="AU185" s="7"/>
     </row>
     <row r="186">
       <c r="A186" s="7" t="inlineStr">
@@ -15043,6 +15232,7 @@
       <c r="AR186" s="7"/>
       <c r="AS186" s="7"/>
       <c r="AT186" s="7"/>
+      <c r="AU186" s="7"/>
     </row>
     <row r="187">
       <c r="A187" s="7" t="inlineStr">
@@ -15123,6 +15313,7 @@
       <c r="AR187" s="7"/>
       <c r="AS187" s="7"/>
       <c r="AT187" s="7"/>
+      <c r="AU187" s="7"/>
     </row>
     <row r="188">
       <c r="A188" s="7" t="inlineStr">
@@ -15203,6 +15394,7 @@
       <c r="AR188" s="7"/>
       <c r="AS188" s="7"/>
       <c r="AT188" s="7"/>
+      <c r="AU188" s="7"/>
     </row>
     <row r="189">
       <c r="A189" s="7" t="inlineStr">
@@ -15283,6 +15475,7 @@
       <c r="AR189" s="7"/>
       <c r="AS189" s="7"/>
       <c r="AT189" s="7"/>
+      <c r="AU189" s="7"/>
     </row>
     <row r="190">
       <c r="A190" s="7" t="inlineStr">
@@ -15363,6 +15556,7 @@
       <c r="AR190" s="7"/>
       <c r="AS190" s="7"/>
       <c r="AT190" s="7"/>
+      <c r="AU190" s="7"/>
     </row>
     <row r="191">
       <c r="A191" s="7" t="inlineStr">
@@ -15443,6 +15637,7 @@
       <c r="AR191" s="7"/>
       <c r="AS191" s="7"/>
       <c r="AT191" s="7"/>
+      <c r="AU191" s="7"/>
     </row>
     <row r="192">
       <c r="A192" s="7" t="inlineStr">
@@ -15523,6 +15718,7 @@
       <c r="AR192" s="7"/>
       <c r="AS192" s="7"/>
       <c r="AT192" s="7"/>
+      <c r="AU192" s="7"/>
     </row>
     <row r="193">
       <c r="A193" s="7" t="inlineStr">
@@ -15607,6 +15803,7 @@
       <c r="AR193" s="7"/>
       <c r="AS193" s="7"/>
       <c r="AT193" s="7"/>
+      <c r="AU193" s="7"/>
     </row>
     <row r="194">
       <c r="A194" s="7" t="inlineStr">
@@ -15691,6 +15888,7 @@
       <c r="AR194" s="7"/>
       <c r="AS194" s="7"/>
       <c r="AT194" s="7"/>
+      <c r="AU194" s="7"/>
     </row>
     <row r="195">
       <c r="A195" s="7" t="inlineStr">
@@ -15775,6 +15973,7 @@
       <c r="AR195" s="7"/>
       <c r="AS195" s="7"/>
       <c r="AT195" s="7"/>
+      <c r="AU195" s="7"/>
     </row>
     <row r="196">
       <c r="A196" s="7" t="inlineStr">
@@ -15851,6 +16050,7 @@
       <c r="AR196" s="7"/>
       <c r="AS196" s="7"/>
       <c r="AT196" s="7"/>
+      <c r="AU196" s="7"/>
     </row>
     <row r="197">
       <c r="A197" s="7" t="inlineStr">
@@ -15935,6 +16135,7 @@
       <c r="AR197" s="7"/>
       <c r="AS197" s="7"/>
       <c r="AT197" s="7"/>
+      <c r="AU197" s="7"/>
     </row>
     <row r="198">
       <c r="A198" s="7" t="inlineStr">
@@ -16011,6 +16212,7 @@
       <c r="AR198" s="7"/>
       <c r="AS198" s="7"/>
       <c r="AT198" s="7"/>
+      <c r="AU198" s="7"/>
     </row>
     <row r="199">
       <c r="A199" s="7" t="inlineStr">
@@ -16095,6 +16297,7 @@
       <c r="AR199" s="7"/>
       <c r="AS199" s="7"/>
       <c r="AT199" s="7"/>
+      <c r="AU199" s="7"/>
     </row>
     <row r="200">
       <c r="A200" s="7" t="inlineStr">
@@ -16179,6 +16382,7 @@
       <c r="AR200" s="7"/>
       <c r="AS200" s="7"/>
       <c r="AT200" s="7"/>
+      <c r="AU200" s="7"/>
     </row>
     <row r="201">
       <c r="A201" s="7" t="inlineStr">
@@ -16255,6 +16459,7 @@
       <c r="AR201" s="7"/>
       <c r="AS201" s="7"/>
       <c r="AT201" s="7"/>
+      <c r="AU201" s="7"/>
     </row>
     <row r="202">
       <c r="A202" s="7" t="inlineStr">
@@ -16339,6 +16544,7 @@
       <c r="AR202" s="7"/>
       <c r="AS202" s="7"/>
       <c r="AT202" s="7"/>
+      <c r="AU202" s="7"/>
     </row>
     <row r="203">
       <c r="A203" s="7" t="inlineStr">
@@ -16423,6 +16629,7 @@
       <c r="AR203" s="7"/>
       <c r="AS203" s="7"/>
       <c r="AT203" s="7"/>
+      <c r="AU203" s="7"/>
     </row>
     <row r="204">
       <c r="A204" s="7" t="inlineStr">
@@ -16511,6 +16718,7 @@
       </c>
       <c r="AS204" s="7"/>
       <c r="AT204" s="7"/>
+      <c r="AU204" s="7"/>
     </row>
     <row r="205">
       <c r="A205" s="7" t="inlineStr">
@@ -16599,6 +16807,7 @@
       <c r="AR205" s="7"/>
       <c r="AS205" s="7"/>
       <c r="AT205" s="7"/>
+      <c r="AU205" s="7"/>
     </row>
     <row r="206">
       <c r="A206" s="7" t="inlineStr">
@@ -16687,6 +16896,7 @@
       </c>
       <c r="AS206" s="7"/>
       <c r="AT206" s="7"/>
+      <c r="AU206" s="7"/>
     </row>
     <row r="207">
       <c r="A207" s="7" t="inlineStr">
@@ -16767,6 +16977,7 @@
       <c r="AR207" s="7"/>
       <c r="AS207" s="7"/>
       <c r="AT207" s="7"/>
+      <c r="AU207" s="7"/>
     </row>
     <row r="208">
       <c r="A208" s="7" t="inlineStr">
@@ -16851,6 +17062,7 @@
       </c>
       <c r="AS208" s="7"/>
       <c r="AT208" s="7"/>
+      <c r="AU208" s="7"/>
     </row>
     <row r="209">
       <c r="A209" s="7" t="inlineStr">
@@ -16939,6 +17151,7 @@
       </c>
       <c r="AS209" s="7"/>
       <c r="AT209" s="7"/>
+      <c r="AU209" s="7"/>
     </row>
     <row r="210">
       <c r="A210" s="7" t="inlineStr">
@@ -17023,6 +17236,7 @@
       </c>
       <c r="AS210" s="7"/>
       <c r="AT210" s="7"/>
+      <c r="AU210" s="7"/>
     </row>
     <row r="211">
       <c r="A211" s="7" t="inlineStr">
@@ -17099,6 +17313,7 @@
       <c r="AR211" s="7"/>
       <c r="AS211" s="7"/>
       <c r="AT211" s="7"/>
+      <c r="AU211" s="7"/>
     </row>
     <row r="212">
       <c r="A212" s="7" t="inlineStr">
@@ -17175,6 +17390,7 @@
       <c r="AR212" s="7"/>
       <c r="AS212" s="7"/>
       <c r="AT212" s="7"/>
+      <c r="AU212" s="7"/>
     </row>
     <row r="213">
       <c r="A213" s="7" t="inlineStr">
@@ -17255,6 +17471,7 @@
       </c>
       <c r="AS213" s="7"/>
       <c r="AT213" s="7"/>
+      <c r="AU213" s="7"/>
     </row>
     <row r="214">
       <c r="A214" s="7" t="inlineStr">
@@ -17331,6 +17548,7 @@
       <c r="AR214" s="7"/>
       <c r="AS214" s="7"/>
       <c r="AT214" s="7"/>
+      <c r="AU214" s="7"/>
     </row>
     <row r="215">
       <c r="A215" s="7" t="inlineStr">
@@ -17403,6 +17621,7 @@
       <c r="AR215" s="7"/>
       <c r="AS215" s="7"/>
       <c r="AT215" s="7"/>
+      <c r="AU215" s="7"/>
     </row>
     <row r="216">
       <c r="A216" s="7" t="inlineStr">
@@ -17475,6 +17694,7 @@
       <c r="AR216" s="7"/>
       <c r="AS216" s="7"/>
       <c r="AT216" s="7"/>
+      <c r="AU216" s="7"/>
     </row>
     <row r="217">
       <c r="A217" s="7" t="inlineStr">
@@ -17551,6 +17771,7 @@
       </c>
       <c r="AS217" s="7"/>
       <c r="AT217" s="7"/>
+      <c r="AU217" s="7"/>
     </row>
     <row r="218">
       <c r="A218" s="7" t="inlineStr">
@@ -17623,6 +17844,7 @@
       <c r="AR218" s="7"/>
       <c r="AS218" s="7"/>
       <c r="AT218" s="7"/>
+      <c r="AU218" s="7"/>
     </row>
     <row r="219">
       <c r="A219" s="7" t="inlineStr">
@@ -17699,6 +17921,7 @@
       </c>
       <c r="AS219" s="7"/>
       <c r="AT219" s="7"/>
+      <c r="AU219" s="7"/>
     </row>
     <row r="220">
       <c r="A220" s="7" t="inlineStr">
@@ -17771,6 +17994,7 @@
       <c r="AR220" s="7"/>
       <c r="AS220" s="7"/>
       <c r="AT220" s="7"/>
+      <c r="AU220" s="7"/>
     </row>
     <row r="221">
       <c r="A221" s="7" t="inlineStr">
@@ -17847,6 +18071,7 @@
       </c>
       <c r="AS221" s="7"/>
       <c r="AT221" s="7"/>
+      <c r="AU221" s="7"/>
     </row>
     <row r="222">
       <c r="A222" s="7" t="inlineStr">
@@ -17927,6 +18152,7 @@
         </is>
       </c>
       <c r="AT222" s="7"/>
+      <c r="AU222" s="7"/>
     </row>
     <row r="223">
       <c r="A223" s="7" t="inlineStr">
@@ -18003,6 +18229,7 @@
       </c>
       <c r="AS223" s="7"/>
       <c r="AT223" s="7"/>
+      <c r="AU223" s="7"/>
     </row>
     <row r="224">
       <c r="A224" s="7" t="inlineStr">
@@ -18079,6 +18306,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AU224" s="7"/>
     </row>
     <row r="225">
       <c r="A225" s="7" t="inlineStr">
@@ -18151,6 +18379,7 @@
       <c r="AR225" s="7"/>
       <c r="AS225" s="7"/>
       <c r="AT225" s="7"/>
+      <c r="AU225" s="7"/>
     </row>
     <row r="226">
       <c r="A226" s="7" t="inlineStr">
@@ -18223,6 +18452,7 @@
       <c r="AR226" s="7"/>
       <c r="AS226" s="7"/>
       <c r="AT226" s="7"/>
+      <c r="AU226" s="7"/>
     </row>
     <row r="227">
       <c r="A227" s="7" t="inlineStr">
@@ -18295,6 +18525,7 @@
       <c r="AR227" s="7"/>
       <c r="AS227" s="7"/>
       <c r="AT227" s="7"/>
+      <c r="AU227" s="7"/>
     </row>
     <row r="228">
       <c r="A228" s="7" t="inlineStr">
@@ -18371,6 +18602,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AU228" s="7"/>
     </row>
     <row r="229">
       <c r="A229" s="7" t="inlineStr">
@@ -18443,6 +18675,7 @@
       <c r="AR229" s="7"/>
       <c r="AS229" s="7"/>
       <c r="AT229" s="7"/>
+      <c r="AU229" s="7"/>
     </row>
     <row r="230">
       <c r="A230" s="7" t="inlineStr">
@@ -18519,6 +18752,453 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AU230" s="7"/>
+    </row>
+    <row r="231">
+      <c r="A231" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_231</t>
+        </is>
+      </c>
+      <c r="B231" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UI</t>
+        </is>
+      </c>
+      <c r="C231" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">팔레트 단추</t>
+        </is>
+      </c>
+      <c r="D231" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#213 개정</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">팔레트 노드 · 모듈 · 벨트 요소 단추가 그림 가득 + 하단 반투명 라벨 띠 위 이름(낱말 단위 두 줄 · 한 줄에 들면 한 줄)인가?</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#213 · AU 실측(1024×768): 「기초 / 가공소」 · 「복합 / 가공소」 두 줄 · 576×1024 는 못 봄</t>
+        </is>
+      </c>
+      <c r="G231" s="7"/>
+      <c r="H231" s="7"/>
+      <c r="I231" s="7"/>
+      <c r="J231" s="7"/>
+      <c r="K231" s="7"/>
+      <c r="L231" s="7"/>
+      <c r="M231" s="7"/>
+      <c r="N231" s="7"/>
+      <c r="O231" s="7"/>
+      <c r="P231" s="7"/>
+      <c r="Q231" s="7"/>
+      <c r="R231" s="7"/>
+      <c r="S231" s="7"/>
+      <c r="T231" s="7"/>
+      <c r="U231" s="7"/>
+      <c r="V231" s="7"/>
+      <c r="W231" s="7"/>
+      <c r="X231" s="7"/>
+      <c r="Y231" s="7"/>
+      <c r="Z231" s="7"/>
+      <c r="AA231" s="7"/>
+      <c r="AB231" s="7"/>
+      <c r="AC231" s="7"/>
+      <c r="AD231" s="7"/>
+      <c r="AE231" s="7"/>
+      <c r="AF231" s="7"/>
+      <c r="AG231" s="7"/>
+      <c r="AH231" s="7"/>
+      <c r="AI231" s="7"/>
+      <c r="AJ231" s="7"/>
+      <c r="AK231" s="7"/>
+      <c r="AL231" s="7"/>
+      <c r="AM231" s="7"/>
+      <c r="AN231" s="7"/>
+      <c r="AO231" s="7"/>
+      <c r="AP231" s="7"/>
+      <c r="AQ231" s="7"/>
+      <c r="AR231" s="7"/>
+      <c r="AS231" s="7"/>
+      <c r="AT231" s="7"/>
+      <c r="AU231" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_232</t>
+        </is>
+      </c>
+      <c r="B232" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UI</t>
+        </is>
+      </c>
+      <c r="C232" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">안내 줄 잔존</t>
+        </is>
+      </c>
+      <c r="D232" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#214</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t xml:space="preserve">「처음부터」 뒤 · 튜토리얼 막 중 보드 왼쪽 아래에 「보호막 · [고철] 20」 같은 비용 안내 줄이 안 남는가?</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#214 · 처음부터 때 노드 고르기도 풀고 · 노드 잠금 국면이면 고르기 해제 · 튜토리얼 중 비용 줄 숨김 · AU 못 봄</t>
+        </is>
+      </c>
+      <c r="G232" s="7"/>
+      <c r="H232" s="7"/>
+      <c r="I232" s="7"/>
+      <c r="J232" s="7"/>
+      <c r="K232" s="7"/>
+      <c r="L232" s="7"/>
+      <c r="M232" s="7"/>
+      <c r="N232" s="7"/>
+      <c r="O232" s="7"/>
+      <c r="P232" s="7"/>
+      <c r="Q232" s="7"/>
+      <c r="R232" s="7"/>
+      <c r="S232" s="7"/>
+      <c r="T232" s="7"/>
+      <c r="U232" s="7"/>
+      <c r="V232" s="7"/>
+      <c r="W232" s="7"/>
+      <c r="X232" s="7"/>
+      <c r="Y232" s="7"/>
+      <c r="Z232" s="7"/>
+      <c r="AA232" s="7"/>
+      <c r="AB232" s="7"/>
+      <c r="AC232" s="7"/>
+      <c r="AD232" s="7"/>
+      <c r="AE232" s="7"/>
+      <c r="AF232" s="7"/>
+      <c r="AG232" s="7"/>
+      <c r="AH232" s="7"/>
+      <c r="AI232" s="7"/>
+      <c r="AJ232" s="7"/>
+      <c r="AK232" s="7"/>
+      <c r="AL232" s="7"/>
+      <c r="AM232" s="7"/>
+      <c r="AN232" s="7"/>
+      <c r="AO232" s="7"/>
+      <c r="AP232" s="7"/>
+      <c r="AQ232" s="7"/>
+      <c r="AR232" s="7"/>
+      <c r="AS232" s="7"/>
+      <c r="AT232" s="7"/>
+      <c r="AU232" s="7"/>
+    </row>
+    <row r="233">
+      <c r="A233" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_233</t>
+        </is>
+      </c>
+      <c r="B233" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼</t>
+        </is>
+      </c>
+      <c r="C233" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S5 문안</t>
+        </is>
+      </c>
+      <c r="D233" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#215</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S5 걸음 ③ 「물류 탭에서 분류기를 고른 뒤 이 칸을 탭하세요」 · ④ 「복합 탭에서 복합 가공소를 고른 뒤 이 칸을 탭하세요」인가?</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#215 · 탭 이름을 PaletteCategories.LabelOf 로 읽음 · AU 못 봄(자연 S5)</t>
+        </is>
+      </c>
+      <c r="G233" s="7"/>
+      <c r="H233" s="7"/>
+      <c r="I233" s="7"/>
+      <c r="J233" s="7"/>
+      <c r="K233" s="7"/>
+      <c r="L233" s="7"/>
+      <c r="M233" s="7"/>
+      <c r="N233" s="7"/>
+      <c r="O233" s="7"/>
+      <c r="P233" s="7"/>
+      <c r="Q233" s="7"/>
+      <c r="R233" s="7"/>
+      <c r="S233" s="7"/>
+      <c r="T233" s="7"/>
+      <c r="U233" s="7"/>
+      <c r="V233" s="7"/>
+      <c r="W233" s="7"/>
+      <c r="X233" s="7"/>
+      <c r="Y233" s="7"/>
+      <c r="Z233" s="7"/>
+      <c r="AA233" s="7"/>
+      <c r="AB233" s="7"/>
+      <c r="AC233" s="7"/>
+      <c r="AD233" s="7"/>
+      <c r="AE233" s="7"/>
+      <c r="AF233" s="7"/>
+      <c r="AG233" s="7"/>
+      <c r="AH233" s="7"/>
+      <c r="AI233" s="7"/>
+      <c r="AJ233" s="7"/>
+      <c r="AK233" s="7"/>
+      <c r="AL233" s="7"/>
+      <c r="AM233" s="7"/>
+      <c r="AN233" s="7"/>
+      <c r="AO233" s="7"/>
+      <c r="AP233" s="7"/>
+      <c r="AQ233" s="7"/>
+      <c r="AR233" s="7"/>
+      <c r="AS233" s="7"/>
+      <c r="AT233" s="7"/>
+      <c r="AU233" s="7"/>
+    </row>
+    <row r="234">
+      <c r="A234" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_234</t>
+        </is>
+      </c>
+      <c r="B234" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼</t>
+        </is>
+      </c>
+      <c r="C234" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S5 자동 완성</t>
+        </is>
+      </c>
+      <c r="D234" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#216</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S5 걸음 ⑤ 끝 뒤 표준탄 갈래(9,8)~(2,4) · 병합기(2,5)가 0.15초 간격으로 저절로 깔리고 「이렇게 이으면 표준탄도 마운트에 닿습니다」가 한 번 뜨며 판이 프리셋과 같아지는가?</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#216 · 꼬리 칸 목록 = PresetBoards.ExplosiveTail(프리셋과 한 자리 · 하네스 프리셋 표 불변) · 고철 0 · 플레이어 칸 건너뜀 ⚠️ · AU 못 봄(자연 S5)</t>
+        </is>
+      </c>
+      <c r="G234" s="7"/>
+      <c r="H234" s="7"/>
+      <c r="I234" s="7"/>
+      <c r="J234" s="7"/>
+      <c r="K234" s="7"/>
+      <c r="L234" s="7"/>
+      <c r="M234" s="7"/>
+      <c r="N234" s="7"/>
+      <c r="O234" s="7"/>
+      <c r="P234" s="7"/>
+      <c r="Q234" s="7"/>
+      <c r="R234" s="7"/>
+      <c r="S234" s="7"/>
+      <c r="T234" s="7"/>
+      <c r="U234" s="7"/>
+      <c r="V234" s="7"/>
+      <c r="W234" s="7"/>
+      <c r="X234" s="7"/>
+      <c r="Y234" s="7"/>
+      <c r="Z234" s="7"/>
+      <c r="AA234" s="7"/>
+      <c r="AB234" s="7"/>
+      <c r="AC234" s="7"/>
+      <c r="AD234" s="7"/>
+      <c r="AE234" s="7"/>
+      <c r="AF234" s="7"/>
+      <c r="AG234" s="7"/>
+      <c r="AH234" s="7"/>
+      <c r="AI234" s="7"/>
+      <c r="AJ234" s="7"/>
+      <c r="AK234" s="7"/>
+      <c r="AL234" s="7"/>
+      <c r="AM234" s="7"/>
+      <c r="AN234" s="7"/>
+      <c r="AO234" s="7"/>
+      <c r="AP234" s="7"/>
+      <c r="AQ234" s="7"/>
+      <c r="AR234" s="7"/>
+      <c r="AS234" s="7"/>
+      <c r="AT234" s="7"/>
+      <c r="AU234" s="7"/>
+    </row>
+    <row r="235">
+      <c r="A235" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_235</t>
+        </is>
+      </c>
+      <c r="B235" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C235" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">쪼갠 발 표적</t>
+        </is>
+      </c>
+      <c r="D235" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#217</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">탄 하나를 쪼갠 세 발이 한 표적에게만 가고(앞 발에 죽으면 나머지 버림) 다른 탄종 발은 따로 고르는가?</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#217 · 시험 SplitShots_StayOnOneTarget · 하네스: S1뒤 28.2→29.7 · S2전 Win 54.8→LoseTimeout 53/55 · S3전 43.9→44.9 · S4뒤 50.5→53.5 · AU 화면 못 봄</t>
+        </is>
+      </c>
+      <c r="G235" s="7"/>
+      <c r="H235" s="7"/>
+      <c r="I235" s="7"/>
+      <c r="J235" s="7"/>
+      <c r="K235" s="7"/>
+      <c r="L235" s="7"/>
+      <c r="M235" s="7"/>
+      <c r="N235" s="7"/>
+      <c r="O235" s="7"/>
+      <c r="P235" s="7"/>
+      <c r="Q235" s="7"/>
+      <c r="R235" s="7"/>
+      <c r="S235" s="7"/>
+      <c r="T235" s="7"/>
+      <c r="U235" s="7"/>
+      <c r="V235" s="7"/>
+      <c r="W235" s="7"/>
+      <c r="X235" s="7"/>
+      <c r="Y235" s="7"/>
+      <c r="Z235" s="7"/>
+      <c r="AA235" s="7"/>
+      <c r="AB235" s="7"/>
+      <c r="AC235" s="7"/>
+      <c r="AD235" s="7"/>
+      <c r="AE235" s="7"/>
+      <c r="AF235" s="7"/>
+      <c r="AG235" s="7"/>
+      <c r="AH235" s="7"/>
+      <c r="AI235" s="7"/>
+      <c r="AJ235" s="7"/>
+      <c r="AK235" s="7"/>
+      <c r="AL235" s="7"/>
+      <c r="AM235" s="7"/>
+      <c r="AN235" s="7"/>
+      <c r="AO235" s="7"/>
+      <c r="AP235" s="7"/>
+      <c r="AQ235" s="7"/>
+      <c r="AR235" s="7"/>
+      <c r="AS235" s="7"/>
+      <c r="AT235" s="7"/>
+      <c r="AU235" s="7"/>
+    </row>
+    <row r="236">
+      <c r="A236" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_236</t>
+        </is>
+      </c>
+      <c r="B236" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UI</t>
+        </is>
+      </c>
+      <c r="C236" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">배지 목표 줄</t>
+        </is>
+      </c>
+      <c r="D236" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#218</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t xml:space="preserve">모든 판 도전 배지 목표 줄이 「목표: {주제}」만인가?(「전투력 N 넘기기」 없음)</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#218 · AU 실측: S4 「목표: 로봇 B 해금 · 합체」 ✅</t>
+        </is>
+      </c>
+      <c r="G236" s="7"/>
+      <c r="H236" s="7"/>
+      <c r="I236" s="7"/>
+      <c r="J236" s="7"/>
+      <c r="K236" s="7"/>
+      <c r="L236" s="7"/>
+      <c r="M236" s="7"/>
+      <c r="N236" s="7"/>
+      <c r="O236" s="7"/>
+      <c r="P236" s="7"/>
+      <c r="Q236" s="7"/>
+      <c r="R236" s="7"/>
+      <c r="S236" s="7"/>
+      <c r="T236" s="7"/>
+      <c r="U236" s="7"/>
+      <c r="V236" s="7"/>
+      <c r="W236" s="7"/>
+      <c r="X236" s="7"/>
+      <c r="Y236" s="7"/>
+      <c r="Z236" s="7"/>
+      <c r="AA236" s="7"/>
+      <c r="AB236" s="7"/>
+      <c r="AC236" s="7"/>
+      <c r="AD236" s="7"/>
+      <c r="AE236" s="7"/>
+      <c r="AF236" s="7"/>
+      <c r="AG236" s="7"/>
+      <c r="AH236" s="7"/>
+      <c r="AI236" s="7"/>
+      <c r="AJ236" s="7"/>
+      <c r="AK236" s="7"/>
+      <c r="AL236" s="7"/>
+      <c r="AM236" s="7"/>
+      <c r="AN236" s="7"/>
+      <c r="AO236" s="7"/>
+      <c r="AP236" s="7"/>
+      <c r="AQ236" s="7"/>
+      <c r="AR236" s="7"/>
+      <c r="AS236" s="7"/>
+      <c r="AT236" s="7"/>
+      <c r="AU236" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="26">
@@ -18547,9 +19227,9 @@
     <mergeCell ref="B92:B99"/>
     <mergeCell ref="B100:B106"/>
     <mergeCell ref="B107:B111"/>
-    <mergeCell ref="G7:AT7"/>
+    <mergeCell ref="G7:AU7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:AT230">
+  <conditionalFormatting sqref="G9:AU236">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
QA AV(7efab39 · CID_237~241)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -203,8 +203,9 @@
     <col min="45" max="45" width="12" customWidth="1"/>
     <col min="46" max="46" width="12" customWidth="1"/>
     <col min="47" max="47" width="12" customWidth="1"/>
-    <col min="48" max="48" width="11" customWidth="1"/>
+    <col min="48" max="48" width="12" customWidth="1"/>
     <col min="49" max="49" width="11" customWidth="1"/>
+    <col min="50" max="50" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -522,6 +523,11 @@
       <c r="AU6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">8133 22d9191 갈아엎음(10-20 11:20) · 사용자 육안(10-20 아침) #213~#218 · 결함 ⑨ 가름 ‖ 시험 1691/1685/0/6 · 전투 12줄 = #217 로 네 줄 바뀜(S2 전 LoseTimeout 53/55 · 판정 요청) · 프리셋 표 불변.</t>
+        </is>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8133 7efab39(10-20 14:19) · 883dd43 #219 · 0d984fd #220 · bd3e690 #221 #222 ④ · 86a6d0b #224 · 7efab39 #225 #223 #222수정 #217ⓐ #224수정 ‖ 시험 1709/1703/0/6 · 전투 12줄: S2전 Win 54.8 복귀 · S5전 Win 53.6 · S5뒤 33.4 · S6뒤 Win 54.9 · ⚠️ #223 대조: B 가득 + 즉시 합체 = S6 시간 초과(화면도 같음)</t>
         </is>
       </c>
     </row>
@@ -593,14 +599,15 @@
       <c r="AS7" s="2"/>
       <c r="AT7" s="2"/>
       <c r="AU7" s="2"/>
-      <c r="AV7" s="2" t="inlineStr">
+      <c r="AV7" s="2"/>
+      <c r="AW7" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">버전</t>
         </is>
       </c>
-      <c r="AW7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">22d9191</t>
+      <c r="AX7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7efab39</t>
         </is>
       </c>
     </row>
@@ -830,11 +837,16 @@
       </c>
       <c r="AV8" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">7efab39</t>
+        </is>
+      </c>
+      <c r="AW8" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">PASSrate</t>
         </is>
       </c>
-      <c r="AW8" s="7">
-        <f>COUNTIF(AU9:AU236,"Pass")</f>
+      <c r="AX8" s="7">
+        <f>COUNTIF(AV9:AV241,"Pass")</f>
       </c>
     </row>
     <row r="9">
@@ -945,13 +957,14 @@
       <c r="AS9" s="7"/>
       <c r="AT9" s="7"/>
       <c r="AU9" s="7"/>
-      <c r="AV9" s="2" t="inlineStr">
+      <c r="AV9" s="7"/>
+      <c r="AW9" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">FAILrate</t>
         </is>
       </c>
-      <c r="AW9" s="7">
-        <f>COUNTIF(AU9:AU236,"Fail")+COUNTIF(AU9:AU236,"Broken")</f>
+      <c r="AX9" s="7">
+        <f>COUNTIF(AV9:AV241,"Fail")+COUNTIF(AV9:AV241,"Broken")</f>
       </c>
     </row>
     <row r="10">
@@ -1026,13 +1039,14 @@
       <c r="AS10" s="7"/>
       <c r="AT10" s="7"/>
       <c r="AU10" s="7"/>
-      <c r="AV10" s="2" t="inlineStr">
+      <c r="AV10" s="7"/>
+      <c r="AW10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">N/A</t>
         </is>
       </c>
-      <c r="AW10" s="7">
-        <f>COUNTIF(AU9:AU236,"N/A")</f>
+      <c r="AX10" s="7">
+        <f>COUNTIF(AV9:AV241,"N/A")</f>
       </c>
     </row>
     <row r="11">
@@ -1107,13 +1121,14 @@
       <c r="AS11" s="7"/>
       <c r="AT11" s="7"/>
       <c r="AU11" s="7"/>
-      <c r="AV11" s="2" t="inlineStr">
+      <c r="AV11" s="7"/>
+      <c r="AW11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">전체 개수</t>
         </is>
       </c>
-      <c r="AW11" s="7">
-        <v>228</v>
+      <c r="AX11" s="7">
+        <v>233</v>
       </c>
     </row>
     <row r="12">
@@ -1188,13 +1203,14 @@
       <c r="AS12" s="7"/>
       <c r="AT12" s="7"/>
       <c r="AU12" s="7"/>
-      <c r="AV12" s="2" t="inlineStr">
+      <c r="AV12" s="7"/>
+      <c r="AW12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">진행율</t>
         </is>
       </c>
-      <c r="AW12" s="7">
-        <f>TEXT((COUNTA(AU9:AU236))/228,"0.00%")</f>
+      <c r="AX12" s="7">
+        <f>TEXT((COUNTA(AV9:AV241))/233,"0.00%")</f>
       </c>
     </row>
     <row r="13">
@@ -1273,6 +1289,7 @@
       <c r="AS13" s="7"/>
       <c r="AT13" s="7"/>
       <c r="AU13" s="7"/>
+      <c r="AV13" s="7"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -1341,6 +1358,7 @@
       <c r="AS14" s="7"/>
       <c r="AT14" s="7"/>
       <c r="AU14" s="7"/>
+      <c r="AV14" s="7"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -1445,6 +1463,7 @@
       <c r="AS15" s="7"/>
       <c r="AT15" s="7"/>
       <c r="AU15" s="7"/>
+      <c r="AV15" s="7"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -1549,6 +1568,7 @@
       <c r="AS16" s="7"/>
       <c r="AT16" s="7"/>
       <c r="AU16" s="7"/>
+      <c r="AV16" s="7"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -1658,6 +1678,7 @@
       <c r="AS17" s="7"/>
       <c r="AT17" s="7"/>
       <c r="AU17" s="7"/>
+      <c r="AV17" s="7"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -1731,6 +1752,7 @@
       <c r="AS18" s="7"/>
       <c r="AT18" s="7"/>
       <c r="AU18" s="7"/>
+      <c r="AV18" s="7"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -1799,6 +1821,7 @@
       <c r="AS19" s="7"/>
       <c r="AT19" s="7"/>
       <c r="AU19" s="7"/>
+      <c r="AV19" s="7"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1867,6 +1890,7 @@
       <c r="AS20" s="7"/>
       <c r="AT20" s="7"/>
       <c r="AU20" s="7"/>
+      <c r="AV20" s="7"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1971,6 +1995,7 @@
       <c r="AS21" s="7"/>
       <c r="AT21" s="7"/>
       <c r="AU21" s="7"/>
+      <c r="AV21" s="7"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -2068,6 +2093,7 @@
       <c r="AS22" s="7"/>
       <c r="AT22" s="7"/>
       <c r="AU22" s="7"/>
+      <c r="AV22" s="7"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -2144,6 +2170,7 @@
       <c r="AS23" s="7"/>
       <c r="AT23" s="7"/>
       <c r="AU23" s="7"/>
+      <c r="AV23" s="7"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -2212,6 +2239,7 @@
       <c r="AS24" s="7"/>
       <c r="AT24" s="7"/>
       <c r="AU24" s="7"/>
+      <c r="AV24" s="7"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -2280,6 +2308,7 @@
       <c r="AS25" s="7"/>
       <c r="AT25" s="7"/>
       <c r="AU25" s="7"/>
+      <c r="AV25" s="7"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -2377,6 +2406,7 @@
       <c r="AS26" s="7"/>
       <c r="AT26" s="7"/>
       <c r="AU26" s="7"/>
+      <c r="AV26" s="7"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -2449,6 +2479,7 @@
       <c r="AS27" s="7"/>
       <c r="AT27" s="7"/>
       <c r="AU27" s="7"/>
+      <c r="AV27" s="7"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -2530,6 +2561,7 @@
       <c r="AS28" s="7"/>
       <c r="AT28" s="7"/>
       <c r="AU28" s="7"/>
+      <c r="AV28" s="7"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -2606,6 +2638,7 @@
       <c r="AS29" s="7"/>
       <c r="AT29" s="7"/>
       <c r="AU29" s="7"/>
+      <c r="AV29" s="7"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -2706,6 +2739,7 @@
       <c r="AS30" s="7"/>
       <c r="AT30" s="7"/>
       <c r="AU30" s="7"/>
+      <c r="AV30" s="7"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
@@ -2811,6 +2845,7 @@
       <c r="AS31" s="7"/>
       <c r="AT31" s="7"/>
       <c r="AU31" s="7"/>
+      <c r="AV31" s="7"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
@@ -2903,6 +2938,7 @@
       <c r="AS32" s="7"/>
       <c r="AT32" s="7"/>
       <c r="AU32" s="7"/>
+      <c r="AV32" s="7"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -3003,6 +3039,7 @@
       <c r="AS33" s="7"/>
       <c r="AT33" s="7"/>
       <c r="AU33" s="7"/>
+      <c r="AV33" s="7"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
@@ -3103,6 +3140,7 @@
       <c r="AS34" s="7"/>
       <c r="AT34" s="7"/>
       <c r="AU34" s="7"/>
+      <c r="AV34" s="7"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -3212,6 +3250,7 @@
       <c r="AS35" s="7"/>
       <c r="AT35" s="7"/>
       <c r="AU35" s="7"/>
+      <c r="AV35" s="7"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -3296,6 +3335,7 @@
       <c r="AS36" s="7"/>
       <c r="AT36" s="7"/>
       <c r="AU36" s="7"/>
+      <c r="AV36" s="7"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -3364,6 +3404,7 @@
       <c r="AS37" s="7"/>
       <c r="AT37" s="7"/>
       <c r="AU37" s="7"/>
+      <c r="AV37" s="7"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -3453,6 +3494,7 @@
       <c r="AS38" s="7"/>
       <c r="AT38" s="7"/>
       <c r="AU38" s="7"/>
+      <c r="AV38" s="7"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -3553,6 +3595,7 @@
       <c r="AS39" s="7"/>
       <c r="AT39" s="7"/>
       <c r="AU39" s="7"/>
+      <c r="AV39" s="7"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -3654,6 +3697,7 @@
       <c r="AS40" s="7"/>
       <c r="AT40" s="7"/>
       <c r="AU40" s="7"/>
+      <c r="AV40" s="7"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -3750,6 +3794,7 @@
       <c r="AS41" s="7"/>
       <c r="AT41" s="7"/>
       <c r="AU41" s="7"/>
+      <c r="AV41" s="7"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
@@ -3830,6 +3875,7 @@
       <c r="AS42" s="7"/>
       <c r="AT42" s="7"/>
       <c r="AU42" s="7"/>
+      <c r="AV42" s="7"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -3930,6 +3976,7 @@
       <c r="AS43" s="7"/>
       <c r="AT43" s="7"/>
       <c r="AU43" s="7"/>
+      <c r="AV43" s="7"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
@@ -4003,6 +4050,7 @@
       <c r="AS44" s="7"/>
       <c r="AT44" s="7"/>
       <c r="AU44" s="7"/>
+      <c r="AV44" s="7"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -4099,6 +4147,7 @@
       <c r="AS45" s="7"/>
       <c r="AT45" s="7"/>
       <c r="AU45" s="7"/>
+      <c r="AV45" s="7"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -4195,6 +4244,7 @@
       <c r="AS46" s="7"/>
       <c r="AT46" s="7"/>
       <c r="AU46" s="7"/>
+      <c r="AV46" s="7"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -4268,6 +4318,7 @@
       <c r="AS47" s="7"/>
       <c r="AT47" s="7"/>
       <c r="AU47" s="7"/>
+      <c r="AV47" s="7"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -4336,6 +4387,7 @@
       <c r="AS48" s="7"/>
       <c r="AT48" s="7"/>
       <c r="AU48" s="7"/>
+      <c r="AV48" s="7"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -4404,6 +4456,7 @@
       <c r="AS49" s="7"/>
       <c r="AT49" s="7"/>
       <c r="AU49" s="7"/>
+      <c r="AV49" s="7"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -4496,6 +4549,7 @@
       <c r="AS50" s="7"/>
       <c r="AT50" s="7"/>
       <c r="AU50" s="7"/>
+      <c r="AV50" s="7"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -4588,6 +4642,7 @@
       <c r="AS51" s="7"/>
       <c r="AT51" s="7"/>
       <c r="AU51" s="7"/>
+      <c r="AV51" s="7"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -4661,6 +4716,7 @@
       <c r="AS52" s="7"/>
       <c r="AT52" s="7"/>
       <c r="AU52" s="7"/>
+      <c r="AV52" s="7"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -4734,6 +4790,7 @@
       <c r="AS53" s="7"/>
       <c r="AT53" s="7"/>
       <c r="AU53" s="7"/>
+      <c r="AV53" s="7"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -4802,6 +4859,7 @@
       <c r="AS54" s="7"/>
       <c r="AT54" s="7"/>
       <c r="AU54" s="7"/>
+      <c r="AV54" s="7"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
@@ -4906,6 +4964,7 @@
       <c r="AS55" s="7"/>
       <c r="AT55" s="7"/>
       <c r="AU55" s="7"/>
+      <c r="AV55" s="7"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -4990,6 +5049,7 @@
       <c r="AS56" s="7"/>
       <c r="AT56" s="7"/>
       <c r="AU56" s="7"/>
+      <c r="AV56" s="7"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
@@ -5083,6 +5143,7 @@
       <c r="AS57" s="7"/>
       <c r="AT57" s="7"/>
       <c r="AU57" s="7"/>
+      <c r="AV57" s="7"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -5184,6 +5245,7 @@
       <c r="AS58" s="7"/>
       <c r="AT58" s="7"/>
       <c r="AU58" s="7"/>
+      <c r="AV58" s="7"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -5252,6 +5314,7 @@
       <c r="AS59" s="7"/>
       <c r="AT59" s="7"/>
       <c r="AU59" s="7"/>
+      <c r="AV59" s="7"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -5320,6 +5383,7 @@
       <c r="AS60" s="7"/>
       <c r="AT60" s="7"/>
       <c r="AU60" s="7"/>
+      <c r="AV60" s="7"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -5400,6 +5464,7 @@
       <c r="AS61" s="7"/>
       <c r="AT61" s="7"/>
       <c r="AU61" s="7"/>
+      <c r="AV61" s="7"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
@@ -5488,6 +5553,7 @@
       <c r="AS62" s="7"/>
       <c r="AT62" s="7"/>
       <c r="AU62" s="7"/>
+      <c r="AV62" s="7"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -5568,6 +5634,7 @@
       <c r="AS63" s="7"/>
       <c r="AT63" s="7"/>
       <c r="AU63" s="7"/>
+      <c r="AV63" s="7"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
@@ -5636,6 +5703,7 @@
       <c r="AS64" s="7"/>
       <c r="AT64" s="7"/>
       <c r="AU64" s="7"/>
+      <c r="AV64" s="7"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
@@ -5709,6 +5777,7 @@
       <c r="AS65" s="7"/>
       <c r="AT65" s="7"/>
       <c r="AU65" s="7"/>
+      <c r="AV65" s="7"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
@@ -5789,6 +5858,7 @@
       <c r="AS66" s="7"/>
       <c r="AT66" s="7"/>
       <c r="AU66" s="7"/>
+      <c r="AV66" s="7"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
@@ -5857,6 +5927,7 @@
       <c r="AS67" s="7"/>
       <c r="AT67" s="7"/>
       <c r="AU67" s="7"/>
+      <c r="AV67" s="7"/>
     </row>
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
@@ -5929,6 +6000,7 @@
       <c r="AS68" s="7"/>
       <c r="AT68" s="7"/>
       <c r="AU68" s="7"/>
+      <c r="AV68" s="7"/>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
@@ -6033,6 +6105,7 @@
       <c r="AS69" s="7"/>
       <c r="AT69" s="7"/>
       <c r="AU69" s="7"/>
+      <c r="AV69" s="7"/>
     </row>
     <row r="70">
       <c r="A70" s="7" t="inlineStr">
@@ -6101,6 +6174,7 @@
       <c r="AS70" s="7"/>
       <c r="AT70" s="7"/>
       <c r="AU70" s="7"/>
+      <c r="AV70" s="7"/>
     </row>
     <row r="71">
       <c r="A71" s="7" t="inlineStr">
@@ -6174,6 +6248,7 @@
       <c r="AS71" s="7"/>
       <c r="AT71" s="7"/>
       <c r="AU71" s="7"/>
+      <c r="AV71" s="7"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
@@ -6258,6 +6333,7 @@
       <c r="AS72" s="7"/>
       <c r="AT72" s="7"/>
       <c r="AU72" s="7"/>
+      <c r="AV72" s="7"/>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
@@ -6331,6 +6407,7 @@
       <c r="AS73" s="7"/>
       <c r="AT73" s="7"/>
       <c r="AU73" s="7"/>
+      <c r="AV73" s="7"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -6399,6 +6476,7 @@
       <c r="AS74" s="7"/>
       <c r="AT74" s="7"/>
       <c r="AU74" s="7"/>
+      <c r="AV74" s="7"/>
     </row>
     <row r="75">
       <c r="A75" s="7" t="inlineStr">
@@ -6467,6 +6545,7 @@
       <c r="AS75" s="7"/>
       <c r="AT75" s="7"/>
       <c r="AU75" s="7"/>
+      <c r="AV75" s="7"/>
     </row>
     <row r="76">
       <c r="A76" s="7" t="inlineStr">
@@ -6535,6 +6614,7 @@
       <c r="AS76" s="7"/>
       <c r="AT76" s="7"/>
       <c r="AU76" s="7"/>
+      <c r="AV76" s="7"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -6607,6 +6687,7 @@
       <c r="AS77" s="7"/>
       <c r="AT77" s="7"/>
       <c r="AU77" s="7"/>
+      <c r="AV77" s="7"/>
     </row>
     <row r="78">
       <c r="A78" s="7" t="inlineStr">
@@ -6675,6 +6756,7 @@
       <c r="AS78" s="7"/>
       <c r="AT78" s="7"/>
       <c r="AU78" s="7"/>
+      <c r="AV78" s="7"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -6748,6 +6830,7 @@
       <c r="AS79" s="7"/>
       <c r="AT79" s="7"/>
       <c r="AU79" s="7"/>
+      <c r="AV79" s="7"/>
     </row>
     <row r="80">
       <c r="A80" s="7" t="inlineStr">
@@ -6832,6 +6915,7 @@
       <c r="AS80" s="7"/>
       <c r="AT80" s="7"/>
       <c r="AU80" s="7"/>
+      <c r="AV80" s="7"/>
     </row>
     <row r="81">
       <c r="A81" s="7" t="inlineStr">
@@ -6904,6 +6988,7 @@
       <c r="AS81" s="7"/>
       <c r="AT81" s="7"/>
       <c r="AU81" s="7"/>
+      <c r="AV81" s="7"/>
     </row>
     <row r="82">
       <c r="A82" s="7" t="inlineStr">
@@ -6972,6 +7057,7 @@
       <c r="AS82" s="7"/>
       <c r="AT82" s="7"/>
       <c r="AU82" s="7"/>
+      <c r="AV82" s="7"/>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
@@ -7045,6 +7131,7 @@
       <c r="AS83" s="7"/>
       <c r="AT83" s="7"/>
       <c r="AU83" s="7"/>
+      <c r="AV83" s="7"/>
     </row>
     <row r="84">
       <c r="A84" s="7" t="inlineStr">
@@ -7113,6 +7200,7 @@
       <c r="AS84" s="7"/>
       <c r="AT84" s="7"/>
       <c r="AU84" s="7"/>
+      <c r="AV84" s="7"/>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
@@ -7181,6 +7269,7 @@
       <c r="AS85" s="7"/>
       <c r="AT85" s="7"/>
       <c r="AU85" s="7"/>
+      <c r="AV85" s="7"/>
     </row>
     <row r="86">
       <c r="A86" s="7" t="inlineStr">
@@ -7254,6 +7343,7 @@
       <c r="AS86" s="7"/>
       <c r="AT86" s="7"/>
       <c r="AU86" s="7"/>
+      <c r="AV86" s="7"/>
     </row>
     <row r="87">
       <c r="A87" s="7" t="inlineStr">
@@ -7322,6 +7412,7 @@
       <c r="AS87" s="7"/>
       <c r="AT87" s="7"/>
       <c r="AU87" s="7"/>
+      <c r="AV87" s="7"/>
     </row>
     <row r="88">
       <c r="A88" s="7" t="inlineStr">
@@ -7390,6 +7481,7 @@
       <c r="AS88" s="7"/>
       <c r="AT88" s="7"/>
       <c r="AU88" s="7"/>
+      <c r="AV88" s="7"/>
     </row>
     <row r="89">
       <c r="A89" s="7" t="inlineStr">
@@ -7458,6 +7550,7 @@
       <c r="AS89" s="7"/>
       <c r="AT89" s="7"/>
       <c r="AU89" s="7"/>
+      <c r="AV89" s="7"/>
     </row>
     <row r="90">
       <c r="A90" s="7" t="inlineStr">
@@ -7555,6 +7648,7 @@
       <c r="AS90" s="7"/>
       <c r="AT90" s="7"/>
       <c r="AU90" s="7"/>
+      <c r="AV90" s="7"/>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
@@ -7623,6 +7717,7 @@
       <c r="AS91" s="7"/>
       <c r="AT91" s="7"/>
       <c r="AU91" s="7"/>
+      <c r="AV91" s="7"/>
     </row>
     <row r="92">
       <c r="A92" s="7" t="inlineStr">
@@ -7727,6 +7822,7 @@
       <c r="AS92" s="7"/>
       <c r="AT92" s="7"/>
       <c r="AU92" s="7"/>
+      <c r="AV92" s="7"/>
     </row>
     <row r="93">
       <c r="A93" s="7" t="inlineStr">
@@ -7836,6 +7932,7 @@
       <c r="AS93" s="7"/>
       <c r="AT93" s="7"/>
       <c r="AU93" s="7"/>
+      <c r="AV93" s="7"/>
     </row>
     <row r="94">
       <c r="A94" s="7" t="inlineStr">
@@ -7909,6 +8006,7 @@
       <c r="AS94" s="7"/>
       <c r="AT94" s="7"/>
       <c r="AU94" s="7"/>
+      <c r="AV94" s="7"/>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
@@ -7982,6 +8080,7 @@
       <c r="AS95" s="7"/>
       <c r="AT95" s="7"/>
       <c r="AU95" s="7"/>
+      <c r="AV95" s="7"/>
     </row>
     <row r="96">
       <c r="A96" s="7" t="inlineStr">
@@ -8074,6 +8173,7 @@
       <c r="AS96" s="7"/>
       <c r="AT96" s="7"/>
       <c r="AU96" s="7"/>
+      <c r="AV96" s="7"/>
     </row>
     <row r="97">
       <c r="A97" s="7" t="inlineStr">
@@ -8142,6 +8242,7 @@
       <c r="AS97" s="7"/>
       <c r="AT97" s="7"/>
       <c r="AU97" s="7"/>
+      <c r="AV97" s="7"/>
     </row>
     <row r="98">
       <c r="A98" s="7" t="inlineStr">
@@ -8210,6 +8311,7 @@
       <c r="AS98" s="7"/>
       <c r="AT98" s="7"/>
       <c r="AU98" s="7"/>
+      <c r="AV98" s="7"/>
     </row>
     <row r="99">
       <c r="A99" s="7" t="inlineStr">
@@ -8278,6 +8380,7 @@
       <c r="AS99" s="7"/>
       <c r="AT99" s="7"/>
       <c r="AU99" s="7"/>
+      <c r="AV99" s="7"/>
     </row>
     <row r="100">
       <c r="A100" s="7" t="inlineStr">
@@ -8355,6 +8458,7 @@
       <c r="AS100" s="7"/>
       <c r="AT100" s="7"/>
       <c r="AU100" s="7"/>
+      <c r="AV100" s="7"/>
     </row>
     <row r="101">
       <c r="A101" s="7" t="inlineStr">
@@ -8423,6 +8527,7 @@
       <c r="AS101" s="7"/>
       <c r="AT101" s="7"/>
       <c r="AU101" s="7"/>
+      <c r="AV101" s="7"/>
     </row>
     <row r="102">
       <c r="A102" s="7" t="inlineStr">
@@ -8491,6 +8596,7 @@
       <c r="AS102" s="7"/>
       <c r="AT102" s="7"/>
       <c r="AU102" s="7"/>
+      <c r="AV102" s="7"/>
     </row>
     <row r="103">
       <c r="A103" s="7" t="inlineStr">
@@ -8559,6 +8665,7 @@
       <c r="AS103" s="7"/>
       <c r="AT103" s="7"/>
       <c r="AU103" s="7"/>
+      <c r="AV103" s="7"/>
     </row>
     <row r="104">
       <c r="A104" s="7" t="inlineStr">
@@ -8632,6 +8739,7 @@
       <c r="AS104" s="7"/>
       <c r="AT104" s="7"/>
       <c r="AU104" s="7"/>
+      <c r="AV104" s="7"/>
     </row>
     <row r="105">
       <c r="A105" s="7" t="inlineStr">
@@ -8700,6 +8808,7 @@
       <c r="AS105" s="7"/>
       <c r="AT105" s="7"/>
       <c r="AU105" s="7"/>
+      <c r="AV105" s="7"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
@@ -8768,6 +8877,7 @@
       <c r="AS106" s="7"/>
       <c r="AT106" s="7"/>
       <c r="AU106" s="7"/>
+      <c r="AV106" s="7"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="inlineStr">
@@ -8836,6 +8946,7 @@
       <c r="AS107" s="7"/>
       <c r="AT107" s="7"/>
       <c r="AU107" s="7"/>
+      <c r="AV107" s="7"/>
     </row>
     <row r="108">
       <c r="A108" s="7" t="inlineStr">
@@ -8908,6 +9019,7 @@
       <c r="AS108" s="7"/>
       <c r="AT108" s="7"/>
       <c r="AU108" s="7"/>
+      <c r="AV108" s="7"/>
     </row>
     <row r="109">
       <c r="A109" s="7" t="inlineStr">
@@ -8985,6 +9097,7 @@
       <c r="AS109" s="7"/>
       <c r="AT109" s="7"/>
       <c r="AU109" s="7"/>
+      <c r="AV109" s="7"/>
     </row>
     <row r="110">
       <c r="A110" s="7" t="inlineStr">
@@ -9070,6 +9183,7 @@
       <c r="AS110" s="7"/>
       <c r="AT110" s="7"/>
       <c r="AU110" s="7"/>
+      <c r="AV110" s="7"/>
     </row>
     <row r="111">
       <c r="A111" s="7" t="inlineStr">
@@ -9158,6 +9272,7 @@
       <c r="AS111" s="7"/>
       <c r="AT111" s="7"/>
       <c r="AU111" s="7"/>
+      <c r="AV111" s="7"/>
     </row>
     <row r="112">
       <c r="A112" s="7" t="inlineStr">
@@ -9243,6 +9358,7 @@
       <c r="AS112" s="7"/>
       <c r="AT112" s="7"/>
       <c r="AU112" s="7"/>
+      <c r="AV112" s="7"/>
     </row>
     <row r="113">
       <c r="A113" s="7" t="inlineStr">
@@ -9320,6 +9436,7 @@
       <c r="AS113" s="7"/>
       <c r="AT113" s="7"/>
       <c r="AU113" s="7"/>
+      <c r="AV113" s="7"/>
     </row>
     <row r="114">
       <c r="A114" s="7" t="inlineStr">
@@ -9413,6 +9530,7 @@
       <c r="AS114" s="7"/>
       <c r="AT114" s="7"/>
       <c r="AU114" s="7"/>
+      <c r="AV114" s="7"/>
     </row>
     <row r="115">
       <c r="A115" s="7" t="inlineStr">
@@ -9498,6 +9616,7 @@
       <c r="AS115" s="7"/>
       <c r="AT115" s="7"/>
       <c r="AU115" s="7"/>
+      <c r="AV115" s="7"/>
     </row>
     <row r="116">
       <c r="A116" s="7" t="inlineStr">
@@ -9591,6 +9710,7 @@
       <c r="AS116" s="7"/>
       <c r="AT116" s="7"/>
       <c r="AU116" s="7"/>
+      <c r="AV116" s="7"/>
     </row>
     <row r="117">
       <c r="A117" s="7" t="inlineStr">
@@ -9680,6 +9800,7 @@
       <c r="AS117" s="7"/>
       <c r="AT117" s="7"/>
       <c r="AU117" s="7"/>
+      <c r="AV117" s="7"/>
     </row>
     <row r="118">
       <c r="A118" s="7" t="inlineStr">
@@ -9769,6 +9890,7 @@
       <c r="AS118" s="7"/>
       <c r="AT118" s="7"/>
       <c r="AU118" s="7"/>
+      <c r="AV118" s="7"/>
     </row>
     <row r="119">
       <c r="A119" s="7" t="inlineStr">
@@ -9854,6 +9976,7 @@
       <c r="AS119" s="7"/>
       <c r="AT119" s="7"/>
       <c r="AU119" s="7"/>
+      <c r="AV119" s="7"/>
     </row>
     <row r="120">
       <c r="A120" s="7" t="inlineStr">
@@ -9931,6 +10054,7 @@
       <c r="AS120" s="7"/>
       <c r="AT120" s="7"/>
       <c r="AU120" s="7"/>
+      <c r="AV120" s="7"/>
     </row>
     <row r="121">
       <c r="A121" s="7" t="inlineStr">
@@ -10020,6 +10144,7 @@
       <c r="AS121" s="7"/>
       <c r="AT121" s="7"/>
       <c r="AU121" s="7"/>
+      <c r="AV121" s="7"/>
     </row>
     <row r="122">
       <c r="A122" s="7" t="inlineStr">
@@ -10109,6 +10234,7 @@
       <c r="AS122" s="7"/>
       <c r="AT122" s="7"/>
       <c r="AU122" s="7"/>
+      <c r="AV122" s="7"/>
     </row>
     <row r="123">
       <c r="A123" s="7" t="inlineStr">
@@ -10186,6 +10312,7 @@
       <c r="AS123" s="7"/>
       <c r="AT123" s="7"/>
       <c r="AU123" s="7"/>
+      <c r="AV123" s="7"/>
     </row>
     <row r="124">
       <c r="A124" s="7" t="inlineStr">
@@ -10271,6 +10398,7 @@
       <c r="AS124" s="7"/>
       <c r="AT124" s="7"/>
       <c r="AU124" s="7"/>
+      <c r="AV124" s="7"/>
     </row>
     <row r="125">
       <c r="A125" s="7" t="inlineStr">
@@ -10348,6 +10476,7 @@
       <c r="AS125" s="7"/>
       <c r="AT125" s="7"/>
       <c r="AU125" s="7"/>
+      <c r="AV125" s="7"/>
     </row>
     <row r="126">
       <c r="A126" s="7" t="inlineStr">
@@ -10425,6 +10554,7 @@
       <c r="AS126" s="7"/>
       <c r="AT126" s="7"/>
       <c r="AU126" s="7"/>
+      <c r="AV126" s="7"/>
     </row>
     <row r="127">
       <c r="A127" s="7" t="inlineStr">
@@ -10506,6 +10636,7 @@
       <c r="AS127" s="7"/>
       <c r="AT127" s="7"/>
       <c r="AU127" s="7"/>
+      <c r="AV127" s="7"/>
     </row>
     <row r="128">
       <c r="A128" s="7" t="inlineStr">
@@ -10587,6 +10718,7 @@
       <c r="AS128" s="7"/>
       <c r="AT128" s="7"/>
       <c r="AU128" s="7"/>
+      <c r="AV128" s="7"/>
     </row>
     <row r="129">
       <c r="A129" s="7" t="inlineStr">
@@ -10668,6 +10800,7 @@
       <c r="AS129" s="7"/>
       <c r="AT129" s="7"/>
       <c r="AU129" s="7"/>
+      <c r="AV129" s="7"/>
     </row>
     <row r="130">
       <c r="A130" s="7" t="inlineStr">
@@ -10745,6 +10878,7 @@
       <c r="AS130" s="7"/>
       <c r="AT130" s="7"/>
       <c r="AU130" s="7"/>
+      <c r="AV130" s="7"/>
     </row>
     <row r="131">
       <c r="A131" s="7" t="inlineStr">
@@ -10830,6 +10964,7 @@
       <c r="AS131" s="7"/>
       <c r="AT131" s="7"/>
       <c r="AU131" s="7"/>
+      <c r="AV131" s="7"/>
     </row>
     <row r="132">
       <c r="A132" s="7" t="inlineStr">
@@ -10919,6 +11054,7 @@
       <c r="AS132" s="7"/>
       <c r="AT132" s="7"/>
       <c r="AU132" s="7"/>
+      <c r="AV132" s="7"/>
     </row>
     <row r="133">
       <c r="A133" s="7" t="inlineStr">
@@ -11008,6 +11144,7 @@
       <c r="AS133" s="7"/>
       <c r="AT133" s="7"/>
       <c r="AU133" s="7"/>
+      <c r="AV133" s="7"/>
     </row>
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
@@ -11093,6 +11230,7 @@
       <c r="AS134" s="7"/>
       <c r="AT134" s="7"/>
       <c r="AU134" s="7"/>
+      <c r="AV134" s="7"/>
     </row>
     <row r="135">
       <c r="A135" s="7" t="inlineStr">
@@ -11178,6 +11316,7 @@
       <c r="AS135" s="7"/>
       <c r="AT135" s="7"/>
       <c r="AU135" s="7"/>
+      <c r="AV135" s="7"/>
     </row>
     <row r="136">
       <c r="A136" s="7" t="inlineStr">
@@ -11263,6 +11402,7 @@
       <c r="AS136" s="7"/>
       <c r="AT136" s="7"/>
       <c r="AU136" s="7"/>
+      <c r="AV136" s="7"/>
     </row>
     <row r="137">
       <c r="A137" s="7" t="inlineStr">
@@ -11344,6 +11484,7 @@
       <c r="AS137" s="7"/>
       <c r="AT137" s="7"/>
       <c r="AU137" s="7"/>
+      <c r="AV137" s="7"/>
     </row>
     <row r="138">
       <c r="A138" s="7" t="inlineStr">
@@ -11425,6 +11566,7 @@
       <c r="AS138" s="7"/>
       <c r="AT138" s="7"/>
       <c r="AU138" s="7"/>
+      <c r="AV138" s="7"/>
     </row>
     <row r="139">
       <c r="A139" s="7" t="inlineStr">
@@ -11506,6 +11648,7 @@
       <c r="AS139" s="7"/>
       <c r="AT139" s="7"/>
       <c r="AU139" s="7"/>
+      <c r="AV139" s="7"/>
     </row>
     <row r="140">
       <c r="A140" s="7" t="inlineStr">
@@ -11583,6 +11726,7 @@
       <c r="AS140" s="7"/>
       <c r="AT140" s="7"/>
       <c r="AU140" s="7"/>
+      <c r="AV140" s="7"/>
     </row>
     <row r="141">
       <c r="A141" s="7" t="inlineStr">
@@ -11672,6 +11816,7 @@
       <c r="AS141" s="7"/>
       <c r="AT141" s="7"/>
       <c r="AU141" s="7"/>
+      <c r="AV141" s="7"/>
     </row>
     <row r="142">
       <c r="A142" s="7" t="inlineStr">
@@ -11749,6 +11894,7 @@
       <c r="AS142" s="7"/>
       <c r="AT142" s="7"/>
       <c r="AU142" s="7"/>
+      <c r="AV142" s="7"/>
     </row>
     <row r="143">
       <c r="A143" s="7" t="inlineStr">
@@ -11826,6 +11972,7 @@
       <c r="AS143" s="7"/>
       <c r="AT143" s="7"/>
       <c r="AU143" s="7"/>
+      <c r="AV143" s="7"/>
     </row>
     <row r="144">
       <c r="A144" s="7" t="inlineStr">
@@ -11903,6 +12050,7 @@
       <c r="AS144" s="7"/>
       <c r="AT144" s="7"/>
       <c r="AU144" s="7"/>
+      <c r="AV144" s="7"/>
     </row>
     <row r="145">
       <c r="A145" s="7" t="inlineStr">
@@ -11996,6 +12144,7 @@
       <c r="AS145" s="7"/>
       <c r="AT145" s="7"/>
       <c r="AU145" s="7"/>
+      <c r="AV145" s="7"/>
     </row>
     <row r="146">
       <c r="A146" s="7" t="inlineStr">
@@ -12077,6 +12226,7 @@
       <c r="AS146" s="7"/>
       <c r="AT146" s="7"/>
       <c r="AU146" s="7"/>
+      <c r="AV146" s="7"/>
     </row>
     <row r="147">
       <c r="A147" s="7" t="inlineStr">
@@ -12170,6 +12320,7 @@
       <c r="AS147" s="7"/>
       <c r="AT147" s="7"/>
       <c r="AU147" s="7"/>
+      <c r="AV147" s="7"/>
     </row>
     <row r="148">
       <c r="A148" s="7" t="inlineStr">
@@ -12247,6 +12398,7 @@
       <c r="AS148" s="7"/>
       <c r="AT148" s="7"/>
       <c r="AU148" s="7"/>
+      <c r="AV148" s="7"/>
     </row>
     <row r="149">
       <c r="A149" s="7" t="inlineStr">
@@ -12332,6 +12484,7 @@
       <c r="AS149" s="7"/>
       <c r="AT149" s="7"/>
       <c r="AU149" s="7"/>
+      <c r="AV149" s="7"/>
     </row>
     <row r="150">
       <c r="A150" s="7" t="inlineStr">
@@ -12421,6 +12574,7 @@
       <c r="AS150" s="7"/>
       <c r="AT150" s="7"/>
       <c r="AU150" s="7"/>
+      <c r="AV150" s="7"/>
     </row>
     <row r="151">
       <c r="A151" s="7" t="inlineStr">
@@ -12502,6 +12656,7 @@
       <c r="AS151" s="7"/>
       <c r="AT151" s="7"/>
       <c r="AU151" s="7"/>
+      <c r="AV151" s="7"/>
     </row>
     <row r="152">
       <c r="A152" s="7" t="inlineStr">
@@ -12587,6 +12742,7 @@
       <c r="AS152" s="7"/>
       <c r="AT152" s="7"/>
       <c r="AU152" s="7"/>
+      <c r="AV152" s="7"/>
     </row>
     <row r="153">
       <c r="A153" s="7" t="inlineStr">
@@ -12676,6 +12832,7 @@
       <c r="AS153" s="7"/>
       <c r="AT153" s="7"/>
       <c r="AU153" s="7"/>
+      <c r="AV153" s="7"/>
     </row>
     <row r="154">
       <c r="A154" s="7" t="inlineStr">
@@ -12749,6 +12906,7 @@
       <c r="AS154" s="7"/>
       <c r="AT154" s="7"/>
       <c r="AU154" s="7"/>
+      <c r="AV154" s="7"/>
     </row>
     <row r="155">
       <c r="A155" s="7" t="inlineStr">
@@ -12826,6 +12984,7 @@
       <c r="AS155" s="7"/>
       <c r="AT155" s="7"/>
       <c r="AU155" s="7"/>
+      <c r="AV155" s="7"/>
     </row>
     <row r="156">
       <c r="A156" s="7" t="inlineStr">
@@ -12907,6 +13066,7 @@
       <c r="AS156" s="7"/>
       <c r="AT156" s="7"/>
       <c r="AU156" s="7"/>
+      <c r="AV156" s="7"/>
     </row>
     <row r="157">
       <c r="A157" s="7" t="inlineStr">
@@ -12984,6 +13144,7 @@
       <c r="AS157" s="7"/>
       <c r="AT157" s="7"/>
       <c r="AU157" s="7"/>
+      <c r="AV157" s="7"/>
     </row>
     <row r="158">
       <c r="A158" s="7" t="inlineStr">
@@ -13061,6 +13222,7 @@
       <c r="AS158" s="7"/>
       <c r="AT158" s="7"/>
       <c r="AU158" s="7"/>
+      <c r="AV158" s="7"/>
     </row>
     <row r="159">
       <c r="A159" s="7" t="inlineStr">
@@ -13138,6 +13300,7 @@
       <c r="AS159" s="7"/>
       <c r="AT159" s="7"/>
       <c r="AU159" s="7"/>
+      <c r="AV159" s="7"/>
     </row>
     <row r="160">
       <c r="A160" s="7" t="inlineStr">
@@ -13215,6 +13378,7 @@
       <c r="AS160" s="7"/>
       <c r="AT160" s="7"/>
       <c r="AU160" s="7"/>
+      <c r="AV160" s="7"/>
     </row>
     <row r="161">
       <c r="A161" s="7" t="inlineStr">
@@ -13296,6 +13460,7 @@
       <c r="AS161" s="7"/>
       <c r="AT161" s="7"/>
       <c r="AU161" s="7"/>
+      <c r="AV161" s="7"/>
     </row>
     <row r="162">
       <c r="A162" s="7" t="inlineStr">
@@ -13373,6 +13538,7 @@
       <c r="AS162" s="7"/>
       <c r="AT162" s="7"/>
       <c r="AU162" s="7"/>
+      <c r="AV162" s="7"/>
     </row>
     <row r="163">
       <c r="A163" s="7" t="inlineStr">
@@ -13450,6 +13616,7 @@
       <c r="AS163" s="7"/>
       <c r="AT163" s="7"/>
       <c r="AU163" s="7"/>
+      <c r="AV163" s="7"/>
     </row>
     <row r="164">
       <c r="A164" s="7" t="inlineStr">
@@ -13527,6 +13694,7 @@
       <c r="AS164" s="7"/>
       <c r="AT164" s="7"/>
       <c r="AU164" s="7"/>
+      <c r="AV164" s="7"/>
     </row>
     <row r="165">
       <c r="A165" s="7" t="inlineStr">
@@ -13604,6 +13772,7 @@
       <c r="AS165" s="7"/>
       <c r="AT165" s="7"/>
       <c r="AU165" s="7"/>
+      <c r="AV165" s="7"/>
     </row>
     <row r="166">
       <c r="A166" s="7" t="inlineStr">
@@ -13689,6 +13858,7 @@
       <c r="AS166" s="7"/>
       <c r="AT166" s="7"/>
       <c r="AU166" s="7"/>
+      <c r="AV166" s="7"/>
     </row>
     <row r="167">
       <c r="A167" s="7" t="inlineStr">
@@ -13770,6 +13940,7 @@
       <c r="AS167" s="7"/>
       <c r="AT167" s="7"/>
       <c r="AU167" s="7"/>
+      <c r="AV167" s="7"/>
     </row>
     <row r="168">
       <c r="A168" s="7" t="inlineStr">
@@ -13847,6 +14018,7 @@
       <c r="AS168" s="7"/>
       <c r="AT168" s="7"/>
       <c r="AU168" s="7"/>
+      <c r="AV168" s="7"/>
     </row>
     <row r="169">
       <c r="A169" s="7" t="inlineStr">
@@ -13924,6 +14096,7 @@
       <c r="AS169" s="7"/>
       <c r="AT169" s="7"/>
       <c r="AU169" s="7"/>
+      <c r="AV169" s="7"/>
     </row>
     <row r="170">
       <c r="A170" s="7" t="inlineStr">
@@ -14005,6 +14178,7 @@
       <c r="AS170" s="7"/>
       <c r="AT170" s="7"/>
       <c r="AU170" s="7"/>
+      <c r="AV170" s="7"/>
     </row>
     <row r="171">
       <c r="A171" s="7" t="inlineStr">
@@ -14078,6 +14252,7 @@
       <c r="AS171" s="7"/>
       <c r="AT171" s="7"/>
       <c r="AU171" s="7"/>
+      <c r="AV171" s="7"/>
     </row>
     <row r="172">
       <c r="A172" s="7" t="inlineStr">
@@ -14151,6 +14326,7 @@
       <c r="AS172" s="7"/>
       <c r="AT172" s="7"/>
       <c r="AU172" s="7"/>
+      <c r="AV172" s="7"/>
     </row>
     <row r="173">
       <c r="A173" s="7" t="inlineStr">
@@ -14232,6 +14408,7 @@
       <c r="AS173" s="7"/>
       <c r="AT173" s="7"/>
       <c r="AU173" s="7"/>
+      <c r="AV173" s="7"/>
     </row>
     <row r="174">
       <c r="A174" s="7" t="inlineStr">
@@ -14309,6 +14486,7 @@
       <c r="AS174" s="7"/>
       <c r="AT174" s="7"/>
       <c r="AU174" s="7"/>
+      <c r="AV174" s="7"/>
     </row>
     <row r="175">
       <c r="A175" s="7" t="inlineStr">
@@ -14390,6 +14568,7 @@
       <c r="AS175" s="7"/>
       <c r="AT175" s="7"/>
       <c r="AU175" s="7"/>
+      <c r="AV175" s="7"/>
     </row>
     <row r="176">
       <c r="A176" s="7" t="inlineStr">
@@ -14467,6 +14646,7 @@
       <c r="AS176" s="7"/>
       <c r="AT176" s="7"/>
       <c r="AU176" s="7"/>
+      <c r="AV176" s="7"/>
     </row>
     <row r="177">
       <c r="A177" s="7" t="inlineStr">
@@ -14544,6 +14724,7 @@
       <c r="AS177" s="7"/>
       <c r="AT177" s="7"/>
       <c r="AU177" s="7"/>
+      <c r="AV177" s="7"/>
     </row>
     <row r="178">
       <c r="A178" s="7" t="inlineStr">
@@ -14621,6 +14802,7 @@
       <c r="AS178" s="7"/>
       <c r="AT178" s="7"/>
       <c r="AU178" s="7"/>
+      <c r="AV178" s="7"/>
     </row>
     <row r="179">
       <c r="A179" s="7" t="inlineStr">
@@ -14698,6 +14880,7 @@
       <c r="AS179" s="7"/>
       <c r="AT179" s="7"/>
       <c r="AU179" s="7"/>
+      <c r="AV179" s="7"/>
     </row>
     <row r="180">
       <c r="A180" s="7" t="inlineStr">
@@ -14775,6 +14958,7 @@
       <c r="AS180" s="7"/>
       <c r="AT180" s="7"/>
       <c r="AU180" s="7"/>
+      <c r="AV180" s="7"/>
     </row>
     <row r="181">
       <c r="A181" s="7" t="inlineStr">
@@ -14852,6 +15036,7 @@
       <c r="AS181" s="7"/>
       <c r="AT181" s="7"/>
       <c r="AU181" s="7"/>
+      <c r="AV181" s="7"/>
     </row>
     <row r="182">
       <c r="A182" s="7" t="inlineStr">
@@ -14929,6 +15114,7 @@
       <c r="AS182" s="7"/>
       <c r="AT182" s="7"/>
       <c r="AU182" s="7"/>
+      <c r="AV182" s="7"/>
     </row>
     <row r="183">
       <c r="A183" s="7" t="inlineStr">
@@ -15006,6 +15192,7 @@
       <c r="AS183" s="7"/>
       <c r="AT183" s="7"/>
       <c r="AU183" s="7"/>
+      <c r="AV183" s="7"/>
     </row>
     <row r="184">
       <c r="A184" s="7" t="inlineStr">
@@ -15079,6 +15266,7 @@
       <c r="AS184" s="7"/>
       <c r="AT184" s="7"/>
       <c r="AU184" s="7"/>
+      <c r="AV184" s="7"/>
     </row>
     <row r="185">
       <c r="A185" s="7" t="inlineStr">
@@ -15156,6 +15344,7 @@
       <c r="AS185" s="7"/>
       <c r="AT185" s="7"/>
       <c r="AU185" s="7"/>
+      <c r="AV185" s="7"/>
     </row>
     <row r="186">
       <c r="A186" s="7" t="inlineStr">
@@ -15233,6 +15422,7 @@
       <c r="AS186" s="7"/>
       <c r="AT186" s="7"/>
       <c r="AU186" s="7"/>
+      <c r="AV186" s="7"/>
     </row>
     <row r="187">
       <c r="A187" s="7" t="inlineStr">
@@ -15314,6 +15504,7 @@
       <c r="AS187" s="7"/>
       <c r="AT187" s="7"/>
       <c r="AU187" s="7"/>
+      <c r="AV187" s="7"/>
     </row>
     <row r="188">
       <c r="A188" s="7" t="inlineStr">
@@ -15395,6 +15586,7 @@
       <c r="AS188" s="7"/>
       <c r="AT188" s="7"/>
       <c r="AU188" s="7"/>
+      <c r="AV188" s="7"/>
     </row>
     <row r="189">
       <c r="A189" s="7" t="inlineStr">
@@ -15476,6 +15668,7 @@
       <c r="AS189" s="7"/>
       <c r="AT189" s="7"/>
       <c r="AU189" s="7"/>
+      <c r="AV189" s="7"/>
     </row>
     <row r="190">
       <c r="A190" s="7" t="inlineStr">
@@ -15557,6 +15750,7 @@
       <c r="AS190" s="7"/>
       <c r="AT190" s="7"/>
       <c r="AU190" s="7"/>
+      <c r="AV190" s="7"/>
     </row>
     <row r="191">
       <c r="A191" s="7" t="inlineStr">
@@ -15638,6 +15832,7 @@
       <c r="AS191" s="7"/>
       <c r="AT191" s="7"/>
       <c r="AU191" s="7"/>
+      <c r="AV191" s="7"/>
     </row>
     <row r="192">
       <c r="A192" s="7" t="inlineStr">
@@ -15719,6 +15914,7 @@
       <c r="AS192" s="7"/>
       <c r="AT192" s="7"/>
       <c r="AU192" s="7"/>
+      <c r="AV192" s="7"/>
     </row>
     <row r="193">
       <c r="A193" s="7" t="inlineStr">
@@ -15804,6 +16000,7 @@
       <c r="AS193" s="7"/>
       <c r="AT193" s="7"/>
       <c r="AU193" s="7"/>
+      <c r="AV193" s="7"/>
     </row>
     <row r="194">
       <c r="A194" s="7" t="inlineStr">
@@ -15889,6 +16086,7 @@
       <c r="AS194" s="7"/>
       <c r="AT194" s="7"/>
       <c r="AU194" s="7"/>
+      <c r="AV194" s="7"/>
     </row>
     <row r="195">
       <c r="A195" s="7" t="inlineStr">
@@ -15974,6 +16172,7 @@
       <c r="AS195" s="7"/>
       <c r="AT195" s="7"/>
       <c r="AU195" s="7"/>
+      <c r="AV195" s="7"/>
     </row>
     <row r="196">
       <c r="A196" s="7" t="inlineStr">
@@ -16051,6 +16250,7 @@
       <c r="AS196" s="7"/>
       <c r="AT196" s="7"/>
       <c r="AU196" s="7"/>
+      <c r="AV196" s="7"/>
     </row>
     <row r="197">
       <c r="A197" s="7" t="inlineStr">
@@ -16136,6 +16336,7 @@
       <c r="AS197" s="7"/>
       <c r="AT197" s="7"/>
       <c r="AU197" s="7"/>
+      <c r="AV197" s="7"/>
     </row>
     <row r="198">
       <c r="A198" s="7" t="inlineStr">
@@ -16213,6 +16414,7 @@
       <c r="AS198" s="7"/>
       <c r="AT198" s="7"/>
       <c r="AU198" s="7"/>
+      <c r="AV198" s="7"/>
     </row>
     <row r="199">
       <c r="A199" s="7" t="inlineStr">
@@ -16298,6 +16500,7 @@
       <c r="AS199" s="7"/>
       <c r="AT199" s="7"/>
       <c r="AU199" s="7"/>
+      <c r="AV199" s="7"/>
     </row>
     <row r="200">
       <c r="A200" s="7" t="inlineStr">
@@ -16383,6 +16586,7 @@
       <c r="AS200" s="7"/>
       <c r="AT200" s="7"/>
       <c r="AU200" s="7"/>
+      <c r="AV200" s="7"/>
     </row>
     <row r="201">
       <c r="A201" s="7" t="inlineStr">
@@ -16460,6 +16664,7 @@
       <c r="AS201" s="7"/>
       <c r="AT201" s="7"/>
       <c r="AU201" s="7"/>
+      <c r="AV201" s="7"/>
     </row>
     <row r="202">
       <c r="A202" s="7" t="inlineStr">
@@ -16545,6 +16750,7 @@
       <c r="AS202" s="7"/>
       <c r="AT202" s="7"/>
       <c r="AU202" s="7"/>
+      <c r="AV202" s="7"/>
     </row>
     <row r="203">
       <c r="A203" s="7" t="inlineStr">
@@ -16630,6 +16836,7 @@
       <c r="AS203" s="7"/>
       <c r="AT203" s="7"/>
       <c r="AU203" s="7"/>
+      <c r="AV203" s="7"/>
     </row>
     <row r="204">
       <c r="A204" s="7" t="inlineStr">
@@ -16719,6 +16926,7 @@
       <c r="AS204" s="7"/>
       <c r="AT204" s="7"/>
       <c r="AU204" s="7"/>
+      <c r="AV204" s="7"/>
     </row>
     <row r="205">
       <c r="A205" s="7" t="inlineStr">
@@ -16808,6 +17016,7 @@
       <c r="AS205" s="7"/>
       <c r="AT205" s="7"/>
       <c r="AU205" s="7"/>
+      <c r="AV205" s="7"/>
     </row>
     <row r="206">
       <c r="A206" s="7" t="inlineStr">
@@ -16897,6 +17106,7 @@
       <c r="AS206" s="7"/>
       <c r="AT206" s="7"/>
       <c r="AU206" s="7"/>
+      <c r="AV206" s="7"/>
     </row>
     <row r="207">
       <c r="A207" s="7" t="inlineStr">
@@ -16978,6 +17188,7 @@
       <c r="AS207" s="7"/>
       <c r="AT207" s="7"/>
       <c r="AU207" s="7"/>
+      <c r="AV207" s="7"/>
     </row>
     <row r="208">
       <c r="A208" s="7" t="inlineStr">
@@ -17063,6 +17274,7 @@
       <c r="AS208" s="7"/>
       <c r="AT208" s="7"/>
       <c r="AU208" s="7"/>
+      <c r="AV208" s="7"/>
     </row>
     <row r="209">
       <c r="A209" s="7" t="inlineStr">
@@ -17152,6 +17364,7 @@
       <c r="AS209" s="7"/>
       <c r="AT209" s="7"/>
       <c r="AU209" s="7"/>
+      <c r="AV209" s="7"/>
     </row>
     <row r="210">
       <c r="A210" s="7" t="inlineStr">
@@ -17237,6 +17450,7 @@
       <c r="AS210" s="7"/>
       <c r="AT210" s="7"/>
       <c r="AU210" s="7"/>
+      <c r="AV210" s="7"/>
     </row>
     <row r="211">
       <c r="A211" s="7" t="inlineStr">
@@ -17314,6 +17528,7 @@
       <c r="AS211" s="7"/>
       <c r="AT211" s="7"/>
       <c r="AU211" s="7"/>
+      <c r="AV211" s="7"/>
     </row>
     <row r="212">
       <c r="A212" s="7" t="inlineStr">
@@ -17391,6 +17606,7 @@
       <c r="AS212" s="7"/>
       <c r="AT212" s="7"/>
       <c r="AU212" s="7"/>
+      <c r="AV212" s="7"/>
     </row>
     <row r="213">
       <c r="A213" s="7" t="inlineStr">
@@ -17472,6 +17688,7 @@
       <c r="AS213" s="7"/>
       <c r="AT213" s="7"/>
       <c r="AU213" s="7"/>
+      <c r="AV213" s="7"/>
     </row>
     <row r="214">
       <c r="A214" s="7" t="inlineStr">
@@ -17549,6 +17766,7 @@
       <c r="AS214" s="7"/>
       <c r="AT214" s="7"/>
       <c r="AU214" s="7"/>
+      <c r="AV214" s="7"/>
     </row>
     <row r="215">
       <c r="A215" s="7" t="inlineStr">
@@ -17622,6 +17840,7 @@
       <c r="AS215" s="7"/>
       <c r="AT215" s="7"/>
       <c r="AU215" s="7"/>
+      <c r="AV215" s="7"/>
     </row>
     <row r="216">
       <c r="A216" s="7" t="inlineStr">
@@ -17695,6 +17914,7 @@
       <c r="AS216" s="7"/>
       <c r="AT216" s="7"/>
       <c r="AU216" s="7"/>
+      <c r="AV216" s="7"/>
     </row>
     <row r="217">
       <c r="A217" s="7" t="inlineStr">
@@ -17772,6 +17992,7 @@
       <c r="AS217" s="7"/>
       <c r="AT217" s="7"/>
       <c r="AU217" s="7"/>
+      <c r="AV217" s="7"/>
     </row>
     <row r="218">
       <c r="A218" s="7" t="inlineStr">
@@ -17845,6 +18066,7 @@
       <c r="AS218" s="7"/>
       <c r="AT218" s="7"/>
       <c r="AU218" s="7"/>
+      <c r="AV218" s="7"/>
     </row>
     <row r="219">
       <c r="A219" s="7" t="inlineStr">
@@ -17922,6 +18144,7 @@
       <c r="AS219" s="7"/>
       <c r="AT219" s="7"/>
       <c r="AU219" s="7"/>
+      <c r="AV219" s="7"/>
     </row>
     <row r="220">
       <c r="A220" s="7" t="inlineStr">
@@ -17995,6 +18218,7 @@
       <c r="AS220" s="7"/>
       <c r="AT220" s="7"/>
       <c r="AU220" s="7"/>
+      <c r="AV220" s="7"/>
     </row>
     <row r="221">
       <c r="A221" s="7" t="inlineStr">
@@ -18072,6 +18296,7 @@
       <c r="AS221" s="7"/>
       <c r="AT221" s="7"/>
       <c r="AU221" s="7"/>
+      <c r="AV221" s="7"/>
     </row>
     <row r="222">
       <c r="A222" s="7" t="inlineStr">
@@ -18153,6 +18378,7 @@
       </c>
       <c r="AT222" s="7"/>
       <c r="AU222" s="7"/>
+      <c r="AV222" s="7"/>
     </row>
     <row r="223">
       <c r="A223" s="7" t="inlineStr">
@@ -18230,6 +18456,7 @@
       <c r="AS223" s="7"/>
       <c r="AT223" s="7"/>
       <c r="AU223" s="7"/>
+      <c r="AV223" s="7"/>
     </row>
     <row r="224">
       <c r="A224" s="7" t="inlineStr">
@@ -18307,6 +18534,7 @@
         </is>
       </c>
       <c r="AU224" s="7"/>
+      <c r="AV224" s="7"/>
     </row>
     <row r="225">
       <c r="A225" s="7" t="inlineStr">
@@ -18380,6 +18608,7 @@
       <c r="AS225" s="7"/>
       <c r="AT225" s="7"/>
       <c r="AU225" s="7"/>
+      <c r="AV225" s="7"/>
     </row>
     <row r="226">
       <c r="A226" s="7" t="inlineStr">
@@ -18453,6 +18682,7 @@
       <c r="AS226" s="7"/>
       <c r="AT226" s="7"/>
       <c r="AU226" s="7"/>
+      <c r="AV226" s="7"/>
     </row>
     <row r="227">
       <c r="A227" s="7" t="inlineStr">
@@ -18526,6 +18756,7 @@
       <c r="AS227" s="7"/>
       <c r="AT227" s="7"/>
       <c r="AU227" s="7"/>
+      <c r="AV227" s="7"/>
     </row>
     <row r="228">
       <c r="A228" s="7" t="inlineStr">
@@ -18603,6 +18834,7 @@
         </is>
       </c>
       <c r="AU228" s="7"/>
+      <c r="AV228" s="7"/>
     </row>
     <row r="229">
       <c r="A229" s="7" t="inlineStr">
@@ -18676,6 +18908,7 @@
       <c r="AS229" s="7"/>
       <c r="AT229" s="7"/>
       <c r="AU229" s="7"/>
+      <c r="AV229" s="7"/>
     </row>
     <row r="230">
       <c r="A230" s="7" t="inlineStr">
@@ -18753,6 +18986,7 @@
         </is>
       </c>
       <c r="AU230" s="7"/>
+      <c r="AV230" s="7"/>
     </row>
     <row r="231">
       <c r="A231" s="7" t="inlineStr">
@@ -18830,6 +19064,7 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AV231" s="7"/>
     </row>
     <row r="232">
       <c r="A232" s="7" t="inlineStr">
@@ -18903,6 +19138,7 @@
       <c r="AS232" s="7"/>
       <c r="AT232" s="7"/>
       <c r="AU232" s="7"/>
+      <c r="AV232" s="7"/>
     </row>
     <row r="233">
       <c r="A233" s="7" t="inlineStr">
@@ -18976,6 +19212,7 @@
       <c r="AS233" s="7"/>
       <c r="AT233" s="7"/>
       <c r="AU233" s="7"/>
+      <c r="AV233" s="7"/>
     </row>
     <row r="234">
       <c r="A234" s="7" t="inlineStr">
@@ -19049,6 +19286,7 @@
       <c r="AS234" s="7"/>
       <c r="AT234" s="7"/>
       <c r="AU234" s="7"/>
+      <c r="AV234" s="7"/>
     </row>
     <row r="235">
       <c r="A235" s="7" t="inlineStr">
@@ -19078,7 +19316,7 @@
       </c>
       <c r="F235" t="inlineStr">
         <is>
-          <t xml:space="preserve">#217 · 시험 SplitShots_StayOnOneTarget · 하네스: S1뒤 28.2→29.7 · S2전 Win 54.8→LoseTimeout 53/55 · S3전 43.9→44.9 · S4뒤 50.5→53.5 · AU 화면 못 봄</t>
+          <t xml:space="preserve">#217 · 시험 SplitShots_StayOnOneTarget · 하네스: S1뒤 28.2→29.7 · S2전 Win 54.8→LoseTimeout 53/55 · S3전 43.9→44.9 · S4뒤 50.5→53.5 · AU 화면 못 봄 · AV — #217 ⓐ(죽으면 남은 발 다음 표적) · S2전 Win 54.8 복귀</t>
         </is>
       </c>
       <c r="G235" s="7"/>
@@ -19122,6 +19360,11 @@
       <c r="AS235" s="7"/>
       <c r="AT235" s="7"/>
       <c r="AU235" s="7"/>
+      <c r="AV235" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="7" t="inlineStr">
@@ -19199,6 +19442,397 @@
           <t xml:space="preserve">Pass</t>
         </is>
       </c>
+      <c r="AV236" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_237</t>
+        </is>
+      </c>
+      <c r="B237" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UI</t>
+        </is>
+      </c>
+      <c r="C237" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">팔레트 라벨 맞춤</t>
+        </is>
+      </c>
+      <c r="D237" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#219 · #220</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t xml:space="preserve">팔레트 노드 · 모듈 · 벨트 요소 라벨이 같은 크기로 단추 사각 안에 드는가(창 셋)?</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PaletteLabelFit 시험(30/60/110px) · 화면 39cc2c0 세 창 단추 안 ✅ · 0d984fd 차례 보정은 캡처 잘림으로 화면 못 봄</t>
+        </is>
+      </c>
+      <c r="G237" s="7"/>
+      <c r="H237" s="7"/>
+      <c r="I237" s="7"/>
+      <c r="J237" s="7"/>
+      <c r="K237" s="7"/>
+      <c r="L237" s="7"/>
+      <c r="M237" s="7"/>
+      <c r="N237" s="7"/>
+      <c r="O237" s="7"/>
+      <c r="P237" s="7"/>
+      <c r="Q237" s="7"/>
+      <c r="R237" s="7"/>
+      <c r="S237" s="7"/>
+      <c r="T237" s="7"/>
+      <c r="U237" s="7"/>
+      <c r="V237" s="7"/>
+      <c r="W237" s="7"/>
+      <c r="X237" s="7"/>
+      <c r="Y237" s="7"/>
+      <c r="Z237" s="7"/>
+      <c r="AA237" s="7"/>
+      <c r="AB237" s="7"/>
+      <c r="AC237" s="7"/>
+      <c r="AD237" s="7"/>
+      <c r="AE237" s="7"/>
+      <c r="AF237" s="7"/>
+      <c r="AG237" s="7"/>
+      <c r="AH237" s="7"/>
+      <c r="AI237" s="7"/>
+      <c r="AJ237" s="7"/>
+      <c r="AK237" s="7"/>
+      <c r="AL237" s="7"/>
+      <c r="AM237" s="7"/>
+      <c r="AN237" s="7"/>
+      <c r="AO237" s="7"/>
+      <c r="AP237" s="7"/>
+      <c r="AQ237" s="7"/>
+      <c r="AR237" s="7"/>
+      <c r="AS237" s="7"/>
+      <c r="AT237" s="7"/>
+      <c r="AU237" s="7"/>
+      <c r="AV237" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_238</t>
+        </is>
+      </c>
+      <c r="B238" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UI</t>
+        </is>
+      </c>
+      <c r="C238" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">프로필 칩</t>
+        </is>
+      </c>
+      <c r="D238" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#221</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HUD 프로필 칩이 이름만이고 「전투력 N」이 없는가?</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t xml:space="preserve">화면 bd3e690 「MechPilot01」만 ✅</t>
+        </is>
+      </c>
+      <c r="G238" s="7"/>
+      <c r="H238" s="7"/>
+      <c r="I238" s="7"/>
+      <c r="J238" s="7"/>
+      <c r="K238" s="7"/>
+      <c r="L238" s="7"/>
+      <c r="M238" s="7"/>
+      <c r="N238" s="7"/>
+      <c r="O238" s="7"/>
+      <c r="P238" s="7"/>
+      <c r="Q238" s="7"/>
+      <c r="R238" s="7"/>
+      <c r="S238" s="7"/>
+      <c r="T238" s="7"/>
+      <c r="U238" s="7"/>
+      <c r="V238" s="7"/>
+      <c r="W238" s="7"/>
+      <c r="X238" s="7"/>
+      <c r="Y238" s="7"/>
+      <c r="Z238" s="7"/>
+      <c r="AA238" s="7"/>
+      <c r="AB238" s="7"/>
+      <c r="AC238" s="7"/>
+      <c r="AD238" s="7"/>
+      <c r="AE238" s="7"/>
+      <c r="AF238" s="7"/>
+      <c r="AG238" s="7"/>
+      <c r="AH238" s="7"/>
+      <c r="AI238" s="7"/>
+      <c r="AJ238" s="7"/>
+      <c r="AK238" s="7"/>
+      <c r="AL238" s="7"/>
+      <c r="AM238" s="7"/>
+      <c r="AN238" s="7"/>
+      <c r="AO238" s="7"/>
+      <c r="AP238" s="7"/>
+      <c r="AQ238" s="7"/>
+      <c r="AR238" s="7"/>
+      <c r="AS238" s="7"/>
+      <c r="AT238" s="7"/>
+      <c r="AU238" s="7"/>
+      <c r="AV238" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_239</t>
+        </is>
+      </c>
+      <c r="B239" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UI</t>
+        </is>
+      </c>
+      <c r="C239" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">배지 목표 줄</t>
+        </is>
+      </c>
+      <c r="D239" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#224</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t xml:space="preserve">파밍 배지 「파밍: {주제}」 한 줄 · 도전 「목표: {주제}」가 카드 안에 드는가?</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BadgeLineFit 시험 · 화면 7efab39 S6 「파밍: 자유 플레이 · 보스」 한 줄 ✅</t>
+        </is>
+      </c>
+      <c r="G239" s="7"/>
+      <c r="H239" s="7"/>
+      <c r="I239" s="7"/>
+      <c r="J239" s="7"/>
+      <c r="K239" s="7"/>
+      <c r="L239" s="7"/>
+      <c r="M239" s="7"/>
+      <c r="N239" s="7"/>
+      <c r="O239" s="7"/>
+      <c r="P239" s="7"/>
+      <c r="Q239" s="7"/>
+      <c r="R239" s="7"/>
+      <c r="S239" s="7"/>
+      <c r="T239" s="7"/>
+      <c r="U239" s="7"/>
+      <c r="V239" s="7"/>
+      <c r="W239" s="7"/>
+      <c r="X239" s="7"/>
+      <c r="Y239" s="7"/>
+      <c r="Z239" s="7"/>
+      <c r="AA239" s="7"/>
+      <c r="AB239" s="7"/>
+      <c r="AC239" s="7"/>
+      <c r="AD239" s="7"/>
+      <c r="AE239" s="7"/>
+      <c r="AF239" s="7"/>
+      <c r="AG239" s="7"/>
+      <c r="AH239" s="7"/>
+      <c r="AI239" s="7"/>
+      <c r="AJ239" s="7"/>
+      <c r="AK239" s="7"/>
+      <c r="AL239" s="7"/>
+      <c r="AM239" s="7"/>
+      <c r="AN239" s="7"/>
+      <c r="AO239" s="7"/>
+      <c r="AP239" s="7"/>
+      <c r="AQ239" s="7"/>
+      <c r="AR239" s="7"/>
+      <c r="AS239" s="7"/>
+      <c r="AT239" s="7"/>
+      <c r="AU239" s="7"/>
+      <c r="AV239" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_240</t>
+        </is>
+      </c>
+      <c r="B240" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전투</t>
+        </is>
+      </c>
+      <c r="C240" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">도전 진입 만재</t>
+        </is>
+      </c>
+      <c r="D240" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#223</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t xml:space="preserve">S4 · S5 · S6 도전(다시 도전 포함)이 마운트 A·B 가득으로 시작하고 판을 넘는가?</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t xml:space="preserve">하네스 Docs/261020_fill223.md: B 가득 + 즉시 합체 = S6 시작 보드 Timeout 411 · 프리셋 Timeout 6874 · S5 프리셋 Timeout(B 0 이면 Win 31.0) / 45초 합체는 Win · 화면 7efab39 처음부터 → S6 → B 강화 → 도전(A 40 · B 38) → 즉시 합체 → 시간 초과(보스 ≈30%) — 7635b57 같은 길 승리(00:41)</t>
+        </is>
+      </c>
+      <c r="G240" s="7"/>
+      <c r="H240" s="7"/>
+      <c r="I240" s="7"/>
+      <c r="J240" s="7"/>
+      <c r="K240" s="7"/>
+      <c r="L240" s="7"/>
+      <c r="M240" s="7"/>
+      <c r="N240" s="7"/>
+      <c r="O240" s="7"/>
+      <c r="P240" s="7"/>
+      <c r="Q240" s="7"/>
+      <c r="R240" s="7"/>
+      <c r="S240" s="7"/>
+      <c r="T240" s="7"/>
+      <c r="U240" s="7"/>
+      <c r="V240" s="7"/>
+      <c r="W240" s="7"/>
+      <c r="X240" s="7"/>
+      <c r="Y240" s="7"/>
+      <c r="Z240" s="7"/>
+      <c r="AA240" s="7"/>
+      <c r="AB240" s="7"/>
+      <c r="AC240" s="7"/>
+      <c r="AD240" s="7"/>
+      <c r="AE240" s="7"/>
+      <c r="AF240" s="7"/>
+      <c r="AG240" s="7"/>
+      <c r="AH240" s="7"/>
+      <c r="AI240" s="7"/>
+      <c r="AJ240" s="7"/>
+      <c r="AK240" s="7"/>
+      <c r="AL240" s="7"/>
+      <c r="AM240" s="7"/>
+      <c r="AN240" s="7"/>
+      <c r="AO240" s="7"/>
+      <c r="AP240" s="7"/>
+      <c r="AQ240" s="7"/>
+      <c r="AR240" s="7"/>
+      <c r="AS240" s="7"/>
+      <c r="AT240" s="7"/>
+      <c r="AU240" s="7"/>
+      <c r="AV240" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CID_241</t>
+        </is>
+      </c>
+      <c r="B241" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">튜토리얼</t>
+        </is>
+      </c>
+      <c r="C241" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">처음부터 프리셋</t>
+        </is>
+      </c>
+      <c r="D241" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">#225</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t xml:space="preserve">바로가기 S5/S6 를 누른 저장에서 「처음부터」 뒤 자연 진행 S5 의 A 판이 시작 보드이고 폭발탄 막이 뜨는가?</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t xml:space="preserve">코드 가름: 처음부터 경로에 프리셋을 되살리는 자리 없음 · 방어 = 플래그 · 자동 완성 끔 + 시작 판 즉시 게시 · 화면 못 봄(T1 끌기)</t>
+        </is>
+      </c>
+      <c r="G241" s="7"/>
+      <c r="H241" s="7"/>
+      <c r="I241" s="7"/>
+      <c r="J241" s="7"/>
+      <c r="K241" s="7"/>
+      <c r="L241" s="7"/>
+      <c r="M241" s="7"/>
+      <c r="N241" s="7"/>
+      <c r="O241" s="7"/>
+      <c r="P241" s="7"/>
+      <c r="Q241" s="7"/>
+      <c r="R241" s="7"/>
+      <c r="S241" s="7"/>
+      <c r="T241" s="7"/>
+      <c r="U241" s="7"/>
+      <c r="V241" s="7"/>
+      <c r="W241" s="7"/>
+      <c r="X241" s="7"/>
+      <c r="Y241" s="7"/>
+      <c r="Z241" s="7"/>
+      <c r="AA241" s="7"/>
+      <c r="AB241" s="7"/>
+      <c r="AC241" s="7"/>
+      <c r="AD241" s="7"/>
+      <c r="AE241" s="7"/>
+      <c r="AF241" s="7"/>
+      <c r="AG241" s="7"/>
+      <c r="AH241" s="7"/>
+      <c r="AI241" s="7"/>
+      <c r="AJ241" s="7"/>
+      <c r="AK241" s="7"/>
+      <c r="AL241" s="7"/>
+      <c r="AM241" s="7"/>
+      <c r="AN241" s="7"/>
+      <c r="AO241" s="7"/>
+      <c r="AP241" s="7"/>
+      <c r="AQ241" s="7"/>
+      <c r="AR241" s="7"/>
+      <c r="AS241" s="7"/>
+      <c r="AT241" s="7"/>
+      <c r="AU241" s="7"/>
+      <c r="AV241" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="26">
@@ -19227,9 +19861,9 @@
     <mergeCell ref="B92:B99"/>
     <mergeCell ref="B100:B106"/>
     <mergeCell ref="B107:B111"/>
-    <mergeCell ref="G7:AU7"/>
+    <mergeCell ref="G7:AV7"/>
   </mergeCells>
-  <conditionalFormatting sqref="G9:AU236">
+  <conditionalFormatting sqref="G9:AV241">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>

</xml_diff>

<commit_message>
QA AV: CID_200 Pass(10-20 플랜 화면 S6 승리)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/QA/MechBoardIdle_QA_261014.xlsx
+++ b/Docs/QA/MechBoardIdle_QA_261014.xlsx
@@ -17218,7 +17218,7 @@
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t xml:space="preserve">4a6f983 사용자 육안 = 시간 초과(보스 ≈30%) · 조건 = 옛 저장(#197 전 A 판 리셋 · HUD 전투력 0) — 새 저장으로 재확인 자리 · AQ Fail — 시간 초과 · 보스 ≈40% 남음. 🗑️(정정) 「A 판이 폭발탄 1·2걸음만 된 채」는 틀림 — 바로가기 S6 점프가 #167 폭발탄 프리셋으로 A 판을 덮었다(새로고침 뒤 복합 가공소 확인). 조건 = 바로가기 S6 · A 판 폭발탄 프리셋 · A·B 강화 · 마운트 탄 0/200 · HUD 전투력 3→0 · 합체 1회 · AR Pass(보이는 창) — 처음부터 → S6 → B 막 강화 → 도전(A 1/40 · B 31/40 · 게이지 100%) → 즉시 합체 → 승리 남은 00:41. AQ Fail 은 숨긴 창(배경 탭) 조건</t>
+          <t xml:space="preserve">4a6f983 사용자 육안 = 시간 초과(보스 ≈30%) · 조건 = 옛 저장(#197 전 A 판 리셋 · HUD 전투력 0) — 새 저장으로 재확인 자리 · AQ Fail — 시간 초과 · 보스 ≈40% 남음. 🗑️(정정) 「A 판이 폭발탄 1·2걸음만 된 채」는 틀림 — 바로가기 S6 점프가 #167 폭발탄 프리셋으로 A 판을 덮었다(새로고침 뒤 복합 가공소 확인). 조건 = 바로가기 S6 · A 판 폭발탄 프리셋 · A·B 강화 · 마운트 탄 0/200 · HUD 전투력 3→0 · 합체 1회 · AR Pass(보이는 창) — 처음부터 → S6 → B 막 강화 → 도전(A 1/40 · B 31/40 · 게이지 100%) → 즉시 합체 → 승리 남은 00:41. AQ Fail 은 숨긴 창(배경 탭) 조건 · AV Pass — 10-20 플랜 화면 · 보이는 창 · 느린 프레임(게임 1초 ≈ 실 3~4초) · 4576641 · 처음부터 → S6 → B 강화 → 도전(A 39/40 · B 40/40 · 게이지 14%) → 합체(≈8초) → 승리 남은 00:32 · 파동 폭주 없음</t>
         </is>
       </c>
       <c r="G208" s="7"/>
@@ -17274,7 +17274,11 @@
       <c r="AS208" s="7"/>
       <c r="AT208" s="7"/>
       <c r="AU208" s="7"/>
-      <c r="AV208" s="7"/>
+      <c r="AV208" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pass</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="7" t="inlineStr">

</xml_diff>